<commit_message>
nfl hold refresh 2026-10-17 14:13 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8447,7 +8447,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-16 15:37 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-17 14:13 UTC.</t>
         </is>
       </c>
     </row>
@@ -57415,7 +57415,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-16 15:37 UTC</t>
+          <t>2026-10-17 14:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-18 14:35 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8447,7 +8447,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-17 14:13 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-18 14:35 UTC.</t>
         </is>
       </c>
     </row>
@@ -57415,7 +57415,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-17 14:13 UTC</t>
+          <t>2026-10-18 14:35 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-19 18:47 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8516,7 +8516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-19 17:22 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-19 18:47 UTC.</t>
         </is>
       </c>
     </row>
@@ -61196,7 +61196,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-19 17:22 UTC</t>
+          <t>2026-10-19 18:47 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-19 20:18 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -5865,13 +5865,13 @@
         <v>0.01856</v>
       </c>
       <c r="E69" s="15" t="n">
-        <v>116043796.66</v>
+        <v>232358252.76</v>
       </c>
       <c r="F69" s="15" t="n">
-        <v>31198857.72</v>
+        <v>52374618.16</v>
       </c>
       <c r="G69" s="16" t="n">
-        <v>0.26885</v>
+        <v>0.2254</v>
       </c>
       <c r="H69" s="17" t="inlineStr">
         <is>
@@ -5879,13 +5879,13 @@
         </is>
       </c>
       <c r="I69" s="15" t="n">
-        <v>939830431.46</v>
+        <v>1056144887.56</v>
       </c>
       <c r="J69" s="15" t="n">
-        <v>46489637.58</v>
+        <v>67665398.02</v>
       </c>
       <c r="K69" s="18" t="n">
-        <v>0.04947</v>
+        <v>0.06407</v>
       </c>
       <c r="L69" s="19" t="n">
         <v>245</v>
@@ -5936,13 +5936,13 @@
       <c r="C70" s="9" t="n"/>
       <c r="D70" s="10" t="n"/>
       <c r="E70" s="9" t="n">
-        <v>3394421.97</v>
+        <v>10166981.32</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>3436808.97</v>
+        <v>10150454.73</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>1.01249</v>
+        <v>0.99837</v>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
@@ -5950,13 +5950,13 @@
         </is>
       </c>
       <c r="I70" s="9" t="n">
-        <v>3394421.97</v>
+        <v>10166981.32</v>
       </c>
       <c r="J70" s="9" t="n">
-        <v>3436808.97</v>
+        <v>10150454.73</v>
       </c>
       <c r="K70" s="12" t="n">
-        <v>1.01249</v>
+        <v>0.99837</v>
       </c>
       <c r="L70" s="13" t="n"/>
       <c r="M70" s="13" t="n"/>
@@ -7371,13 +7371,13 @@
         <v>0.01885</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>504663323.83</v>
+        <v>627776458.8</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>95578138.56</v>
+        <v>123490105.41</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.18939</v>
+        <v>0.19671</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
@@ -7385,13 +7385,13 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>2783638743.97</v>
+        <v>2906751878.94</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>138537529.67</v>
+        <v>166449496.52</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.04977</v>
+        <v>0.05726</v>
       </c>
       <c r="L20" s="13" t="n">
         <v>625</v>
@@ -7923,10 +7923,10 @@
         <v>-0.8</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>33954624.9</v>
+        <v>114910846.96</v>
       </c>
       <c r="M10" s="10" t="n">
-        <v>0.1878</v>
+        <v>0.2195</v>
       </c>
     </row>
     <row r="11">
@@ -8516,7 +8516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-19 18:47 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-19 20:18 UTC.</t>
         </is>
       </c>
     </row>
@@ -10009,26 +10009,26 @@
         </is>
       </c>
       <c r="D13" s="15" t="n">
-        <v>2076306.62</v>
+        <v>4639033.49</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>6060270.87</v>
+        <v>13249507.62</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.1302</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>0.0242</v>
+        <v>0.0653</v>
       </c>
       <c r="H13" s="16" t="n"/>
       <c r="I13" s="16" t="n">
-        <v>0.1198</v>
+        <v>0.1168</v>
       </c>
       <c r="J13" s="19" t="n">
-        <v>46752</v>
+        <v>103496</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>77003</v>
+        <v>166554</v>
       </c>
       <c r="L13" s="31" t="n">
         <v>0</v>
@@ -12403,26 +12403,26 @@
         </is>
       </c>
       <c r="D70" s="9" t="n">
-        <v>86574.78999999999</v>
+        <v>196872.77</v>
       </c>
       <c r="E70" s="9" t="n">
-        <v>1408284.06</v>
+        <v>4009737.61</v>
       </c>
       <c r="F70" s="10" t="n">
-        <v>0.6026</v>
+        <v>0.3535</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>0.5231</v>
+        <v>0.2665</v>
       </c>
       <c r="H70" s="10" t="n"/>
       <c r="I70" s="10" t="n">
-        <v>0.0321</v>
+        <v>0.0313</v>
       </c>
       <c r="J70" s="13" t="n">
-        <v>7020</v>
+        <v>16510</v>
       </c>
       <c r="K70" s="13" t="n">
-        <v>11461</v>
+        <v>24175</v>
       </c>
       <c r="L70" s="32" t="n">
         <v>0</v>
@@ -12445,26 +12445,26 @@
         </is>
       </c>
       <c r="D71" s="15" t="n">
-        <v>680941.92</v>
+        <v>1401486.21</v>
       </c>
       <c r="E71" s="15" t="n">
-        <v>780876.74</v>
+        <v>1193927.74</v>
       </c>
       <c r="F71" s="16" t="n">
-        <v>-0.0004</v>
+        <v>0.0447</v>
       </c>
       <c r="G71" s="16" t="n">
-        <v>-0.0621</v>
+        <v>-0.0101</v>
       </c>
       <c r="H71" s="16" t="n"/>
       <c r="I71" s="16" t="n">
-        <v>0.3085</v>
+        <v>0.3169</v>
       </c>
       <c r="J71" s="19" t="n">
-        <v>3644</v>
+        <v>7254</v>
       </c>
       <c r="K71" s="19" t="n">
-        <v>11483</v>
+        <v>21993</v>
       </c>
       <c r="L71" s="31" t="n">
         <v>0</v>
@@ -12487,26 +12487,26 @@
         </is>
       </c>
       <c r="D72" s="9" t="n">
-        <v>502341.31</v>
+        <v>1137953.09</v>
       </c>
       <c r="E72" s="9" t="n">
-        <v>834848.13</v>
+        <v>1393941.47</v>
       </c>
       <c r="F72" s="10" t="n">
-        <v>0.0423</v>
+        <v>0.1458</v>
       </c>
       <c r="G72" s="10" t="n">
-        <v>-0.0246</v>
+        <v>0.0847</v>
       </c>
       <c r="H72" s="10" t="n"/>
       <c r="I72" s="10" t="n">
-        <v>0.2183</v>
+        <v>0.2184</v>
       </c>
       <c r="J72" s="13" t="n">
-        <v>6529</v>
+        <v>13583</v>
       </c>
       <c r="K72" s="13" t="n">
-        <v>13719</v>
+        <v>28119</v>
       </c>
       <c r="L72" s="32" t="n">
         <v>0</v>
@@ -12529,26 +12529,26 @@
         </is>
       </c>
       <c r="D73" s="15" t="n">
-        <v>315788.74</v>
+        <v>701610.6800000001</v>
       </c>
       <c r="E73" s="15" t="n">
-        <v>594223.78</v>
+        <v>1114284.65</v>
       </c>
       <c r="F73" s="16" t="n">
-        <v>0.1052</v>
+        <v>0.154</v>
       </c>
       <c r="G73" s="16" t="n">
-        <v>0.038</v>
+        <v>0.08840000000000001</v>
       </c>
       <c r="H73" s="16" t="n"/>
       <c r="I73" s="16" t="n">
-        <v>0.1609</v>
+        <v>0.1598</v>
       </c>
       <c r="J73" s="19" t="n">
-        <v>6793</v>
+        <v>14552</v>
       </c>
       <c r="K73" s="19" t="n">
-        <v>10187</v>
+        <v>22690</v>
       </c>
       <c r="L73" s="31" t="n">
         <v>0</v>
@@ -12571,26 +12571,26 @@
         </is>
       </c>
       <c r="D74" s="9" t="n">
-        <v>175036.42</v>
+        <v>447576.43</v>
       </c>
       <c r="E74" s="9" t="n">
-        <v>490373.2</v>
+        <v>1160837.95</v>
       </c>
       <c r="F74" s="10" t="n">
-        <v>0.0955</v>
+        <v>0.1045</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>0.0218</v>
+        <v>0.0349</v>
       </c>
       <c r="H74" s="10" t="n"/>
       <c r="I74" s="10" t="n">
-        <v>0.1249</v>
+        <v>0.1232</v>
       </c>
       <c r="J74" s="13" t="n">
-        <v>5734</v>
+        <v>12724</v>
       </c>
       <c r="K74" s="13" t="n">
-        <v>7797</v>
+        <v>17646</v>
       </c>
       <c r="L74" s="32" t="n">
         <v>0</v>
@@ -12613,26 +12613,26 @@
         </is>
       </c>
       <c r="D75" s="15" t="n">
-        <v>197778.76</v>
+        <v>474095.8</v>
       </c>
       <c r="E75" s="15" t="n">
-        <v>925005.71</v>
+        <v>1885619.14</v>
       </c>
       <c r="F75" s="16" t="n">
-        <v>0.1709</v>
+        <v>0.1976</v>
       </c>
       <c r="G75" s="16" t="n">
-        <v>0.09039999999999999</v>
+        <v>0.1196</v>
       </c>
       <c r="H75" s="16" t="n"/>
       <c r="I75" s="16" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0764</v>
       </c>
       <c r="J75" s="19" t="n">
-        <v>9344</v>
+        <v>21261</v>
       </c>
       <c r="K75" s="19" t="n">
-        <v>12274</v>
+        <v>28692</v>
       </c>
       <c r="L75" s="31" t="n">
         <v>0</v>
@@ -12655,26 +12655,26 @@
         </is>
       </c>
       <c r="D76" s="9" t="n">
-        <v>117844.67</v>
+        <v>279438.5</v>
       </c>
       <c r="E76" s="9" t="n">
-        <v>1026659.24</v>
+        <v>2491159.06</v>
       </c>
       <c r="F76" s="10" t="n">
-        <v>0.3025</v>
+        <v>0.2047</v>
       </c>
       <c r="G76" s="10" t="n">
-        <v>0.2208</v>
+        <v>0.1214</v>
       </c>
       <c r="H76" s="10" t="n"/>
       <c r="I76" s="10" t="n">
-        <v>0.0408</v>
+        <v>0.0446</v>
       </c>
       <c r="J76" s="13" t="n">
-        <v>7688</v>
+        <v>17612</v>
       </c>
       <c r="K76" s="13" t="n">
-        <v>10082</v>
+        <v>23239</v>
       </c>
       <c r="L76" s="32" t="n">
         <v>0</v>
@@ -13999,26 +13999,26 @@
         </is>
       </c>
       <c r="D108" s="9" t="n">
-        <v>40906854.55</v>
+        <v>53155308.32</v>
       </c>
       <c r="E108" s="9" t="n">
-        <v>75997426.04000001</v>
+        <v>111141974.55</v>
       </c>
       <c r="F108" s="10" t="n">
-        <v>0.3312</v>
+        <v>0.287</v>
       </c>
       <c r="G108" s="10" t="n">
-        <v>0.2781</v>
+        <v>0.2319</v>
       </c>
       <c r="H108" s="10" t="n"/>
       <c r="I108" s="10" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.1081</v>
       </c>
       <c r="J108" s="13" t="n">
-        <v>638094</v>
+        <v>798506</v>
       </c>
       <c r="K108" s="13" t="n">
-        <v>1137900</v>
+        <v>1483184</v>
       </c>
       <c r="L108" s="32" t="n">
         <v>0</v>
@@ -15889,26 +15889,26 @@
         </is>
       </c>
       <c r="D153" s="15" t="n">
-        <v>3063768.95</v>
+        <v>3613975.49</v>
       </c>
       <c r="E153" s="15" t="n">
-        <v>30286559.59</v>
+        <v>39515981.75</v>
       </c>
       <c r="F153" s="16" t="n">
-        <v>0.5453</v>
+        <v>0.4951</v>
       </c>
       <c r="G153" s="16" t="n">
-        <v>0.4758</v>
+        <v>0.4215</v>
       </c>
       <c r="H153" s="16" t="n"/>
       <c r="I153" s="16" t="n">
-        <v>0.0321</v>
+        <v>0.0413</v>
       </c>
       <c r="J153" s="19" t="n">
-        <v>203113</v>
+        <v>241669</v>
       </c>
       <c r="K153" s="19" t="n">
-        <v>290632</v>
+        <v>344040</v>
       </c>
       <c r="L153" s="31" t="n">
         <v>0</v>
@@ -15931,26 +15931,26 @@
         </is>
       </c>
       <c r="D154" s="9" t="n">
-        <v>15604440.58</v>
+        <v>21773163.68</v>
       </c>
       <c r="E154" s="9" t="n">
-        <v>10659018.28</v>
+        <v>17561417.12</v>
       </c>
       <c r="F154" s="10" t="n">
-        <v>0.1492</v>
+        <v>0.1382</v>
       </c>
       <c r="G154" s="10" t="n">
-        <v>0.1032</v>
+        <v>0.0901</v>
       </c>
       <c r="H154" s="10" t="n"/>
       <c r="I154" s="10" t="n">
-        <v>0.2967</v>
+        <v>0.3085</v>
       </c>
       <c r="J154" s="13" t="n">
-        <v>55780</v>
+        <v>78852</v>
       </c>
       <c r="K154" s="13" t="n">
-        <v>211661</v>
+        <v>317462</v>
       </c>
       <c r="L154" s="32" t="n">
         <v>0</v>
@@ -15973,26 +15973,26 @@
         </is>
       </c>
       <c r="D155" s="15" t="n">
-        <v>8149958</v>
+        <v>10378403.76</v>
       </c>
       <c r="E155" s="15" t="n">
-        <v>6990748.79</v>
+        <v>11117341.43</v>
       </c>
       <c r="F155" s="16" t="n">
-        <v>0.3359</v>
+        <v>0.2934</v>
       </c>
       <c r="G155" s="16" t="n">
-        <v>0.2845</v>
+        <v>0.24</v>
       </c>
       <c r="H155" s="16" t="n"/>
       <c r="I155" s="16" t="n">
-        <v>0.1701</v>
+        <v>0.1858</v>
       </c>
       <c r="J155" s="19" t="n">
-        <v>69796</v>
+        <v>91112</v>
       </c>
       <c r="K155" s="19" t="n">
-        <v>160469</v>
+        <v>212245</v>
       </c>
       <c r="L155" s="31" t="n">
         <v>0</v>
@@ -16015,26 +16015,26 @@
         </is>
       </c>
       <c r="D156" s="9" t="n">
-        <v>5125275.45</v>
+        <v>6542029.25</v>
       </c>
       <c r="E156" s="9" t="n">
-        <v>6688333.51</v>
+        <v>10919517.98</v>
       </c>
       <c r="F156" s="10" t="n">
-        <v>0.4169</v>
+        <v>0.3753</v>
       </c>
       <c r="G156" s="10" t="n">
-        <v>0.3612</v>
+        <v>0.3172</v>
       </c>
       <c r="H156" s="10" t="n"/>
       <c r="I156" s="10" t="n">
-        <v>0.1092</v>
+        <v>0.1277</v>
       </c>
       <c r="J156" s="13" t="n">
-        <v>71271</v>
+        <v>93361</v>
       </c>
       <c r="K156" s="13" t="n">
-        <v>131097</v>
+        <v>178049</v>
       </c>
       <c r="L156" s="32" t="n">
         <v>0</v>
@@ -16057,26 +16057,26 @@
         </is>
       </c>
       <c r="D157" s="15" t="n">
-        <v>2904771.26</v>
+        <v>3575188.13</v>
       </c>
       <c r="E157" s="15" t="n">
-        <v>4395944.33</v>
+        <v>7308717.77</v>
       </c>
       <c r="F157" s="16" t="n">
-        <v>0.4679</v>
+        <v>0.4104</v>
       </c>
       <c r="G157" s="16" t="n">
-        <v>0.4109</v>
+        <v>0.3507</v>
       </c>
       <c r="H157" s="16" t="n"/>
       <c r="I157" s="16" t="n">
-        <v>0.07829999999999999</v>
+        <v>0.09669999999999999</v>
       </c>
       <c r="J157" s="19" t="n">
-        <v>56982</v>
+        <v>71814</v>
       </c>
       <c r="K157" s="19" t="n">
-        <v>85460</v>
+        <v>110890</v>
       </c>
       <c r="L157" s="31" t="n">
         <v>0</v>
@@ -16099,26 +16099,26 @@
         </is>
       </c>
       <c r="D158" s="9" t="n">
-        <v>3652654.05</v>
+        <v>4479161.42</v>
       </c>
       <c r="E158" s="9" t="n">
-        <v>8401695.18</v>
+        <v>13011533.05</v>
       </c>
       <c r="F158" s="10" t="n">
-        <v>0.5397</v>
+        <v>0.4676</v>
       </c>
       <c r="G158" s="10" t="n">
-        <v>0.4796</v>
+        <v>0.4044</v>
       </c>
       <c r="H158" s="10" t="n"/>
       <c r="I158" s="10" t="n">
-        <v>0.0566</v>
+        <v>0.0746</v>
       </c>
       <c r="J158" s="13" t="n">
-        <v>99806</v>
+        <v>122637</v>
       </c>
       <c r="K158" s="13" t="n">
-        <v>144290</v>
+        <v>180715</v>
       </c>
       <c r="L158" s="32" t="n">
         <v>0</v>
@@ -16141,26 +16141,26 @@
         </is>
       </c>
       <c r="D159" s="15" t="n">
-        <v>2405986.26</v>
+        <v>2793386.59</v>
       </c>
       <c r="E159" s="15" t="n">
-        <v>8575126.35</v>
+        <v>11707465.45</v>
       </c>
       <c r="F159" s="16" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.4995</v>
       </c>
       <c r="G159" s="16" t="n">
-        <v>0.4959</v>
+        <v>0.4332</v>
       </c>
       <c r="H159" s="16" t="n"/>
       <c r="I159" s="16" t="n">
-        <v>0.0513</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="J159" s="19" t="n">
-        <v>81346</v>
+        <v>99061</v>
       </c>
       <c r="K159" s="19" t="n">
-        <v>114291</v>
+        <v>139783</v>
       </c>
       <c r="L159" s="31" t="n">
         <v>0</v>
@@ -16603,26 +16603,26 @@
         </is>
       </c>
       <c r="D170" s="9" t="n">
-        <v>9544957.16</v>
+        <v>16259183.52</v>
       </c>
       <c r="E170" s="9" t="n">
-        <v>7006213.23</v>
+        <v>12956752.55</v>
       </c>
       <c r="F170" s="10" t="n">
-        <v>0.3692</v>
+        <v>0.356</v>
       </c>
       <c r="G170" s="10" t="n">
-        <v>0.3149</v>
+        <v>0.3024</v>
       </c>
       <c r="H170" s="10" t="n"/>
       <c r="I170" s="10" t="n">
-        <v>0.0851</v>
+        <v>0.0927</v>
       </c>
       <c r="J170" s="13" t="n">
-        <v>164557</v>
+        <v>285750</v>
       </c>
       <c r="K170" s="13" t="n">
-        <v>348849</v>
+        <v>595535</v>
       </c>
       <c r="L170" s="32" t="n">
         <v>0</v>
@@ -19585,26 +19585,26 @@
         </is>
       </c>
       <c r="D241" s="15" t="n">
-        <v>185917.74</v>
+        <v>472175.63</v>
       </c>
       <c r="E241" s="15" t="n">
-        <v>47631.11</v>
+        <v>392050.53</v>
       </c>
       <c r="F241" s="16" t="n">
-        <v>0.5459000000000001</v>
+        <v>0.2525</v>
       </c>
       <c r="G241" s="16" t="n">
-        <v>0.5047</v>
+        <v>0.2239</v>
       </c>
       <c r="H241" s="16" t="n"/>
       <c r="I241" s="16" t="n">
-        <v>0.0241</v>
+        <v>0.0326</v>
       </c>
       <c r="J241" s="19" t="n">
-        <v>8790</v>
+        <v>14197</v>
       </c>
       <c r="K241" s="19" t="n">
-        <v>13443</v>
+        <v>24878</v>
       </c>
       <c r="L241" s="31" t="n">
         <v>0</v>
@@ -19627,26 +19627,26 @@
         </is>
       </c>
       <c r="D242" s="9" t="n">
-        <v>5333907.39</v>
+        <v>8709588.59</v>
       </c>
       <c r="E242" s="9" t="n">
-        <v>2772403.86</v>
+        <v>4533512.07</v>
       </c>
       <c r="F242" s="10" t="n">
-        <v>0.2509</v>
+        <v>0.2577</v>
       </c>
       <c r="G242" s="10" t="n">
-        <v>0.2002</v>
+        <v>0.2076</v>
       </c>
       <c r="H242" s="10" t="n"/>
       <c r="I242" s="10" t="n">
-        <v>0.2313</v>
+        <v>0.2328</v>
       </c>
       <c r="J242" s="13" t="n">
-        <v>20164</v>
+        <v>34777</v>
       </c>
       <c r="K242" s="13" t="n">
-        <v>127072</v>
+        <v>207524</v>
       </c>
       <c r="L242" s="32" t="n">
         <v>0</v>
@@ -19669,26 +19669,26 @@
         </is>
       </c>
       <c r="D243" s="15" t="n">
-        <v>1631580.99</v>
+        <v>2785695.25</v>
       </c>
       <c r="E243" s="15" t="n">
-        <v>1466506.56</v>
+        <v>2425218.26</v>
       </c>
       <c r="F243" s="16" t="n">
-        <v>0.3617</v>
+        <v>0.38</v>
       </c>
       <c r="G243" s="16" t="n">
-        <v>0.3041</v>
+        <v>0.3228</v>
       </c>
       <c r="H243" s="16" t="n"/>
       <c r="I243" s="16" t="n">
-        <v>0.1343</v>
+        <v>0.1447</v>
       </c>
       <c r="J243" s="19" t="n">
-        <v>32210</v>
+        <v>55252</v>
       </c>
       <c r="K243" s="19" t="n">
-        <v>60479</v>
+        <v>102299</v>
       </c>
       <c r="L243" s="31" t="n">
         <v>0</v>
@@ -19711,26 +19711,26 @@
         </is>
       </c>
       <c r="D244" s="9" t="n">
-        <v>1134708.92</v>
+        <v>1933069.3</v>
       </c>
       <c r="E244" s="9" t="n">
-        <v>1165848.05</v>
+        <v>1882261.34</v>
       </c>
       <c r="F244" s="10" t="n">
-        <v>0.5219</v>
+        <v>0.454</v>
       </c>
       <c r="G244" s="10" t="n">
-        <v>0.4662</v>
+        <v>0.3972</v>
       </c>
       <c r="H244" s="10" t="n"/>
       <c r="I244" s="10" t="n">
-        <v>0.0819</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="J244" s="13" t="n">
-        <v>32016</v>
+        <v>55617</v>
       </c>
       <c r="K244" s="13" t="n">
-        <v>51192</v>
+        <v>88262</v>
       </c>
       <c r="L244" s="32" t="n">
         <v>0</v>
@@ -19753,26 +19753,26 @@
         </is>
       </c>
       <c r="D245" s="15" t="n">
-        <v>455466.18</v>
+        <v>851471.2</v>
       </c>
       <c r="E245" s="15" t="n">
-        <v>548795.77</v>
+        <v>1087375.82</v>
       </c>
       <c r="F245" s="16" t="n">
-        <v>0.6659</v>
+        <v>0.5916</v>
       </c>
       <c r="G245" s="16" t="n">
-        <v>0.6005</v>
+        <v>0.5262</v>
       </c>
       <c r="H245" s="16" t="n"/>
       <c r="I245" s="16" t="n">
-        <v>0.0496</v>
+        <v>0.0618</v>
       </c>
       <c r="J245" s="19" t="n">
-        <v>22580</v>
+        <v>40228</v>
       </c>
       <c r="K245" s="19" t="n">
-        <v>28484</v>
+        <v>52602</v>
       </c>
       <c r="L245" s="31" t="n">
         <v>0</v>
@@ -19795,26 +19795,26 @@
         </is>
       </c>
       <c r="D246" s="9" t="n">
-        <v>565396.3199999999</v>
+        <v>1006735.89</v>
       </c>
       <c r="E246" s="9" t="n">
-        <v>776902.67</v>
+        <v>1795455.89</v>
       </c>
       <c r="F246" s="10" t="n">
-        <v>0.6949</v>
+        <v>0.6306</v>
       </c>
       <c r="G246" s="10" t="n">
-        <v>0.6294</v>
+        <v>0.5645</v>
       </c>
       <c r="H246" s="10" t="n"/>
       <c r="I246" s="10" t="n">
-        <v>0.0274</v>
+        <v>0.0335</v>
       </c>
       <c r="J246" s="13" t="n">
-        <v>29835</v>
+        <v>52884</v>
       </c>
       <c r="K246" s="13" t="n">
-        <v>45498</v>
+        <v>78566</v>
       </c>
       <c r="L246" s="32" t="n">
         <v>0</v>
@@ -19837,26 +19837,26 @@
         </is>
       </c>
       <c r="D247" s="15" t="n">
-        <v>237979.61</v>
+        <v>500447.66</v>
       </c>
       <c r="E247" s="15" t="n">
-        <v>228125.21</v>
+        <v>840878.63</v>
       </c>
       <c r="F247" s="16" t="n">
-        <v>0.8629</v>
+        <v>0.697</v>
       </c>
       <c r="G247" s="16" t="n">
-        <v>0.7951</v>
+        <v>0.6395</v>
       </c>
       <c r="H247" s="16" t="n"/>
       <c r="I247" s="16" t="n">
-        <v>0.0127</v>
+        <v>0.0169</v>
       </c>
       <c r="J247" s="19" t="n">
-        <v>18962</v>
+        <v>32795</v>
       </c>
       <c r="K247" s="19" t="n">
-        <v>22681</v>
+        <v>41404</v>
       </c>
       <c r="L247" s="31" t="n">
         <v>0</v>
@@ -20509,26 +20509,26 @@
         </is>
       </c>
       <c r="D263" s="15" t="n">
-        <v>3134447.66</v>
+        <v>4614239.69</v>
       </c>
       <c r="E263" s="15" t="n">
-        <v>11077474.42</v>
+        <v>12393478.9</v>
       </c>
       <c r="F263" s="16" t="n">
-        <v>0.1622</v>
+        <v>0.1834</v>
       </c>
       <c r="G263" s="16" t="n">
-        <v>0.1084</v>
+        <v>0.1299</v>
       </c>
       <c r="H263" s="16" t="n"/>
       <c r="I263" s="16" t="n">
-        <v>0.1258</v>
+        <v>0.1288</v>
       </c>
       <c r="J263" s="19" t="n">
-        <v>50401</v>
+        <v>72199</v>
       </c>
       <c r="K263" s="19" t="n">
-        <v>142497</v>
+        <v>203609</v>
       </c>
       <c r="L263" s="31" t="n">
         <v>0</v>
@@ -24793,26 +24793,26 @@
         </is>
       </c>
       <c r="D365" s="15" t="n">
-        <v>106707.99</v>
+        <v>114759.6</v>
       </c>
       <c r="E365" s="15" t="n">
-        <v>3394150.93</v>
+        <v>3395004.68</v>
       </c>
       <c r="F365" s="16" t="n">
-        <v>0.6274999999999999</v>
+        <v>0.654</v>
       </c>
       <c r="G365" s="16" t="n">
-        <v>0.5514</v>
+        <v>0.5785</v>
       </c>
       <c r="H365" s="16" t="n"/>
       <c r="I365" s="16" t="n">
-        <v>0.0302</v>
+        <v>0.0273</v>
       </c>
       <c r="J365" s="19" t="n">
-        <v>6992</v>
+        <v>7759</v>
       </c>
       <c r="K365" s="19" t="n">
-        <v>21516</v>
+        <v>22609</v>
       </c>
       <c r="L365" s="31" t="n">
         <v>0</v>
@@ -24835,26 +24835,26 @@
         </is>
       </c>
       <c r="D366" s="9" t="n">
-        <v>1334389.84</v>
+        <v>2077101.92</v>
       </c>
       <c r="E366" s="9" t="n">
-        <v>794516.9300000001</v>
+        <v>1137970.7</v>
       </c>
       <c r="F366" s="10" t="n">
-        <v>0.1206</v>
+        <v>0.09320000000000001</v>
       </c>
       <c r="G366" s="10" t="n">
-        <v>0.0746</v>
+        <v>0.0485</v>
       </c>
       <c r="H366" s="10" t="n"/>
       <c r="I366" s="10" t="n">
-        <v>0.3118</v>
+        <v>0.3117</v>
       </c>
       <c r="J366" s="13" t="n">
-        <v>7491</v>
+        <v>12232</v>
       </c>
       <c r="K366" s="13" t="n">
-        <v>26269</v>
+        <v>41665</v>
       </c>
       <c r="L366" s="32" t="n">
         <v>0</v>
@@ -24877,26 +24877,26 @@
         </is>
       </c>
       <c r="D367" s="15" t="n">
-        <v>751560.99</v>
+        <v>1007634.37</v>
       </c>
       <c r="E367" s="15" t="n">
-        <v>915737.99</v>
+        <v>1113439.17</v>
       </c>
       <c r="F367" s="16" t="n">
-        <v>0.1942</v>
+        <v>0.1515</v>
       </c>
       <c r="G367" s="16" t="n">
-        <v>0.1451</v>
+        <v>0.1002</v>
       </c>
       <c r="H367" s="16" t="n"/>
       <c r="I367" s="16" t="n">
-        <v>0.2203</v>
+        <v>0.2114</v>
       </c>
       <c r="J367" s="19" t="n">
-        <v>6363</v>
+        <v>9888</v>
       </c>
       <c r="K367" s="19" t="n">
-        <v>19369</v>
+        <v>30439</v>
       </c>
       <c r="L367" s="31" t="n">
         <v>0</v>
@@ -24919,26 +24919,26 @@
         </is>
       </c>
       <c r="D368" s="9" t="n">
-        <v>357051.23</v>
+        <v>533580.78</v>
       </c>
       <c r="E368" s="9" t="n">
-        <v>683564.4300000001</v>
+        <v>913057.83</v>
       </c>
       <c r="F368" s="10" t="n">
-        <v>0.1727</v>
+        <v>0.2568</v>
       </c>
       <c r="G368" s="10" t="n">
-        <v>0.1174</v>
+        <v>0.1994</v>
       </c>
       <c r="H368" s="10" t="n"/>
       <c r="I368" s="10" t="n">
-        <v>0.1521</v>
+        <v>0.1451</v>
       </c>
       <c r="J368" s="13" t="n">
-        <v>6899</v>
+        <v>10415</v>
       </c>
       <c r="K368" s="13" t="n">
-        <v>14903</v>
+        <v>23290</v>
       </c>
       <c r="L368" s="32" t="n">
         <v>0</v>
@@ -24961,26 +24961,26 @@
         </is>
       </c>
       <c r="D369" s="15" t="n">
-        <v>180978.45</v>
+        <v>326155.76</v>
       </c>
       <c r="E369" s="15" t="n">
-        <v>478600.7</v>
+        <v>864369.35</v>
       </c>
       <c r="F369" s="16" t="n">
-        <v>0.1561</v>
+        <v>0.3362</v>
       </c>
       <c r="G369" s="16" t="n">
-        <v>0.096</v>
+        <v>0.2711</v>
       </c>
       <c r="H369" s="16" t="n"/>
       <c r="I369" s="16" t="n">
-        <v>0.0992</v>
+        <v>0.0819</v>
       </c>
       <c r="J369" s="19" t="n">
-        <v>5069</v>
+        <v>8325</v>
       </c>
       <c r="K369" s="19" t="n">
-        <v>10249</v>
+        <v>21427</v>
       </c>
       <c r="L369" s="31" t="n">
         <v>0</v>
@@ -25003,26 +25003,26 @@
         </is>
       </c>
       <c r="D370" s="9" t="n">
-        <v>226869.52</v>
+        <v>348361.96</v>
       </c>
       <c r="E370" s="9" t="n">
-        <v>1555082.27</v>
+        <v>1675455.53</v>
       </c>
       <c r="F370" s="10" t="n">
-        <v>-0.0385</v>
+        <v>0.2821</v>
       </c>
       <c r="G370" s="10" t="n">
-        <v>-0.1183</v>
+        <v>0.2071</v>
       </c>
       <c r="H370" s="10" t="n"/>
       <c r="I370" s="10" t="n">
-        <v>0.0617</v>
+        <v>0.0529</v>
       </c>
       <c r="J370" s="13" t="n">
-        <v>9159</v>
+        <v>13043</v>
       </c>
       <c r="K370" s="13" t="n">
-        <v>19768</v>
+        <v>31137</v>
       </c>
       <c r="L370" s="32" t="n">
         <v>0</v>
@@ -25045,26 +25045,26 @@
         </is>
       </c>
       <c r="D371" s="15" t="n">
-        <v>176889.63</v>
+        <v>206645.31</v>
       </c>
       <c r="E371" s="15" t="n">
-        <v>3255821.18</v>
+        <v>3294181.65</v>
       </c>
       <c r="F371" s="16" t="n">
-        <v>0.3009</v>
+        <v>0.3875</v>
       </c>
       <c r="G371" s="16" t="n">
-        <v>0.2241</v>
+        <v>0.3122</v>
       </c>
       <c r="H371" s="16" t="n"/>
       <c r="I371" s="16" t="n">
-        <v>0.0323</v>
+        <v>0.0285</v>
       </c>
       <c r="J371" s="19" t="n">
-        <v>8428</v>
+        <v>10537</v>
       </c>
       <c r="K371" s="19" t="n">
-        <v>30423</v>
+        <v>33042</v>
       </c>
       <c r="L371" s="31" t="n">
         <v>0</v>
@@ -26319,31 +26319,31 @@
         </is>
       </c>
       <c r="D400" s="9" t="n">
-        <v>33954624.9</v>
+        <v>114910846.96</v>
       </c>
       <c r="E400" s="9" t="n">
-        <v>84085135.65000001</v>
+        <v>211976300.01</v>
       </c>
       <c r="F400" s="10" t="n">
-        <v>0.1878</v>
+        <v>0.2195</v>
       </c>
       <c r="G400" s="10" t="n">
-        <v>0.1262</v>
+        <v>0.1639</v>
       </c>
       <c r="H400" s="10" t="n">
-        <v>0.152</v>
+        <v>0.1183</v>
       </c>
       <c r="I400" s="10" t="n">
-        <v>0.0766</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="J400" s="13" t="n">
-        <v>951576</v>
+        <v>2210360</v>
       </c>
       <c r="K400" s="13" t="n">
-        <v>1926060</v>
+        <v>4676070</v>
       </c>
       <c r="L400" s="32" t="n">
-        <v>0.5442</v>
+        <v>0.4437</v>
       </c>
     </row>
     <row r="401">
@@ -34891,31 +34891,31 @@
         </is>
       </c>
       <c r="D595" s="15" t="n">
-        <v>3075500.61</v>
+        <v>7212672.01</v>
       </c>
       <c r="E595" s="15" t="n">
-        <v>38940373.65</v>
+        <v>86185959.48999999</v>
       </c>
       <c r="F595" s="16" t="n">
-        <v>0.7124</v>
+        <v>0.678</v>
       </c>
       <c r="G595" s="16" t="n">
-        <v>0.6387</v>
+        <v>0.6058</v>
       </c>
       <c r="H595" s="16" t="n">
-        <v>0.541</v>
+        <v>0.4735</v>
       </c>
       <c r="I595" s="16" t="n">
-        <v>0.0119</v>
+        <v>0.0149</v>
       </c>
       <c r="J595" s="19" t="n">
-        <v>203482</v>
+        <v>443767</v>
       </c>
       <c r="K595" s="19" t="n">
-        <v>381719</v>
+        <v>813247</v>
       </c>
       <c r="L595" s="31" t="n">
-        <v>0.6551</v>
+        <v>0.5498</v>
       </c>
     </row>
     <row r="596">
@@ -34935,31 +34935,31 @@
         </is>
       </c>
       <c r="D596" s="9" t="n">
-        <v>9385921.77</v>
+        <v>34731296.41</v>
       </c>
       <c r="E596" s="9" t="n">
-        <v>6856606.55</v>
+        <v>21044773.82</v>
       </c>
       <c r="F596" s="10" t="n">
-        <v>0.154</v>
+        <v>0.1057</v>
       </c>
       <c r="G596" s="10" t="n">
-        <v>0.0997</v>
+        <v>0.057</v>
       </c>
       <c r="H596" s="10" t="n">
-        <v>0.0367</v>
+        <v>0.0299</v>
       </c>
       <c r="I596" s="10" t="n">
-        <v>0.2435</v>
+        <v>0.2529</v>
       </c>
       <c r="J596" s="13" t="n">
-        <v>52088</v>
+        <v>142898</v>
       </c>
       <c r="K596" s="13" t="n">
-        <v>240105</v>
+        <v>641016</v>
       </c>
       <c r="L596" s="32" t="n">
-        <v>0.4697</v>
+        <v>0.4011</v>
       </c>
     </row>
     <row r="597">
@@ -34979,31 +34979,31 @@
         </is>
       </c>
       <c r="D597" s="15" t="n">
-        <v>5268787.7</v>
+        <v>21672341.65</v>
       </c>
       <c r="E597" s="15" t="n">
-        <v>2440928.66</v>
+        <v>11328100.01</v>
       </c>
       <c r="F597" s="16" t="n">
-        <v>-0.0109</v>
+        <v>0.1362</v>
       </c>
       <c r="G597" s="16" t="n">
-        <v>-0.067</v>
+        <v>0.0848</v>
       </c>
       <c r="H597" s="16" t="n">
-        <v>0.0877</v>
+        <v>0.0587</v>
       </c>
       <c r="I597" s="16" t="n">
-        <v>0.1661</v>
+        <v>0.1735</v>
       </c>
       <c r="J597" s="19" t="n">
-        <v>94708</v>
+        <v>244326</v>
       </c>
       <c r="K597" s="19" t="n">
-        <v>217189</v>
+        <v>618459</v>
       </c>
       <c r="L597" s="31" t="n">
-        <v>0.5202</v>
+        <v>0.4059</v>
       </c>
     </row>
     <row r="598">
@@ -35023,31 +35023,31 @@
         </is>
       </c>
       <c r="D598" s="9" t="n">
-        <v>4843103.28</v>
+        <v>16621570.28</v>
       </c>
       <c r="E598" s="9" t="n">
-        <v>4159382.85</v>
+        <v>13294816.87</v>
       </c>
       <c r="F598" s="10" t="n">
-        <v>-0.0026</v>
+        <v>0.0992</v>
       </c>
       <c r="G598" s="10" t="n">
-        <v>-0.0624</v>
+        <v>0.0444</v>
       </c>
       <c r="H598" s="10" t="n">
-        <v>0.1328</v>
+        <v>0.0999</v>
       </c>
       <c r="I598" s="10" t="n">
-        <v>0.1217</v>
+        <v>0.1271</v>
       </c>
       <c r="J598" s="13" t="n">
-        <v>122820</v>
+        <v>294833</v>
       </c>
       <c r="K598" s="13" t="n">
-        <v>257387</v>
+        <v>620399</v>
       </c>
       <c r="L598" s="32" t="n">
-        <v>0.5315</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="599">
@@ -35067,31 +35067,31 @@
         </is>
       </c>
       <c r="D599" s="15" t="n">
-        <v>3332641.04</v>
+        <v>11005891.12</v>
       </c>
       <c r="E599" s="15" t="n">
-        <v>5317814.46</v>
+        <v>13210194.5</v>
       </c>
       <c r="F599" s="16" t="n">
-        <v>-0.1384</v>
+        <v>0.1241</v>
       </c>
       <c r="G599" s="16" t="n">
-        <v>-0.2032</v>
+        <v>0.06710000000000001</v>
       </c>
       <c r="H599" s="16" t="n">
-        <v>0.1702</v>
+        <v>0.1353</v>
       </c>
       <c r="I599" s="16" t="n">
-        <v>0.0953</v>
+        <v>0.09810000000000001</v>
       </c>
       <c r="J599" s="19" t="n">
-        <v>114149</v>
+        <v>261949</v>
       </c>
       <c r="K599" s="19" t="n">
-        <v>180068</v>
+        <v>439771</v>
       </c>
       <c r="L599" s="31" t="n">
-        <v>0.5369</v>
+        <v>0.442</v>
       </c>
     </row>
     <row r="600">
@@ -35111,31 +35111,31 @@
         </is>
       </c>
       <c r="D600" s="9" t="n">
-        <v>4386776.78</v>
+        <v>13930929.12</v>
       </c>
       <c r="E600" s="9" t="n">
-        <v>11517715.42</v>
+        <v>34282458.42</v>
       </c>
       <c r="F600" s="10" t="n">
-        <v>0.301</v>
+        <v>0.3776</v>
       </c>
       <c r="G600" s="10" t="n">
-        <v>0.2322</v>
+        <v>0.3146</v>
       </c>
       <c r="H600" s="10" t="n">
-        <v>0.2328</v>
+        <v>0.1943</v>
       </c>
       <c r="I600" s="10" t="n">
-        <v>0.0581</v>
+        <v>0.0616</v>
       </c>
       <c r="J600" s="13" t="n">
-        <v>189693</v>
+        <v>436479</v>
       </c>
       <c r="K600" s="13" t="n">
-        <v>303415</v>
+        <v>776965</v>
       </c>
       <c r="L600" s="32" t="n">
-        <v>0.6066</v>
+        <v>0.4969</v>
       </c>
     </row>
     <row r="601">
@@ -35155,31 +35155,31 @@
         </is>
       </c>
       <c r="D601" s="15" t="n">
-        <v>3661893.72</v>
+        <v>9736146.380000001</v>
       </c>
       <c r="E601" s="15" t="n">
-        <v>14852314.06</v>
+        <v>32629996.9</v>
       </c>
       <c r="F601" s="16" t="n">
-        <v>0.5328000000000001</v>
+        <v>0.5579</v>
       </c>
       <c r="G601" s="16" t="n">
-        <v>0.464</v>
+        <v>0.4921</v>
       </c>
       <c r="H601" s="16" t="n">
-        <v>0.3431</v>
+        <v>0.3162</v>
       </c>
       <c r="I601" s="16" t="n">
-        <v>0.0296</v>
+        <v>0.0331</v>
       </c>
       <c r="J601" s="19" t="n">
-        <v>174636</v>
+        <v>386108</v>
       </c>
       <c r="K601" s="19" t="n">
-        <v>346177</v>
+        <v>766213</v>
       </c>
       <c r="L601" s="31" t="n">
-        <v>0.6254999999999999</v>
+        <v>0.5331</v>
       </c>
     </row>
     <row r="602">
@@ -35619,7 +35619,7 @@
         </is>
       </c>
       <c r="D612" s="9" t="n">
-        <v>9837150.98</v>
+        <v>9837163.289999999</v>
       </c>
       <c r="E612" s="9" t="n">
         <v>60052235.9</v>
@@ -35635,10 +35635,10 @@
         <v>0.0536</v>
       </c>
       <c r="J612" s="13" t="n">
-        <v>367836</v>
+        <v>367837</v>
       </c>
       <c r="K612" s="13" t="n">
-        <v>522286</v>
+        <v>522287</v>
       </c>
       <c r="L612" s="32" t="n">
         <v>0.6417</v>
@@ -35661,29 +35661,29 @@
         </is>
       </c>
       <c r="D613" s="15" t="n">
-        <v>5166813.85</v>
+        <v>10578903.27</v>
       </c>
       <c r="E613" s="15" t="n">
-        <v>30945991.71</v>
+        <v>61460146.15</v>
       </c>
       <c r="F613" s="16" t="n">
-        <v>0.4713</v>
+        <v>0.436</v>
       </c>
       <c r="G613" s="16" t="n">
-        <v>0.401</v>
+        <v>0.3666</v>
       </c>
       <c r="H613" s="16" t="n"/>
       <c r="I613" s="16" t="n">
-        <v>0.029</v>
+        <v>0.0414</v>
       </c>
       <c r="J613" s="19" t="n">
-        <v>238416</v>
+        <v>440254</v>
       </c>
       <c r="K613" s="19" t="n">
-        <v>337631</v>
+        <v>607867</v>
       </c>
       <c r="L613" s="31" t="n">
-        <v>0.5535</v>
+        <v>0.5063</v>
       </c>
     </row>
     <row r="614">
@@ -38769,7 +38769,7 @@
         </is>
       </c>
       <c r="D687" s="15" t="n">
-        <v>1093544.03</v>
+        <v>1093556.35</v>
       </c>
       <c r="E687" s="15" t="n">
         <v>1908846.56</v>
@@ -38785,10 +38785,10 @@
         <v>0.1538</v>
       </c>
       <c r="J687" s="19" t="n">
-        <v>18820</v>
+        <v>18821</v>
       </c>
       <c r="K687" s="19" t="n">
-        <v>27422</v>
+        <v>27423</v>
       </c>
       <c r="L687" s="31" t="n">
         <v>0.5726</v>
@@ -38937,29 +38937,29 @@
         </is>
       </c>
       <c r="D691" s="15" t="n">
-        <v>1890668.07</v>
+        <v>3130216.34</v>
       </c>
       <c r="E691" s="15" t="n">
-        <v>21658686.04</v>
+        <v>41397838.26</v>
       </c>
       <c r="F691" s="16" t="n">
-        <v>0.6832</v>
+        <v>0.6782</v>
       </c>
       <c r="G691" s="16" t="n">
-        <v>0.6021</v>
+        <v>0.5962</v>
       </c>
       <c r="H691" s="16" t="n"/>
       <c r="I691" s="16" t="n">
-        <v>0.0106</v>
+        <v>0.0114</v>
       </c>
       <c r="J691" s="19" t="n">
-        <v>148143</v>
+        <v>254315</v>
       </c>
       <c r="K691" s="19" t="n">
-        <v>222823</v>
+        <v>359463</v>
       </c>
       <c r="L691" s="31" t="n">
-        <v>0.6542</v>
+        <v>0.5918</v>
       </c>
     </row>
     <row r="692">
@@ -38979,29 +38979,29 @@
         </is>
       </c>
       <c r="D692" s="9" t="n">
-        <v>547821.74</v>
+        <v>1253725.22</v>
       </c>
       <c r="E692" s="9" t="n">
-        <v>271571.45</v>
+        <v>696964.75</v>
       </c>
       <c r="F692" s="10" t="n">
-        <v>0.1497</v>
+        <v>0.0983</v>
       </c>
       <c r="G692" s="10" t="n">
-        <v>0.1031</v>
+        <v>0.0504</v>
       </c>
       <c r="H692" s="10" t="n"/>
       <c r="I692" s="10" t="n">
-        <v>0.2604</v>
+        <v>0.2905</v>
       </c>
       <c r="J692" s="13" t="n">
-        <v>3222</v>
+        <v>7856</v>
       </c>
       <c r="K692" s="13" t="n">
-        <v>6026</v>
+        <v>16031</v>
       </c>
       <c r="L692" s="32" t="n">
-        <v>0.461</v>
+        <v>0.4411</v>
       </c>
     </row>
     <row r="693">
@@ -39021,29 +39021,29 @@
         </is>
       </c>
       <c r="D693" s="15" t="n">
-        <v>526475.51</v>
+        <v>1224883.5</v>
       </c>
       <c r="E693" s="15" t="n">
-        <v>571228.8199999999</v>
+        <v>1223196.68</v>
       </c>
       <c r="F693" s="16" t="n">
-        <v>0.4927</v>
+        <v>0.3168</v>
       </c>
       <c r="G693" s="16" t="n">
-        <v>0.4323</v>
+        <v>0.2594</v>
       </c>
       <c r="H693" s="16" t="n"/>
       <c r="I693" s="16" t="n">
-        <v>0.145</v>
+        <v>0.1908</v>
       </c>
       <c r="J693" s="19" t="n">
-        <v>6641</v>
+        <v>14671</v>
       </c>
       <c r="K693" s="19" t="n">
-        <v>10025</v>
+        <v>22773</v>
       </c>
       <c r="L693" s="31" t="n">
-        <v>0.471</v>
+        <v>0.4596</v>
       </c>
     </row>
     <row r="694">
@@ -39063,29 +39063,29 @@
         </is>
       </c>
       <c r="D694" s="9" t="n">
-        <v>429470.22</v>
+        <v>1054960.23</v>
       </c>
       <c r="E694" s="9" t="n">
-        <v>645783.03</v>
+        <v>1566789.57</v>
       </c>
       <c r="F694" s="10" t="n">
-        <v>0.3217</v>
+        <v>0.3124</v>
       </c>
       <c r="G694" s="10" t="n">
-        <v>0.2603</v>
+        <v>0.2519</v>
       </c>
       <c r="H694" s="10" t="n"/>
       <c r="I694" s="10" t="n">
-        <v>0.0919</v>
+        <v>0.1355</v>
       </c>
       <c r="J694" s="13" t="n">
-        <v>9260</v>
+        <v>19942</v>
       </c>
       <c r="K694" s="13" t="n">
-        <v>12278</v>
+        <v>27847</v>
       </c>
       <c r="L694" s="32" t="n">
-        <v>0.4247</v>
+        <v>0.4408</v>
       </c>
     </row>
     <row r="695">
@@ -39105,29 +39105,29 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>406249.54</v>
+        <v>987186.8</v>
       </c>
       <c r="E695" s="15" t="n">
-        <v>969757.1</v>
+        <v>2013902.97</v>
       </c>
       <c r="F695" s="16" t="n">
-        <v>0.487</v>
+        <v>0.3815</v>
       </c>
       <c r="G695" s="16" t="n">
-        <v>0.4187</v>
+        <v>0.3168</v>
       </c>
       <c r="H695" s="16" t="n"/>
       <c r="I695" s="16" t="n">
-        <v>0.06619999999999999</v>
+        <v>0.095</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>10837</v>
+        <v>22288</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>13902</v>
+        <v>29914</v>
       </c>
       <c r="L695" s="31" t="n">
-        <v>0.5092</v>
+        <v>0.4755</v>
       </c>
     </row>
     <row r="696">
@@ -39147,29 +39147,29 @@
         </is>
       </c>
       <c r="D696" s="9" t="n">
-        <v>667367.03</v>
+        <v>1433665.27</v>
       </c>
       <c r="E696" s="9" t="n">
-        <v>2386089.06</v>
+        <v>5025901.17</v>
       </c>
       <c r="F696" s="10" t="n">
-        <v>0.1725</v>
+        <v>0.3786</v>
       </c>
       <c r="G696" s="10" t="n">
-        <v>0.102</v>
+        <v>0.307</v>
       </c>
       <c r="H696" s="10" t="n"/>
       <c r="I696" s="10" t="n">
-        <v>0.0435</v>
+        <v>0.0605</v>
       </c>
       <c r="J696" s="13" t="n">
-        <v>24126</v>
+        <v>49354</v>
       </c>
       <c r="K696" s="13" t="n">
-        <v>29233</v>
+        <v>62778</v>
       </c>
       <c r="L696" s="32" t="n">
-        <v>0.5465</v>
+        <v>0.5004</v>
       </c>
     </row>
     <row r="697">
@@ -39189,29 +39189,29 @@
         </is>
       </c>
       <c r="D697" s="15" t="n">
-        <v>698761.74</v>
+        <v>1494265.9</v>
       </c>
       <c r="E697" s="15" t="n">
-        <v>4442876.22</v>
+        <v>9535552.75</v>
       </c>
       <c r="F697" s="16" t="n">
-        <v>0.5022</v>
+        <v>0.4879</v>
       </c>
       <c r="G697" s="16" t="n">
-        <v>0.4283</v>
+        <v>0.4097</v>
       </c>
       <c r="H697" s="16" t="n"/>
       <c r="I697" s="16" t="n">
-        <v>0.0253</v>
+        <v>0.0336</v>
       </c>
       <c r="J697" s="19" t="n">
-        <v>36187</v>
+        <v>71828</v>
       </c>
       <c r="K697" s="19" t="n">
-        <v>43344</v>
+        <v>89061</v>
       </c>
       <c r="L697" s="31" t="n">
-        <v>0.5272</v>
+        <v>0.4924</v>
       </c>
     </row>
     <row r="698">
@@ -40071,29 +40071,29 @@
         </is>
       </c>
       <c r="D718" s="9" t="n">
-        <v>11604814.78</v>
+        <v>18273106.65</v>
       </c>
       <c r="E718" s="9" t="n">
-        <v>16991670.27</v>
+        <v>33474226.13</v>
       </c>
       <c r="F718" s="10" t="n">
-        <v>0.473</v>
+        <v>0.4433</v>
       </c>
       <c r="G718" s="10" t="n">
-        <v>0.4137</v>
+        <v>0.3829</v>
       </c>
       <c r="H718" s="10" t="n"/>
       <c r="I718" s="10" t="n">
-        <v>0.0675</v>
+        <v>0.0731</v>
       </c>
       <c r="J718" s="13" t="n">
-        <v>191877</v>
+        <v>290594</v>
       </c>
       <c r="K718" s="13" t="n">
-        <v>338429</v>
+        <v>514969</v>
       </c>
       <c r="L718" s="32" t="n">
-        <v>0.3532</v>
+        <v>0.3488</v>
       </c>
     </row>
     <row r="719">
@@ -45993,29 +45993,29 @@
         </is>
       </c>
       <c r="D859" s="15" t="n">
-        <v>589807.5</v>
+        <v>907749.34</v>
       </c>
       <c r="E859" s="15" t="n">
-        <v>3439818.38</v>
+        <v>6629349.37</v>
       </c>
       <c r="F859" s="16" t="n">
-        <v>0.7778</v>
+        <v>0.7979000000000001</v>
       </c>
       <c r="G859" s="16" t="n">
-        <v>0.7079</v>
+        <v>0.7262999999999999</v>
       </c>
       <c r="H859" s="16" t="n"/>
       <c r="I859" s="16" t="n">
-        <v>0.0167</v>
+        <v>0.0173</v>
       </c>
       <c r="J859" s="19" t="n">
-        <v>39957</v>
+        <v>61885</v>
       </c>
       <c r="K859" s="19" t="n">
-        <v>52832</v>
+        <v>80793</v>
       </c>
       <c r="L859" s="31" t="n">
-        <v>0.4435</v>
+        <v>0.4272</v>
       </c>
     </row>
     <row r="860">
@@ -46035,29 +46035,29 @@
         </is>
       </c>
       <c r="D860" s="9" t="n">
-        <v>4294387.91</v>
+        <v>6491506.38</v>
       </c>
       <c r="E860" s="9" t="n">
-        <v>2622599.69</v>
+        <v>4708839.08</v>
       </c>
       <c r="F860" s="10" t="n">
-        <v>0.4479</v>
+        <v>0.3923</v>
       </c>
       <c r="G860" s="10" t="n">
-        <v>0.395</v>
+        <v>0.3395</v>
       </c>
       <c r="H860" s="10" t="n"/>
       <c r="I860" s="10" t="n">
-        <v>0.2702</v>
+        <v>0.2763</v>
       </c>
       <c r="J860" s="13" t="n">
-        <v>9837</v>
+        <v>15326</v>
       </c>
       <c r="K860" s="13" t="n">
-        <v>70419</v>
+        <v>102933</v>
       </c>
       <c r="L860" s="32" t="n">
-        <v>0.3456</v>
+        <v>0.3481</v>
       </c>
     </row>
     <row r="861">
@@ -46077,29 +46077,29 @@
         </is>
       </c>
       <c r="D861" s="15" t="n">
-        <v>2706399.06</v>
+        <v>4101808.97</v>
       </c>
       <c r="E861" s="15" t="n">
-        <v>1993918.82</v>
+        <v>3867800.25</v>
       </c>
       <c r="F861" s="16" t="n">
-        <v>0.4522</v>
+        <v>0.3735</v>
       </c>
       <c r="G861" s="16" t="n">
-        <v>0.3943</v>
+        <v>0.3151</v>
       </c>
       <c r="H861" s="16" t="n"/>
       <c r="I861" s="16" t="n">
-        <v>0.1527</v>
+        <v>0.1611</v>
       </c>
       <c r="J861" s="19" t="n">
-        <v>21356</v>
+        <v>32637</v>
       </c>
       <c r="K861" s="19" t="n">
-        <v>56715</v>
+        <v>82503</v>
       </c>
       <c r="L861" s="31" t="n">
-        <v>0.3128</v>
+        <v>0.3106</v>
       </c>
     </row>
     <row r="862">
@@ -46119,29 +46119,29 @@
         </is>
       </c>
       <c r="D862" s="9" t="n">
-        <v>1429775.93</v>
+        <v>2463078.47</v>
       </c>
       <c r="E862" s="9" t="n">
-        <v>1886420.19</v>
+        <v>4144422.03</v>
       </c>
       <c r="F862" s="10" t="n">
-        <v>0.3721</v>
+        <v>0.3231</v>
       </c>
       <c r="G862" s="10" t="n">
-        <v>0.3088</v>
+        <v>0.2592</v>
       </c>
       <c r="H862" s="10" t="n"/>
       <c r="I862" s="10" t="n">
-        <v>0.0926</v>
+        <v>0.1028</v>
       </c>
       <c r="J862" s="13" t="n">
-        <v>25984</v>
+        <v>39006</v>
       </c>
       <c r="K862" s="13" t="n">
-        <v>38259</v>
+        <v>61662</v>
       </c>
       <c r="L862" s="32" t="n">
-        <v>0.3644</v>
+        <v>0.341</v>
       </c>
     </row>
     <row r="863">
@@ -46161,29 +46161,29 @@
         </is>
       </c>
       <c r="D863" s="15" t="n">
-        <v>913409.09</v>
+        <v>1551654.64</v>
       </c>
       <c r="E863" s="15" t="n">
-        <v>1484270.54</v>
+        <v>3580812.88</v>
       </c>
       <c r="F863" s="16" t="n">
-        <v>0.552</v>
+        <v>0.5822000000000001</v>
       </c>
       <c r="G863" s="16" t="n">
-        <v>0.4885</v>
+        <v>0.5154</v>
       </c>
       <c r="H863" s="16" t="n"/>
       <c r="I863" s="16" t="n">
-        <v>0.0591</v>
+        <v>0.0692</v>
       </c>
       <c r="J863" s="19" t="n">
-        <v>22479</v>
+        <v>33723</v>
       </c>
       <c r="K863" s="19" t="n">
-        <v>29081</v>
+        <v>47103</v>
       </c>
       <c r="L863" s="31" t="n">
-        <v>0.3888</v>
+        <v>0.3601</v>
       </c>
     </row>
     <row r="864">
@@ -46203,29 +46203,29 @@
         </is>
       </c>
       <c r="D864" s="9" t="n">
-        <v>1016972.47</v>
+        <v>1671037.44</v>
       </c>
       <c r="E864" s="9" t="n">
-        <v>2777752.1</v>
+        <v>5413739.24</v>
       </c>
       <c r="F864" s="10" t="n">
-        <v>0.503</v>
+        <v>0.5717</v>
       </c>
       <c r="G864" s="10" t="n">
-        <v>0.4355</v>
+        <v>0.5021</v>
       </c>
       <c r="H864" s="10" t="n"/>
       <c r="I864" s="10" t="n">
-        <v>0.0449</v>
+        <v>0.0491</v>
       </c>
       <c r="J864" s="13" t="n">
-        <v>38037</v>
+        <v>56891</v>
       </c>
       <c r="K864" s="13" t="n">
-        <v>48358</v>
+        <v>74515</v>
       </c>
       <c r="L864" s="32" t="n">
-        <v>0.3759</v>
+        <v>0.381</v>
       </c>
     </row>
     <row r="865">
@@ -46245,29 +46245,29 @@
         </is>
       </c>
       <c r="D865" s="15" t="n">
-        <v>654062.84</v>
+        <v>1086271.41</v>
       </c>
       <c r="E865" s="15" t="n">
-        <v>2786890.53</v>
+        <v>5129263.29</v>
       </c>
       <c r="F865" s="16" t="n">
-        <v>0.5131</v>
+        <v>0.5911999999999999</v>
       </c>
       <c r="G865" s="16" t="n">
-        <v>0.4417</v>
+        <v>0.5185999999999999</v>
       </c>
       <c r="H865" s="16" t="n"/>
       <c r="I865" s="16" t="n">
-        <v>0.0271</v>
+        <v>0.03</v>
       </c>
       <c r="J865" s="19" t="n">
-        <v>34227</v>
+        <v>51126</v>
       </c>
       <c r="K865" s="19" t="n">
-        <v>42765</v>
+        <v>65460</v>
       </c>
       <c r="L865" s="31" t="n">
-        <v>0.3794</v>
+        <v>0.384</v>
       </c>
     </row>
     <row r="866">
@@ -46665,29 +46665,29 @@
         </is>
       </c>
       <c r="D875" s="15" t="n">
-        <v>6526583.92</v>
+        <v>8116162.42</v>
       </c>
       <c r="E875" s="15" t="n">
-        <v>18847669.74</v>
+        <v>24286138.43</v>
       </c>
       <c r="F875" s="16" t="n">
-        <v>0.5044999999999999</v>
+        <v>0.4907</v>
       </c>
       <c r="G875" s="16" t="n">
-        <v>0.443</v>
+        <v>0.428</v>
       </c>
       <c r="H875" s="16" t="n"/>
       <c r="I875" s="16" t="n">
-        <v>0.05</v>
+        <v>0.0523</v>
       </c>
       <c r="J875" s="19" t="n">
-        <v>126682</v>
+        <v>155743</v>
       </c>
       <c r="K875" s="19" t="n">
-        <v>191050</v>
+        <v>231383</v>
       </c>
       <c r="L875" s="31" t="n">
-        <v>0.7532</v>
+        <v>0.7796999999999999</v>
       </c>
     </row>
     <row r="876">
@@ -49353,29 +49353,29 @@
         </is>
       </c>
       <c r="D939" s="15" t="n">
-        <v>1162501.05</v>
+        <v>1509055.64</v>
       </c>
       <c r="E939" s="15" t="n">
-        <v>8757276.369999999</v>
+        <v>11148366.61</v>
       </c>
       <c r="F939" s="16" t="n">
-        <v>0.8492</v>
+        <v>0.8524</v>
       </c>
       <c r="G939" s="16" t="n">
-        <v>0.7782</v>
+        <v>0.7804</v>
       </c>
       <c r="H939" s="16" t="n"/>
       <c r="I939" s="16" t="n">
-        <v>0.011</v>
+        <v>0.0115</v>
       </c>
       <c r="J939" s="19" t="n">
-        <v>52145</v>
+        <v>64858</v>
       </c>
       <c r="K939" s="19" t="n">
-        <v>77988</v>
+        <v>96508</v>
       </c>
       <c r="L939" s="31" t="n">
-        <v>0.8706</v>
+        <v>0.8895999999999999</v>
       </c>
     </row>
     <row r="940">
@@ -49395,29 +49395,29 @@
         </is>
       </c>
       <c r="D940" s="9" t="n">
-        <v>1226211.12</v>
+        <v>1560867.86</v>
       </c>
       <c r="E940" s="9" t="n">
-        <v>577149.73</v>
+        <v>752646.47</v>
       </c>
       <c r="F940" s="10" t="n">
-        <v>0.1357</v>
+        <v>0.0731</v>
       </c>
       <c r="G940" s="10" t="n">
-        <v>0.0878</v>
+        <v>0.0247</v>
       </c>
       <c r="H940" s="10" t="n"/>
       <c r="I940" s="10" t="n">
-        <v>0.3144</v>
+        <v>0.33</v>
       </c>
       <c r="J940" s="13" t="n">
-        <v>3969</v>
+        <v>5439</v>
       </c>
       <c r="K940" s="13" t="n">
-        <v>9958</v>
+        <v>12552</v>
       </c>
       <c r="L940" s="32" t="n">
-        <v>0.7471</v>
+        <v>0.7337</v>
       </c>
     </row>
     <row r="941">
@@ -49437,29 +49437,29 @@
         </is>
       </c>
       <c r="D941" s="15" t="n">
-        <v>1043571.83</v>
+        <v>1248767.88</v>
       </c>
       <c r="E941" s="15" t="n">
-        <v>887611.34</v>
+        <v>1086075.31</v>
       </c>
       <c r="F941" s="16" t="n">
-        <v>0.4069</v>
+        <v>0.3948</v>
       </c>
       <c r="G941" s="16" t="n">
-        <v>0.3505</v>
+        <v>0.3371</v>
       </c>
       <c r="H941" s="16" t="n"/>
       <c r="I941" s="16" t="n">
-        <v>0.1732</v>
+        <v>0.1793</v>
       </c>
       <c r="J941" s="19" t="n">
-        <v>8122</v>
+        <v>10154</v>
       </c>
       <c r="K941" s="19" t="n">
-        <v>14294</v>
+        <v>16975</v>
       </c>
       <c r="L941" s="31" t="n">
-        <v>0.6412</v>
+        <v>0.6848</v>
       </c>
     </row>
     <row r="942">
@@ -49479,29 +49479,29 @@
         </is>
       </c>
       <c r="D942" s="9" t="n">
-        <v>893069.53</v>
+        <v>1074862.34</v>
       </c>
       <c r="E942" s="9" t="n">
-        <v>1313695.47</v>
+        <v>1619100.09</v>
       </c>
       <c r="F942" s="10" t="n">
-        <v>0.4433</v>
+        <v>0.4119</v>
       </c>
       <c r="G942" s="10" t="n">
-        <v>0.3828</v>
+        <v>0.3507</v>
       </c>
       <c r="H942" s="10" t="n"/>
       <c r="I942" s="10" t="n">
-        <v>0.1052</v>
+        <v>0.1063</v>
       </c>
       <c r="J942" s="13" t="n">
-        <v>10896</v>
+        <v>13080</v>
       </c>
       <c r="K942" s="13" t="n">
-        <v>17700</v>
+        <v>20401</v>
       </c>
       <c r="L942" s="32" t="n">
-        <v>0.6688</v>
+        <v>0.7167</v>
       </c>
     </row>
     <row r="943">
@@ -49521,29 +49521,29 @@
         </is>
       </c>
       <c r="D943" s="15" t="n">
-        <v>565357.52</v>
+        <v>685689.92</v>
       </c>
       <c r="E943" s="15" t="n">
-        <v>1092451.96</v>
+        <v>1620699.38</v>
       </c>
       <c r="F943" s="16" t="n">
-        <v>0.451</v>
+        <v>0.4778</v>
       </c>
       <c r="G943" s="16" t="n">
-        <v>0.3871</v>
+        <v>0.4122</v>
       </c>
       <c r="H943" s="16" t="n"/>
       <c r="I943" s="16" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0658</v>
       </c>
       <c r="J943" s="19" t="n">
-        <v>10068</v>
+        <v>12144</v>
       </c>
       <c r="K943" s="19" t="n">
-        <v>15159</v>
+        <v>17769</v>
       </c>
       <c r="L943" s="31" t="n">
-        <v>0.7135</v>
+        <v>0.7519</v>
       </c>
     </row>
     <row r="944">
@@ -49563,29 +49563,29 @@
         </is>
       </c>
       <c r="D944" s="9" t="n">
-        <v>821056.27</v>
+        <v>1065781.2</v>
       </c>
       <c r="E944" s="9" t="n">
-        <v>2727388.58</v>
+        <v>3517054.86</v>
       </c>
       <c r="F944" s="10" t="n">
-        <v>0.5026</v>
+        <v>0.5115</v>
       </c>
       <c r="G944" s="10" t="n">
-        <v>0.433</v>
+        <v>0.4407</v>
       </c>
       <c r="H944" s="10" t="n"/>
       <c r="I944" s="10" t="n">
-        <v>0.04</v>
+        <v>0.0416</v>
       </c>
       <c r="J944" s="13" t="n">
-        <v>20385</v>
+        <v>24621</v>
       </c>
       <c r="K944" s="13" t="n">
-        <v>28461</v>
+        <v>33630</v>
       </c>
       <c r="L944" s="32" t="n">
-        <v>0.7812</v>
+        <v>0.8214</v>
       </c>
     </row>
     <row r="945">
@@ -49605,29 +49605,29 @@
         </is>
       </c>
       <c r="D945" s="15" t="n">
-        <v>814816.59</v>
+        <v>971137.58</v>
       </c>
       <c r="E945" s="15" t="n">
-        <v>3492096.29</v>
+        <v>4542195.73</v>
       </c>
       <c r="F945" s="16" t="n">
-        <v>0.7987</v>
+        <v>0.7964</v>
       </c>
       <c r="G945" s="16" t="n">
-        <v>0.7328</v>
+        <v>0.7284</v>
       </c>
       <c r="H945" s="16" t="n"/>
       <c r="I945" s="16" t="n">
-        <v>0.0232</v>
+        <v>0.0224</v>
       </c>
       <c r="J945" s="19" t="n">
-        <v>21097</v>
+        <v>25447</v>
       </c>
       <c r="K945" s="19" t="n">
-        <v>27490</v>
+        <v>33548</v>
       </c>
       <c r="L945" s="31" t="n">
-        <v>0.8299</v>
+        <v>0.8483000000000001</v>
       </c>
     </row>
     <row r="946">
@@ -49983,26 +49983,26 @@
         </is>
       </c>
       <c r="D954" s="9" t="n">
-        <v>4268308.29</v>
+        <v>10071359.86</v>
       </c>
       <c r="E954" s="9" t="n">
-        <v>7994148.56</v>
+        <v>24287962.28</v>
       </c>
       <c r="F954" s="10" t="n">
-        <v>-0.0636</v>
+        <v>-0.0023</v>
       </c>
       <c r="G954" s="10" t="n">
-        <v>-0.1234</v>
+        <v>-0.0593</v>
       </c>
       <c r="H954" s="10" t="n"/>
       <c r="I954" s="10" t="n">
-        <v>0.1363</v>
+        <v>0.1288</v>
       </c>
       <c r="J954" s="13" t="n">
-        <v>82691</v>
+        <v>185707</v>
       </c>
       <c r="K954" s="13" t="n">
-        <v>187297</v>
+        <v>458089</v>
       </c>
       <c r="L954" s="32" t="n">
         <v>0</v>
@@ -52377,26 +52377,26 @@
         </is>
       </c>
       <c r="D1011" s="15" t="n">
-        <v>267916.13</v>
+        <v>1007980.31</v>
       </c>
       <c r="E1011" s="15" t="n">
-        <v>1540543.18</v>
+        <v>7510663.8</v>
       </c>
       <c r="F1011" s="16" t="n">
-        <v>0.4735</v>
+        <v>0.0107</v>
       </c>
       <c r="G1011" s="16" t="n">
-        <v>0.42</v>
+        <v>-0.03</v>
       </c>
       <c r="H1011" s="16" t="n"/>
       <c r="I1011" s="16" t="n">
-        <v>0.0301</v>
+        <v>0.0431</v>
       </c>
       <c r="J1011" s="19" t="n">
-        <v>12225</v>
+        <v>30415</v>
       </c>
       <c r="K1011" s="19" t="n">
-        <v>28471</v>
+        <v>90487</v>
       </c>
       <c r="L1011" s="31" t="n">
         <v>0</v>
@@ -52419,26 +52419,26 @@
         </is>
       </c>
       <c r="D1012" s="9" t="n">
-        <v>1894582.89</v>
+        <v>4185043.47</v>
       </c>
       <c r="E1012" s="9" t="n">
-        <v>2998924.71</v>
+        <v>4394532.25</v>
       </c>
       <c r="F1012" s="10" t="n">
-        <v>-0.0141</v>
+        <v>0.0095</v>
       </c>
       <c r="G1012" s="10" t="n">
-        <v>-0.07199999999999999</v>
+        <v>-0.0433</v>
       </c>
       <c r="H1012" s="10" t="n"/>
       <c r="I1012" s="10" t="n">
-        <v>0.2538</v>
+        <v>0.2555</v>
       </c>
       <c r="J1012" s="13" t="n">
-        <v>13788</v>
+        <v>27511</v>
       </c>
       <c r="K1012" s="13" t="n">
-        <v>48539</v>
+        <v>99319</v>
       </c>
       <c r="L1012" s="32" t="n">
         <v>0</v>
@@ -52461,26 +52461,26 @@
         </is>
       </c>
       <c r="D1013" s="15" t="n">
-        <v>919264.1800000001</v>
+        <v>2039971.03</v>
       </c>
       <c r="E1013" s="15" t="n">
-        <v>499700.84</v>
+        <v>1377764.42</v>
       </c>
       <c r="F1013" s="16" t="n">
-        <v>-0.0346</v>
+        <v>-0.0021</v>
       </c>
       <c r="G1013" s="16" t="n">
-        <v>-0.0919</v>
+        <v>-0.0591</v>
       </c>
       <c r="H1013" s="16" t="n"/>
       <c r="I1013" s="16" t="n">
-        <v>0.2073</v>
+        <v>0.198</v>
       </c>
       <c r="J1013" s="19" t="n">
-        <v>14093</v>
+        <v>30372</v>
       </c>
       <c r="K1013" s="19" t="n">
-        <v>34966</v>
+        <v>72600</v>
       </c>
       <c r="L1013" s="31" t="n">
         <v>0</v>
@@ -52503,26 +52503,26 @@
         </is>
       </c>
       <c r="D1014" s="9" t="n">
-        <v>490855.47</v>
+        <v>1138528.72</v>
       </c>
       <c r="E1014" s="9" t="n">
-        <v>672918</v>
+        <v>1665390.01</v>
       </c>
       <c r="F1014" s="10" t="n">
-        <v>-0.3256</v>
+        <v>-0.0342</v>
       </c>
       <c r="G1014" s="10" t="n">
-        <v>-0.3856</v>
+        <v>-0.09569999999999999</v>
       </c>
       <c r="H1014" s="10" t="n"/>
       <c r="I1014" s="10" t="n">
-        <v>0.1659</v>
+        <v>0.1502</v>
       </c>
       <c r="J1014" s="13" t="n">
-        <v>12239</v>
+        <v>27428</v>
       </c>
       <c r="K1014" s="13" t="n">
-        <v>23105</v>
+        <v>52033</v>
       </c>
       <c r="L1014" s="32" t="n">
         <v>0</v>
@@ -52545,26 +52545,26 @@
         </is>
       </c>
       <c r="D1015" s="15" t="n">
-        <v>249880.06</v>
+        <v>609333.03</v>
       </c>
       <c r="E1015" s="15" t="n">
-        <v>398337.37</v>
+        <v>1165691.14</v>
       </c>
       <c r="F1015" s="16" t="n">
-        <v>-0.305</v>
+        <v>-0.1449</v>
       </c>
       <c r="G1015" s="16" t="n">
-        <v>-0.3766</v>
+        <v>-0.2138</v>
       </c>
       <c r="H1015" s="16" t="n"/>
       <c r="I1015" s="16" t="n">
-        <v>0.1253</v>
+        <v>0.119</v>
       </c>
       <c r="J1015" s="19" t="n">
-        <v>7712</v>
+        <v>18003</v>
       </c>
       <c r="K1015" s="19" t="n">
-        <v>13287</v>
+        <v>32526</v>
       </c>
       <c r="L1015" s="31" t="n">
         <v>0</v>
@@ -52587,26 +52587,26 @@
         </is>
       </c>
       <c r="D1016" s="9" t="n">
-        <v>282395.94</v>
+        <v>724505.05</v>
       </c>
       <c r="E1016" s="9" t="n">
-        <v>647320.79</v>
+        <v>3241087.42</v>
       </c>
       <c r="F1016" s="10" t="n">
-        <v>-0.5798</v>
+        <v>-0.0316</v>
       </c>
       <c r="G1016" s="10" t="n">
-        <v>-0.6489</v>
+        <v>-0.1056</v>
       </c>
       <c r="H1016" s="10" t="n"/>
       <c r="I1016" s="10" t="n">
-        <v>0.0887</v>
+        <v>0.0824</v>
       </c>
       <c r="J1016" s="13" t="n">
-        <v>11562</v>
+        <v>27159</v>
       </c>
       <c r="K1016" s="13" t="n">
-        <v>20964</v>
+        <v>63379</v>
       </c>
       <c r="L1016" s="32" t="n">
         <v>0</v>
@@ -52629,26 +52629,26 @@
         </is>
       </c>
       <c r="D1017" s="15" t="n">
-        <v>163413.62</v>
+        <v>365998.25</v>
       </c>
       <c r="E1017" s="15" t="n">
-        <v>1236403.67</v>
+        <v>4932833.24</v>
       </c>
       <c r="F1017" s="16" t="n">
-        <v>0.3677</v>
+        <v>0.22</v>
       </c>
       <c r="G1017" s="16" t="n">
-        <v>0.2957</v>
+        <v>0.1372</v>
       </c>
       <c r="H1017" s="16" t="n"/>
       <c r="I1017" s="16" t="n">
-        <v>0.0415</v>
+        <v>0.0428</v>
       </c>
       <c r="J1017" s="19" t="n">
-        <v>11072</v>
+        <v>24819</v>
       </c>
       <c r="K1017" s="19" t="n">
-        <v>17965</v>
+        <v>47745</v>
       </c>
       <c r="L1017" s="31" t="n">
         <v>0</v>
@@ -53091,26 +53091,26 @@
         </is>
       </c>
       <c r="D1028" s="9" t="n">
-        <v>129516401.41</v>
+        <v>130335435.15</v>
       </c>
       <c r="E1028" s="9" t="n">
-        <v>426028581.12</v>
+        <v>426921978.41</v>
       </c>
       <c r="F1028" s="10" t="n">
-        <v>0.1959</v>
+        <v>0.1964</v>
       </c>
       <c r="G1028" s="10" t="n">
-        <v>0.1393</v>
+        <v>0.1397</v>
       </c>
       <c r="H1028" s="10" t="n"/>
       <c r="I1028" s="10" t="n">
-        <v>0.1012</v>
+        <v>0.1013</v>
       </c>
       <c r="J1028" s="13" t="n">
-        <v>2948104</v>
+        <v>2953338</v>
       </c>
       <c r="K1028" s="13" t="n">
-        <v>5741210</v>
+        <v>5760824</v>
       </c>
       <c r="L1028" s="32" t="n">
         <v>0</v>
@@ -53133,26 +53133,26 @@
         </is>
       </c>
       <c r="D1029" s="15" t="n">
-        <v>82777376.36</v>
+        <v>151977339.51</v>
       </c>
       <c r="E1029" s="15" t="n">
-        <v>346321931.67</v>
+        <v>635745335.75</v>
       </c>
       <c r="F1029" s="16" t="n">
-        <v>0.0822</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="G1029" s="16" t="n">
-        <v>0.024</v>
+        <v>0.0287</v>
       </c>
       <c r="H1029" s="16" t="n"/>
       <c r="I1029" s="16" t="n">
-        <v>0.09520000000000001</v>
+        <v>0.0973</v>
       </c>
       <c r="J1029" s="19" t="n">
-        <v>2148083</v>
+        <v>3808198</v>
       </c>
       <c r="K1029" s="19" t="n">
-        <v>4014551</v>
+        <v>7301656</v>
       </c>
       <c r="L1029" s="31" t="n">
         <v>0</v>
@@ -56115,13 +56115,13 @@
         </is>
       </c>
       <c r="D1100" s="9" t="n">
-        <v>13631387.6</v>
+        <v>13632486.1</v>
       </c>
       <c r="E1100" s="9" t="n">
-        <v>195763590.23</v>
+        <v>195798279.71</v>
       </c>
       <c r="F1100" s="10" t="n">
-        <v>0.4978</v>
+        <v>0.4977</v>
       </c>
       <c r="G1100" s="10" t="n">
         <v>0.4165</v>
@@ -56131,10 +56131,10 @@
         <v>0.0256</v>
       </c>
       <c r="J1100" s="13" t="n">
-        <v>1037301</v>
+        <v>1037374</v>
       </c>
       <c r="K1100" s="13" t="n">
-        <v>1670839</v>
+        <v>1671010</v>
       </c>
       <c r="L1100" s="32" t="n">
         <v>0</v>
@@ -56157,26 +56157,26 @@
         </is>
       </c>
       <c r="D1101" s="15" t="n">
-        <v>36484036.51</v>
+        <v>36928896.3</v>
       </c>
       <c r="E1101" s="15" t="n">
-        <v>18857890.71</v>
+        <v>19098536.55</v>
       </c>
       <c r="F1101" s="16" t="n">
-        <v>0.0912</v>
+        <v>0.0926</v>
       </c>
       <c r="G1101" s="16" t="n">
-        <v>0.0497</v>
+        <v>0.051</v>
       </c>
       <c r="H1101" s="16" t="n"/>
       <c r="I1101" s="16" t="n">
         <v>0.315</v>
       </c>
       <c r="J1101" s="19" t="n">
-        <v>158555</v>
+        <v>159475</v>
       </c>
       <c r="K1101" s="19" t="n">
-        <v>675260</v>
+        <v>682883</v>
       </c>
       <c r="L1101" s="31" t="n">
         <v>0</v>
@@ -56199,26 +56199,26 @@
         </is>
       </c>
       <c r="D1102" s="9" t="n">
-        <v>23101175.25</v>
+        <v>23303680.58</v>
       </c>
       <c r="E1102" s="9" t="n">
-        <v>20820117.72</v>
+        <v>21060268.13</v>
       </c>
       <c r="F1102" s="10" t="n">
-        <v>0.1243</v>
+        <v>0.1248</v>
       </c>
       <c r="G1102" s="10" t="n">
-        <v>0.0747</v>
+        <v>0.0751</v>
       </c>
       <c r="H1102" s="10" t="n"/>
       <c r="I1102" s="10" t="n">
-        <v>0.2355</v>
+        <v>0.2354</v>
       </c>
       <c r="J1102" s="13" t="n">
-        <v>229436</v>
+        <v>230659</v>
       </c>
       <c r="K1102" s="13" t="n">
-        <v>594197</v>
+        <v>599011</v>
       </c>
       <c r="L1102" s="32" t="n">
         <v>0</v>
@@ -56241,26 +56241,26 @@
         </is>
       </c>
       <c r="D1103" s="15" t="n">
-        <v>16640566.83</v>
+        <v>16734018.51</v>
       </c>
       <c r="E1103" s="15" t="n">
-        <v>25018524.77</v>
+        <v>25187202.12</v>
       </c>
       <c r="F1103" s="16" t="n">
-        <v>0.1535</v>
+        <v>0.1549</v>
       </c>
       <c r="G1103" s="16" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.0985</v>
       </c>
       <c r="H1103" s="16" t="n"/>
       <c r="I1103" s="16" t="n">
-        <v>0.1817</v>
+        <v>0.1815</v>
       </c>
       <c r="J1103" s="19" t="n">
-        <v>261495</v>
+        <v>262504</v>
       </c>
       <c r="K1103" s="19" t="n">
-        <v>549834</v>
+        <v>552722</v>
       </c>
       <c r="L1103" s="31" t="n">
         <v>0</v>
@@ -56283,26 +56283,26 @@
         </is>
       </c>
       <c r="D1104" s="9" t="n">
-        <v>11545931.79</v>
+        <v>11584474.04</v>
       </c>
       <c r="E1104" s="9" t="n">
-        <v>24700809.51</v>
+        <v>24786032.7</v>
       </c>
       <c r="F1104" s="10" t="n">
-        <v>0.2293</v>
+        <v>0.2307</v>
       </c>
       <c r="G1104" s="10" t="n">
-        <v>0.1684</v>
+        <v>0.1698</v>
       </c>
       <c r="H1104" s="10" t="n"/>
       <c r="I1104" s="10" t="n">
-        <v>0.1445</v>
+        <v>0.1443</v>
       </c>
       <c r="J1104" s="13" t="n">
-        <v>249244</v>
+        <v>249937</v>
       </c>
       <c r="K1104" s="13" t="n">
-        <v>460026</v>
+        <v>461821</v>
       </c>
       <c r="L1104" s="32" t="n">
         <v>0</v>
@@ -56325,26 +56325,26 @@
         </is>
       </c>
       <c r="D1105" s="15" t="n">
-        <v>15823537.96</v>
+        <v>15854106.91</v>
       </c>
       <c r="E1105" s="15" t="n">
-        <v>59330133.55</v>
+        <v>59410234.51</v>
       </c>
       <c r="F1105" s="16" t="n">
-        <v>0.2185</v>
+        <v>0.2195</v>
       </c>
       <c r="G1105" s="16" t="n">
-        <v>0.153</v>
+        <v>0.154</v>
       </c>
       <c r="H1105" s="16" t="n"/>
       <c r="I1105" s="16" t="n">
-        <v>0.1052</v>
+        <v>0.1051</v>
       </c>
       <c r="J1105" s="19" t="n">
-        <v>469445</v>
+        <v>470385</v>
       </c>
       <c r="K1105" s="19" t="n">
-        <v>867665</v>
+        <v>869373</v>
       </c>
       <c r="L1105" s="31" t="n">
         <v>0</v>
@@ -56367,26 +56367,26 @@
         </is>
       </c>
       <c r="D1106" s="9" t="n">
-        <v>12289765.47</v>
+        <v>12297772.72</v>
       </c>
       <c r="E1106" s="9" t="n">
-        <v>81537514.62</v>
+        <v>81581424.69</v>
       </c>
       <c r="F1106" s="10" t="n">
-        <v>0.3033</v>
+        <v>0.3036</v>
       </c>
       <c r="G1106" s="10" t="n">
-        <v>0.2309</v>
+        <v>0.2313</v>
       </c>
       <c r="H1106" s="10" t="n"/>
       <c r="I1106" s="10" t="n">
         <v>0.0643</v>
       </c>
       <c r="J1106" s="13" t="n">
-        <v>542628</v>
+        <v>543004</v>
       </c>
       <c r="K1106" s="13" t="n">
-        <v>923389</v>
+        <v>924004</v>
       </c>
       <c r="L1106" s="32" t="n">
         <v>0</v>
@@ -56409,26 +56409,26 @@
         </is>
       </c>
       <c r="D1107" s="15" t="n">
-        <v>11227658.99</v>
+        <v>18798799.93</v>
       </c>
       <c r="E1107" s="15" t="n">
-        <v>182996707.85</v>
+        <v>319571908.03</v>
       </c>
       <c r="F1107" s="16" t="n">
-        <v>0.3936</v>
+        <v>0.4217</v>
       </c>
       <c r="G1107" s="16" t="n">
-        <v>0.3129</v>
+        <v>0.3399</v>
       </c>
       <c r="H1107" s="16" t="n"/>
       <c r="I1107" s="16" t="n">
-        <v>0.0277</v>
+        <v>0.0272</v>
       </c>
       <c r="J1107" s="19" t="n">
-        <v>861831</v>
+        <v>1453931</v>
       </c>
       <c r="K1107" s="19" t="n">
-        <v>1359058</v>
+        <v>2270467</v>
       </c>
       <c r="L1107" s="31" t="n">
         <v>0</v>
@@ -56451,26 +56451,26 @@
         </is>
       </c>
       <c r="D1108" s="9" t="n">
-        <v>20828995.57</v>
+        <v>39786009.98</v>
       </c>
       <c r="E1108" s="9" t="n">
-        <v>10664575.05</v>
+        <v>20006818.38</v>
       </c>
       <c r="F1108" s="10" t="n">
-        <v>0.0367</v>
+        <v>-0.0013</v>
       </c>
       <c r="G1108" s="10" t="n">
-        <v>-0.0052</v>
+        <v>-0.0428</v>
       </c>
       <c r="H1108" s="10" t="n"/>
       <c r="I1108" s="10" t="n">
-        <v>0.3031</v>
+        <v>0.3039</v>
       </c>
       <c r="J1108" s="13" t="n">
-        <v>96276</v>
+        <v>176095</v>
       </c>
       <c r="K1108" s="13" t="n">
-        <v>403275</v>
+        <v>754130</v>
       </c>
       <c r="L1108" s="32" t="n">
         <v>0</v>
@@ -56493,26 +56493,26 @@
         </is>
       </c>
       <c r="D1109" s="15" t="n">
-        <v>14271512.22</v>
+        <v>25986686.48</v>
       </c>
       <c r="E1109" s="15" t="n">
-        <v>13870247.16</v>
+        <v>25609140.89</v>
       </c>
       <c r="F1109" s="16" t="n">
-        <v>0.048</v>
+        <v>0.026</v>
       </c>
       <c r="G1109" s="16" t="n">
-        <v>-0.0019</v>
+        <v>-0.0249</v>
       </c>
       <c r="H1109" s="16" t="n"/>
       <c r="I1109" s="16" t="n">
-        <v>0.2325</v>
+        <v>0.2357</v>
       </c>
       <c r="J1109" s="19" t="n">
-        <v>144856</v>
+        <v>263423</v>
       </c>
       <c r="K1109" s="19" t="n">
-        <v>382385</v>
+        <v>702937</v>
       </c>
       <c r="L1109" s="31" t="n">
         <v>0</v>
@@ -56535,26 +56535,26 @@
         </is>
       </c>
       <c r="D1110" s="9" t="n">
-        <v>10419193.24</v>
+        <v>19378152.15</v>
       </c>
       <c r="E1110" s="9" t="n">
-        <v>15467400.21</v>
+        <v>30969589.13</v>
       </c>
       <c r="F1110" s="10" t="n">
-        <v>0.0148</v>
+        <v>0.0299</v>
       </c>
       <c r="G1110" s="10" t="n">
-        <v>-0.0407</v>
+        <v>-0.027</v>
       </c>
       <c r="H1110" s="10" t="n"/>
       <c r="I1110" s="10" t="n">
-        <v>0.1832</v>
+        <v>0.1879</v>
       </c>
       <c r="J1110" s="13" t="n">
-        <v>168231</v>
+        <v>306128</v>
       </c>
       <c r="K1110" s="13" t="n">
-        <v>339950</v>
+        <v>658168</v>
       </c>
       <c r="L1110" s="32" t="n">
         <v>0</v>
@@ -56577,26 +56577,26 @@
         </is>
       </c>
       <c r="D1111" s="15" t="n">
-        <v>7949605.67</v>
+        <v>14026152.75</v>
       </c>
       <c r="E1111" s="15" t="n">
-        <v>17754869.53</v>
+        <v>33963946.59</v>
       </c>
       <c r="F1111" s="16" t="n">
-        <v>-0.0037</v>
+        <v>0.0452</v>
       </c>
       <c r="G1111" s="16" t="n">
-        <v>-0.06320000000000001</v>
+        <v>-0.0166</v>
       </c>
       <c r="H1111" s="16" t="n"/>
       <c r="I1111" s="16" t="n">
-        <v>0.1477</v>
+        <v>0.1504</v>
       </c>
       <c r="J1111" s="19" t="n">
-        <v>167018</v>
+        <v>302846</v>
       </c>
       <c r="K1111" s="19" t="n">
-        <v>309540</v>
+        <v>583201</v>
       </c>
       <c r="L1111" s="31" t="n">
         <v>0</v>
@@ -56619,26 +56619,26 @@
         </is>
       </c>
       <c r="D1112" s="9" t="n">
-        <v>9467601.9</v>
+        <v>18083448.04</v>
       </c>
       <c r="E1112" s="9" t="n">
-        <v>37863333.19</v>
+        <v>76377364.84</v>
       </c>
       <c r="F1112" s="10" t="n">
-        <v>-0.0026</v>
+        <v>0.07149999999999999</v>
       </c>
       <c r="G1112" s="10" t="n">
-        <v>-0.0707</v>
+        <v>0.0022</v>
       </c>
       <c r="H1112" s="10" t="n"/>
       <c r="I1112" s="10" t="n">
-        <v>0.1114</v>
+        <v>0.1109</v>
       </c>
       <c r="J1112" s="13" t="n">
-        <v>313657</v>
+        <v>578525</v>
       </c>
       <c r="K1112" s="13" t="n">
-        <v>513660</v>
+        <v>1015024</v>
       </c>
       <c r="L1112" s="32" t="n">
         <v>0</v>
@@ -56661,26 +56661,26 @@
         </is>
       </c>
       <c r="D1113" s="15" t="n">
-        <v>8612808.77</v>
+        <v>15918090.19</v>
       </c>
       <c r="E1113" s="15" t="n">
-        <v>67704798.69</v>
+        <v>129246567.89</v>
       </c>
       <c r="F1113" s="16" t="n">
-        <v>0.09710000000000001</v>
+        <v>0.14</v>
       </c>
       <c r="G1113" s="16" t="n">
-        <v>0.024</v>
+        <v>0.0655</v>
       </c>
       <c r="H1113" s="16" t="n"/>
       <c r="I1113" s="16" t="n">
-        <v>0.0688</v>
+        <v>0.0663</v>
       </c>
       <c r="J1113" s="19" t="n">
-        <v>396214</v>
+        <v>727250</v>
       </c>
       <c r="K1113" s="19" t="n">
-        <v>706683</v>
+        <v>1317729</v>
       </c>
       <c r="L1113" s="31" t="n">
         <v>0</v>
@@ -57123,26 +57123,26 @@
         </is>
       </c>
       <c r="D1124" s="9" t="n">
-        <v>7466832.7</v>
+        <v>12557624.64</v>
       </c>
       <c r="E1124" s="9" t="n">
-        <v>17807497.69</v>
+        <v>30426704.74</v>
       </c>
       <c r="F1124" s="10" t="n">
-        <v>0.2709</v>
+        <v>0.2247</v>
       </c>
       <c r="G1124" s="10" t="n">
-        <v>0.2101</v>
+        <v>0.1632</v>
       </c>
       <c r="H1124" s="10" t="n"/>
       <c r="I1124" s="10" t="n">
-        <v>0.0927</v>
+        <v>0.1146</v>
       </c>
       <c r="J1124" s="13" t="n">
-        <v>125019</v>
+        <v>213085</v>
       </c>
       <c r="K1124" s="13" t="n">
-        <v>210474</v>
+        <v>357174</v>
       </c>
       <c r="L1124" s="32" t="n">
         <v>0</v>
@@ -60105,26 +60105,26 @@
         </is>
       </c>
       <c r="D1195" s="15" t="n">
-        <v>434657.67</v>
+        <v>665564.5699999999</v>
       </c>
       <c r="E1195" s="15" t="n">
-        <v>4292597.67</v>
+        <v>7960554.33</v>
       </c>
       <c r="F1195" s="16" t="n">
-        <v>0.6567</v>
+        <v>0.3603</v>
       </c>
       <c r="G1195" s="16" t="n">
-        <v>0.5827</v>
+        <v>0.2806</v>
       </c>
       <c r="H1195" s="16" t="n"/>
       <c r="I1195" s="16" t="n">
-        <v>0.027</v>
+        <v>0.0408</v>
       </c>
       <c r="J1195" s="19" t="n">
-        <v>25936</v>
+        <v>42644</v>
       </c>
       <c r="K1195" s="19" t="n">
-        <v>41410</v>
+        <v>64425</v>
       </c>
       <c r="L1195" s="31" t="n">
         <v>0</v>
@@ -60147,26 +60147,26 @@
         </is>
       </c>
       <c r="D1196" s="9" t="n">
-        <v>1827837.88</v>
+        <v>3129801.72</v>
       </c>
       <c r="E1196" s="9" t="n">
-        <v>1307646</v>
+        <v>2056350.06</v>
       </c>
       <c r="F1196" s="10" t="n">
-        <v>0.187</v>
+        <v>0.1951</v>
       </c>
       <c r="G1196" s="10" t="n">
-        <v>0.1364</v>
+        <v>0.1438</v>
       </c>
       <c r="H1196" s="10" t="n"/>
       <c r="I1196" s="10" t="n">
-        <v>0.304</v>
+        <v>0.32</v>
       </c>
       <c r="J1196" s="13" t="n">
-        <v>7573</v>
+        <v>12701</v>
       </c>
       <c r="K1196" s="13" t="n">
-        <v>21867</v>
+        <v>38775</v>
       </c>
       <c r="L1196" s="32" t="n">
         <v>0</v>
@@ -60189,26 +60189,26 @@
         </is>
       </c>
       <c r="D1197" s="15" t="n">
-        <v>1857031.6</v>
+        <v>3269246.63</v>
       </c>
       <c r="E1197" s="15" t="n">
-        <v>2187515.7</v>
+        <v>3302856.55</v>
       </c>
       <c r="F1197" s="16" t="n">
-        <v>0.2141</v>
+        <v>0.1998</v>
       </c>
       <c r="G1197" s="16" t="n">
-        <v>0.1572</v>
+        <v>0.1427</v>
       </c>
       <c r="H1197" s="16" t="n"/>
       <c r="I1197" s="16" t="n">
-        <v>0.1957</v>
+        <v>0.2195</v>
       </c>
       <c r="J1197" s="19" t="n">
-        <v>15073</v>
+        <v>26910</v>
       </c>
       <c r="K1197" s="19" t="n">
-        <v>31386</v>
+        <v>57086</v>
       </c>
       <c r="L1197" s="31" t="n">
         <v>0</v>
@@ -60231,26 +60231,26 @@
         </is>
       </c>
       <c r="D1198" s="9" t="n">
-        <v>1299271.75</v>
+        <v>2059095.67</v>
       </c>
       <c r="E1198" s="9" t="n">
-        <v>2273683.88</v>
+        <v>3519746.04</v>
       </c>
       <c r="F1198" s="10" t="n">
-        <v>0.1575</v>
+        <v>0.1366</v>
       </c>
       <c r="G1198" s="10" t="n">
-        <v>0.096</v>
+        <v>0.0742</v>
       </c>
       <c r="H1198" s="10" t="n"/>
       <c r="I1198" s="10" t="n">
-        <v>0.1263</v>
+        <v>0.1502</v>
       </c>
       <c r="J1198" s="13" t="n">
-        <v>17518</v>
+        <v>29976</v>
       </c>
       <c r="K1198" s="13" t="n">
-        <v>28215</v>
+        <v>46146</v>
       </c>
       <c r="L1198" s="32" t="n">
         <v>0</v>
@@ -60273,26 +60273,26 @@
         </is>
       </c>
       <c r="D1199" s="15" t="n">
-        <v>768726.6800000001</v>
+        <v>1273940.96</v>
       </c>
       <c r="E1199" s="15" t="n">
-        <v>1974771.55</v>
+        <v>2996901.57</v>
       </c>
       <c r="F1199" s="16" t="n">
-        <v>0.3012</v>
+        <v>0.2749</v>
       </c>
       <c r="G1199" s="16" t="n">
-        <v>0.2316</v>
+        <v>0.2066</v>
       </c>
       <c r="H1199" s="16" t="n"/>
       <c r="I1199" s="16" t="n">
-        <v>0.0887</v>
+        <v>0.1132</v>
       </c>
       <c r="J1199" s="19" t="n">
-        <v>15270</v>
+        <v>26099</v>
       </c>
       <c r="K1199" s="19" t="n">
-        <v>24546</v>
+        <v>40356</v>
       </c>
       <c r="L1199" s="31" t="n">
         <v>0</v>
@@ -60315,26 +60315,26 @@
         </is>
       </c>
       <c r="D1200" s="9" t="n">
-        <v>830647.96</v>
+        <v>1402017.54</v>
       </c>
       <c r="E1200" s="9" t="n">
-        <v>3018165.91</v>
+        <v>4783033.14</v>
       </c>
       <c r="F1200" s="10" t="n">
-        <v>0.3907</v>
+        <v>0.2982</v>
       </c>
       <c r="G1200" s="10" t="n">
-        <v>0.3216</v>
+        <v>0.2281</v>
       </c>
       <c r="H1200" s="10" t="n"/>
       <c r="I1200" s="10" t="n">
-        <v>0.0582</v>
+        <v>0.0815</v>
       </c>
       <c r="J1200" s="13" t="n">
-        <v>24315</v>
+        <v>41857</v>
       </c>
       <c r="K1200" s="13" t="n">
-        <v>33535</v>
+        <v>58039</v>
       </c>
       <c r="L1200" s="32" t="n">
         <v>0</v>
@@ -60357,26 +60357,26 @@
         </is>
       </c>
       <c r="D1201" s="15" t="n">
-        <v>448659.15</v>
+        <v>757957.55</v>
       </c>
       <c r="E1201" s="15" t="n">
-        <v>2753116.98</v>
+        <v>5807263.05</v>
       </c>
       <c r="F1201" s="16" t="n">
-        <v>0.5283</v>
+        <v>0.3542</v>
       </c>
       <c r="G1201" s="16" t="n">
-        <v>0.455</v>
+        <v>0.2779</v>
       </c>
       <c r="H1201" s="16" t="n"/>
       <c r="I1201" s="16" t="n">
-        <v>0.0337</v>
+        <v>0.0562</v>
       </c>
       <c r="J1201" s="19" t="n">
-        <v>19334</v>
+        <v>32898</v>
       </c>
       <c r="K1201" s="19" t="n">
-        <v>29515</v>
+        <v>52347</v>
       </c>
       <c r="L1201" s="31" t="n">
         <v>0</v>
@@ -61196,7 +61196,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-19 18:47 UTC</t>
+          <t>2026-10-19 20:18 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-21 16:35 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -1679,7 +1679,7 @@
         <v>21766760.99</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1234384.02</v>
+        <v>1234384.01</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>0.05671</v>
@@ -1692,7 +1692,7 @@
         <v>21766760.99</v>
       </c>
       <c r="J9" s="15" t="n">
-        <v>1234384.02</v>
+        <v>1234384.01</v>
       </c>
       <c r="K9" s="18" t="n"/>
       <c r="L9" s="19" t="n">
@@ -2892,7 +2892,7 @@
         </is>
       </c>
       <c r="I26" s="9" t="n">
-        <v>499580423.51</v>
+        <v>499580423.5</v>
       </c>
       <c r="J26" s="9" t="n">
         <v>6582164.99</v>
@@ -3049,7 +3049,7 @@
         <v>691271126.84</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>44338006.62</v>
+        <v>44338006.61</v>
       </c>
       <c r="K28" s="12" t="n">
         <v>0.06414</v>
@@ -5933,22 +5933,22 @@
         <v>46320</v>
       </c>
       <c r="B70" s="9" t="n">
-        <v>78255216.66</v>
+        <v>157372428.15</v>
       </c>
       <c r="C70" s="9" t="n">
-        <v>3467465.95</v>
+        <v>6857933.43</v>
       </c>
       <c r="D70" s="10" t="n">
-        <v>0.04431</v>
+        <v>0.04358</v>
       </c>
       <c r="E70" s="9" t="n">
-        <v>25357758.93</v>
+        <v>49773819.72</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>9501292.24</v>
+        <v>18335625.38</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>0.37469</v>
+        <v>0.36838</v>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
@@ -5956,19 +5956,19 @@
         </is>
       </c>
       <c r="I70" s="9" t="n">
-        <v>103612975.59</v>
+        <v>207146247.87</v>
       </c>
       <c r="J70" s="9" t="n">
-        <v>12968758.2</v>
+        <v>25193558.81</v>
       </c>
       <c r="K70" s="12" t="n">
-        <v>0.12517</v>
+        <v>0.12162</v>
       </c>
       <c r="L70" s="13" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="M70" s="13" t="n">
-        <v>-317</v>
+        <v>-513</v>
       </c>
       <c r="N70" s="9" t="n">
         <v>64762756.4</v>
@@ -5976,8 +5976,12 @@
       <c r="O70" s="10" t="n">
         <v>0.05704</v>
       </c>
-      <c r="P70" s="9" t="n"/>
-      <c r="Q70" s="10" t="n"/>
+      <c r="P70" s="9" t="n">
+        <v>52982190.33</v>
+      </c>
+      <c r="Q70" s="10" t="n">
+        <v>0.05527</v>
+      </c>
       <c r="R70" s="9" t="n">
         <v>9057675.779999999</v>
       </c>
@@ -5985,13 +5989,17 @@
         <v>-0.06547</v>
       </c>
       <c r="T70" s="9" t="n">
-        <v>4434784.48</v>
+        <v>13930969.8</v>
       </c>
       <c r="U70" s="10" t="n">
-        <v>0.08269</v>
-      </c>
-      <c r="V70" s="9" t="n"/>
-      <c r="W70" s="10" t="n"/>
+        <v>0.06711</v>
+      </c>
+      <c r="V70" s="9" t="n">
+        <v>16638835.85</v>
+      </c>
+      <c r="W70" s="10" t="n">
+        <v>-0.00637</v>
+      </c>
       <c r="X70" s="9" t="n"/>
       <c r="Y70" s="10" t="n"/>
       <c r="Z70" s="9" t="n"/>
@@ -7384,22 +7392,22 @@
         <v>46296</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>2357230636.81</v>
+        <v>2436347848.3</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>46426857.06</v>
+        <v>49817324.54</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.0197</v>
+        <v>0.02045</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>652262996.6</v>
+        <v>676690867.52</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>126375268.68</v>
+        <v>135221781.75</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.19375</v>
+        <v>0.19983</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
@@ -7407,19 +7415,19 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>3009493633.41</v>
+        <v>3113038715.82</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>172802125.74</v>
+        <v>185039106.29</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.05742</v>
+        <v>0.05944</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>631</v>
+        <v>648</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>154</v>
+        <v>130</v>
       </c>
       <c r="N20" s="9" t="n">
         <v>1072027977.53</v>
@@ -7428,10 +7436,10 @@
         <v>0.01175</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>90714884.14</v>
+        <v>143697074.47</v>
       </c>
       <c r="Q20" s="10" t="n">
-        <v>0.0336</v>
+        <v>0.04159</v>
       </c>
       <c r="R20" s="9" t="n">
         <v>298312041.27</v>
@@ -7440,16 +7448,16 @@
         <v>0.04584</v>
       </c>
       <c r="T20" s="9" t="n">
-        <v>89370002.97</v>
+        <v>98866188.29000001</v>
       </c>
       <c r="U20" s="10" t="n">
-        <v>0.02357</v>
+        <v>0.02706</v>
       </c>
       <c r="V20" s="9" t="n">
-        <v>806805730.89</v>
+        <v>823444566.73</v>
       </c>
       <c r="W20" s="10" t="n">
-        <v>0.01859</v>
+        <v>0.01809</v>
       </c>
       <c r="X20" s="9" t="n"/>
       <c r="Y20" s="10" t="n"/>
@@ -7988,10 +7996,10 @@
         <v>8.6</v>
       </c>
       <c r="L11" s="15" t="n">
-        <v>19163529.07</v>
+        <v>27876873.41</v>
       </c>
       <c r="M11" s="16" t="n">
-        <v>0.4144</v>
+        <v>0.3732</v>
       </c>
     </row>
     <row r="12">
@@ -8550,7 +8558,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-20 16:05 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-21 16:34 UTC.</t>
         </is>
       </c>
     </row>
@@ -10085,26 +10093,26 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>142030.76</v>
+        <v>789950.65</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>682086.48</v>
+        <v>1823775.13</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.1362</v>
+        <v>0.404</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.07679999999999999</v>
+        <v>0.3456</v>
       </c>
       <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n">
-        <v>0.0866</v>
+        <v>0.06859999999999999</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>2459</v>
+        <v>18975</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>6106</v>
+        <v>29483</v>
       </c>
       <c r="L14" s="32" t="n">
         <v>0</v>
@@ -12773,26 +12781,26 @@
         </is>
       </c>
       <c r="D78" s="9" t="n">
-        <v>8935.379999999999</v>
+        <v>63961.69</v>
       </c>
       <c r="E78" s="9" t="n">
-        <v>548675.99</v>
+        <v>1008625.06</v>
       </c>
       <c r="F78" s="10" t="n">
-        <v>0.845</v>
+        <v>0.8423</v>
       </c>
       <c r="G78" s="10" t="n">
-        <v>0.7644</v>
+        <v>0.775</v>
       </c>
       <c r="H78" s="10" t="n"/>
       <c r="I78" s="10" t="n">
-        <v>0.007</v>
+        <v>0.0163</v>
       </c>
       <c r="J78" s="13" t="n">
-        <v>431</v>
+        <v>4783</v>
       </c>
       <c r="K78" s="13" t="n">
-        <v>2896</v>
+        <v>9357</v>
       </c>
       <c r="L78" s="32" t="n">
         <v>0</v>
@@ -12815,26 +12823,26 @@
         </is>
       </c>
       <c r="D79" s="15" t="n">
-        <v>47977.32</v>
+        <v>202548.9</v>
       </c>
       <c r="E79" s="15" t="n">
-        <v>14814.01</v>
+        <v>96121.2</v>
       </c>
       <c r="F79" s="16" t="n">
-        <v>-0.3979</v>
+        <v>0.1729</v>
       </c>
       <c r="G79" s="16" t="n">
-        <v>-0.4494</v>
+        <v>0.1235</v>
       </c>
       <c r="H79" s="16" t="n"/>
       <c r="I79" s="16" t="n">
-        <v>0.336</v>
+        <v>0.3054</v>
       </c>
       <c r="J79" s="19" t="n">
-        <v>247</v>
+        <v>1192</v>
       </c>
       <c r="K79" s="19" t="n">
-        <v>737</v>
+        <v>3077</v>
       </c>
       <c r="L79" s="31" t="n">
         <v>0</v>
@@ -12857,26 +12865,26 @@
         </is>
       </c>
       <c r="D80" s="9" t="n">
-        <v>36129.92</v>
+        <v>197824.14</v>
       </c>
       <c r="E80" s="9" t="n">
-        <v>31020.45</v>
+        <v>123062.5</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>0.0544</v>
+        <v>0.3015</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>-0.007</v>
+        <v>0.2444</v>
       </c>
       <c r="H80" s="10" t="n"/>
       <c r="I80" s="10" t="n">
-        <v>0.1686</v>
+        <v>0.1666</v>
       </c>
       <c r="J80" s="13" t="n">
-        <v>350</v>
+        <v>2041</v>
       </c>
       <c r="K80" s="13" t="n">
-        <v>580</v>
+        <v>3387</v>
       </c>
       <c r="L80" s="32" t="n">
         <v>0</v>
@@ -12899,26 +12907,26 @@
         </is>
       </c>
       <c r="D81" s="15" t="n">
-        <v>15752.16</v>
+        <v>121501.67</v>
       </c>
       <c r="E81" s="15" t="n">
-        <v>27561.68</v>
+        <v>110775.03</v>
       </c>
       <c r="F81" s="16" t="n">
-        <v>0.644</v>
+        <v>0.5625</v>
       </c>
       <c r="G81" s="16" t="n">
-        <v>0.5790999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="H81" s="16" t="n"/>
       <c r="I81" s="16" t="n">
-        <v>0.0863</v>
+        <v>0.0887</v>
       </c>
       <c r="J81" s="19" t="n">
-        <v>336</v>
+        <v>2300</v>
       </c>
       <c r="K81" s="19" t="n">
-        <v>459</v>
+        <v>3207</v>
       </c>
       <c r="L81" s="31" t="n">
         <v>0</v>
@@ -12941,26 +12949,26 @@
         </is>
       </c>
       <c r="D82" s="9" t="n">
-        <v>13571.47</v>
+        <v>70960.57000000001</v>
       </c>
       <c r="E82" s="9" t="n">
-        <v>4959.59</v>
+        <v>78655.84</v>
       </c>
       <c r="F82" s="10" t="n">
-        <v>0.5027</v>
+        <v>0.4666</v>
       </c>
       <c r="G82" s="10" t="n">
-        <v>0.442</v>
+        <v>0.4028</v>
       </c>
       <c r="H82" s="10" t="n"/>
       <c r="I82" s="10" t="n">
-        <v>0.0643</v>
+        <v>0.07439999999999999</v>
       </c>
       <c r="J82" s="13" t="n">
-        <v>311</v>
+        <v>2123</v>
       </c>
       <c r="K82" s="13" t="n">
-        <v>504</v>
+        <v>2775</v>
       </c>
       <c r="L82" s="32" t="n">
         <v>0</v>
@@ -12983,26 +12991,26 @@
         </is>
       </c>
       <c r="D83" s="15" t="n">
-        <v>11179.62</v>
+        <v>86018.75</v>
       </c>
       <c r="E83" s="15" t="n">
-        <v>27261.32</v>
+        <v>206540.07</v>
       </c>
       <c r="F83" s="16" t="n">
-        <v>0.7292999999999999</v>
+        <v>0.3768</v>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0.6664</v>
+        <v>0.3147</v>
       </c>
       <c r="H83" s="16" t="n"/>
       <c r="I83" s="16" t="n">
-        <v>0.029</v>
+        <v>0.031</v>
       </c>
       <c r="J83" s="19" t="n">
-        <v>414</v>
+        <v>3543</v>
       </c>
       <c r="K83" s="19" t="n">
-        <v>451</v>
+        <v>4152</v>
       </c>
       <c r="L83" s="31" t="n">
         <v>0</v>
@@ -13025,26 +13033,26 @@
         </is>
       </c>
       <c r="D84" s="9" t="n">
-        <v>8484.889999999999</v>
+        <v>47134.93</v>
       </c>
       <c r="E84" s="9" t="n">
-        <v>27793.42</v>
+        <v>199995.44</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>0.4478</v>
+        <v>0.7802</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>0.3924</v>
+        <v>0.7146</v>
       </c>
       <c r="H84" s="10" t="n"/>
       <c r="I84" s="10" t="n">
-        <v>0.0189</v>
+        <v>0.0157</v>
       </c>
       <c r="J84" s="13" t="n">
-        <v>370</v>
+        <v>2993</v>
       </c>
       <c r="K84" s="13" t="n">
-        <v>479</v>
+        <v>3528</v>
       </c>
       <c r="L84" s="32" t="n">
         <v>0</v>
@@ -14411,26 +14419,26 @@
         </is>
       </c>
       <c r="D117" s="15" t="n">
-        <v>419565.78</v>
+        <v>1608230.32</v>
       </c>
       <c r="E117" s="15" t="n">
-        <v>709064.1800000001</v>
+        <v>1217175.74</v>
       </c>
       <c r="F117" s="16" t="n">
-        <v>0.9656</v>
+        <v>0.6938</v>
       </c>
       <c r="G117" s="16" t="n">
-        <v>0.906</v>
+        <v>0.643</v>
       </c>
       <c r="H117" s="16" t="n"/>
       <c r="I117" s="16" t="n">
-        <v>0</v>
+        <v>0.0285</v>
       </c>
       <c r="J117" s="19" t="n">
-        <v>15353</v>
+        <v>27368</v>
       </c>
       <c r="K117" s="19" t="n">
-        <v>26413</v>
+        <v>58665</v>
       </c>
       <c r="L117" s="31" t="n">
         <v>0</v>
@@ -16595,26 +16603,26 @@
         </is>
       </c>
       <c r="D169" s="15" t="n">
-        <v>129182.5</v>
+        <v>167105.66</v>
       </c>
       <c r="E169" s="15" t="n">
-        <v>353066.29</v>
+        <v>411678.23</v>
       </c>
       <c r="F169" s="16" t="n">
-        <v>1.0187</v>
+        <v>1.0229</v>
       </c>
       <c r="G169" s="16" t="n">
-        <v>0.9473</v>
+        <v>0.952</v>
       </c>
       <c r="H169" s="16" t="n"/>
       <c r="I169" s="16" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="J169" s="19" t="n">
-        <v>7736</v>
+        <v>10025</v>
       </c>
       <c r="K169" s="19" t="n">
-        <v>16845</v>
+        <v>25272</v>
       </c>
       <c r="L169" s="31" t="n">
         <v>0</v>
@@ -16637,26 +16645,26 @@
         </is>
       </c>
       <c r="D170" s="9" t="n">
-        <v>43528.95</v>
+        <v>687676.72</v>
       </c>
       <c r="E170" s="9" t="n">
-        <v>15875.91</v>
+        <v>261903.93</v>
       </c>
       <c r="F170" s="10" t="n">
-        <v>0.9741</v>
+        <v>0.4961</v>
       </c>
       <c r="G170" s="10" t="n">
-        <v>0.9236</v>
+        <v>0.454</v>
       </c>
       <c r="H170" s="10" t="n"/>
       <c r="I170" s="10" t="n">
-        <v>0</v>
+        <v>0.1866</v>
       </c>
       <c r="J170" s="13" t="n">
-        <v>359</v>
+        <v>2572</v>
       </c>
       <c r="K170" s="13" t="n">
-        <v>554</v>
+        <v>7784</v>
       </c>
       <c r="L170" s="32" t="n">
         <v>0</v>
@@ -16679,26 +16687,26 @@
         </is>
       </c>
       <c r="D171" s="15" t="n">
-        <v>43046.57</v>
+        <v>390434.92</v>
       </c>
       <c r="E171" s="15" t="n">
-        <v>33835.68</v>
+        <v>157621.43</v>
       </c>
       <c r="F171" s="16" t="n">
-        <v>0.8951</v>
+        <v>0.7148</v>
       </c>
       <c r="G171" s="16" t="n">
-        <v>0.8535</v>
+        <v>0.6627999999999999</v>
       </c>
       <c r="H171" s="16" t="n"/>
       <c r="I171" s="16" t="n">
-        <v>0</v>
+        <v>0.0625</v>
       </c>
       <c r="J171" s="19" t="n">
-        <v>731</v>
+        <v>3422</v>
       </c>
       <c r="K171" s="19" t="n">
-        <v>929</v>
+        <v>11460</v>
       </c>
       <c r="L171" s="31" t="n">
         <v>0</v>
@@ -16721,26 +16729,26 @@
         </is>
       </c>
       <c r="D172" s="9" t="n">
-        <v>61547.71</v>
+        <v>127571.05</v>
       </c>
       <c r="E172" s="9" t="n">
-        <v>45002.81</v>
+        <v>56335.08</v>
       </c>
       <c r="F172" s="10" t="n">
-        <v>0.9267</v>
+        <v>0.8021</v>
       </c>
       <c r="G172" s="10" t="n">
-        <v>0.8779</v>
+        <v>0.7511</v>
       </c>
       <c r="H172" s="10" t="n"/>
       <c r="I172" s="10" t="n">
-        <v>0</v>
+        <v>0.0233</v>
       </c>
       <c r="J172" s="13" t="n">
-        <v>1116</v>
+        <v>2531</v>
       </c>
       <c r="K172" s="13" t="n">
-        <v>1513</v>
+        <v>3353</v>
       </c>
       <c r="L172" s="32" t="n">
         <v>0</v>
@@ -16763,26 +16771,26 @@
         </is>
       </c>
       <c r="D173" s="15" t="n">
-        <v>40846.93</v>
+        <v>67596.85000000001</v>
       </c>
       <c r="E173" s="15" t="n">
-        <v>61445.02</v>
+        <v>75044.21000000001</v>
       </c>
       <c r="F173" s="16" t="n">
-        <v>0.959</v>
+        <v>0.9728</v>
       </c>
       <c r="G173" s="16" t="n">
-        <v>0.9033</v>
+        <v>0.9155</v>
       </c>
       <c r="H173" s="16" t="n"/>
       <c r="I173" s="16" t="n">
-        <v>0</v>
+        <v>0.0045</v>
       </c>
       <c r="J173" s="19" t="n">
-        <v>1137</v>
+        <v>1992</v>
       </c>
       <c r="K173" s="19" t="n">
-        <v>1419</v>
+        <v>2498</v>
       </c>
       <c r="L173" s="31" t="n">
         <v>0</v>
@@ -16805,26 +16813,26 @@
         </is>
       </c>
       <c r="D174" s="9" t="n">
-        <v>56213.57</v>
+        <v>109878.76</v>
       </c>
       <c r="E174" s="9" t="n">
-        <v>82977.91</v>
+        <v>105902.39</v>
       </c>
       <c r="F174" s="10" t="n">
-        <v>0.9625</v>
+        <v>0.9457</v>
       </c>
       <c r="G174" s="10" t="n">
-        <v>0.9025</v>
+        <v>0.8883</v>
       </c>
       <c r="H174" s="10" t="n"/>
       <c r="I174" s="10" t="n">
-        <v>0</v>
+        <v>0.0026</v>
       </c>
       <c r="J174" s="13" t="n">
-        <v>2067</v>
+        <v>3906</v>
       </c>
       <c r="K174" s="13" t="n">
-        <v>2358</v>
+        <v>4613</v>
       </c>
       <c r="L174" s="32" t="n">
         <v>0</v>
@@ -16847,26 +16855,26 @@
         </is>
       </c>
       <c r="D175" s="15" t="n">
-        <v>45199.55</v>
+        <v>57966.37</v>
       </c>
       <c r="E175" s="15" t="n">
-        <v>116860.55</v>
+        <v>148690.47</v>
       </c>
       <c r="F175" s="16" t="n">
-        <v>0.9356</v>
+        <v>0.9084</v>
       </c>
       <c r="G175" s="16" t="n">
-        <v>0.8665</v>
+        <v>0.8403</v>
       </c>
       <c r="H175" s="16" t="n"/>
       <c r="I175" s="16" t="n">
-        <v>0</v>
+        <v>0.0014</v>
       </c>
       <c r="J175" s="19" t="n">
-        <v>2207</v>
+        <v>2920</v>
       </c>
       <c r="K175" s="19" t="n">
-        <v>2795</v>
+        <v>3685</v>
       </c>
       <c r="L175" s="31" t="n">
         <v>0</v>
@@ -17351,26 +17359,26 @@
         </is>
       </c>
       <c r="D187" s="15" t="n">
-        <v>624131.91</v>
+        <v>897376.26</v>
       </c>
       <c r="E187" s="15" t="n">
-        <v>23601.66</v>
+        <v>1925015.98</v>
       </c>
       <c r="F187" s="16" t="n">
-        <v>-0.2062</v>
+        <v>-0.1383</v>
       </c>
       <c r="G187" s="16" t="n">
-        <v>-0.2567</v>
+        <v>-0.1918</v>
       </c>
       <c r="H187" s="16" t="n"/>
       <c r="I187" s="16" t="n">
-        <v>0.1264</v>
+        <v>0.142</v>
       </c>
       <c r="J187" s="19" t="n">
-        <v>12948</v>
+        <v>20369</v>
       </c>
       <c r="K187" s="19" t="n">
-        <v>21770</v>
+        <v>34908</v>
       </c>
       <c r="L187" s="31" t="n">
         <v>0</v>
@@ -20627,26 +20635,26 @@
         </is>
       </c>
       <c r="D265" s="15" t="n">
-        <v>6762.42</v>
+        <v>17032.09</v>
       </c>
       <c r="E265" s="15" t="n">
-        <v>0</v>
+        <v>236357.21</v>
       </c>
       <c r="F265" s="16" t="n">
-        <v>0.7975</v>
+        <v>0.4042</v>
       </c>
       <c r="G265" s="16" t="n">
-        <v>0.7309</v>
+        <v>0.3663</v>
       </c>
       <c r="H265" s="16" t="n"/>
       <c r="I265" s="16" t="n">
-        <v>0.0328</v>
+        <v>0.0385</v>
       </c>
       <c r="J265" s="19" t="n">
-        <v>579</v>
+        <v>908</v>
       </c>
       <c r="K265" s="19" t="n">
-        <v>641</v>
+        <v>1026</v>
       </c>
       <c r="L265" s="31" t="n">
         <v>0</v>
@@ -20669,26 +20677,26 @@
         </is>
       </c>
       <c r="D266" s="9" t="n">
-        <v>284920.18</v>
+        <v>430966.7</v>
       </c>
       <c r="E266" s="9" t="n">
-        <v>13427.87</v>
+        <v>202744.47</v>
       </c>
       <c r="F266" s="10" t="n">
-        <v>-0.5718</v>
+        <v>-0.4086</v>
       </c>
       <c r="G266" s="10" t="n">
-        <v>-0.6161</v>
+        <v>-0.4582</v>
       </c>
       <c r="H266" s="10" t="n"/>
       <c r="I266" s="10" t="n">
-        <v>0.2892</v>
+        <v>0.2984</v>
       </c>
       <c r="J266" s="13" t="n">
-        <v>1556</v>
+        <v>2785</v>
       </c>
       <c r="K266" s="13" t="n">
-        <v>5870</v>
+        <v>10379</v>
       </c>
       <c r="L266" s="32" t="n">
         <v>0</v>
@@ -20711,26 +20719,26 @@
         </is>
       </c>
       <c r="D267" s="15" t="n">
-        <v>108635.18</v>
+        <v>150963.12</v>
       </c>
       <c r="E267" s="15" t="n">
-        <v>4919.51</v>
+        <v>210605.51</v>
       </c>
       <c r="F267" s="16" t="n">
-        <v>-0.5523</v>
+        <v>-0.371</v>
       </c>
       <c r="G267" s="16" t="n">
-        <v>-0.6046</v>
+        <v>-0.4288</v>
       </c>
       <c r="H267" s="16" t="n"/>
       <c r="I267" s="16" t="n">
-        <v>0.2372</v>
+        <v>0.2461</v>
       </c>
       <c r="J267" s="19" t="n">
-        <v>2352</v>
+        <v>3905</v>
       </c>
       <c r="K267" s="19" t="n">
-        <v>3895</v>
+        <v>6244</v>
       </c>
       <c r="L267" s="31" t="n">
         <v>0</v>
@@ -20753,26 +20761,26 @@
         </is>
       </c>
       <c r="D268" s="9" t="n">
-        <v>96261.31</v>
+        <v>118911.85</v>
       </c>
       <c r="E268" s="9" t="n">
-        <v>1533.45</v>
+        <v>245958.8</v>
       </c>
       <c r="F268" s="10" t="n">
-        <v>0.1039</v>
+        <v>0.1266</v>
       </c>
       <c r="G268" s="10" t="n">
-        <v>0.0553</v>
+        <v>0.0727</v>
       </c>
       <c r="H268" s="10" t="n"/>
       <c r="I268" s="10" t="n">
-        <v>0.1398</v>
+        <v>0.1603</v>
       </c>
       <c r="J268" s="13" t="n">
-        <v>2311</v>
+        <v>3549</v>
       </c>
       <c r="K268" s="13" t="n">
-        <v>3222</v>
+        <v>4890</v>
       </c>
       <c r="L268" s="32" t="n">
         <v>0</v>
@@ -20795,26 +20803,26 @@
         </is>
       </c>
       <c r="D269" s="15" t="n">
-        <v>51515.78</v>
+        <v>63314.99</v>
       </c>
       <c r="E269" s="15" t="n">
-        <v>1156.66</v>
+        <v>198639.55</v>
       </c>
       <c r="F269" s="16" t="n">
-        <v>0.5098</v>
+        <v>0.3724</v>
       </c>
       <c r="G269" s="16" t="n">
-        <v>0.4502</v>
+        <v>0.3065</v>
       </c>
       <c r="H269" s="16" t="n"/>
       <c r="I269" s="16" t="n">
-        <v>0.0771</v>
+        <v>0.0916</v>
       </c>
       <c r="J269" s="19" t="n">
-        <v>1867</v>
+        <v>2872</v>
       </c>
       <c r="K269" s="19" t="n">
-        <v>2297</v>
+        <v>3519</v>
       </c>
       <c r="L269" s="31" t="n">
         <v>0</v>
@@ -20837,26 +20845,26 @@
         </is>
       </c>
       <c r="D270" s="9" t="n">
-        <v>51792.25</v>
+        <v>64114.66</v>
       </c>
       <c r="E270" s="9" t="n">
-        <v>1509.83</v>
+        <v>319604.9</v>
       </c>
       <c r="F270" s="10" t="n">
-        <v>0.6056</v>
+        <v>0.5386</v>
       </c>
       <c r="G270" s="10" t="n">
-        <v>0.5407</v>
+        <v>0.4693</v>
       </c>
       <c r="H270" s="10" t="n"/>
       <c r="I270" s="10" t="n">
-        <v>0.0451</v>
+        <v>0.0495</v>
       </c>
       <c r="J270" s="13" t="n">
-        <v>2639</v>
+        <v>3919</v>
       </c>
       <c r="K270" s="13" t="n">
-        <v>3528</v>
+        <v>5227</v>
       </c>
       <c r="L270" s="32" t="n">
         <v>0</v>
@@ -20879,26 +20887,26 @@
         </is>
       </c>
       <c r="D271" s="15" t="n">
-        <v>24244.79</v>
+        <v>52072.86</v>
       </c>
       <c r="E271" s="15" t="n">
-        <v>1054.33</v>
+        <v>511105.54</v>
       </c>
       <c r="F271" s="16" t="n">
-        <v>0.8738</v>
+        <v>0.5376</v>
       </c>
       <c r="G271" s="16" t="n">
-        <v>0.8066</v>
+        <v>0.4932</v>
       </c>
       <c r="H271" s="16" t="n"/>
       <c r="I271" s="16" t="n">
-        <v>0.014</v>
+        <v>0.0165</v>
       </c>
       <c r="J271" s="19" t="n">
-        <v>1644</v>
+        <v>2431</v>
       </c>
       <c r="K271" s="19" t="n">
-        <v>2317</v>
+        <v>3623</v>
       </c>
       <c r="L271" s="31" t="n">
         <v>0</v>
@@ -21593,26 +21601,26 @@
         </is>
       </c>
       <c r="D288" s="9" t="n">
-        <v>11284.41</v>
+        <v>8369875.58</v>
       </c>
       <c r="E288" s="9" t="n">
-        <v>39829.95</v>
+        <v>16936057.2</v>
       </c>
       <c r="F288" s="10" t="n">
-        <v>0.9905</v>
+        <v>0.4738</v>
       </c>
       <c r="G288" s="10" t="n">
-        <v>0.9252</v>
+        <v>0.4146</v>
       </c>
       <c r="H288" s="10" t="n"/>
       <c r="I288" s="10" t="n">
-        <v>0</v>
+        <v>0.0629</v>
       </c>
       <c r="J288" s="13" t="n">
-        <v>1001</v>
+        <v>206966</v>
       </c>
       <c r="K288" s="13" t="n">
-        <v>1289</v>
+        <v>434008</v>
       </c>
       <c r="L288" s="32" t="n">
         <v>0</v>
@@ -26171,26 +26179,26 @@
         </is>
       </c>
       <c r="D397" s="15" t="n">
-        <v>2478.07</v>
+        <v>645702.85</v>
       </c>
       <c r="E397" s="15" t="n">
-        <v>22298.13</v>
+        <v>7014941.95</v>
       </c>
       <c r="F397" s="16" t="n">
-        <v>1.0516</v>
+        <v>0.9721</v>
       </c>
       <c r="G397" s="16" t="n">
-        <v>0.982</v>
+        <v>0.9054</v>
       </c>
       <c r="H397" s="16" t="n"/>
       <c r="I397" s="16" t="n">
-        <v>0</v>
+        <v>0.0048</v>
       </c>
       <c r="J397" s="19" t="n">
-        <v>372</v>
+        <v>45910</v>
       </c>
       <c r="K397" s="19" t="n">
-        <v>468</v>
+        <v>95256</v>
       </c>
       <c r="L397" s="31" t="n">
         <v>0</v>
@@ -26213,26 +26221,26 @@
         </is>
       </c>
       <c r="D398" s="9" t="n">
-        <v>1364.35</v>
+        <v>2952080</v>
       </c>
       <c r="E398" s="9" t="n">
-        <v>972.67</v>
+        <v>2479769.51</v>
       </c>
       <c r="F398" s="10" t="n">
-        <v>0.8804</v>
+        <v>0.246</v>
       </c>
       <c r="G398" s="10" t="n">
-        <v>0.8215</v>
+        <v>0.1894</v>
       </c>
       <c r="H398" s="10" t="n"/>
       <c r="I398" s="10" t="n">
-        <v>0</v>
+        <v>0.2448</v>
       </c>
       <c r="J398" s="13" t="n">
-        <v>41</v>
+        <v>14336</v>
       </c>
       <c r="K398" s="13" t="n">
-        <v>91</v>
+        <v>67993</v>
       </c>
       <c r="L398" s="32" t="n">
         <v>0</v>
@@ -26255,26 +26263,26 @@
         </is>
       </c>
       <c r="D399" s="15" t="n">
-        <v>1663.34</v>
+        <v>1669946.17</v>
       </c>
       <c r="E399" s="15" t="n">
-        <v>262.63</v>
+        <v>1164351.78</v>
       </c>
       <c r="F399" s="16" t="n">
-        <v>0.9691</v>
+        <v>0.3145</v>
       </c>
       <c r="G399" s="16" t="n">
-        <v>0.9115</v>
+        <v>0.2579</v>
       </c>
       <c r="H399" s="16" t="n"/>
       <c r="I399" s="16" t="n">
-        <v>0</v>
+        <v>0.1382</v>
       </c>
       <c r="J399" s="19" t="n">
-        <v>83</v>
+        <v>24854</v>
       </c>
       <c r="K399" s="19" t="n">
-        <v>105</v>
+        <v>67571</v>
       </c>
       <c r="L399" s="31" t="n">
         <v>0</v>
@@ -26297,26 +26305,26 @@
         </is>
       </c>
       <c r="D400" s="9" t="n">
-        <v>2030.12</v>
+        <v>1030756</v>
       </c>
       <c r="E400" s="9" t="n">
-        <v>2113.98</v>
+        <v>1020494.68</v>
       </c>
       <c r="F400" s="10" t="n">
-        <v>1.04</v>
+        <v>0.604</v>
       </c>
       <c r="G400" s="10" t="n">
-        <v>0.9791</v>
+        <v>0.5452</v>
       </c>
       <c r="H400" s="10" t="n"/>
       <c r="I400" s="10" t="n">
-        <v>0</v>
+        <v>0.0873</v>
       </c>
       <c r="J400" s="13" t="n">
-        <v>97</v>
+        <v>27871</v>
       </c>
       <c r="K400" s="13" t="n">
-        <v>127</v>
+        <v>44836</v>
       </c>
       <c r="L400" s="32" t="n">
         <v>0</v>
@@ -26339,26 +26347,26 @@
         </is>
       </c>
       <c r="D401" s="15" t="n">
-        <v>1025.55</v>
+        <v>630393.5600000001</v>
       </c>
       <c r="E401" s="15" t="n">
-        <v>753.0700000000001</v>
+        <v>576542.35</v>
       </c>
       <c r="F401" s="16" t="n">
-        <v>1.0091</v>
+        <v>0.5928</v>
       </c>
       <c r="G401" s="16" t="n">
-        <v>0.947</v>
+        <v>0.5314</v>
       </c>
       <c r="H401" s="16" t="n"/>
       <c r="I401" s="16" t="n">
-        <v>0</v>
+        <v>0.0636</v>
       </c>
       <c r="J401" s="19" t="n">
-        <v>74</v>
+        <v>22618</v>
       </c>
       <c r="K401" s="19" t="n">
-        <v>85</v>
+        <v>35026</v>
       </c>
       <c r="L401" s="31" t="n">
         <v>0</v>
@@ -26381,26 +26389,26 @@
         </is>
       </c>
       <c r="D402" s="9" t="n">
-        <v>1298.23</v>
+        <v>785515.38</v>
       </c>
       <c r="E402" s="9" t="n">
-        <v>4306.31</v>
+        <v>1313099.31</v>
       </c>
       <c r="F402" s="10" t="n">
-        <v>0.9832</v>
+        <v>0.7115</v>
       </c>
       <c r="G402" s="10" t="n">
-        <v>0.9111</v>
+        <v>0.6492</v>
       </c>
       <c r="H402" s="10" t="n"/>
       <c r="I402" s="10" t="n">
-        <v>0</v>
+        <v>0.0366</v>
       </c>
       <c r="J402" s="13" t="n">
-        <v>147</v>
+        <v>37815</v>
       </c>
       <c r="K402" s="13" t="n">
-        <v>188</v>
+        <v>50143</v>
       </c>
       <c r="L402" s="32" t="n">
         <v>0</v>
@@ -26423,26 +26431,26 @@
         </is>
       </c>
       <c r="D403" s="15" t="n">
-        <v>1424.75</v>
+        <v>655481.62</v>
       </c>
       <c r="E403" s="15" t="n">
-        <v>9123.17</v>
+        <v>3366857.62</v>
       </c>
       <c r="F403" s="16" t="n">
-        <v>0.9373</v>
+        <v>0.8098</v>
       </c>
       <c r="G403" s="16" t="n">
-        <v>0.8618</v>
+        <v>0.7456</v>
       </c>
       <c r="H403" s="16" t="n"/>
       <c r="I403" s="16" t="n">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="J403" s="19" t="n">
-        <v>187</v>
+        <v>33562</v>
       </c>
       <c r="K403" s="19" t="n">
-        <v>225</v>
+        <v>73183</v>
       </c>
       <c r="L403" s="31" t="n">
         <v>0</v>
@@ -27741,31 +27749,31 @@
         </is>
       </c>
       <c r="D433" s="15" t="n">
-        <v>19163529.07</v>
+        <v>27876873.41</v>
       </c>
       <c r="E433" s="15" t="n">
-        <v>29096000.56</v>
+        <v>37987244.76</v>
       </c>
       <c r="F433" s="16" t="n">
-        <v>0.4144</v>
+        <v>0.3732</v>
       </c>
       <c r="G433" s="16" t="n">
-        <v>0.3548</v>
+        <v>0.3195</v>
       </c>
       <c r="H433" s="16" t="n">
-        <v>0.1201</v>
+        <v>0.1203</v>
       </c>
       <c r="I433" s="16" t="n">
-        <v>0.0832</v>
+        <v>0.0998</v>
       </c>
       <c r="J433" s="19" t="n">
-        <v>416961</v>
+        <v>563557</v>
       </c>
       <c r="K433" s="19" t="n">
-        <v>879295</v>
+        <v>1122369</v>
       </c>
       <c r="L433" s="31" t="n">
-        <v>0.7733</v>
+        <v>0.5714</v>
       </c>
     </row>
     <row r="434">
@@ -36621,31 +36629,31 @@
         </is>
       </c>
       <c r="D635" s="15" t="n">
-        <v>2126572.06</v>
+        <v>2382816.39</v>
       </c>
       <c r="E635" s="15" t="n">
-        <v>12594160.16</v>
+        <v>14345686.04</v>
       </c>
       <c r="F635" s="16" t="n">
-        <v>0.7942</v>
+        <v>0.7859</v>
       </c>
       <c r="G635" s="16" t="n">
-        <v>0.7222</v>
+        <v>0.7151</v>
       </c>
       <c r="H635" s="16" t="n">
-        <v>0.5038</v>
+        <v>0.5065</v>
       </c>
       <c r="I635" s="16" t="n">
-        <v>0.0178</v>
+        <v>0.021</v>
       </c>
       <c r="J635" s="19" t="n">
-        <v>122338</v>
+        <v>137327</v>
       </c>
       <c r="K635" s="19" t="n">
-        <v>237256</v>
+        <v>255969</v>
       </c>
       <c r="L635" s="31" t="n">
-        <v>0.6673</v>
+        <v>0.6146</v>
       </c>
     </row>
     <row r="636">
@@ -36665,31 +36673,31 @@
         </is>
       </c>
       <c r="D636" s="9" t="n">
-        <v>4503217.77</v>
+        <v>7372698.27</v>
       </c>
       <c r="E636" s="9" t="n">
-        <v>4319291.41</v>
+        <v>6460768.27</v>
       </c>
       <c r="F636" s="10" t="n">
-        <v>0.0756</v>
+        <v>0.1808</v>
       </c>
       <c r="G636" s="10" t="n">
-        <v>0.0202</v>
+        <v>0.1317</v>
       </c>
       <c r="H636" s="10" t="n">
-        <v>0.0191</v>
+        <v>0.0198</v>
       </c>
       <c r="I636" s="10" t="n">
-        <v>0.2903</v>
+        <v>0.2849</v>
       </c>
       <c r="J636" s="13" t="n">
-        <v>15709</v>
+        <v>27842</v>
       </c>
       <c r="K636" s="13" t="n">
-        <v>75610</v>
+        <v>126549</v>
       </c>
       <c r="L636" s="32" t="n">
-        <v>0.7995</v>
+        <v>0.5368000000000001</v>
       </c>
     </row>
     <row r="637">
@@ -36709,31 +36717,31 @@
         </is>
       </c>
       <c r="D637" s="15" t="n">
-        <v>2565204.89</v>
+        <v>4243385.66</v>
       </c>
       <c r="E637" s="15" t="n">
-        <v>1288889.22</v>
+        <v>1997960.07</v>
       </c>
       <c r="F637" s="16" t="n">
-        <v>0.2335</v>
+        <v>0.2042</v>
       </c>
       <c r="G637" s="16" t="n">
-        <v>0.1817</v>
+        <v>0.1584</v>
       </c>
       <c r="H637" s="16" t="n">
-        <v>0.0625</v>
+        <v>0.0629</v>
       </c>
       <c r="I637" s="16" t="n">
-        <v>0.2286</v>
+        <v>0.2272</v>
       </c>
       <c r="J637" s="19" t="n">
-        <v>30752</v>
+        <v>52643</v>
       </c>
       <c r="K637" s="19" t="n">
-        <v>65105</v>
+        <v>103255</v>
       </c>
       <c r="L637" s="31" t="n">
-        <v>0.8335</v>
+        <v>0.5506</v>
       </c>
     </row>
     <row r="638">
@@ -36753,31 +36761,31 @@
         </is>
       </c>
       <c r="D638" s="9" t="n">
-        <v>2582084.54</v>
+        <v>3956831.51</v>
       </c>
       <c r="E638" s="9" t="n">
-        <v>1661131.29</v>
+        <v>2479619.7</v>
       </c>
       <c r="F638" s="10" t="n">
-        <v>0.2924</v>
+        <v>0.2317</v>
       </c>
       <c r="G638" s="10" t="n">
-        <v>0.2381</v>
+        <v>0.1827</v>
       </c>
       <c r="H638" s="10" t="n">
-        <v>0.0915</v>
+        <v>0.0922</v>
       </c>
       <c r="I638" s="10" t="n">
-        <v>0.1704</v>
+        <v>0.176</v>
       </c>
       <c r="J638" s="13" t="n">
-        <v>43209</v>
+        <v>68226</v>
       </c>
       <c r="K638" s="13" t="n">
-        <v>92285</v>
+        <v>131573</v>
       </c>
       <c r="L638" s="32" t="n">
-        <v>0.7614</v>
+        <v>0.5419</v>
       </c>
     </row>
     <row r="639">
@@ -36797,31 +36805,31 @@
         </is>
       </c>
       <c r="D639" s="15" t="n">
-        <v>2146681.85</v>
+        <v>3075031.01</v>
       </c>
       <c r="E639" s="15" t="n">
-        <v>1730740.71</v>
+        <v>2381296.53</v>
       </c>
       <c r="F639" s="16" t="n">
-        <v>0.4728</v>
+        <v>0.4155</v>
       </c>
       <c r="G639" s="16" t="n">
-        <v>0.4137</v>
+        <v>0.3618</v>
       </c>
       <c r="H639" s="16" t="n">
-        <v>0.1854</v>
+        <v>0.1823</v>
       </c>
       <c r="I639" s="16" t="n">
-        <v>0.1197</v>
+        <v>0.1309</v>
       </c>
       <c r="J639" s="19" t="n">
-        <v>43542</v>
+        <v>64666</v>
       </c>
       <c r="K639" s="19" t="n">
-        <v>94843</v>
+        <v>125865</v>
       </c>
       <c r="L639" s="31" t="n">
-        <v>0.7837</v>
+        <v>0.5915</v>
       </c>
     </row>
     <row r="640">
@@ -36841,31 +36849,31 @@
         </is>
       </c>
       <c r="D640" s="9" t="n">
-        <v>2811558.53</v>
+        <v>3777157.98</v>
       </c>
       <c r="E640" s="9" t="n">
-        <v>3565998.3</v>
+        <v>4970088.48</v>
       </c>
       <c r="F640" s="10" t="n">
-        <v>0.6017</v>
+        <v>0.5399</v>
       </c>
       <c r="G640" s="10" t="n">
-        <v>0.5384</v>
+        <v>0.4811</v>
       </c>
       <c r="H640" s="10" t="n">
-        <v>0.2373</v>
+        <v>0.2376</v>
       </c>
       <c r="I640" s="10" t="n">
-        <v>0.0708</v>
+        <v>0.08119999999999999</v>
       </c>
       <c r="J640" s="13" t="n">
-        <v>79230</v>
+        <v>108658</v>
       </c>
       <c r="K640" s="13" t="n">
-        <v>141124</v>
+        <v>178324</v>
       </c>
       <c r="L640" s="32" t="n">
-        <v>0.7901</v>
+        <v>0.6189</v>
       </c>
     </row>
     <row r="641">
@@ -36885,31 +36893,31 @@
         </is>
       </c>
       <c r="D641" s="15" t="n">
-        <v>2428209.44</v>
+        <v>3068952.59</v>
       </c>
       <c r="E641" s="15" t="n">
-        <v>3935789.48</v>
+        <v>5351825.67</v>
       </c>
       <c r="F641" s="16" t="n">
-        <v>0.7621</v>
+        <v>0.6838</v>
       </c>
       <c r="G641" s="16" t="n">
-        <v>0.6963</v>
+        <v>0.6217</v>
       </c>
       <c r="H641" s="16" t="n">
-        <v>0.3496</v>
+        <v>0.3482</v>
       </c>
       <c r="I641" s="16" t="n">
-        <v>0.0334</v>
+        <v>0.04</v>
       </c>
       <c r="J641" s="19" t="n">
-        <v>82181</v>
+        <v>104195</v>
       </c>
       <c r="K641" s="19" t="n">
-        <v>173072</v>
+        <v>200834</v>
       </c>
       <c r="L641" s="31" t="n">
-        <v>0.7377</v>
+        <v>0.6091</v>
       </c>
     </row>
     <row r="642">
@@ -37391,26 +37399,26 @@
         </is>
       </c>
       <c r="D653" s="15" t="n">
-        <v>9896975.279999999</v>
+        <v>9897635.68</v>
       </c>
       <c r="E653" s="15" t="n">
-        <v>50610765.13</v>
+        <v>50614019</v>
       </c>
       <c r="F653" s="16" t="n">
-        <v>0.3374</v>
+        <v>0.3372</v>
       </c>
       <c r="G653" s="16" t="n">
-        <v>0.2697</v>
+        <v>0.2695</v>
       </c>
       <c r="H653" s="16" t="n"/>
       <c r="I653" s="16" t="n">
         <v>0.0573</v>
       </c>
       <c r="J653" s="19" t="n">
-        <v>365768</v>
+        <v>365798</v>
       </c>
       <c r="K653" s="19" t="n">
-        <v>516271</v>
+        <v>516318</v>
       </c>
       <c r="L653" s="31" t="n">
         <v>0.449</v>
@@ -37433,29 +37441,29 @@
         </is>
       </c>
       <c r="D654" s="9" t="n">
-        <v>3768374.71</v>
+        <v>5552561.44</v>
       </c>
       <c r="E654" s="9" t="n">
-        <v>21423287.2</v>
+        <v>30841051.46</v>
       </c>
       <c r="F654" s="10" t="n">
-        <v>0.4153</v>
+        <v>0.3462</v>
       </c>
       <c r="G654" s="10" t="n">
-        <v>0.3487</v>
+        <v>0.2809</v>
       </c>
       <c r="H654" s="10" t="n"/>
       <c r="I654" s="10" t="n">
-        <v>0.0418</v>
+        <v>0.0633</v>
       </c>
       <c r="J654" s="13" t="n">
-        <v>165230</v>
+        <v>221623</v>
       </c>
       <c r="K654" s="13" t="n">
-        <v>229559</v>
+        <v>308208</v>
       </c>
       <c r="L654" s="32" t="n">
-        <v>0.836</v>
+        <v>0.6375</v>
       </c>
     </row>
     <row r="655">
@@ -40709,26 +40717,26 @@
         </is>
       </c>
       <c r="D732" s="9" t="n">
-        <v>2336015.38</v>
+        <v>2336050.19</v>
       </c>
       <c r="E732" s="9" t="n">
-        <v>30864233.1</v>
+        <v>30865240.19</v>
       </c>
       <c r="F732" s="10" t="n">
-        <v>0.5873</v>
+        <v>0.5869</v>
       </c>
       <c r="G732" s="10" t="n">
-        <v>0.5034999999999999</v>
+        <v>0.5031</v>
       </c>
       <c r="H732" s="10" t="n"/>
       <c r="I732" s="10" t="n">
         <v>0.0168</v>
       </c>
       <c r="J732" s="13" t="n">
-        <v>186935</v>
+        <v>186941</v>
       </c>
       <c r="K732" s="13" t="n">
-        <v>270092</v>
+        <v>270105</v>
       </c>
       <c r="L732" s="32" t="n">
         <v>0.5448</v>
@@ -40751,29 +40759,29 @@
         </is>
       </c>
       <c r="D733" s="15" t="n">
-        <v>1488662.03</v>
+        <v>1488971.46</v>
       </c>
       <c r="E733" s="15" t="n">
-        <v>881317.0600000001</v>
+        <v>881625.16</v>
       </c>
       <c r="F733" s="16" t="n">
-        <v>0.0692</v>
+        <v>0.06909999999999999</v>
       </c>
       <c r="G733" s="16" t="n">
-        <v>0.0227</v>
+        <v>0.0226</v>
       </c>
       <c r="H733" s="16" t="n"/>
       <c r="I733" s="16" t="n">
-        <v>0.3022</v>
+        <v>0.3024</v>
       </c>
       <c r="J733" s="19" t="n">
-        <v>8634</v>
+        <v>8640</v>
       </c>
       <c r="K733" s="19" t="n">
-        <v>19668</v>
+        <v>19676</v>
       </c>
       <c r="L733" s="31" t="n">
-        <v>0.3863</v>
+        <v>0.3862</v>
       </c>
     </row>
     <row r="734">
@@ -40793,26 +40801,26 @@
         </is>
       </c>
       <c r="D734" s="9" t="n">
-        <v>1400646.69</v>
+        <v>1400720.72</v>
       </c>
       <c r="E734" s="9" t="n">
-        <v>1407600.06</v>
+        <v>1407740.02</v>
       </c>
       <c r="F734" s="10" t="n">
-        <v>0.2761</v>
+        <v>0.276</v>
       </c>
       <c r="G734" s="10" t="n">
-        <v>0.2205</v>
+        <v>0.2204</v>
       </c>
       <c r="H734" s="10" t="n"/>
       <c r="I734" s="10" t="n">
-        <v>0.2097</v>
+        <v>0.2098</v>
       </c>
       <c r="J734" s="13" t="n">
-        <v>16002</v>
+        <v>16006</v>
       </c>
       <c r="K734" s="13" t="n">
-        <v>26456</v>
+        <v>26463</v>
       </c>
       <c r="L734" s="32" t="n">
         <v>0.4022</v>
@@ -40835,10 +40843,10 @@
         </is>
       </c>
       <c r="D735" s="15" t="n">
-        <v>1116938.71</v>
+        <v>1117128.73</v>
       </c>
       <c r="E735" s="15" t="n">
-        <v>1725416.65</v>
+        <v>1725507.23</v>
       </c>
       <c r="F735" s="16" t="n">
         <v>0.2488</v>
@@ -40848,16 +40856,16 @@
       </c>
       <c r="H735" s="16" t="n"/>
       <c r="I735" s="16" t="n">
-        <v>0.1526</v>
+        <v>0.1527</v>
       </c>
       <c r="J735" s="19" t="n">
-        <v>20945</v>
+        <v>20950</v>
       </c>
       <c r="K735" s="19" t="n">
-        <v>29988</v>
+        <v>29995</v>
       </c>
       <c r="L735" s="31" t="n">
-        <v>0.3912</v>
+        <v>0.3913</v>
       </c>
     </row>
     <row r="736">
@@ -40877,26 +40885,26 @@
         </is>
       </c>
       <c r="D736" s="9" t="n">
-        <v>972376.28</v>
+        <v>972390.35</v>
       </c>
       <c r="E736" s="9" t="n">
-        <v>2123280.92</v>
+        <v>2123377.24</v>
       </c>
       <c r="F736" s="10" t="n">
-        <v>0.3403</v>
+        <v>0.3402</v>
       </c>
       <c r="G736" s="10" t="n">
-        <v>0.275</v>
+        <v>0.2748</v>
       </c>
       <c r="H736" s="10" t="n"/>
       <c r="I736" s="10" t="n">
-        <v>0.1115</v>
+        <v>0.1116</v>
       </c>
       <c r="J736" s="13" t="n">
-        <v>22490</v>
+        <v>22492</v>
       </c>
       <c r="K736" s="13" t="n">
-        <v>30574</v>
+        <v>30576</v>
       </c>
       <c r="L736" s="32" t="n">
         <v>0.4498</v>
@@ -40919,10 +40927,10 @@
         </is>
       </c>
       <c r="D737" s="15" t="n">
-        <v>1312610.71</v>
+        <v>1312615.66</v>
       </c>
       <c r="E737" s="15" t="n">
-        <v>5012979.61</v>
+        <v>5012998.28</v>
       </c>
       <c r="F737" s="16" t="n">
         <v>0.2778</v>
@@ -40935,10 +40943,10 @@
         <v>0.0731</v>
       </c>
       <c r="J737" s="19" t="n">
-        <v>46875</v>
+        <v>46879</v>
       </c>
       <c r="K737" s="19" t="n">
-        <v>60115</v>
+        <v>60119</v>
       </c>
       <c r="L737" s="31" t="n">
         <v>0.4558</v>
@@ -40961,26 +40969,26 @@
         </is>
       </c>
       <c r="D738" s="9" t="n">
-        <v>1269725.47</v>
+        <v>1269758.58</v>
       </c>
       <c r="E738" s="9" t="n">
-        <v>8595937.73</v>
+        <v>8597530.869999999</v>
       </c>
       <c r="F738" s="10" t="n">
-        <v>0.3973</v>
+        <v>0.3969</v>
       </c>
       <c r="G738" s="10" t="n">
-        <v>0.318</v>
+        <v>0.3176</v>
       </c>
       <c r="H738" s="10" t="n"/>
       <c r="I738" s="10" t="n">
         <v>0.0425</v>
       </c>
       <c r="J738" s="13" t="n">
-        <v>63887</v>
+        <v>63890</v>
       </c>
       <c r="K738" s="13" t="n">
-        <v>79378</v>
+        <v>79384</v>
       </c>
       <c r="L738" s="32" t="n">
         <v>0.4412</v>
@@ -41003,29 +41011,29 @@
         </is>
       </c>
       <c r="D739" s="15" t="n">
-        <v>1260224.87</v>
+        <v>1526127.6</v>
       </c>
       <c r="E739" s="15" t="n">
-        <v>16984455.5</v>
+        <v>21743041.34</v>
       </c>
       <c r="F739" s="16" t="n">
-        <v>0.774</v>
+        <v>0.7499</v>
       </c>
       <c r="G739" s="16" t="n">
-        <v>0.6967</v>
+        <v>0.6712</v>
       </c>
       <c r="H739" s="16" t="n"/>
       <c r="I739" s="16" t="n">
-        <v>0.0074</v>
+        <v>0.013</v>
       </c>
       <c r="J739" s="19" t="n">
-        <v>104757</v>
+        <v>129562</v>
       </c>
       <c r="K739" s="19" t="n">
-        <v>145417</v>
+        <v>176984</v>
       </c>
       <c r="L739" s="31" t="n">
-        <v>0.7823</v>
+        <v>0.6856</v>
       </c>
     </row>
     <row r="740">
@@ -41045,29 +41053,29 @@
         </is>
       </c>
       <c r="D740" s="9" t="n">
-        <v>366911.43</v>
+        <v>713382.0699999999</v>
       </c>
       <c r="E740" s="9" t="n">
-        <v>134003.03</v>
+        <v>333765.27</v>
       </c>
       <c r="F740" s="10" t="n">
-        <v>0.2516</v>
+        <v>0.2173</v>
       </c>
       <c r="G740" s="10" t="n">
-        <v>0.2059</v>
+        <v>0.1765</v>
       </c>
       <c r="H740" s="10" t="n"/>
       <c r="I740" s="10" t="n">
-        <v>0.3534</v>
+        <v>0.3564</v>
       </c>
       <c r="J740" s="13" t="n">
-        <v>1893</v>
+        <v>3432</v>
       </c>
       <c r="K740" s="13" t="n">
-        <v>5651</v>
+        <v>10013</v>
       </c>
       <c r="L740" s="32" t="n">
-        <v>0.9008</v>
+        <v>0.5651</v>
       </c>
     </row>
     <row r="741">
@@ -41087,29 +41095,29 @@
         </is>
       </c>
       <c r="D741" s="15" t="n">
-        <v>459579.03</v>
+        <v>870756.5699999999</v>
       </c>
       <c r="E741" s="15" t="n">
-        <v>234353.03</v>
+        <v>740051.22</v>
       </c>
       <c r="F741" s="16" t="n">
-        <v>-0.0427</v>
+        <v>0.0477</v>
       </c>
       <c r="G741" s="16" t="n">
-        <v>-0.0955</v>
+        <v>-0.0047</v>
       </c>
       <c r="H741" s="16" t="n"/>
       <c r="I741" s="16" t="n">
-        <v>0.2631</v>
+        <v>0.2892</v>
       </c>
       <c r="J741" s="19" t="n">
-        <v>4640</v>
+        <v>8269</v>
       </c>
       <c r="K741" s="19" t="n">
-        <v>9082</v>
+        <v>16776</v>
       </c>
       <c r="L741" s="31" t="n">
-        <v>0.9185</v>
+        <v>0.6055</v>
       </c>
     </row>
     <row r="742">
@@ -41129,29 +41137,29 @@
         </is>
       </c>
       <c r="D742" s="9" t="n">
-        <v>359571.8</v>
+        <v>559064.24</v>
       </c>
       <c r="E742" s="9" t="n">
-        <v>419477.03</v>
+        <v>1150749.92</v>
       </c>
       <c r="F742" s="10" t="n">
-        <v>-0.001</v>
+        <v>0.1007</v>
       </c>
       <c r="G742" s="10" t="n">
-        <v>-0.0613</v>
+        <v>0.0373</v>
       </c>
       <c r="H742" s="10" t="n"/>
       <c r="I742" s="10" t="n">
-        <v>0.1828</v>
+        <v>0.2165</v>
       </c>
       <c r="J742" s="13" t="n">
-        <v>6314</v>
+        <v>10476</v>
       </c>
       <c r="K742" s="13" t="n">
-        <v>8525</v>
+        <v>14629</v>
       </c>
       <c r="L742" s="32" t="n">
-        <v>0.9109</v>
+        <v>0.6606</v>
       </c>
     </row>
     <row r="743">
@@ -41171,29 +41179,29 @@
         </is>
       </c>
       <c r="D743" s="15" t="n">
-        <v>282181.79</v>
+        <v>448941.17</v>
       </c>
       <c r="E743" s="15" t="n">
-        <v>358144.69</v>
+        <v>936068.63</v>
       </c>
       <c r="F743" s="16" t="n">
-        <v>0.1259</v>
+        <v>0.0458</v>
       </c>
       <c r="G743" s="16" t="n">
-        <v>0.0623</v>
+        <v>-0.018</v>
       </c>
       <c r="H743" s="16" t="n"/>
       <c r="I743" s="16" t="n">
-        <v>0.1344</v>
+        <v>0.1716</v>
       </c>
       <c r="J743" s="19" t="n">
-        <v>6993</v>
+        <v>11290</v>
       </c>
       <c r="K743" s="19" t="n">
-        <v>8877</v>
+        <v>14877</v>
       </c>
       <c r="L743" s="31" t="n">
-        <v>0.8355</v>
+        <v>0.5872000000000001</v>
       </c>
     </row>
     <row r="744">
@@ -41213,29 +41221,29 @@
         </is>
       </c>
       <c r="D744" s="9" t="n">
-        <v>493845.78</v>
+        <v>720689.46</v>
       </c>
       <c r="E744" s="9" t="n">
-        <v>945993.17</v>
+        <v>2093586.73</v>
       </c>
       <c r="F744" s="10" t="n">
-        <v>0.3805</v>
+        <v>0.2894</v>
       </c>
       <c r="G744" s="10" t="n">
-        <v>0.3135</v>
+        <v>0.22</v>
       </c>
       <c r="H744" s="10" t="n"/>
       <c r="I744" s="10" t="n">
-        <v>0.08</v>
+        <v>0.1079</v>
       </c>
       <c r="J744" s="13" t="n">
-        <v>16572</v>
+        <v>24908</v>
       </c>
       <c r="K744" s="13" t="n">
-        <v>21010</v>
+        <v>32102</v>
       </c>
       <c r="L744" s="32" t="n">
-        <v>0.8381999999999999</v>
+        <v>0.6377</v>
       </c>
     </row>
     <row r="745">
@@ -41255,29 +41263,29 @@
         </is>
       </c>
       <c r="D745" s="15" t="n">
-        <v>546060</v>
+        <v>713600.33</v>
       </c>
       <c r="E745" s="15" t="n">
-        <v>2346860.76</v>
+        <v>3843788.34</v>
       </c>
       <c r="F745" s="16" t="n">
-        <v>0.5382</v>
+        <v>0.4142</v>
       </c>
       <c r="G745" s="16" t="n">
-        <v>0.4653</v>
+        <v>0.3392</v>
       </c>
       <c r="H745" s="16" t="n"/>
       <c r="I745" s="16" t="n">
-        <v>0.0346</v>
+        <v>0.0548</v>
       </c>
       <c r="J745" s="19" t="n">
-        <v>24061</v>
+        <v>33686</v>
       </c>
       <c r="K745" s="19" t="n">
-        <v>30997</v>
+        <v>42827</v>
       </c>
       <c r="L745" s="31" t="n">
-        <v>0.7955</v>
+        <v>0.6595</v>
       </c>
     </row>
     <row r="746">
@@ -42179,29 +42187,29 @@
         </is>
       </c>
       <c r="D767" s="15" t="n">
-        <v>3277288.75</v>
+        <v>5483453.56</v>
       </c>
       <c r="E767" s="15" t="n">
-        <v>3750388.45</v>
+        <v>9874841.9</v>
       </c>
       <c r="F767" s="16" t="n">
-        <v>-0.032</v>
+        <v>0.075</v>
       </c>
       <c r="G767" s="16" t="n">
-        <v>-0.08690000000000001</v>
+        <v>0.0205</v>
       </c>
       <c r="H767" s="16" t="n"/>
       <c r="I767" s="16" t="n">
-        <v>0.0979</v>
+        <v>0.1246</v>
       </c>
       <c r="J767" s="19" t="n">
-        <v>53382</v>
+        <v>81877</v>
       </c>
       <c r="K767" s="19" t="n">
-        <v>82049</v>
+        <v>135202</v>
       </c>
       <c r="L767" s="31" t="n">
-        <v>0.89</v>
+        <v>0.6022999999999999</v>
       </c>
     </row>
     <row r="768">
@@ -48395,29 +48403,29 @@
         </is>
       </c>
       <c r="D915" s="15" t="n">
-        <v>203924.15</v>
+        <v>276988.77</v>
       </c>
       <c r="E915" s="15" t="n">
-        <v>1944479.75</v>
+        <v>2820085.75</v>
       </c>
       <c r="F915" s="16" t="n">
-        <v>0.7613</v>
+        <v>0.7255</v>
       </c>
       <c r="G915" s="16" t="n">
-        <v>0.6875</v>
+        <v>0.6533</v>
       </c>
       <c r="H915" s="16" t="n"/>
       <c r="I915" s="16" t="n">
-        <v>0.0164</v>
+        <v>0.0209</v>
       </c>
       <c r="J915" s="19" t="n">
-        <v>15907</v>
+        <v>20770</v>
       </c>
       <c r="K915" s="19" t="n">
-        <v>20270</v>
+        <v>28144</v>
       </c>
       <c r="L915" s="31" t="n">
-        <v>0.7203000000000001</v>
+        <v>0.5886</v>
       </c>
     </row>
     <row r="916">
@@ -48437,29 +48445,29 @@
         </is>
       </c>
       <c r="D916" s="9" t="n">
-        <v>1158675.89</v>
+        <v>2291959.42</v>
       </c>
       <c r="E916" s="9" t="n">
-        <v>261996.41</v>
+        <v>1803708.95</v>
       </c>
       <c r="F916" s="10" t="n">
-        <v>-0.4709</v>
+        <v>-0.1659</v>
       </c>
       <c r="G916" s="10" t="n">
-        <v>-0.5169</v>
+        <v>-0.2085</v>
       </c>
       <c r="H916" s="10" t="n"/>
       <c r="I916" s="10" t="n">
-        <v>0.3402</v>
+        <v>0.3334</v>
       </c>
       <c r="J916" s="13" t="n">
-        <v>2184</v>
+        <v>4736</v>
       </c>
       <c r="K916" s="13" t="n">
-        <v>13646</v>
+        <v>28199</v>
       </c>
       <c r="L916" s="32" t="n">
-        <v>0.9823</v>
+        <v>0.5687</v>
       </c>
     </row>
     <row r="917">
@@ -48479,29 +48487,29 @@
         </is>
       </c>
       <c r="D917" s="15" t="n">
-        <v>581812.35</v>
+        <v>982662.75</v>
       </c>
       <c r="E917" s="15" t="n">
-        <v>127423.29</v>
+        <v>941500.36</v>
       </c>
       <c r="F917" s="16" t="n">
-        <v>-0.0655</v>
+        <v>0.0703</v>
       </c>
       <c r="G917" s="16" t="n">
-        <v>-0.1172</v>
+        <v>0.0156</v>
       </c>
       <c r="H917" s="16" t="n"/>
       <c r="I917" s="16" t="n">
-        <v>0.2542</v>
+        <v>0.264</v>
       </c>
       <c r="J917" s="19" t="n">
-        <v>4665</v>
+        <v>9099</v>
       </c>
       <c r="K917" s="19" t="n">
-        <v>8334</v>
+        <v>16566</v>
       </c>
       <c r="L917" s="31" t="n">
-        <v>0.9351</v>
+        <v>0.6165</v>
       </c>
     </row>
     <row r="918">
@@ -48521,29 +48529,29 @@
         </is>
       </c>
       <c r="D918" s="9" t="n">
-        <v>430573.93</v>
+        <v>711252.12</v>
       </c>
       <c r="E918" s="9" t="n">
-        <v>162506.22</v>
+        <v>840514.73</v>
       </c>
       <c r="F918" s="10" t="n">
-        <v>-0.0173</v>
+        <v>0.1526</v>
       </c>
       <c r="G918" s="10" t="n">
-        <v>-0.0727</v>
+        <v>0.0916</v>
       </c>
       <c r="H918" s="10" t="n"/>
       <c r="I918" s="10" t="n">
-        <v>0.1932</v>
+        <v>0.2098</v>
       </c>
       <c r="J918" s="13" t="n">
-        <v>5715</v>
+        <v>10275</v>
       </c>
       <c r="K918" s="13" t="n">
-        <v>7811</v>
+        <v>14718</v>
       </c>
       <c r="L918" s="32" t="n">
-        <v>0.8797</v>
+        <v>0.6247</v>
       </c>
     </row>
     <row r="919">
@@ -48563,29 +48571,29 @@
         </is>
       </c>
       <c r="D919" s="15" t="n">
-        <v>291014.52</v>
+        <v>426478.87</v>
       </c>
       <c r="E919" s="15" t="n">
-        <v>160470.66</v>
+        <v>760356.08</v>
       </c>
       <c r="F919" s="16" t="n">
-        <v>0.2036</v>
+        <v>0.2153</v>
       </c>
       <c r="G919" s="16" t="n">
-        <v>0.1445</v>
+        <v>0.1525</v>
       </c>
       <c r="H919" s="16" t="n"/>
       <c r="I919" s="16" t="n">
-        <v>0.1266</v>
+        <v>0.1494</v>
       </c>
       <c r="J919" s="19" t="n">
-        <v>5385</v>
+        <v>8746</v>
       </c>
       <c r="K919" s="19" t="n">
-        <v>7609</v>
+        <v>12415</v>
       </c>
       <c r="L919" s="31" t="n">
-        <v>0.8073</v>
+        <v>0.6299</v>
       </c>
     </row>
     <row r="920">
@@ -48605,29 +48613,29 @@
         </is>
       </c>
       <c r="D920" s="9" t="n">
-        <v>375121.52</v>
+        <v>493474.78</v>
       </c>
       <c r="E920" s="9" t="n">
-        <v>416549.08</v>
+        <v>1255610.88</v>
       </c>
       <c r="F920" s="10" t="n">
-        <v>0.3764</v>
+        <v>0.3216</v>
       </c>
       <c r="G920" s="10" t="n">
-        <v>0.3122</v>
+        <v>0.2511</v>
       </c>
       <c r="H920" s="10" t="n"/>
       <c r="I920" s="10" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.1086</v>
       </c>
       <c r="J920" s="13" t="n">
-        <v>9704</v>
+        <v>14550</v>
       </c>
       <c r="K920" s="13" t="n">
-        <v>12933</v>
+        <v>19148</v>
       </c>
       <c r="L920" s="32" t="n">
-        <v>0.794</v>
+        <v>0.6616</v>
       </c>
     </row>
     <row r="921">
@@ -48647,29 +48655,29 @@
         </is>
       </c>
       <c r="D921" s="15" t="n">
-        <v>236166.39</v>
+        <v>300636.86</v>
       </c>
       <c r="E921" s="15" t="n">
-        <v>676963.04</v>
+        <v>1453065.16</v>
       </c>
       <c r="F921" s="16" t="n">
-        <v>0.5535</v>
+        <v>0.5396</v>
       </c>
       <c r="G921" s="16" t="n">
-        <v>0.4837</v>
+        <v>0.4655</v>
       </c>
       <c r="H921" s="16" t="n"/>
       <c r="I921" s="16" t="n">
-        <v>0.0403</v>
+        <v>0.0542</v>
       </c>
       <c r="J921" s="19" t="n">
-        <v>9822</v>
+        <v>13701</v>
       </c>
       <c r="K921" s="19" t="n">
-        <v>11446</v>
+        <v>16012</v>
       </c>
       <c r="L921" s="31" t="n">
-        <v>0.7461</v>
+        <v>0.6354</v>
       </c>
     </row>
     <row r="922">
@@ -49109,29 +49117,29 @@
         </is>
       </c>
       <c r="D932" s="9" t="n">
-        <v>1035654.53</v>
+        <v>1148293.19</v>
       </c>
       <c r="E932" s="9" t="n">
-        <v>3524999.1</v>
+        <v>3979184.96</v>
       </c>
       <c r="F932" s="10" t="n">
-        <v>0.8037</v>
+        <v>0.7647</v>
       </c>
       <c r="G932" s="10" t="n">
-        <v>0.7377</v>
+        <v>0.6969</v>
       </c>
       <c r="H932" s="10" t="n"/>
       <c r="I932" s="10" t="n">
-        <v>0.0172</v>
+        <v>0.0199</v>
       </c>
       <c r="J932" s="13" t="n">
-        <v>30157</v>
+        <v>33391</v>
       </c>
       <c r="K932" s="13" t="n">
-        <v>40376</v>
+        <v>44348</v>
       </c>
       <c r="L932" s="32" t="n">
-        <v>0.8692</v>
+        <v>0.8258</v>
       </c>
     </row>
     <row r="933">
@@ -52091,29 +52099,29 @@
         </is>
       </c>
       <c r="D1003" s="15" t="n">
-        <v>510752.64</v>
+        <v>539069.2</v>
       </c>
       <c r="E1003" s="15" t="n">
-        <v>2602741.4</v>
+        <v>2693869.74</v>
       </c>
       <c r="F1003" s="16" t="n">
-        <v>0.9189000000000001</v>
+        <v>0.9265</v>
       </c>
       <c r="G1003" s="16" t="n">
-        <v>0.8483000000000001</v>
+        <v>0.8558</v>
       </c>
       <c r="H1003" s="16" t="n"/>
       <c r="I1003" s="16" t="n">
-        <v>0.0054</v>
+        <v>0.0059</v>
       </c>
       <c r="J1003" s="19" t="n">
-        <v>21691</v>
+        <v>23197</v>
       </c>
       <c r="K1003" s="19" t="n">
-        <v>30422</v>
+        <v>32135</v>
       </c>
       <c r="L1003" s="31" t="n">
-        <v>0.9264</v>
+        <v>0.8944</v>
       </c>
     </row>
     <row r="1004">
@@ -52133,29 +52141,29 @@
         </is>
       </c>
       <c r="D1004" s="9" t="n">
-        <v>69082.39</v>
+        <v>90771.09</v>
       </c>
       <c r="E1004" s="9" t="n">
-        <v>22010.36</v>
+        <v>42511.89</v>
       </c>
       <c r="F1004" s="10" t="n">
-        <v>0.4438</v>
+        <v>0.4862</v>
       </c>
       <c r="G1004" s="10" t="n">
-        <v>0.3973</v>
+        <v>0.4366</v>
       </c>
       <c r="H1004" s="10" t="n"/>
       <c r="I1004" s="10" t="n">
-        <v>0.1509</v>
+        <v>0.1707</v>
       </c>
       <c r="J1004" s="13" t="n">
-        <v>318</v>
+        <v>451</v>
       </c>
       <c r="K1004" s="13" t="n">
-        <v>461</v>
+        <v>732</v>
       </c>
       <c r="L1004" s="32" t="n">
-        <v>0.3784</v>
+        <v>0.3394</v>
       </c>
     </row>
     <row r="1005">
@@ -52175,29 +52183,29 @@
         </is>
       </c>
       <c r="D1005" s="15" t="n">
-        <v>40505.39</v>
+        <v>50140.87</v>
       </c>
       <c r="E1005" s="15" t="n">
-        <v>22359.74</v>
+        <v>38055.84</v>
       </c>
       <c r="F1005" s="16" t="n">
-        <v>0.1155</v>
+        <v>0.1518</v>
       </c>
       <c r="G1005" s="16" t="n">
-        <v>0.0698</v>
+        <v>0.0977</v>
       </c>
       <c r="H1005" s="16" t="n"/>
       <c r="I1005" s="16" t="n">
-        <v>0.2056</v>
+        <v>0.194</v>
       </c>
       <c r="J1005" s="19" t="n">
-        <v>501</v>
+        <v>701</v>
       </c>
       <c r="K1005" s="19" t="n">
-        <v>592</v>
+        <v>874</v>
       </c>
       <c r="L1005" s="31" t="n">
-        <v>0.8851</v>
+        <v>0.8075</v>
       </c>
     </row>
     <row r="1006">
@@ -52217,29 +52225,29 @@
         </is>
       </c>
       <c r="D1006" s="9" t="n">
-        <v>54821.2</v>
+        <v>64373.77</v>
       </c>
       <c r="E1006" s="9" t="n">
-        <v>53646.45</v>
+        <v>71704.57000000001</v>
       </c>
       <c r="F1006" s="10" t="n">
-        <v>0.5894</v>
+        <v>0.5954</v>
       </c>
       <c r="G1006" s="10" t="n">
-        <v>0.5312</v>
+        <v>0.5354</v>
       </c>
       <c r="H1006" s="10" t="n"/>
       <c r="I1006" s="10" t="n">
-        <v>0.1061</v>
+        <v>0.1007</v>
       </c>
       <c r="J1006" s="13" t="n">
-        <v>735</v>
+        <v>973</v>
       </c>
       <c r="K1006" s="13" t="n">
-        <v>867</v>
+        <v>1191</v>
       </c>
       <c r="L1006" s="32" t="n">
-        <v>0.8242</v>
+        <v>0.7672</v>
       </c>
     </row>
     <row r="1007">
@@ -52259,29 +52267,29 @@
         </is>
       </c>
       <c r="D1007" s="15" t="n">
-        <v>73067.00999999999</v>
+        <v>88425.63</v>
       </c>
       <c r="E1007" s="15" t="n">
-        <v>152665.88</v>
+        <v>342241.31</v>
       </c>
       <c r="F1007" s="16" t="n">
-        <v>0.7020999999999999</v>
+        <v>0.2795</v>
       </c>
       <c r="G1007" s="16" t="n">
-        <v>0.6405999999999999</v>
+        <v>0.1956</v>
       </c>
       <c r="H1007" s="16" t="n"/>
       <c r="I1007" s="16" t="n">
-        <v>0.0621</v>
+        <v>0.0609</v>
       </c>
       <c r="J1007" s="19" t="n">
-        <v>869</v>
+        <v>1116</v>
       </c>
       <c r="K1007" s="19" t="n">
-        <v>1000</v>
+        <v>1301</v>
       </c>
       <c r="L1007" s="31" t="n">
-        <v>0.8762</v>
+        <v>0.8516</v>
       </c>
     </row>
     <row r="1008">
@@ -52301,29 +52309,29 @@
         </is>
       </c>
       <c r="D1008" s="9" t="n">
-        <v>140474.92</v>
+        <v>154157.43</v>
       </c>
       <c r="E1008" s="9" t="n">
-        <v>209161.26</v>
+        <v>280861.72</v>
       </c>
       <c r="F1008" s="10" t="n">
-        <v>0.793</v>
+        <v>0.7563</v>
       </c>
       <c r="G1008" s="10" t="n">
-        <v>0.7256</v>
+        <v>0.6899</v>
       </c>
       <c r="H1008" s="10" t="n"/>
       <c r="I1008" s="10" t="n">
-        <v>0.0301</v>
+        <v>0.0323</v>
       </c>
       <c r="J1008" s="13" t="n">
-        <v>2590</v>
+        <v>3067</v>
       </c>
       <c r="K1008" s="13" t="n">
-        <v>2972</v>
+        <v>3555</v>
       </c>
       <c r="L1008" s="32" t="n">
-        <v>0.8912</v>
+        <v>0.8614000000000001</v>
       </c>
     </row>
     <row r="1009">
@@ -52343,29 +52351,29 @@
         </is>
       </c>
       <c r="D1009" s="15" t="n">
-        <v>146950.99</v>
+        <v>161355.2</v>
       </c>
       <c r="E1009" s="15" t="n">
-        <v>462414</v>
+        <v>509939.9</v>
       </c>
       <c r="F1009" s="16" t="n">
-        <v>0.9028</v>
+        <v>0.9129</v>
       </c>
       <c r="G1009" s="16" t="n">
-        <v>0.8343</v>
+        <v>0.8443000000000001</v>
       </c>
       <c r="H1009" s="16" t="n"/>
       <c r="I1009" s="16" t="n">
-        <v>0.0119</v>
+        <v>0.0126</v>
       </c>
       <c r="J1009" s="19" t="n">
-        <v>3453</v>
+        <v>3886</v>
       </c>
       <c r="K1009" s="19" t="n">
-        <v>4062</v>
+        <v>4560</v>
       </c>
       <c r="L1009" s="31" t="n">
-        <v>0.8892</v>
+        <v>0.851</v>
       </c>
     </row>
     <row r="1010">
@@ -52763,26 +52771,26 @@
         </is>
       </c>
       <c r="D1019" s="15" t="n">
-        <v>706839.34</v>
+        <v>2194185.13</v>
       </c>
       <c r="E1019" s="15" t="n">
-        <v>653175.1</v>
+        <v>2768391.26</v>
       </c>
       <c r="F1019" s="16" t="n">
-        <v>0.7833</v>
+        <v>0.3072</v>
       </c>
       <c r="G1019" s="16" t="n">
-        <v>0.7271</v>
+        <v>0.251</v>
       </c>
       <c r="H1019" s="16" t="n"/>
       <c r="I1019" s="16" t="n">
-        <v>0.0658</v>
+        <v>0.09619999999999999</v>
       </c>
       <c r="J1019" s="19" t="n">
-        <v>11087</v>
+        <v>38202</v>
       </c>
       <c r="K1019" s="19" t="n">
-        <v>29369</v>
+        <v>104297</v>
       </c>
       <c r="L1019" s="31" t="n">
         <v>0</v>
@@ -55451,26 +55459,26 @@
         </is>
       </c>
       <c r="D1083" s="15" t="n">
-        <v>19641.56</v>
+        <v>112709.83</v>
       </c>
       <c r="E1083" s="15" t="n">
-        <v>30886.84</v>
+        <v>400355.64</v>
       </c>
       <c r="F1083" s="16" t="n">
-        <v>1.0013</v>
+        <v>0.8177</v>
       </c>
       <c r="G1083" s="16" t="n">
-        <v>0.9317</v>
+        <v>0.7532</v>
       </c>
       <c r="H1083" s="16" t="n"/>
       <c r="I1083" s="16" t="n">
-        <v>0.01</v>
+        <v>0.0209</v>
       </c>
       <c r="J1083" s="19" t="n">
-        <v>1403</v>
+        <v>5417</v>
       </c>
       <c r="K1083" s="19" t="n">
-        <v>5905</v>
+        <v>24209</v>
       </c>
       <c r="L1083" s="31" t="n">
         <v>0</v>
@@ -55493,26 +55501,26 @@
         </is>
       </c>
       <c r="D1084" s="9" t="n">
-        <v>314312.32</v>
+        <v>863638.87</v>
       </c>
       <c r="E1084" s="9" t="n">
-        <v>415585.84</v>
+        <v>944860.6</v>
       </c>
       <c r="F1084" s="10" t="n">
-        <v>0.9258</v>
+        <v>0.3192</v>
       </c>
       <c r="G1084" s="10" t="n">
-        <v>0.8725000000000001</v>
+        <v>0.2662</v>
       </c>
       <c r="H1084" s="10" t="n"/>
       <c r="I1084" s="10" t="n">
-        <v>0.1778</v>
+        <v>0.236</v>
       </c>
       <c r="J1084" s="13" t="n">
-        <v>1777</v>
+        <v>5770</v>
       </c>
       <c r="K1084" s="13" t="n">
-        <v>6873</v>
+        <v>18767</v>
       </c>
       <c r="L1084" s="32" t="n">
         <v>0</v>
@@ -55535,26 +55543,26 @@
         </is>
       </c>
       <c r="D1085" s="15" t="n">
-        <v>174412.5</v>
+        <v>510146.88</v>
       </c>
       <c r="E1085" s="15" t="n">
-        <v>71412.00999999999</v>
+        <v>295142.55</v>
       </c>
       <c r="F1085" s="16" t="n">
-        <v>0.6105</v>
+        <v>0.1569</v>
       </c>
       <c r="G1085" s="16" t="n">
-        <v>0.554</v>
+        <v>0.1015</v>
       </c>
       <c r="H1085" s="16" t="n"/>
       <c r="I1085" s="16" t="n">
-        <v>0.0896</v>
+        <v>0.1488</v>
       </c>
       <c r="J1085" s="19" t="n">
-        <v>2020</v>
+        <v>6510</v>
       </c>
       <c r="K1085" s="19" t="n">
-        <v>5661</v>
+        <v>15222</v>
       </c>
       <c r="L1085" s="31" t="n">
         <v>0</v>
@@ -55577,26 +55585,26 @@
         </is>
       </c>
       <c r="D1086" s="9" t="n">
-        <v>116816.39</v>
+        <v>292855.57</v>
       </c>
       <c r="E1086" s="9" t="n">
-        <v>24629.56</v>
+        <v>226119.52</v>
       </c>
       <c r="F1086" s="10" t="n">
-        <v>0.6301</v>
+        <v>0.3254</v>
       </c>
       <c r="G1086" s="10" t="n">
-        <v>0.5741000000000001</v>
+        <v>0.2665</v>
       </c>
       <c r="H1086" s="10" t="n"/>
       <c r="I1086" s="10" t="n">
-        <v>0.0548</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="J1086" s="13" t="n">
-        <v>2153</v>
+        <v>6023</v>
       </c>
       <c r="K1086" s="13" t="n">
-        <v>5626</v>
+        <v>12175</v>
       </c>
       <c r="L1086" s="32" t="n">
         <v>0</v>
@@ -55619,26 +55627,26 @@
         </is>
       </c>
       <c r="D1087" s="15" t="n">
-        <v>34806.45</v>
+        <v>154626.34</v>
       </c>
       <c r="E1087" s="15" t="n">
-        <v>4782.63</v>
+        <v>65947.07000000001</v>
       </c>
       <c r="F1087" s="16" t="n">
-        <v>0.8427</v>
+        <v>0.0494</v>
       </c>
       <c r="G1087" s="16" t="n">
-        <v>0.7829</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="H1087" s="16" t="n"/>
       <c r="I1087" s="16" t="n">
-        <v>0.036</v>
+        <v>0.0645</v>
       </c>
       <c r="J1087" s="19" t="n">
-        <v>1056</v>
+        <v>3751</v>
       </c>
       <c r="K1087" s="19" t="n">
-        <v>1340</v>
+        <v>5840</v>
       </c>
       <c r="L1087" s="31" t="n">
         <v>0</v>
@@ -55661,26 +55669,26 @@
         </is>
       </c>
       <c r="D1088" s="9" t="n">
-        <v>30680.23</v>
+        <v>142469.97</v>
       </c>
       <c r="E1088" s="9" t="n">
-        <v>71019.75</v>
+        <v>260570.96</v>
       </c>
       <c r="F1088" s="10" t="n">
-        <v>0.6252</v>
+        <v>0.262</v>
       </c>
       <c r="G1088" s="10" t="n">
-        <v>0.5605</v>
+        <v>0.2041</v>
       </c>
       <c r="H1088" s="10" t="n"/>
       <c r="I1088" s="10" t="n">
-        <v>0.0263</v>
+        <v>0.0484</v>
       </c>
       <c r="J1088" s="13" t="n">
-        <v>1519</v>
+        <v>5599</v>
       </c>
       <c r="K1088" s="13" t="n">
-        <v>2205</v>
+        <v>8045</v>
       </c>
       <c r="L1088" s="32" t="n">
         <v>0</v>
@@ -55703,26 +55711,26 @@
         </is>
       </c>
       <c r="D1089" s="15" t="n">
-        <v>16169.88</v>
+        <v>117737.67</v>
       </c>
       <c r="E1089" s="15" t="n">
-        <v>34858.47</v>
+        <v>575394.91</v>
       </c>
       <c r="F1089" s="16" t="n">
-        <v>0.8919</v>
+        <v>0.7305</v>
       </c>
       <c r="G1089" s="16" t="n">
-        <v>0.8225</v>
+        <v>0.6659</v>
       </c>
       <c r="H1089" s="16" t="n"/>
       <c r="I1089" s="16" t="n">
-        <v>0.019</v>
+        <v>0.024</v>
       </c>
       <c r="J1089" s="19" t="n">
-        <v>1159</v>
+        <v>5132</v>
       </c>
       <c r="K1089" s="19" t="n">
-        <v>1759</v>
+        <v>20039</v>
       </c>
       <c r="L1089" s="31" t="n">
         <v>0</v>
@@ -56207,26 +56215,26 @@
         </is>
       </c>
       <c r="D1101" s="15" t="n">
-        <v>151245773.1</v>
+        <v>151932450.44</v>
       </c>
       <c r="E1101" s="15" t="n">
-        <v>606356308.99</v>
+        <v>606872937.3099999</v>
       </c>
       <c r="F1101" s="16" t="n">
-        <v>0.07630000000000001</v>
+        <v>0.0762</v>
       </c>
       <c r="G1101" s="16" t="n">
         <v>0.018</v>
       </c>
       <c r="H1101" s="16" t="n"/>
       <c r="I1101" s="16" t="n">
-        <v>0.1027</v>
+        <v>0.1029</v>
       </c>
       <c r="J1101" s="19" t="n">
-        <v>3668122</v>
+        <v>3671001</v>
       </c>
       <c r="K1101" s="19" t="n">
-        <v>7084499</v>
+        <v>7097111</v>
       </c>
       <c r="L1101" s="31" t="n">
         <v>0</v>
@@ -56249,26 +56257,26 @@
         </is>
       </c>
       <c r="D1102" s="9" t="n">
-        <v>13355643.98</v>
+        <v>43726865.08</v>
       </c>
       <c r="E1102" s="9" t="n">
-        <v>82001280.94</v>
+        <v>198541152.32</v>
       </c>
       <c r="F1102" s="10" t="n">
-        <v>0.1853</v>
+        <v>0.2122</v>
       </c>
       <c r="G1102" s="10" t="n">
-        <v>0.1248</v>
+        <v>0.1538</v>
       </c>
       <c r="H1102" s="10" t="n"/>
       <c r="I1102" s="10" t="n">
-        <v>0.0828</v>
+        <v>0.0872</v>
       </c>
       <c r="J1102" s="13" t="n">
-        <v>430868</v>
+        <v>1144021</v>
       </c>
       <c r="K1102" s="13" t="n">
-        <v>824524</v>
+        <v>2251660</v>
       </c>
       <c r="L1102" s="32" t="n">
         <v>0</v>
@@ -59525,26 +59533,26 @@
         </is>
       </c>
       <c r="D1180" s="9" t="n">
-        <v>17526700.98</v>
+        <v>17527780.03</v>
       </c>
       <c r="E1180" s="9" t="n">
-        <v>296116658.82</v>
+        <v>296133942.32</v>
       </c>
       <c r="F1180" s="10" t="n">
-        <v>0.387</v>
+        <v>0.3868</v>
       </c>
       <c r="G1180" s="10" t="n">
-        <v>0.3052</v>
+        <v>0.3049</v>
       </c>
       <c r="H1180" s="10" t="n"/>
       <c r="I1180" s="10" t="n">
         <v>0.0298</v>
       </c>
       <c r="J1180" s="13" t="n">
-        <v>1340812</v>
+        <v>1340854</v>
       </c>
       <c r="K1180" s="13" t="n">
-        <v>2084198</v>
+        <v>2084261</v>
       </c>
       <c r="L1180" s="32" t="n">
         <v>0</v>
@@ -59567,26 +59575,26 @@
         </is>
       </c>
       <c r="D1181" s="15" t="n">
-        <v>40441452.55</v>
+        <v>40919055.23</v>
       </c>
       <c r="E1181" s="15" t="n">
-        <v>20536062</v>
+        <v>20758772.01</v>
       </c>
       <c r="F1181" s="16" t="n">
-        <v>0.0014</v>
+        <v>0.0026</v>
       </c>
       <c r="G1181" s="16" t="n">
-        <v>-0.0401</v>
+        <v>-0.039</v>
       </c>
       <c r="H1181" s="16" t="n"/>
       <c r="I1181" s="16" t="n">
-        <v>0.3057</v>
+        <v>0.3061</v>
       </c>
       <c r="J1181" s="19" t="n">
-        <v>178966</v>
+        <v>179969</v>
       </c>
       <c r="K1181" s="19" t="n">
-        <v>770006</v>
+        <v>776573</v>
       </c>
       <c r="L1181" s="31" t="n">
         <v>0</v>
@@ -59609,26 +59617,26 @@
         </is>
       </c>
       <c r="D1182" s="9" t="n">
-        <v>26235476.96</v>
+        <v>26404603.36</v>
       </c>
       <c r="E1182" s="9" t="n">
-        <v>25918110.3</v>
+        <v>26088317.89</v>
       </c>
       <c r="F1182" s="10" t="n">
-        <v>0.0257</v>
+        <v>0.0262</v>
       </c>
       <c r="G1182" s="10" t="n">
-        <v>-0.025</v>
+        <v>-0.0247</v>
       </c>
       <c r="H1182" s="10" t="n"/>
       <c r="I1182" s="10" t="n">
-        <v>0.2382</v>
+        <v>0.2383</v>
       </c>
       <c r="J1182" s="13" t="n">
-        <v>265642</v>
+        <v>266468</v>
       </c>
       <c r="K1182" s="13" t="n">
-        <v>710527</v>
+        <v>714370</v>
       </c>
       <c r="L1182" s="32" t="n">
         <v>0</v>
@@ -59651,26 +59659,26 @@
         </is>
       </c>
       <c r="D1183" s="15" t="n">
-        <v>19463336.15</v>
+        <v>19480688.72</v>
       </c>
       <c r="E1183" s="15" t="n">
-        <v>31147346.96</v>
+        <v>31181555.27</v>
       </c>
       <c r="F1183" s="16" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="G1183" s="16" t="n">
-        <v>-0.0301</v>
+        <v>-0.03</v>
       </c>
       <c r="H1183" s="16" t="n"/>
       <c r="I1183" s="16" t="n">
         <v>0.1908</v>
       </c>
       <c r="J1183" s="19" t="n">
-        <v>306636</v>
+        <v>307053</v>
       </c>
       <c r="K1183" s="19" t="n">
-        <v>660712</v>
+        <v>661656</v>
       </c>
       <c r="L1183" s="31" t="n">
         <v>0</v>
@@ -59693,26 +59701,26 @@
         </is>
       </c>
       <c r="D1184" s="9" t="n">
-        <v>14012392.33</v>
+        <v>14023253.68</v>
       </c>
       <c r="E1184" s="9" t="n">
-        <v>33831742.98</v>
+        <v>33857622.22</v>
       </c>
       <c r="F1184" s="10" t="n">
-        <v>0.0388</v>
+        <v>0.0392</v>
       </c>
       <c r="G1184" s="10" t="n">
-        <v>-0.023</v>
+        <v>-0.0225</v>
       </c>
       <c r="H1184" s="10" t="n"/>
       <c r="I1184" s="10" t="n">
         <v>0.1539</v>
       </c>
       <c r="J1184" s="13" t="n">
-        <v>301026</v>
+        <v>301282</v>
       </c>
       <c r="K1184" s="13" t="n">
-        <v>581217</v>
+        <v>581810</v>
       </c>
       <c r="L1184" s="32" t="n">
         <v>0</v>
@@ -59735,26 +59743,26 @@
         </is>
       </c>
       <c r="D1185" s="15" t="n">
-        <v>17984742.28</v>
+        <v>17993532.2</v>
       </c>
       <c r="E1185" s="15" t="n">
-        <v>75289562.56</v>
+        <v>75325795.97</v>
       </c>
       <c r="F1185" s="16" t="n">
-        <v>0.0594</v>
+        <v>0.0582</v>
       </c>
       <c r="G1185" s="16" t="n">
-        <v>-0.0098</v>
+        <v>-0.011</v>
       </c>
       <c r="H1185" s="16" t="n"/>
       <c r="I1185" s="16" t="n">
         <v>0.1144</v>
       </c>
       <c r="J1185" s="19" t="n">
-        <v>570149</v>
+        <v>570400</v>
       </c>
       <c r="K1185" s="19" t="n">
-        <v>1004835</v>
+        <v>1005326</v>
       </c>
       <c r="L1185" s="31" t="n">
         <v>0</v>
@@ -59777,26 +59785,26 @@
         </is>
       </c>
       <c r="D1186" s="9" t="n">
-        <v>15581671.85</v>
+        <v>15583537.22</v>
       </c>
       <c r="E1186" s="9" t="n">
-        <v>123516825.37</v>
+        <v>123526931.63</v>
       </c>
       <c r="F1186" s="10" t="n">
         <v>0.1212</v>
       </c>
       <c r="G1186" s="10" t="n">
-        <v>0.0472</v>
+        <v>0.0471</v>
       </c>
       <c r="H1186" s="10" t="n"/>
       <c r="I1186" s="10" t="n">
-        <v>0.0693</v>
+        <v>0.0694</v>
       </c>
       <c r="J1186" s="13" t="n">
-        <v>704891</v>
+        <v>704975</v>
       </c>
       <c r="K1186" s="13" t="n">
-        <v>1273004</v>
+        <v>1273115</v>
       </c>
       <c r="L1186" s="32" t="n">
         <v>0</v>
@@ -59819,26 +59827,26 @@
         </is>
       </c>
       <c r="D1187" s="15" t="n">
-        <v>2340285.46</v>
+        <v>6620353.75</v>
       </c>
       <c r="E1187" s="15" t="n">
-        <v>51361742.61</v>
+        <v>116963099.56</v>
       </c>
       <c r="F1187" s="16" t="n">
-        <v>0.4996</v>
+        <v>0.5511</v>
       </c>
       <c r="G1187" s="16" t="n">
-        <v>0.4141</v>
+        <v>0.4717</v>
       </c>
       <c r="H1187" s="16" t="n"/>
       <c r="I1187" s="16" t="n">
-        <v>0.0207</v>
+        <v>0.0221</v>
       </c>
       <c r="J1187" s="19" t="n">
-        <v>197314</v>
+        <v>491041</v>
       </c>
       <c r="K1187" s="19" t="n">
-        <v>340607</v>
+        <v>822895</v>
       </c>
       <c r="L1187" s="31" t="n">
         <v>0</v>
@@ -59861,26 +59869,26 @@
         </is>
       </c>
       <c r="D1188" s="9" t="n">
-        <v>3571522.62</v>
+        <v>10479063.64</v>
       </c>
       <c r="E1188" s="9" t="n">
-        <v>1774022.2</v>
+        <v>5392763.97</v>
       </c>
       <c r="F1188" s="10" t="n">
-        <v>0.1124</v>
+        <v>0.09429999999999999</v>
       </c>
       <c r="G1188" s="10" t="n">
-        <v>0.074</v>
+        <v>0.0539</v>
       </c>
       <c r="H1188" s="10" t="n"/>
       <c r="I1188" s="10" t="n">
-        <v>0.2985</v>
+        <v>0.3071</v>
       </c>
       <c r="J1188" s="13" t="n">
-        <v>18187</v>
+        <v>48047</v>
       </c>
       <c r="K1188" s="13" t="n">
-        <v>69768</v>
+        <v>192701</v>
       </c>
       <c r="L1188" s="32" t="n">
         <v>0</v>
@@ -59903,26 +59911,26 @@
         </is>
       </c>
       <c r="D1189" s="15" t="n">
-        <v>2089612.37</v>
+        <v>6715174.79</v>
       </c>
       <c r="E1189" s="15" t="n">
-        <v>2090595.13</v>
+        <v>6218363.71</v>
       </c>
       <c r="F1189" s="16" t="n">
-        <v>0.0644</v>
+        <v>0.06909999999999999</v>
       </c>
       <c r="G1189" s="16" t="n">
-        <v>0.0134</v>
+        <v>0.0195</v>
       </c>
       <c r="H1189" s="16" t="n"/>
       <c r="I1189" s="16" t="n">
-        <v>0.2266</v>
+        <v>0.2333</v>
       </c>
       <c r="J1189" s="19" t="n">
-        <v>25935</v>
+        <v>69071</v>
       </c>
       <c r="K1189" s="19" t="n">
-        <v>62346</v>
+        <v>172679</v>
       </c>
       <c r="L1189" s="31" t="n">
         <v>0</v>
@@ -59945,26 +59953,26 @@
         </is>
       </c>
       <c r="D1190" s="9" t="n">
-        <v>1481840.85</v>
+        <v>5444561.22</v>
       </c>
       <c r="E1190" s="9" t="n">
-        <v>2512227.38</v>
+        <v>7488148.39</v>
       </c>
       <c r="F1190" s="10" t="n">
-        <v>0.0737</v>
+        <v>0.1132</v>
       </c>
       <c r="G1190" s="10" t="n">
-        <v>0.0178</v>
+        <v>0.0594</v>
       </c>
       <c r="H1190" s="10" t="n"/>
       <c r="I1190" s="10" t="n">
-        <v>0.1779</v>
+        <v>0.187</v>
       </c>
       <c r="J1190" s="13" t="n">
-        <v>29511</v>
+        <v>80938</v>
       </c>
       <c r="K1190" s="13" t="n">
-        <v>58370</v>
+        <v>174970</v>
       </c>
       <c r="L1190" s="32" t="n">
         <v>0</v>
@@ -59987,26 +59995,26 @@
         </is>
       </c>
       <c r="D1191" s="15" t="n">
-        <v>1003281.01</v>
+        <v>3634193.55</v>
       </c>
       <c r="E1191" s="15" t="n">
-        <v>2631018.73</v>
+        <v>7810635.94</v>
       </c>
       <c r="F1191" s="16" t="n">
-        <v>0.0946</v>
+        <v>0.1073</v>
       </c>
       <c r="G1191" s="16" t="n">
-        <v>0.03</v>
+        <v>0.0449</v>
       </c>
       <c r="H1191" s="16" t="n"/>
       <c r="I1191" s="16" t="n">
-        <v>0.145</v>
+        <v>0.1527</v>
       </c>
       <c r="J1191" s="19" t="n">
-        <v>29268</v>
+        <v>78854</v>
       </c>
       <c r="K1191" s="19" t="n">
-        <v>49188</v>
+        <v>152189</v>
       </c>
       <c r="L1191" s="31" t="n">
         <v>0</v>
@@ -60029,26 +60037,26 @@
         </is>
       </c>
       <c r="D1192" s="9" t="n">
-        <v>1370663.54</v>
+        <v>5490548.72</v>
       </c>
       <c r="E1192" s="9" t="n">
-        <v>6125359.52</v>
+        <v>19558022.4</v>
       </c>
       <c r="F1192" s="10" t="n">
-        <v>0.1902</v>
+        <v>0.1786</v>
       </c>
       <c r="G1192" s="10" t="n">
-        <v>0.1197</v>
+        <v>0.1124</v>
       </c>
       <c r="H1192" s="10" t="n"/>
       <c r="I1192" s="10" t="n">
-        <v>0.1093</v>
+        <v>0.1101</v>
       </c>
       <c r="J1192" s="13" t="n">
-        <v>56060</v>
+        <v>158776</v>
       </c>
       <c r="K1192" s="13" t="n">
-        <v>91099</v>
+        <v>303782</v>
       </c>
       <c r="L1192" s="32" t="n">
         <v>0</v>
@@ -60071,26 +60079,26 @@
         </is>
       </c>
       <c r="D1193" s="15" t="n">
-        <v>1498438.12</v>
+        <v>5342969.41</v>
       </c>
       <c r="E1193" s="15" t="n">
-        <v>15506315.37</v>
+        <v>35110118.35</v>
       </c>
       <c r="F1193" s="16" t="n">
-        <v>0.2037</v>
+        <v>0.4102</v>
       </c>
       <c r="G1193" s="16" t="n">
-        <v>0.1238</v>
+        <v>0.3379</v>
       </c>
       <c r="H1193" s="16" t="n"/>
       <c r="I1193" s="16" t="n">
-        <v>0.06279999999999999</v>
+        <v>0.0615</v>
       </c>
       <c r="J1193" s="19" t="n">
-        <v>74593</v>
+        <v>217294</v>
       </c>
       <c r="K1193" s="19" t="n">
-        <v>153146</v>
+        <v>432444</v>
       </c>
       <c r="L1193" s="31" t="n">
         <v>0</v>
@@ -60575,26 +60583,26 @@
         </is>
       </c>
       <c r="D1205" s="15" t="n">
-        <v>53837.3</v>
+        <v>1494928.17</v>
       </c>
       <c r="E1205" s="15" t="n">
-        <v>144726.8</v>
+        <v>1312927.84</v>
       </c>
       <c r="F1205" s="16" t="n">
-        <v>0.8569</v>
+        <v>0.5211</v>
       </c>
       <c r="G1205" s="16" t="n">
-        <v>0.7923</v>
+        <v>0.4655</v>
       </c>
       <c r="H1205" s="16" t="n"/>
       <c r="I1205" s="16" t="n">
-        <v>0.0044</v>
+        <v>0.0378</v>
       </c>
       <c r="J1205" s="19" t="n">
-        <v>2283</v>
+        <v>25015</v>
       </c>
       <c r="K1205" s="19" t="n">
-        <v>2936</v>
+        <v>34242</v>
       </c>
       <c r="L1205" s="31" t="n">
         <v>0</v>
@@ -63851,26 +63859,26 @@
         </is>
       </c>
       <c r="D1283" s="15" t="n">
-        <v>8671.4</v>
+        <v>91660.8</v>
       </c>
       <c r="E1283" s="15" t="n">
-        <v>38558.08</v>
+        <v>377220.94</v>
       </c>
       <c r="F1283" s="16" t="n">
-        <v>0.8988</v>
+        <v>0.4359</v>
       </c>
       <c r="G1283" s="16" t="n">
-        <v>0.8287</v>
+        <v>0.3712</v>
       </c>
       <c r="H1283" s="16" t="n"/>
       <c r="I1283" s="16" t="n">
-        <v>0.0043</v>
+        <v>0.0057</v>
       </c>
       <c r="J1283" s="19" t="n">
-        <v>929</v>
+        <v>6148</v>
       </c>
       <c r="K1283" s="19" t="n">
-        <v>1158</v>
+        <v>7696</v>
       </c>
       <c r="L1283" s="31" t="n">
         <v>0</v>
@@ -63893,26 +63901,26 @@
         </is>
       </c>
       <c r="D1284" s="9" t="n">
-        <v>5974.59</v>
+        <v>375267.55</v>
       </c>
       <c r="E1284" s="9" t="n">
-        <v>1684.28</v>
+        <v>77652.03999999999</v>
       </c>
       <c r="F1284" s="10" t="n">
-        <v>0.9883999999999999</v>
+        <v>0.5082</v>
       </c>
       <c r="G1284" s="10" t="n">
-        <v>0.9362</v>
+        <v>0.4583</v>
       </c>
       <c r="H1284" s="10" t="n"/>
       <c r="I1284" s="10" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.2109</v>
       </c>
       <c r="J1284" s="13" t="n">
-        <v>107</v>
+        <v>1380</v>
       </c>
       <c r="K1284" s="13" t="n">
-        <v>231</v>
+        <v>3053</v>
       </c>
       <c r="L1284" s="32" t="n">
         <v>0</v>
@@ -63935,26 +63943,26 @@
         </is>
       </c>
       <c r="D1285" s="15" t="n">
-        <v>11247.27</v>
+        <v>402150</v>
       </c>
       <c r="E1285" s="15" t="n">
-        <v>7626.37</v>
+        <v>56647.05</v>
       </c>
       <c r="F1285" s="16" t="n">
-        <v>0.7502</v>
+        <v>0.1826</v>
       </c>
       <c r="G1285" s="16" t="n">
-        <v>0.7013</v>
+        <v>0.1296</v>
       </c>
       <c r="H1285" s="16" t="n"/>
       <c r="I1285" s="16" t="n">
-        <v>0.0279</v>
+        <v>0.104</v>
       </c>
       <c r="J1285" s="19" t="n">
-        <v>179</v>
+        <v>2626</v>
       </c>
       <c r="K1285" s="19" t="n">
-        <v>222</v>
+        <v>4056</v>
       </c>
       <c r="L1285" s="31" t="n">
         <v>0</v>
@@ -63977,26 +63985,26 @@
         </is>
       </c>
       <c r="D1286" s="9" t="n">
-        <v>7065.98</v>
+        <v>232991.87</v>
       </c>
       <c r="E1286" s="9" t="n">
-        <v>11037.89</v>
+        <v>113587.59</v>
       </c>
       <c r="F1286" s="10" t="n">
-        <v>0.6873</v>
+        <v>0.6991000000000001</v>
       </c>
       <c r="G1286" s="10" t="n">
-        <v>0.6127</v>
+        <v>0.644</v>
       </c>
       <c r="H1286" s="10" t="n"/>
       <c r="I1286" s="10" t="n">
-        <v>0</v>
+        <v>0.0536</v>
       </c>
       <c r="J1286" s="13" t="n">
-        <v>231</v>
+        <v>3133</v>
       </c>
       <c r="K1286" s="13" t="n">
-        <v>289</v>
+        <v>4397</v>
       </c>
       <c r="L1286" s="32" t="n">
         <v>0</v>
@@ -64019,26 +64027,26 @@
         </is>
       </c>
       <c r="D1287" s="15" t="n">
-        <v>5095.94</v>
+        <v>155344.25</v>
       </c>
       <c r="E1287" s="15" t="n">
-        <v>18009.98</v>
+        <v>197885.13</v>
       </c>
       <c r="F1287" s="16" t="n">
-        <v>0.8804999999999999</v>
+        <v>0.6581</v>
       </c>
       <c r="G1287" s="16" t="n">
-        <v>0.8071</v>
+        <v>0.5987</v>
       </c>
       <c r="H1287" s="16" t="n"/>
       <c r="I1287" s="16" t="n">
-        <v>0</v>
+        <v>0.0268</v>
       </c>
       <c r="J1287" s="19" t="n">
-        <v>206</v>
+        <v>2838</v>
       </c>
       <c r="K1287" s="19" t="n">
-        <v>266</v>
+        <v>4166</v>
       </c>
       <c r="L1287" s="31" t="n">
         <v>0</v>
@@ -64061,26 +64069,26 @@
         </is>
       </c>
       <c r="D1288" s="9" t="n">
-        <v>10247.51</v>
+        <v>156380.54</v>
       </c>
       <c r="E1288" s="9" t="n">
-        <v>28331.64</v>
+        <v>363073.33</v>
       </c>
       <c r="F1288" s="10" t="n">
-        <v>0.9981</v>
+        <v>0.8548</v>
       </c>
       <c r="G1288" s="10" t="n">
-        <v>0.9353</v>
+        <v>0.7919</v>
       </c>
       <c r="H1288" s="10" t="n"/>
       <c r="I1288" s="10" t="n">
-        <v>0</v>
+        <v>0.0152</v>
       </c>
       <c r="J1288" s="13" t="n">
-        <v>311</v>
+        <v>4808</v>
       </c>
       <c r="K1288" s="13" t="n">
-        <v>360</v>
+        <v>6121</v>
       </c>
       <c r="L1288" s="32" t="n">
         <v>0</v>
@@ -64103,26 +64111,26 @@
         </is>
       </c>
       <c r="D1289" s="15" t="n">
-        <v>5534.6</v>
+        <v>81133.17</v>
       </c>
       <c r="E1289" s="15" t="n">
-        <v>39478.56</v>
+        <v>126861.76</v>
       </c>
       <c r="F1289" s="16" t="n">
-        <v>0.7995</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="G1289" s="16" t="n">
-        <v>0.7158</v>
+        <v>0.8736</v>
       </c>
       <c r="H1289" s="16" t="n"/>
       <c r="I1289" s="16" t="n">
-        <v>0</v>
+        <v>0.0073</v>
       </c>
       <c r="J1289" s="19" t="n">
-        <v>320</v>
+        <v>4082</v>
       </c>
       <c r="K1289" s="19" t="n">
-        <v>410</v>
+        <v>4753</v>
       </c>
       <c r="L1289" s="31" t="n">
         <v>0</v>
@@ -64942,7 +64950,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-20 16:05 UTC</t>
+          <t>2026-10-21 16:34 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-22 16:31 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -1679,7 +1679,7 @@
         <v>21766760.99</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1234384.01</v>
+        <v>1234384.02</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>0.05671</v>
@@ -1692,7 +1692,7 @@
         <v>21766760.99</v>
       </c>
       <c r="J9" s="15" t="n">
-        <v>1234384.01</v>
+        <v>1234384.02</v>
       </c>
       <c r="K9" s="18" t="n"/>
       <c r="L9" s="19" t="n">
@@ -2892,7 +2892,7 @@
         </is>
       </c>
       <c r="I26" s="9" t="n">
-        <v>499580423.5</v>
+        <v>499580423.51</v>
       </c>
       <c r="J26" s="9" t="n">
         <v>6582164.99</v>
@@ -3049,7 +3049,7 @@
         <v>691271126.84</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>44338006.61</v>
+        <v>44338006.62</v>
       </c>
       <c r="K28" s="12" t="n">
         <v>0.06414</v>
@@ -5933,22 +5933,22 @@
         <v>46320</v>
       </c>
       <c r="B70" s="9" t="n">
-        <v>157372428.15</v>
+        <v>230834189.48</v>
       </c>
       <c r="C70" s="9" t="n">
-        <v>6857933.43</v>
+        <v>9891551.23</v>
       </c>
       <c r="D70" s="10" t="n">
-        <v>0.04358</v>
+        <v>0.04285</v>
       </c>
       <c r="E70" s="9" t="n">
-        <v>49773819.72</v>
+        <v>67747126.03</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>18335625.38</v>
+        <v>14711168.37</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>0.36838</v>
+        <v>0.21715</v>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
@@ -5956,19 +5956,19 @@
         </is>
       </c>
       <c r="I70" s="9" t="n">
-        <v>207146247.87</v>
+        <v>298581315.51</v>
       </c>
       <c r="J70" s="9" t="n">
-        <v>25193558.81</v>
+        <v>24602719.6</v>
       </c>
       <c r="K70" s="12" t="n">
-        <v>0.12162</v>
+        <v>0.0824</v>
       </c>
       <c r="L70" s="13" t="n">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="M70" s="13" t="n">
-        <v>-513</v>
+        <v>-374</v>
       </c>
       <c r="N70" s="9" t="n">
         <v>64762756.4</v>
@@ -5977,10 +5977,10 @@
         <v>0.05704</v>
       </c>
       <c r="P70" s="9" t="n">
-        <v>52982190.33</v>
+        <v>113298952.38</v>
       </c>
       <c r="Q70" s="10" t="n">
-        <v>0.05527</v>
+        <v>0.04748</v>
       </c>
       <c r="R70" s="9" t="n">
         <v>9057675.779999999</v>
@@ -5989,16 +5989,16 @@
         <v>-0.06547</v>
       </c>
       <c r="T70" s="9" t="n">
-        <v>13930969.8</v>
+        <v>15967573.79</v>
       </c>
       <c r="U70" s="10" t="n">
-        <v>0.06711</v>
+        <v>0.07665</v>
       </c>
       <c r="V70" s="9" t="n">
-        <v>16638835.85</v>
+        <v>27747231.13</v>
       </c>
       <c r="W70" s="10" t="n">
-        <v>-0.00637</v>
+        <v>0.00676</v>
       </c>
       <c r="X70" s="9" t="n"/>
       <c r="Y70" s="10" t="n"/>
@@ -7392,22 +7392,22 @@
         <v>46296</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>2436347848.3</v>
+        <v>2509809609.62</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>49817324.54</v>
+        <v>52850942.34</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.02045</v>
+        <v>0.02106</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>676690867.52</v>
+        <v>694672460.79</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>135221781.75</v>
+        <v>131605821.07</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.19983</v>
+        <v>0.18945</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
@@ -7415,19 +7415,19 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>3113038715.82</v>
+        <v>3204482070.41</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>185039106.29</v>
+        <v>184456763.41</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.05944</v>
+        <v>0.05756</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>648</v>
+        <v>662</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="N20" s="9" t="n">
         <v>1072027977.53</v>
@@ -7436,10 +7436,10 @@
         <v>0.01175</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>143697074.47</v>
+        <v>204013836.52</v>
       </c>
       <c r="Q20" s="10" t="n">
-        <v>0.04159</v>
+        <v>0.04131</v>
       </c>
       <c r="R20" s="9" t="n">
         <v>298312041.27</v>
@@ -7448,16 +7448,16 @@
         <v>0.04584</v>
       </c>
       <c r="T20" s="9" t="n">
-        <v>98866188.29000001</v>
+        <v>100902792.28</v>
       </c>
       <c r="U20" s="10" t="n">
-        <v>0.02706</v>
+        <v>0.02937</v>
       </c>
       <c r="V20" s="9" t="n">
-        <v>823444566.73</v>
+        <v>834552962.02</v>
       </c>
       <c r="W20" s="10" t="n">
-        <v>0.01809</v>
+        <v>0.0182</v>
       </c>
       <c r="X20" s="9" t="n"/>
       <c r="Y20" s="10" t="n"/>
@@ -8558,7 +8558,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-21 16:34 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-22 16:31 UTC.</t>
         </is>
       </c>
     </row>
@@ -10093,26 +10093,26 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>789950.65</v>
+        <v>2062239.18</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>1823775.13</v>
+        <v>6132442.66</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.404</v>
+        <v>0.3085</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.3456</v>
+        <v>0.2491</v>
       </c>
       <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.0891</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>18975</v>
+        <v>41361</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>29483</v>
+        <v>63489</v>
       </c>
       <c r="L14" s="32" t="n">
         <v>0</v>
@@ -12781,26 +12781,26 @@
         </is>
       </c>
       <c r="D78" s="9" t="n">
-        <v>63961.69</v>
+        <v>119345.55</v>
       </c>
       <c r="E78" s="9" t="n">
-        <v>1008625.06</v>
+        <v>2728144.04</v>
       </c>
       <c r="F78" s="10" t="n">
-        <v>0.8423</v>
+        <v>0.5097</v>
       </c>
       <c r="G78" s="10" t="n">
-        <v>0.775</v>
+        <v>0.4406</v>
       </c>
       <c r="H78" s="10" t="n"/>
       <c r="I78" s="10" t="n">
-        <v>0.0163</v>
+        <v>0.0278</v>
       </c>
       <c r="J78" s="13" t="n">
-        <v>4783</v>
+        <v>9284</v>
       </c>
       <c r="K78" s="13" t="n">
-        <v>9357</v>
+        <v>14897</v>
       </c>
       <c r="L78" s="32" t="n">
         <v>0</v>
@@ -12823,26 +12823,26 @@
         </is>
       </c>
       <c r="D79" s="15" t="n">
-        <v>202548.9</v>
+        <v>553792.55</v>
       </c>
       <c r="E79" s="15" t="n">
-        <v>96121.2</v>
+        <v>390392.73</v>
       </c>
       <c r="F79" s="16" t="n">
-        <v>0.1729</v>
+        <v>0.1723</v>
       </c>
       <c r="G79" s="16" t="n">
-        <v>0.1235</v>
+        <v>0.1219</v>
       </c>
       <c r="H79" s="16" t="n"/>
       <c r="I79" s="16" t="n">
-        <v>0.3054</v>
+        <v>0.3044</v>
       </c>
       <c r="J79" s="19" t="n">
-        <v>1192</v>
+        <v>2618</v>
       </c>
       <c r="K79" s="19" t="n">
-        <v>3077</v>
+        <v>7043</v>
       </c>
       <c r="L79" s="31" t="n">
         <v>0</v>
@@ -12865,26 +12865,26 @@
         </is>
       </c>
       <c r="D80" s="9" t="n">
-        <v>197824.14</v>
+        <v>510902.65</v>
       </c>
       <c r="E80" s="9" t="n">
-        <v>123062.5</v>
+        <v>508884.73</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>0.3015</v>
+        <v>0.2906</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>0.2444</v>
+        <v>0.2323</v>
       </c>
       <c r="H80" s="10" t="n"/>
       <c r="I80" s="10" t="n">
-        <v>0.1666</v>
+        <v>0.1924</v>
       </c>
       <c r="J80" s="13" t="n">
-        <v>2041</v>
+        <v>4750</v>
       </c>
       <c r="K80" s="13" t="n">
-        <v>3387</v>
+        <v>8416</v>
       </c>
       <c r="L80" s="32" t="n">
         <v>0</v>
@@ -12907,26 +12907,26 @@
         </is>
       </c>
       <c r="D81" s="15" t="n">
-        <v>121501.67</v>
+        <v>343297.97</v>
       </c>
       <c r="E81" s="15" t="n">
-        <v>110775.03</v>
+        <v>474455.89</v>
       </c>
       <c r="F81" s="16" t="n">
-        <v>0.5625</v>
+        <v>0.3262</v>
       </c>
       <c r="G81" s="16" t="n">
-        <v>0.5</v>
+        <v>0.2645</v>
       </c>
       <c r="H81" s="16" t="n"/>
       <c r="I81" s="16" t="n">
-        <v>0.0887</v>
+        <v>0.1203</v>
       </c>
       <c r="J81" s="19" t="n">
-        <v>2300</v>
+        <v>5577</v>
       </c>
       <c r="K81" s="19" t="n">
-        <v>3207</v>
+        <v>8317</v>
       </c>
       <c r="L81" s="31" t="n">
         <v>0</v>
@@ -12949,26 +12949,26 @@
         </is>
       </c>
       <c r="D82" s="9" t="n">
-        <v>70960.57000000001</v>
+        <v>194650.23</v>
       </c>
       <c r="E82" s="9" t="n">
-        <v>78655.84</v>
+        <v>422566.62</v>
       </c>
       <c r="F82" s="10" t="n">
-        <v>0.4666</v>
+        <v>0.2725</v>
       </c>
       <c r="G82" s="10" t="n">
-        <v>0.4028</v>
+        <v>0.208</v>
       </c>
       <c r="H82" s="10" t="n"/>
       <c r="I82" s="10" t="n">
-        <v>0.07439999999999999</v>
+        <v>0.0898</v>
       </c>
       <c r="J82" s="13" t="n">
-        <v>2123</v>
+        <v>4831</v>
       </c>
       <c r="K82" s="13" t="n">
-        <v>2775</v>
+        <v>6917</v>
       </c>
       <c r="L82" s="32" t="n">
         <v>0</v>
@@ -12991,26 +12991,26 @@
         </is>
       </c>
       <c r="D83" s="15" t="n">
-        <v>86018.75</v>
+        <v>222131.91</v>
       </c>
       <c r="E83" s="15" t="n">
-        <v>206540.07</v>
+        <v>969049.4300000001</v>
       </c>
       <c r="F83" s="16" t="n">
-        <v>0.3768</v>
+        <v>0.4333</v>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0.3147</v>
+        <v>0.3661</v>
       </c>
       <c r="H83" s="16" t="n"/>
       <c r="I83" s="16" t="n">
-        <v>0.031</v>
+        <v>0.0536</v>
       </c>
       <c r="J83" s="19" t="n">
-        <v>3543</v>
+        <v>7784</v>
       </c>
       <c r="K83" s="19" t="n">
-        <v>4152</v>
+        <v>9573</v>
       </c>
       <c r="L83" s="31" t="n">
         <v>0</v>
@@ -13033,26 +13033,26 @@
         </is>
       </c>
       <c r="D84" s="9" t="n">
-        <v>47134.93</v>
+        <v>118118.32</v>
       </c>
       <c r="E84" s="9" t="n">
-        <v>199995.44</v>
+        <v>638949.23</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>0.7802</v>
+        <v>0.5955</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>0.7146</v>
+        <v>0.5269</v>
       </c>
       <c r="H84" s="10" t="n"/>
       <c r="I84" s="10" t="n">
-        <v>0.0157</v>
+        <v>0.0299</v>
       </c>
       <c r="J84" s="13" t="n">
-        <v>2993</v>
+        <v>6517</v>
       </c>
       <c r="K84" s="13" t="n">
-        <v>3528</v>
+        <v>8326</v>
       </c>
       <c r="L84" s="32" t="n">
         <v>0</v>
@@ -14419,26 +14419,26 @@
         </is>
       </c>
       <c r="D117" s="15" t="n">
-        <v>1608230.32</v>
+        <v>2380079.75</v>
       </c>
       <c r="E117" s="15" t="n">
-        <v>1217175.74</v>
+        <v>2790676.8</v>
       </c>
       <c r="F117" s="16" t="n">
-        <v>0.6938</v>
+        <v>0.451</v>
       </c>
       <c r="G117" s="16" t="n">
-        <v>0.643</v>
+        <v>0.3981</v>
       </c>
       <c r="H117" s="16" t="n"/>
       <c r="I117" s="16" t="n">
-        <v>0.0285</v>
+        <v>0.0785</v>
       </c>
       <c r="J117" s="19" t="n">
-        <v>27368</v>
+        <v>35347</v>
       </c>
       <c r="K117" s="19" t="n">
-        <v>58665</v>
+        <v>81307</v>
       </c>
       <c r="L117" s="31" t="n">
         <v>0</v>
@@ -16603,26 +16603,26 @@
         </is>
       </c>
       <c r="D169" s="15" t="n">
-        <v>167105.66</v>
+        <v>172620.02</v>
       </c>
       <c r="E169" s="15" t="n">
-        <v>411678.23</v>
+        <v>452068.08</v>
       </c>
       <c r="F169" s="16" t="n">
-        <v>1.0229</v>
+        <v>1.0238</v>
       </c>
       <c r="G169" s="16" t="n">
-        <v>0.952</v>
+        <v>0.9529</v>
       </c>
       <c r="H169" s="16" t="n"/>
       <c r="I169" s="16" t="n">
         <v>0.0005</v>
       </c>
       <c r="J169" s="19" t="n">
-        <v>10025</v>
+        <v>10392</v>
       </c>
       <c r="K169" s="19" t="n">
-        <v>25272</v>
+        <v>26977</v>
       </c>
       <c r="L169" s="31" t="n">
         <v>0</v>
@@ -16645,26 +16645,26 @@
         </is>
       </c>
       <c r="D170" s="9" t="n">
-        <v>687676.72</v>
+        <v>1198140.41</v>
       </c>
       <c r="E170" s="9" t="n">
-        <v>261903.93</v>
+        <v>843154</v>
       </c>
       <c r="F170" s="10" t="n">
-        <v>0.4961</v>
+        <v>0.2334</v>
       </c>
       <c r="G170" s="10" t="n">
-        <v>0.454</v>
+        <v>0.1869</v>
       </c>
       <c r="H170" s="10" t="n"/>
       <c r="I170" s="10" t="n">
-        <v>0.1866</v>
+        <v>0.2804</v>
       </c>
       <c r="J170" s="13" t="n">
-        <v>2572</v>
+        <v>5331</v>
       </c>
       <c r="K170" s="13" t="n">
-        <v>7784</v>
+        <v>17441</v>
       </c>
       <c r="L170" s="32" t="n">
         <v>0</v>
@@ -16687,26 +16687,26 @@
         </is>
       </c>
       <c r="D171" s="15" t="n">
-        <v>390434.92</v>
+        <v>575088.16</v>
       </c>
       <c r="E171" s="15" t="n">
-        <v>157621.43</v>
+        <v>775354.85</v>
       </c>
       <c r="F171" s="16" t="n">
-        <v>0.7148</v>
+        <v>0.5246</v>
       </c>
       <c r="G171" s="16" t="n">
-        <v>0.6627999999999999</v>
+        <v>0.4681</v>
       </c>
       <c r="H171" s="16" t="n"/>
       <c r="I171" s="16" t="n">
-        <v>0.0625</v>
+        <v>0.1422</v>
       </c>
       <c r="J171" s="19" t="n">
-        <v>3422</v>
+        <v>5768</v>
       </c>
       <c r="K171" s="19" t="n">
-        <v>11460</v>
+        <v>19530</v>
       </c>
       <c r="L171" s="31" t="n">
         <v>0</v>
@@ -16729,26 +16729,26 @@
         </is>
       </c>
       <c r="D172" s="9" t="n">
-        <v>127571.05</v>
+        <v>171227.99</v>
       </c>
       <c r="E172" s="9" t="n">
-        <v>56335.08</v>
+        <v>176127.87</v>
       </c>
       <c r="F172" s="10" t="n">
-        <v>0.8021</v>
+        <v>0.5233</v>
       </c>
       <c r="G172" s="10" t="n">
-        <v>0.7511</v>
+        <v>0.4679</v>
       </c>
       <c r="H172" s="10" t="n"/>
       <c r="I172" s="10" t="n">
-        <v>0.0233</v>
+        <v>0.08649999999999999</v>
       </c>
       <c r="J172" s="13" t="n">
-        <v>2531</v>
+        <v>3643</v>
       </c>
       <c r="K172" s="13" t="n">
-        <v>3353</v>
+        <v>4865</v>
       </c>
       <c r="L172" s="32" t="n">
         <v>0</v>
@@ -16771,26 +16771,26 @@
         </is>
       </c>
       <c r="D173" s="15" t="n">
-        <v>67596.85000000001</v>
+        <v>84656.11</v>
       </c>
       <c r="E173" s="15" t="n">
-        <v>75044.21000000001</v>
+        <v>153148.07</v>
       </c>
       <c r="F173" s="16" t="n">
-        <v>0.9728</v>
+        <v>0.8007</v>
       </c>
       <c r="G173" s="16" t="n">
-        <v>0.9155</v>
+        <v>0.7438</v>
       </c>
       <c r="H173" s="16" t="n"/>
       <c r="I173" s="16" t="n">
-        <v>0.0045</v>
+        <v>0.0348</v>
       </c>
       <c r="J173" s="19" t="n">
-        <v>1992</v>
+        <v>2502</v>
       </c>
       <c r="K173" s="19" t="n">
-        <v>2498</v>
+        <v>3154</v>
       </c>
       <c r="L173" s="31" t="n">
         <v>0</v>
@@ -16813,26 +16813,26 @@
         </is>
       </c>
       <c r="D174" s="9" t="n">
-        <v>109878.76</v>
+        <v>118926.05</v>
       </c>
       <c r="E174" s="9" t="n">
-        <v>105902.39</v>
+        <v>221996.28</v>
       </c>
       <c r="F174" s="10" t="n">
-        <v>0.9457</v>
+        <v>0.8773</v>
       </c>
       <c r="G174" s="10" t="n">
-        <v>0.8883</v>
+        <v>0.8168</v>
       </c>
       <c r="H174" s="10" t="n"/>
       <c r="I174" s="10" t="n">
-        <v>0.0026</v>
+        <v>0.0098</v>
       </c>
       <c r="J174" s="13" t="n">
-        <v>3906</v>
+        <v>4610</v>
       </c>
       <c r="K174" s="13" t="n">
-        <v>4613</v>
+        <v>5450</v>
       </c>
       <c r="L174" s="32" t="n">
         <v>0</v>
@@ -16855,26 +16855,26 @@
         </is>
       </c>
       <c r="D175" s="15" t="n">
-        <v>57966.37</v>
+        <v>59421.01</v>
       </c>
       <c r="E175" s="15" t="n">
-        <v>148690.47</v>
+        <v>168827.66</v>
       </c>
       <c r="F175" s="16" t="n">
-        <v>0.9084</v>
+        <v>0.9038</v>
       </c>
       <c r="G175" s="16" t="n">
-        <v>0.8403</v>
+        <v>0.8355</v>
       </c>
       <c r="H175" s="16" t="n"/>
       <c r="I175" s="16" t="n">
-        <v>0.0014</v>
+        <v>0.0026</v>
       </c>
       <c r="J175" s="19" t="n">
-        <v>2920</v>
+        <v>3101</v>
       </c>
       <c r="K175" s="19" t="n">
-        <v>3685</v>
+        <v>3890</v>
       </c>
       <c r="L175" s="31" t="n">
         <v>0</v>
@@ -21601,26 +21601,26 @@
         </is>
       </c>
       <c r="D288" s="9" t="n">
-        <v>8369875.58</v>
+        <v>20957680.45</v>
       </c>
       <c r="E288" s="9" t="n">
-        <v>16936057.2</v>
+        <v>39767946.81</v>
       </c>
       <c r="F288" s="10" t="n">
-        <v>0.4738</v>
+        <v>-0.0166</v>
       </c>
       <c r="G288" s="10" t="n">
-        <v>0.4146</v>
+        <v>-0.077</v>
       </c>
       <c r="H288" s="10" t="n"/>
       <c r="I288" s="10" t="n">
-        <v>0.0629</v>
+        <v>0.1216</v>
       </c>
       <c r="J288" s="13" t="n">
-        <v>206966</v>
+        <v>490938</v>
       </c>
       <c r="K288" s="13" t="n">
-        <v>434008</v>
+        <v>1015531</v>
       </c>
       <c r="L288" s="32" t="n">
         <v>0</v>
@@ -26179,26 +26179,26 @@
         </is>
       </c>
       <c r="D397" s="15" t="n">
-        <v>645702.85</v>
+        <v>1486167.44</v>
       </c>
       <c r="E397" s="15" t="n">
-        <v>7014941.95</v>
+        <v>12296298.56</v>
       </c>
       <c r="F397" s="16" t="n">
-        <v>0.9721</v>
+        <v>-0.8596</v>
       </c>
       <c r="G397" s="16" t="n">
-        <v>0.9054</v>
+        <v>-0.9268</v>
       </c>
       <c r="H397" s="16" t="n"/>
       <c r="I397" s="16" t="n">
-        <v>0.0048</v>
+        <v>0.0582</v>
       </c>
       <c r="J397" s="19" t="n">
-        <v>45910</v>
+        <v>105041</v>
       </c>
       <c r="K397" s="19" t="n">
-        <v>95256</v>
+        <v>207263</v>
       </c>
       <c r="L397" s="31" t="n">
         <v>0</v>
@@ -26221,26 +26221,26 @@
         </is>
       </c>
       <c r="D398" s="9" t="n">
-        <v>2952080</v>
+        <v>7911790.13</v>
       </c>
       <c r="E398" s="9" t="n">
-        <v>2479769.51</v>
+        <v>7150674.57</v>
       </c>
       <c r="F398" s="10" t="n">
-        <v>0.246</v>
+        <v>0.0541</v>
       </c>
       <c r="G398" s="10" t="n">
-        <v>0.1894</v>
+        <v>-0.0037</v>
       </c>
       <c r="H398" s="10" t="n"/>
       <c r="I398" s="10" t="n">
-        <v>0.2448</v>
+        <v>0.3003</v>
       </c>
       <c r="J398" s="13" t="n">
-        <v>14336</v>
+        <v>37735</v>
       </c>
       <c r="K398" s="13" t="n">
-        <v>67993</v>
+        <v>160474</v>
       </c>
       <c r="L398" s="32" t="n">
         <v>0</v>
@@ -26263,26 +26263,26 @@
         </is>
       </c>
       <c r="D399" s="15" t="n">
-        <v>1669946.17</v>
+        <v>3857524.77</v>
       </c>
       <c r="E399" s="15" t="n">
-        <v>1164351.78</v>
+        <v>2953027.72</v>
       </c>
       <c r="F399" s="16" t="n">
-        <v>0.3145</v>
+        <v>0.0221</v>
       </c>
       <c r="G399" s="16" t="n">
-        <v>0.2579</v>
+        <v>-0.0353</v>
       </c>
       <c r="H399" s="16" t="n"/>
       <c r="I399" s="16" t="n">
-        <v>0.1382</v>
+        <v>0.206</v>
       </c>
       <c r="J399" s="19" t="n">
-        <v>24854</v>
+        <v>60153</v>
       </c>
       <c r="K399" s="19" t="n">
-        <v>67571</v>
+        <v>136152</v>
       </c>
       <c r="L399" s="31" t="n">
         <v>0</v>
@@ -26305,26 +26305,26 @@
         </is>
       </c>
       <c r="D400" s="9" t="n">
-        <v>1030756</v>
+        <v>2615936.81</v>
       </c>
       <c r="E400" s="9" t="n">
-        <v>1020494.68</v>
+        <v>2406819.01</v>
       </c>
       <c r="F400" s="10" t="n">
-        <v>0.604</v>
+        <v>0.1113</v>
       </c>
       <c r="G400" s="10" t="n">
-        <v>0.5452</v>
+        <v>0.0519</v>
       </c>
       <c r="H400" s="10" t="n"/>
       <c r="I400" s="10" t="n">
-        <v>0.0873</v>
+        <v>0.1537</v>
       </c>
       <c r="J400" s="13" t="n">
-        <v>27871</v>
+        <v>66696</v>
       </c>
       <c r="K400" s="13" t="n">
-        <v>44836</v>
+        <v>107021</v>
       </c>
       <c r="L400" s="32" t="n">
         <v>0</v>
@@ -26347,26 +26347,26 @@
         </is>
       </c>
       <c r="D401" s="15" t="n">
-        <v>630393.5600000001</v>
+        <v>1528456.69</v>
       </c>
       <c r="E401" s="15" t="n">
-        <v>576542.35</v>
+        <v>1632979.71</v>
       </c>
       <c r="F401" s="16" t="n">
-        <v>0.5928</v>
+        <v>0.0048</v>
       </c>
       <c r="G401" s="16" t="n">
-        <v>0.5314</v>
+        <v>-0.0581</v>
       </c>
       <c r="H401" s="16" t="n"/>
       <c r="I401" s="16" t="n">
-        <v>0.0636</v>
+        <v>0.122</v>
       </c>
       <c r="J401" s="19" t="n">
-        <v>22618</v>
+        <v>54157</v>
       </c>
       <c r="K401" s="19" t="n">
-        <v>35026</v>
+        <v>81306</v>
       </c>
       <c r="L401" s="31" t="n">
         <v>0</v>
@@ -26389,26 +26389,26 @@
         </is>
       </c>
       <c r="D402" s="9" t="n">
-        <v>785515.38</v>
+        <v>1861947.6</v>
       </c>
       <c r="E402" s="9" t="n">
-        <v>1313099.31</v>
+        <v>3125214</v>
       </c>
       <c r="F402" s="10" t="n">
-        <v>0.7115</v>
+        <v>0.0426</v>
       </c>
       <c r="G402" s="10" t="n">
-        <v>0.6492</v>
+        <v>-0.0211</v>
       </c>
       <c r="H402" s="10" t="n"/>
       <c r="I402" s="10" t="n">
-        <v>0.0366</v>
+        <v>0.0882</v>
       </c>
       <c r="J402" s="13" t="n">
-        <v>37815</v>
+        <v>88681</v>
       </c>
       <c r="K402" s="13" t="n">
-        <v>50143</v>
+        <v>124054</v>
       </c>
       <c r="L402" s="32" t="n">
         <v>0</v>
@@ -26431,26 +26431,26 @@
         </is>
       </c>
       <c r="D403" s="15" t="n">
-        <v>655481.62</v>
+        <v>1695857.01</v>
       </c>
       <c r="E403" s="15" t="n">
-        <v>3366857.62</v>
+        <v>10202933.25</v>
       </c>
       <c r="F403" s="16" t="n">
-        <v>0.8098</v>
+        <v>0.0223</v>
       </c>
       <c r="G403" s="16" t="n">
-        <v>0.7456</v>
+        <v>-0.046</v>
       </c>
       <c r="H403" s="16" t="n"/>
       <c r="I403" s="16" t="n">
-        <v>0.018</v>
+        <v>0.066</v>
       </c>
       <c r="J403" s="19" t="n">
-        <v>33562</v>
+        <v>78475</v>
       </c>
       <c r="K403" s="19" t="n">
-        <v>73183</v>
+        <v>199261</v>
       </c>
       <c r="L403" s="31" t="n">
         <v>0</v>
@@ -37402,7 +37402,7 @@
         <v>9897635.68</v>
       </c>
       <c r="E653" s="15" t="n">
-        <v>50614019</v>
+        <v>50614019.95</v>
       </c>
       <c r="F653" s="16" t="n">
         <v>0.3372</v>
@@ -37415,10 +37415,10 @@
         <v>0.0573</v>
       </c>
       <c r="J653" s="19" t="n">
-        <v>365798</v>
+        <v>365799</v>
       </c>
       <c r="K653" s="19" t="n">
-        <v>516318</v>
+        <v>516319</v>
       </c>
       <c r="L653" s="31" t="n">
         <v>0.449</v>
@@ -37441,29 +37441,29 @@
         </is>
       </c>
       <c r="D654" s="9" t="n">
-        <v>5552561.44</v>
+        <v>5883424.11</v>
       </c>
       <c r="E654" s="9" t="n">
-        <v>30841051.46</v>
+        <v>33683179.93</v>
       </c>
       <c r="F654" s="10" t="n">
-        <v>0.3462</v>
+        <v>0.3335</v>
       </c>
       <c r="G654" s="10" t="n">
-        <v>0.2809</v>
+        <v>0.2681</v>
       </c>
       <c r="H654" s="10" t="n"/>
       <c r="I654" s="10" t="n">
-        <v>0.0633</v>
+        <v>0.0641</v>
       </c>
       <c r="J654" s="13" t="n">
-        <v>221623</v>
+        <v>236162</v>
       </c>
       <c r="K654" s="13" t="n">
-        <v>308208</v>
+        <v>327042</v>
       </c>
       <c r="L654" s="32" t="n">
-        <v>0.6375</v>
+        <v>0.6099</v>
       </c>
     </row>
     <row r="655">
@@ -40804,7 +40804,7 @@
         <v>1400720.72</v>
       </c>
       <c r="E734" s="9" t="n">
-        <v>1407740.02</v>
+        <v>1407740.98</v>
       </c>
       <c r="F734" s="10" t="n">
         <v>0.276</v>
@@ -40817,10 +40817,10 @@
         <v>0.2098</v>
       </c>
       <c r="J734" s="13" t="n">
-        <v>16006</v>
+        <v>16007</v>
       </c>
       <c r="K734" s="13" t="n">
-        <v>26463</v>
+        <v>26464</v>
       </c>
       <c r="L734" s="32" t="n">
         <v>0.4022</v>
@@ -41011,29 +41011,29 @@
         </is>
       </c>
       <c r="D739" s="15" t="n">
-        <v>1526127.6</v>
+        <v>1638396.24</v>
       </c>
       <c r="E739" s="15" t="n">
-        <v>21743041.34</v>
+        <v>24103698.28</v>
       </c>
       <c r="F739" s="16" t="n">
-        <v>0.7499</v>
+        <v>0.7214</v>
       </c>
       <c r="G739" s="16" t="n">
-        <v>0.6712</v>
+        <v>0.6423</v>
       </c>
       <c r="H739" s="16" t="n"/>
       <c r="I739" s="16" t="n">
-        <v>0.013</v>
+        <v>0.0142</v>
       </c>
       <c r="J739" s="19" t="n">
-        <v>129562</v>
+        <v>139243</v>
       </c>
       <c r="K739" s="19" t="n">
-        <v>176984</v>
+        <v>190228</v>
       </c>
       <c r="L739" s="31" t="n">
-        <v>0.6856</v>
+        <v>0.6486</v>
       </c>
     </row>
     <row r="740">
@@ -41053,29 +41053,29 @@
         </is>
       </c>
       <c r="D740" s="9" t="n">
-        <v>713382.0699999999</v>
+        <v>723907.92</v>
       </c>
       <c r="E740" s="9" t="n">
-        <v>333765.27</v>
+        <v>336608.99</v>
       </c>
       <c r="F740" s="10" t="n">
-        <v>0.2173</v>
+        <v>0.2155</v>
       </c>
       <c r="G740" s="10" t="n">
-        <v>0.1765</v>
+        <v>0.1748</v>
       </c>
       <c r="H740" s="10" t="n"/>
       <c r="I740" s="10" t="n">
-        <v>0.3564</v>
+        <v>0.3497</v>
       </c>
       <c r="J740" s="13" t="n">
-        <v>3432</v>
+        <v>3563</v>
       </c>
       <c r="K740" s="13" t="n">
-        <v>10013</v>
+        <v>10193</v>
       </c>
       <c r="L740" s="32" t="n">
-        <v>0.5651</v>
+        <v>0.5591</v>
       </c>
     </row>
     <row r="741">
@@ -41095,29 +41095,29 @@
         </is>
       </c>
       <c r="D741" s="15" t="n">
-        <v>870756.5699999999</v>
+        <v>881711.33</v>
       </c>
       <c r="E741" s="15" t="n">
-        <v>740051.22</v>
+        <v>747959.14</v>
       </c>
       <c r="F741" s="16" t="n">
-        <v>0.0477</v>
+        <v>0.0417</v>
       </c>
       <c r="G741" s="16" t="n">
-        <v>-0.0047</v>
+        <v>-0.0108</v>
       </c>
       <c r="H741" s="16" t="n"/>
       <c r="I741" s="16" t="n">
-        <v>0.2892</v>
+        <v>0.2878</v>
       </c>
       <c r="J741" s="19" t="n">
-        <v>8269</v>
+        <v>8545</v>
       </c>
       <c r="K741" s="19" t="n">
-        <v>16776</v>
+        <v>17103</v>
       </c>
       <c r="L741" s="31" t="n">
-        <v>0.6055</v>
+        <v>0.6027</v>
       </c>
     </row>
     <row r="742">
@@ -41137,29 +41137,29 @@
         </is>
       </c>
       <c r="D742" s="9" t="n">
-        <v>559064.24</v>
+        <v>575257.27</v>
       </c>
       <c r="E742" s="9" t="n">
-        <v>1150749.92</v>
+        <v>1165771.54</v>
       </c>
       <c r="F742" s="10" t="n">
-        <v>0.1007</v>
+        <v>0.0827</v>
       </c>
       <c r="G742" s="10" t="n">
-        <v>0.0373</v>
+        <v>0.0195</v>
       </c>
       <c r="H742" s="10" t="n"/>
       <c r="I742" s="10" t="n">
-        <v>0.2165</v>
+        <v>0.218</v>
       </c>
       <c r="J742" s="13" t="n">
-        <v>10476</v>
+        <v>10915</v>
       </c>
       <c r="K742" s="13" t="n">
-        <v>14629</v>
+        <v>15130</v>
       </c>
       <c r="L742" s="32" t="n">
-        <v>0.6606</v>
+        <v>0.6513</v>
       </c>
     </row>
     <row r="743">
@@ -41179,29 +41179,29 @@
         </is>
       </c>
       <c r="D743" s="15" t="n">
-        <v>448941.17</v>
+        <v>486709.96</v>
       </c>
       <c r="E743" s="15" t="n">
-        <v>936068.63</v>
+        <v>981043.5699999999</v>
       </c>
       <c r="F743" s="16" t="n">
-        <v>0.0458</v>
+        <v>0.0203</v>
       </c>
       <c r="G743" s="16" t="n">
-        <v>-0.018</v>
+        <v>-0.0429</v>
       </c>
       <c r="H743" s="16" t="n"/>
       <c r="I743" s="16" t="n">
-        <v>0.1716</v>
+        <v>0.1736</v>
       </c>
       <c r="J743" s="19" t="n">
-        <v>11290</v>
+        <v>11793</v>
       </c>
       <c r="K743" s="19" t="n">
-        <v>14877</v>
+        <v>15442</v>
       </c>
       <c r="L743" s="31" t="n">
-        <v>0.5872000000000001</v>
+        <v>0.5508</v>
       </c>
     </row>
     <row r="744">
@@ -41221,29 +41221,29 @@
         </is>
       </c>
       <c r="D744" s="9" t="n">
-        <v>720689.46</v>
+        <v>755018.47</v>
       </c>
       <c r="E744" s="9" t="n">
-        <v>2093586.73</v>
+        <v>2188484.66</v>
       </c>
       <c r="F744" s="10" t="n">
-        <v>0.2894</v>
+        <v>0.2636</v>
       </c>
       <c r="G744" s="10" t="n">
-        <v>0.22</v>
+        <v>0.1942</v>
       </c>
       <c r="H744" s="10" t="n"/>
       <c r="I744" s="10" t="n">
-        <v>0.1079</v>
+        <v>0.1116</v>
       </c>
       <c r="J744" s="13" t="n">
-        <v>24908</v>
+        <v>26257</v>
       </c>
       <c r="K744" s="13" t="n">
-        <v>32102</v>
+        <v>33663</v>
       </c>
       <c r="L744" s="32" t="n">
-        <v>0.6377</v>
+        <v>0.6178</v>
       </c>
     </row>
     <row r="745">
@@ -41263,29 +41263,29 @@
         </is>
       </c>
       <c r="D745" s="15" t="n">
-        <v>713600.33</v>
+        <v>822422.9300000001</v>
       </c>
       <c r="E745" s="15" t="n">
-        <v>3843788.34</v>
+        <v>4159613.74</v>
       </c>
       <c r="F745" s="16" t="n">
-        <v>0.4142</v>
+        <v>0.4026</v>
       </c>
       <c r="G745" s="16" t="n">
-        <v>0.3392</v>
+        <v>0.3292</v>
       </c>
       <c r="H745" s="16" t="n"/>
       <c r="I745" s="16" t="n">
-        <v>0.0548</v>
+        <v>0.0586</v>
       </c>
       <c r="J745" s="19" t="n">
-        <v>33686</v>
+        <v>35846</v>
       </c>
       <c r="K745" s="19" t="n">
-        <v>42827</v>
+        <v>45283</v>
       </c>
       <c r="L745" s="31" t="n">
-        <v>0.6595</v>
+        <v>0.5836</v>
       </c>
     </row>
     <row r="746">
@@ -42187,29 +42187,29 @@
         </is>
       </c>
       <c r="D767" s="15" t="n">
-        <v>5483453.56</v>
+        <v>5728396.3</v>
       </c>
       <c r="E767" s="15" t="n">
-        <v>9874841.9</v>
+        <v>10713899.56</v>
       </c>
       <c r="F767" s="16" t="n">
-        <v>0.075</v>
+        <v>0.08840000000000001</v>
       </c>
       <c r="G767" s="16" t="n">
-        <v>0.0205</v>
+        <v>0.0329</v>
       </c>
       <c r="H767" s="16" t="n"/>
       <c r="I767" s="16" t="n">
-        <v>0.1246</v>
+        <v>0.1203</v>
       </c>
       <c r="J767" s="19" t="n">
-        <v>81877</v>
+        <v>86568</v>
       </c>
       <c r="K767" s="19" t="n">
-        <v>135202</v>
+        <v>141180</v>
       </c>
       <c r="L767" s="31" t="n">
-        <v>0.6022999999999999</v>
+        <v>0.5798</v>
       </c>
     </row>
     <row r="768">
@@ -48403,29 +48403,29 @@
         </is>
       </c>
       <c r="D915" s="15" t="n">
-        <v>276988.77</v>
+        <v>292227.67</v>
       </c>
       <c r="E915" s="15" t="n">
-        <v>2820085.75</v>
+        <v>3073006.16</v>
       </c>
       <c r="F915" s="16" t="n">
-        <v>0.7255</v>
+        <v>0.7371</v>
       </c>
       <c r="G915" s="16" t="n">
-        <v>0.6533</v>
+        <v>0.665</v>
       </c>
       <c r="H915" s="16" t="n"/>
       <c r="I915" s="16" t="n">
-        <v>0.0209</v>
+        <v>0.0201</v>
       </c>
       <c r="J915" s="19" t="n">
-        <v>20770</v>
+        <v>22508</v>
       </c>
       <c r="K915" s="19" t="n">
-        <v>28144</v>
+        <v>30273</v>
       </c>
       <c r="L915" s="31" t="n">
-        <v>0.5886</v>
+        <v>0.5588</v>
       </c>
     </row>
     <row r="916">
@@ -48445,29 +48445,29 @@
         </is>
       </c>
       <c r="D916" s="9" t="n">
-        <v>2291959.42</v>
+        <v>2406218.79</v>
       </c>
       <c r="E916" s="9" t="n">
-        <v>1803708.95</v>
+        <v>2093183.78</v>
       </c>
       <c r="F916" s="10" t="n">
-        <v>-0.1659</v>
+        <v>-0.1479</v>
       </c>
       <c r="G916" s="10" t="n">
-        <v>-0.2085</v>
+        <v>-0.1929</v>
       </c>
       <c r="H916" s="10" t="n"/>
       <c r="I916" s="10" t="n">
-        <v>0.3334</v>
+        <v>0.3198</v>
       </c>
       <c r="J916" s="13" t="n">
-        <v>4736</v>
+        <v>5038</v>
       </c>
       <c r="K916" s="13" t="n">
-        <v>28199</v>
+        <v>28913</v>
       </c>
       <c r="L916" s="32" t="n">
-        <v>0.5687</v>
+        <v>0.5425</v>
       </c>
     </row>
     <row r="917">
@@ -48487,29 +48487,29 @@
         </is>
       </c>
       <c r="D917" s="15" t="n">
-        <v>982662.75</v>
+        <v>1038988.12</v>
       </c>
       <c r="E917" s="15" t="n">
-        <v>941500.36</v>
+        <v>960900.15</v>
       </c>
       <c r="F917" s="16" t="n">
-        <v>0.0703</v>
+        <v>0.1065</v>
       </c>
       <c r="G917" s="16" t="n">
-        <v>0.0156</v>
+        <v>0.0514</v>
       </c>
       <c r="H917" s="16" t="n"/>
       <c r="I917" s="16" t="n">
-        <v>0.264</v>
+        <v>0.258</v>
       </c>
       <c r="J917" s="19" t="n">
-        <v>9099</v>
+        <v>9473</v>
       </c>
       <c r="K917" s="19" t="n">
-        <v>16566</v>
+        <v>17083</v>
       </c>
       <c r="L917" s="31" t="n">
-        <v>0.6165</v>
+        <v>0.5841</v>
       </c>
     </row>
     <row r="918">
@@ -48529,29 +48529,29 @@
         </is>
       </c>
       <c r="D918" s="9" t="n">
-        <v>711252.12</v>
+        <v>732812.42</v>
       </c>
       <c r="E918" s="9" t="n">
-        <v>840514.73</v>
+        <v>865290.91</v>
       </c>
       <c r="F918" s="10" t="n">
-        <v>0.1526</v>
+        <v>0.1566</v>
       </c>
       <c r="G918" s="10" t="n">
-        <v>0.0916</v>
+        <v>0.0954</v>
       </c>
       <c r="H918" s="10" t="n"/>
       <c r="I918" s="10" t="n">
-        <v>0.2098</v>
+        <v>0.206</v>
       </c>
       <c r="J918" s="13" t="n">
-        <v>10275</v>
+        <v>10698</v>
       </c>
       <c r="K918" s="13" t="n">
-        <v>14718</v>
+        <v>15311</v>
       </c>
       <c r="L918" s="32" t="n">
-        <v>0.6247</v>
+        <v>0.6149</v>
       </c>
     </row>
     <row r="919">
@@ -48571,29 +48571,29 @@
         </is>
       </c>
       <c r="D919" s="15" t="n">
-        <v>426478.87</v>
+        <v>441662.29</v>
       </c>
       <c r="E919" s="15" t="n">
-        <v>760356.08</v>
+        <v>794404.73</v>
       </c>
       <c r="F919" s="16" t="n">
-        <v>0.2153</v>
+        <v>0.1946</v>
       </c>
       <c r="G919" s="16" t="n">
-        <v>0.1525</v>
+        <v>0.1317</v>
       </c>
       <c r="H919" s="16" t="n"/>
       <c r="I919" s="16" t="n">
-        <v>0.1494</v>
+        <v>0.1463</v>
       </c>
       <c r="J919" s="19" t="n">
-        <v>8746</v>
+        <v>9114</v>
       </c>
       <c r="K919" s="19" t="n">
-        <v>12415</v>
+        <v>12821</v>
       </c>
       <c r="L919" s="31" t="n">
-        <v>0.6299</v>
+        <v>0.6248</v>
       </c>
     </row>
     <row r="920">
@@ -48613,29 +48613,29 @@
         </is>
       </c>
       <c r="D920" s="9" t="n">
-        <v>493474.78</v>
+        <v>505807.52</v>
       </c>
       <c r="E920" s="9" t="n">
-        <v>1255610.88</v>
+        <v>1300235.15</v>
       </c>
       <c r="F920" s="10" t="n">
-        <v>0.3216</v>
+        <v>0.3311</v>
       </c>
       <c r="G920" s="10" t="n">
-        <v>0.2511</v>
+        <v>0.2605</v>
       </c>
       <c r="H920" s="10" t="n"/>
       <c r="I920" s="10" t="n">
-        <v>0.1086</v>
+        <v>0.1058</v>
       </c>
       <c r="J920" s="13" t="n">
-        <v>14550</v>
+        <v>15259</v>
       </c>
       <c r="K920" s="13" t="n">
-        <v>19148</v>
+        <v>19919</v>
       </c>
       <c r="L920" s="32" t="n">
-        <v>0.6616</v>
+        <v>0.6479</v>
       </c>
     </row>
     <row r="921">
@@ -48655,29 +48655,29 @@
         </is>
       </c>
       <c r="D921" s="15" t="n">
-        <v>300636.86</v>
+        <v>310679.49</v>
       </c>
       <c r="E921" s="15" t="n">
-        <v>1453065.16</v>
+        <v>1626878.69</v>
       </c>
       <c r="F921" s="16" t="n">
-        <v>0.5396</v>
+        <v>0.5417</v>
       </c>
       <c r="G921" s="16" t="n">
-        <v>0.4655</v>
+        <v>0.4672</v>
       </c>
       <c r="H921" s="16" t="n"/>
       <c r="I921" s="16" t="n">
-        <v>0.0542</v>
+        <v>0.052</v>
       </c>
       <c r="J921" s="19" t="n">
-        <v>13701</v>
+        <v>14478</v>
       </c>
       <c r="K921" s="19" t="n">
-        <v>16012</v>
+        <v>16860</v>
       </c>
       <c r="L921" s="31" t="n">
-        <v>0.6354</v>
+        <v>0.6161</v>
       </c>
     </row>
     <row r="922">
@@ -49117,29 +49117,29 @@
         </is>
       </c>
       <c r="D932" s="9" t="n">
-        <v>1148293.19</v>
+        <v>1198339.07</v>
       </c>
       <c r="E932" s="9" t="n">
-        <v>3979184.96</v>
+        <v>4263679.11</v>
       </c>
       <c r="F932" s="10" t="n">
-        <v>0.7647</v>
+        <v>0.7712</v>
       </c>
       <c r="G932" s="10" t="n">
-        <v>0.6969</v>
+        <v>0.7033</v>
       </c>
       <c r="H932" s="10" t="n"/>
       <c r="I932" s="10" t="n">
-        <v>0.0199</v>
+        <v>0.0194</v>
       </c>
       <c r="J932" s="13" t="n">
-        <v>33391</v>
+        <v>35039</v>
       </c>
       <c r="K932" s="13" t="n">
-        <v>44348</v>
+        <v>46605</v>
       </c>
       <c r="L932" s="32" t="n">
-        <v>0.8258</v>
+        <v>0.7917999999999999</v>
       </c>
     </row>
     <row r="933">
@@ -52099,29 +52099,29 @@
         </is>
       </c>
       <c r="D1003" s="15" t="n">
-        <v>539069.2</v>
+        <v>551802.4300000001</v>
       </c>
       <c r="E1003" s="15" t="n">
-        <v>2693869.74</v>
+        <v>2780012.14</v>
       </c>
       <c r="F1003" s="16" t="n">
-        <v>0.9265</v>
+        <v>0.9288</v>
       </c>
       <c r="G1003" s="16" t="n">
-        <v>0.8558</v>
+        <v>0.8583</v>
       </c>
       <c r="H1003" s="16" t="n"/>
       <c r="I1003" s="16" t="n">
-        <v>0.0059</v>
+        <v>0.0057</v>
       </c>
       <c r="J1003" s="19" t="n">
-        <v>23197</v>
+        <v>24066</v>
       </c>
       <c r="K1003" s="19" t="n">
-        <v>32135</v>
+        <v>33202</v>
       </c>
       <c r="L1003" s="31" t="n">
-        <v>0.8944</v>
+        <v>0.8744</v>
       </c>
     </row>
     <row r="1004">
@@ -52141,29 +52141,29 @@
         </is>
       </c>
       <c r="D1004" s="9" t="n">
-        <v>90771.09</v>
+        <v>101232.93</v>
       </c>
       <c r="E1004" s="9" t="n">
-        <v>42511.89</v>
+        <v>94809.7</v>
       </c>
       <c r="F1004" s="10" t="n">
-        <v>0.4862</v>
+        <v>0.5261</v>
       </c>
       <c r="G1004" s="10" t="n">
-        <v>0.4366</v>
+        <v>0.4749</v>
       </c>
       <c r="H1004" s="10" t="n"/>
       <c r="I1004" s="10" t="n">
-        <v>0.1707</v>
+        <v>0.1649</v>
       </c>
       <c r="J1004" s="13" t="n">
-        <v>451</v>
+        <v>473</v>
       </c>
       <c r="K1004" s="13" t="n">
-        <v>732</v>
+        <v>779</v>
       </c>
       <c r="L1004" s="32" t="n">
-        <v>0.3394</v>
+        <v>0.3049</v>
       </c>
     </row>
     <row r="1005">
@@ -52183,29 +52183,29 @@
         </is>
       </c>
       <c r="D1005" s="15" t="n">
-        <v>50140.87</v>
+        <v>52065.34</v>
       </c>
       <c r="E1005" s="15" t="n">
-        <v>38055.84</v>
+        <v>43609.77</v>
       </c>
       <c r="F1005" s="16" t="n">
-        <v>0.1518</v>
+        <v>0.1682</v>
       </c>
       <c r="G1005" s="16" t="n">
-        <v>0.0977</v>
+        <v>0.1129</v>
       </c>
       <c r="H1005" s="16" t="n"/>
       <c r="I1005" s="16" t="n">
-        <v>0.194</v>
+        <v>0.1829</v>
       </c>
       <c r="J1005" s="19" t="n">
-        <v>701</v>
+        <v>771</v>
       </c>
       <c r="K1005" s="19" t="n">
-        <v>874</v>
+        <v>949</v>
       </c>
       <c r="L1005" s="31" t="n">
-        <v>0.8075</v>
+        <v>0.7786</v>
       </c>
     </row>
     <row r="1006">
@@ -52225,29 +52225,29 @@
         </is>
       </c>
       <c r="D1006" s="9" t="n">
-        <v>64373.77</v>
+        <v>69879.28</v>
       </c>
       <c r="E1006" s="9" t="n">
-        <v>71704.57000000001</v>
+        <v>82534.91</v>
       </c>
       <c r="F1006" s="10" t="n">
-        <v>0.5954</v>
+        <v>0.6143999999999999</v>
       </c>
       <c r="G1006" s="10" t="n">
-        <v>0.5354</v>
+        <v>0.5541</v>
       </c>
       <c r="H1006" s="10" t="n"/>
       <c r="I1006" s="10" t="n">
-        <v>0.1007</v>
+        <v>0.09370000000000001</v>
       </c>
       <c r="J1006" s="13" t="n">
-        <v>973</v>
+        <v>1078</v>
       </c>
       <c r="K1006" s="13" t="n">
-        <v>1191</v>
+        <v>1312</v>
       </c>
       <c r="L1006" s="32" t="n">
-        <v>0.7672</v>
+        <v>0.7081</v>
       </c>
     </row>
     <row r="1007">
@@ -52267,29 +52267,29 @@
         </is>
       </c>
       <c r="D1007" s="15" t="n">
-        <v>88425.63</v>
+        <v>91921.74000000001</v>
       </c>
       <c r="E1007" s="15" t="n">
-        <v>342241.31</v>
+        <v>362974.88</v>
       </c>
       <c r="F1007" s="16" t="n">
-        <v>0.2795</v>
+        <v>0.2831</v>
       </c>
       <c r="G1007" s="16" t="n">
-        <v>0.1956</v>
+        <v>0.1983</v>
       </c>
       <c r="H1007" s="16" t="n"/>
       <c r="I1007" s="16" t="n">
-        <v>0.0609</v>
+        <v>0.0558</v>
       </c>
       <c r="J1007" s="19" t="n">
-        <v>1116</v>
+        <v>1219</v>
       </c>
       <c r="K1007" s="19" t="n">
-        <v>1301</v>
+        <v>1419</v>
       </c>
       <c r="L1007" s="31" t="n">
-        <v>0.8516</v>
+        <v>0.8192</v>
       </c>
     </row>
     <row r="1008">
@@ -52309,29 +52309,29 @@
         </is>
       </c>
       <c r="D1008" s="9" t="n">
-        <v>154157.43</v>
+        <v>160540.29</v>
       </c>
       <c r="E1008" s="9" t="n">
-        <v>280861.72</v>
+        <v>318797.58</v>
       </c>
       <c r="F1008" s="10" t="n">
-        <v>0.7563</v>
+        <v>0.7702</v>
       </c>
       <c r="G1008" s="10" t="n">
-        <v>0.6899</v>
+        <v>0.7035</v>
       </c>
       <c r="H1008" s="10" t="n"/>
       <c r="I1008" s="10" t="n">
-        <v>0.0323</v>
+        <v>0.0318</v>
       </c>
       <c r="J1008" s="13" t="n">
-        <v>3067</v>
+        <v>3274</v>
       </c>
       <c r="K1008" s="13" t="n">
-        <v>3555</v>
+        <v>3937</v>
       </c>
       <c r="L1008" s="32" t="n">
-        <v>0.8614000000000001</v>
+        <v>0.8272</v>
       </c>
     </row>
     <row r="1009">
@@ -52351,29 +52351,29 @@
         </is>
       </c>
       <c r="D1009" s="15" t="n">
-        <v>161355.2</v>
+        <v>170897.05</v>
       </c>
       <c r="E1009" s="15" t="n">
-        <v>509939.9</v>
+        <v>580940.13</v>
       </c>
       <c r="F1009" s="16" t="n">
-        <v>0.9129</v>
+        <v>0.9191</v>
       </c>
       <c r="G1009" s="16" t="n">
-        <v>0.8443000000000001</v>
+        <v>0.8504</v>
       </c>
       <c r="H1009" s="16" t="n"/>
       <c r="I1009" s="16" t="n">
-        <v>0.0126</v>
+        <v>0.012</v>
       </c>
       <c r="J1009" s="19" t="n">
-        <v>3886</v>
+        <v>4158</v>
       </c>
       <c r="K1009" s="19" t="n">
-        <v>4560</v>
+        <v>5007</v>
       </c>
       <c r="L1009" s="31" t="n">
-        <v>0.851</v>
+        <v>0.8036</v>
       </c>
     </row>
     <row r="1010">
@@ -52771,26 +52771,26 @@
         </is>
       </c>
       <c r="D1019" s="15" t="n">
-        <v>2194185.13</v>
+        <v>3761117</v>
       </c>
       <c r="E1019" s="15" t="n">
-        <v>2768391.26</v>
+        <v>10181039.4</v>
       </c>
       <c r="F1019" s="16" t="n">
-        <v>0.3072</v>
+        <v>0.2452</v>
       </c>
       <c r="G1019" s="16" t="n">
-        <v>0.251</v>
+        <v>0.1904</v>
       </c>
       <c r="H1019" s="16" t="n"/>
       <c r="I1019" s="16" t="n">
-        <v>0.09619999999999999</v>
+        <v>0.1111</v>
       </c>
       <c r="J1019" s="19" t="n">
-        <v>38202</v>
+        <v>60182</v>
       </c>
       <c r="K1019" s="19" t="n">
-        <v>104297</v>
+        <v>155631</v>
       </c>
       <c r="L1019" s="31" t="n">
         <v>0</v>
@@ -55459,26 +55459,26 @@
         </is>
       </c>
       <c r="D1083" s="15" t="n">
-        <v>112709.83</v>
+        <v>140082.98</v>
       </c>
       <c r="E1083" s="15" t="n">
-        <v>400355.64</v>
+        <v>3539504.62</v>
       </c>
       <c r="F1083" s="16" t="n">
-        <v>0.8177</v>
+        <v>0.8312</v>
       </c>
       <c r="G1083" s="16" t="n">
-        <v>0.7532</v>
+        <v>0.7625999999999999</v>
       </c>
       <c r="H1083" s="16" t="n"/>
       <c r="I1083" s="16" t="n">
-        <v>0.0209</v>
+        <v>0.0254</v>
       </c>
       <c r="J1083" s="19" t="n">
-        <v>5417</v>
+        <v>7643</v>
       </c>
       <c r="K1083" s="19" t="n">
-        <v>24209</v>
+        <v>29077</v>
       </c>
       <c r="L1083" s="31" t="n">
         <v>0</v>
@@ -55501,26 +55501,26 @@
         </is>
       </c>
       <c r="D1084" s="9" t="n">
-        <v>863638.87</v>
+        <v>1643226.8</v>
       </c>
       <c r="E1084" s="9" t="n">
-        <v>944860.6</v>
+        <v>1488514.8</v>
       </c>
       <c r="F1084" s="10" t="n">
-        <v>0.3192</v>
+        <v>0.2281</v>
       </c>
       <c r="G1084" s="10" t="n">
-        <v>0.2662</v>
+        <v>0.1801</v>
       </c>
       <c r="H1084" s="10" t="n"/>
       <c r="I1084" s="10" t="n">
-        <v>0.236</v>
+        <v>0.2427</v>
       </c>
       <c r="J1084" s="13" t="n">
-        <v>5770</v>
+        <v>9690</v>
       </c>
       <c r="K1084" s="13" t="n">
-        <v>18767</v>
+        <v>33617</v>
       </c>
       <c r="L1084" s="32" t="n">
         <v>0</v>
@@ -55543,26 +55543,26 @@
         </is>
       </c>
       <c r="D1085" s="15" t="n">
-        <v>510146.88</v>
+        <v>860192.47</v>
       </c>
       <c r="E1085" s="15" t="n">
-        <v>295142.55</v>
+        <v>648869.47</v>
       </c>
       <c r="F1085" s="16" t="n">
-        <v>0.1569</v>
+        <v>0.1239</v>
       </c>
       <c r="G1085" s="16" t="n">
-        <v>0.1015</v>
+        <v>0.0678</v>
       </c>
       <c r="H1085" s="16" t="n"/>
       <c r="I1085" s="16" t="n">
-        <v>0.1488</v>
+        <v>0.1651</v>
       </c>
       <c r="J1085" s="19" t="n">
-        <v>6510</v>
+        <v>10760</v>
       </c>
       <c r="K1085" s="19" t="n">
-        <v>15222</v>
+        <v>25498</v>
       </c>
       <c r="L1085" s="31" t="n">
         <v>0</v>
@@ -55585,26 +55585,26 @@
         </is>
       </c>
       <c r="D1086" s="9" t="n">
-        <v>292855.57</v>
+        <v>498427.51</v>
       </c>
       <c r="E1086" s="9" t="n">
-        <v>226119.52</v>
+        <v>727135.91</v>
       </c>
       <c r="F1086" s="10" t="n">
-        <v>0.3254</v>
+        <v>0.259</v>
       </c>
       <c r="G1086" s="10" t="n">
-        <v>0.2665</v>
+        <v>0.199</v>
       </c>
       <c r="H1086" s="10" t="n"/>
       <c r="I1086" s="10" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.1164</v>
       </c>
       <c r="J1086" s="13" t="n">
-        <v>6023</v>
+        <v>9752</v>
       </c>
       <c r="K1086" s="13" t="n">
-        <v>12175</v>
+        <v>19987</v>
       </c>
       <c r="L1086" s="32" t="n">
         <v>0</v>
@@ -55627,26 +55627,26 @@
         </is>
       </c>
       <c r="D1087" s="15" t="n">
-        <v>154626.34</v>
+        <v>236016.44</v>
       </c>
       <c r="E1087" s="15" t="n">
-        <v>65947.07000000001</v>
+        <v>354154.05</v>
       </c>
       <c r="F1087" s="16" t="n">
-        <v>0.0494</v>
+        <v>0.0487</v>
       </c>
       <c r="G1087" s="16" t="n">
-        <v>-0.008800000000000001</v>
+        <v>-0.0134</v>
       </c>
       <c r="H1087" s="16" t="n"/>
       <c r="I1087" s="16" t="n">
-        <v>0.0645</v>
+        <v>0.0815</v>
       </c>
       <c r="J1087" s="19" t="n">
-        <v>3751</v>
+        <v>5893</v>
       </c>
       <c r="K1087" s="19" t="n">
-        <v>5840</v>
+        <v>9374</v>
       </c>
       <c r="L1087" s="31" t="n">
         <v>0</v>
@@ -55669,26 +55669,26 @@
         </is>
       </c>
       <c r="D1088" s="9" t="n">
-        <v>142469.97</v>
+        <v>227750.23</v>
       </c>
       <c r="E1088" s="9" t="n">
-        <v>260570.96</v>
+        <v>807563.36</v>
       </c>
       <c r="F1088" s="10" t="n">
-        <v>0.262</v>
+        <v>0.3087</v>
       </c>
       <c r="G1088" s="10" t="n">
-        <v>0.2041</v>
+        <v>0.2451</v>
       </c>
       <c r="H1088" s="10" t="n"/>
       <c r="I1088" s="10" t="n">
-        <v>0.0484</v>
+        <v>0.0598</v>
       </c>
       <c r="J1088" s="13" t="n">
-        <v>5599</v>
+        <v>8785</v>
       </c>
       <c r="K1088" s="13" t="n">
-        <v>8045</v>
+        <v>13111</v>
       </c>
       <c r="L1088" s="32" t="n">
         <v>0</v>
@@ -55711,26 +55711,26 @@
         </is>
       </c>
       <c r="D1089" s="15" t="n">
-        <v>117737.67</v>
+        <v>155420.57</v>
       </c>
       <c r="E1089" s="15" t="n">
-        <v>575394.91</v>
+        <v>2615297.18</v>
       </c>
       <c r="F1089" s="16" t="n">
-        <v>0.7305</v>
+        <v>0.7308</v>
       </c>
       <c r="G1089" s="16" t="n">
-        <v>0.6659</v>
+        <v>0.6642</v>
       </c>
       <c r="H1089" s="16" t="n"/>
       <c r="I1089" s="16" t="n">
-        <v>0.024</v>
+        <v>0.0295</v>
       </c>
       <c r="J1089" s="19" t="n">
-        <v>5132</v>
+        <v>7659</v>
       </c>
       <c r="K1089" s="19" t="n">
-        <v>20039</v>
+        <v>24967</v>
       </c>
       <c r="L1089" s="31" t="n">
         <v>0</v>
@@ -56215,13 +56215,13 @@
         </is>
       </c>
       <c r="D1101" s="15" t="n">
-        <v>151932450.44</v>
+        <v>151943202.19</v>
       </c>
       <c r="E1101" s="15" t="n">
-        <v>606872937.3099999</v>
+        <v>606885933.46</v>
       </c>
       <c r="F1101" s="16" t="n">
-        <v>0.0762</v>
+        <v>0.07630000000000001</v>
       </c>
       <c r="G1101" s="16" t="n">
         <v>0.018</v>
@@ -56231,10 +56231,10 @@
         <v>0.1029</v>
       </c>
       <c r="J1101" s="19" t="n">
-        <v>3671001</v>
+        <v>3671150</v>
       </c>
       <c r="K1101" s="19" t="n">
-        <v>7097111</v>
+        <v>7097443</v>
       </c>
       <c r="L1101" s="31" t="n">
         <v>0</v>
@@ -56257,26 +56257,26 @@
         </is>
       </c>
       <c r="D1102" s="9" t="n">
-        <v>43726865.08</v>
+        <v>74236517.09999999</v>
       </c>
       <c r="E1102" s="9" t="n">
-        <v>198541152.32</v>
+        <v>334462876.84</v>
       </c>
       <c r="F1102" s="10" t="n">
-        <v>0.2122</v>
+        <v>0.1713</v>
       </c>
       <c r="G1102" s="10" t="n">
-        <v>0.1538</v>
+        <v>0.1128</v>
       </c>
       <c r="H1102" s="10" t="n"/>
       <c r="I1102" s="10" t="n">
-        <v>0.0872</v>
+        <v>0.0968</v>
       </c>
       <c r="J1102" s="13" t="n">
-        <v>1144021</v>
+        <v>1810079</v>
       </c>
       <c r="K1102" s="13" t="n">
-        <v>2251660</v>
+        <v>3633079</v>
       </c>
       <c r="L1102" s="32" t="n">
         <v>0</v>
@@ -59533,10 +59533,10 @@
         </is>
       </c>
       <c r="D1180" s="9" t="n">
-        <v>17527780.03</v>
+        <v>17527781.9</v>
       </c>
       <c r="E1180" s="9" t="n">
-        <v>296133942.32</v>
+        <v>296133965.96</v>
       </c>
       <c r="F1180" s="10" t="n">
         <v>0.3868</v>
@@ -59549,10 +59549,10 @@
         <v>0.0298</v>
       </c>
       <c r="J1180" s="13" t="n">
-        <v>1340854</v>
+        <v>1340855</v>
       </c>
       <c r="K1180" s="13" t="n">
-        <v>2084261</v>
+        <v>2084263</v>
       </c>
       <c r="L1180" s="32" t="n">
         <v>0</v>
@@ -59575,26 +59575,26 @@
         </is>
       </c>
       <c r="D1181" s="15" t="n">
-        <v>40919055.23</v>
+        <v>40928654.79</v>
       </c>
       <c r="E1181" s="15" t="n">
-        <v>20758772.01</v>
+        <v>20763452.89</v>
       </c>
       <c r="F1181" s="16" t="n">
         <v>0.0026</v>
       </c>
       <c r="G1181" s="16" t="n">
-        <v>-0.039</v>
+        <v>-0.0389</v>
       </c>
       <c r="H1181" s="16" t="n"/>
       <c r="I1181" s="16" t="n">
         <v>0.3061</v>
       </c>
       <c r="J1181" s="19" t="n">
-        <v>179969</v>
+        <v>180075</v>
       </c>
       <c r="K1181" s="19" t="n">
-        <v>776573</v>
+        <v>776825</v>
       </c>
       <c r="L1181" s="31" t="n">
         <v>0</v>
@@ -59617,26 +59617,26 @@
         </is>
       </c>
       <c r="D1182" s="9" t="n">
-        <v>26404603.36</v>
+        <v>26405659.51</v>
       </c>
       <c r="E1182" s="9" t="n">
-        <v>26088317.89</v>
+        <v>26088934.78</v>
       </c>
       <c r="F1182" s="10" t="n">
         <v>0.0262</v>
       </c>
       <c r="G1182" s="10" t="n">
-        <v>-0.0247</v>
+        <v>-0.0246</v>
       </c>
       <c r="H1182" s="10" t="n"/>
       <c r="I1182" s="10" t="n">
         <v>0.2383</v>
       </c>
       <c r="J1182" s="13" t="n">
-        <v>266468</v>
+        <v>266496</v>
       </c>
       <c r="K1182" s="13" t="n">
-        <v>714370</v>
+        <v>714422</v>
       </c>
       <c r="L1182" s="32" t="n">
         <v>0</v>
@@ -59659,7 +59659,7 @@
         </is>
       </c>
       <c r="D1183" s="15" t="n">
-        <v>19480688.72</v>
+        <v>19480757.02</v>
       </c>
       <c r="E1183" s="15" t="n">
         <v>31181555.27</v>
@@ -59675,10 +59675,10 @@
         <v>0.1908</v>
       </c>
       <c r="J1183" s="19" t="n">
-        <v>307053</v>
+        <v>307055</v>
       </c>
       <c r="K1183" s="19" t="n">
-        <v>661656</v>
+        <v>661659</v>
       </c>
       <c r="L1183" s="31" t="n">
         <v>0</v>
@@ -59701,10 +59701,10 @@
         </is>
       </c>
       <c r="D1184" s="9" t="n">
-        <v>14023253.68</v>
+        <v>14023258.4</v>
       </c>
       <c r="E1184" s="9" t="n">
-        <v>33857622.22</v>
+        <v>33857654.51</v>
       </c>
       <c r="F1184" s="10" t="n">
         <v>0.0392</v>
@@ -59717,10 +59717,10 @@
         <v>0.1539</v>
       </c>
       <c r="J1184" s="13" t="n">
-        <v>301282</v>
+        <v>301286</v>
       </c>
       <c r="K1184" s="13" t="n">
-        <v>581810</v>
+        <v>581814</v>
       </c>
       <c r="L1184" s="32" t="n">
         <v>0</v>
@@ -59743,26 +59743,26 @@
         </is>
       </c>
       <c r="D1185" s="15" t="n">
-        <v>17993532.2</v>
+        <v>17993544.42</v>
       </c>
       <c r="E1185" s="15" t="n">
-        <v>75325795.97</v>
+        <v>75332498.70999999</v>
       </c>
       <c r="F1185" s="16" t="n">
-        <v>0.0582</v>
+        <v>0.0586</v>
       </c>
       <c r="G1185" s="16" t="n">
-        <v>-0.011</v>
+        <v>-0.0106</v>
       </c>
       <c r="H1185" s="16" t="n"/>
       <c r="I1185" s="16" t="n">
         <v>0.1144</v>
       </c>
       <c r="J1185" s="19" t="n">
-        <v>570400</v>
+        <v>570403</v>
       </c>
       <c r="K1185" s="19" t="n">
-        <v>1005326</v>
+        <v>1005335</v>
       </c>
       <c r="L1185" s="31" t="n">
         <v>0</v>
@@ -59785,10 +59785,10 @@
         </is>
       </c>
       <c r="D1186" s="9" t="n">
-        <v>15583537.22</v>
+        <v>15583546.15</v>
       </c>
       <c r="E1186" s="9" t="n">
-        <v>123526931.63</v>
+        <v>123527871.35</v>
       </c>
       <c r="F1186" s="10" t="n">
         <v>0.1212</v>
@@ -59801,10 +59801,10 @@
         <v>0.0694</v>
       </c>
       <c r="J1186" s="13" t="n">
-        <v>704975</v>
+        <v>704980</v>
       </c>
       <c r="K1186" s="13" t="n">
-        <v>1273115</v>
+        <v>1273125</v>
       </c>
       <c r="L1186" s="32" t="n">
         <v>0</v>
@@ -59827,26 +59827,26 @@
         </is>
       </c>
       <c r="D1187" s="15" t="n">
-        <v>6620353.75</v>
+        <v>10429384.86</v>
       </c>
       <c r="E1187" s="15" t="n">
-        <v>116963099.56</v>
+        <v>182922141.45</v>
       </c>
       <c r="F1187" s="16" t="n">
-        <v>0.5511</v>
+        <v>0.4665</v>
       </c>
       <c r="G1187" s="16" t="n">
-        <v>0.4717</v>
+        <v>0.3874</v>
       </c>
       <c r="H1187" s="16" t="n"/>
       <c r="I1187" s="16" t="n">
-        <v>0.0221</v>
+        <v>0.0273</v>
       </c>
       <c r="J1187" s="19" t="n">
-        <v>491041</v>
+        <v>736977</v>
       </c>
       <c r="K1187" s="19" t="n">
-        <v>822895</v>
+        <v>1220851</v>
       </c>
       <c r="L1187" s="31" t="n">
         <v>0</v>
@@ -59869,26 +59869,26 @@
         </is>
       </c>
       <c r="D1188" s="9" t="n">
-        <v>10479063.64</v>
+        <v>17321110.88</v>
       </c>
       <c r="E1188" s="9" t="n">
-        <v>5392763.97</v>
+        <v>8787233.859999999</v>
       </c>
       <c r="F1188" s="10" t="n">
-        <v>0.09429999999999999</v>
+        <v>0.0488</v>
       </c>
       <c r="G1188" s="10" t="n">
-        <v>0.0539</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="H1188" s="10" t="n"/>
       <c r="I1188" s="10" t="n">
-        <v>0.3071</v>
+        <v>0.3124</v>
       </c>
       <c r="J1188" s="13" t="n">
-        <v>48047</v>
+        <v>78658</v>
       </c>
       <c r="K1188" s="13" t="n">
-        <v>192701</v>
+        <v>317790</v>
       </c>
       <c r="L1188" s="32" t="n">
         <v>0</v>
@@ -59911,26 +59911,26 @@
         </is>
       </c>
       <c r="D1189" s="15" t="n">
-        <v>6715174.79</v>
+        <v>11335832.97</v>
       </c>
       <c r="E1189" s="15" t="n">
-        <v>6218363.71</v>
+        <v>11018336.63</v>
       </c>
       <c r="F1189" s="16" t="n">
-        <v>0.06909999999999999</v>
+        <v>0.022</v>
       </c>
       <c r="G1189" s="16" t="n">
-        <v>0.0195</v>
+        <v>-0.0282</v>
       </c>
       <c r="H1189" s="16" t="n"/>
       <c r="I1189" s="16" t="n">
-        <v>0.2333</v>
+        <v>0.2467</v>
       </c>
       <c r="J1189" s="19" t="n">
-        <v>69071</v>
+        <v>113869</v>
       </c>
       <c r="K1189" s="19" t="n">
-        <v>172679</v>
+        <v>286932</v>
       </c>
       <c r="L1189" s="31" t="n">
         <v>0</v>
@@ -59953,26 +59953,26 @@
         </is>
       </c>
       <c r="D1190" s="9" t="n">
-        <v>5444561.22</v>
+        <v>9502769.300000001</v>
       </c>
       <c r="E1190" s="9" t="n">
-        <v>7488148.39</v>
+        <v>13573874.66</v>
       </c>
       <c r="F1190" s="10" t="n">
-        <v>0.1132</v>
+        <v>0.09379999999999999</v>
       </c>
       <c r="G1190" s="10" t="n">
-        <v>0.0594</v>
+        <v>0.0394</v>
       </c>
       <c r="H1190" s="10" t="n"/>
       <c r="I1190" s="10" t="n">
-        <v>0.187</v>
+        <v>0.2013</v>
       </c>
       <c r="J1190" s="13" t="n">
-        <v>80938</v>
+        <v>132657</v>
       </c>
       <c r="K1190" s="13" t="n">
-        <v>174970</v>
+        <v>296106</v>
       </c>
       <c r="L1190" s="32" t="n">
         <v>0</v>
@@ -59995,26 +59995,26 @@
         </is>
       </c>
       <c r="D1191" s="15" t="n">
-        <v>3634193.55</v>
+        <v>6487649.5</v>
       </c>
       <c r="E1191" s="15" t="n">
-        <v>7810635.94</v>
+        <v>13719664.03</v>
       </c>
       <c r="F1191" s="16" t="n">
-        <v>0.1073</v>
+        <v>0.0979</v>
       </c>
       <c r="G1191" s="16" t="n">
-        <v>0.0449</v>
+        <v>0.0358</v>
       </c>
       <c r="H1191" s="16" t="n"/>
       <c r="I1191" s="16" t="n">
-        <v>0.1527</v>
+        <v>0.1646</v>
       </c>
       <c r="J1191" s="19" t="n">
-        <v>78854</v>
+        <v>129319</v>
       </c>
       <c r="K1191" s="19" t="n">
-        <v>152189</v>
+        <v>260750</v>
       </c>
       <c r="L1191" s="31" t="n">
         <v>0</v>
@@ -60037,26 +60037,26 @@
         </is>
       </c>
       <c r="D1192" s="9" t="n">
-        <v>5490548.72</v>
+        <v>10010303.1</v>
       </c>
       <c r="E1192" s="9" t="n">
-        <v>19558022.4</v>
+        <v>35798453.17</v>
       </c>
       <c r="F1192" s="10" t="n">
-        <v>0.1786</v>
+        <v>0.1718</v>
       </c>
       <c r="G1192" s="10" t="n">
-        <v>0.1124</v>
+        <v>0.1054</v>
       </c>
       <c r="H1192" s="10" t="n"/>
       <c r="I1192" s="10" t="n">
-        <v>0.1101</v>
+        <v>0.1182</v>
       </c>
       <c r="J1192" s="13" t="n">
-        <v>158776</v>
+        <v>261795</v>
       </c>
       <c r="K1192" s="13" t="n">
-        <v>303782</v>
+        <v>527524</v>
       </c>
       <c r="L1192" s="32" t="n">
         <v>0</v>
@@ -60079,26 +60079,26 @@
         </is>
       </c>
       <c r="D1193" s="15" t="n">
-        <v>5342969.41</v>
+        <v>9149466.51</v>
       </c>
       <c r="E1193" s="15" t="n">
-        <v>35110118.35</v>
+        <v>68643173.05</v>
       </c>
       <c r="F1193" s="16" t="n">
-        <v>0.4102</v>
+        <v>0.3835</v>
       </c>
       <c r="G1193" s="16" t="n">
-        <v>0.3379</v>
+        <v>0.3108</v>
       </c>
       <c r="H1193" s="16" t="n"/>
       <c r="I1193" s="16" t="n">
-        <v>0.0615</v>
+        <v>0.0659</v>
       </c>
       <c r="J1193" s="19" t="n">
-        <v>217294</v>
+        <v>356804</v>
       </c>
       <c r="K1193" s="19" t="n">
-        <v>432444</v>
+        <v>723126</v>
       </c>
       <c r="L1193" s="31" t="n">
         <v>0</v>
@@ -60583,26 +60583,26 @@
         </is>
       </c>
       <c r="D1205" s="15" t="n">
-        <v>1494928.17</v>
+        <v>2984297</v>
       </c>
       <c r="E1205" s="15" t="n">
-        <v>1312927.84</v>
+        <v>7942844.01</v>
       </c>
       <c r="F1205" s="16" t="n">
-        <v>0.5211</v>
+        <v>0.2728</v>
       </c>
       <c r="G1205" s="16" t="n">
-        <v>0.4655</v>
+        <v>0.2133</v>
       </c>
       <c r="H1205" s="16" t="n"/>
       <c r="I1205" s="16" t="n">
-        <v>0.0378</v>
+        <v>0.0834</v>
       </c>
       <c r="J1205" s="19" t="n">
-        <v>25015</v>
+        <v>51820</v>
       </c>
       <c r="K1205" s="19" t="n">
-        <v>34242</v>
+        <v>75580</v>
       </c>
       <c r="L1205" s="31" t="n">
         <v>0</v>
@@ -63859,26 +63859,26 @@
         </is>
       </c>
       <c r="D1283" s="15" t="n">
-        <v>91660.8</v>
+        <v>165373.44</v>
       </c>
       <c r="E1283" s="15" t="n">
-        <v>377220.94</v>
+        <v>2095456.54</v>
       </c>
       <c r="F1283" s="16" t="n">
-        <v>0.4359</v>
+        <v>0.4392</v>
       </c>
       <c r="G1283" s="16" t="n">
-        <v>0.3712</v>
+        <v>0.3747</v>
       </c>
       <c r="H1283" s="16" t="n"/>
       <c r="I1283" s="16" t="n">
-        <v>0.0057</v>
+        <v>0.0189</v>
       </c>
       <c r="J1283" s="19" t="n">
-        <v>6148</v>
+        <v>11534</v>
       </c>
       <c r="K1283" s="19" t="n">
-        <v>7696</v>
+        <v>14314</v>
       </c>
       <c r="L1283" s="31" t="n">
         <v>0</v>
@@ -63901,26 +63901,26 @@
         </is>
       </c>
       <c r="D1284" s="9" t="n">
-        <v>375267.55</v>
+        <v>840038.26</v>
       </c>
       <c r="E1284" s="9" t="n">
-        <v>77652.03999999999</v>
+        <v>542849.8199999999</v>
       </c>
       <c r="F1284" s="10" t="n">
-        <v>0.5082</v>
+        <v>0.2094</v>
       </c>
       <c r="G1284" s="10" t="n">
-        <v>0.4583</v>
+        <v>0.156</v>
       </c>
       <c r="H1284" s="10" t="n"/>
       <c r="I1284" s="10" t="n">
-        <v>0.2109</v>
+        <v>0.2869</v>
       </c>
       <c r="J1284" s="13" t="n">
-        <v>1380</v>
+        <v>3290</v>
       </c>
       <c r="K1284" s="13" t="n">
-        <v>3053</v>
+        <v>8299</v>
       </c>
       <c r="L1284" s="32" t="n">
         <v>0</v>
@@ -63943,26 +63943,26 @@
         </is>
       </c>
       <c r="D1285" s="15" t="n">
-        <v>402150</v>
+        <v>723977.65</v>
       </c>
       <c r="E1285" s="15" t="n">
-        <v>56647.05</v>
+        <v>548879.08</v>
       </c>
       <c r="F1285" s="16" t="n">
-        <v>0.1826</v>
+        <v>0.122</v>
       </c>
       <c r="G1285" s="16" t="n">
-        <v>0.1296</v>
+        <v>0.06560000000000001</v>
       </c>
       <c r="H1285" s="16" t="n"/>
       <c r="I1285" s="16" t="n">
-        <v>0.104</v>
+        <v>0.1853</v>
       </c>
       <c r="J1285" s="19" t="n">
-        <v>2626</v>
+        <v>5851</v>
       </c>
       <c r="K1285" s="19" t="n">
-        <v>4056</v>
+        <v>10002</v>
       </c>
       <c r="L1285" s="31" t="n">
         <v>0</v>
@@ -63985,26 +63985,26 @@
         </is>
       </c>
       <c r="D1286" s="9" t="n">
-        <v>232991.87</v>
+        <v>476299.71</v>
       </c>
       <c r="E1286" s="9" t="n">
-        <v>113587.59</v>
+        <v>698966.0600000001</v>
       </c>
       <c r="F1286" s="10" t="n">
-        <v>0.6991000000000001</v>
+        <v>0.2752</v>
       </c>
       <c r="G1286" s="10" t="n">
-        <v>0.644</v>
+        <v>0.2143</v>
       </c>
       <c r="H1286" s="10" t="n"/>
       <c r="I1286" s="10" t="n">
-        <v>0.0536</v>
+        <v>0.1217</v>
       </c>
       <c r="J1286" s="13" t="n">
-        <v>3133</v>
+        <v>6699</v>
       </c>
       <c r="K1286" s="13" t="n">
-        <v>4397</v>
+        <v>10317</v>
       </c>
       <c r="L1286" s="32" t="n">
         <v>0</v>
@@ -64027,26 +64027,26 @@
         </is>
       </c>
       <c r="D1287" s="15" t="n">
-        <v>155344.25</v>
+        <v>313742.91</v>
       </c>
       <c r="E1287" s="15" t="n">
-        <v>197885.13</v>
+        <v>887407.13</v>
       </c>
       <c r="F1287" s="16" t="n">
-        <v>0.6581</v>
+        <v>0.4036</v>
       </c>
       <c r="G1287" s="16" t="n">
-        <v>0.5987</v>
+        <v>0.3392</v>
       </c>
       <c r="H1287" s="16" t="n"/>
       <c r="I1287" s="16" t="n">
-        <v>0.0268</v>
+        <v>0.0814</v>
       </c>
       <c r="J1287" s="19" t="n">
-        <v>2838</v>
+        <v>6022</v>
       </c>
       <c r="K1287" s="19" t="n">
-        <v>4166</v>
+        <v>9257</v>
       </c>
       <c r="L1287" s="31" t="n">
         <v>0</v>
@@ -64069,26 +64069,26 @@
         </is>
       </c>
       <c r="D1288" s="9" t="n">
-        <v>156380.54</v>
+        <v>285126.79</v>
       </c>
       <c r="E1288" s="9" t="n">
-        <v>363073.33</v>
+        <v>1368909.74</v>
       </c>
       <c r="F1288" s="10" t="n">
-        <v>0.8548</v>
+        <v>0.4798</v>
       </c>
       <c r="G1288" s="10" t="n">
-        <v>0.7919</v>
+        <v>0.4102</v>
       </c>
       <c r="H1288" s="10" t="n"/>
       <c r="I1288" s="10" t="n">
-        <v>0.0152</v>
+        <v>0.0523</v>
       </c>
       <c r="J1288" s="13" t="n">
-        <v>4808</v>
+        <v>9830</v>
       </c>
       <c r="K1288" s="13" t="n">
-        <v>6121</v>
+        <v>12678</v>
       </c>
       <c r="L1288" s="32" t="n">
         <v>0</v>
@@ -64111,26 +64111,26 @@
         </is>
       </c>
       <c r="D1289" s="15" t="n">
-        <v>81133.17</v>
+        <v>179738.23</v>
       </c>
       <c r="E1289" s="15" t="n">
-        <v>126861.76</v>
+        <v>1800375.63</v>
       </c>
       <c r="F1289" s="16" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.4596</v>
       </c>
       <c r="G1289" s="16" t="n">
-        <v>0.8736</v>
+        <v>0.3926</v>
       </c>
       <c r="H1289" s="16" t="n"/>
       <c r="I1289" s="16" t="n">
-        <v>0.0073</v>
+        <v>0.0299</v>
       </c>
       <c r="J1289" s="19" t="n">
-        <v>4082</v>
+        <v>8594</v>
       </c>
       <c r="K1289" s="19" t="n">
-        <v>4753</v>
+        <v>10713</v>
       </c>
       <c r="L1289" s="31" t="n">
         <v>0</v>
@@ -64950,7 +64950,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-21 16:34 UTC</t>
+          <t>2026-10-22 16:31 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-23 16:21 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -1679,7 +1679,7 @@
         <v>21766760.99</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1234384.02</v>
+        <v>1234384.01</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>0.05671</v>
@@ -1692,7 +1692,7 @@
         <v>21766760.99</v>
       </c>
       <c r="J9" s="15" t="n">
-        <v>1234384.02</v>
+        <v>1234384.01</v>
       </c>
       <c r="K9" s="18" t="n"/>
       <c r="L9" s="19" t="n">
@@ -2892,7 +2892,7 @@
         </is>
       </c>
       <c r="I26" s="9" t="n">
-        <v>499580423.51</v>
+        <v>499580423.5</v>
       </c>
       <c r="J26" s="9" t="n">
         <v>6582164.99</v>
@@ -3049,7 +3049,7 @@
         <v>691271126.84</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>44338006.62</v>
+        <v>44338006.61</v>
       </c>
       <c r="K28" s="12" t="n">
         <v>0.06414</v>
@@ -5933,22 +5933,22 @@
         <v>46320</v>
       </c>
       <c r="B70" s="9" t="n">
-        <v>230834189.48</v>
+        <v>335232092.44</v>
       </c>
       <c r="C70" s="9" t="n">
-        <v>9891551.23</v>
+        <v>14588409.01</v>
       </c>
       <c r="D70" s="10" t="n">
-        <v>0.04285</v>
+        <v>0.04352</v>
       </c>
       <c r="E70" s="9" t="n">
-        <v>67747126.03</v>
+        <v>98163244.3</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>14711168.37</v>
+        <v>16162082.18</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>0.21715</v>
+        <v>0.16464</v>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
@@ -5956,31 +5956,31 @@
         </is>
       </c>
       <c r="I70" s="9" t="n">
-        <v>298581315.51</v>
+        <v>433395336.74</v>
       </c>
       <c r="J70" s="9" t="n">
-        <v>24602719.6</v>
+        <v>30750491.19</v>
       </c>
       <c r="K70" s="12" t="n">
-        <v>0.0824</v>
+        <v>0.07095</v>
       </c>
       <c r="L70" s="13" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="M70" s="13" t="n">
-        <v>-374</v>
+        <v>-5</v>
       </c>
       <c r="N70" s="9" t="n">
-        <v>64762756.4</v>
+        <v>114230395.94</v>
       </c>
       <c r="O70" s="10" t="n">
-        <v>0.05704</v>
+        <v>0.08209</v>
       </c>
       <c r="P70" s="9" t="n">
-        <v>113298952.38</v>
+        <v>144714656.37</v>
       </c>
       <c r="Q70" s="10" t="n">
-        <v>0.04748</v>
+        <v>0.02468</v>
       </c>
       <c r="R70" s="9" t="n">
         <v>9057675.779999999</v>
@@ -5989,16 +5989,16 @@
         <v>-0.06547</v>
       </c>
       <c r="T70" s="9" t="n">
-        <v>15967573.79</v>
+        <v>24765380.95</v>
       </c>
       <c r="U70" s="10" t="n">
-        <v>0.07665</v>
+        <v>0.05437</v>
       </c>
       <c r="V70" s="9" t="n">
-        <v>27747231.13</v>
+        <v>42463983.39</v>
       </c>
       <c r="W70" s="10" t="n">
-        <v>0.00676</v>
+        <v>0.02087</v>
       </c>
       <c r="X70" s="9" t="n"/>
       <c r="Y70" s="10" t="n"/>
@@ -7392,22 +7392,22 @@
         <v>46296</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>2509809609.62</v>
+        <v>2614207512.58</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>52850942.34</v>
+        <v>57547800.12</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.02106</v>
+        <v>0.02201</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>694672460.79</v>
+        <v>725233243.29</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>131605821.07</v>
+        <v>133204891.18</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.18945</v>
+        <v>0.18367</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
@@ -7415,31 +7415,31 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>3204482070.41</v>
+        <v>3339440755.87</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>184456763.41</v>
+        <v>190752691.31</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.05756</v>
+        <v>0.05712</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>662</v>
+        <v>680</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="N20" s="9" t="n">
-        <v>1072027977.53</v>
+        <v>1121495617.07</v>
       </c>
       <c r="O20" s="10" t="n">
-        <v>0.01175</v>
+        <v>0.0163</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>204013836.52</v>
+        <v>235429540.52</v>
       </c>
       <c r="Q20" s="10" t="n">
-        <v>0.04131</v>
+        <v>0.02812</v>
       </c>
       <c r="R20" s="9" t="n">
         <v>298312041.27</v>
@@ -7448,16 +7448,16 @@
         <v>0.04584</v>
       </c>
       <c r="T20" s="9" t="n">
-        <v>100902792.28</v>
+        <v>109700599.44</v>
       </c>
       <c r="U20" s="10" t="n">
-        <v>0.02937</v>
+        <v>0.02814</v>
       </c>
       <c r="V20" s="9" t="n">
-        <v>834552962.02</v>
+        <v>849269714.28</v>
       </c>
       <c r="W20" s="10" t="n">
-        <v>0.0182</v>
+        <v>0.01871</v>
       </c>
       <c r="X20" s="9" t="n"/>
       <c r="Y20" s="10" t="n"/>
@@ -7984,22 +7984,22 @@
         <v>-0.0249</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>64762756.41</v>
+        <v>114230395.95</v>
       </c>
       <c r="I11" s="16" t="n">
-        <v>0.057</v>
+        <v>0.08210000000000001</v>
       </c>
       <c r="J11" s="19" t="n">
-        <v>178</v>
+        <v>631</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>8.6</v>
+        <v>3.4</v>
       </c>
       <c r="L11" s="15" t="n">
-        <v>27876873.41</v>
+        <v>35584131.75</v>
       </c>
       <c r="M11" s="16" t="n">
-        <v>0.3732</v>
+        <v>0.2263</v>
       </c>
     </row>
     <row r="12">
@@ -8558,14 +8558,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-22 16:31 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-23 16:21 UTC.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>Season 2026 to date  ·  93 games</t>
+          <t>Season 2026 to date  ·  94 games</t>
         </is>
       </c>
     </row>
@@ -8628,31 +8628,31 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>1073039036.780001</v>
+        <v>1094486670.650001</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.02289108361212028</v>
+        <v>0.02639592486114302</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>-0.002015418149641269</v>
+        <v>0.001453189228019952</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0.04570345615853073</v>
+        <v>0.04955673129564912</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>0.006659456887698806</v>
+        <v>0.006749446889558886</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>390.4399927083192</v>
+        <v>428.0728440609023</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>-0.01221988262968555</v>
+        <v>-0.008887055809646919</v>
       </c>
       <c r="I6" s="29" t="n">
-        <v>-6.215836630760569</v>
+        <v>-6.11880545588273</v>
       </c>
       <c r="J6" s="15" t="n">
-        <v>33407060.86</v>
+        <v>34124364.63999999</v>
       </c>
     </row>
     <row r="7">
@@ -8662,31 +8662,31 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>298754195.3900002</v>
+        <v>304912384.6100002</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.06772996316783206</v>
+        <v>0.0651479548310499</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>0.03853673945890759</v>
+        <v>0.03595118995911224</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.09744475751780644</v>
+        <v>0.08985606126429682</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.001716904371627406</v>
+        <v>0.001825606710714355</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>957.2785314617904</v>
+        <v>880.3045455358247</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>0.0005301349576246206</v>
+        <v>0.0009134536781841853</v>
       </c>
       <c r="I7" s="30" t="n">
-        <v>-10.51944869527048</v>
+        <v>-9.453304968098424</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>10901997.57</v>
+        <v>11128069</v>
       </c>
     </row>
     <row r="8">
@@ -8696,31 +8696,31 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>154819897.07</v>
+        <v>162423843.45</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.005852962617526463</v>
+        <v>0.01213908695989551</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>-0.02224932980314891</v>
+        <v>-0.01556039720718724</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>-0.07964040745649988</v>
+        <v>-0.05680795482964646</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>-0.009899265698560002</v>
+        <v>-0.009343761331756351</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>-697.4114175793987</v>
+        <v>-474.6419349789011</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>0.004922796293828473</v>
+        <v>0.004044327699925969</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>5.826351558889748</v>
+        <v>4.036919181212047</v>
       </c>
       <c r="J8" s="15" t="n">
-        <v>5438492.560000002</v>
+        <v>5623820.890000002</v>
       </c>
     </row>
     <row r="9">
@@ -8730,31 +8730,31 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>285472746.82</v>
+        <v>295974023.85</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>-0.002511828389881752</v>
+        <v>-0.001470542192650604</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>-0.02704149967375861</v>
+        <v>-0.02577057172377259</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>-0.03707478172878582</v>
+        <v>-0.03478429504223865</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>-0.008822196858139382</v>
+        <v>-0.00871848457142016</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-282.5258487064644</v>
+        <v>-260.6581047081849</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-0.01993172804217448</v>
+        <v>-0.01950377115797173</v>
       </c>
       <c r="I9" s="30" t="n">
-        <v>1.636968672735572</v>
+        <v>1.656232582738445</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>7138556.300000002</v>
+        <v>7335037.760000002</v>
       </c>
     </row>
     <row r="10">
@@ -8764,31 +8764,31 @@
         </is>
       </c>
       <c r="B10" s="15" t="n">
-        <v>128321989.42</v>
+        <v>131157655.96</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>0.05064766848905357</v>
+        <v>0.05187481371331455</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>0.02673165632409816</v>
+        <v>0.02796520594359058</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>0.05609811746594821</v>
+        <v>0.0579103549052363</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>0.007368308141252288</v>
+        <v>0.007446872488217138</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>487.2980932469592</v>
+        <v>504.6348241701916</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>0.0178715612929296</v>
+        <v>0.0189215400014692</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>-3.720285644534563</v>
+        <v>-3.786675211426286</v>
       </c>
       <c r="J10" s="15" t="n">
-        <v>3068950.259999999</v>
+        <v>3135928.109999998</v>
       </c>
     </row>
     <row r="11">
@@ -8798,31 +8798,31 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>32104762.19000001</v>
+        <v>33025688.69000001</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.004140767628592104</v>
+        <v>0.006287045879617653</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>-0.01793505575877932</v>
+        <v>-0.01575331539286063</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0.03877010443479054</v>
+        <v>0.04185210604019338</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.003485053525472333</v>
+        <v>0.003503934173786229</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>352.8505090931821</v>
+        <v>383.4817186640715</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-0.03592638718647231</v>
+        <v>-0.03419908744734319</v>
       </c>
       <c r="I11" s="30" t="n">
-        <v>-3.610377138754659</v>
+        <v>-3.51805540179019</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>708739.0599999999</v>
+        <v>727898.11</v>
       </c>
     </row>
     <row r="12">
@@ -8832,31 +8832,31 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>1972512627.669998</v>
+        <v>2021980267.209998</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>0.02616910061608782</v>
+        <v>0.0283396702575479</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>0.0005275498394295148</v>
+        <v>0.002742483114165862</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>0.02671544928668358</v>
+        <v>0.02907683462791388</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>0.0003305688781501375</v>
+        <v>0.0004443182116283221</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>263.8488040853345</v>
+        <v>286.3251641628556</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>-0.008648507576792896</v>
+        <v>-0.006514635616847445</v>
       </c>
       <c r="I12" s="29" t="n">
-        <v>-3.75530687523528</v>
+        <v>-3.690635906225312</v>
       </c>
       <c r="J12" s="15" t="n">
-        <v>60663796.60999995</v>
+        <v>62075118.50999995</v>
       </c>
     </row>
     <row r="14">
@@ -9236,11 +9236,11 @@
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>W06 (Mon)</t>
+          <t>W06 (Mon) + W07 (Thu)</t>
         </is>
       </c>
       <c r="D26" s="19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
@@ -9248,25 +9248,25 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>64762756.41</v>
+        <v>114230395.95</v>
       </c>
       <c r="G26" s="16" t="n">
-        <v>0.057</v>
+        <v>0.08210000000000001</v>
       </c>
       <c r="H26" s="16" t="n">
-        <v>0.0364</v>
+        <v>0.0601</v>
       </c>
       <c r="I26" s="15" t="n">
-        <v>-2359737.5</v>
+        <v>-6864385.52</v>
       </c>
       <c r="J26" s="15" t="n">
-        <v>14687145.08</v>
+        <v>28774143.02</v>
       </c>
       <c r="K26" s="16" t="n">
-        <v>0.0193</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="L26" s="16" t="n">
-        <v>0.0015</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="27">
@@ -10093,26 +10093,26 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>2062239.18</v>
+        <v>2601249.42</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>6132442.66</v>
+        <v>8123757</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.3085</v>
+        <v>0.2702</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.2491</v>
+        <v>0.2114</v>
       </c>
       <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n">
-        <v>0.0891</v>
+        <v>0.09710000000000001</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>41361</v>
+        <v>53647</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>63489</v>
+        <v>84735</v>
       </c>
       <c r="L14" s="32" t="n">
         <v>0</v>
@@ -12781,26 +12781,26 @@
         </is>
       </c>
       <c r="D78" s="9" t="n">
-        <v>119345.55</v>
+        <v>177021.41</v>
       </c>
       <c r="E78" s="9" t="n">
-        <v>2728144.04</v>
+        <v>3346744.33</v>
       </c>
       <c r="F78" s="10" t="n">
-        <v>0.5097</v>
+        <v>0.5244</v>
       </c>
       <c r="G78" s="10" t="n">
-        <v>0.4406</v>
+        <v>0.4523</v>
       </c>
       <c r="H78" s="10" t="n"/>
       <c r="I78" s="10" t="n">
-        <v>0.0278</v>
+        <v>0.032</v>
       </c>
       <c r="J78" s="13" t="n">
-        <v>9284</v>
+        <v>12922</v>
       </c>
       <c r="K78" s="13" t="n">
-        <v>14897</v>
+        <v>23482</v>
       </c>
       <c r="L78" s="32" t="n">
         <v>0</v>
@@ -12823,26 +12823,26 @@
         </is>
       </c>
       <c r="D79" s="15" t="n">
-        <v>553792.55</v>
+        <v>662404.51</v>
       </c>
       <c r="E79" s="15" t="n">
-        <v>390392.73</v>
+        <v>513155.23</v>
       </c>
       <c r="F79" s="16" t="n">
-        <v>0.1723</v>
+        <v>0.1484</v>
       </c>
       <c r="G79" s="16" t="n">
-        <v>0.1219</v>
+        <v>0.0983</v>
       </c>
       <c r="H79" s="16" t="n"/>
       <c r="I79" s="16" t="n">
-        <v>0.3044</v>
+        <v>0.3092</v>
       </c>
       <c r="J79" s="19" t="n">
-        <v>2618</v>
+        <v>3338</v>
       </c>
       <c r="K79" s="19" t="n">
-        <v>7043</v>
+        <v>8496</v>
       </c>
       <c r="L79" s="31" t="n">
         <v>0</v>
@@ -12865,26 +12865,26 @@
         </is>
       </c>
       <c r="D80" s="9" t="n">
-        <v>510902.65</v>
+        <v>655687.21</v>
       </c>
       <c r="E80" s="9" t="n">
-        <v>508884.73</v>
+        <v>639736.3199999999</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>0.2906</v>
+        <v>0.232</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>0.2323</v>
+        <v>0.1787</v>
       </c>
       <c r="H80" s="10" t="n"/>
       <c r="I80" s="10" t="n">
-        <v>0.1924</v>
+        <v>0.2037</v>
       </c>
       <c r="J80" s="13" t="n">
-        <v>4750</v>
+        <v>5891</v>
       </c>
       <c r="K80" s="13" t="n">
-        <v>8416</v>
+        <v>10143</v>
       </c>
       <c r="L80" s="32" t="n">
         <v>0</v>
@@ -12907,26 +12907,26 @@
         </is>
       </c>
       <c r="D81" s="15" t="n">
-        <v>343297.97</v>
+        <v>411291.81</v>
       </c>
       <c r="E81" s="15" t="n">
-        <v>474455.89</v>
+        <v>643296.55</v>
       </c>
       <c r="F81" s="16" t="n">
-        <v>0.3262</v>
+        <v>0.3064</v>
       </c>
       <c r="G81" s="16" t="n">
-        <v>0.2645</v>
+        <v>0.2446</v>
       </c>
       <c r="H81" s="16" t="n"/>
       <c r="I81" s="16" t="n">
-        <v>0.1203</v>
+        <v>0.1346</v>
       </c>
       <c r="J81" s="19" t="n">
-        <v>5577</v>
+        <v>6841</v>
       </c>
       <c r="K81" s="19" t="n">
-        <v>8317</v>
+        <v>10048</v>
       </c>
       <c r="L81" s="31" t="n">
         <v>0</v>
@@ -12949,26 +12949,26 @@
         </is>
       </c>
       <c r="D82" s="9" t="n">
-        <v>194650.23</v>
+        <v>243068.2</v>
       </c>
       <c r="E82" s="9" t="n">
-        <v>422566.62</v>
+        <v>557837.67</v>
       </c>
       <c r="F82" s="10" t="n">
-        <v>0.2725</v>
+        <v>0.1625</v>
       </c>
       <c r="G82" s="10" t="n">
-        <v>0.208</v>
+        <v>0.0982</v>
       </c>
       <c r="H82" s="10" t="n"/>
       <c r="I82" s="10" t="n">
-        <v>0.0898</v>
+        <v>0.1039</v>
       </c>
       <c r="J82" s="13" t="n">
-        <v>4831</v>
+        <v>6032</v>
       </c>
       <c r="K82" s="13" t="n">
-        <v>6917</v>
+        <v>8498</v>
       </c>
       <c r="L82" s="32" t="n">
         <v>0</v>
@@ -12991,26 +12991,26 @@
         </is>
       </c>
       <c r="D83" s="15" t="n">
-        <v>222131.91</v>
+        <v>291507.78</v>
       </c>
       <c r="E83" s="15" t="n">
-        <v>969049.4300000001</v>
+        <v>1269733.89</v>
       </c>
       <c r="F83" s="16" t="n">
-        <v>0.4333</v>
+        <v>0.4065</v>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0.3661</v>
+        <v>0.3402</v>
       </c>
       <c r="H83" s="16" t="n"/>
       <c r="I83" s="16" t="n">
-        <v>0.0536</v>
+        <v>0.0646</v>
       </c>
       <c r="J83" s="19" t="n">
-        <v>7784</v>
+        <v>9960</v>
       </c>
       <c r="K83" s="19" t="n">
-        <v>9573</v>
+        <v>12434</v>
       </c>
       <c r="L83" s="31" t="n">
         <v>0</v>
@@ -13033,26 +13033,26 @@
         </is>
       </c>
       <c r="D84" s="9" t="n">
-        <v>118118.32</v>
+        <v>160268.52</v>
       </c>
       <c r="E84" s="9" t="n">
-        <v>638949.23</v>
+        <v>1153253.02</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>0.5955</v>
+        <v>0.472</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>0.5269</v>
+        <v>0.399</v>
       </c>
       <c r="H84" s="10" t="n"/>
       <c r="I84" s="10" t="n">
-        <v>0.0299</v>
+        <v>0.0431</v>
       </c>
       <c r="J84" s="13" t="n">
-        <v>6517</v>
+        <v>8663</v>
       </c>
       <c r="K84" s="13" t="n">
-        <v>8326</v>
+        <v>11634</v>
       </c>
       <c r="L84" s="32" t="n">
         <v>0</v>
@@ -14419,26 +14419,26 @@
         </is>
       </c>
       <c r="D117" s="15" t="n">
-        <v>2380079.75</v>
+        <v>4147608.73</v>
       </c>
       <c r="E117" s="15" t="n">
-        <v>2790676.8</v>
+        <v>3859558</v>
       </c>
       <c r="F117" s="16" t="n">
-        <v>0.451</v>
+        <v>0.5436</v>
       </c>
       <c r="G117" s="16" t="n">
-        <v>0.3981</v>
+        <v>0.4942</v>
       </c>
       <c r="H117" s="16" t="n"/>
       <c r="I117" s="16" t="n">
-        <v>0.0785</v>
+        <v>0.08169999999999999</v>
       </c>
       <c r="J117" s="19" t="n">
-        <v>35347</v>
+        <v>54447</v>
       </c>
       <c r="K117" s="19" t="n">
-        <v>81307</v>
+        <v>126695</v>
       </c>
       <c r="L117" s="31" t="n">
         <v>0</v>
@@ -16603,26 +16603,26 @@
         </is>
       </c>
       <c r="D169" s="15" t="n">
-        <v>172620.02</v>
+        <v>274870.41</v>
       </c>
       <c r="E169" s="15" t="n">
-        <v>452068.08</v>
+        <v>633116.1899999999</v>
       </c>
       <c r="F169" s="16" t="n">
-        <v>1.0238</v>
+        <v>1.0231</v>
       </c>
       <c r="G169" s="16" t="n">
-        <v>0.9529</v>
+        <v>0.9528</v>
       </c>
       <c r="H169" s="16" t="n"/>
       <c r="I169" s="16" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="J169" s="19" t="n">
-        <v>10392</v>
+        <v>17127</v>
       </c>
       <c r="K169" s="19" t="n">
-        <v>26977</v>
+        <v>39178</v>
       </c>
       <c r="L169" s="31" t="n">
         <v>0</v>
@@ -16645,26 +16645,26 @@
         </is>
       </c>
       <c r="D170" s="9" t="n">
-        <v>1198140.41</v>
+        <v>1992458.84</v>
       </c>
       <c r="E170" s="9" t="n">
-        <v>843154</v>
+        <v>1453501.28</v>
       </c>
       <c r="F170" s="10" t="n">
-        <v>0.2334</v>
+        <v>0.3114</v>
       </c>
       <c r="G170" s="10" t="n">
-        <v>0.1869</v>
+        <v>0.2672</v>
       </c>
       <c r="H170" s="10" t="n"/>
       <c r="I170" s="10" t="n">
-        <v>0.2804</v>
+        <v>0.2862</v>
       </c>
       <c r="J170" s="13" t="n">
-        <v>5331</v>
+        <v>8364</v>
       </c>
       <c r="K170" s="13" t="n">
-        <v>17441</v>
+        <v>28036</v>
       </c>
       <c r="L170" s="32" t="n">
         <v>0</v>
@@ -16687,26 +16687,26 @@
         </is>
       </c>
       <c r="D171" s="15" t="n">
-        <v>575088.16</v>
+        <v>1192552.19</v>
       </c>
       <c r="E171" s="15" t="n">
-        <v>775354.85</v>
+        <v>890131</v>
       </c>
       <c r="F171" s="16" t="n">
-        <v>0.5246</v>
+        <v>0.6911</v>
       </c>
       <c r="G171" s="16" t="n">
-        <v>0.4681</v>
+        <v>0.6424</v>
       </c>
       <c r="H171" s="16" t="n"/>
       <c r="I171" s="16" t="n">
-        <v>0.1422</v>
+        <v>0.1534</v>
       </c>
       <c r="J171" s="19" t="n">
-        <v>5768</v>
+        <v>8551</v>
       </c>
       <c r="K171" s="19" t="n">
-        <v>19530</v>
+        <v>30536</v>
       </c>
       <c r="L171" s="31" t="n">
         <v>0</v>
@@ -16729,26 +16729,26 @@
         </is>
       </c>
       <c r="D172" s="9" t="n">
-        <v>171227.99</v>
+        <v>253265.07</v>
       </c>
       <c r="E172" s="9" t="n">
-        <v>176127.87</v>
+        <v>212265.18</v>
       </c>
       <c r="F172" s="10" t="n">
-        <v>0.5233</v>
+        <v>0.6125</v>
       </c>
       <c r="G172" s="10" t="n">
-        <v>0.4679</v>
+        <v>0.5589</v>
       </c>
       <c r="H172" s="10" t="n"/>
       <c r="I172" s="10" t="n">
-        <v>0.08649999999999999</v>
+        <v>0.0914</v>
       </c>
       <c r="J172" s="13" t="n">
-        <v>3643</v>
+        <v>5273</v>
       </c>
       <c r="K172" s="13" t="n">
-        <v>4865</v>
+        <v>7405</v>
       </c>
       <c r="L172" s="32" t="n">
         <v>0</v>
@@ -16771,26 +16771,26 @@
         </is>
       </c>
       <c r="D173" s="15" t="n">
-        <v>84656.11</v>
+        <v>118346.4</v>
       </c>
       <c r="E173" s="15" t="n">
-        <v>153148.07</v>
+        <v>167729.32</v>
       </c>
       <c r="F173" s="16" t="n">
-        <v>0.8007</v>
+        <v>0.7287</v>
       </c>
       <c r="G173" s="16" t="n">
-        <v>0.7438</v>
+        <v>0.6732</v>
       </c>
       <c r="H173" s="16" t="n"/>
       <c r="I173" s="16" t="n">
-        <v>0.0348</v>
+        <v>0.0398</v>
       </c>
       <c r="J173" s="19" t="n">
-        <v>2502</v>
+        <v>3468</v>
       </c>
       <c r="K173" s="19" t="n">
-        <v>3154</v>
+        <v>4447</v>
       </c>
       <c r="L173" s="31" t="n">
         <v>0</v>
@@ -16813,26 +16813,26 @@
         </is>
       </c>
       <c r="D174" s="9" t="n">
-        <v>118926.05</v>
+        <v>219955.62</v>
       </c>
       <c r="E174" s="9" t="n">
-        <v>221996.28</v>
+        <v>318797.51</v>
       </c>
       <c r="F174" s="10" t="n">
-        <v>0.8773</v>
+        <v>0.9011</v>
       </c>
       <c r="G174" s="10" t="n">
-        <v>0.8168</v>
+        <v>0.8413</v>
       </c>
       <c r="H174" s="10" t="n"/>
       <c r="I174" s="10" t="n">
-        <v>0.0098</v>
+        <v>0.0131</v>
       </c>
       <c r="J174" s="13" t="n">
-        <v>4610</v>
+        <v>7092</v>
       </c>
       <c r="K174" s="13" t="n">
-        <v>5450</v>
+        <v>11250</v>
       </c>
       <c r="L174" s="32" t="n">
         <v>0</v>
@@ -16855,26 +16855,26 @@
         </is>
       </c>
       <c r="D175" s="15" t="n">
-        <v>59421.01</v>
+        <v>96160.19</v>
       </c>
       <c r="E175" s="15" t="n">
-        <v>168827.66</v>
+        <v>184017.52</v>
       </c>
       <c r="F175" s="16" t="n">
-        <v>0.9038</v>
+        <v>0.9294</v>
       </c>
       <c r="G175" s="16" t="n">
-        <v>0.8355</v>
+        <v>0.864</v>
       </c>
       <c r="H175" s="16" t="n"/>
       <c r="I175" s="16" t="n">
-        <v>0.0026</v>
+        <v>0.0037</v>
       </c>
       <c r="J175" s="19" t="n">
-        <v>3101</v>
+        <v>4572</v>
       </c>
       <c r="K175" s="19" t="n">
-        <v>3890</v>
+        <v>5843</v>
       </c>
       <c r="L175" s="31" t="n">
         <v>0</v>
@@ -21601,26 +21601,26 @@
         </is>
       </c>
       <c r="D288" s="9" t="n">
-        <v>20957680.45</v>
+        <v>32916729.55</v>
       </c>
       <c r="E288" s="9" t="n">
-        <v>39767946.81</v>
+        <v>81755726.12</v>
       </c>
       <c r="F288" s="10" t="n">
-        <v>-0.0166</v>
+        <v>0.0281</v>
       </c>
       <c r="G288" s="10" t="n">
-        <v>-0.077</v>
+        <v>-0.0335</v>
       </c>
       <c r="H288" s="10" t="n"/>
       <c r="I288" s="10" t="n">
-        <v>0.1216</v>
+        <v>0.1346</v>
       </c>
       <c r="J288" s="13" t="n">
-        <v>490938</v>
+        <v>751329</v>
       </c>
       <c r="K288" s="13" t="n">
-        <v>1015531</v>
+        <v>1543785</v>
       </c>
       <c r="L288" s="32" t="n">
         <v>0</v>
@@ -26179,26 +26179,26 @@
         </is>
       </c>
       <c r="D397" s="15" t="n">
-        <v>1486167.44</v>
+        <v>2359613.28</v>
       </c>
       <c r="E397" s="15" t="n">
-        <v>12296298.56</v>
+        <v>27529453.84</v>
       </c>
       <c r="F397" s="16" t="n">
-        <v>-0.8596</v>
+        <v>-0.214</v>
       </c>
       <c r="G397" s="16" t="n">
-        <v>-0.9268</v>
+        <v>-0.2917</v>
       </c>
       <c r="H397" s="16" t="n"/>
       <c r="I397" s="16" t="n">
-        <v>0.0582</v>
+        <v>0.0667</v>
       </c>
       <c r="J397" s="19" t="n">
-        <v>105041</v>
+        <v>162834</v>
       </c>
       <c r="K397" s="19" t="n">
-        <v>207263</v>
+        <v>348420</v>
       </c>
       <c r="L397" s="31" t="n">
         <v>0</v>
@@ -26221,26 +26221,26 @@
         </is>
       </c>
       <c r="D398" s="9" t="n">
-        <v>7911790.13</v>
+        <v>13014165.11</v>
       </c>
       <c r="E398" s="9" t="n">
-        <v>7150674.57</v>
+        <v>12239365.48</v>
       </c>
       <c r="F398" s="10" t="n">
-        <v>0.0541</v>
+        <v>0.0072</v>
       </c>
       <c r="G398" s="10" t="n">
-        <v>-0.0037</v>
+        <v>-0.0492</v>
       </c>
       <c r="H398" s="10" t="n"/>
       <c r="I398" s="10" t="n">
-        <v>0.3003</v>
+        <v>0.3075</v>
       </c>
       <c r="J398" s="13" t="n">
-        <v>37735</v>
+        <v>61738</v>
       </c>
       <c r="K398" s="13" t="n">
-        <v>160474</v>
+        <v>257344</v>
       </c>
       <c r="L398" s="32" t="n">
         <v>0</v>
@@ -26263,26 +26263,26 @@
         </is>
       </c>
       <c r="D399" s="15" t="n">
-        <v>3857524.77</v>
+        <v>6203570.84</v>
       </c>
       <c r="E399" s="15" t="n">
-        <v>2953027.72</v>
+        <v>6169653.79</v>
       </c>
       <c r="F399" s="16" t="n">
-        <v>0.0221</v>
+        <v>0.0023</v>
       </c>
       <c r="G399" s="16" t="n">
-        <v>-0.0353</v>
+        <v>-0.0553</v>
       </c>
       <c r="H399" s="16" t="n"/>
       <c r="I399" s="16" t="n">
-        <v>0.206</v>
+        <v>0.2187</v>
       </c>
       <c r="J399" s="19" t="n">
-        <v>60153</v>
+        <v>91912</v>
       </c>
       <c r="K399" s="19" t="n">
-        <v>136152</v>
+        <v>202174</v>
       </c>
       <c r="L399" s="31" t="n">
         <v>0</v>
@@ -26305,26 +26305,26 @@
         </is>
       </c>
       <c r="D400" s="9" t="n">
-        <v>2615936.81</v>
+        <v>3904810.22</v>
       </c>
       <c r="E400" s="9" t="n">
-        <v>2406819.01</v>
+        <v>5377283.13</v>
       </c>
       <c r="F400" s="10" t="n">
-        <v>0.1113</v>
+        <v>0.1017</v>
       </c>
       <c r="G400" s="10" t="n">
-        <v>0.0519</v>
+        <v>0.0397</v>
       </c>
       <c r="H400" s="10" t="n"/>
       <c r="I400" s="10" t="n">
-        <v>0.1537</v>
+        <v>0.167</v>
       </c>
       <c r="J400" s="13" t="n">
-        <v>66696</v>
+        <v>101141</v>
       </c>
       <c r="K400" s="13" t="n">
-        <v>107021</v>
+        <v>162945</v>
       </c>
       <c r="L400" s="32" t="n">
         <v>0</v>
@@ -26347,26 +26347,26 @@
         </is>
       </c>
       <c r="D401" s="15" t="n">
-        <v>1528456.69</v>
+        <v>2266538.77</v>
       </c>
       <c r="E401" s="15" t="n">
-        <v>1632979.71</v>
+        <v>3911671.7</v>
       </c>
       <c r="F401" s="16" t="n">
-        <v>0.0048</v>
+        <v>0.0958</v>
       </c>
       <c r="G401" s="16" t="n">
-        <v>-0.0581</v>
+        <v>0.0306</v>
       </c>
       <c r="H401" s="16" t="n"/>
       <c r="I401" s="16" t="n">
-        <v>0.122</v>
+        <v>0.1365</v>
       </c>
       <c r="J401" s="19" t="n">
-        <v>54157</v>
+        <v>81532</v>
       </c>
       <c r="K401" s="19" t="n">
-        <v>81306</v>
+        <v>123226</v>
       </c>
       <c r="L401" s="31" t="n">
         <v>0</v>
@@ -26389,26 +26389,26 @@
         </is>
       </c>
       <c r="D402" s="9" t="n">
-        <v>1861947.6</v>
+        <v>2788575.93</v>
       </c>
       <c r="E402" s="9" t="n">
-        <v>3125214</v>
+        <v>7749499.65</v>
       </c>
       <c r="F402" s="10" t="n">
-        <v>0.0426</v>
+        <v>0.1264</v>
       </c>
       <c r="G402" s="10" t="n">
-        <v>-0.0211</v>
+        <v>0.0586</v>
       </c>
       <c r="H402" s="10" t="n"/>
       <c r="I402" s="10" t="n">
-        <v>0.0882</v>
+        <v>0.1038</v>
       </c>
       <c r="J402" s="13" t="n">
-        <v>88681</v>
+        <v>133119</v>
       </c>
       <c r="K402" s="13" t="n">
-        <v>124054</v>
+        <v>188333</v>
       </c>
       <c r="L402" s="32" t="n">
         <v>0</v>
@@ -26431,26 +26431,26 @@
         </is>
       </c>
       <c r="D403" s="15" t="n">
-        <v>1695857.01</v>
+        <v>2379455.41</v>
       </c>
       <c r="E403" s="15" t="n">
-        <v>10202933.25</v>
+        <v>18778798.53</v>
       </c>
       <c r="F403" s="16" t="n">
-        <v>0.0223</v>
+        <v>0.1489</v>
       </c>
       <c r="G403" s="16" t="n">
-        <v>-0.046</v>
+        <v>0.0765</v>
       </c>
       <c r="H403" s="16" t="n"/>
       <c r="I403" s="16" t="n">
-        <v>0.066</v>
+        <v>0.07870000000000001</v>
       </c>
       <c r="J403" s="19" t="n">
-        <v>78475</v>
+        <v>119053</v>
       </c>
       <c r="K403" s="19" t="n">
-        <v>199261</v>
+        <v>261343</v>
       </c>
       <c r="L403" s="31" t="n">
         <v>0</v>
@@ -27749,31 +27749,31 @@
         </is>
       </c>
       <c r="D433" s="15" t="n">
-        <v>27876873.41</v>
+        <v>35584131.75</v>
       </c>
       <c r="E433" s="15" t="n">
-        <v>37987244.76</v>
+        <v>50456879.64</v>
       </c>
       <c r="F433" s="16" t="n">
-        <v>0.3732</v>
+        <v>0.2263</v>
       </c>
       <c r="G433" s="16" t="n">
-        <v>0.3195</v>
+        <v>0.1708</v>
       </c>
       <c r="H433" s="16" t="n">
-        <v>0.1203</v>
+        <v>0.1241</v>
       </c>
       <c r="I433" s="16" t="n">
-        <v>0.0998</v>
+        <v>0.1155</v>
       </c>
       <c r="J433" s="19" t="n">
-        <v>563557</v>
+        <v>775797</v>
       </c>
       <c r="K433" s="19" t="n">
-        <v>1122369</v>
+        <v>1547571</v>
       </c>
       <c r="L433" s="31" t="n">
-        <v>0.5714</v>
+        <v>0.6609</v>
       </c>
     </row>
     <row r="434">
@@ -36629,31 +36629,31 @@
         </is>
       </c>
       <c r="D635" s="15" t="n">
-        <v>2382816.39</v>
+        <v>2968363.67</v>
       </c>
       <c r="E635" s="15" t="n">
-        <v>14345686.04</v>
+        <v>18589653.77</v>
       </c>
       <c r="F635" s="16" t="n">
-        <v>0.7859</v>
+        <v>0.7371</v>
       </c>
       <c r="G635" s="16" t="n">
-        <v>0.7151</v>
+        <v>0.6657999999999999</v>
       </c>
       <c r="H635" s="16" t="n">
-        <v>0.5065</v>
+        <v>0.4961</v>
       </c>
       <c r="I635" s="16" t="n">
-        <v>0.021</v>
+        <v>0.025</v>
       </c>
       <c r="J635" s="19" t="n">
-        <v>137327</v>
+        <v>172173</v>
       </c>
       <c r="K635" s="19" t="n">
-        <v>255969</v>
+        <v>336468</v>
       </c>
       <c r="L635" s="31" t="n">
-        <v>0.6146</v>
+        <v>0.6882</v>
       </c>
     </row>
     <row r="636">
@@ -36673,31 +36673,31 @@
         </is>
       </c>
       <c r="D636" s="9" t="n">
-        <v>7372698.27</v>
+        <v>9587171.49</v>
       </c>
       <c r="E636" s="9" t="n">
-        <v>6460768.27</v>
+        <v>8016614.73</v>
       </c>
       <c r="F636" s="10" t="n">
-        <v>0.1808</v>
+        <v>0.053</v>
       </c>
       <c r="G636" s="10" t="n">
-        <v>0.1317</v>
+        <v>0.002</v>
       </c>
       <c r="H636" s="10" t="n">
-        <v>0.0198</v>
+        <v>0.0229</v>
       </c>
       <c r="I636" s="10" t="n">
-        <v>0.2849</v>
+        <v>0.2784</v>
       </c>
       <c r="J636" s="13" t="n">
-        <v>27842</v>
+        <v>41943</v>
       </c>
       <c r="K636" s="13" t="n">
-        <v>126549</v>
+        <v>187101</v>
       </c>
       <c r="L636" s="32" t="n">
-        <v>0.5368000000000001</v>
+        <v>0.6368</v>
       </c>
     </row>
     <row r="637">
@@ -36717,31 +36717,31 @@
         </is>
       </c>
       <c r="D637" s="15" t="n">
-        <v>4243385.66</v>
+        <v>5486012.85</v>
       </c>
       <c r="E637" s="15" t="n">
-        <v>1997960.07</v>
+        <v>2685131.29</v>
       </c>
       <c r="F637" s="16" t="n">
-        <v>0.2042</v>
+        <v>0.0969</v>
       </c>
       <c r="G637" s="16" t="n">
-        <v>0.1584</v>
+        <v>0.0484</v>
       </c>
       <c r="H637" s="16" t="n">
-        <v>0.0629</v>
+        <v>0.0601</v>
       </c>
       <c r="I637" s="16" t="n">
-        <v>0.2272</v>
+        <v>0.233</v>
       </c>
       <c r="J637" s="19" t="n">
-        <v>52643</v>
+        <v>77690</v>
       </c>
       <c r="K637" s="19" t="n">
-        <v>103255</v>
+        <v>154450</v>
       </c>
       <c r="L637" s="31" t="n">
-        <v>0.5506</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="638">
@@ -36761,31 +36761,31 @@
         </is>
       </c>
       <c r="D638" s="9" t="n">
-        <v>3956831.51</v>
+        <v>5208226.48</v>
       </c>
       <c r="E638" s="9" t="n">
-        <v>2479619.7</v>
+        <v>3440591.94</v>
       </c>
       <c r="F638" s="10" t="n">
-        <v>0.2317</v>
+        <v>0.0577</v>
       </c>
       <c r="G638" s="10" t="n">
-        <v>0.1827</v>
+        <v>0.0059</v>
       </c>
       <c r="H638" s="10" t="n">
-        <v>0.0922</v>
+        <v>0.1002</v>
       </c>
       <c r="I638" s="10" t="n">
-        <v>0.176</v>
+        <v>0.187</v>
       </c>
       <c r="J638" s="13" t="n">
-        <v>68226</v>
+        <v>99509</v>
       </c>
       <c r="K638" s="13" t="n">
-        <v>131573</v>
+        <v>196729</v>
       </c>
       <c r="L638" s="32" t="n">
-        <v>0.5419</v>
+        <v>0.6505</v>
       </c>
     </row>
     <row r="639">
@@ -36805,31 +36805,31 @@
         </is>
       </c>
       <c r="D639" s="15" t="n">
-        <v>3075031.01</v>
+        <v>3782645.31</v>
       </c>
       <c r="E639" s="15" t="n">
-        <v>2381296.53</v>
+        <v>3331643.06</v>
       </c>
       <c r="F639" s="16" t="n">
-        <v>0.4155</v>
+        <v>0.259</v>
       </c>
       <c r="G639" s="16" t="n">
-        <v>0.3618</v>
+        <v>0.2035</v>
       </c>
       <c r="H639" s="16" t="n">
-        <v>0.1823</v>
+        <v>0.1699</v>
       </c>
       <c r="I639" s="16" t="n">
-        <v>0.1309</v>
+        <v>0.1498</v>
       </c>
       <c r="J639" s="19" t="n">
-        <v>64666</v>
+        <v>91964</v>
       </c>
       <c r="K639" s="19" t="n">
-        <v>125865</v>
+        <v>161857</v>
       </c>
       <c r="L639" s="31" t="n">
-        <v>0.5915</v>
+        <v>0.6663</v>
       </c>
     </row>
     <row r="640">
@@ -36849,31 +36849,31 @@
         </is>
       </c>
       <c r="D640" s="9" t="n">
-        <v>3777157.98</v>
+        <v>4739522.59</v>
       </c>
       <c r="E640" s="9" t="n">
-        <v>4970088.48</v>
+        <v>6730932.94</v>
       </c>
       <c r="F640" s="10" t="n">
-        <v>0.5399</v>
+        <v>0.3309</v>
       </c>
       <c r="G640" s="10" t="n">
-        <v>0.4811</v>
+        <v>0.2707</v>
       </c>
       <c r="H640" s="10" t="n">
-        <v>0.2376</v>
+        <v>0.2276</v>
       </c>
       <c r="I640" s="10" t="n">
-        <v>0.08119999999999999</v>
+        <v>0.1012</v>
       </c>
       <c r="J640" s="13" t="n">
-        <v>108658</v>
+        <v>151829</v>
       </c>
       <c r="K640" s="13" t="n">
-        <v>178324</v>
+        <v>235259</v>
       </c>
       <c r="L640" s="32" t="n">
-        <v>0.6189</v>
+        <v>0.6937</v>
       </c>
     </row>
     <row r="641">
@@ -36893,31 +36893,31 @@
         </is>
       </c>
       <c r="D641" s="15" t="n">
-        <v>3068952.59</v>
+        <v>3812189.36</v>
       </c>
       <c r="E641" s="15" t="n">
-        <v>5351825.67</v>
+        <v>7662311.91</v>
       </c>
       <c r="F641" s="16" t="n">
-        <v>0.6838</v>
+        <v>0.5179</v>
       </c>
       <c r="G641" s="16" t="n">
-        <v>0.6217</v>
+        <v>0.4545</v>
       </c>
       <c r="H641" s="16" t="n">
-        <v>0.3482</v>
+        <v>0.3416</v>
       </c>
       <c r="I641" s="16" t="n">
-        <v>0.04</v>
+        <v>0.0555</v>
       </c>
       <c r="J641" s="19" t="n">
-        <v>104195</v>
+        <v>140689</v>
       </c>
       <c r="K641" s="19" t="n">
-        <v>200834</v>
+        <v>275707</v>
       </c>
       <c r="L641" s="31" t="n">
-        <v>0.6091</v>
+        <v>0.6839</v>
       </c>
     </row>
     <row r="642">
@@ -37441,29 +37441,29 @@
         </is>
       </c>
       <c r="D654" s="9" t="n">
-        <v>5883424.11</v>
+        <v>6883889.3</v>
       </c>
       <c r="E654" s="9" t="n">
-        <v>33683179.93</v>
+        <v>38759180.98</v>
       </c>
       <c r="F654" s="10" t="n">
-        <v>0.3335</v>
+        <v>0.33</v>
       </c>
       <c r="G654" s="10" t="n">
-        <v>0.2681</v>
+        <v>0.2646</v>
       </c>
       <c r="H654" s="10" t="n"/>
       <c r="I654" s="10" t="n">
-        <v>0.0641</v>
+        <v>0.0634</v>
       </c>
       <c r="J654" s="13" t="n">
-        <v>236162</v>
+        <v>276725</v>
       </c>
       <c r="K654" s="13" t="n">
-        <v>327042</v>
+        <v>378164</v>
       </c>
       <c r="L654" s="32" t="n">
-        <v>0.6099</v>
+        <v>0.6597</v>
       </c>
     </row>
     <row r="655">
@@ -41011,29 +41011,29 @@
         </is>
       </c>
       <c r="D739" s="15" t="n">
-        <v>1638396.24</v>
+        <v>1929103.83</v>
       </c>
       <c r="E739" s="15" t="n">
-        <v>24103698.28</v>
+        <v>27757514.56</v>
       </c>
       <c r="F739" s="16" t="n">
-        <v>0.7214</v>
+        <v>0.7066</v>
       </c>
       <c r="G739" s="16" t="n">
-        <v>0.6423</v>
+        <v>0.6284</v>
       </c>
       <c r="H739" s="16" t="n"/>
       <c r="I739" s="16" t="n">
-        <v>0.0142</v>
+        <v>0.0148</v>
       </c>
       <c r="J739" s="19" t="n">
-        <v>139243</v>
+        <v>162994</v>
       </c>
       <c r="K739" s="19" t="n">
-        <v>190228</v>
+        <v>220323</v>
       </c>
       <c r="L739" s="31" t="n">
-        <v>0.6486</v>
+        <v>0.6899</v>
       </c>
     </row>
     <row r="740">
@@ -41053,29 +41053,29 @@
         </is>
       </c>
       <c r="D740" s="9" t="n">
-        <v>723907.92</v>
+        <v>854460.53</v>
       </c>
       <c r="E740" s="9" t="n">
-        <v>336608.99</v>
+        <v>374003.51</v>
       </c>
       <c r="F740" s="10" t="n">
-        <v>0.2155</v>
+        <v>0.1993</v>
       </c>
       <c r="G740" s="10" t="n">
-        <v>0.1748</v>
+        <v>0.1576</v>
       </c>
       <c r="H740" s="10" t="n"/>
       <c r="I740" s="10" t="n">
-        <v>0.3497</v>
+        <v>0.348</v>
       </c>
       <c r="J740" s="13" t="n">
-        <v>3563</v>
+        <v>4359</v>
       </c>
       <c r="K740" s="13" t="n">
-        <v>10193</v>
+        <v>11426</v>
       </c>
       <c r="L740" s="32" t="n">
-        <v>0.5591</v>
+        <v>0.6219</v>
       </c>
     </row>
     <row r="741">
@@ -41095,29 +41095,29 @@
         </is>
       </c>
       <c r="D741" s="15" t="n">
-        <v>881711.33</v>
+        <v>988917.9</v>
       </c>
       <c r="E741" s="15" t="n">
-        <v>747959.14</v>
+        <v>810893.2</v>
       </c>
       <c r="F741" s="16" t="n">
-        <v>0.0417</v>
+        <v>0.0553</v>
       </c>
       <c r="G741" s="16" t="n">
-        <v>-0.0108</v>
+        <v>0.0024</v>
       </c>
       <c r="H741" s="16" t="n"/>
       <c r="I741" s="16" t="n">
-        <v>0.2878</v>
+        <v>0.2824</v>
       </c>
       <c r="J741" s="19" t="n">
-        <v>8545</v>
+        <v>9896</v>
       </c>
       <c r="K741" s="19" t="n">
-        <v>17103</v>
+        <v>18946</v>
       </c>
       <c r="L741" s="31" t="n">
-        <v>0.6027</v>
+        <v>0.6454</v>
       </c>
     </row>
     <row r="742">
@@ -41137,29 +41137,29 @@
         </is>
       </c>
       <c r="D742" s="9" t="n">
-        <v>575257.27</v>
+        <v>685530.0699999999</v>
       </c>
       <c r="E742" s="9" t="n">
-        <v>1165771.54</v>
+        <v>1270846.77</v>
       </c>
       <c r="F742" s="10" t="n">
-        <v>0.0827</v>
+        <v>0.0725</v>
       </c>
       <c r="G742" s="10" t="n">
-        <v>0.0195</v>
+        <v>0.0097</v>
       </c>
       <c r="H742" s="10" t="n"/>
       <c r="I742" s="10" t="n">
-        <v>0.218</v>
+        <v>0.2119</v>
       </c>
       <c r="J742" s="13" t="n">
-        <v>10915</v>
+        <v>12787</v>
       </c>
       <c r="K742" s="13" t="n">
-        <v>15130</v>
+        <v>17506</v>
       </c>
       <c r="L742" s="32" t="n">
-        <v>0.6513</v>
+        <v>0.7019</v>
       </c>
     </row>
     <row r="743">
@@ -41179,29 +41179,29 @@
         </is>
       </c>
       <c r="D743" s="15" t="n">
-        <v>486709.96</v>
+        <v>582953.45</v>
       </c>
       <c r="E743" s="15" t="n">
-        <v>981043.5699999999</v>
+        <v>1087743.92</v>
       </c>
       <c r="F743" s="16" t="n">
-        <v>0.0203</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="G743" s="16" t="n">
-        <v>-0.0429</v>
+        <v>0.0197</v>
       </c>
       <c r="H743" s="16" t="n"/>
       <c r="I743" s="16" t="n">
-        <v>0.1736</v>
+        <v>0.1701</v>
       </c>
       <c r="J743" s="19" t="n">
-        <v>11793</v>
+        <v>13760</v>
       </c>
       <c r="K743" s="19" t="n">
-        <v>15442</v>
+        <v>17846</v>
       </c>
       <c r="L743" s="31" t="n">
-        <v>0.5508</v>
+        <v>0.6208</v>
       </c>
     </row>
     <row r="744">
@@ -41221,29 +41221,29 @@
         </is>
       </c>
       <c r="D744" s="9" t="n">
-        <v>755018.47</v>
+        <v>892393.95</v>
       </c>
       <c r="E744" s="9" t="n">
-        <v>2188484.66</v>
+        <v>2566852.42</v>
       </c>
       <c r="F744" s="10" t="n">
-        <v>0.2636</v>
+        <v>0.2523</v>
       </c>
       <c r="G744" s="10" t="n">
-        <v>0.1942</v>
+        <v>0.1828</v>
       </c>
       <c r="H744" s="10" t="n"/>
       <c r="I744" s="10" t="n">
-        <v>0.1116</v>
+        <v>0.1092</v>
       </c>
       <c r="J744" s="13" t="n">
-        <v>26257</v>
+        <v>30799</v>
       </c>
       <c r="K744" s="13" t="n">
-        <v>33663</v>
+        <v>39273</v>
       </c>
       <c r="L744" s="32" t="n">
-        <v>0.6178</v>
+        <v>0.6681</v>
       </c>
     </row>
     <row r="745">
@@ -41263,29 +41263,29 @@
         </is>
       </c>
       <c r="D745" s="15" t="n">
-        <v>822422.9300000001</v>
+        <v>950529.58</v>
       </c>
       <c r="E745" s="15" t="n">
-        <v>4159613.74</v>
+        <v>4891326.59</v>
       </c>
       <c r="F745" s="16" t="n">
-        <v>0.4026</v>
+        <v>0.3793</v>
       </c>
       <c r="G745" s="16" t="n">
-        <v>0.3292</v>
+        <v>0.3057</v>
       </c>
       <c r="H745" s="16" t="n"/>
       <c r="I745" s="16" t="n">
-        <v>0.0586</v>
+        <v>0.0574</v>
       </c>
       <c r="J745" s="19" t="n">
-        <v>35846</v>
+        <v>42130</v>
       </c>
       <c r="K745" s="19" t="n">
-        <v>45283</v>
+        <v>52844</v>
       </c>
       <c r="L745" s="31" t="n">
-        <v>0.5836</v>
+        <v>0.6328</v>
       </c>
     </row>
     <row r="746">
@@ -42187,29 +42187,29 @@
         </is>
       </c>
       <c r="D767" s="15" t="n">
-        <v>5728396.3</v>
+        <v>9677381.960000001</v>
       </c>
       <c r="E767" s="15" t="n">
-        <v>10713899.56</v>
+        <v>13822086.59</v>
       </c>
       <c r="F767" s="16" t="n">
-        <v>0.08840000000000001</v>
+        <v>0.0324</v>
       </c>
       <c r="G767" s="16" t="n">
-        <v>0.0329</v>
+        <v>-0.024</v>
       </c>
       <c r="H767" s="16" t="n"/>
       <c r="I767" s="16" t="n">
-        <v>0.1203</v>
+        <v>0.1104</v>
       </c>
       <c r="J767" s="19" t="n">
-        <v>86568</v>
+        <v>167005</v>
       </c>
       <c r="K767" s="19" t="n">
-        <v>141180</v>
+        <v>271121</v>
       </c>
       <c r="L767" s="31" t="n">
-        <v>0.5798</v>
+        <v>0.7433999999999999</v>
       </c>
     </row>
     <row r="768">
@@ -48403,29 +48403,29 @@
         </is>
       </c>
       <c r="D915" s="15" t="n">
-        <v>292227.67</v>
+        <v>744122.5</v>
       </c>
       <c r="E915" s="15" t="n">
-        <v>3073006.16</v>
+        <v>4064712.31</v>
       </c>
       <c r="F915" s="16" t="n">
-        <v>0.7371</v>
+        <v>0.5653</v>
       </c>
       <c r="G915" s="16" t="n">
-        <v>0.665</v>
+        <v>0.4972</v>
       </c>
       <c r="H915" s="16" t="n"/>
       <c r="I915" s="16" t="n">
-        <v>0.0201</v>
+        <v>0.0203</v>
       </c>
       <c r="J915" s="19" t="n">
-        <v>22508</v>
+        <v>49211</v>
       </c>
       <c r="K915" s="19" t="n">
-        <v>30273</v>
+        <v>73690</v>
       </c>
       <c r="L915" s="31" t="n">
-        <v>0.5588</v>
+        <v>0.8229</v>
       </c>
     </row>
     <row r="916">
@@ -48445,29 +48445,29 @@
         </is>
       </c>
       <c r="D916" s="9" t="n">
-        <v>2406218.79</v>
+        <v>3443621.3</v>
       </c>
       <c r="E916" s="9" t="n">
-        <v>2093183.78</v>
+        <v>2678020.6</v>
       </c>
       <c r="F916" s="10" t="n">
-        <v>-0.1479</v>
+        <v>-0.1527</v>
       </c>
       <c r="G916" s="10" t="n">
-        <v>-0.1929</v>
+        <v>-0.2008</v>
       </c>
       <c r="H916" s="10" t="n"/>
       <c r="I916" s="10" t="n">
-        <v>0.3198</v>
+        <v>0.3269</v>
       </c>
       <c r="J916" s="13" t="n">
-        <v>5038</v>
+        <v>8404</v>
       </c>
       <c r="K916" s="13" t="n">
-        <v>28913</v>
+        <v>42001</v>
       </c>
       <c r="L916" s="32" t="n">
-        <v>0.5425</v>
+        <v>0.6704</v>
       </c>
     </row>
     <row r="917">
@@ -48487,29 +48487,29 @@
         </is>
       </c>
       <c r="D917" s="15" t="n">
-        <v>1038988.12</v>
+        <v>1932692.87</v>
       </c>
       <c r="E917" s="15" t="n">
-        <v>960900.15</v>
+        <v>1181256.81</v>
       </c>
       <c r="F917" s="16" t="n">
-        <v>0.1065</v>
+        <v>-0.1392</v>
       </c>
       <c r="G917" s="16" t="n">
-        <v>0.0514</v>
+        <v>-0.1937</v>
       </c>
       <c r="H917" s="16" t="n"/>
       <c r="I917" s="16" t="n">
-        <v>0.258</v>
+        <v>0.2574</v>
       </c>
       <c r="J917" s="19" t="n">
-        <v>9473</v>
+        <v>16790</v>
       </c>
       <c r="K917" s="19" t="n">
-        <v>17083</v>
+        <v>38224</v>
       </c>
       <c r="L917" s="31" t="n">
-        <v>0.5841</v>
+        <v>0.763</v>
       </c>
     </row>
     <row r="918">
@@ -48529,29 +48529,29 @@
         </is>
       </c>
       <c r="D918" s="9" t="n">
-        <v>732812.42</v>
+        <v>1288822.6</v>
       </c>
       <c r="E918" s="9" t="n">
-        <v>865290.91</v>
+        <v>1130042.97</v>
       </c>
       <c r="F918" s="10" t="n">
-        <v>0.1566</v>
+        <v>0.0755</v>
       </c>
       <c r="G918" s="10" t="n">
-        <v>0.0954</v>
+        <v>0.016</v>
       </c>
       <c r="H918" s="10" t="n"/>
       <c r="I918" s="10" t="n">
-        <v>0.206</v>
+        <v>0.192</v>
       </c>
       <c r="J918" s="13" t="n">
-        <v>10698</v>
+        <v>18973</v>
       </c>
       <c r="K918" s="13" t="n">
-        <v>15311</v>
+        <v>26045</v>
       </c>
       <c r="L918" s="32" t="n">
-        <v>0.6149</v>
+        <v>0.7795</v>
       </c>
     </row>
     <row r="919">
@@ -48571,29 +48571,29 @@
         </is>
       </c>
       <c r="D919" s="15" t="n">
-        <v>441662.29</v>
+        <v>731869.21</v>
       </c>
       <c r="E919" s="15" t="n">
-        <v>794404.73</v>
+        <v>951924.3</v>
       </c>
       <c r="F919" s="16" t="n">
-        <v>0.1946</v>
+        <v>0.1142</v>
       </c>
       <c r="G919" s="16" t="n">
-        <v>0.1317</v>
+        <v>0.0529</v>
       </c>
       <c r="H919" s="16" t="n"/>
       <c r="I919" s="16" t="n">
-        <v>0.1463</v>
+        <v>0.1429</v>
       </c>
       <c r="J919" s="19" t="n">
-        <v>9114</v>
+        <v>16288</v>
       </c>
       <c r="K919" s="19" t="n">
-        <v>12821</v>
+        <v>21376</v>
       </c>
       <c r="L919" s="31" t="n">
-        <v>0.6248</v>
+        <v>0.7693</v>
       </c>
     </row>
     <row r="920">
@@ -48613,29 +48613,29 @@
         </is>
       </c>
       <c r="D920" s="9" t="n">
-        <v>505807.52</v>
+        <v>921062.34</v>
       </c>
       <c r="E920" s="9" t="n">
-        <v>1300235.15</v>
+        <v>1654872.84</v>
       </c>
       <c r="F920" s="10" t="n">
-        <v>0.3311</v>
+        <v>0.2539</v>
       </c>
       <c r="G920" s="10" t="n">
-        <v>0.2605</v>
+        <v>0.188</v>
       </c>
       <c r="H920" s="10" t="n"/>
       <c r="I920" s="10" t="n">
-        <v>0.1058</v>
+        <v>0.09959999999999999</v>
       </c>
       <c r="J920" s="13" t="n">
-        <v>15259</v>
+        <v>28880</v>
       </c>
       <c r="K920" s="13" t="n">
-        <v>19919</v>
+        <v>36243</v>
       </c>
       <c r="L920" s="32" t="n">
-        <v>0.6479</v>
+        <v>0.8032</v>
       </c>
     </row>
     <row r="921">
@@ -48655,29 +48655,29 @@
         </is>
       </c>
       <c r="D921" s="15" t="n">
-        <v>310679.49</v>
+        <v>615191.14</v>
       </c>
       <c r="E921" s="15" t="n">
-        <v>1626878.69</v>
+        <v>2161256.77</v>
       </c>
       <c r="F921" s="16" t="n">
-        <v>0.5417</v>
+        <v>0.4442</v>
       </c>
       <c r="G921" s="16" t="n">
-        <v>0.4672</v>
+        <v>0.375</v>
       </c>
       <c r="H921" s="16" t="n"/>
       <c r="I921" s="16" t="n">
-        <v>0.052</v>
+        <v>0.0532</v>
       </c>
       <c r="J921" s="19" t="n">
-        <v>14478</v>
+        <v>28459</v>
       </c>
       <c r="K921" s="19" t="n">
-        <v>16860</v>
+        <v>33542</v>
       </c>
       <c r="L921" s="31" t="n">
-        <v>0.6161</v>
+        <v>0.7986</v>
       </c>
     </row>
     <row r="922">
@@ -49117,29 +49117,29 @@
         </is>
       </c>
       <c r="D932" s="9" t="n">
-        <v>1198339.07</v>
+        <v>3076342.28</v>
       </c>
       <c r="E932" s="9" t="n">
-        <v>4263679.11</v>
+        <v>5563991.12</v>
       </c>
       <c r="F932" s="10" t="n">
-        <v>0.7712</v>
+        <v>0.5797</v>
       </c>
       <c r="G932" s="10" t="n">
-        <v>0.7033</v>
+        <v>0.5195</v>
       </c>
       <c r="H932" s="10" t="n"/>
       <c r="I932" s="10" t="n">
-        <v>0.0194</v>
+        <v>0.0393</v>
       </c>
       <c r="J932" s="13" t="n">
-        <v>35039</v>
+        <v>72495</v>
       </c>
       <c r="K932" s="13" t="n">
-        <v>46605</v>
+        <v>102846</v>
       </c>
       <c r="L932" s="32" t="n">
-        <v>0.7917999999999999</v>
+        <v>0.901</v>
       </c>
     </row>
     <row r="933">
@@ -52099,29 +52099,29 @@
         </is>
       </c>
       <c r="D1003" s="15" t="n">
-        <v>551802.4300000001</v>
+        <v>830530.21</v>
       </c>
       <c r="E1003" s="15" t="n">
-        <v>2780012.14</v>
+        <v>3380588.38</v>
       </c>
       <c r="F1003" s="16" t="n">
-        <v>0.9288</v>
+        <v>0.9094</v>
       </c>
       <c r="G1003" s="16" t="n">
-        <v>0.8583</v>
+        <v>0.8406</v>
       </c>
       <c r="H1003" s="16" t="n"/>
       <c r="I1003" s="16" t="n">
-        <v>0.0057</v>
+        <v>0.0074</v>
       </c>
       <c r="J1003" s="19" t="n">
-        <v>24066</v>
+        <v>38608</v>
       </c>
       <c r="K1003" s="19" t="n">
-        <v>33202</v>
+        <v>54884</v>
       </c>
       <c r="L1003" s="31" t="n">
-        <v>0.8744</v>
+        <v>0.8847</v>
       </c>
     </row>
     <row r="1004">
@@ -52141,29 +52141,29 @@
         </is>
       </c>
       <c r="D1004" s="9" t="n">
-        <v>101232.93</v>
+        <v>327597.09</v>
       </c>
       <c r="E1004" s="9" t="n">
-        <v>94809.7</v>
+        <v>120528.39</v>
       </c>
       <c r="F1004" s="10" t="n">
-        <v>0.5261</v>
+        <v>0.2446</v>
       </c>
       <c r="G1004" s="10" t="n">
-        <v>0.4749</v>
+        <v>0.2002</v>
       </c>
       <c r="H1004" s="10" t="n"/>
       <c r="I1004" s="10" t="n">
-        <v>0.1649</v>
+        <v>0.2683</v>
       </c>
       <c r="J1004" s="13" t="n">
-        <v>473</v>
+        <v>1297</v>
       </c>
       <c r="K1004" s="13" t="n">
-        <v>779</v>
+        <v>2663</v>
       </c>
       <c r="L1004" s="32" t="n">
-        <v>0.3049</v>
+        <v>0.7684</v>
       </c>
     </row>
     <row r="1005">
@@ -52183,29 +52183,29 @@
         </is>
       </c>
       <c r="D1005" s="15" t="n">
-        <v>52065.34</v>
+        <v>348532.94</v>
       </c>
       <c r="E1005" s="15" t="n">
-        <v>43609.77</v>
+        <v>70397.49000000001</v>
       </c>
       <c r="F1005" s="16" t="n">
-        <v>0.1682</v>
+        <v>0.2285</v>
       </c>
       <c r="G1005" s="16" t="n">
-        <v>0.1129</v>
+        <v>0.1799</v>
       </c>
       <c r="H1005" s="16" t="n"/>
       <c r="I1005" s="16" t="n">
-        <v>0.1829</v>
+        <v>0.2063</v>
       </c>
       <c r="J1005" s="19" t="n">
-        <v>771</v>
+        <v>2903</v>
       </c>
       <c r="K1005" s="19" t="n">
-        <v>949</v>
+        <v>4493</v>
       </c>
       <c r="L1005" s="31" t="n">
-        <v>0.7786</v>
+        <v>0.9579</v>
       </c>
     </row>
     <row r="1006">
@@ -52225,29 +52225,29 @@
         </is>
       </c>
       <c r="D1006" s="9" t="n">
-        <v>69879.28</v>
+        <v>433612.53</v>
       </c>
       <c r="E1006" s="9" t="n">
-        <v>82534.91</v>
+        <v>150889.82</v>
       </c>
       <c r="F1006" s="10" t="n">
-        <v>0.6143999999999999</v>
+        <v>0.3322</v>
       </c>
       <c r="G1006" s="10" t="n">
-        <v>0.5541</v>
+        <v>0.2788</v>
       </c>
       <c r="H1006" s="10" t="n"/>
       <c r="I1006" s="10" t="n">
-        <v>0.09370000000000001</v>
+        <v>0.1326</v>
       </c>
       <c r="J1006" s="13" t="n">
-        <v>1078</v>
+        <v>4517</v>
       </c>
       <c r="K1006" s="13" t="n">
-        <v>1312</v>
+        <v>7557</v>
       </c>
       <c r="L1006" s="32" t="n">
-        <v>0.7081</v>
+        <v>0.946</v>
       </c>
     </row>
     <row r="1007">
@@ -52267,29 +52267,29 @@
         </is>
       </c>
       <c r="D1007" s="15" t="n">
-        <v>91921.74000000001</v>
+        <v>297772.82</v>
       </c>
       <c r="E1007" s="15" t="n">
-        <v>362974.88</v>
+        <v>460294.09</v>
       </c>
       <c r="F1007" s="16" t="n">
-        <v>0.2831</v>
+        <v>0.4944</v>
       </c>
       <c r="G1007" s="16" t="n">
-        <v>0.1983</v>
+        <v>0.4284</v>
       </c>
       <c r="H1007" s="16" t="n"/>
       <c r="I1007" s="16" t="n">
-        <v>0.0558</v>
+        <v>0.0726</v>
       </c>
       <c r="J1007" s="19" t="n">
-        <v>1219</v>
+        <v>4446</v>
       </c>
       <c r="K1007" s="19" t="n">
-        <v>1419</v>
+        <v>6036</v>
       </c>
       <c r="L1007" s="31" t="n">
-        <v>0.8192</v>
+        <v>0.9371</v>
       </c>
     </row>
     <row r="1008">
@@ -52309,29 +52309,29 @@
         </is>
       </c>
       <c r="D1008" s="9" t="n">
-        <v>160540.29</v>
+        <v>489960.58</v>
       </c>
       <c r="E1008" s="9" t="n">
-        <v>318797.58</v>
+        <v>541309.28</v>
       </c>
       <c r="F1008" s="10" t="n">
-        <v>0.7702</v>
+        <v>0.6294</v>
       </c>
       <c r="G1008" s="10" t="n">
-        <v>0.7035</v>
+        <v>0.5665</v>
       </c>
       <c r="H1008" s="10" t="n"/>
       <c r="I1008" s="10" t="n">
-        <v>0.0318</v>
+        <v>0.0444</v>
       </c>
       <c r="J1008" s="13" t="n">
-        <v>3274</v>
+        <v>10318</v>
       </c>
       <c r="K1008" s="13" t="n">
-        <v>3937</v>
+        <v>14914</v>
       </c>
       <c r="L1008" s="32" t="n">
-        <v>0.8272</v>
+        <v>0.9287</v>
       </c>
     </row>
     <row r="1009">
@@ -52351,29 +52351,29 @@
         </is>
       </c>
       <c r="D1009" s="15" t="n">
-        <v>170897.05</v>
+        <v>348336.1</v>
       </c>
       <c r="E1009" s="15" t="n">
-        <v>580940.13</v>
+        <v>839983.67</v>
       </c>
       <c r="F1009" s="16" t="n">
-        <v>0.9191</v>
+        <v>0.7715</v>
       </c>
       <c r="G1009" s="16" t="n">
-        <v>0.8504</v>
+        <v>0.7057</v>
       </c>
       <c r="H1009" s="16" t="n"/>
       <c r="I1009" s="16" t="n">
-        <v>0.012</v>
+        <v>0.0229</v>
       </c>
       <c r="J1009" s="19" t="n">
-        <v>4158</v>
+        <v>10406</v>
       </c>
       <c r="K1009" s="19" t="n">
-        <v>5007</v>
+        <v>12299</v>
       </c>
       <c r="L1009" s="31" t="n">
-        <v>0.8036</v>
+        <v>0.8815</v>
       </c>
     </row>
     <row r="1010">
@@ -52771,26 +52771,26 @@
         </is>
       </c>
       <c r="D1019" s="15" t="n">
-        <v>3761117</v>
+        <v>4883704.82</v>
       </c>
       <c r="E1019" s="15" t="n">
-        <v>10181039.4</v>
+        <v>11410902.52</v>
       </c>
       <c r="F1019" s="16" t="n">
-        <v>0.2452</v>
+        <v>0.2947</v>
       </c>
       <c r="G1019" s="16" t="n">
-        <v>0.1904</v>
+        <v>0.2396</v>
       </c>
       <c r="H1019" s="16" t="n"/>
       <c r="I1019" s="16" t="n">
-        <v>0.1111</v>
+        <v>0.1034</v>
       </c>
       <c r="J1019" s="19" t="n">
-        <v>60182</v>
+        <v>83650</v>
       </c>
       <c r="K1019" s="19" t="n">
-        <v>155631</v>
+        <v>217106</v>
       </c>
       <c r="L1019" s="31" t="n">
         <v>0</v>
@@ -55459,26 +55459,26 @@
         </is>
       </c>
       <c r="D1083" s="15" t="n">
-        <v>140082.98</v>
+        <v>233801.06</v>
       </c>
       <c r="E1083" s="15" t="n">
-        <v>3539504.62</v>
+        <v>3759790.86</v>
       </c>
       <c r="F1083" s="16" t="n">
-        <v>0.8312</v>
+        <v>0.8228</v>
       </c>
       <c r="G1083" s="16" t="n">
-        <v>0.7625999999999999</v>
+        <v>0.7577</v>
       </c>
       <c r="H1083" s="16" t="n"/>
       <c r="I1083" s="16" t="n">
-        <v>0.0254</v>
+        <v>0.0242</v>
       </c>
       <c r="J1083" s="19" t="n">
-        <v>7643</v>
+        <v>11853</v>
       </c>
       <c r="K1083" s="19" t="n">
-        <v>29077</v>
+        <v>43020</v>
       </c>
       <c r="L1083" s="31" t="n">
         <v>0</v>
@@ -55501,26 +55501,26 @@
         </is>
       </c>
       <c r="D1084" s="9" t="n">
-        <v>1643226.8</v>
+        <v>2049166.03</v>
       </c>
       <c r="E1084" s="9" t="n">
-        <v>1488514.8</v>
+        <v>1733859.95</v>
       </c>
       <c r="F1084" s="10" t="n">
-        <v>0.2281</v>
+        <v>0.2517</v>
       </c>
       <c r="G1084" s="10" t="n">
-        <v>0.1801</v>
+        <v>0.2032</v>
       </c>
       <c r="H1084" s="10" t="n"/>
       <c r="I1084" s="10" t="n">
-        <v>0.2427</v>
+        <v>0.2375</v>
       </c>
       <c r="J1084" s="13" t="n">
-        <v>9690</v>
+        <v>13089</v>
       </c>
       <c r="K1084" s="13" t="n">
-        <v>33617</v>
+        <v>44052</v>
       </c>
       <c r="L1084" s="32" t="n">
         <v>0</v>
@@ -55543,26 +55543,26 @@
         </is>
       </c>
       <c r="D1085" s="15" t="n">
-        <v>860192.47</v>
+        <v>1119827.3</v>
       </c>
       <c r="E1085" s="15" t="n">
-        <v>648869.47</v>
+        <v>856873.38</v>
       </c>
       <c r="F1085" s="16" t="n">
-        <v>0.1239</v>
+        <v>0.1568</v>
       </c>
       <c r="G1085" s="16" t="n">
-        <v>0.0678</v>
+        <v>0.1007</v>
       </c>
       <c r="H1085" s="16" t="n"/>
       <c r="I1085" s="16" t="n">
-        <v>0.1651</v>
+        <v>0.1559</v>
       </c>
       <c r="J1085" s="19" t="n">
-        <v>10760</v>
+        <v>14470</v>
       </c>
       <c r="K1085" s="19" t="n">
-        <v>25498</v>
+        <v>33322</v>
       </c>
       <c r="L1085" s="31" t="n">
         <v>0</v>
@@ -55585,26 +55585,26 @@
         </is>
       </c>
       <c r="D1086" s="9" t="n">
-        <v>498427.51</v>
+        <v>619609.3100000001</v>
       </c>
       <c r="E1086" s="9" t="n">
-        <v>727135.91</v>
+        <v>885983.88</v>
       </c>
       <c r="F1086" s="10" t="n">
-        <v>0.259</v>
+        <v>0.325</v>
       </c>
       <c r="G1086" s="10" t="n">
-        <v>0.199</v>
+        <v>0.2646</v>
       </c>
       <c r="H1086" s="10" t="n"/>
       <c r="I1086" s="10" t="n">
-        <v>0.1164</v>
+        <v>0.1107</v>
       </c>
       <c r="J1086" s="13" t="n">
-        <v>9752</v>
+        <v>13030</v>
       </c>
       <c r="K1086" s="13" t="n">
-        <v>19987</v>
+        <v>25430</v>
       </c>
       <c r="L1086" s="32" t="n">
         <v>0</v>
@@ -55627,26 +55627,26 @@
         </is>
       </c>
       <c r="D1087" s="15" t="n">
-        <v>236016.44</v>
+        <v>316586.42</v>
       </c>
       <c r="E1087" s="15" t="n">
-        <v>354154.05</v>
+        <v>373916.57</v>
       </c>
       <c r="F1087" s="16" t="n">
-        <v>0.0487</v>
+        <v>0.193</v>
       </c>
       <c r="G1087" s="16" t="n">
-        <v>-0.0134</v>
+        <v>0.1318</v>
       </c>
       <c r="H1087" s="16" t="n"/>
       <c r="I1087" s="16" t="n">
-        <v>0.0815</v>
+        <v>0.07480000000000001</v>
       </c>
       <c r="J1087" s="19" t="n">
-        <v>5893</v>
+        <v>8213</v>
       </c>
       <c r="K1087" s="19" t="n">
-        <v>9374</v>
+        <v>13215</v>
       </c>
       <c r="L1087" s="31" t="n">
         <v>0</v>
@@ -55669,26 +55669,26 @@
         </is>
       </c>
       <c r="D1088" s="9" t="n">
-        <v>227750.23</v>
+        <v>315943.21</v>
       </c>
       <c r="E1088" s="9" t="n">
-        <v>807563.36</v>
+        <v>940013.1899999999</v>
       </c>
       <c r="F1088" s="10" t="n">
-        <v>0.3087</v>
+        <v>0.3836</v>
       </c>
       <c r="G1088" s="10" t="n">
-        <v>0.2451</v>
+        <v>0.3211</v>
       </c>
       <c r="H1088" s="10" t="n"/>
       <c r="I1088" s="10" t="n">
-        <v>0.0598</v>
+        <v>0.0526</v>
       </c>
       <c r="J1088" s="13" t="n">
-        <v>8785</v>
+        <v>12339</v>
       </c>
       <c r="K1088" s="13" t="n">
-        <v>13111</v>
+        <v>18515</v>
       </c>
       <c r="L1088" s="32" t="n">
         <v>0</v>
@@ -55711,26 +55711,26 @@
         </is>
       </c>
       <c r="D1089" s="15" t="n">
-        <v>155420.57</v>
+        <v>228771.5</v>
       </c>
       <c r="E1089" s="15" t="n">
-        <v>2615297.18</v>
+        <v>2860464.67</v>
       </c>
       <c r="F1089" s="16" t="n">
-        <v>0.7308</v>
+        <v>0.7504</v>
       </c>
       <c r="G1089" s="16" t="n">
-        <v>0.6642</v>
+        <v>0.6845</v>
       </c>
       <c r="H1089" s="16" t="n"/>
       <c r="I1089" s="16" t="n">
-        <v>0.0295</v>
+        <v>0.0276</v>
       </c>
       <c r="J1089" s="19" t="n">
-        <v>7659</v>
+        <v>10656</v>
       </c>
       <c r="K1089" s="19" t="n">
-        <v>24967</v>
+        <v>39552</v>
       </c>
       <c r="L1089" s="31" t="n">
         <v>0</v>
@@ -56257,26 +56257,26 @@
         </is>
       </c>
       <c r="D1102" s="9" t="n">
-        <v>74236517.09999999</v>
+        <v>97276496.69</v>
       </c>
       <c r="E1102" s="9" t="n">
-        <v>334462876.84</v>
+        <v>444710231.06</v>
       </c>
       <c r="F1102" s="10" t="n">
-        <v>0.1713</v>
+        <v>0.1584</v>
       </c>
       <c r="G1102" s="10" t="n">
-        <v>0.1128</v>
+        <v>0.0997</v>
       </c>
       <c r="H1102" s="10" t="n"/>
       <c r="I1102" s="10" t="n">
-        <v>0.0968</v>
+        <v>0.1006</v>
       </c>
       <c r="J1102" s="13" t="n">
-        <v>1810079</v>
+        <v>2329488</v>
       </c>
       <c r="K1102" s="13" t="n">
-        <v>3633079</v>
+        <v>4639002</v>
       </c>
       <c r="L1102" s="32" t="n">
         <v>0</v>
@@ -59827,26 +59827,26 @@
         </is>
       </c>
       <c r="D1187" s="15" t="n">
-        <v>10429384.86</v>
+        <v>13541589.95</v>
       </c>
       <c r="E1187" s="15" t="n">
-        <v>182922141.45</v>
+        <v>239009617.82</v>
       </c>
       <c r="F1187" s="16" t="n">
-        <v>0.4665</v>
+        <v>0.4579</v>
       </c>
       <c r="G1187" s="16" t="n">
-        <v>0.3874</v>
+        <v>0.3791</v>
       </c>
       <c r="H1187" s="16" t="n"/>
       <c r="I1187" s="16" t="n">
-        <v>0.0273</v>
+        <v>0.0297</v>
       </c>
       <c r="J1187" s="19" t="n">
-        <v>736977</v>
+        <v>941203</v>
       </c>
       <c r="K1187" s="19" t="n">
-        <v>1220851</v>
+        <v>1549179</v>
       </c>
       <c r="L1187" s="31" t="n">
         <v>0</v>
@@ -59869,26 +59869,26 @@
         </is>
       </c>
       <c r="D1188" s="9" t="n">
-        <v>17321110.88</v>
+        <v>23063810.81</v>
       </c>
       <c r="E1188" s="9" t="n">
-        <v>8787233.859999999</v>
+        <v>12050164.86</v>
       </c>
       <c r="F1188" s="10" t="n">
-        <v>0.0488</v>
+        <v>0.0296</v>
       </c>
       <c r="G1188" s="10" t="n">
-        <v>0.008399999999999999</v>
+        <v>-0.0112</v>
       </c>
       <c r="H1188" s="10" t="n"/>
       <c r="I1188" s="10" t="n">
-        <v>0.3124</v>
+        <v>0.3182</v>
       </c>
       <c r="J1188" s="13" t="n">
-        <v>78658</v>
+        <v>102535</v>
       </c>
       <c r="K1188" s="13" t="n">
-        <v>317790</v>
+        <v>423974</v>
       </c>
       <c r="L1188" s="32" t="n">
         <v>0</v>
@@ -59911,26 +59911,26 @@
         </is>
       </c>
       <c r="D1189" s="15" t="n">
-        <v>11335832.97</v>
+        <v>15470906.95</v>
       </c>
       <c r="E1189" s="15" t="n">
-        <v>11018336.63</v>
+        <v>15399606.21</v>
       </c>
       <c r="F1189" s="16" t="n">
-        <v>0.022</v>
+        <v>0.0267</v>
       </c>
       <c r="G1189" s="16" t="n">
-        <v>-0.0282</v>
+        <v>-0.0236</v>
       </c>
       <c r="H1189" s="16" t="n"/>
       <c r="I1189" s="16" t="n">
-        <v>0.2467</v>
+        <v>0.2512</v>
       </c>
       <c r="J1189" s="19" t="n">
-        <v>113869</v>
+        <v>149747</v>
       </c>
       <c r="K1189" s="19" t="n">
-        <v>286932</v>
+        <v>381136</v>
       </c>
       <c r="L1189" s="31" t="n">
         <v>0</v>
@@ -59953,26 +59953,26 @@
         </is>
       </c>
       <c r="D1190" s="9" t="n">
-        <v>9502769.300000001</v>
+        <v>12463040.53</v>
       </c>
       <c r="E1190" s="9" t="n">
-        <v>13573874.66</v>
+        <v>18409126.48</v>
       </c>
       <c r="F1190" s="10" t="n">
-        <v>0.09379999999999999</v>
+        <v>0.0818</v>
       </c>
       <c r="G1190" s="10" t="n">
-        <v>0.0394</v>
+        <v>0.0269</v>
       </c>
       <c r="H1190" s="10" t="n"/>
       <c r="I1190" s="10" t="n">
-        <v>0.2013</v>
+        <v>0.2049</v>
       </c>
       <c r="J1190" s="13" t="n">
-        <v>132657</v>
+        <v>173839</v>
       </c>
       <c r="K1190" s="13" t="n">
-        <v>296106</v>
+        <v>383703</v>
       </c>
       <c r="L1190" s="32" t="n">
         <v>0</v>
@@ -59995,26 +59995,26 @@
         </is>
       </c>
       <c r="D1191" s="15" t="n">
-        <v>6487649.5</v>
+        <v>8419647.26</v>
       </c>
       <c r="E1191" s="15" t="n">
-        <v>13719664.03</v>
+        <v>21696895.32</v>
       </c>
       <c r="F1191" s="16" t="n">
-        <v>0.0979</v>
+        <v>0.0872</v>
       </c>
       <c r="G1191" s="16" t="n">
-        <v>0.0358</v>
+        <v>0.0241</v>
       </c>
       <c r="H1191" s="16" t="n"/>
       <c r="I1191" s="16" t="n">
-        <v>0.1646</v>
+        <v>0.1672</v>
       </c>
       <c r="J1191" s="19" t="n">
-        <v>129319</v>
+        <v>169889</v>
       </c>
       <c r="K1191" s="19" t="n">
-        <v>260750</v>
+        <v>345740</v>
       </c>
       <c r="L1191" s="31" t="n">
         <v>0</v>
@@ -60037,26 +60037,26 @@
         </is>
       </c>
       <c r="D1192" s="9" t="n">
-        <v>10010303.1</v>
+        <v>12488624.76</v>
       </c>
       <c r="E1192" s="9" t="n">
-        <v>35798453.17</v>
+        <v>47155271.58</v>
       </c>
       <c r="F1192" s="10" t="n">
-        <v>0.1718</v>
+        <v>0.1658</v>
       </c>
       <c r="G1192" s="10" t="n">
-        <v>0.1054</v>
+        <v>0.0983</v>
       </c>
       <c r="H1192" s="10" t="n"/>
       <c r="I1192" s="10" t="n">
-        <v>0.1182</v>
+        <v>0.1205</v>
       </c>
       <c r="J1192" s="13" t="n">
-        <v>261795</v>
+        <v>338387</v>
       </c>
       <c r="K1192" s="13" t="n">
-        <v>527524</v>
+        <v>655665</v>
       </c>
       <c r="L1192" s="32" t="n">
         <v>0</v>
@@ -60079,26 +60079,26 @@
         </is>
       </c>
       <c r="D1193" s="15" t="n">
-        <v>9149466.51</v>
+        <v>11828876.43</v>
       </c>
       <c r="E1193" s="15" t="n">
-        <v>68643173.05</v>
+        <v>90989548.8</v>
       </c>
       <c r="F1193" s="16" t="n">
-        <v>0.3835</v>
+        <v>0.3624</v>
       </c>
       <c r="G1193" s="16" t="n">
-        <v>0.3108</v>
+        <v>0.2892</v>
       </c>
       <c r="H1193" s="16" t="n"/>
       <c r="I1193" s="16" t="n">
-        <v>0.0659</v>
+        <v>0.0689</v>
       </c>
       <c r="J1193" s="19" t="n">
-        <v>356804</v>
+        <v>453888</v>
       </c>
       <c r="K1193" s="19" t="n">
-        <v>723126</v>
+        <v>899605</v>
       </c>
       <c r="L1193" s="31" t="n">
         <v>0</v>
@@ -60583,26 +60583,26 @@
         </is>
       </c>
       <c r="D1205" s="15" t="n">
-        <v>2984297</v>
+        <v>4646574.42</v>
       </c>
       <c r="E1205" s="15" t="n">
-        <v>7942844.01</v>
+        <v>11289991.74</v>
       </c>
       <c r="F1205" s="16" t="n">
-        <v>0.2728</v>
+        <v>0.2341</v>
       </c>
       <c r="G1205" s="16" t="n">
-        <v>0.2133</v>
+        <v>0.1758</v>
       </c>
       <c r="H1205" s="16" t="n"/>
       <c r="I1205" s="16" t="n">
-        <v>0.0834</v>
+        <v>0.103</v>
       </c>
       <c r="J1205" s="19" t="n">
-        <v>51820</v>
+        <v>73865</v>
       </c>
       <c r="K1205" s="19" t="n">
-        <v>75580</v>
+        <v>111678</v>
       </c>
       <c r="L1205" s="31" t="n">
         <v>0</v>
@@ -63859,26 +63859,26 @@
         </is>
       </c>
       <c r="D1283" s="15" t="n">
-        <v>165373.44</v>
+        <v>243890.18</v>
       </c>
       <c r="E1283" s="15" t="n">
-        <v>2095456.54</v>
+        <v>2986584.8</v>
       </c>
       <c r="F1283" s="16" t="n">
-        <v>0.4392</v>
+        <v>0.5927</v>
       </c>
       <c r="G1283" s="16" t="n">
-        <v>0.3747</v>
+        <v>0.5232</v>
       </c>
       <c r="H1283" s="16" t="n"/>
       <c r="I1283" s="16" t="n">
-        <v>0.0189</v>
+        <v>0.0259</v>
       </c>
       <c r="J1283" s="19" t="n">
-        <v>11534</v>
+        <v>15993</v>
       </c>
       <c r="K1283" s="19" t="n">
-        <v>14314</v>
+        <v>19808</v>
       </c>
       <c r="L1283" s="31" t="n">
         <v>0</v>
@@ -63901,26 +63901,26 @@
         </is>
       </c>
       <c r="D1284" s="9" t="n">
-        <v>840038.26</v>
+        <v>1369656.14</v>
       </c>
       <c r="E1284" s="9" t="n">
-        <v>542849.8199999999</v>
+        <v>924648.9</v>
       </c>
       <c r="F1284" s="10" t="n">
-        <v>0.2094</v>
+        <v>0.1408</v>
       </c>
       <c r="G1284" s="10" t="n">
-        <v>0.156</v>
+        <v>0.0895</v>
       </c>
       <c r="H1284" s="10" t="n"/>
       <c r="I1284" s="10" t="n">
-        <v>0.2869</v>
+        <v>0.3027</v>
       </c>
       <c r="J1284" s="13" t="n">
-        <v>3290</v>
+        <v>5074</v>
       </c>
       <c r="K1284" s="13" t="n">
-        <v>8299</v>
+        <v>13085</v>
       </c>
       <c r="L1284" s="32" t="n">
         <v>0</v>
@@ -63943,26 +63943,26 @@
         </is>
       </c>
       <c r="D1285" s="15" t="n">
-        <v>723977.65</v>
+        <v>1087524.21</v>
       </c>
       <c r="E1285" s="15" t="n">
-        <v>548879.08</v>
+        <v>884828.58</v>
       </c>
       <c r="F1285" s="16" t="n">
-        <v>0.122</v>
+        <v>0.1529</v>
       </c>
       <c r="G1285" s="16" t="n">
-        <v>0.06560000000000001</v>
+        <v>0.0979</v>
       </c>
       <c r="H1285" s="16" t="n"/>
       <c r="I1285" s="16" t="n">
-        <v>0.1853</v>
+        <v>0.203</v>
       </c>
       <c r="J1285" s="19" t="n">
-        <v>5851</v>
+        <v>8632</v>
       </c>
       <c r="K1285" s="19" t="n">
-        <v>10002</v>
+        <v>15616</v>
       </c>
       <c r="L1285" s="31" t="n">
         <v>0</v>
@@ -63985,26 +63985,26 @@
         </is>
       </c>
       <c r="D1286" s="9" t="n">
-        <v>476299.71</v>
+        <v>780033.5</v>
       </c>
       <c r="E1286" s="9" t="n">
-        <v>698966.0600000001</v>
+        <v>1189362.37</v>
       </c>
       <c r="F1286" s="10" t="n">
-        <v>0.2752</v>
+        <v>0.16</v>
       </c>
       <c r="G1286" s="10" t="n">
-        <v>0.2143</v>
+        <v>0.101</v>
       </c>
       <c r="H1286" s="10" t="n"/>
       <c r="I1286" s="10" t="n">
-        <v>0.1217</v>
+        <v>0.1523</v>
       </c>
       <c r="J1286" s="13" t="n">
-        <v>6699</v>
+        <v>9836</v>
       </c>
       <c r="K1286" s="13" t="n">
-        <v>10317</v>
+        <v>16387</v>
       </c>
       <c r="L1286" s="32" t="n">
         <v>0</v>
@@ -64027,26 +64027,26 @@
         </is>
       </c>
       <c r="D1287" s="15" t="n">
-        <v>313742.91</v>
+        <v>480461.42</v>
       </c>
       <c r="E1287" s="15" t="n">
-        <v>887407.13</v>
+        <v>1187501.54</v>
       </c>
       <c r="F1287" s="16" t="n">
-        <v>0.4036</v>
+        <v>0.3725</v>
       </c>
       <c r="G1287" s="16" t="n">
-        <v>0.3392</v>
+        <v>0.3092</v>
       </c>
       <c r="H1287" s="16" t="n"/>
       <c r="I1287" s="16" t="n">
-        <v>0.0814</v>
+        <v>0.1056</v>
       </c>
       <c r="J1287" s="19" t="n">
-        <v>6022</v>
+        <v>8521</v>
       </c>
       <c r="K1287" s="19" t="n">
-        <v>9257</v>
+        <v>13726</v>
       </c>
       <c r="L1287" s="31" t="n">
         <v>0</v>
@@ -64069,26 +64069,26 @@
         </is>
       </c>
       <c r="D1288" s="9" t="n">
-        <v>285126.79</v>
+        <v>427491.76</v>
       </c>
       <c r="E1288" s="9" t="n">
-        <v>1368909.74</v>
+        <v>1865601.49</v>
       </c>
       <c r="F1288" s="10" t="n">
-        <v>0.4798</v>
+        <v>0.3725</v>
       </c>
       <c r="G1288" s="10" t="n">
-        <v>0.4102</v>
+        <v>0.3027</v>
       </c>
       <c r="H1288" s="10" t="n"/>
       <c r="I1288" s="10" t="n">
-        <v>0.0523</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="J1288" s="13" t="n">
-        <v>9830</v>
+        <v>13909</v>
       </c>
       <c r="K1288" s="13" t="n">
-        <v>12678</v>
+        <v>18127</v>
       </c>
       <c r="L1288" s="32" t="n">
         <v>0</v>
@@ -64111,26 +64111,26 @@
         </is>
       </c>
       <c r="D1289" s="15" t="n">
-        <v>179738.23</v>
+        <v>257517.22</v>
       </c>
       <c r="E1289" s="15" t="n">
-        <v>1800375.63</v>
+        <v>2251464.06</v>
       </c>
       <c r="F1289" s="16" t="n">
-        <v>0.4596</v>
+        <v>0.4702</v>
       </c>
       <c r="G1289" s="16" t="n">
-        <v>0.3926</v>
+        <v>0.4018</v>
       </c>
       <c r="H1289" s="16" t="n"/>
       <c r="I1289" s="16" t="n">
-        <v>0.0299</v>
+        <v>0.0455</v>
       </c>
       <c r="J1289" s="19" t="n">
-        <v>8594</v>
+        <v>11900</v>
       </c>
       <c r="K1289" s="19" t="n">
-        <v>10713</v>
+        <v>14929</v>
       </c>
       <c r="L1289" s="31" t="n">
         <v>0</v>
@@ -64891,22 +64891,22 @@
         </is>
       </c>
       <c r="B12" s="33" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C12" s="34" t="n">
-        <v>1072027977.53</v>
+        <v>1121495617.070001</v>
       </c>
       <c r="D12" s="35" t="n">
-        <v>0.01175022377589718</v>
+        <v>0.01629961006691922</v>
       </c>
       <c r="E12" s="35" t="n">
-        <v>-0.002391850907225632</v>
+        <v>0.003868149360494195</v>
       </c>
       <c r="F12" s="35" t="n">
-        <v>-0.003002532195100902</v>
+        <v>-0.002597900886440029</v>
       </c>
       <c r="G12" s="33" t="n">
-        <v>6.106812878752706</v>
+        <v>64.66050246934223</v>
       </c>
       <c r="H12" s="36" t="n"/>
       <c r="I12" s="36" t="n"/>
@@ -64950,7 +64950,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-22 16:31 UTC</t>
+          <t>2026-10-23 16:21 UTC</t>
         </is>
       </c>
     </row>
@@ -64986,7 +64986,7 @@
       </c>
       <c r="B4" s="38" t="inlineStr">
         <is>
-          <t>477 (2025 post: from 2026-01-10, 2025 pre: from 2025-07-31, 2025 reg: from 2025-09-04, 2026 pre: from 2026-08-06, 2026 reg: from 2026-09-09)</t>
+          <t>478 (2025 post: from 2026-01-10, 2025 pre: from 2025-07-31, 2025 reg: from 2025-09-04, 2026 pre: from 2026-08-06, 2026 reg: from 2026-09-09)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-26 01:24 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Weekly'!$A$6:$A$70</f>
+              <f>'Weekly'!$A$6:$A$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly'!$D$6:$D$70</f>
+              <f>'Weekly'!$D$6:$D$71</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -404,12 +404,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Weekly'!$A$6:$A$70</f>
+              <f>'Weekly'!$A$6:$A$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly'!$G$6:$G$70</f>
+              <f>'Weekly'!$G$6:$G$71</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -440,12 +440,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Weekly'!$A$6:$A$70</f>
+              <f>'Weekly'!$A$6:$A$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly'!$K$6:$K$70</f>
+              <f>'Weekly'!$K$6:$K$71</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -527,12 +527,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Weekly'!$A$6:$A$70</f>
+              <f>'Weekly'!$A$6:$A$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly'!$B$6:$B$70</f>
+              <f>'Weekly'!$B$6:$B$71</f>
             </numRef>
           </val>
         </ser>
@@ -555,12 +555,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Weekly'!$A$6:$A$70</f>
+              <f>'Weekly'!$A$6:$A$71</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly'!$E$6:$E$70</f>
+              <f>'Weekly'!$E$6:$E$71</f>
             </numRef>
           </val>
         </ser>
@@ -889,7 +889,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>72</row>
+      <row>73</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="3240000"/>
@@ -911,7 +911,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>91</row>
+      <row>92</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="3240000"/>
@@ -1271,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA70"/>
+  <dimension ref="A1:AA71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5933,13 +5933,13 @@
         <v>46320</v>
       </c>
       <c r="B70" s="9" t="n">
-        <v>671730107.84</v>
+        <v>847609310.39</v>
       </c>
       <c r="C70" s="9" t="n">
-        <v>27463157.96</v>
+        <v>31476670.69</v>
       </c>
       <c r="D70" s="10" t="n">
-        <v>0.04088</v>
+        <v>0.03714</v>
       </c>
       <c r="E70" s="9" t="n">
         <v>190635589.58</v>
@@ -5956,31 +5956,31 @@
         </is>
       </c>
       <c r="I70" s="9" t="n">
-        <v>862365697.42</v>
+        <v>1038244899.97</v>
       </c>
       <c r="J70" s="9" t="n">
-        <v>48544677.93</v>
+        <v>52558190.67</v>
       </c>
       <c r="K70" s="12" t="n">
-        <v>0.05629</v>
+        <v>0.05062</v>
       </c>
       <c r="L70" s="13" t="n">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="M70" s="13" t="n">
-        <v>24</v>
+        <v>-40</v>
       </c>
       <c r="N70" s="9" t="n">
-        <v>114230395.94</v>
+        <v>280748074.82</v>
       </c>
       <c r="O70" s="10" t="n">
-        <v>0.08209</v>
+        <v>0.04804</v>
       </c>
       <c r="P70" s="9" t="n">
-        <v>260214508.82</v>
+        <v>268456984.88</v>
       </c>
       <c r="Q70" s="10" t="n">
-        <v>0.02988</v>
+        <v>0.0285</v>
       </c>
       <c r="R70" s="9" t="n">
         <v>42293945.77</v>
@@ -5989,10 +5989,10 @@
         <v>-0.08223</v>
       </c>
       <c r="T70" s="9" t="n">
-        <v>32131392.55</v>
+        <v>33250440.17</v>
       </c>
       <c r="U70" s="10" t="n">
-        <v>0.04579</v>
+        <v>0.04511</v>
       </c>
       <c r="V70" s="9" t="n">
         <v>222859864.76</v>
@@ -6004,6 +6004,53 @@
       <c r="Y70" s="10" t="n"/>
       <c r="Z70" s="9" t="n"/>
       <c r="AA70" s="10" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B71" s="15" t="n"/>
+      <c r="C71" s="15" t="n"/>
+      <c r="D71" s="16" t="n"/>
+      <c r="E71" s="15" t="n">
+        <v>876862.78</v>
+      </c>
+      <c r="F71" s="15" t="n">
+        <v>877292</v>
+      </c>
+      <c r="G71" s="16" t="n">
+        <v>1.00049</v>
+      </c>
+      <c r="H71" s="17" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="I71" s="15" t="n">
+        <v>876862.78</v>
+      </c>
+      <c r="J71" s="15" t="n">
+        <v>877292</v>
+      </c>
+      <c r="K71" s="18" t="n">
+        <v>1.00049</v>
+      </c>
+      <c r="L71" s="19" t="n"/>
+      <c r="M71" s="19" t="n"/>
+      <c r="N71" s="15" t="n"/>
+      <c r="O71" s="16" t="n"/>
+      <c r="P71" s="15" t="n"/>
+      <c r="Q71" s="16" t="n"/>
+      <c r="R71" s="15" t="n"/>
+      <c r="S71" s="16" t="n"/>
+      <c r="T71" s="15" t="n"/>
+      <c r="U71" s="16" t="n"/>
+      <c r="V71" s="15" t="n"/>
+      <c r="W71" s="16" t="n"/>
+      <c r="X71" s="15" t="n"/>
+      <c r="Y71" s="16" t="n"/>
+      <c r="Z71" s="15" t="n"/>
+      <c r="AA71" s="16" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -6020,7 +6067,7 @@
     <mergeCell ref="N4:O4"/>
     <mergeCell ref="T4:U4"/>
   </mergeCells>
-  <conditionalFormatting sqref="C6:C70">
+  <conditionalFormatting sqref="C6:C71">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6028,7 +6075,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D6:D70">
+  <conditionalFormatting sqref="D6:D71">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6036,7 +6083,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F6:F70">
+  <conditionalFormatting sqref="F6:F71">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6044,7 +6091,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G6:G70">
+  <conditionalFormatting sqref="G6:G71">
     <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6052,7 +6099,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J6:J70">
+  <conditionalFormatting sqref="J6:J71">
     <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6060,7 +6107,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K70">
+  <conditionalFormatting sqref="K6:K71">
     <cfRule type="cellIs" priority="11" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6068,7 +6115,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M6:M70">
+  <conditionalFormatting sqref="M6:M71">
     <cfRule type="cellIs" priority="13" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6076,7 +6123,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O6:O70">
+  <conditionalFormatting sqref="O6:O71">
     <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6084,7 +6131,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q6:Q70">
+  <conditionalFormatting sqref="Q6:Q71">
     <cfRule type="cellIs" priority="17" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6092,7 +6139,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S6:S70">
+  <conditionalFormatting sqref="S6:S71">
     <cfRule type="cellIs" priority="19" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6100,7 +6147,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U6:U70">
+  <conditionalFormatting sqref="U6:U71">
     <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6108,7 +6155,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W6:W70">
+  <conditionalFormatting sqref="W6:W71">
     <cfRule type="cellIs" priority="23" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6116,7 +6163,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y6:Y70">
+  <conditionalFormatting sqref="Y6:Y71">
     <cfRule type="cellIs" priority="25" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -6124,7 +6171,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA6:AA70">
+  <conditionalFormatting sqref="AA6:AA71">
     <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -7392,13 +7439,13 @@
         <v>46296</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>2950705527.98</v>
+        <v>3126584730.54</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>70422549.06999999</v>
+        <v>74436061.8</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.02387</v>
+        <v>0.02381</v>
       </c>
       <c r="E20" s="9" t="n">
         <v>818307638.95</v>
@@ -7415,31 +7462,31 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>3769013166.94</v>
+        <v>3944892369.49</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>209146969.88</v>
+        <v>213160482.62</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.05549</v>
+        <v>0.05403</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>820</v>
+        <v>835</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="N20" s="9" t="n">
-        <v>1121495617.07</v>
+        <v>1288013295.95</v>
       </c>
       <c r="O20" s="10" t="n">
-        <v>0.0163</v>
+        <v>0.01738</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>350929392.97</v>
+        <v>359171869.02</v>
       </c>
       <c r="Q20" s="10" t="n">
-        <v>0.03084</v>
+        <v>0.02979</v>
       </c>
       <c r="R20" s="9" t="n">
         <v>331548311.27</v>
@@ -7448,10 +7495,10 @@
         <v>0.03254</v>
       </c>
       <c r="T20" s="9" t="n">
-        <v>117066611.04</v>
+        <v>118185658.66</v>
       </c>
       <c r="U20" s="10" t="n">
-        <v>0.02743</v>
+        <v>0.02741</v>
       </c>
       <c r="V20" s="9" t="n">
         <v>1029665595.64</v>
@@ -7984,16 +8031,16 @@
         <v>-0.0249</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>114230395.95</v>
+        <v>280748074.85</v>
       </c>
       <c r="I11" s="16" t="n">
-        <v>0.08210000000000001</v>
+        <v>0.048</v>
       </c>
       <c r="J11" s="19" t="n">
-        <v>631</v>
+        <v>125</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>3.4</v>
+        <v>0.9</v>
       </c>
       <c r="L11" s="15" t="n">
         <v>42124229.67</v>
@@ -8558,14 +8605,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-25 15:55 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 01:24 UTC.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>Season 2026 to date  ·  94 games</t>
+          <t>Season 2026 to date  ·  105 games</t>
         </is>
       </c>
     </row>
@@ -8628,31 +8675,31 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>1094486670.650001</v>
+        <v>1177587505.920001</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.02639592486114302</v>
+        <v>0.02652917218715998</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.001453189228019952</v>
+        <v>0.001565361827238364</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0.04955673129564912</v>
+        <v>0.04115042953902844</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>0.006749446889558886</v>
+        <v>0.006616802309398866</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>428.0728440609023</v>
+        <v>345.3362722962958</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>-0.008887055809646919</v>
+        <v>-0.006844318350949435</v>
       </c>
       <c r="I6" s="29" t="n">
-        <v>-6.11880545588273</v>
+        <v>-5.798445239256158</v>
       </c>
       <c r="J6" s="15" t="n">
-        <v>34124364.63999999</v>
+        <v>36746338.99999999</v>
       </c>
     </row>
     <row r="7">
@@ -8662,31 +8709,31 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>304912384.6100002</v>
+        <v>330209434.9200001</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.0651479548310499</v>
+        <v>0.0606204215056715</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>0.03595118995911224</v>
+        <v>0.03136627517172338</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.08985606126429682</v>
+        <v>0.07747731461304155</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.001825606710714355</v>
+        <v>0.001117843520402102</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>880.3045455358247</v>
+        <v>763.5947109263946</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>0.0009134536781841853</v>
+        <v>0.0008831874703495228</v>
       </c>
       <c r="I7" s="30" t="n">
-        <v>-9.453304968098424</v>
+        <v>-7.946091892656172</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>11128069</v>
+        <v>12074993.91</v>
       </c>
     </row>
     <row r="8">
@@ -8696,31 +8743,31 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>162423843.45</v>
+        <v>174260918.48</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.01213908695989551</v>
+        <v>0.01563732863208081</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>-0.01556039720718724</v>
+        <v>-0.01209220907579367</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>-0.05680795482964646</v>
+        <v>-0.04789334495583976</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>-0.009343761331756351</v>
+        <v>-0.009910783396611922</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>-474.6419349789011</v>
+        <v>-379.8256155922784</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>0.004044327699925969</v>
+        <v>0.004872361828775336</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>4.036919181212047</v>
+        <v>3.150992547510586</v>
       </c>
       <c r="J8" s="15" t="n">
-        <v>5623820.890000002</v>
+        <v>6040218.430000002</v>
       </c>
     </row>
     <row r="9">
@@ -8730,31 +8777,31 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>295974023.85</v>
+        <v>326085843.4999999</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>-0.001470542192650604</v>
+        <v>0.0001533715154978737</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>-0.02577057172377259</v>
+        <v>-0.02350590162924385</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>-0.03478429504223865</v>
+        <v>-0.03152201082195837</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>-0.00871848457142016</v>
+        <v>-0.008992339212826344</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-260.6581047081849</v>
+        <v>-225.2967160913202</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-0.01950377115797173</v>
+        <v>-0.01814844593178638</v>
       </c>
       <c r="I9" s="30" t="n">
-        <v>1.656232582738445</v>
+        <v>1.243153871491366</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>7335037.760000002</v>
+        <v>7862893.960000002</v>
       </c>
     </row>
     <row r="10">
@@ -8764,31 +8811,31 @@
         </is>
       </c>
       <c r="B10" s="15" t="n">
-        <v>131157655.96</v>
+        <v>140584131.19</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>0.05187481371331455</v>
+        <v>0.05207653465600221</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>0.02796520594359058</v>
+        <v>0.02834885912275345</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>0.0579103549052363</v>
+        <v>0.05684385622285867</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>0.007446872488217138</v>
+        <v>0.007493619724425039</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>504.6348241701916</v>
+        <v>493.5023649843363</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>0.0189215400014692</v>
+        <v>0.01993339325894341</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>-3.786675211426286</v>
+        <v>-3.65885315866659</v>
       </c>
       <c r="J10" s="15" t="n">
-        <v>3135928.109999998</v>
+        <v>3335734.649999999</v>
       </c>
     </row>
     <row r="11">
@@ -8798,31 +8845,31 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>33025688.69000001</v>
+        <v>39770112.08</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.006287045879617653</v>
+        <v>0.001432955227417087</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>-0.01575331539286063</v>
+        <v>-0.0193504483581028</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0.04185210604019338</v>
+        <v>0.05228542659668419</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.003503934173786229</v>
+        <v>0.003420810626991917</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>383.4817186640715</v>
+        <v>488.6461596969227</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-0.03419908744734319</v>
+        <v>-0.03932289993345896</v>
       </c>
       <c r="I11" s="30" t="n">
-        <v>-3.51805540179019</v>
+        <v>-4.159202510328733</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>727898.11</v>
+        <v>826558.2899999997</v>
       </c>
     </row>
     <row r="12">
@@ -8832,31 +8879,31 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>2021980267.209998</v>
+        <v>2188497946.089999</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>0.0283396702575479</v>
+        <v>0.02806078372141843</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>0.002742483114165862</v>
+        <v>0.002579156882502222</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>0.02907683462791388</v>
+        <v>0.02503314364135891</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>0.0004443182116283221</v>
+        <v>9.222376466407526e-05</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>286.3251641628556</v>
+        <v>249.4091987669484</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>-0.006514635616847445</v>
+        <v>-0.005237662358274827</v>
       </c>
       <c r="I12" s="29" t="n">
-        <v>-3.690635906225312</v>
+        <v>-3.498465115538365</v>
       </c>
       <c r="J12" s="15" t="n">
-        <v>62075118.50999995</v>
+        <v>66886738.23999994</v>
       </c>
     </row>
     <row r="14">
@@ -9236,11 +9283,11 @@
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>W06 (Mon) + W07 (Thu)</t>
+          <t>W07 (Thu/Sun) + W06 (Mon)</t>
         </is>
       </c>
       <c r="D26" s="19" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
@@ -9248,25 +9295,25 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>114230395.95</v>
+        <v>280748074.85</v>
       </c>
       <c r="G26" s="16" t="n">
-        <v>0.08210000000000001</v>
+        <v>0.048</v>
       </c>
       <c r="H26" s="16" t="n">
-        <v>0.0601</v>
+        <v>0.0248</v>
       </c>
       <c r="I26" s="15" t="n">
-        <v>-6864385.52</v>
+        <v>-6963618.34</v>
       </c>
       <c r="J26" s="15" t="n">
-        <v>28774143.02</v>
+        <v>68004756.01000001</v>
       </c>
       <c r="K26" s="16" t="n">
-        <v>0.06610000000000001</v>
+        <v>0.0111</v>
       </c>
       <c r="L26" s="16" t="n">
-        <v>0.003</v>
+        <v>-0.0014</v>
       </c>
     </row>
     <row r="27">
@@ -64891,22 +64938,22 @@
         </is>
       </c>
       <c r="B12" s="33" t="n">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="C12" s="34" t="n">
-        <v>1121495617.070001</v>
+        <v>1288013295.950002</v>
       </c>
       <c r="D12" s="35" t="n">
-        <v>0.01629961006691922</v>
+        <v>0.01738231648725858</v>
       </c>
       <c r="E12" s="35" t="n">
-        <v>0.003868149360494195</v>
+        <v>-0.0004084194164633934</v>
       </c>
       <c r="F12" s="35" t="n">
-        <v>-0.002597900886440029</v>
+        <v>-0.002860618263766299</v>
       </c>
       <c r="G12" s="33" t="n">
-        <v>64.66050246934223</v>
+        <v>24.52198847302906</v>
       </c>
       <c r="H12" s="36" t="n"/>
       <c r="I12" s="36" t="n"/>
@@ -64950,7 +64997,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-25 15:55 UTC</t>
+          <t>2026-10-26 01:24 UTC</t>
         </is>
       </c>
     </row>
@@ -64986,7 +65033,7 @@
       </c>
       <c r="B4" s="38" t="inlineStr">
         <is>
-          <t>478 (2025 post: from 2026-01-10, 2025 pre: from 2025-07-31, 2025 reg: from 2025-09-04, 2026 pre: from 2026-08-06, 2026 reg: from 2026-09-09)</t>
+          <t>489 (2025 post: from 2026-01-10, 2025 pre: from 2025-07-31, 2025 reg: from 2025-09-04, 2026 pre: from 2026-08-06, 2026 reg: from 2026-09-09)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-26 06:37 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -5933,13 +5933,13 @@
         <v>46320</v>
       </c>
       <c r="B70" s="9" t="n">
-        <v>847609310.39</v>
+        <v>925649567.11</v>
       </c>
       <c r="C70" s="9" t="n">
-        <v>31476670.69</v>
+        <v>43771811.93</v>
       </c>
       <c r="D70" s="10" t="n">
-        <v>0.03714</v>
+        <v>0.04729</v>
       </c>
       <c r="E70" s="9" t="n">
         <v>190635589.58</v>
@@ -5956,31 +5956,31 @@
         </is>
       </c>
       <c r="I70" s="9" t="n">
-        <v>1038244899.97</v>
+        <v>1116285156.69</v>
       </c>
       <c r="J70" s="9" t="n">
-        <v>52558190.67</v>
+        <v>64853331.9</v>
       </c>
       <c r="K70" s="12" t="n">
-        <v>0.05062</v>
+        <v>0.0581</v>
       </c>
       <c r="L70" s="13" t="n">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="M70" s="13" t="n">
-        <v>-40</v>
+        <v>194</v>
       </c>
       <c r="N70" s="9" t="n">
-        <v>280748074.82</v>
+        <v>329514184.7</v>
       </c>
       <c r="O70" s="10" t="n">
-        <v>0.04804</v>
+        <v>0.0723</v>
       </c>
       <c r="P70" s="9" t="n">
-        <v>268456984.88</v>
+        <v>295271366.54</v>
       </c>
       <c r="Q70" s="10" t="n">
-        <v>0.0285</v>
+        <v>0.0321</v>
       </c>
       <c r="R70" s="9" t="n">
         <v>42293945.77</v>
@@ -5989,10 +5989,10 @@
         <v>-0.08223</v>
       </c>
       <c r="T70" s="9" t="n">
-        <v>33250440.17</v>
+        <v>35710205.34</v>
       </c>
       <c r="U70" s="10" t="n">
-        <v>0.04511</v>
+        <v>0.04564</v>
       </c>
       <c r="V70" s="9" t="n">
         <v>222859864.76</v>
@@ -7439,13 +7439,13 @@
         <v>46296</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>3126584730.54</v>
+        <v>3204624987.25</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>74436061.8</v>
+        <v>86731203.04000001</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.02381</v>
+        <v>0.02706</v>
       </c>
       <c r="E20" s="9" t="n">
         <v>818307638.95</v>
@@ -7462,31 +7462,31 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>3944892369.49</v>
+        <v>4022932626.21</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>213160482.62</v>
+        <v>225455623.85</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.05403</v>
+        <v>0.05604</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>835</v>
+        <v>844</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>119</v>
+        <v>179</v>
       </c>
       <c r="N20" s="9" t="n">
-        <v>1288013295.95</v>
+        <v>1336779405.83</v>
       </c>
       <c r="O20" s="10" t="n">
-        <v>0.01738</v>
+        <v>0.02448</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>359171869.02</v>
+        <v>385986250.68</v>
       </c>
       <c r="Q20" s="10" t="n">
-        <v>0.02979</v>
+        <v>0.03245</v>
       </c>
       <c r="R20" s="9" t="n">
         <v>331548311.27</v>
@@ -7495,10 +7495,10 @@
         <v>0.03254</v>
       </c>
       <c r="T20" s="9" t="n">
-        <v>118185658.66</v>
+        <v>120645423.84</v>
       </c>
       <c r="U20" s="10" t="n">
-        <v>0.02741</v>
+        <v>0.02793</v>
       </c>
       <c r="V20" s="9" t="n">
         <v>1029665595.64</v>
@@ -8031,16 +8031,16 @@
         <v>-0.0249</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>280748074.85</v>
+        <v>329514184.73</v>
       </c>
       <c r="I11" s="16" t="n">
-        <v>0.048</v>
+        <v>0.0723</v>
       </c>
       <c r="J11" s="19" t="n">
-        <v>125</v>
+        <v>638</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>0.9</v>
+        <v>-2.1</v>
       </c>
       <c r="L11" s="15" t="n">
         <v>42124229.67</v>
@@ -8605,14 +8605,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 01:24 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 06:37 UTC.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>Season 2026 to date  ·  105 games</t>
+          <t>Season 2026 to date  ·  106 games</t>
         </is>
       </c>
     </row>
@@ -8675,31 +8675,31 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>1177587505.920001</v>
+        <v>1203063512.840001</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.02652917218715998</v>
+        <v>0.03325192332993666</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.001565361827238364</v>
+        <v>0.008252447276505826</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0.04115042953902844</v>
+        <v>0.05907392792828259</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>0.006616802309398866</v>
+        <v>0.00685817135234109</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>345.3362722962958</v>
+        <v>522.157565759415</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>-0.006844318350949435</v>
+        <v>-0.002728430564084517</v>
       </c>
       <c r="I6" s="29" t="n">
-        <v>-5.798445239256158</v>
+        <v>-6.379054876118246</v>
       </c>
       <c r="J6" s="15" t="n">
-        <v>36746338.99999999</v>
+        <v>37594946.86999998</v>
       </c>
     </row>
     <row r="7">
@@ -8709,31 +8709,31 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>330209434.9200001</v>
+        <v>338221215.0100002</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.0606204215056715</v>
+        <v>0.05889745943172436</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>0.03136627517172338</v>
+        <v>0.02963517264788861</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.07747731461304155</v>
+        <v>0.0706345135696871</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.001117843520402102</v>
+        <v>0.001158348085698785</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>763.5947109263946</v>
+        <v>694.7616548398831</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>0.0008831874703495228</v>
+        <v>0.002241268524286087</v>
       </c>
       <c r="I7" s="30" t="n">
-        <v>-7.946091892656172</v>
+        <v>-7.19147113293037</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>12074993.91</v>
+        <v>12371407.73</v>
       </c>
     </row>
     <row r="8">
@@ -8743,31 +8743,31 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>174260918.48</v>
+        <v>176833649.73</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.01563732863208081</v>
+        <v>0.01616389756341204</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>-0.01209220907579367</v>
+        <v>-0.01155224881191506</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>-0.04789334495583976</v>
+        <v>-0.04492103863558515</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>-0.009910783396611922</v>
+        <v>-0.009724010218640524</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>-379.8256155922784</v>
+        <v>-351.9702841694462</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>0.004872361828775336</v>
+        <v>0.004241608985911144</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>3.150992547510586</v>
+        <v>2.687823146813515</v>
       </c>
       <c r="J8" s="15" t="n">
-        <v>6040218.430000002</v>
+        <v>6126434.190000003</v>
       </c>
     </row>
     <row r="9">
@@ -8777,31 +8777,31 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>326085843.4999999</v>
+        <v>334745646.3</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>0.0001533715154978737</v>
+        <v>0.003432345252879835</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>-0.02350590162924385</v>
+        <v>-0.02013707922569628</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>-0.03152201082195837</v>
+        <v>-0.02569385834525074</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>-0.008992339212826344</v>
+        <v>-0.009132857521749537</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-225.2967160913202</v>
+        <v>-165.6100082350121</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-0.01814844593178638</v>
+        <v>-0.01645858797779771</v>
       </c>
       <c r="I9" s="30" t="n">
-        <v>1.243153871491366</v>
+        <v>0.9841026518185889</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>7862893.960000002</v>
+        <v>8043924.890000002</v>
       </c>
     </row>
     <row r="10">
@@ -8811,31 +8811,31 @@
         </is>
       </c>
       <c r="B10" s="15" t="n">
-        <v>140584131.19</v>
+        <v>143197099.59</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>0.05207653465600221</v>
+        <v>0.05256653578565681</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>0.02834885912275345</v>
+        <v>0.0288003182453285</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>0.05684385622285867</v>
+        <v>0.05856794778761725</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>0.007493619724425039</v>
+        <v>0.007491629752250475</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>493.5023649843363</v>
+        <v>510.7631803536677</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>0.01993339325894341</v>
+        <v>0.02000946746123027</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>-3.65885315866659</v>
+        <v>-3.737199077232269</v>
       </c>
       <c r="J10" s="15" t="n">
-        <v>3335734.649999999</v>
+        <v>3403253.419999999</v>
       </c>
     </row>
     <row r="11">
@@ -8845,31 +8845,31 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>39770112.08</v>
+        <v>41202932.5</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.001432955227417087</v>
+        <v>0.007043584094408801</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>-0.0193504483581028</v>
+        <v>-0.01350472396594588</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0.05228542659668419</v>
+        <v>0.06532371027830339</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.003420810626991917</v>
+        <v>0.003299162604491962</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>488.6461596969227</v>
+        <v>620.2454767381142</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-0.03932289993345896</v>
+        <v>-0.03523063322097789</v>
       </c>
       <c r="I11" s="30" t="n">
-        <v>-4.159202510328733</v>
+        <v>-4.851089022357201</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>826558.2899999997</v>
+        <v>846650.5499999997</v>
       </c>
     </row>
     <row r="12">
@@ -8879,31 +8879,31 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>2188497946.089999</v>
+        <v>2237264055.969998</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>0.02806078372141843</v>
+        <v>0.03207016230316717</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>0.002579156882502222</v>
+        <v>0.00658640367491677</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>0.02503314364135891</v>
+        <v>0.03221140168963393</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>9.222376466407526e-05</v>
+        <v>0.0002181690106810668</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>249.4091987669484</v>
+        <v>319.9323267895287</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>-0.005237662358274827</v>
+        <v>-0.002400850321273368</v>
       </c>
       <c r="I12" s="29" t="n">
-        <v>-3.498465115538365</v>
+        <v>-3.797477985579214</v>
       </c>
       <c r="J12" s="15" t="n">
-        <v>66886738.23999994</v>
+        <v>68386617.64999995</v>
       </c>
     </row>
     <row r="14">
@@ -9287,7 +9287,7 @@
         </is>
       </c>
       <c r="D26" s="19" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
@@ -9295,25 +9295,25 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>280748074.85</v>
+        <v>329514184.73</v>
       </c>
       <c r="G26" s="16" t="n">
-        <v>0.048</v>
+        <v>0.0723</v>
       </c>
       <c r="H26" s="16" t="n">
-        <v>0.0248</v>
+        <v>0.0487</v>
       </c>
       <c r="I26" s="15" t="n">
-        <v>-6963618.34</v>
+        <v>-16054663</v>
       </c>
       <c r="J26" s="15" t="n">
-        <v>68004756.01000001</v>
+        <v>83787151.59</v>
       </c>
       <c r="K26" s="16" t="n">
-        <v>0.0111</v>
+        <v>0.0635</v>
       </c>
       <c r="L26" s="16" t="n">
-        <v>-0.0014</v>
+        <v>-0.0002</v>
       </c>
     </row>
     <row r="27">
@@ -64938,22 +64938,22 @@
         </is>
       </c>
       <c r="B12" s="33" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C12" s="34" t="n">
-        <v>1288013295.950002</v>
+        <v>1336779405.830002</v>
       </c>
       <c r="D12" s="35" t="n">
-        <v>0.01738231648725858</v>
+        <v>0.02448205624448547</v>
       </c>
       <c r="E12" s="35" t="n">
-        <v>-0.0004084194164633934</v>
+        <v>0.01392706053118594</v>
       </c>
       <c r="F12" s="35" t="n">
-        <v>-0.002860618263766299</v>
+        <v>-0.002485049685752307</v>
       </c>
       <c r="G12" s="33" t="n">
-        <v>24.52198847302906</v>
+        <v>164.1211021693825</v>
       </c>
       <c r="H12" s="36" t="n"/>
       <c r="I12" s="36" t="n"/>
@@ -64997,7 +64997,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-26 01:24 UTC</t>
+          <t>2026-10-26 06:37 UTC</t>
         </is>
       </c>
     </row>
@@ -65033,7 +65033,7 @@
       </c>
       <c r="B4" s="38" t="inlineStr">
         <is>
-          <t>489 (2025 post: from 2026-01-10, 2025 pre: from 2025-07-31, 2025 reg: from 2025-09-04, 2026 pre: from 2026-08-06, 2026 reg: from 2026-09-09)</t>
+          <t>490 (2025 post: from 2026-01-10, 2025 pre: from 2025-07-31, 2025 reg: from 2025-09-04, 2026 pre: from 2026-08-06, 2026 reg: from 2026-09-09)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-26 07:26 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -5942,13 +5942,13 @@
         <v>0.04729</v>
       </c>
       <c r="E70" s="9" t="n">
-        <v>190635589.58</v>
+        <v>275422584.52</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>21081519.97</v>
+        <v>51631072.56</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>0.11059</v>
+        <v>0.18746</v>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
@@ -5956,13 +5956,13 @@
         </is>
       </c>
       <c r="I70" s="9" t="n">
-        <v>1116285156.69</v>
+        <v>1201072151.63</v>
       </c>
       <c r="J70" s="9" t="n">
-        <v>64853331.9</v>
+        <v>95402884.48</v>
       </c>
       <c r="K70" s="12" t="n">
-        <v>0.0581</v>
+        <v>0.07943</v>
       </c>
       <c r="L70" s="13" t="n">
         <v>219</v>
@@ -6013,13 +6013,13 @@
       <c r="C71" s="15" t="n"/>
       <c r="D71" s="16" t="n"/>
       <c r="E71" s="15" t="n">
-        <v>876862.78</v>
+        <v>4531424.11</v>
       </c>
       <c r="F71" s="15" t="n">
-        <v>877292</v>
+        <v>4307281.36</v>
       </c>
       <c r="G71" s="16" t="n">
-        <v>1.00049</v>
+        <v>0.9505400000000001</v>
       </c>
       <c r="H71" s="17" t="inlineStr">
         <is>
@@ -6027,13 +6027,13 @@
         </is>
       </c>
       <c r="I71" s="15" t="n">
-        <v>876862.78</v>
+        <v>4531424.11</v>
       </c>
       <c r="J71" s="15" t="n">
-        <v>877292</v>
+        <v>4307281.36</v>
       </c>
       <c r="K71" s="18" t="n">
-        <v>1.00049</v>
+        <v>0.9505400000000001</v>
       </c>
       <c r="L71" s="19" t="n"/>
       <c r="M71" s="19" t="n"/>
@@ -7448,13 +7448,13 @@
         <v>0.02706</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>818307638.95</v>
+        <v>906434238.4400001</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>138724420.81</v>
+        <v>172391256.19</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.16953</v>
+        <v>0.19019</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
@@ -7462,13 +7462,13 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>4022932626.21</v>
+        <v>4111059225.7</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>225455623.85</v>
+        <v>259122459.23</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.05604</v>
+        <v>0.06303</v>
       </c>
       <c r="L20" s="13" t="n">
         <v>844</v>
@@ -8043,10 +8043,10 @@
         <v>-2.1</v>
       </c>
       <c r="L11" s="15" t="n">
-        <v>42124229.67</v>
+        <v>102929410.54</v>
       </c>
       <c r="M11" s="16" t="n">
-        <v>0.176</v>
+        <v>0.3365</v>
       </c>
     </row>
     <row r="12">
@@ -8605,7 +8605,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 06:37 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 07:26 UTC.</t>
         </is>
       </c>
     </row>
@@ -10140,26 +10140,26 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>6742160.2</v>
+        <v>7811593.26</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>18541715.73</v>
+        <v>22002791.93</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.09569999999999999</v>
+        <v>0.0992</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.0363</v>
+        <v>0.0398</v>
       </c>
       <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n">
-        <v>0.1121</v>
+        <v>0.1164</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>129647</v>
+        <v>148526</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>207434</v>
+        <v>239817</v>
       </c>
       <c r="L14" s="32" t="n">
         <v>0</v>
@@ -12828,26 +12828,26 @@
         </is>
       </c>
       <c r="D78" s="9" t="n">
-        <v>447248.48</v>
+        <v>502434.77</v>
       </c>
       <c r="E78" s="9" t="n">
-        <v>7146753.07</v>
+        <v>7996013.84</v>
       </c>
       <c r="F78" s="10" t="n">
-        <v>0.4329</v>
+        <v>0.4547</v>
       </c>
       <c r="G78" s="10" t="n">
-        <v>0.3596</v>
+        <v>0.3804</v>
       </c>
       <c r="H78" s="10" t="n"/>
       <c r="I78" s="10" t="n">
-        <v>0.0295</v>
+        <v>0.0318</v>
       </c>
       <c r="J78" s="13" t="n">
-        <v>31600</v>
+        <v>35761</v>
       </c>
       <c r="K78" s="13" t="n">
-        <v>49787</v>
+        <v>56908</v>
       </c>
       <c r="L78" s="32" t="n">
         <v>0</v>
@@ -12870,26 +12870,26 @@
         </is>
       </c>
       <c r="D79" s="15" t="n">
-        <v>1831414.31</v>
+        <v>2188064.88</v>
       </c>
       <c r="E79" s="15" t="n">
-        <v>1224434.35</v>
+        <v>1454751.52</v>
       </c>
       <c r="F79" s="16" t="n">
-        <v>-0.0454</v>
+        <v>-0.0314</v>
       </c>
       <c r="G79" s="16" t="n">
-        <v>-0.09370000000000001</v>
+        <v>-0.079</v>
       </c>
       <c r="H79" s="16" t="n"/>
       <c r="I79" s="16" t="n">
-        <v>0.3349</v>
+        <v>0.3376</v>
       </c>
       <c r="J79" s="19" t="n">
-        <v>7643</v>
+        <v>8988</v>
       </c>
       <c r="K79" s="19" t="n">
-        <v>23182</v>
+        <v>27634</v>
       </c>
       <c r="L79" s="31" t="n">
         <v>0</v>
@@ -12912,26 +12912,26 @@
         </is>
       </c>
       <c r="D80" s="9" t="n">
-        <v>1556283.51</v>
+        <v>1818012.77</v>
       </c>
       <c r="E80" s="9" t="n">
-        <v>1426069.28</v>
+        <v>1714248.23</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>0.1273</v>
+        <v>0.1211</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>0.0725</v>
+        <v>0.06619999999999999</v>
       </c>
       <c r="H80" s="10" t="n"/>
       <c r="I80" s="10" t="n">
-        <v>0.2328</v>
+        <v>0.2368</v>
       </c>
       <c r="J80" s="13" t="n">
-        <v>13854</v>
+        <v>16019</v>
       </c>
       <c r="K80" s="13" t="n">
-        <v>26222</v>
+        <v>31080</v>
       </c>
       <c r="L80" s="32" t="n">
         <v>0</v>
@@ -12954,26 +12954,26 @@
         </is>
       </c>
       <c r="D81" s="15" t="n">
-        <v>1060603.1</v>
+        <v>1194554.76</v>
       </c>
       <c r="E81" s="15" t="n">
-        <v>1491541.88</v>
+        <v>1842469.43</v>
       </c>
       <c r="F81" s="16" t="n">
-        <v>0.0519</v>
+        <v>0.0271</v>
       </c>
       <c r="G81" s="16" t="n">
-        <v>-0.009599999999999999</v>
+        <v>-0.0354</v>
       </c>
       <c r="H81" s="16" t="n"/>
       <c r="I81" s="16" t="n">
-        <v>0.1695</v>
+        <v>0.1736</v>
       </c>
       <c r="J81" s="19" t="n">
-        <v>16043</v>
+        <v>18530</v>
       </c>
       <c r="K81" s="19" t="n">
-        <v>25339</v>
+        <v>29295</v>
       </c>
       <c r="L81" s="31" t="n">
         <v>0</v>
@@ -12996,26 +12996,26 @@
         </is>
       </c>
       <c r="D82" s="9" t="n">
-        <v>661442.6800000001</v>
+        <v>758222.03</v>
       </c>
       <c r="E82" s="9" t="n">
-        <v>1328527.37</v>
+        <v>1638623.52</v>
       </c>
       <c r="F82" s="10" t="n">
-        <v>0.0738</v>
+        <v>0.1253</v>
       </c>
       <c r="G82" s="10" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.0596</v>
       </c>
       <c r="H82" s="10" t="n"/>
       <c r="I82" s="10" t="n">
-        <v>0.1273</v>
+        <v>0.1294</v>
       </c>
       <c r="J82" s="13" t="n">
-        <v>14441</v>
+        <v>16473</v>
       </c>
       <c r="K82" s="13" t="n">
-        <v>20793</v>
+        <v>23742</v>
       </c>
       <c r="L82" s="32" t="n">
         <v>0</v>
@@ -13038,26 +13038,26 @@
         </is>
       </c>
       <c r="D83" s="15" t="n">
-        <v>748111.54</v>
+        <v>851672.7</v>
       </c>
       <c r="E83" s="15" t="n">
-        <v>2762288.31</v>
+        <v>3310612.36</v>
       </c>
       <c r="F83" s="16" t="n">
-        <v>0.1481</v>
+        <v>0.1078</v>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.0365</v>
       </c>
       <c r="H83" s="16" t="n"/>
       <c r="I83" s="16" t="n">
-        <v>0.0866</v>
+        <v>0.09180000000000001</v>
       </c>
       <c r="J83" s="19" t="n">
-        <v>24733</v>
+        <v>28285</v>
       </c>
       <c r="K83" s="19" t="n">
-        <v>33292</v>
+        <v>38158</v>
       </c>
       <c r="L83" s="31" t="n">
         <v>0</v>
@@ -13080,26 +13080,26 @@
         </is>
       </c>
       <c r="D84" s="9" t="n">
-        <v>437056.58</v>
+        <v>498631.35</v>
       </c>
       <c r="E84" s="9" t="n">
-        <v>3162101.47</v>
+        <v>4046073.03</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>0.2784</v>
+        <v>0.3523</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>0.205</v>
+        <v>0.2771</v>
       </c>
       <c r="H84" s="10" t="n"/>
       <c r="I84" s="10" t="n">
-        <v>0.0525</v>
+        <v>0.0564</v>
       </c>
       <c r="J84" s="13" t="n">
-        <v>21333</v>
+        <v>24470</v>
       </c>
       <c r="K84" s="13" t="n">
-        <v>28819</v>
+        <v>33000</v>
       </c>
       <c r="L84" s="32" t="n">
         <v>0</v>
@@ -14466,26 +14466,26 @@
         </is>
       </c>
       <c r="D117" s="15" t="n">
-        <v>37658165.99</v>
+        <v>42162046.89</v>
       </c>
       <c r="E117" s="15" t="n">
-        <v>76726578.41</v>
+        <v>90570755.62</v>
       </c>
       <c r="F117" s="16" t="n">
-        <v>0.2288</v>
+        <v>0.2191</v>
       </c>
       <c r="G117" s="16" t="n">
-        <v>0.1742</v>
+        <v>0.1637</v>
       </c>
       <c r="H117" s="16" t="n"/>
       <c r="I117" s="16" t="n">
-        <v>0.0951</v>
+        <v>0.1041</v>
       </c>
       <c r="J117" s="19" t="n">
-        <v>597565</v>
+        <v>652279</v>
       </c>
       <c r="K117" s="19" t="n">
-        <v>1113287</v>
+        <v>1233926</v>
       </c>
       <c r="L117" s="31" t="n">
         <v>0</v>
@@ -16650,26 +16650,26 @@
         </is>
       </c>
       <c r="D169" s="15" t="n">
-        <v>2953533.49</v>
+        <v>3058468.79</v>
       </c>
       <c r="E169" s="15" t="n">
-        <v>28011265.92</v>
+        <v>30813737.89</v>
       </c>
       <c r="F169" s="16" t="n">
-        <v>0.7218</v>
+        <v>0.7104</v>
       </c>
       <c r="G169" s="16" t="n">
-        <v>0.6536</v>
+        <v>0.6405</v>
       </c>
       <c r="H169" s="16" t="n"/>
       <c r="I169" s="16" t="n">
-        <v>0.0145</v>
+        <v>0.0158</v>
       </c>
       <c r="J169" s="19" t="n">
-        <v>185867</v>
+        <v>194789</v>
       </c>
       <c r="K169" s="19" t="n">
-        <v>300039</v>
+        <v>313057</v>
       </c>
       <c r="L169" s="31" t="n">
         <v>0</v>
@@ -16692,26 +16692,26 @@
         </is>
       </c>
       <c r="D170" s="9" t="n">
-        <v>14589586.25</v>
+        <v>17154492.26</v>
       </c>
       <c r="E170" s="9" t="n">
-        <v>13172510.68</v>
+        <v>16463025.86</v>
       </c>
       <c r="F170" s="10" t="n">
-        <v>0.046</v>
+        <v>0.0471</v>
       </c>
       <c r="G170" s="10" t="n">
-        <v>-0.0014</v>
+        <v>-0.0012</v>
       </c>
       <c r="H170" s="10" t="n"/>
       <c r="I170" s="10" t="n">
-        <v>0.3308</v>
+        <v>0.3366</v>
       </c>
       <c r="J170" s="13" t="n">
-        <v>57604</v>
+        <v>66323</v>
       </c>
       <c r="K170" s="13" t="n">
-        <v>200691</v>
+        <v>244592</v>
       </c>
       <c r="L170" s="32" t="n">
         <v>0</v>
@@ -16734,26 +16734,26 @@
         </is>
       </c>
       <c r="D171" s="15" t="n">
-        <v>7927640.06</v>
+        <v>8661722.18</v>
       </c>
       <c r="E171" s="15" t="n">
-        <v>7012246.33</v>
+        <v>9147312.15</v>
       </c>
       <c r="F171" s="16" t="n">
-        <v>0.1782</v>
+        <v>0.1845</v>
       </c>
       <c r="G171" s="16" t="n">
-        <v>0.1257</v>
+        <v>0.1306</v>
       </c>
       <c r="H171" s="16" t="n"/>
       <c r="I171" s="16" t="n">
-        <v>0.202</v>
+        <v>0.2111</v>
       </c>
       <c r="J171" s="19" t="n">
-        <v>66416</v>
+        <v>74880</v>
       </c>
       <c r="K171" s="19" t="n">
-        <v>158628</v>
+        <v>177385</v>
       </c>
       <c r="L171" s="31" t="n">
         <v>0</v>
@@ -16776,26 +16776,26 @@
         </is>
       </c>
       <c r="D172" s="9" t="n">
-        <v>4408503.88</v>
+        <v>4871762.92</v>
       </c>
       <c r="E172" s="9" t="n">
-        <v>5861372.28</v>
+        <v>7306578.36</v>
       </c>
       <c r="F172" s="10" t="n">
-        <v>0.2136</v>
+        <v>0.1881</v>
       </c>
       <c r="G172" s="10" t="n">
-        <v>0.156</v>
+        <v>0.1294</v>
       </c>
       <c r="H172" s="10" t="n"/>
       <c r="I172" s="10" t="n">
-        <v>0.1328</v>
+        <v>0.1429</v>
       </c>
       <c r="J172" s="13" t="n">
-        <v>64241</v>
+        <v>72381</v>
       </c>
       <c r="K172" s="13" t="n">
-        <v>110326</v>
+        <v>124705</v>
       </c>
       <c r="L172" s="32" t="n">
         <v>0</v>
@@ -16818,26 +16818,26 @@
         </is>
       </c>
       <c r="D173" s="15" t="n">
-        <v>2520033.67</v>
+        <v>2741146.2</v>
       </c>
       <c r="E173" s="15" t="n">
-        <v>4762368.23</v>
+        <v>5868871.08</v>
       </c>
       <c r="F173" s="16" t="n">
-        <v>0.2765</v>
+        <v>0.2844</v>
       </c>
       <c r="G173" s="16" t="n">
-        <v>0.2168</v>
+        <v>0.2233</v>
       </c>
       <c r="H173" s="16" t="n"/>
       <c r="I173" s="16" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.1038</v>
       </c>
       <c r="J173" s="19" t="n">
-        <v>53177</v>
+        <v>58774</v>
       </c>
       <c r="K173" s="19" t="n">
-        <v>85100</v>
+        <v>94004</v>
       </c>
       <c r="L173" s="31" t="n">
         <v>0</v>
@@ -16860,26 +16860,26 @@
         </is>
       </c>
       <c r="D174" s="9" t="n">
-        <v>3295565.22</v>
+        <v>3556440.7</v>
       </c>
       <c r="E174" s="9" t="n">
-        <v>9392555.35</v>
+        <v>11145240.84</v>
       </c>
       <c r="F174" s="10" t="n">
-        <v>0.4867</v>
+        <v>0.4827</v>
       </c>
       <c r="G174" s="10" t="n">
-        <v>0.4229</v>
+        <v>0.4177</v>
       </c>
       <c r="H174" s="10" t="n"/>
       <c r="I174" s="10" t="n">
-        <v>0.0543</v>
+        <v>0.063</v>
       </c>
       <c r="J174" s="13" t="n">
-        <v>96328</v>
+        <v>104745</v>
       </c>
       <c r="K174" s="13" t="n">
-        <v>153885</v>
+        <v>166065</v>
       </c>
       <c r="L174" s="32" t="n">
         <v>0</v>
@@ -16902,26 +16902,26 @@
         </is>
       </c>
       <c r="D175" s="15" t="n">
-        <v>1963303.4</v>
+        <v>2118013.83</v>
       </c>
       <c r="E175" s="15" t="n">
-        <v>8514259.619999999</v>
+        <v>9825989.439999999</v>
       </c>
       <c r="F175" s="16" t="n">
-        <v>0.5888</v>
+        <v>0.5887</v>
       </c>
       <c r="G175" s="16" t="n">
-        <v>0.5234</v>
+        <v>0.5219</v>
       </c>
       <c r="H175" s="16" t="n"/>
       <c r="I175" s="16" t="n">
-        <v>0.0394</v>
+        <v>0.0454</v>
       </c>
       <c r="J175" s="19" t="n">
-        <v>73932</v>
+        <v>80387</v>
       </c>
       <c r="K175" s="19" t="n">
-        <v>104618</v>
+        <v>114118</v>
       </c>
       <c r="L175" s="31" t="n">
         <v>0</v>
@@ -17406,26 +17406,26 @@
         </is>
       </c>
       <c r="D187" s="15" t="n">
-        <v>3659269.07</v>
+        <v>4149539.61</v>
       </c>
       <c r="E187" s="15" t="n">
-        <v>6252838.43</v>
+        <v>9377518.939999999</v>
       </c>
       <c r="F187" s="16" t="n">
-        <v>-0.0021</v>
+        <v>0.0219</v>
       </c>
       <c r="G187" s="16" t="n">
-        <v>-0.0555</v>
+        <v>-0.0346</v>
       </c>
       <c r="H187" s="16" t="n"/>
       <c r="I187" s="16" t="n">
-        <v>0.123</v>
+        <v>0.1346</v>
       </c>
       <c r="J187" s="19" t="n">
-        <v>82404</v>
+        <v>95674</v>
       </c>
       <c r="K187" s="19" t="n">
-        <v>146260</v>
+        <v>171417</v>
       </c>
       <c r="L187" s="31" t="n">
         <v>0</v>
@@ -20682,26 +20682,26 @@
         </is>
       </c>
       <c r="D265" s="15" t="n">
-        <v>124103.52</v>
+        <v>146213.69</v>
       </c>
       <c r="E265" s="15" t="n">
-        <v>465293.62</v>
+        <v>881557.51</v>
       </c>
       <c r="F265" s="16" t="n">
-        <v>0.431</v>
+        <v>0.3886</v>
       </c>
       <c r="G265" s="16" t="n">
-        <v>0.4065</v>
+        <v>0.363</v>
       </c>
       <c r="H265" s="16" t="n"/>
       <c r="I265" s="16" t="n">
-        <v>0.05</v>
+        <v>0.0536</v>
       </c>
       <c r="J265" s="19" t="n">
-        <v>3517</v>
+        <v>4194</v>
       </c>
       <c r="K265" s="19" t="n">
-        <v>5945</v>
+        <v>7084</v>
       </c>
       <c r="L265" s="31" t="n">
         <v>0</v>
@@ -20724,26 +20724,26 @@
         </is>
       </c>
       <c r="D266" s="9" t="n">
-        <v>1700088.8</v>
+        <v>1984699.16</v>
       </c>
       <c r="E266" s="9" t="n">
-        <v>865823.6800000001</v>
+        <v>1370502.22</v>
       </c>
       <c r="F266" s="10" t="n">
-        <v>-0.0211</v>
+        <v>0.016</v>
       </c>
       <c r="G266" s="10" t="n">
-        <v>-0.0687</v>
+        <v>-0.0338</v>
       </c>
       <c r="H266" s="10" t="n"/>
       <c r="I266" s="10" t="n">
-        <v>0.2434</v>
+        <v>0.2447</v>
       </c>
       <c r="J266" s="13" t="n">
-        <v>9839</v>
+        <v>11616</v>
       </c>
       <c r="K266" s="13" t="n">
-        <v>42665</v>
+        <v>51061</v>
       </c>
       <c r="L266" s="32" t="n">
         <v>0</v>
@@ -20766,26 +20766,26 @@
         </is>
       </c>
       <c r="D267" s="15" t="n">
-        <v>667340.01</v>
+        <v>745527.17</v>
       </c>
       <c r="E267" s="15" t="n">
-        <v>1149023.22</v>
+        <v>1390466</v>
       </c>
       <c r="F267" s="16" t="n">
-        <v>0.0322</v>
+        <v>0.0473</v>
       </c>
       <c r="G267" s="16" t="n">
-        <v>-0.0269</v>
+        <v>-0.0135</v>
       </c>
       <c r="H267" s="16" t="n"/>
       <c r="I267" s="16" t="n">
-        <v>0.1841</v>
+        <v>0.1899</v>
       </c>
       <c r="J267" s="19" t="n">
-        <v>15466</v>
+        <v>17879</v>
       </c>
       <c r="K267" s="19" t="n">
-        <v>25814</v>
+        <v>29611</v>
       </c>
       <c r="L267" s="31" t="n">
         <v>0</v>
@@ -20808,26 +20808,26 @@
         </is>
       </c>
       <c r="D268" s="9" t="n">
-        <v>478102.37</v>
+        <v>516186.59</v>
       </c>
       <c r="E268" s="9" t="n">
-        <v>698311.51</v>
+        <v>988443.84</v>
       </c>
       <c r="F268" s="10" t="n">
-        <v>0.091</v>
+        <v>0.0383</v>
       </c>
       <c r="G268" s="10" t="n">
-        <v>0.0341</v>
+        <v>-0.022</v>
       </c>
       <c r="H268" s="10" t="n"/>
       <c r="I268" s="10" t="n">
-        <v>0.1329</v>
+        <v>0.1469</v>
       </c>
       <c r="J268" s="13" t="n">
-        <v>15213</v>
+        <v>17538</v>
       </c>
       <c r="K268" s="13" t="n">
-        <v>20942</v>
+        <v>24073</v>
       </c>
       <c r="L268" s="32" t="n">
         <v>0</v>
@@ -20850,26 +20850,26 @@
         </is>
       </c>
       <c r="D269" s="15" t="n">
-        <v>257075.49</v>
+        <v>279635.59</v>
       </c>
       <c r="E269" s="15" t="n">
-        <v>669822.39</v>
+        <v>1047853.65</v>
       </c>
       <c r="F269" s="16" t="n">
-        <v>0.0574</v>
+        <v>0.0716</v>
       </c>
       <c r="G269" s="16" t="n">
-        <v>-0.0075</v>
+        <v>0.0014</v>
       </c>
       <c r="H269" s="16" t="n"/>
       <c r="I269" s="16" t="n">
-        <v>0.09370000000000001</v>
+        <v>0.1114</v>
       </c>
       <c r="J269" s="19" t="n">
-        <v>11910</v>
+        <v>13710</v>
       </c>
       <c r="K269" s="19" t="n">
-        <v>15038</v>
+        <v>17351</v>
       </c>
       <c r="L269" s="31" t="n">
         <v>0</v>
@@ -20892,26 +20892,26 @@
         </is>
       </c>
       <c r="D270" s="9" t="n">
-        <v>275332.87</v>
+        <v>303605.27</v>
       </c>
       <c r="E270" s="9" t="n">
-        <v>1322804.02</v>
+        <v>1960000.42</v>
       </c>
       <c r="F270" s="10" t="n">
-        <v>-0.2782</v>
+        <v>-0.176</v>
       </c>
       <c r="G270" s="10" t="n">
-        <v>-0.3477</v>
+        <v>-0.2546</v>
       </c>
       <c r="H270" s="10" t="n"/>
       <c r="I270" s="10" t="n">
-        <v>0.0678</v>
+        <v>0.08550000000000001</v>
       </c>
       <c r="J270" s="13" t="n">
-        <v>16330</v>
+        <v>18876</v>
       </c>
       <c r="K270" s="13" t="n">
-        <v>22739</v>
+        <v>26540</v>
       </c>
       <c r="L270" s="32" t="n">
         <v>0</v>
@@ -20934,26 +20934,26 @@
         </is>
       </c>
       <c r="D271" s="15" t="n">
-        <v>157226.03</v>
+        <v>173672.14</v>
       </c>
       <c r="E271" s="15" t="n">
-        <v>1081759.99</v>
+        <v>1738695.3</v>
       </c>
       <c r="F271" s="16" t="n">
-        <v>-0.1806</v>
+        <v>-0.1109</v>
       </c>
       <c r="G271" s="16" t="n">
-        <v>-0.2386</v>
+        <v>-0.1793</v>
       </c>
       <c r="H271" s="16" t="n"/>
       <c r="I271" s="16" t="n">
-        <v>0.0467</v>
+        <v>0.0588</v>
       </c>
       <c r="J271" s="19" t="n">
-        <v>10129</v>
+        <v>11861</v>
       </c>
       <c r="K271" s="19" t="n">
-        <v>13117</v>
+        <v>15697</v>
       </c>
       <c r="L271" s="31" t="n">
         <v>0</v>
@@ -21648,26 +21648,26 @@
         </is>
       </c>
       <c r="D288" s="9" t="n">
-        <v>61340956.65</v>
+        <v>70439414.03</v>
       </c>
       <c r="E288" s="9" t="n">
-        <v>151931602.04</v>
+        <v>172548158.41</v>
       </c>
       <c r="F288" s="10" t="n">
-        <v>-0.0372</v>
+        <v>-0.0018</v>
       </c>
       <c r="G288" s="10" t="n">
-        <v>-0.0989</v>
+        <v>-0.06320000000000001</v>
       </c>
       <c r="H288" s="10" t="n"/>
       <c r="I288" s="10" t="n">
-        <v>0.1208</v>
+        <v>0.1237</v>
       </c>
       <c r="J288" s="13" t="n">
-        <v>1339733</v>
+        <v>1519981</v>
       </c>
       <c r="K288" s="13" t="n">
-        <v>2874586</v>
+        <v>3304531</v>
       </c>
       <c r="L288" s="32" t="n">
         <v>0</v>
@@ -26226,26 +26226,26 @@
         </is>
       </c>
       <c r="D397" s="15" t="n">
-        <v>5279994.57</v>
+        <v>6083299.99</v>
       </c>
       <c r="E397" s="15" t="n">
-        <v>46162026.34</v>
+        <v>50430186.27</v>
       </c>
       <c r="F397" s="16" t="n">
-        <v>0.1694</v>
+        <v>0.2249</v>
       </c>
       <c r="G397" s="16" t="n">
-        <v>0.0949</v>
+        <v>0.1495</v>
       </c>
       <c r="H397" s="16" t="n"/>
       <c r="I397" s="16" t="n">
-        <v>0.0451</v>
+        <v>0.0436</v>
       </c>
       <c r="J397" s="19" t="n">
-        <v>345279</v>
+        <v>401958</v>
       </c>
       <c r="K397" s="19" t="n">
-        <v>752326</v>
+        <v>880097</v>
       </c>
       <c r="L397" s="31" t="n">
         <v>0</v>
@@ -26268,26 +26268,26 @@
         </is>
       </c>
       <c r="D398" s="9" t="n">
-        <v>22846315.4</v>
+        <v>26594678.51</v>
       </c>
       <c r="E398" s="9" t="n">
-        <v>21111906.23</v>
+        <v>24285547.09</v>
       </c>
       <c r="F398" s="10" t="n">
-        <v>0.0475</v>
+        <v>0.0408</v>
       </c>
       <c r="G398" s="10" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.014</v>
       </c>
       <c r="H398" s="10" t="n"/>
       <c r="I398" s="10" t="n">
-        <v>0.3062</v>
+        <v>0.3115</v>
       </c>
       <c r="J398" s="13" t="n">
-        <v>105880</v>
+        <v>121853</v>
       </c>
       <c r="K398" s="13" t="n">
-        <v>425579</v>
+        <v>480919</v>
       </c>
       <c r="L398" s="32" t="n">
         <v>0</v>
@@ -26310,26 +26310,26 @@
         </is>
       </c>
       <c r="D399" s="15" t="n">
-        <v>11280144.46</v>
+        <v>12716351.03</v>
       </c>
       <c r="E399" s="15" t="n">
-        <v>10574692.03</v>
+        <v>12046791.44</v>
       </c>
       <c r="F399" s="16" t="n">
-        <v>0.0425</v>
+        <v>0.0546</v>
       </c>
       <c r="G399" s="16" t="n">
-        <v>-0.0136</v>
+        <v>-0.0012</v>
       </c>
       <c r="H399" s="16" t="n"/>
       <c r="I399" s="16" t="n">
-        <v>0.2165</v>
+        <v>0.2226</v>
       </c>
       <c r="J399" s="19" t="n">
-        <v>150317</v>
+        <v>168780</v>
       </c>
       <c r="K399" s="19" t="n">
-        <v>337714</v>
+        <v>380998</v>
       </c>
       <c r="L399" s="31" t="n">
         <v>0</v>
@@ -26352,26 +26352,26 @@
         </is>
       </c>
       <c r="D400" s="9" t="n">
-        <v>7568869.05</v>
+        <v>8657509.26</v>
       </c>
       <c r="E400" s="9" t="n">
-        <v>10028223.07</v>
+        <v>11509818.04</v>
       </c>
       <c r="F400" s="10" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.1224</v>
       </c>
       <c r="G400" s="10" t="n">
-        <v>0.0259</v>
+        <v>0.0614</v>
       </c>
       <c r="H400" s="10" t="n"/>
       <c r="I400" s="10" t="n">
-        <v>0.1618</v>
+        <v>0.1683</v>
       </c>
       <c r="J400" s="13" t="n">
-        <v>166080</v>
+        <v>185881</v>
       </c>
       <c r="K400" s="13" t="n">
-        <v>293499</v>
+        <v>333867</v>
       </c>
       <c r="L400" s="32" t="n">
         <v>0</v>
@@ -26394,26 +26394,26 @@
         </is>
       </c>
       <c r="D401" s="15" t="n">
-        <v>4550836.59</v>
+        <v>5219839.49</v>
       </c>
       <c r="E401" s="15" t="n">
-        <v>8020809.6</v>
+        <v>9548701.880000001</v>
       </c>
       <c r="F401" s="16" t="n">
-        <v>0.1101</v>
+        <v>0.1537</v>
       </c>
       <c r="G401" s="16" t="n">
-        <v>0.0452</v>
+        <v>0.0885</v>
       </c>
       <c r="H401" s="16" t="n"/>
       <c r="I401" s="16" t="n">
-        <v>0.1312</v>
+        <v>0.1359</v>
       </c>
       <c r="J401" s="19" t="n">
-        <v>137335</v>
+        <v>154036</v>
       </c>
       <c r="K401" s="19" t="n">
-        <v>231982</v>
+        <v>267297</v>
       </c>
       <c r="L401" s="31" t="n">
         <v>0</v>
@@ -26436,26 +26436,26 @@
         </is>
       </c>
       <c r="D402" s="9" t="n">
-        <v>5425005.74</v>
+        <v>6374699.1</v>
       </c>
       <c r="E402" s="9" t="n">
-        <v>13795580.49</v>
+        <v>19191439.28</v>
       </c>
       <c r="F402" s="10" t="n">
-        <v>0.1743</v>
+        <v>0.2303</v>
       </c>
       <c r="G402" s="10" t="n">
-        <v>0.107</v>
+        <v>0.1621</v>
       </c>
       <c r="H402" s="10" t="n"/>
       <c r="I402" s="10" t="n">
-        <v>0.0964</v>
+        <v>0.1006</v>
       </c>
       <c r="J402" s="13" t="n">
-        <v>227612</v>
+        <v>256577</v>
       </c>
       <c r="K402" s="13" t="n">
-        <v>347972</v>
+        <v>442638</v>
       </c>
       <c r="L402" s="32" t="n">
         <v>0</v>
@@ -26478,26 +26478,26 @@
         </is>
       </c>
       <c r="D403" s="15" t="n">
-        <v>4389790.85</v>
+        <v>4793036.65</v>
       </c>
       <c r="E403" s="15" t="n">
-        <v>42238364.28</v>
+        <v>45535674.41</v>
       </c>
       <c r="F403" s="16" t="n">
-        <v>-1.5596</v>
+        <v>-1.3773</v>
       </c>
       <c r="G403" s="16" t="n">
-        <v>-1.6436</v>
+        <v>-1.4605</v>
       </c>
       <c r="H403" s="16" t="n"/>
       <c r="I403" s="16" t="n">
-        <v>0.0699</v>
+        <v>0.073</v>
       </c>
       <c r="J403" s="19" t="n">
-        <v>207230</v>
+        <v>230896</v>
       </c>
       <c r="K403" s="19" t="n">
-        <v>485514</v>
+        <v>518715</v>
       </c>
       <c r="L403" s="31" t="n">
         <v>0</v>
@@ -27796,31 +27796,31 @@
         </is>
       </c>
       <c r="D433" s="15" t="n">
-        <v>42124229.67</v>
+        <v>102929410.54</v>
       </c>
       <c r="E433" s="15" t="n">
-        <v>57596750.56</v>
+        <v>195454778.86</v>
       </c>
       <c r="F433" s="16" t="n">
-        <v>0.176</v>
+        <v>0.3365</v>
       </c>
       <c r="G433" s="16" t="n">
-        <v>0.123</v>
+        <v>0.2795</v>
       </c>
       <c r="H433" s="16" t="n">
-        <v>0.1247</v>
+        <v>0.107</v>
       </c>
       <c r="I433" s="16" t="n">
-        <v>0.127</v>
+        <v>0.0843</v>
       </c>
       <c r="J433" s="19" t="n">
-        <v>877857</v>
+        <v>2031771</v>
       </c>
       <c r="K433" s="19" t="n">
-        <v>1727031</v>
+        <v>4240605</v>
       </c>
       <c r="L433" s="31" t="n">
-        <v>0.5777</v>
+        <v>0.5588</v>
       </c>
     </row>
     <row r="434">
@@ -36676,31 +36676,31 @@
         </is>
       </c>
       <c r="D635" s="15" t="n">
-        <v>3175451.41</v>
+        <v>6629554.42</v>
       </c>
       <c r="E635" s="15" t="n">
-        <v>20441613.52</v>
+        <v>84760953.86</v>
       </c>
       <c r="F635" s="16" t="n">
-        <v>0.7059</v>
+        <v>0.7929</v>
       </c>
       <c r="G635" s="16" t="n">
-        <v>0.6351</v>
+        <v>0.7188</v>
       </c>
       <c r="H635" s="16" t="n">
-        <v>0.4975</v>
+        <v>0.47</v>
       </c>
       <c r="I635" s="16" t="n">
-        <v>0.0282</v>
+        <v>0.0174</v>
       </c>
       <c r="J635" s="19" t="n">
-        <v>183426</v>
+        <v>418522</v>
       </c>
       <c r="K635" s="19" t="n">
-        <v>356954</v>
+        <v>821873</v>
       </c>
       <c r="L635" s="31" t="n">
-        <v>0.6556</v>
+        <v>0.6696</v>
       </c>
     </row>
     <row r="636">
@@ -36720,31 +36720,31 @@
         </is>
       </c>
       <c r="D636" s="9" t="n">
-        <v>11602566.02</v>
+        <v>31322916.58</v>
       </c>
       <c r="E636" s="9" t="n">
-        <v>9658664.779999999</v>
+        <v>20968754.01</v>
       </c>
       <c r="F636" s="10" t="n">
-        <v>0.0311</v>
+        <v>0.1772</v>
       </c>
       <c r="G636" s="10" t="n">
-        <v>-0.0186</v>
+        <v>0.1263</v>
       </c>
       <c r="H636" s="10" t="n">
-        <v>0.0234</v>
+        <v>0.028</v>
       </c>
       <c r="I636" s="10" t="n">
-        <v>0.2803</v>
+        <v>0.245</v>
       </c>
       <c r="J636" s="13" t="n">
-        <v>51178</v>
+        <v>129494</v>
       </c>
       <c r="K636" s="13" t="n">
-        <v>226673</v>
+        <v>567908</v>
       </c>
       <c r="L636" s="32" t="n">
-        <v>0.5484</v>
+        <v>0.5165</v>
       </c>
     </row>
     <row r="637">
@@ -36764,31 +36764,31 @@
         </is>
       </c>
       <c r="D637" s="15" t="n">
-        <v>6618709.47</v>
+        <v>19404486.89</v>
       </c>
       <c r="E637" s="15" t="n">
-        <v>3217738.61</v>
+        <v>10910099.18</v>
       </c>
       <c r="F637" s="16" t="n">
-        <v>0.059</v>
+        <v>0.2216</v>
       </c>
       <c r="G637" s="16" t="n">
-        <v>0.0126</v>
+        <v>0.1691</v>
       </c>
       <c r="H637" s="16" t="n">
-        <v>0.0606</v>
+        <v>0.0501</v>
       </c>
       <c r="I637" s="16" t="n">
-        <v>0.2408</v>
+        <v>0.1722</v>
       </c>
       <c r="J637" s="19" t="n">
-        <v>92909</v>
+        <v>220966</v>
       </c>
       <c r="K637" s="19" t="n">
-        <v>181771</v>
+        <v>514790</v>
       </c>
       <c r="L637" s="31" t="n">
-        <v>0.5617</v>
+        <v>0.5122</v>
       </c>
     </row>
     <row r="638">
@@ -36808,31 +36808,31 @@
         </is>
       </c>
       <c r="D638" s="9" t="n">
-        <v>6301186.86</v>
+        <v>14776564.36</v>
       </c>
       <c r="E638" s="9" t="n">
-        <v>4026933.18</v>
+        <v>13515691.86</v>
       </c>
       <c r="F638" s="10" t="n">
-        <v>0.023</v>
+        <v>0.2792</v>
       </c>
       <c r="G638" s="10" t="n">
-        <v>-0.0259</v>
+        <v>0.2222</v>
       </c>
       <c r="H638" s="10" t="n">
-        <v>0.1027</v>
+        <v>0.0843</v>
       </c>
       <c r="I638" s="10" t="n">
-        <v>0.1968</v>
+        <v>0.1241</v>
       </c>
       <c r="J638" s="13" t="n">
-        <v>116756</v>
+        <v>268987</v>
       </c>
       <c r="K638" s="13" t="n">
-        <v>225062</v>
+        <v>540700</v>
       </c>
       <c r="L638" s="32" t="n">
-        <v>0.5607</v>
+        <v>0.5590000000000001</v>
       </c>
     </row>
     <row r="639">
@@ -36852,31 +36852,31 @@
         </is>
       </c>
       <c r="D639" s="15" t="n">
-        <v>4482613.1</v>
+        <v>10017881.43</v>
       </c>
       <c r="E639" s="15" t="n">
-        <v>3939669.01</v>
+        <v>12019286.95</v>
       </c>
       <c r="F639" s="16" t="n">
-        <v>0.2037</v>
+        <v>0.4617</v>
       </c>
       <c r="G639" s="16" t="n">
-        <v>0.1512</v>
+        <v>0.4031</v>
       </c>
       <c r="H639" s="16" t="n">
-        <v>0.1698</v>
+        <v>0.119</v>
       </c>
       <c r="I639" s="16" t="n">
-        <v>0.1623</v>
+        <v>0.0963</v>
       </c>
       <c r="J639" s="19" t="n">
-        <v>106158</v>
+        <v>240200</v>
       </c>
       <c r="K639" s="19" t="n">
-        <v>180270</v>
+        <v>426809</v>
       </c>
       <c r="L639" s="31" t="n">
-        <v>0.5782</v>
+        <v>0.5841</v>
       </c>
     </row>
     <row r="640">
@@ -36896,31 +36896,31 @@
         </is>
       </c>
       <c r="D640" s="9" t="n">
-        <v>5630781.98</v>
+        <v>12503337.58</v>
       </c>
       <c r="E640" s="9" t="n">
-        <v>7589986.71</v>
+        <v>25564122.33</v>
       </c>
       <c r="F640" s="10" t="n">
-        <v>0.2615</v>
+        <v>0.4777</v>
       </c>
       <c r="G640" s="10" t="n">
-        <v>0.2051</v>
+        <v>0.4147</v>
       </c>
       <c r="H640" s="10" t="n">
-        <v>0.2282</v>
+        <v>0.191</v>
       </c>
       <c r="I640" s="10" t="n">
-        <v>0.1129</v>
+        <v>0.0625</v>
       </c>
       <c r="J640" s="13" t="n">
-        <v>171850</v>
+        <v>403982</v>
       </c>
       <c r="K640" s="13" t="n">
-        <v>260417</v>
+        <v>726664</v>
       </c>
       <c r="L640" s="32" t="n">
-        <v>0.6012999999999999</v>
+        <v>0.6032</v>
       </c>
     </row>
     <row r="641">
@@ -36940,31 +36940,31 @@
         </is>
       </c>
       <c r="D641" s="15" t="n">
-        <v>4312920.84</v>
+        <v>8274669.28</v>
       </c>
       <c r="E641" s="15" t="n">
-        <v>8722144.74</v>
+        <v>27715870.68</v>
       </c>
       <c r="F641" s="16" t="n">
-        <v>0.4385</v>
+        <v>0.5802</v>
       </c>
       <c r="G641" s="16" t="n">
-        <v>0.3775</v>
+        <v>0.5143</v>
       </c>
       <c r="H641" s="16" t="n">
-        <v>0.3426</v>
+        <v>0.3004</v>
       </c>
       <c r="I641" s="16" t="n">
-        <v>0.06419999999999999</v>
+        <v>0.0359</v>
       </c>
       <c r="J641" s="19" t="n">
-        <v>155580</v>
+        <v>349620</v>
       </c>
       <c r="K641" s="19" t="n">
-        <v>295884</v>
+        <v>641861</v>
       </c>
       <c r="L641" s="31" t="n">
-        <v>0.6172</v>
+        <v>0.6408</v>
       </c>
     </row>
     <row r="642">
@@ -37488,29 +37488,29 @@
         </is>
       </c>
       <c r="D654" s="9" t="n">
-        <v>8319011.3</v>
+        <v>13425865.55</v>
       </c>
       <c r="E654" s="9" t="n">
-        <v>52078219.26</v>
+        <v>78976163.79000001</v>
       </c>
       <c r="F654" s="10" t="n">
-        <v>0.3449</v>
+        <v>0.346</v>
       </c>
       <c r="G654" s="10" t="n">
-        <v>0.2779</v>
+        <v>0.28</v>
       </c>
       <c r="H654" s="10" t="n"/>
       <c r="I654" s="10" t="n">
         <v>0.0587</v>
       </c>
       <c r="J654" s="13" t="n">
-        <v>346827</v>
+        <v>508897</v>
       </c>
       <c r="K654" s="13" t="n">
-        <v>475171</v>
+        <v>691754</v>
       </c>
       <c r="L654" s="32" t="n">
-        <v>0.5658</v>
+        <v>0.5457</v>
       </c>
     </row>
     <row r="655">
@@ -41058,29 +41058,29 @@
         </is>
       </c>
       <c r="D739" s="15" t="n">
-        <v>2443341.79</v>
+        <v>3373365.76</v>
       </c>
       <c r="E739" s="15" t="n">
-        <v>36806255.26</v>
+        <v>52518955.28</v>
       </c>
       <c r="F739" s="16" t="n">
-        <v>0.6264</v>
+        <v>0.6208</v>
       </c>
       <c r="G739" s="16" t="n">
-        <v>0.5481</v>
+        <v>0.5421</v>
       </c>
       <c r="H739" s="16" t="n"/>
       <c r="I739" s="16" t="n">
-        <v>0.0142</v>
+        <v>0.0141</v>
       </c>
       <c r="J739" s="19" t="n">
-        <v>205376</v>
+        <v>278296</v>
       </c>
       <c r="K739" s="19" t="n">
-        <v>281846</v>
+        <v>373023</v>
       </c>
       <c r="L739" s="31" t="n">
-        <v>0.5645</v>
+        <v>0.5618</v>
       </c>
     </row>
     <row r="740">
@@ -41100,29 +41100,29 @@
         </is>
       </c>
       <c r="D740" s="9" t="n">
-        <v>973330.61</v>
+        <v>1794111.11</v>
       </c>
       <c r="E740" s="9" t="n">
-        <v>492861.27</v>
+        <v>947688.9399999999</v>
       </c>
       <c r="F740" s="10" t="n">
-        <v>0.2403</v>
+        <v>0.2089</v>
       </c>
       <c r="G740" s="10" t="n">
-        <v>0.197</v>
+        <v>0.1661</v>
       </c>
       <c r="H740" s="10" t="n"/>
       <c r="I740" s="10" t="n">
-        <v>0.334</v>
+        <v>0.33</v>
       </c>
       <c r="J740" s="13" t="n">
-        <v>5282</v>
+        <v>9317</v>
       </c>
       <c r="K740" s="13" t="n">
-        <v>13010</v>
+        <v>23481</v>
       </c>
       <c r="L740" s="32" t="n">
-        <v>0.5731000000000001</v>
+        <v>0.5024</v>
       </c>
     </row>
     <row r="741">
@@ -41142,29 +41142,29 @@
         </is>
       </c>
       <c r="D741" s="15" t="n">
-        <v>1099939.21</v>
+        <v>1832181.65</v>
       </c>
       <c r="E741" s="15" t="n">
-        <v>972287.35</v>
+        <v>1738735.54</v>
       </c>
       <c r="F741" s="16" t="n">
-        <v>0.0775</v>
+        <v>0.1327</v>
       </c>
       <c r="G741" s="16" t="n">
-        <v>0.0239</v>
+        <v>0.07829999999999999</v>
       </c>
       <c r="H741" s="16" t="n"/>
       <c r="I741" s="16" t="n">
-        <v>0.2696</v>
+        <v>0.2407</v>
       </c>
       <c r="J741" s="19" t="n">
-        <v>11798</v>
+        <v>19895</v>
       </c>
       <c r="K741" s="19" t="n">
-        <v>21688</v>
+        <v>35709</v>
       </c>
       <c r="L741" s="31" t="n">
-        <v>0.5916</v>
+        <v>0.5664</v>
       </c>
     </row>
     <row r="742">
@@ -41184,29 +41184,29 @@
         </is>
       </c>
       <c r="D742" s="9" t="n">
-        <v>811918.6800000001</v>
+        <v>1492185.47</v>
       </c>
       <c r="E742" s="9" t="n">
-        <v>1622742.47</v>
+        <v>2549511.1</v>
       </c>
       <c r="F742" s="10" t="n">
-        <v>0.128</v>
+        <v>0.2081</v>
       </c>
       <c r="G742" s="10" t="n">
-        <v>0.0643</v>
+        <v>0.1446</v>
       </c>
       <c r="H742" s="10" t="n"/>
       <c r="I742" s="10" t="n">
-        <v>0.1991</v>
+        <v>0.1742</v>
       </c>
       <c r="J742" s="13" t="n">
-        <v>15626</v>
+        <v>26653</v>
       </c>
       <c r="K742" s="13" t="n">
-        <v>21313</v>
+        <v>38128</v>
       </c>
       <c r="L742" s="32" t="n">
-        <v>0.61</v>
+        <v>0.5714</v>
       </c>
     </row>
     <row r="743">
@@ -41226,29 +41226,29 @@
         </is>
       </c>
       <c r="D743" s="15" t="n">
-        <v>697250.02</v>
+        <v>1201921.94</v>
       </c>
       <c r="E743" s="15" t="n">
-        <v>1701972.85</v>
+        <v>3153162.49</v>
       </c>
       <c r="F743" s="16" t="n">
-        <v>0.1309</v>
+        <v>0.2208</v>
       </c>
       <c r="G743" s="16" t="n">
-        <v>0.065</v>
+        <v>0.1534</v>
       </c>
       <c r="H743" s="16" t="n"/>
       <c r="I743" s="16" t="n">
-        <v>0.1568</v>
+        <v>0.1343</v>
       </c>
       <c r="J743" s="19" t="n">
-        <v>17120</v>
+        <v>28948</v>
       </c>
       <c r="K743" s="19" t="n">
-        <v>22063</v>
+        <v>38274</v>
       </c>
       <c r="L743" s="31" t="n">
-        <v>0.551</v>
+        <v>0.539</v>
       </c>
     </row>
     <row r="744">
@@ -41268,29 +41268,29 @@
         </is>
       </c>
       <c r="D744" s="9" t="n">
-        <v>1111852.88</v>
+        <v>1957777.49</v>
       </c>
       <c r="E744" s="9" t="n">
-        <v>3578866.98</v>
+        <v>6608718.79</v>
       </c>
       <c r="F744" s="10" t="n">
-        <v>0.2648</v>
+        <v>0.2602</v>
       </c>
       <c r="G744" s="10" t="n">
-        <v>0.1942</v>
+        <v>0.1919</v>
       </c>
       <c r="H744" s="10" t="n"/>
       <c r="I744" s="10" t="n">
-        <v>0.1</v>
+        <v>0.0878</v>
       </c>
       <c r="J744" s="13" t="n">
-        <v>38518</v>
+        <v>62960</v>
       </c>
       <c r="K744" s="13" t="n">
-        <v>48937</v>
+        <v>80025</v>
       </c>
       <c r="L744" s="32" t="n">
-        <v>0.5571</v>
+        <v>0.5335</v>
       </c>
     </row>
     <row r="745">
@@ -41310,29 +41310,29 @@
         </is>
       </c>
       <c r="D745" s="15" t="n">
-        <v>1181378.1</v>
+        <v>1774322.14</v>
       </c>
       <c r="E745" s="15" t="n">
-        <v>6903233.07</v>
+        <v>11459391.65</v>
       </c>
       <c r="F745" s="16" t="n">
-        <v>0.4485</v>
+        <v>0.4779</v>
       </c>
       <c r="G745" s="16" t="n">
-        <v>0.3735</v>
+        <v>0.4018</v>
       </c>
       <c r="H745" s="16" t="n"/>
       <c r="I745" s="16" t="n">
-        <v>0.0535</v>
+        <v>0.0489</v>
       </c>
       <c r="J745" s="19" t="n">
-        <v>53107</v>
+        <v>82828</v>
       </c>
       <c r="K745" s="19" t="n">
-        <v>66314</v>
+        <v>103114</v>
       </c>
       <c r="L745" s="31" t="n">
-        <v>0.525</v>
+        <v>0.5338000000000001</v>
       </c>
     </row>
     <row r="746">
@@ -42234,29 +42234,29 @@
         </is>
       </c>
       <c r="D767" s="15" t="n">
-        <v>12611960.81</v>
+        <v>20077930.89</v>
       </c>
       <c r="E767" s="15" t="n">
-        <v>28240767.41</v>
+        <v>50838059.41</v>
       </c>
       <c r="F767" s="16" t="n">
-        <v>0.0725</v>
+        <v>0.1692</v>
       </c>
       <c r="G767" s="16" t="n">
-        <v>0.0127</v>
+        <v>0.1088</v>
       </c>
       <c r="H767" s="16" t="n"/>
       <c r="I767" s="16" t="n">
-        <v>0.1087</v>
+        <v>0.0843</v>
       </c>
       <c r="J767" s="19" t="n">
-        <v>231850</v>
+        <v>393594</v>
       </c>
       <c r="K767" s="19" t="n">
-        <v>382475</v>
+        <v>618685</v>
       </c>
       <c r="L767" s="31" t="n">
-        <v>0.602</v>
+        <v>0.604</v>
       </c>
     </row>
     <row r="768">
@@ -48450,29 +48450,29 @@
         </is>
       </c>
       <c r="D915" s="15" t="n">
-        <v>940836.46</v>
+        <v>1748076.87</v>
       </c>
       <c r="E915" s="15" t="n">
-        <v>9290472.369999999</v>
+        <v>19680716.72</v>
       </c>
       <c r="F915" s="16" t="n">
-        <v>0.59</v>
+        <v>0.6987</v>
       </c>
       <c r="G915" s="16" t="n">
-        <v>0.516</v>
+        <v>0.6246</v>
       </c>
       <c r="H915" s="16" t="n"/>
       <c r="I915" s="16" t="n">
-        <v>0.0198</v>
+        <v>0.0135</v>
       </c>
       <c r="J915" s="19" t="n">
-        <v>69180</v>
+        <v>130763</v>
       </c>
       <c r="K915" s="19" t="n">
-        <v>100704</v>
+        <v>183221</v>
       </c>
       <c r="L915" s="31" t="n">
-        <v>0.6805</v>
+        <v>0.6114000000000001</v>
       </c>
     </row>
     <row r="916">
@@ -48492,29 +48492,29 @@
         </is>
       </c>
       <c r="D916" s="9" t="n">
-        <v>4761873.38</v>
+        <v>7072915.11</v>
       </c>
       <c r="E916" s="9" t="n">
-        <v>4146731.61</v>
+        <v>5441957.98</v>
       </c>
       <c r="F916" s="10" t="n">
-        <v>-0.1038</v>
+        <v>-0.0804</v>
       </c>
       <c r="G916" s="10" t="n">
-        <v>-0.1542</v>
+        <v>-0.1313</v>
       </c>
       <c r="H916" s="10" t="n"/>
       <c r="I916" s="10" t="n">
-        <v>0.316</v>
+        <v>0.3216</v>
       </c>
       <c r="J916" s="13" t="n">
-        <v>12150</v>
+        <v>17477</v>
       </c>
       <c r="K916" s="13" t="n">
-        <v>61580</v>
+        <v>78006</v>
       </c>
       <c r="L916" s="32" t="n">
-        <v>0.5132</v>
+        <v>0.5737</v>
       </c>
     </row>
     <row r="917">
@@ -48534,29 +48534,29 @@
         </is>
       </c>
       <c r="D917" s="15" t="n">
-        <v>2449451.79</v>
+        <v>3565576.81</v>
       </c>
       <c r="E917" s="15" t="n">
-        <v>2608804.43</v>
+        <v>3286887.14</v>
       </c>
       <c r="F917" s="16" t="n">
-        <v>-0.0696</v>
+        <v>0.0158</v>
       </c>
       <c r="G917" s="16" t="n">
-        <v>-0.1279</v>
+        <v>-0.0413</v>
       </c>
       <c r="H917" s="16" t="n"/>
       <c r="I917" s="16" t="n">
-        <v>0.2536</v>
+        <v>0.2349</v>
       </c>
       <c r="J917" s="19" t="n">
-        <v>23352</v>
+        <v>32476</v>
       </c>
       <c r="K917" s="19" t="n">
-        <v>52995</v>
+        <v>70553</v>
       </c>
       <c r="L917" s="31" t="n">
-        <v>0.6372</v>
+        <v>0.6283</v>
       </c>
     </row>
     <row r="918">
@@ -48576,29 +48576,29 @@
         </is>
       </c>
       <c r="D918" s="9" t="n">
-        <v>1597502.07</v>
+        <v>2523574.89</v>
       </c>
       <c r="E918" s="9" t="n">
-        <v>2109404.57</v>
+        <v>3189453.25</v>
       </c>
       <c r="F918" s="10" t="n">
-        <v>0.1384</v>
+        <v>0.2309</v>
       </c>
       <c r="G918" s="10" t="n">
-        <v>0.0762</v>
+        <v>0.169</v>
       </c>
       <c r="H918" s="10" t="n"/>
       <c r="I918" s="10" t="n">
-        <v>0.1882</v>
+        <v>0.1642</v>
       </c>
       <c r="J918" s="13" t="n">
-        <v>26025</v>
+        <v>38637</v>
       </c>
       <c r="K918" s="13" t="n">
-        <v>35670</v>
+        <v>55622</v>
       </c>
       <c r="L918" s="32" t="n">
-        <v>0.6613</v>
+        <v>0.6434</v>
       </c>
     </row>
     <row r="919">
@@ -48618,29 +48618,29 @@
         </is>
       </c>
       <c r="D919" s="15" t="n">
-        <v>926710.15</v>
+        <v>1620694.1</v>
       </c>
       <c r="E919" s="15" t="n">
-        <v>1881681.34</v>
+        <v>3060715.75</v>
       </c>
       <c r="F919" s="16" t="n">
-        <v>0.1945</v>
+        <v>0.3003</v>
       </c>
       <c r="G919" s="16" t="n">
-        <v>0.1293</v>
+        <v>0.2347</v>
       </c>
       <c r="H919" s="16" t="n"/>
       <c r="I919" s="16" t="n">
-        <v>0.143</v>
+        <v>0.1187</v>
       </c>
       <c r="J919" s="19" t="n">
-        <v>22323</v>
+        <v>35183</v>
       </c>
       <c r="K919" s="19" t="n">
-        <v>29171</v>
+        <v>47664</v>
       </c>
       <c r="L919" s="31" t="n">
-        <v>0.6421</v>
+        <v>0.5937</v>
       </c>
     </row>
     <row r="920">
@@ -48660,29 +48660,29 @@
         </is>
       </c>
       <c r="D920" s="9" t="n">
-        <v>1134113.37</v>
+        <v>2064457.97</v>
       </c>
       <c r="E920" s="9" t="n">
-        <v>3336096.4</v>
+        <v>6468160.54</v>
       </c>
       <c r="F920" s="10" t="n">
-        <v>0.2822</v>
+        <v>0.4026</v>
       </c>
       <c r="G920" s="10" t="n">
-        <v>0.2106</v>
+        <v>0.3314</v>
       </c>
       <c r="H920" s="10" t="n"/>
       <c r="I920" s="10" t="n">
-        <v>0.098</v>
+        <v>0.073</v>
       </c>
       <c r="J920" s="13" t="n">
-        <v>39764</v>
+        <v>69200</v>
       </c>
       <c r="K920" s="13" t="n">
-        <v>49831</v>
+        <v>90051</v>
       </c>
       <c r="L920" s="32" t="n">
-        <v>0.6843</v>
+        <v>0.6254</v>
       </c>
     </row>
     <row r="921">
@@ -48702,29 +48702,29 @@
         </is>
       </c>
       <c r="D921" s="15" t="n">
-        <v>801473.6</v>
+        <v>1482635.15</v>
       </c>
       <c r="E921" s="15" t="n">
-        <v>4867576.69</v>
+        <v>9710168.02</v>
       </c>
       <c r="F921" s="16" t="n">
-        <v>0.3766</v>
+        <v>0.5309</v>
       </c>
       <c r="G921" s="16" t="n">
-        <v>0.3025</v>
+        <v>0.457</v>
       </c>
       <c r="H921" s="16" t="n"/>
       <c r="I921" s="16" t="n">
-        <v>0.0535</v>
+        <v>0.0369</v>
       </c>
       <c r="J921" s="19" t="n">
-        <v>39056</v>
+        <v>69858</v>
       </c>
       <c r="K921" s="19" t="n">
-        <v>52524</v>
+        <v>93568</v>
       </c>
       <c r="L921" s="31" t="n">
-        <v>0.649</v>
+        <v>0.596</v>
       </c>
     </row>
     <row r="922">
@@ -49164,29 +49164,29 @@
         </is>
       </c>
       <c r="D932" s="9" t="n">
-        <v>5787399.79</v>
+        <v>7112808.67</v>
       </c>
       <c r="E932" s="9" t="n">
-        <v>18652338.77</v>
+        <v>23562518.2</v>
       </c>
       <c r="F932" s="10" t="n">
-        <v>0.5235</v>
+        <v>0.423</v>
       </c>
       <c r="G932" s="10" t="n">
-        <v>0.4597</v>
+        <v>0.3588</v>
       </c>
       <c r="H932" s="10" t="n"/>
       <c r="I932" s="10" t="n">
-        <v>0.0443</v>
+        <v>0.0537</v>
       </c>
       <c r="J932" s="13" t="n">
-        <v>131992</v>
+        <v>151770</v>
       </c>
       <c r="K932" s="13" t="n">
-        <v>192719</v>
+        <v>217447</v>
       </c>
       <c r="L932" s="32" t="n">
-        <v>0.544</v>
+        <v>0.6244</v>
       </c>
     </row>
     <row r="933">
@@ -52146,29 +52146,29 @@
         </is>
       </c>
       <c r="D1003" s="15" t="n">
-        <v>1328733.45</v>
+        <v>1488704.64</v>
       </c>
       <c r="E1003" s="15" t="n">
-        <v>9022015.279999999</v>
+        <v>11257584.23</v>
       </c>
       <c r="F1003" s="16" t="n">
-        <v>0.8463000000000001</v>
+        <v>0.8159</v>
       </c>
       <c r="G1003" s="16" t="n">
-        <v>0.7751</v>
+        <v>0.7432</v>
       </c>
       <c r="H1003" s="16" t="n"/>
       <c r="I1003" s="16" t="n">
-        <v>0.0078</v>
+        <v>0.0094</v>
       </c>
       <c r="J1003" s="19" t="n">
-        <v>65217</v>
+        <v>72200</v>
       </c>
       <c r="K1003" s="19" t="n">
-        <v>89417</v>
+        <v>97771</v>
       </c>
       <c r="L1003" s="31" t="n">
-        <v>0.6092</v>
+        <v>0.6449</v>
       </c>
     </row>
     <row r="1004">
@@ -52188,29 +52188,29 @@
         </is>
       </c>
       <c r="D1004" s="9" t="n">
-        <v>934274.96</v>
+        <v>1399299.15</v>
       </c>
       <c r="E1004" s="9" t="n">
-        <v>674034.54</v>
+        <v>983092.04</v>
       </c>
       <c r="F1004" s="10" t="n">
-        <v>0.1796</v>
+        <v>0.0324</v>
       </c>
       <c r="G1004" s="10" t="n">
-        <v>0.1318</v>
+        <v>-0.0169</v>
       </c>
       <c r="H1004" s="10" t="n"/>
       <c r="I1004" s="10" t="n">
-        <v>0.2888</v>
+        <v>0.3473</v>
       </c>
       <c r="J1004" s="13" t="n">
-        <v>3258</v>
+        <v>4881</v>
       </c>
       <c r="K1004" s="13" t="n">
-        <v>8754</v>
+        <v>11795</v>
       </c>
       <c r="L1004" s="32" t="n">
-        <v>0.3551</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="1005">
@@ -52230,29 +52230,29 @@
         </is>
       </c>
       <c r="D1005" s="15" t="n">
-        <v>811199.89</v>
+        <v>973715.01</v>
       </c>
       <c r="E1005" s="15" t="n">
-        <v>868307.71</v>
+        <v>1067929.39</v>
       </c>
       <c r="F1005" s="16" t="n">
-        <v>0.2432</v>
+        <v>0.2012</v>
       </c>
       <c r="G1005" s="16" t="n">
-        <v>0.1875</v>
+        <v>0.1441</v>
       </c>
       <c r="H1005" s="16" t="n"/>
       <c r="I1005" s="16" t="n">
-        <v>0.1853</v>
+        <v>0.1956</v>
       </c>
       <c r="J1005" s="19" t="n">
-        <v>6850</v>
+        <v>8633</v>
       </c>
       <c r="K1005" s="19" t="n">
-        <v>13809</v>
+        <v>16071</v>
       </c>
       <c r="L1005" s="31" t="n">
-        <v>0.4941</v>
+        <v>0.5775</v>
       </c>
     </row>
     <row r="1006">
@@ -52272,29 +52272,29 @@
         </is>
       </c>
       <c r="D1006" s="9" t="n">
-        <v>790499.64</v>
+        <v>920145.01</v>
       </c>
       <c r="E1006" s="9" t="n">
-        <v>1250683.09</v>
+        <v>1454771.84</v>
       </c>
       <c r="F1006" s="10" t="n">
-        <v>0.3817</v>
+        <v>0.3678</v>
       </c>
       <c r="G1006" s="10" t="n">
-        <v>0.3193</v>
+        <v>0.3051</v>
       </c>
       <c r="H1006" s="10" t="n"/>
       <c r="I1006" s="10" t="n">
-        <v>0.1259</v>
+        <v>0.1346</v>
       </c>
       <c r="J1006" s="13" t="n">
-        <v>9190</v>
+        <v>11020</v>
       </c>
       <c r="K1006" s="13" t="n">
-        <v>16807</v>
+        <v>18961</v>
       </c>
       <c r="L1006" s="32" t="n">
-        <v>0.5593</v>
+        <v>0.6192</v>
       </c>
     </row>
     <row r="1007">
@@ -52314,29 +52314,29 @@
         </is>
       </c>
       <c r="D1007" s="15" t="n">
-        <v>516119.06</v>
+        <v>627554.58</v>
       </c>
       <c r="E1007" s="15" t="n">
-        <v>1412386.03</v>
+        <v>1779617.7</v>
       </c>
       <c r="F1007" s="16" t="n">
-        <v>0.5197000000000001</v>
+        <v>0.3994</v>
       </c>
       <c r="G1007" s="16" t="n">
-        <v>0.45</v>
+        <v>0.3291</v>
       </c>
       <c r="H1007" s="16" t="n"/>
       <c r="I1007" s="16" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0848</v>
       </c>
       <c r="J1007" s="19" t="n">
-        <v>8778</v>
+        <v>10359</v>
       </c>
       <c r="K1007" s="19" t="n">
-        <v>12648</v>
+        <v>14556</v>
       </c>
       <c r="L1007" s="31" t="n">
-        <v>0.6229</v>
+        <v>0.6863</v>
       </c>
     </row>
     <row r="1008">
@@ -52356,29 +52356,29 @@
         </is>
       </c>
       <c r="D1008" s="9" t="n">
-        <v>782164.61</v>
+        <v>943079.13</v>
       </c>
       <c r="E1008" s="9" t="n">
-        <v>2548289.1</v>
+        <v>3254599.14</v>
       </c>
       <c r="F1008" s="10" t="n">
-        <v>0.6152</v>
+        <v>0.5296</v>
       </c>
       <c r="G1008" s="10" t="n">
-        <v>0.5444</v>
+        <v>0.4574</v>
       </c>
       <c r="H1008" s="10" t="n"/>
       <c r="I1008" s="10" t="n">
-        <v>0.0443</v>
+        <v>0.0503</v>
       </c>
       <c r="J1008" s="13" t="n">
-        <v>19503</v>
+        <v>22577</v>
       </c>
       <c r="K1008" s="13" t="n">
-        <v>27743</v>
+        <v>31360</v>
       </c>
       <c r="L1008" s="32" t="n">
-        <v>0.6387</v>
+        <v>0.6981000000000001</v>
       </c>
     </row>
     <row r="1009">
@@ -52398,29 +52398,29 @@
         </is>
       </c>
       <c r="D1009" s="15" t="n">
-        <v>624408.1899999999</v>
+        <v>760311.15</v>
       </c>
       <c r="E1009" s="15" t="n">
-        <v>2876623.03</v>
+        <v>3764923.87</v>
       </c>
       <c r="F1009" s="16" t="n">
-        <v>0.7832</v>
+        <v>0.6111</v>
       </c>
       <c r="G1009" s="16" t="n">
-        <v>0.7127</v>
+        <v>0.5395</v>
       </c>
       <c r="H1009" s="16" t="n"/>
       <c r="I1009" s="16" t="n">
-        <v>0.0229</v>
+        <v>0.0264</v>
       </c>
       <c r="J1009" s="19" t="n">
-        <v>19196</v>
+        <v>22100</v>
       </c>
       <c r="K1009" s="19" t="n">
-        <v>23541</v>
+        <v>26933</v>
       </c>
       <c r="L1009" s="31" t="n">
-        <v>0.5492</v>
+        <v>0.6232</v>
       </c>
     </row>
     <row r="1010">
@@ -52818,26 +52818,26 @@
         </is>
       </c>
       <c r="D1019" s="15" t="n">
-        <v>7060685.14</v>
+        <v>7801878.9</v>
       </c>
       <c r="E1019" s="15" t="n">
-        <v>16438394.38</v>
+        <v>18179641.38</v>
       </c>
       <c r="F1019" s="16" t="n">
-        <v>0.2032</v>
+        <v>0.2154</v>
       </c>
       <c r="G1019" s="16" t="n">
-        <v>0.1484</v>
+        <v>0.1605</v>
       </c>
       <c r="H1019" s="16" t="n"/>
       <c r="I1019" s="16" t="n">
-        <v>0.1086</v>
+        <v>0.1101</v>
       </c>
       <c r="J1019" s="19" t="n">
-        <v>120542</v>
+        <v>133295</v>
       </c>
       <c r="K1019" s="19" t="n">
-        <v>293430</v>
+        <v>318089</v>
       </c>
       <c r="L1019" s="31" t="n">
         <v>0</v>
@@ -55506,26 +55506,26 @@
         </is>
       </c>
       <c r="D1083" s="15" t="n">
-        <v>307790.14</v>
+        <v>313560.69</v>
       </c>
       <c r="E1083" s="15" t="n">
-        <v>5597443.12</v>
+        <v>5823349.63</v>
       </c>
       <c r="F1083" s="16" t="n">
-        <v>0.7215</v>
+        <v>0.7224</v>
       </c>
       <c r="G1083" s="16" t="n">
-        <v>0.6534</v>
+        <v>0.6541</v>
       </c>
       <c r="H1083" s="16" t="n"/>
       <c r="I1083" s="16" t="n">
-        <v>0.027</v>
+        <v>0.0276</v>
       </c>
       <c r="J1083" s="19" t="n">
-        <v>16461</v>
+        <v>17111</v>
       </c>
       <c r="K1083" s="19" t="n">
-        <v>56304</v>
+        <v>57134</v>
       </c>
       <c r="L1083" s="31" t="n">
         <v>0</v>
@@ -55548,26 +55548,26 @@
         </is>
       </c>
       <c r="D1084" s="9" t="n">
-        <v>3024041.33</v>
+        <v>3388390.21</v>
       </c>
       <c r="E1084" s="9" t="n">
-        <v>2642444.32</v>
+        <v>2926327.77</v>
       </c>
       <c r="F1084" s="10" t="n">
-        <v>0.1555</v>
+        <v>0.1572</v>
       </c>
       <c r="G1084" s="10" t="n">
-        <v>0.1063</v>
+        <v>0.1079</v>
       </c>
       <c r="H1084" s="10" t="n"/>
       <c r="I1084" s="10" t="n">
-        <v>0.2431</v>
+        <v>0.243</v>
       </c>
       <c r="J1084" s="13" t="n">
-        <v>19642</v>
+        <v>22255</v>
       </c>
       <c r="K1084" s="13" t="n">
-        <v>63536</v>
+        <v>70784</v>
       </c>
       <c r="L1084" s="32" t="n">
         <v>0</v>
@@ -55590,26 +55590,26 @@
         </is>
       </c>
       <c r="D1085" s="15" t="n">
-        <v>1624798.15</v>
+        <v>1804675.99</v>
       </c>
       <c r="E1085" s="15" t="n">
-        <v>1177115.29</v>
+        <v>1356134.87</v>
       </c>
       <c r="F1085" s="16" t="n">
-        <v>0.0645</v>
+        <v>0.0882</v>
       </c>
       <c r="G1085" s="16" t="n">
-        <v>0.0106</v>
+        <v>0.034</v>
       </c>
       <c r="H1085" s="16" t="n"/>
       <c r="I1085" s="16" t="n">
-        <v>0.1639</v>
+        <v>0.1642</v>
       </c>
       <c r="J1085" s="19" t="n">
-        <v>20961</v>
+        <v>23684</v>
       </c>
       <c r="K1085" s="19" t="n">
-        <v>45776</v>
+        <v>51657</v>
       </c>
       <c r="L1085" s="31" t="n">
         <v>0</v>
@@ -55632,26 +55632,26 @@
         </is>
       </c>
       <c r="D1086" s="9" t="n">
-        <v>882416.52</v>
+        <v>980536.92</v>
       </c>
       <c r="E1086" s="9" t="n">
-        <v>1269326.87</v>
+        <v>1518001.2</v>
       </c>
       <c r="F1086" s="10" t="n">
-        <v>0.2639</v>
+        <v>0.2997</v>
       </c>
       <c r="G1086" s="10" t="n">
-        <v>0.2045</v>
+        <v>0.2398</v>
       </c>
       <c r="H1086" s="10" t="n"/>
       <c r="I1086" s="10" t="n">
-        <v>0.1129</v>
+        <v>0.1125</v>
       </c>
       <c r="J1086" s="13" t="n">
-        <v>18852</v>
+        <v>21014</v>
       </c>
       <c r="K1086" s="13" t="n">
-        <v>34950</v>
+        <v>38583</v>
       </c>
       <c r="L1086" s="32" t="n">
         <v>0</v>
@@ -55674,26 +55674,26 @@
         </is>
       </c>
       <c r="D1087" s="15" t="n">
-        <v>469058.94</v>
+        <v>508289.9</v>
       </c>
       <c r="E1087" s="15" t="n">
-        <v>784322.64</v>
+        <v>944251.4399999999</v>
       </c>
       <c r="F1087" s="16" t="n">
-        <v>0.0214</v>
+        <v>0.0818</v>
       </c>
       <c r="G1087" s="16" t="n">
-        <v>-0.0394</v>
+        <v>0.0209</v>
       </c>
       <c r="H1087" s="16" t="n"/>
       <c r="I1087" s="16" t="n">
         <v>0.07829999999999999</v>
       </c>
       <c r="J1087" s="19" t="n">
-        <v>11779</v>
+        <v>13162</v>
       </c>
       <c r="K1087" s="19" t="n">
-        <v>18962</v>
+        <v>21547</v>
       </c>
       <c r="L1087" s="31" t="n">
         <v>0</v>
@@ -55716,26 +55716,26 @@
         </is>
       </c>
       <c r="D1088" s="9" t="n">
-        <v>458461.06</v>
+        <v>495358.3</v>
       </c>
       <c r="E1088" s="9" t="n">
-        <v>1502591.77</v>
+        <v>1817891.54</v>
       </c>
       <c r="F1088" s="10" t="n">
-        <v>0.4117</v>
+        <v>0.4191</v>
       </c>
       <c r="G1088" s="10" t="n">
-        <v>0.3486</v>
+        <v>0.3553</v>
       </c>
       <c r="H1088" s="10" t="n"/>
       <c r="I1088" s="10" t="n">
-        <v>0.0527</v>
+        <v>0.0529</v>
       </c>
       <c r="J1088" s="13" t="n">
-        <v>17711</v>
+        <v>19516</v>
       </c>
       <c r="K1088" s="13" t="n">
-        <v>26875</v>
+        <v>29312</v>
       </c>
       <c r="L1088" s="32" t="n">
         <v>0</v>
@@ -55758,26 +55758,26 @@
         </is>
       </c>
       <c r="D1089" s="15" t="n">
-        <v>294119</v>
+        <v>311066.89</v>
       </c>
       <c r="E1089" s="15" t="n">
-        <v>3465150.37</v>
+        <v>3793684.94</v>
       </c>
       <c r="F1089" s="16" t="n">
-        <v>0.6998</v>
+        <v>0.7044</v>
       </c>
       <c r="G1089" s="16" t="n">
-        <v>0.6331</v>
+        <v>0.6371</v>
       </c>
       <c r="H1089" s="16" t="n"/>
       <c r="I1089" s="16" t="n">
-        <v>0.0297</v>
+        <v>0.0291</v>
       </c>
       <c r="J1089" s="19" t="n">
-        <v>15136</v>
+        <v>16553</v>
       </c>
       <c r="K1089" s="19" t="n">
-        <v>47027</v>
+        <v>49072</v>
       </c>
       <c r="L1089" s="31" t="n">
         <v>0</v>
@@ -56304,26 +56304,26 @@
         </is>
       </c>
       <c r="D1102" s="9" t="n">
-        <v>149631251.42</v>
+        <v>173041582.07</v>
       </c>
       <c r="E1102" s="9" t="n">
-        <v>660404073.71</v>
+        <v>769592665.4</v>
       </c>
       <c r="F1102" s="10" t="n">
-        <v>0.1792</v>
+        <v>0.1624</v>
       </c>
       <c r="G1102" s="10" t="n">
-        <v>0.1205</v>
+        <v>0.1035</v>
       </c>
       <c r="H1102" s="10" t="n"/>
       <c r="I1102" s="10" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.09320000000000001</v>
       </c>
       <c r="J1102" s="13" t="n">
-        <v>3643230</v>
+        <v>4242855</v>
       </c>
       <c r="K1102" s="13" t="n">
-        <v>7105485</v>
+        <v>8164342</v>
       </c>
       <c r="L1102" s="32" t="n">
         <v>0</v>
@@ -59874,26 +59874,26 @@
         </is>
       </c>
       <c r="D1187" s="15" t="n">
-        <v>19672343.15</v>
+        <v>22126280.09</v>
       </c>
       <c r="E1187" s="15" t="n">
-        <v>345643037.93</v>
+        <v>393137874.88</v>
       </c>
       <c r="F1187" s="16" t="n">
-        <v>0.5057</v>
+        <v>0.4792</v>
       </c>
       <c r="G1187" s="16" t="n">
-        <v>0.4273</v>
+        <v>0.3995</v>
       </c>
       <c r="H1187" s="16" t="n"/>
       <c r="I1187" s="16" t="n">
-        <v>0.026</v>
+        <v>0.0258</v>
       </c>
       <c r="J1187" s="19" t="n">
-        <v>1429741</v>
+        <v>1641425</v>
       </c>
       <c r="K1187" s="19" t="n">
-        <v>2270439</v>
+        <v>2550350</v>
       </c>
       <c r="L1187" s="31" t="n">
         <v>0</v>
@@ -59916,26 +59916,26 @@
         </is>
       </c>
       <c r="D1188" s="9" t="n">
-        <v>37386148.11</v>
+        <v>44373033.51</v>
       </c>
       <c r="E1188" s="9" t="n">
-        <v>19721777.72</v>
+        <v>23076566.87</v>
       </c>
       <c r="F1188" s="10" t="n">
-        <v>0.0517</v>
+        <v>0.0373</v>
       </c>
       <c r="G1188" s="10" t="n">
-        <v>0.0098</v>
+        <v>-0.0046</v>
       </c>
       <c r="H1188" s="10" t="n"/>
       <c r="I1188" s="10" t="n">
-        <v>0.3107</v>
+        <v>0.3084</v>
       </c>
       <c r="J1188" s="13" t="n">
-        <v>164384</v>
+        <v>190962</v>
       </c>
       <c r="K1188" s="13" t="n">
-        <v>717634</v>
+        <v>850472</v>
       </c>
       <c r="L1188" s="32" t="n">
         <v>0</v>
@@ -59958,26 +59958,26 @@
         </is>
       </c>
       <c r="D1189" s="15" t="n">
-        <v>24827997.62</v>
+        <v>28991515.83</v>
       </c>
       <c r="E1189" s="15" t="n">
-        <v>24998791.87</v>
+        <v>29347615.6</v>
       </c>
       <c r="F1189" s="16" t="n">
-        <v>0.0545</v>
+        <v>0.0513</v>
       </c>
       <c r="G1189" s="16" t="n">
-        <v>0.0032</v>
+        <v>-0.0001</v>
       </c>
       <c r="H1189" s="16" t="n"/>
       <c r="I1189" s="16" t="n">
-        <v>0.2358</v>
+        <v>0.234</v>
       </c>
       <c r="J1189" s="19" t="n">
-        <v>244021</v>
+        <v>286679</v>
       </c>
       <c r="K1189" s="19" t="n">
-        <v>629823</v>
+        <v>752295</v>
       </c>
       <c r="L1189" s="31" t="n">
         <v>0</v>
@@ -60000,26 +60000,26 @@
         </is>
       </c>
       <c r="D1190" s="9" t="n">
-        <v>19029822.53</v>
+        <v>22059810.53</v>
       </c>
       <c r="E1190" s="9" t="n">
-        <v>29571409.06</v>
+        <v>35507287.71</v>
       </c>
       <c r="F1190" s="10" t="n">
-        <v>0.0861</v>
+        <v>0.07770000000000001</v>
       </c>
       <c r="G1190" s="10" t="n">
-        <v>0.0294</v>
+        <v>0.0205</v>
       </c>
       <c r="H1190" s="10" t="n"/>
       <c r="I1190" s="10" t="n">
-        <v>0.1867</v>
+        <v>0.1851</v>
       </c>
       <c r="J1190" s="13" t="n">
-        <v>283612</v>
+        <v>335942</v>
       </c>
       <c r="K1190" s="13" t="n">
-        <v>611514</v>
+        <v>730295</v>
       </c>
       <c r="L1190" s="32" t="n">
         <v>0</v>
@@ -60042,26 +60042,26 @@
         </is>
       </c>
       <c r="D1191" s="15" t="n">
-        <v>12932127.86</v>
+        <v>14890635.15</v>
       </c>
       <c r="E1191" s="15" t="n">
-        <v>33144333.9</v>
+        <v>39725290.12</v>
       </c>
       <c r="F1191" s="16" t="n">
-        <v>0.1019</v>
+        <v>0.09660000000000001</v>
       </c>
       <c r="G1191" s="16" t="n">
-        <v>0.038</v>
+        <v>0.0323</v>
       </c>
       <c r="H1191" s="16" t="n"/>
       <c r="I1191" s="16" t="n">
-        <v>0.148</v>
+        <v>0.146</v>
       </c>
       <c r="J1191" s="19" t="n">
-        <v>275872</v>
+        <v>327898</v>
       </c>
       <c r="K1191" s="19" t="n">
-        <v>537697</v>
+        <v>625341</v>
       </c>
       <c r="L1191" s="31" t="n">
         <v>0</v>
@@ -60084,26 +60084,26 @@
         </is>
       </c>
       <c r="D1192" s="9" t="n">
-        <v>18507658.05</v>
+        <v>21016961.99</v>
       </c>
       <c r="E1192" s="9" t="n">
-        <v>71330219.26000001</v>
+        <v>92180541.83</v>
       </c>
       <c r="F1192" s="10" t="n">
-        <v>0.2238</v>
+        <v>0.204</v>
       </c>
       <c r="G1192" s="10" t="n">
-        <v>0.1562</v>
+        <v>0.1357</v>
       </c>
       <c r="H1192" s="10" t="n"/>
       <c r="I1192" s="10" t="n">
-        <v>0.106</v>
+        <v>0.1053</v>
       </c>
       <c r="J1192" s="13" t="n">
-        <v>543789</v>
+        <v>640409</v>
       </c>
       <c r="K1192" s="13" t="n">
-        <v>982408</v>
+        <v>1125090</v>
       </c>
       <c r="L1192" s="32" t="n">
         <v>0</v>
@@ -60126,26 +60126,26 @@
         </is>
       </c>
       <c r="D1193" s="15" t="n">
-        <v>17275154.11</v>
+        <v>19583344.97</v>
       </c>
       <c r="E1193" s="15" t="n">
-        <v>135994503.97</v>
+        <v>156617488.4</v>
       </c>
       <c r="F1193" s="16" t="n">
-        <v>0.3753</v>
+        <v>0.3532</v>
       </c>
       <c r="G1193" s="16" t="n">
-        <v>0.3029</v>
+        <v>0.2803</v>
       </c>
       <c r="H1193" s="16" t="n"/>
       <c r="I1193" s="16" t="n">
-        <v>0.0606</v>
+        <v>0.0605</v>
       </c>
       <c r="J1193" s="19" t="n">
-        <v>701811</v>
+        <v>819540</v>
       </c>
       <c r="K1193" s="19" t="n">
-        <v>1355970</v>
+        <v>1530499</v>
       </c>
       <c r="L1193" s="31" t="n">
         <v>0</v>
@@ -60630,26 +60630,26 @@
         </is>
       </c>
       <c r="D1205" s="15" t="n">
-        <v>14544946.33</v>
+        <v>17509247.78</v>
       </c>
       <c r="E1205" s="15" t="n">
-        <v>38995788.53</v>
+        <v>50600636.06</v>
       </c>
       <c r="F1205" s="16" t="n">
-        <v>0.1522</v>
+        <v>0.1874</v>
       </c>
       <c r="G1205" s="16" t="n">
-        <v>0.0921</v>
+        <v>0.1263</v>
       </c>
       <c r="H1205" s="16" t="n"/>
       <c r="I1205" s="16" t="n">
-        <v>0.1017</v>
+        <v>0.1126</v>
       </c>
       <c r="J1205" s="19" t="n">
-        <v>243369</v>
+        <v>293342</v>
       </c>
       <c r="K1205" s="19" t="n">
-        <v>359849</v>
+        <v>438613</v>
       </c>
       <c r="L1205" s="31" t="n">
         <v>0</v>
@@ -63906,26 +63906,26 @@
         </is>
       </c>
       <c r="D1283" s="15" t="n">
-        <v>1021743</v>
+        <v>1238517.28</v>
       </c>
       <c r="E1283" s="15" t="n">
-        <v>14266549.63</v>
+        <v>17465829.02</v>
       </c>
       <c r="F1283" s="16" t="n">
-        <v>0.4846</v>
+        <v>0.5268</v>
       </c>
       <c r="G1283" s="16" t="n">
-        <v>0.4111</v>
+        <v>0.4502</v>
       </c>
       <c r="H1283" s="16" t="n"/>
       <c r="I1283" s="16" t="n">
-        <v>0.0209</v>
+        <v>0.0265</v>
       </c>
       <c r="J1283" s="19" t="n">
-        <v>71033</v>
+        <v>85731</v>
       </c>
       <c r="K1283" s="19" t="n">
-        <v>86259</v>
+        <v>104555</v>
       </c>
       <c r="L1283" s="31" t="n">
         <v>0</v>
@@ -63948,26 +63948,26 @@
         </is>
       </c>
       <c r="D1284" s="9" t="n">
-        <v>4404189.53</v>
+        <v>5150343.34</v>
       </c>
       <c r="E1284" s="9" t="n">
-        <v>3182474.07</v>
+        <v>3970718.3</v>
       </c>
       <c r="F1284" s="10" t="n">
-        <v>0.0424</v>
+        <v>0.0673</v>
       </c>
       <c r="G1284" s="10" t="n">
-        <v>-0.0106</v>
+        <v>0.0141</v>
       </c>
       <c r="H1284" s="10" t="n"/>
       <c r="I1284" s="10" t="n">
-        <v>0.3471</v>
+        <v>0.3506</v>
       </c>
       <c r="J1284" s="13" t="n">
-        <v>14078</v>
+        <v>16741</v>
       </c>
       <c r="K1284" s="13" t="n">
-        <v>42399</v>
+        <v>51905</v>
       </c>
       <c r="L1284" s="32" t="n">
         <v>0</v>
@@ -63990,26 +63990,26 @@
         </is>
       </c>
       <c r="D1285" s="15" t="n">
-        <v>2907431.17</v>
+        <v>3534694.25</v>
       </c>
       <c r="E1285" s="15" t="n">
-        <v>2642744.89</v>
+        <v>3872150.46</v>
       </c>
       <c r="F1285" s="16" t="n">
-        <v>0.1182</v>
+        <v>0.1453</v>
       </c>
       <c r="G1285" s="16" t="n">
-        <v>0.06270000000000001</v>
+        <v>0.0887</v>
       </c>
       <c r="H1285" s="16" t="n"/>
       <c r="I1285" s="16" t="n">
-        <v>0.2199</v>
+        <v>0.229</v>
       </c>
       <c r="J1285" s="19" t="n">
-        <v>23546</v>
+        <v>28951</v>
       </c>
       <c r="K1285" s="19" t="n">
-        <v>40792</v>
+        <v>52170</v>
       </c>
       <c r="L1285" s="31" t="n">
         <v>0</v>
@@ -64032,26 +64032,26 @@
         </is>
       </c>
       <c r="D1286" s="9" t="n">
-        <v>2082522.66</v>
+        <v>2489619.95</v>
       </c>
       <c r="E1286" s="9" t="n">
-        <v>2915964</v>
+        <v>4181137.42</v>
       </c>
       <c r="F1286" s="10" t="n">
-        <v>0.1049</v>
+        <v>0.1203</v>
       </c>
       <c r="G1286" s="10" t="n">
-        <v>0.0454</v>
+        <v>0.0587</v>
       </c>
       <c r="H1286" s="10" t="n"/>
       <c r="I1286" s="10" t="n">
-        <v>0.1604</v>
+        <v>0.1714</v>
       </c>
       <c r="J1286" s="13" t="n">
-        <v>27609</v>
+        <v>33775</v>
       </c>
       <c r="K1286" s="13" t="n">
-        <v>42106</v>
+        <v>52334</v>
       </c>
       <c r="L1286" s="32" t="n">
         <v>0</v>
@@ -64074,26 +64074,26 @@
         </is>
       </c>
       <c r="D1287" s="15" t="n">
-        <v>1405866.26</v>
+        <v>1780955.66</v>
       </c>
       <c r="E1287" s="15" t="n">
-        <v>3197953.9</v>
+        <v>4230021.87</v>
       </c>
       <c r="F1287" s="16" t="n">
-        <v>0.2589</v>
+        <v>0.3167</v>
       </c>
       <c r="G1287" s="16" t="n">
-        <v>0.1947</v>
+        <v>0.2531</v>
       </c>
       <c r="H1287" s="16" t="n"/>
       <c r="I1287" s="16" t="n">
-        <v>0.1213</v>
+        <v>0.1367</v>
       </c>
       <c r="J1287" s="19" t="n">
-        <v>23868</v>
+        <v>29010</v>
       </c>
       <c r="K1287" s="19" t="n">
-        <v>34615</v>
+        <v>42354</v>
       </c>
       <c r="L1287" s="31" t="n">
         <v>0</v>
@@ -64116,26 +64116,26 @@
         </is>
       </c>
       <c r="D1288" s="9" t="n">
-        <v>1725216.1</v>
+        <v>2092677.12</v>
       </c>
       <c r="E1288" s="9" t="n">
-        <v>5841007.6</v>
+        <v>8161580.94</v>
       </c>
       <c r="F1288" s="10" t="n">
-        <v>0.1742</v>
+        <v>0.2098</v>
       </c>
       <c r="G1288" s="10" t="n">
-        <v>0.1057</v>
+        <v>0.1407</v>
       </c>
       <c r="H1288" s="10" t="n"/>
       <c r="I1288" s="10" t="n">
-        <v>0.0854</v>
+        <v>0.1015</v>
       </c>
       <c r="J1288" s="13" t="n">
-        <v>44534</v>
+        <v>53415</v>
       </c>
       <c r="K1288" s="13" t="n">
-        <v>59095</v>
+        <v>71418</v>
       </c>
       <c r="L1288" s="32" t="n">
         <v>0</v>
@@ -64158,26 +64158,26 @@
         </is>
       </c>
       <c r="D1289" s="15" t="n">
-        <v>997977.61</v>
+        <v>1222440.18</v>
       </c>
       <c r="E1289" s="15" t="n">
-        <v>6949094.45</v>
+        <v>8719198.050000001</v>
       </c>
       <c r="F1289" s="16" t="n">
-        <v>0.3053</v>
+        <v>0.3815</v>
       </c>
       <c r="G1289" s="16" t="n">
-        <v>0.2336</v>
+        <v>0.3078</v>
       </c>
       <c r="H1289" s="16" t="n"/>
       <c r="I1289" s="16" t="n">
-        <v>0.0534</v>
+        <v>0.0672</v>
       </c>
       <c r="J1289" s="19" t="n">
-        <v>38701</v>
+        <v>45719</v>
       </c>
       <c r="K1289" s="19" t="n">
-        <v>54583</v>
+        <v>63877</v>
       </c>
       <c r="L1289" s="31" t="n">
         <v>0</v>
@@ -64997,7 +64997,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-26 06:37 UTC</t>
+          <t>2026-10-26 07:26 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-26 14:27 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8605,7 +8605,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 07:26 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 14:27 UTC.</t>
         </is>
       </c>
     </row>
@@ -37488,29 +37488,29 @@
         </is>
       </c>
       <c r="D654" s="9" t="n">
-        <v>13425865.55</v>
+        <v>13434386.18</v>
       </c>
       <c r="E654" s="9" t="n">
-        <v>78976163.79000001</v>
+        <v>79016591.43000001</v>
       </c>
       <c r="F654" s="10" t="n">
-        <v>0.346</v>
+        <v>0.3448</v>
       </c>
       <c r="G654" s="10" t="n">
-        <v>0.28</v>
+        <v>0.2787</v>
       </c>
       <c r="H654" s="10" t="n"/>
       <c r="I654" s="10" t="n">
-        <v>0.0587</v>
+        <v>0.0588</v>
       </c>
       <c r="J654" s="13" t="n">
-        <v>508897</v>
+        <v>509115</v>
       </c>
       <c r="K654" s="13" t="n">
-        <v>691754</v>
+        <v>692036</v>
       </c>
       <c r="L654" s="32" t="n">
-        <v>0.5457</v>
+        <v>0.5456</v>
       </c>
     </row>
     <row r="655">
@@ -41058,29 +41058,29 @@
         </is>
       </c>
       <c r="D739" s="15" t="n">
-        <v>3373365.76</v>
+        <v>3374711.99</v>
       </c>
       <c r="E739" s="15" t="n">
-        <v>52518955.28</v>
+        <v>52525284.47</v>
       </c>
       <c r="F739" s="16" t="n">
-        <v>0.6208</v>
+        <v>0.6192</v>
       </c>
       <c r="G739" s="16" t="n">
-        <v>0.5421</v>
+        <v>0.5404</v>
       </c>
       <c r="H739" s="16" t="n"/>
       <c r="I739" s="16" t="n">
         <v>0.0141</v>
       </c>
       <c r="J739" s="19" t="n">
-        <v>278296</v>
+        <v>278347</v>
       </c>
       <c r="K739" s="19" t="n">
-        <v>373023</v>
+        <v>373086</v>
       </c>
       <c r="L739" s="31" t="n">
-        <v>0.5618</v>
+        <v>0.5616</v>
       </c>
     </row>
     <row r="740">
@@ -41100,29 +41100,29 @@
         </is>
       </c>
       <c r="D740" s="9" t="n">
-        <v>1794111.11</v>
+        <v>1796216.71</v>
       </c>
       <c r="E740" s="9" t="n">
-        <v>947688.9399999999</v>
+        <v>947888.11</v>
       </c>
       <c r="F740" s="10" t="n">
-        <v>0.2089</v>
+        <v>0.2083</v>
       </c>
       <c r="G740" s="10" t="n">
-        <v>0.1661</v>
+        <v>0.1654</v>
       </c>
       <c r="H740" s="10" t="n"/>
       <c r="I740" s="10" t="n">
-        <v>0.33</v>
+        <v>0.3298</v>
       </c>
       <c r="J740" s="13" t="n">
-        <v>9317</v>
+        <v>9353</v>
       </c>
       <c r="K740" s="13" t="n">
-        <v>23481</v>
+        <v>23537</v>
       </c>
       <c r="L740" s="32" t="n">
-        <v>0.5024</v>
+        <v>0.5029</v>
       </c>
     </row>
     <row r="741">
@@ -41142,10 +41142,10 @@
         </is>
       </c>
       <c r="D741" s="15" t="n">
-        <v>1832181.65</v>
+        <v>1833525.19</v>
       </c>
       <c r="E741" s="15" t="n">
-        <v>1738735.54</v>
+        <v>1739906.79</v>
       </c>
       <c r="F741" s="16" t="n">
         <v>0.1327</v>
@@ -41155,16 +41155,16 @@
       </c>
       <c r="H741" s="16" t="n"/>
       <c r="I741" s="16" t="n">
-        <v>0.2407</v>
+        <v>0.2408</v>
       </c>
       <c r="J741" s="19" t="n">
-        <v>19895</v>
+        <v>19929</v>
       </c>
       <c r="K741" s="19" t="n">
-        <v>35709</v>
+        <v>35752</v>
       </c>
       <c r="L741" s="31" t="n">
-        <v>0.5664</v>
+        <v>0.5662</v>
       </c>
     </row>
     <row r="742">
@@ -41184,29 +41184,29 @@
         </is>
       </c>
       <c r="D742" s="9" t="n">
-        <v>1492185.47</v>
+        <v>1493390.18</v>
       </c>
       <c r="E742" s="9" t="n">
-        <v>2549511.1</v>
+        <v>2555996.44</v>
       </c>
       <c r="F742" s="10" t="n">
-        <v>0.2081</v>
+        <v>0.2033</v>
       </c>
       <c r="G742" s="10" t="n">
-        <v>0.1446</v>
+        <v>0.1397</v>
       </c>
       <c r="H742" s="10" t="n"/>
       <c r="I742" s="10" t="n">
-        <v>0.1742</v>
+        <v>0.1745</v>
       </c>
       <c r="J742" s="13" t="n">
-        <v>26653</v>
+        <v>26680</v>
       </c>
       <c r="K742" s="13" t="n">
-        <v>38128</v>
+        <v>38158</v>
       </c>
       <c r="L742" s="32" t="n">
-        <v>0.5714</v>
+        <v>0.5712</v>
       </c>
     </row>
     <row r="743">
@@ -41226,29 +41226,29 @@
         </is>
       </c>
       <c r="D743" s="15" t="n">
-        <v>1201921.94</v>
+        <v>1202428.39</v>
       </c>
       <c r="E743" s="15" t="n">
-        <v>3153162.49</v>
+        <v>3153438.12</v>
       </c>
       <c r="F743" s="16" t="n">
-        <v>0.2208</v>
+        <v>0.2205</v>
       </c>
       <c r="G743" s="16" t="n">
-        <v>0.1534</v>
+        <v>0.1531</v>
       </c>
       <c r="H743" s="16" t="n"/>
       <c r="I743" s="16" t="n">
-        <v>0.1343</v>
+        <v>0.1345</v>
       </c>
       <c r="J743" s="19" t="n">
-        <v>28948</v>
+        <v>28961</v>
       </c>
       <c r="K743" s="19" t="n">
-        <v>38274</v>
+        <v>38290</v>
       </c>
       <c r="L743" s="31" t="n">
-        <v>0.539</v>
+        <v>0.5387999999999999</v>
       </c>
     </row>
     <row r="744">
@@ -41268,29 +41268,29 @@
         </is>
       </c>
       <c r="D744" s="9" t="n">
-        <v>1957777.49</v>
+        <v>1959498.14</v>
       </c>
       <c r="E744" s="9" t="n">
-        <v>6608718.79</v>
+        <v>6633026.8</v>
       </c>
       <c r="F744" s="10" t="n">
-        <v>0.2602</v>
+        <v>0.2598</v>
       </c>
       <c r="G744" s="10" t="n">
-        <v>0.1919</v>
+        <v>0.1915</v>
       </c>
       <c r="H744" s="10" t="n"/>
       <c r="I744" s="10" t="n">
-        <v>0.0878</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="J744" s="13" t="n">
-        <v>62960</v>
+        <v>62991</v>
       </c>
       <c r="K744" s="13" t="n">
-        <v>80025</v>
+        <v>80068</v>
       </c>
       <c r="L744" s="32" t="n">
-        <v>0.5335</v>
+        <v>0.5334</v>
       </c>
     </row>
     <row r="745">
@@ -41310,29 +41310,29 @@
         </is>
       </c>
       <c r="D745" s="15" t="n">
-        <v>1774322.14</v>
+        <v>1774615.58</v>
       </c>
       <c r="E745" s="15" t="n">
-        <v>11459391.65</v>
+        <v>11461050.71</v>
       </c>
       <c r="F745" s="16" t="n">
-        <v>0.4779</v>
+        <v>0.4774</v>
       </c>
       <c r="G745" s="16" t="n">
-        <v>0.4018</v>
+        <v>0.4013</v>
       </c>
       <c r="H745" s="16" t="n"/>
       <c r="I745" s="16" t="n">
-        <v>0.0489</v>
+        <v>0.049</v>
       </c>
       <c r="J745" s="19" t="n">
-        <v>82828</v>
+        <v>82854</v>
       </c>
       <c r="K745" s="19" t="n">
-        <v>103114</v>
+        <v>103145</v>
       </c>
       <c r="L745" s="31" t="n">
-        <v>0.5338000000000001</v>
+        <v>0.5337</v>
       </c>
     </row>
     <row r="746">
@@ -56262,10 +56262,10 @@
         </is>
       </c>
       <c r="D1101" s="15" t="n">
-        <v>151943202.19</v>
+        <v>151943211.91</v>
       </c>
       <c r="E1101" s="15" t="n">
-        <v>606885933.46</v>
+        <v>606885955.53</v>
       </c>
       <c r="F1101" s="16" t="n">
         <v>0.07630000000000001</v>
@@ -56278,10 +56278,10 @@
         <v>0.1029</v>
       </c>
       <c r="J1101" s="19" t="n">
-        <v>3671150</v>
+        <v>3671152</v>
       </c>
       <c r="K1101" s="19" t="n">
-        <v>7097443</v>
+        <v>7097446</v>
       </c>
       <c r="L1101" s="31" t="n">
         <v>0</v>
@@ -56304,26 +56304,26 @@
         </is>
       </c>
       <c r="D1102" s="9" t="n">
-        <v>173041582.07</v>
+        <v>173079510.38</v>
       </c>
       <c r="E1102" s="9" t="n">
-        <v>769592665.4</v>
+        <v>769940496.97</v>
       </c>
       <c r="F1102" s="10" t="n">
-        <v>0.1624</v>
+        <v>0.1623</v>
       </c>
       <c r="G1102" s="10" t="n">
-        <v>0.1035</v>
+        <v>0.1034</v>
       </c>
       <c r="H1102" s="10" t="n"/>
       <c r="I1102" s="10" t="n">
         <v>0.09320000000000001</v>
       </c>
       <c r="J1102" s="13" t="n">
-        <v>4242855</v>
+        <v>4243936</v>
       </c>
       <c r="K1102" s="13" t="n">
-        <v>8164342</v>
+        <v>8166329</v>
       </c>
       <c r="L1102" s="32" t="n">
         <v>0</v>
@@ -59622,7 +59622,7 @@
         </is>
       </c>
       <c r="D1181" s="15" t="n">
-        <v>40928654.79</v>
+        <v>40928664.18</v>
       </c>
       <c r="E1181" s="15" t="n">
         <v>20763452.89</v>
@@ -59638,10 +59638,10 @@
         <v>0.3061</v>
       </c>
       <c r="J1181" s="19" t="n">
-        <v>180075</v>
+        <v>180076</v>
       </c>
       <c r="K1181" s="19" t="n">
-        <v>776825</v>
+        <v>776826</v>
       </c>
       <c r="L1181" s="31" t="n">
         <v>0</v>
@@ -59664,10 +59664,10 @@
         </is>
       </c>
       <c r="D1182" s="9" t="n">
-        <v>26405659.51</v>
+        <v>26405659.85</v>
       </c>
       <c r="E1182" s="9" t="n">
-        <v>26088934.78</v>
+        <v>26088956.84</v>
       </c>
       <c r="F1182" s="10" t="n">
         <v>0.0262</v>
@@ -59680,10 +59680,10 @@
         <v>0.2383</v>
       </c>
       <c r="J1182" s="13" t="n">
-        <v>266496</v>
+        <v>266497</v>
       </c>
       <c r="K1182" s="13" t="n">
-        <v>714422</v>
+        <v>714424</v>
       </c>
       <c r="L1182" s="32" t="n">
         <v>0</v>
@@ -59874,13 +59874,13 @@
         </is>
       </c>
       <c r="D1187" s="15" t="n">
-        <v>22126280.09</v>
+        <v>22129287.86</v>
       </c>
       <c r="E1187" s="15" t="n">
-        <v>393137874.88</v>
+        <v>393164737.13</v>
       </c>
       <c r="F1187" s="16" t="n">
-        <v>0.4792</v>
+        <v>0.4793</v>
       </c>
       <c r="G1187" s="16" t="n">
         <v>0.3995</v>
@@ -59890,10 +59890,10 @@
         <v>0.0258</v>
       </c>
       <c r="J1187" s="19" t="n">
-        <v>1641425</v>
+        <v>1641690</v>
       </c>
       <c r="K1187" s="19" t="n">
-        <v>2550350</v>
+        <v>2550932</v>
       </c>
       <c r="L1187" s="31" t="n">
         <v>0</v>
@@ -59916,10 +59916,10 @@
         </is>
       </c>
       <c r="D1188" s="9" t="n">
-        <v>44373033.51</v>
+        <v>44386665.62</v>
       </c>
       <c r="E1188" s="9" t="n">
-        <v>23076566.87</v>
+        <v>23092351.44</v>
       </c>
       <c r="F1188" s="10" t="n">
         <v>0.0373</v>
@@ -59932,10 +59932,10 @@
         <v>0.3084</v>
       </c>
       <c r="J1188" s="13" t="n">
-        <v>190962</v>
+        <v>191147</v>
       </c>
       <c r="K1188" s="13" t="n">
-        <v>850472</v>
+        <v>850862</v>
       </c>
       <c r="L1188" s="32" t="n">
         <v>0</v>
@@ -59958,10 +59958,10 @@
         </is>
       </c>
       <c r="D1189" s="15" t="n">
-        <v>28991515.83</v>
+        <v>28995809.94</v>
       </c>
       <c r="E1189" s="15" t="n">
-        <v>29347615.6</v>
+        <v>29381447.48</v>
       </c>
       <c r="F1189" s="16" t="n">
         <v>0.0513</v>
@@ -59974,10 +59974,10 @@
         <v>0.234</v>
       </c>
       <c r="J1189" s="19" t="n">
-        <v>286679</v>
+        <v>286812</v>
       </c>
       <c r="K1189" s="19" t="n">
-        <v>752295</v>
+        <v>752503</v>
       </c>
       <c r="L1189" s="31" t="n">
         <v>0</v>
@@ -60000,26 +60000,26 @@
         </is>
       </c>
       <c r="D1190" s="9" t="n">
-        <v>22059810.53</v>
+        <v>22062874.73</v>
       </c>
       <c r="E1190" s="9" t="n">
-        <v>35507287.71</v>
+        <v>35515816.44</v>
       </c>
       <c r="F1190" s="10" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.0776</v>
       </c>
       <c r="G1190" s="10" t="n">
-        <v>0.0205</v>
+        <v>0.0204</v>
       </c>
       <c r="H1190" s="10" t="n"/>
       <c r="I1190" s="10" t="n">
         <v>0.1851</v>
       </c>
       <c r="J1190" s="13" t="n">
-        <v>335942</v>
+        <v>336041</v>
       </c>
       <c r="K1190" s="13" t="n">
-        <v>730295</v>
+        <v>730449</v>
       </c>
       <c r="L1190" s="32" t="n">
         <v>0</v>
@@ -60042,26 +60042,26 @@
         </is>
       </c>
       <c r="D1191" s="15" t="n">
-        <v>14890635.15</v>
+        <v>14896687.79</v>
       </c>
       <c r="E1191" s="15" t="n">
-        <v>39725290.12</v>
+        <v>39778096.16</v>
       </c>
       <c r="F1191" s="16" t="n">
-        <v>0.09660000000000001</v>
+        <v>0.096</v>
       </c>
       <c r="G1191" s="16" t="n">
-        <v>0.0323</v>
+        <v>0.0317</v>
       </c>
       <c r="H1191" s="16" t="n"/>
       <c r="I1191" s="16" t="n">
         <v>0.146</v>
       </c>
       <c r="J1191" s="19" t="n">
-        <v>327898</v>
+        <v>328005</v>
       </c>
       <c r="K1191" s="19" t="n">
-        <v>625341</v>
+        <v>625530</v>
       </c>
       <c r="L1191" s="31" t="n">
         <v>0</v>
@@ -60084,26 +60084,26 @@
         </is>
       </c>
       <c r="D1192" s="9" t="n">
-        <v>21016961.99</v>
+        <v>21022564.99</v>
       </c>
       <c r="E1192" s="9" t="n">
-        <v>92180541.83</v>
+        <v>92275516.8</v>
       </c>
       <c r="F1192" s="10" t="n">
-        <v>0.204</v>
+        <v>0.2038</v>
       </c>
       <c r="G1192" s="10" t="n">
-        <v>0.1357</v>
+        <v>0.1355</v>
       </c>
       <c r="H1192" s="10" t="n"/>
       <c r="I1192" s="10" t="n">
         <v>0.1053</v>
       </c>
       <c r="J1192" s="13" t="n">
-        <v>640409</v>
+        <v>640537</v>
       </c>
       <c r="K1192" s="13" t="n">
-        <v>1125090</v>
+        <v>1125340</v>
       </c>
       <c r="L1192" s="32" t="n">
         <v>0</v>
@@ -60126,26 +60126,26 @@
         </is>
       </c>
       <c r="D1193" s="15" t="n">
-        <v>19583344.97</v>
+        <v>19585619.44</v>
       </c>
       <c r="E1193" s="15" t="n">
-        <v>156617488.4</v>
+        <v>156732531.52</v>
       </c>
       <c r="F1193" s="16" t="n">
-        <v>0.3532</v>
+        <v>0.3531</v>
       </c>
       <c r="G1193" s="16" t="n">
-        <v>0.2803</v>
+        <v>0.2802</v>
       </c>
       <c r="H1193" s="16" t="n"/>
       <c r="I1193" s="16" t="n">
         <v>0.0605</v>
       </c>
       <c r="J1193" s="19" t="n">
-        <v>819540</v>
+        <v>819704</v>
       </c>
       <c r="K1193" s="19" t="n">
-        <v>1530499</v>
+        <v>1530713</v>
       </c>
       <c r="L1193" s="31" t="n">
         <v>0</v>
@@ -64997,7 +64997,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-26 07:26 UTC</t>
+          <t>2026-10-26 14:27 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-26 16:14 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8605,7 +8605,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 14:27 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 16:14 UTC.</t>
         </is>
       </c>
     </row>
@@ -37488,26 +37488,26 @@
         </is>
       </c>
       <c r="D654" s="9" t="n">
-        <v>13434386.18</v>
+        <v>13437069.38</v>
       </c>
       <c r="E654" s="9" t="n">
-        <v>79016591.43000001</v>
+        <v>79019930.55</v>
       </c>
       <c r="F654" s="10" t="n">
-        <v>0.3448</v>
+        <v>0.3444</v>
       </c>
       <c r="G654" s="10" t="n">
-        <v>0.2787</v>
+        <v>0.2783</v>
       </c>
       <c r="H654" s="10" t="n"/>
       <c r="I654" s="10" t="n">
-        <v>0.0588</v>
+        <v>0.0589</v>
       </c>
       <c r="J654" s="13" t="n">
-        <v>509115</v>
+        <v>509152</v>
       </c>
       <c r="K654" s="13" t="n">
-        <v>692036</v>
+        <v>692089</v>
       </c>
       <c r="L654" s="32" t="n">
         <v>0.5456</v>
@@ -41058,26 +41058,26 @@
         </is>
       </c>
       <c r="D739" s="15" t="n">
-        <v>3374711.99</v>
+        <v>3374836</v>
       </c>
       <c r="E739" s="15" t="n">
-        <v>52525284.47</v>
+        <v>52526823.4</v>
       </c>
       <c r="F739" s="16" t="n">
-        <v>0.6192</v>
+        <v>0.6195000000000001</v>
       </c>
       <c r="G739" s="16" t="n">
-        <v>0.5404</v>
+        <v>0.5407999999999999</v>
       </c>
       <c r="H739" s="16" t="n"/>
       <c r="I739" s="16" t="n">
         <v>0.0141</v>
       </c>
       <c r="J739" s="19" t="n">
-        <v>278347</v>
+        <v>278353</v>
       </c>
       <c r="K739" s="19" t="n">
-        <v>373086</v>
+        <v>373093</v>
       </c>
       <c r="L739" s="31" t="n">
         <v>0.5616</v>
@@ -41100,29 +41100,29 @@
         </is>
       </c>
       <c r="D740" s="9" t="n">
-        <v>1796216.71</v>
+        <v>1796333.41</v>
       </c>
       <c r="E740" s="9" t="n">
-        <v>947888.11</v>
+        <v>948125.34</v>
       </c>
       <c r="F740" s="10" t="n">
-        <v>0.2083</v>
+        <v>0.2081</v>
       </c>
       <c r="G740" s="10" t="n">
-        <v>0.1654</v>
+        <v>0.1653</v>
       </c>
       <c r="H740" s="10" t="n"/>
       <c r="I740" s="10" t="n">
-        <v>0.3298</v>
+        <v>0.3296</v>
       </c>
       <c r="J740" s="13" t="n">
-        <v>9353</v>
+        <v>9363</v>
       </c>
       <c r="K740" s="13" t="n">
-        <v>23537</v>
+        <v>23547</v>
       </c>
       <c r="L740" s="32" t="n">
-        <v>0.5029</v>
+        <v>0.503</v>
       </c>
     </row>
     <row r="741">
@@ -41142,29 +41142,29 @@
         </is>
       </c>
       <c r="D741" s="15" t="n">
-        <v>1833525.19</v>
+        <v>1834228.19</v>
       </c>
       <c r="E741" s="15" t="n">
-        <v>1739906.79</v>
+        <v>1740313.04</v>
       </c>
       <c r="F741" s="16" t="n">
         <v>0.1327</v>
       </c>
       <c r="G741" s="16" t="n">
-        <v>0.07829999999999999</v>
+        <v>0.07820000000000001</v>
       </c>
       <c r="H741" s="16" t="n"/>
       <c r="I741" s="16" t="n">
         <v>0.2408</v>
       </c>
       <c r="J741" s="19" t="n">
-        <v>19929</v>
+        <v>19935</v>
       </c>
       <c r="K741" s="19" t="n">
-        <v>35752</v>
+        <v>35760</v>
       </c>
       <c r="L741" s="31" t="n">
-        <v>0.5662</v>
+        <v>0.5663</v>
       </c>
     </row>
     <row r="742">
@@ -41184,29 +41184,29 @@
         </is>
       </c>
       <c r="D742" s="9" t="n">
-        <v>1493390.18</v>
+        <v>1494450.98</v>
       </c>
       <c r="E742" s="9" t="n">
-        <v>2555996.44</v>
+        <v>2556943.05</v>
       </c>
       <c r="F742" s="10" t="n">
-        <v>0.2033</v>
+        <v>0.203</v>
       </c>
       <c r="G742" s="10" t="n">
-        <v>0.1397</v>
+        <v>0.1394</v>
       </c>
       <c r="H742" s="10" t="n"/>
       <c r="I742" s="10" t="n">
-        <v>0.1745</v>
+        <v>0.1747</v>
       </c>
       <c r="J742" s="13" t="n">
-        <v>26680</v>
+        <v>26685</v>
       </c>
       <c r="K742" s="13" t="n">
-        <v>38158</v>
+        <v>38169</v>
       </c>
       <c r="L742" s="32" t="n">
-        <v>0.5712</v>
+        <v>0.5713</v>
       </c>
     </row>
     <row r="743">
@@ -41226,26 +41226,26 @@
         </is>
       </c>
       <c r="D743" s="15" t="n">
-        <v>1202428.39</v>
+        <v>1202641.03</v>
       </c>
       <c r="E743" s="15" t="n">
-        <v>3153438.12</v>
+        <v>3153469.13</v>
       </c>
       <c r="F743" s="16" t="n">
-        <v>0.2205</v>
+        <v>0.22</v>
       </c>
       <c r="G743" s="16" t="n">
-        <v>0.1531</v>
+        <v>0.1526</v>
       </c>
       <c r="H743" s="16" t="n"/>
       <c r="I743" s="16" t="n">
-        <v>0.1345</v>
+        <v>0.1346</v>
       </c>
       <c r="J743" s="19" t="n">
-        <v>28961</v>
+        <v>28965</v>
       </c>
       <c r="K743" s="19" t="n">
-        <v>38290</v>
+        <v>38299</v>
       </c>
       <c r="L743" s="31" t="n">
         <v>0.5387999999999999</v>
@@ -41268,29 +41268,29 @@
         </is>
       </c>
       <c r="D744" s="9" t="n">
-        <v>1959498.14</v>
+        <v>1959903.26</v>
       </c>
       <c r="E744" s="9" t="n">
-        <v>6633026.8</v>
+        <v>6633205.89</v>
       </c>
       <c r="F744" s="10" t="n">
-        <v>0.2598</v>
+        <v>0.2593</v>
       </c>
       <c r="G744" s="10" t="n">
-        <v>0.1915</v>
+        <v>0.191</v>
       </c>
       <c r="H744" s="10" t="n"/>
       <c r="I744" s="10" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="J744" s="13" t="n">
-        <v>62991</v>
+        <v>62993</v>
       </c>
       <c r="K744" s="13" t="n">
-        <v>80068</v>
+        <v>80072</v>
       </c>
       <c r="L744" s="32" t="n">
-        <v>0.5334</v>
+        <v>0.5333</v>
       </c>
     </row>
     <row r="745">
@@ -41310,26 +41310,26 @@
         </is>
       </c>
       <c r="D745" s="15" t="n">
-        <v>1774615.58</v>
+        <v>1774676.51</v>
       </c>
       <c r="E745" s="15" t="n">
         <v>11461050.71</v>
       </c>
       <c r="F745" s="16" t="n">
-        <v>0.4774</v>
+        <v>0.475</v>
       </c>
       <c r="G745" s="16" t="n">
-        <v>0.4013</v>
+        <v>0.3989</v>
       </c>
       <c r="H745" s="16" t="n"/>
       <c r="I745" s="16" t="n">
         <v>0.049</v>
       </c>
       <c r="J745" s="19" t="n">
-        <v>82854</v>
+        <v>82858</v>
       </c>
       <c r="K745" s="19" t="n">
-        <v>103145</v>
+        <v>103149</v>
       </c>
       <c r="L745" s="31" t="n">
         <v>0.5337</v>
@@ -56304,26 +56304,26 @@
         </is>
       </c>
       <c r="D1102" s="9" t="n">
-        <v>173079510.38</v>
+        <v>173081888.21</v>
       </c>
       <c r="E1102" s="9" t="n">
-        <v>769940496.97</v>
+        <v>769961681.36</v>
       </c>
       <c r="F1102" s="10" t="n">
-        <v>0.1623</v>
+        <v>0.162</v>
       </c>
       <c r="G1102" s="10" t="n">
-        <v>0.1034</v>
+        <v>0.1031</v>
       </c>
       <c r="H1102" s="10" t="n"/>
       <c r="I1102" s="10" t="n">
         <v>0.09320000000000001</v>
       </c>
       <c r="J1102" s="13" t="n">
-        <v>4243936</v>
+        <v>4244097</v>
       </c>
       <c r="K1102" s="13" t="n">
-        <v>8166329</v>
+        <v>8166527</v>
       </c>
       <c r="L1102" s="32" t="n">
         <v>0</v>
@@ -59874,26 +59874,26 @@
         </is>
       </c>
       <c r="D1187" s="15" t="n">
-        <v>22129287.86</v>
+        <v>22129967.16</v>
       </c>
       <c r="E1187" s="15" t="n">
-        <v>393164737.13</v>
+        <v>393175493.35</v>
       </c>
       <c r="F1187" s="16" t="n">
-        <v>0.4793</v>
+        <v>0.4772</v>
       </c>
       <c r="G1187" s="16" t="n">
-        <v>0.3995</v>
+        <v>0.3974</v>
       </c>
       <c r="H1187" s="16" t="n"/>
       <c r="I1187" s="16" t="n">
         <v>0.0258</v>
       </c>
       <c r="J1187" s="19" t="n">
-        <v>1641690</v>
+        <v>1641763</v>
       </c>
       <c r="K1187" s="19" t="n">
-        <v>2550932</v>
+        <v>2551017</v>
       </c>
       <c r="L1187" s="31" t="n">
         <v>0</v>
@@ -59916,10 +59916,10 @@
         </is>
       </c>
       <c r="D1188" s="9" t="n">
-        <v>44386665.62</v>
+        <v>44387031.99</v>
       </c>
       <c r="E1188" s="9" t="n">
-        <v>23092351.44</v>
+        <v>23092412.07</v>
       </c>
       <c r="F1188" s="10" t="n">
         <v>0.0373</v>
@@ -59932,10 +59932,10 @@
         <v>0.3084</v>
       </c>
       <c r="J1188" s="13" t="n">
-        <v>191147</v>
+        <v>191160</v>
       </c>
       <c r="K1188" s="13" t="n">
-        <v>850862</v>
+        <v>850879</v>
       </c>
       <c r="L1188" s="32" t="n">
         <v>0</v>
@@ -59958,10 +59958,10 @@
         </is>
       </c>
       <c r="D1189" s="15" t="n">
-        <v>28995809.94</v>
+        <v>28996027.17</v>
       </c>
       <c r="E1189" s="15" t="n">
-        <v>29381447.48</v>
+        <v>29381640.04</v>
       </c>
       <c r="F1189" s="16" t="n">
         <v>0.0513</v>
@@ -59974,10 +59974,10 @@
         <v>0.234</v>
       </c>
       <c r="J1189" s="19" t="n">
-        <v>286812</v>
+        <v>286828</v>
       </c>
       <c r="K1189" s="19" t="n">
-        <v>752503</v>
+        <v>752522</v>
       </c>
       <c r="L1189" s="31" t="n">
         <v>0</v>
@@ -60000,10 +60000,10 @@
         </is>
       </c>
       <c r="D1190" s="9" t="n">
-        <v>22062874.73</v>
+        <v>22062944.84</v>
       </c>
       <c r="E1190" s="9" t="n">
-        <v>35515816.44</v>
+        <v>35515886.43</v>
       </c>
       <c r="F1190" s="10" t="n">
         <v>0.0776</v>
@@ -60016,10 +60016,10 @@
         <v>0.1851</v>
       </c>
       <c r="J1190" s="13" t="n">
-        <v>336041</v>
+        <v>336049</v>
       </c>
       <c r="K1190" s="13" t="n">
-        <v>730449</v>
+        <v>730460</v>
       </c>
       <c r="L1190" s="32" t="n">
         <v>0</v>
@@ -60042,10 +60042,10 @@
         </is>
       </c>
       <c r="D1191" s="15" t="n">
-        <v>14896687.79</v>
+        <v>14897057.82</v>
       </c>
       <c r="E1191" s="15" t="n">
-        <v>39778096.16</v>
+        <v>39781061.29</v>
       </c>
       <c r="F1191" s="16" t="n">
         <v>0.096</v>
@@ -60058,10 +60058,10 @@
         <v>0.146</v>
       </c>
       <c r="J1191" s="19" t="n">
-        <v>328005</v>
+        <v>328018</v>
       </c>
       <c r="K1191" s="19" t="n">
-        <v>625530</v>
+        <v>625543</v>
       </c>
       <c r="L1191" s="31" t="n">
         <v>0</v>
@@ -60084,10 +60084,10 @@
         </is>
       </c>
       <c r="D1192" s="9" t="n">
-        <v>21022564.99</v>
+        <v>21023124.61</v>
       </c>
       <c r="E1192" s="9" t="n">
-        <v>92275516.8</v>
+        <v>92278591.44</v>
       </c>
       <c r="F1192" s="10" t="n">
         <v>0.2038</v>
@@ -60100,10 +60100,10 @@
         <v>0.1053</v>
       </c>
       <c r="J1192" s="13" t="n">
-        <v>640537</v>
+        <v>640554</v>
       </c>
       <c r="K1192" s="13" t="n">
-        <v>1125340</v>
+        <v>1125364</v>
       </c>
       <c r="L1192" s="32" t="n">
         <v>0</v>
@@ -60126,26 +60126,26 @@
         </is>
       </c>
       <c r="D1193" s="15" t="n">
-        <v>19585619.44</v>
+        <v>19585734.62</v>
       </c>
       <c r="E1193" s="15" t="n">
-        <v>156732531.52</v>
+        <v>156736596.74</v>
       </c>
       <c r="F1193" s="16" t="n">
-        <v>0.3531</v>
+        <v>0.3529</v>
       </c>
       <c r="G1193" s="16" t="n">
-        <v>0.2802</v>
+        <v>0.28</v>
       </c>
       <c r="H1193" s="16" t="n"/>
       <c r="I1193" s="16" t="n">
         <v>0.0605</v>
       </c>
       <c r="J1193" s="19" t="n">
-        <v>819704</v>
+        <v>819725</v>
       </c>
       <c r="K1193" s="19" t="n">
-        <v>1530713</v>
+        <v>1530742</v>
       </c>
       <c r="L1193" s="31" t="n">
         <v>0</v>
@@ -64997,7 +64997,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-26 14:27 UTC</t>
+          <t>2026-10-26 16:14 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-26 17:25 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8605,7 +8605,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 16:14 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 17:25 UTC.</t>
         </is>
       </c>
     </row>
@@ -37488,26 +37488,26 @@
         </is>
       </c>
       <c r="D654" s="9" t="n">
-        <v>13437069.38</v>
+        <v>13437463.07</v>
       </c>
       <c r="E654" s="9" t="n">
-        <v>79019930.55</v>
+        <v>79020290.59999999</v>
       </c>
       <c r="F654" s="10" t="n">
-        <v>0.3444</v>
+        <v>0.3443</v>
       </c>
       <c r="G654" s="10" t="n">
-        <v>0.2783</v>
+        <v>0.2782</v>
       </c>
       <c r="H654" s="10" t="n"/>
       <c r="I654" s="10" t="n">
         <v>0.0589</v>
       </c>
       <c r="J654" s="13" t="n">
-        <v>509152</v>
+        <v>509172</v>
       </c>
       <c r="K654" s="13" t="n">
-        <v>692089</v>
+        <v>692110</v>
       </c>
       <c r="L654" s="32" t="n">
         <v>0.5456</v>
@@ -41058,7 +41058,7 @@
         </is>
       </c>
       <c r="D739" s="15" t="n">
-        <v>3374836</v>
+        <v>3374888.2</v>
       </c>
       <c r="E739" s="15" t="n">
         <v>52526823.4</v>
@@ -41074,10 +41074,10 @@
         <v>0.0141</v>
       </c>
       <c r="J739" s="19" t="n">
-        <v>278353</v>
+        <v>278361</v>
       </c>
       <c r="K739" s="19" t="n">
-        <v>373093</v>
+        <v>373101</v>
       </c>
       <c r="L739" s="31" t="n">
         <v>0.5616</v>
@@ -41142,7 +41142,7 @@
         </is>
       </c>
       <c r="D741" s="15" t="n">
-        <v>1834228.19</v>
+        <v>1834232.93</v>
       </c>
       <c r="E741" s="15" t="n">
         <v>1740313.04</v>
@@ -41158,10 +41158,10 @@
         <v>0.2408</v>
       </c>
       <c r="J741" s="19" t="n">
-        <v>19935</v>
+        <v>19936</v>
       </c>
       <c r="K741" s="19" t="n">
-        <v>35760</v>
+        <v>35761</v>
       </c>
       <c r="L741" s="31" t="n">
         <v>0.5663</v>
@@ -41184,26 +41184,26 @@
         </is>
       </c>
       <c r="D742" s="9" t="n">
-        <v>1494450.98</v>
+        <v>1494589.49</v>
       </c>
       <c r="E742" s="9" t="n">
         <v>2556943.05</v>
       </c>
       <c r="F742" s="10" t="n">
-        <v>0.203</v>
+        <v>0.2029</v>
       </c>
       <c r="G742" s="10" t="n">
-        <v>0.1394</v>
+        <v>0.1393</v>
       </c>
       <c r="H742" s="10" t="n"/>
       <c r="I742" s="10" t="n">
         <v>0.1747</v>
       </c>
       <c r="J742" s="13" t="n">
-        <v>26685</v>
+        <v>26687</v>
       </c>
       <c r="K742" s="13" t="n">
-        <v>38169</v>
+        <v>38171</v>
       </c>
       <c r="L742" s="32" t="n">
         <v>0.5713</v>
@@ -41226,26 +41226,26 @@
         </is>
       </c>
       <c r="D743" s="15" t="n">
-        <v>1202641.03</v>
+        <v>1202646.28</v>
       </c>
       <c r="E743" s="15" t="n">
         <v>3153469.13</v>
       </c>
       <c r="F743" s="16" t="n">
-        <v>0.22</v>
+        <v>0.2199</v>
       </c>
       <c r="G743" s="16" t="n">
-        <v>0.1526</v>
+        <v>0.1525</v>
       </c>
       <c r="H743" s="16" t="n"/>
       <c r="I743" s="16" t="n">
         <v>0.1346</v>
       </c>
       <c r="J743" s="19" t="n">
-        <v>28965</v>
+        <v>28966</v>
       </c>
       <c r="K743" s="19" t="n">
-        <v>38299</v>
+        <v>38300</v>
       </c>
       <c r="L743" s="31" t="n">
         <v>0.5387999999999999</v>
@@ -41268,26 +41268,26 @@
         </is>
       </c>
       <c r="D744" s="9" t="n">
-        <v>1959903.26</v>
+        <v>1960029.74</v>
       </c>
       <c r="E744" s="9" t="n">
-        <v>6633205.89</v>
+        <v>6633565.94</v>
       </c>
       <c r="F744" s="10" t="n">
-        <v>0.2593</v>
+        <v>0.2591</v>
       </c>
       <c r="G744" s="10" t="n">
-        <v>0.191</v>
+        <v>0.1907</v>
       </c>
       <c r="H744" s="10" t="n"/>
       <c r="I744" s="10" t="n">
         <v>0.08799999999999999</v>
       </c>
       <c r="J744" s="13" t="n">
-        <v>62993</v>
+        <v>62996</v>
       </c>
       <c r="K744" s="13" t="n">
-        <v>80072</v>
+        <v>80076</v>
       </c>
       <c r="L744" s="32" t="n">
         <v>0.5333</v>
@@ -41310,7 +41310,7 @@
         </is>
       </c>
       <c r="D745" s="15" t="n">
-        <v>1774676.51</v>
+        <v>1774743.02</v>
       </c>
       <c r="E745" s="15" t="n">
         <v>11461050.71</v>
@@ -41323,13 +41323,13 @@
       </c>
       <c r="H745" s="16" t="n"/>
       <c r="I745" s="16" t="n">
-        <v>0.049</v>
+        <v>0.0491</v>
       </c>
       <c r="J745" s="19" t="n">
-        <v>82858</v>
+        <v>82863</v>
       </c>
       <c r="K745" s="19" t="n">
-        <v>103149</v>
+        <v>103154</v>
       </c>
       <c r="L745" s="31" t="n">
         <v>0.5337</v>
@@ -56304,10 +56304,10 @@
         </is>
       </c>
       <c r="D1102" s="9" t="n">
-        <v>173081888.21</v>
+        <v>173084796.16</v>
       </c>
       <c r="E1102" s="9" t="n">
-        <v>769961681.36</v>
+        <v>769962403.87</v>
       </c>
       <c r="F1102" s="10" t="n">
         <v>0.162</v>
@@ -56320,10 +56320,10 @@
         <v>0.09320000000000001</v>
       </c>
       <c r="J1102" s="13" t="n">
-        <v>4244097</v>
+        <v>4244214</v>
       </c>
       <c r="K1102" s="13" t="n">
-        <v>8166527</v>
+        <v>8166666</v>
       </c>
       <c r="L1102" s="32" t="n">
         <v>0</v>
@@ -59874,7 +59874,7 @@
         </is>
       </c>
       <c r="D1187" s="15" t="n">
-        <v>22129967.16</v>
+        <v>22130211.6</v>
       </c>
       <c r="E1187" s="15" t="n">
         <v>393175493.35</v>
@@ -59890,10 +59890,10 @@
         <v>0.0258</v>
       </c>
       <c r="J1187" s="19" t="n">
-        <v>1641763</v>
+        <v>1641808</v>
       </c>
       <c r="K1187" s="19" t="n">
-        <v>2551017</v>
+        <v>2551071</v>
       </c>
       <c r="L1187" s="31" t="n">
         <v>0</v>
@@ -59916,13 +59916,13 @@
         </is>
       </c>
       <c r="D1188" s="9" t="n">
-        <v>44387031.99</v>
+        <v>44387966.05</v>
       </c>
       <c r="E1188" s="9" t="n">
         <v>23092412.07</v>
       </c>
       <c r="F1188" s="10" t="n">
-        <v>0.0373</v>
+        <v>0.0372</v>
       </c>
       <c r="G1188" s="10" t="n">
         <v>-0.0046</v>
@@ -59932,10 +59932,10 @@
         <v>0.3084</v>
       </c>
       <c r="J1188" s="13" t="n">
-        <v>191160</v>
+        <v>191171</v>
       </c>
       <c r="K1188" s="13" t="n">
-        <v>850879</v>
+        <v>850894</v>
       </c>
       <c r="L1188" s="32" t="n">
         <v>0</v>
@@ -59958,10 +59958,10 @@
         </is>
       </c>
       <c r="D1189" s="15" t="n">
-        <v>28996027.17</v>
+        <v>28996394.13</v>
       </c>
       <c r="E1189" s="15" t="n">
-        <v>29381640.04</v>
+        <v>29381660.17</v>
       </c>
       <c r="F1189" s="16" t="n">
         <v>0.0513</v>
@@ -59974,10 +59974,10 @@
         <v>0.234</v>
       </c>
       <c r="J1189" s="19" t="n">
-        <v>286828</v>
+        <v>286842</v>
       </c>
       <c r="K1189" s="19" t="n">
-        <v>752522</v>
+        <v>752538</v>
       </c>
       <c r="L1189" s="31" t="n">
         <v>0</v>
@@ -60000,7 +60000,7 @@
         </is>
       </c>
       <c r="D1190" s="9" t="n">
-        <v>22062944.84</v>
+        <v>22063962.99</v>
       </c>
       <c r="E1190" s="9" t="n">
         <v>35515886.43</v>
@@ -60016,10 +60016,10 @@
         <v>0.1851</v>
       </c>
       <c r="J1190" s="13" t="n">
-        <v>336049</v>
+        <v>336058</v>
       </c>
       <c r="K1190" s="13" t="n">
-        <v>730460</v>
+        <v>730471</v>
       </c>
       <c r="L1190" s="32" t="n">
         <v>0</v>
@@ -60042,7 +60042,7 @@
         </is>
       </c>
       <c r="D1191" s="15" t="n">
-        <v>14897057.82</v>
+        <v>14897072.17</v>
       </c>
       <c r="E1191" s="15" t="n">
         <v>39781061.29</v>
@@ -60058,10 +60058,10 @@
         <v>0.146</v>
       </c>
       <c r="J1191" s="19" t="n">
-        <v>328018</v>
+        <v>328023</v>
       </c>
       <c r="K1191" s="19" t="n">
-        <v>625543</v>
+        <v>625548</v>
       </c>
       <c r="L1191" s="31" t="n">
         <v>0</v>
@@ -60084,10 +60084,10 @@
         </is>
       </c>
       <c r="D1192" s="9" t="n">
-        <v>21023124.61</v>
+        <v>21023307.32</v>
       </c>
       <c r="E1192" s="9" t="n">
-        <v>92278591.44</v>
+        <v>92278592.67</v>
       </c>
       <c r="F1192" s="10" t="n">
         <v>0.2038</v>
@@ -60100,10 +60100,10 @@
         <v>0.1053</v>
       </c>
       <c r="J1192" s="13" t="n">
-        <v>640554</v>
+        <v>640576</v>
       </c>
       <c r="K1192" s="13" t="n">
-        <v>1125364</v>
+        <v>1125389</v>
       </c>
       <c r="L1192" s="32" t="n">
         <v>0</v>
@@ -60126,10 +60126,10 @@
         </is>
       </c>
       <c r="D1193" s="15" t="n">
-        <v>19585734.62</v>
+        <v>19585881.89</v>
       </c>
       <c r="E1193" s="15" t="n">
-        <v>156736596.74</v>
+        <v>156737297.89</v>
       </c>
       <c r="F1193" s="16" t="n">
         <v>0.3529</v>
@@ -60142,10 +60142,10 @@
         <v>0.0605</v>
       </c>
       <c r="J1193" s="19" t="n">
-        <v>819725</v>
+        <v>819736</v>
       </c>
       <c r="K1193" s="19" t="n">
-        <v>1530742</v>
+        <v>1530755</v>
       </c>
       <c r="L1193" s="31" t="n">
         <v>0</v>
@@ -64997,7 +64997,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-26 16:14 UTC</t>
+          <t>2026-10-26 17:25 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-26 18:54 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8605,7 +8605,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 17:25 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-26 18:54 UTC.</t>
         </is>
       </c>
     </row>
@@ -37488,26 +37488,26 @@
         </is>
       </c>
       <c r="D654" s="9" t="n">
-        <v>13437463.07</v>
+        <v>13439772.67</v>
       </c>
       <c r="E654" s="9" t="n">
-        <v>79020290.59999999</v>
+        <v>79026866.89</v>
       </c>
       <c r="F654" s="10" t="n">
-        <v>0.3443</v>
+        <v>0.3441</v>
       </c>
       <c r="G654" s="10" t="n">
-        <v>0.2782</v>
+        <v>0.278</v>
       </c>
       <c r="H654" s="10" t="n"/>
       <c r="I654" s="10" t="n">
         <v>0.0589</v>
       </c>
       <c r="J654" s="13" t="n">
-        <v>509172</v>
+        <v>509217</v>
       </c>
       <c r="K654" s="13" t="n">
-        <v>692110</v>
+        <v>692169</v>
       </c>
       <c r="L654" s="32" t="n">
         <v>0.5456</v>
@@ -41058,26 +41058,26 @@
         </is>
       </c>
       <c r="D739" s="15" t="n">
-        <v>3374888.2</v>
+        <v>3374947.59</v>
       </c>
       <c r="E739" s="15" t="n">
-        <v>52526823.4</v>
+        <v>52526851.11</v>
       </c>
       <c r="F739" s="16" t="n">
         <v>0.6195000000000001</v>
       </c>
       <c r="G739" s="16" t="n">
-        <v>0.5407999999999999</v>
+        <v>0.5407</v>
       </c>
       <c r="H739" s="16" t="n"/>
       <c r="I739" s="16" t="n">
         <v>0.0141</v>
       </c>
       <c r="J739" s="19" t="n">
-        <v>278361</v>
+        <v>278367</v>
       </c>
       <c r="K739" s="19" t="n">
-        <v>373101</v>
+        <v>373110</v>
       </c>
       <c r="L739" s="31" t="n">
         <v>0.5616</v>
@@ -41100,26 +41100,26 @@
         </is>
       </c>
       <c r="D740" s="9" t="n">
-        <v>1796333.41</v>
+        <v>1796650.51</v>
       </c>
       <c r="E740" s="9" t="n">
         <v>948125.34</v>
       </c>
       <c r="F740" s="10" t="n">
-        <v>0.2081</v>
+        <v>0.208</v>
       </c>
       <c r="G740" s="10" t="n">
-        <v>0.1653</v>
+        <v>0.1651</v>
       </c>
       <c r="H740" s="10" t="n"/>
       <c r="I740" s="10" t="n">
         <v>0.3296</v>
       </c>
       <c r="J740" s="13" t="n">
-        <v>9363</v>
+        <v>9365</v>
       </c>
       <c r="K740" s="13" t="n">
-        <v>23547</v>
+        <v>23549</v>
       </c>
       <c r="L740" s="32" t="n">
         <v>0.503</v>
@@ -41142,29 +41142,29 @@
         </is>
       </c>
       <c r="D741" s="15" t="n">
-        <v>1834232.93</v>
+        <v>1834557.11</v>
       </c>
       <c r="E741" s="15" t="n">
         <v>1740313.04</v>
       </c>
       <c r="F741" s="16" t="n">
-        <v>0.1327</v>
+        <v>0.1325</v>
       </c>
       <c r="G741" s="16" t="n">
-        <v>0.07820000000000001</v>
+        <v>0.078</v>
       </c>
       <c r="H741" s="16" t="n"/>
       <c r="I741" s="16" t="n">
-        <v>0.2408</v>
+        <v>0.2411</v>
       </c>
       <c r="J741" s="19" t="n">
-        <v>19936</v>
+        <v>19945</v>
       </c>
       <c r="K741" s="19" t="n">
-        <v>35761</v>
+        <v>35770</v>
       </c>
       <c r="L741" s="31" t="n">
-        <v>0.5663</v>
+        <v>0.5664</v>
       </c>
     </row>
     <row r="742">
@@ -41184,26 +41184,26 @@
         </is>
       </c>
       <c r="D742" s="9" t="n">
-        <v>1494589.49</v>
+        <v>1494729.46</v>
       </c>
       <c r="E742" s="9" t="n">
-        <v>2556943.05</v>
+        <v>2557227.06</v>
       </c>
       <c r="F742" s="10" t="n">
         <v>0.2029</v>
       </c>
       <c r="G742" s="10" t="n">
-        <v>0.1393</v>
+        <v>0.1392</v>
       </c>
       <c r="H742" s="10" t="n"/>
       <c r="I742" s="10" t="n">
-        <v>0.1747</v>
+        <v>0.1748</v>
       </c>
       <c r="J742" s="13" t="n">
-        <v>26687</v>
+        <v>26691</v>
       </c>
       <c r="K742" s="13" t="n">
-        <v>38171</v>
+        <v>38177</v>
       </c>
       <c r="L742" s="32" t="n">
         <v>0.5713</v>
@@ -41226,13 +41226,13 @@
         </is>
       </c>
       <c r="D743" s="15" t="n">
-        <v>1202646.28</v>
+        <v>1202693.25</v>
       </c>
       <c r="E743" s="15" t="n">
         <v>3153469.13</v>
       </c>
       <c r="F743" s="16" t="n">
-        <v>0.2199</v>
+        <v>0.22</v>
       </c>
       <c r="G743" s="16" t="n">
         <v>0.1525</v>
@@ -41242,10 +41242,10 @@
         <v>0.1346</v>
       </c>
       <c r="J743" s="19" t="n">
-        <v>28966</v>
+        <v>28969</v>
       </c>
       <c r="K743" s="19" t="n">
-        <v>38300</v>
+        <v>38303</v>
       </c>
       <c r="L743" s="31" t="n">
         <v>0.5387999999999999</v>
@@ -41268,10 +41268,10 @@
         </is>
       </c>
       <c r="D744" s="9" t="n">
-        <v>1960029.74</v>
+        <v>1960068.19</v>
       </c>
       <c r="E744" s="9" t="n">
-        <v>6633565.94</v>
+        <v>6633680.08</v>
       </c>
       <c r="F744" s="10" t="n">
         <v>0.2591</v>
@@ -41281,13 +41281,13 @@
       </c>
       <c r="H744" s="10" t="n"/>
       <c r="I744" s="10" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.0881</v>
       </c>
       <c r="J744" s="13" t="n">
-        <v>62996</v>
+        <v>63002</v>
       </c>
       <c r="K744" s="13" t="n">
-        <v>80076</v>
+        <v>80084</v>
       </c>
       <c r="L744" s="32" t="n">
         <v>0.5333</v>
@@ -41310,29 +41310,29 @@
         </is>
       </c>
       <c r="D745" s="15" t="n">
-        <v>1774743.02</v>
+        <v>1776126.56</v>
       </c>
       <c r="E745" s="15" t="n">
-        <v>11461050.71</v>
+        <v>11467201.13</v>
       </c>
       <c r="F745" s="16" t="n">
-        <v>0.475</v>
+        <v>0.4738</v>
       </c>
       <c r="G745" s="16" t="n">
-        <v>0.3989</v>
+        <v>0.3976</v>
       </c>
       <c r="H745" s="16" t="n"/>
       <c r="I745" s="16" t="n">
-        <v>0.0491</v>
+        <v>0.0492</v>
       </c>
       <c r="J745" s="19" t="n">
-        <v>82863</v>
+        <v>82878</v>
       </c>
       <c r="K745" s="19" t="n">
-        <v>103154</v>
+        <v>103176</v>
       </c>
       <c r="L745" s="31" t="n">
-        <v>0.5337</v>
+        <v>0.5334</v>
       </c>
     </row>
     <row r="746">
@@ -56304,10 +56304,10 @@
         </is>
       </c>
       <c r="D1102" s="9" t="n">
-        <v>173084796.16</v>
+        <v>173109547.5</v>
       </c>
       <c r="E1102" s="9" t="n">
-        <v>769962403.87</v>
+        <v>769992456.3200001</v>
       </c>
       <c r="F1102" s="10" t="n">
         <v>0.162</v>
@@ -56320,10 +56320,10 @@
         <v>0.09320000000000001</v>
       </c>
       <c r="J1102" s="13" t="n">
-        <v>4244214</v>
+        <v>4244423</v>
       </c>
       <c r="K1102" s="13" t="n">
-        <v>8166666</v>
+        <v>8167036</v>
       </c>
       <c r="L1102" s="32" t="n">
         <v>0</v>
@@ -59874,26 +59874,26 @@
         </is>
       </c>
       <c r="D1187" s="15" t="n">
-        <v>22130211.6</v>
+        <v>22131318.62</v>
       </c>
       <c r="E1187" s="15" t="n">
-        <v>393175493.35</v>
+        <v>393176791.05</v>
       </c>
       <c r="F1187" s="16" t="n">
-        <v>0.4772</v>
+        <v>0.4771</v>
       </c>
       <c r="G1187" s="16" t="n">
-        <v>0.3974</v>
+        <v>0.3973</v>
       </c>
       <c r="H1187" s="16" t="n"/>
       <c r="I1187" s="16" t="n">
         <v>0.0258</v>
       </c>
       <c r="J1187" s="19" t="n">
-        <v>1641808</v>
+        <v>1641852</v>
       </c>
       <c r="K1187" s="19" t="n">
-        <v>2551071</v>
+        <v>2551138</v>
       </c>
       <c r="L1187" s="31" t="n">
         <v>0</v>
@@ -59916,26 +59916,26 @@
         </is>
       </c>
       <c r="D1188" s="9" t="n">
-        <v>44387966.05</v>
+        <v>44398363.98</v>
       </c>
       <c r="E1188" s="9" t="n">
-        <v>23092412.07</v>
+        <v>23112171.32</v>
       </c>
       <c r="F1188" s="10" t="n">
-        <v>0.0372</v>
+        <v>0.0374</v>
       </c>
       <c r="G1188" s="10" t="n">
-        <v>-0.0046</v>
+        <v>-0.0045</v>
       </c>
       <c r="H1188" s="10" t="n"/>
       <c r="I1188" s="10" t="n">
         <v>0.3084</v>
       </c>
       <c r="J1188" s="13" t="n">
-        <v>191171</v>
+        <v>191200</v>
       </c>
       <c r="K1188" s="13" t="n">
-        <v>850894</v>
+        <v>850973</v>
       </c>
       <c r="L1188" s="32" t="n">
         <v>0</v>
@@ -59958,26 +59958,26 @@
         </is>
       </c>
       <c r="D1189" s="15" t="n">
-        <v>28996394.13</v>
+        <v>29007415.17</v>
       </c>
       <c r="E1189" s="15" t="n">
-        <v>29381660.17</v>
+        <v>29381721.85</v>
       </c>
       <c r="F1189" s="16" t="n">
-        <v>0.0513</v>
+        <v>0.0514</v>
       </c>
       <c r="G1189" s="16" t="n">
-        <v>-0.0001</v>
+        <v>-0</v>
       </c>
       <c r="H1189" s="16" t="n"/>
       <c r="I1189" s="16" t="n">
-        <v>0.234</v>
+        <v>0.2341</v>
       </c>
       <c r="J1189" s="19" t="n">
-        <v>286842</v>
+        <v>286869</v>
       </c>
       <c r="K1189" s="19" t="n">
-        <v>752538</v>
+        <v>752616</v>
       </c>
       <c r="L1189" s="31" t="n">
         <v>0</v>
@@ -60000,10 +60000,10 @@
         </is>
       </c>
       <c r="D1190" s="9" t="n">
-        <v>22063962.99</v>
+        <v>22064821.27</v>
       </c>
       <c r="E1190" s="9" t="n">
-        <v>35515886.43</v>
+        <v>35515945.07</v>
       </c>
       <c r="F1190" s="10" t="n">
         <v>0.0776</v>
@@ -60013,13 +60013,13 @@
       </c>
       <c r="H1190" s="10" t="n"/>
       <c r="I1190" s="10" t="n">
-        <v>0.1851</v>
+        <v>0.1852</v>
       </c>
       <c r="J1190" s="13" t="n">
-        <v>336058</v>
+        <v>336072</v>
       </c>
       <c r="K1190" s="13" t="n">
-        <v>730471</v>
+        <v>730494</v>
       </c>
       <c r="L1190" s="32" t="n">
         <v>0</v>
@@ -60042,13 +60042,13 @@
         </is>
       </c>
       <c r="D1191" s="15" t="n">
-        <v>14897072.17</v>
+        <v>14897327.33</v>
       </c>
       <c r="E1191" s="15" t="n">
-        <v>39781061.29</v>
+        <v>39781467.06</v>
       </c>
       <c r="F1191" s="16" t="n">
-        <v>0.096</v>
+        <v>0.0959</v>
       </c>
       <c r="G1191" s="16" t="n">
         <v>0.0317</v>
@@ -60058,10 +60058,10 @@
         <v>0.146</v>
       </c>
       <c r="J1191" s="19" t="n">
-        <v>328023</v>
+        <v>328042</v>
       </c>
       <c r="K1191" s="19" t="n">
-        <v>625548</v>
+        <v>625571</v>
       </c>
       <c r="L1191" s="31" t="n">
         <v>0</v>
@@ -60084,26 +60084,26 @@
         </is>
       </c>
       <c r="D1192" s="9" t="n">
-        <v>21023307.32</v>
+        <v>21024010.55</v>
       </c>
       <c r="E1192" s="9" t="n">
-        <v>92278592.67</v>
+        <v>92282810.98999999</v>
       </c>
       <c r="F1192" s="10" t="n">
         <v>0.2038</v>
       </c>
       <c r="G1192" s="10" t="n">
-        <v>0.1355</v>
+        <v>0.1354</v>
       </c>
       <c r="H1192" s="10" t="n"/>
       <c r="I1192" s="10" t="n">
         <v>0.1053</v>
       </c>
       <c r="J1192" s="13" t="n">
-        <v>640576</v>
+        <v>640623</v>
       </c>
       <c r="K1192" s="13" t="n">
-        <v>1125389</v>
+        <v>1125450</v>
       </c>
       <c r="L1192" s="32" t="n">
         <v>0</v>
@@ -60126,10 +60126,10 @@
         </is>
       </c>
       <c r="D1193" s="15" t="n">
-        <v>19585881.89</v>
+        <v>19586290.57</v>
       </c>
       <c r="E1193" s="15" t="n">
-        <v>156737297.89</v>
+        <v>156741548.99</v>
       </c>
       <c r="F1193" s="16" t="n">
         <v>0.3529</v>
@@ -60142,10 +60142,10 @@
         <v>0.0605</v>
       </c>
       <c r="J1193" s="19" t="n">
-        <v>819736</v>
+        <v>819765</v>
       </c>
       <c r="K1193" s="19" t="n">
-        <v>1530755</v>
+        <v>1530794</v>
       </c>
       <c r="L1193" s="31" t="n">
         <v>0</v>
@@ -64997,7 +64997,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-26 17:25 UTC</t>
+          <t>2026-10-26 18:54 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-27 15:29 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8643,7 +8643,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-27 13:50 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-27 15:28 UTC.</t>
         </is>
       </c>
     </row>
@@ -39222,10 +39222,10 @@
         </is>
       </c>
       <c r="D694" s="9" t="n">
-        <v>13555700.46</v>
+        <v>13555738.91</v>
       </c>
       <c r="E694" s="9" t="n">
-        <v>78768879.25</v>
+        <v>78769140.43000001</v>
       </c>
       <c r="F694" s="10" t="n">
         <v>0.2923</v>
@@ -39238,10 +39238,10 @@
         <v>0.0689</v>
       </c>
       <c r="J694" s="13" t="n">
-        <v>485744</v>
+        <v>485748</v>
       </c>
       <c r="K694" s="13" t="n">
-        <v>669187</v>
+        <v>669193</v>
       </c>
       <c r="L694" s="32" t="n">
         <v>0.527</v>
@@ -39264,29 +39264,29 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>2285239.67</v>
+        <v>2286438.13</v>
       </c>
       <c r="E695" s="15" t="n">
-        <v>14422439.95</v>
+        <v>14425593.65</v>
       </c>
       <c r="F695" s="16" t="n">
-        <v>0.32</v>
+        <v>0.3191</v>
       </c>
       <c r="G695" s="16" t="n">
-        <v>0.2533</v>
+        <v>0.2524</v>
       </c>
       <c r="H695" s="16" t="n"/>
       <c r="I695" s="16" t="n">
-        <v>0.0372</v>
+        <v>0.0374</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>109491</v>
+        <v>109526</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>146016</v>
+        <v>146056</v>
       </c>
       <c r="L695" s="31" t="n">
-        <v>0.7868000000000001</v>
+        <v>0.7869</v>
       </c>
     </row>
     <row r="696">
@@ -42918,10 +42918,10 @@
         </is>
       </c>
       <c r="D782" s="9" t="n">
-        <v>1953137.84</v>
+        <v>1953157.41</v>
       </c>
       <c r="E782" s="9" t="n">
-        <v>2022262.63</v>
+        <v>2022283.53</v>
       </c>
       <c r="F782" s="10" t="n">
         <v>0.1389</v>
@@ -42934,10 +42934,10 @@
         <v>0.2451</v>
       </c>
       <c r="J782" s="13" t="n">
-        <v>20994</v>
+        <v>20995</v>
       </c>
       <c r="K782" s="13" t="n">
-        <v>38544</v>
+        <v>38546</v>
       </c>
       <c r="L782" s="32" t="n">
         <v>0.5301</v>
@@ -42960,10 +42960,10 @@
         </is>
       </c>
       <c r="D783" s="15" t="n">
-        <v>1550883.42</v>
+        <v>1550894.83</v>
       </c>
       <c r="E783" s="15" t="n">
-        <v>2905893.77</v>
+        <v>2905915.81</v>
       </c>
       <c r="F783" s="16" t="n">
         <v>0.1737</v>
@@ -42976,10 +42976,10 @@
         <v>0.1834</v>
       </c>
       <c r="J783" s="19" t="n">
-        <v>28048</v>
+        <v>28049</v>
       </c>
       <c r="K783" s="19" t="n">
-        <v>41158</v>
+        <v>41160</v>
       </c>
       <c r="L783" s="31" t="n">
         <v>0.5454</v>
@@ -43044,10 +43044,10 @@
         </is>
       </c>
       <c r="D785" s="15" t="n">
-        <v>2012584.59</v>
+        <v>2012592.08</v>
       </c>
       <c r="E785" s="15" t="n">
-        <v>7497754.24</v>
+        <v>7497972.48</v>
       </c>
       <c r="F785" s="16" t="n">
         <v>0.1848</v>
@@ -43060,10 +43060,10 @@
         <v>0.0978</v>
       </c>
       <c r="J785" s="19" t="n">
-        <v>64296</v>
+        <v>64298</v>
       </c>
       <c r="K785" s="19" t="n">
-        <v>82608</v>
+        <v>82610</v>
       </c>
       <c r="L785" s="31" t="n">
         <v>0.509</v>
@@ -43128,10 +43128,10 @@
         </is>
       </c>
       <c r="D787" s="15" t="n">
-        <v>691489.23</v>
+        <v>691808.91</v>
       </c>
       <c r="E787" s="15" t="n">
-        <v>10560536.46</v>
+        <v>10560558.16</v>
       </c>
       <c r="F787" s="16" t="n">
         <v>0.6709000000000001</v>
@@ -43141,16 +43141,16 @@
       </c>
       <c r="H787" s="16" t="n"/>
       <c r="I787" s="16" t="n">
-        <v>0.0109</v>
+        <v>0.011</v>
       </c>
       <c r="J787" s="19" t="n">
-        <v>66275</v>
+        <v>66290</v>
       </c>
       <c r="K787" s="19" t="n">
-        <v>85671</v>
+        <v>85687</v>
       </c>
       <c r="L787" s="31" t="n">
-        <v>0.6264</v>
+        <v>0.6266</v>
       </c>
     </row>
     <row r="788">
@@ -43170,10 +43170,10 @@
         </is>
       </c>
       <c r="D788" s="9" t="n">
-        <v>223993.6</v>
+        <v>224066.16</v>
       </c>
       <c r="E788" s="9" t="n">
-        <v>651906.59</v>
+        <v>651962.35</v>
       </c>
       <c r="F788" s="10" t="n">
         <v>-0.4034</v>
@@ -43183,16 +43183,16 @@
       </c>
       <c r="H788" s="10" t="n"/>
       <c r="I788" s="10" t="n">
-        <v>0.3173</v>
+        <v>0.3184</v>
       </c>
       <c r="J788" s="13" t="n">
-        <v>1185</v>
+        <v>1187</v>
       </c>
       <c r="K788" s="13" t="n">
-        <v>2942</v>
+        <v>2945</v>
       </c>
       <c r="L788" s="32" t="n">
-        <v>0.947</v>
+        <v>0.9471000000000001</v>
       </c>
     </row>
     <row r="789">
@@ -43212,26 +43212,26 @@
         </is>
       </c>
       <c r="D789" s="15" t="n">
-        <v>288867.1</v>
+        <v>289364.23</v>
       </c>
       <c r="E789" s="15" t="n">
-        <v>101297.24</v>
+        <v>101302.99</v>
       </c>
       <c r="F789" s="16" t="n">
-        <v>0.0451</v>
+        <v>0.0415</v>
       </c>
       <c r="G789" s="16" t="n">
-        <v>-0.0012</v>
+        <v>-0.0047</v>
       </c>
       <c r="H789" s="16" t="n"/>
       <c r="I789" s="16" t="n">
-        <v>0.2099</v>
+        <v>0.2109</v>
       </c>
       <c r="J789" s="19" t="n">
-        <v>2859</v>
+        <v>2864</v>
       </c>
       <c r="K789" s="19" t="n">
-        <v>4795</v>
+        <v>4801</v>
       </c>
       <c r="L789" s="31" t="n">
         <v>0.9386</v>
@@ -43254,29 +43254,29 @@
         </is>
       </c>
       <c r="D790" s="9" t="n">
-        <v>229623.25</v>
+        <v>229787.99</v>
       </c>
       <c r="E790" s="9" t="n">
         <v>263346.96</v>
       </c>
       <c r="F790" s="10" t="n">
-        <v>0.1919</v>
+        <v>0.1892</v>
       </c>
       <c r="G790" s="10" t="n">
-        <v>0.1307</v>
+        <v>0.1279</v>
       </c>
       <c r="H790" s="10" t="n"/>
       <c r="I790" s="10" t="n">
-        <v>0.1379</v>
+        <v>0.1387</v>
       </c>
       <c r="J790" s="13" t="n">
-        <v>4207</v>
+        <v>4211</v>
       </c>
       <c r="K790" s="13" t="n">
-        <v>5816</v>
+        <v>5821</v>
       </c>
       <c r="L790" s="32" t="n">
-        <v>0.8486</v>
+        <v>0.8487</v>
       </c>
     </row>
     <row r="791">
@@ -43296,26 +43296,26 @@
         </is>
       </c>
       <c r="D791" s="15" t="n">
-        <v>231787.39</v>
+        <v>231834.61</v>
       </c>
       <c r="E791" s="15" t="n">
         <v>232242.15</v>
       </c>
       <c r="F791" s="16" t="n">
-        <v>0.255</v>
+        <v>0.2537</v>
       </c>
       <c r="G791" s="16" t="n">
-        <v>0.1908</v>
+        <v>0.1895</v>
       </c>
       <c r="H791" s="16" t="n"/>
       <c r="I791" s="16" t="n">
-        <v>0.0955</v>
+        <v>0.0961</v>
       </c>
       <c r="J791" s="19" t="n">
-        <v>5317</v>
+        <v>5320</v>
       </c>
       <c r="K791" s="19" t="n">
-        <v>11064</v>
+        <v>11067</v>
       </c>
       <c r="L791" s="31" t="n">
         <v>0.906</v>
@@ -43338,29 +43338,29 @@
         </is>
       </c>
       <c r="D792" s="9" t="n">
-        <v>315372.7</v>
+        <v>315458.88</v>
       </c>
       <c r="E792" s="9" t="n">
-        <v>833100.75</v>
+        <v>833171.25</v>
       </c>
       <c r="F792" s="10" t="n">
-        <v>0.3187</v>
+        <v>0.3182</v>
       </c>
       <c r="G792" s="10" t="n">
-        <v>0.2498</v>
+        <v>0.2493</v>
       </c>
       <c r="H792" s="10" t="n"/>
       <c r="I792" s="10" t="n">
-        <v>0.0572</v>
+        <v>0.0574</v>
       </c>
       <c r="J792" s="13" t="n">
-        <v>12411</v>
+        <v>12415</v>
       </c>
       <c r="K792" s="13" t="n">
-        <v>15196</v>
+        <v>15200</v>
       </c>
       <c r="L792" s="32" t="n">
-        <v>0.7921</v>
+        <v>0.7922</v>
       </c>
     </row>
     <row r="793">
@@ -43380,26 +43380,26 @@
         </is>
       </c>
       <c r="D793" s="15" t="n">
-        <v>304106.4</v>
+        <v>304117.35</v>
       </c>
       <c r="E793" s="15" t="n">
-        <v>1780009.8</v>
+        <v>1783009.79</v>
       </c>
       <c r="F793" s="16" t="n">
-        <v>0.464</v>
+        <v>0.4639</v>
       </c>
       <c r="G793" s="16" t="n">
-        <v>0.3913</v>
+        <v>0.3912</v>
       </c>
       <c r="H793" s="16" t="n"/>
       <c r="I793" s="16" t="n">
         <v>0.0335</v>
       </c>
       <c r="J793" s="19" t="n">
-        <v>17237</v>
+        <v>17239</v>
       </c>
       <c r="K793" s="19" t="n">
-        <v>20532</v>
+        <v>20535</v>
       </c>
       <c r="L793" s="31" t="n">
         <v>0.7465000000000001</v>
@@ -59382,10 +59382,10 @@
         </is>
       </c>
       <c r="D1174" s="9" t="n">
-        <v>175250049.72</v>
+        <v>175252539.5</v>
       </c>
       <c r="E1174" s="9" t="n">
-        <v>770218137.49</v>
+        <v>770228291.42</v>
       </c>
       <c r="F1174" s="10" t="n">
         <v>0.1453</v>
@@ -59398,10 +59398,10 @@
         <v>0.098</v>
       </c>
       <c r="J1174" s="13" t="n">
-        <v>4199992</v>
+        <v>4200121</v>
       </c>
       <c r="K1174" s="13" t="n">
-        <v>8132495</v>
+        <v>8132679</v>
       </c>
       <c r="L1174" s="32" t="n">
         <v>0</v>
@@ -59424,26 +59424,26 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>13367394.93</v>
+        <v>13879135.78</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>61226043.41</v>
+        <v>61253266.5</v>
       </c>
       <c r="F1175" s="16" t="n">
-        <v>0.1058</v>
+        <v>0.1</v>
       </c>
       <c r="G1175" s="16" t="n">
-        <v>0.0499</v>
+        <v>0.046</v>
       </c>
       <c r="H1175" s="16" t="n"/>
       <c r="I1175" s="16" t="n">
-        <v>0.092</v>
+        <v>0.0931</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>367133</v>
+        <v>367837</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>700622</v>
+        <v>701851</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -62994,10 +62994,10 @@
         </is>
       </c>
       <c r="D1260" s="9" t="n">
-        <v>21410918.95</v>
+        <v>21411475.03</v>
       </c>
       <c r="E1260" s="9" t="n">
-        <v>387406547.26</v>
+        <v>387414252.67</v>
       </c>
       <c r="F1260" s="10" t="n">
         <v>0.4393</v>
@@ -63010,10 +63010,10 @@
         <v>0.0283</v>
       </c>
       <c r="J1260" s="13" t="n">
-        <v>1575433</v>
+        <v>1575453</v>
       </c>
       <c r="K1260" s="13" t="n">
-        <v>2452774</v>
+        <v>2452803</v>
       </c>
       <c r="L1260" s="32" t="n">
         <v>0</v>
@@ -63036,10 +63036,10 @@
         </is>
       </c>
       <c r="D1261" s="15" t="n">
-        <v>46102980.16</v>
+        <v>46103396.01</v>
       </c>
       <c r="E1261" s="15" t="n">
-        <v>24144678.74</v>
+        <v>24144787.24</v>
       </c>
       <c r="F1261" s="16" t="n">
         <v>0.0355</v>
@@ -63049,13 +63049,13 @@
       </c>
       <c r="H1261" s="16" t="n"/>
       <c r="I1261" s="16" t="n">
-        <v>0.3097</v>
+        <v>0.3098</v>
       </c>
       <c r="J1261" s="19" t="n">
-        <v>196917</v>
+        <v>196940</v>
       </c>
       <c r="K1261" s="19" t="n">
-        <v>884554</v>
+        <v>884593</v>
       </c>
       <c r="L1261" s="31" t="n">
         <v>0</v>
@@ -63078,10 +63078,10 @@
         </is>
       </c>
       <c r="D1262" s="9" t="n">
-        <v>29711156.69</v>
+        <v>29711834.7</v>
       </c>
       <c r="E1262" s="9" t="n">
-        <v>30950581.51</v>
+        <v>30951396.85</v>
       </c>
       <c r="F1262" s="10" t="n">
         <v>0.0467</v>
@@ -63091,13 +63091,13 @@
       </c>
       <c r="H1262" s="10" t="n"/>
       <c r="I1262" s="10" t="n">
-        <v>0.2367</v>
+        <v>0.2368</v>
       </c>
       <c r="J1262" s="13" t="n">
-        <v>293990</v>
+        <v>294013</v>
       </c>
       <c r="K1262" s="13" t="n">
-        <v>778710</v>
+        <v>778748</v>
       </c>
       <c r="L1262" s="32" t="n">
         <v>0</v>
@@ -63120,10 +63120,10 @@
         </is>
       </c>
       <c r="D1263" s="15" t="n">
-        <v>22401587.77</v>
+        <v>22401808.11</v>
       </c>
       <c r="E1263" s="15" t="n">
-        <v>37031028.3</v>
+        <v>37031435.68</v>
       </c>
       <c r="F1263" s="16" t="n">
         <v>0.0699</v>
@@ -63133,13 +63133,13 @@
       </c>
       <c r="H1263" s="16" t="n"/>
       <c r="I1263" s="16" t="n">
-        <v>0.1883</v>
+        <v>0.1884</v>
       </c>
       <c r="J1263" s="19" t="n">
-        <v>343005</v>
+        <v>343022</v>
       </c>
       <c r="K1263" s="19" t="n">
-        <v>747834</v>
+        <v>747861</v>
       </c>
       <c r="L1263" s="31" t="n">
         <v>0</v>
@@ -63162,10 +63162,10 @@
         </is>
       </c>
       <c r="D1264" s="9" t="n">
-        <v>15048399.56</v>
+        <v>15048492.89</v>
       </c>
       <c r="E1264" s="9" t="n">
-        <v>40861022.52</v>
+        <v>40861294.77</v>
       </c>
       <c r="F1264" s="10" t="n">
         <v>0.0842</v>
@@ -63178,10 +63178,10 @@
         <v>0.1497</v>
       </c>
       <c r="J1264" s="13" t="n">
-        <v>332633</v>
+        <v>332642</v>
       </c>
       <c r="K1264" s="13" t="n">
-        <v>634072</v>
+        <v>634081</v>
       </c>
       <c r="L1264" s="32" t="n">
         <v>0</v>
@@ -63204,10 +63204,10 @@
         </is>
       </c>
       <c r="D1265" s="15" t="n">
-        <v>21124078.68</v>
+        <v>21124358.98</v>
       </c>
       <c r="E1265" s="15" t="n">
-        <v>93730012.76000001</v>
+        <v>93730129.16</v>
       </c>
       <c r="F1265" s="16" t="n">
         <v>0.1842</v>
@@ -63220,10 +63220,10 @@
         <v>0.109</v>
       </c>
       <c r="J1265" s="19" t="n">
-        <v>644423</v>
+        <v>644440</v>
       </c>
       <c r="K1265" s="19" t="n">
-        <v>1132705</v>
+        <v>1132723</v>
       </c>
       <c r="L1265" s="31" t="n">
         <v>0</v>
@@ -63246,10 +63246,10 @@
         </is>
       </c>
       <c r="D1266" s="9" t="n">
-        <v>19450927.91</v>
+        <v>19451173.78</v>
       </c>
       <c r="E1266" s="9" t="n">
-        <v>156094266.4</v>
+        <v>156094995.05</v>
       </c>
       <c r="F1266" s="10" t="n">
         <v>0.3245</v>
@@ -63262,10 +63262,10 @@
         <v>0.0636</v>
       </c>
       <c r="J1266" s="13" t="n">
-        <v>813591</v>
+        <v>813611</v>
       </c>
       <c r="K1266" s="13" t="n">
-        <v>1501846</v>
+        <v>1501870</v>
       </c>
       <c r="L1266" s="32" t="n">
         <v>0</v>
@@ -63288,26 +63288,26 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>2004726.66</v>
+        <v>2009353.42</v>
       </c>
       <c r="E1267" s="15" t="n">
-        <v>35023578.01</v>
+        <v>35039198.49</v>
       </c>
       <c r="F1267" s="16" t="n">
-        <v>0.4669</v>
+        <v>0.4623</v>
       </c>
       <c r="G1267" s="16" t="n">
-        <v>0.3928</v>
+        <v>0.3882</v>
       </c>
       <c r="H1267" s="16" t="n"/>
       <c r="I1267" s="16" t="n">
-        <v>0.0229</v>
+        <v>0.0236</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>162528</v>
+        <v>162742</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>275790</v>
+        <v>276159</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63330,26 +63330,26 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>3932885.81</v>
+        <v>4395812.85</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>1780011.48</v>
+        <v>1781349.18</v>
       </c>
       <c r="F1268" s="10" t="n">
-        <v>0.0236</v>
+        <v>0.0203</v>
       </c>
       <c r="G1268" s="10" t="n">
-        <v>-0.0166</v>
+        <v>-0.0157</v>
       </c>
       <c r="H1268" s="10" t="n"/>
       <c r="I1268" s="10" t="n">
-        <v>0.3016</v>
+        <v>0.302</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>16109</v>
+        <v>16138</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>65506</v>
+        <v>65572</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63372,26 +63372,26 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>2102268.6</v>
+        <v>2109985.22</v>
       </c>
       <c r="E1269" s="15" t="n">
-        <v>1810175.69</v>
+        <v>1810514.38</v>
       </c>
       <c r="F1269" s="16" t="n">
-        <v>0.0457</v>
+        <v>0.0449</v>
       </c>
       <c r="G1269" s="16" t="n">
-        <v>-0.0043</v>
+        <v>-0.005</v>
       </c>
       <c r="H1269" s="16" t="n"/>
       <c r="I1269" s="16" t="n">
-        <v>0.2448</v>
+        <v>0.2456</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>23050</v>
+        <v>23095</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>56839</v>
+        <v>56913</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63414,26 +63414,26 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>1512939.34</v>
+        <v>1521008.28</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>2385785.02</v>
+        <v>2386738.58</v>
       </c>
       <c r="F1270" s="10" t="n">
-        <v>0.0331</v>
+        <v>0.0313</v>
       </c>
       <c r="G1270" s="10" t="n">
-        <v>-0.0241</v>
+        <v>-0.0257</v>
       </c>
       <c r="H1270" s="10" t="n"/>
       <c r="I1270" s="10" t="n">
-        <v>0.2</v>
+        <v>0.201</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>25935</v>
+        <v>25985</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>50618</v>
+        <v>50700</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63456,26 +63456,26 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>953181.8199999999</v>
+        <v>965184.39</v>
       </c>
       <c r="E1271" s="15" t="n">
-        <v>2281817.41</v>
+        <v>2282189.91</v>
       </c>
       <c r="F1271" s="16" t="n">
-        <v>-0.0451</v>
+        <v>-0.0471</v>
       </c>
       <c r="G1271" s="16" t="n">
-        <v>-0.1065</v>
+        <v>-0.1079</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
-        <v>0.1632</v>
+        <v>0.1647</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>25337</v>
+        <v>25397</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>42224</v>
+        <v>42320</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63498,26 +63498,26 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>1372741.93</v>
+        <v>1379272.81</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>5439418.62</v>
+        <v>5444446.01</v>
       </c>
       <c r="F1272" s="10" t="n">
-        <v>0.0151</v>
+        <v>0.012</v>
       </c>
       <c r="G1272" s="10" t="n">
-        <v>-0.0516</v>
+        <v>-0.0546</v>
       </c>
       <c r="H1272" s="10" t="n"/>
       <c r="I1272" s="10" t="n">
-        <v>0.1192</v>
+        <v>0.1208</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>49183</v>
+        <v>49303</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>80378</v>
+        <v>80589</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63540,26 +63540,26 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>1488650.77</v>
+        <v>1498518.81</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>12505257.19</v>
+        <v>12508829.94</v>
       </c>
       <c r="F1273" s="16" t="n">
-        <v>0.1762</v>
+        <v>0.1714</v>
       </c>
       <c r="G1273" s="16" t="n">
-        <v>0.1093</v>
+        <v>0.1047</v>
       </c>
       <c r="H1273" s="16" t="n"/>
       <c r="I1273" s="16" t="n">
-        <v>0.0674</v>
+        <v>0.0693</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>64991</v>
+        <v>65177</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>129267</v>
+        <v>129598</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -68747,7 +68747,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-27 13:50 UTC</t>
+          <t>2026-10-27 15:28 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-27 16:42 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8643,7 +8643,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-27 15:28 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-27 16:42 UTC.</t>
         </is>
       </c>
     </row>
@@ -39264,7 +39264,7 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>2286438.13</v>
+        <v>2286443.2</v>
       </c>
       <c r="E695" s="15" t="n">
         <v>14425593.65</v>
@@ -39273,17 +39273,17 @@
         <v>0.3191</v>
       </c>
       <c r="G695" s="16" t="n">
-        <v>0.2524</v>
+        <v>0.2523</v>
       </c>
       <c r="H695" s="16" t="n"/>
       <c r="I695" s="16" t="n">
         <v>0.0374</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>109526</v>
+        <v>109527</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>146056</v>
+        <v>146057</v>
       </c>
       <c r="L695" s="31" t="n">
         <v>0.7869</v>
@@ -43254,29 +43254,29 @@
         </is>
       </c>
       <c r="D790" s="9" t="n">
-        <v>229787.99</v>
+        <v>229793.07</v>
       </c>
       <c r="E790" s="9" t="n">
         <v>263346.96</v>
       </c>
       <c r="F790" s="10" t="n">
-        <v>0.1892</v>
+        <v>0.1891</v>
       </c>
       <c r="G790" s="10" t="n">
         <v>0.1279</v>
       </c>
       <c r="H790" s="10" t="n"/>
       <c r="I790" s="10" t="n">
-        <v>0.1387</v>
+        <v>0.1389</v>
       </c>
       <c r="J790" s="13" t="n">
-        <v>4211</v>
+        <v>4212</v>
       </c>
       <c r="K790" s="13" t="n">
-        <v>5821</v>
+        <v>5822</v>
       </c>
       <c r="L790" s="32" t="n">
-        <v>0.8487</v>
+        <v>0.8488</v>
       </c>
     </row>
     <row r="791">
@@ -59424,26 +59424,26 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>13879135.78</v>
+        <v>13879812.87</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>61253266.5</v>
+        <v>61259108.46</v>
       </c>
       <c r="F1175" s="16" t="n">
-        <v>0.1</v>
+        <v>0.1001</v>
       </c>
       <c r="G1175" s="16" t="n">
-        <v>0.046</v>
+        <v>0.0461</v>
       </c>
       <c r="H1175" s="16" t="n"/>
       <c r="I1175" s="16" t="n">
-        <v>0.0931</v>
+        <v>0.09320000000000001</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>367837</v>
+        <v>367860</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>701851</v>
+        <v>701881</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -63288,7 +63288,7 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>2009353.42</v>
+        <v>2009383.67</v>
       </c>
       <c r="E1267" s="15" t="n">
         <v>35039198.49</v>
@@ -63304,10 +63304,10 @@
         <v>0.0236</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>162742</v>
+        <v>162743</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>276159</v>
+        <v>276160</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63330,10 +63330,10 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>4395812.85</v>
+        <v>4395851.78</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>1781349.18</v>
+        <v>1781437.19</v>
       </c>
       <c r="F1268" s="10" t="n">
         <v>0.0203</v>
@@ -63346,10 +63346,10 @@
         <v>0.302</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>16138</v>
+        <v>16141</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>65572</v>
+        <v>65576</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63372,7 +63372,7 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>2109985.22</v>
+        <v>2109995.51</v>
       </c>
       <c r="E1269" s="15" t="n">
         <v>1810514.38</v>
@@ -63385,13 +63385,13 @@
       </c>
       <c r="H1269" s="16" t="n"/>
       <c r="I1269" s="16" t="n">
-        <v>0.2456</v>
+        <v>0.2457</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>23095</v>
+        <v>23097</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>56913</v>
+        <v>56915</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63414,10 +63414,10 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>1521008.28</v>
+        <v>1521131.26</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>2386738.58</v>
+        <v>2389107.02</v>
       </c>
       <c r="F1270" s="10" t="n">
         <v>0.0313</v>
@@ -63430,10 +63430,10 @@
         <v>0.201</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>25985</v>
+        <v>25990</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>50700</v>
+        <v>50707</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63456,26 +63456,26 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>965184.39</v>
+        <v>965471.36</v>
       </c>
       <c r="E1271" s="15" t="n">
-        <v>2282189.91</v>
+        <v>2282222.09</v>
       </c>
       <c r="F1271" s="16" t="n">
-        <v>-0.0471</v>
+        <v>-0.0468</v>
       </c>
       <c r="G1271" s="16" t="n">
-        <v>-0.1079</v>
+        <v>-0.1076</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
         <v>0.1647</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>25397</v>
+        <v>25401</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>42320</v>
+        <v>42325</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63498,10 +63498,10 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>1379272.81</v>
+        <v>1379294.2</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>5444446.01</v>
+        <v>5445208.45</v>
       </c>
       <c r="F1272" s="10" t="n">
         <v>0.012</v>
@@ -63514,10 +63514,10 @@
         <v>0.1208</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>49303</v>
+        <v>49306</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>80589</v>
+        <v>80594</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63540,26 +63540,26 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>1498518.81</v>
+        <v>1498685.09</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>12508829.94</v>
+        <v>12511420.84</v>
       </c>
       <c r="F1273" s="16" t="n">
-        <v>0.1714</v>
+        <v>0.1715</v>
       </c>
       <c r="G1273" s="16" t="n">
-        <v>0.1047</v>
+        <v>0.1048</v>
       </c>
       <c r="H1273" s="16" t="n"/>
       <c r="I1273" s="16" t="n">
         <v>0.0693</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>65177</v>
+        <v>65182</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>129598</v>
+        <v>129604</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -68747,7 +68747,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-27 15:28 UTC</t>
+          <t>2026-10-27 16:42 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-28 14:47 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -6010,22 +6010,22 @@
         <v>46327</v>
       </c>
       <c r="B71" s="15" t="n">
-        <v>107910297.51</v>
+        <v>195776960.82</v>
       </c>
       <c r="C71" s="15" t="n">
-        <v>5026243.49</v>
+        <v>11300764.39</v>
       </c>
       <c r="D71" s="16" t="n">
-        <v>0.04658</v>
+        <v>0.05772</v>
       </c>
       <c r="E71" s="15" t="n">
-        <v>23618300.46</v>
+        <v>23752659.5</v>
       </c>
       <c r="F71" s="15" t="n">
-        <v>5060430.1</v>
+        <v>5029166.96</v>
       </c>
       <c r="G71" s="16" t="n">
-        <v>0.21426</v>
+        <v>0.21173</v>
       </c>
       <c r="H71" s="17" t="inlineStr">
         <is>
@@ -6033,19 +6033,19 @@
         </is>
       </c>
       <c r="I71" s="15" t="n">
-        <v>131528597.97</v>
+        <v>219529620.32</v>
       </c>
       <c r="J71" s="15" t="n">
-        <v>10086673.59</v>
+        <v>16329931.35</v>
       </c>
       <c r="K71" s="18" t="n">
-        <v>0.07668999999999999</v>
+        <v>0.07439</v>
       </c>
       <c r="L71" s="19" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="M71" s="19" t="n">
-        <v>511</v>
+        <v>1022</v>
       </c>
       <c r="N71" s="15" t="n">
         <v>46236350.82</v>
@@ -6054,25 +6054,29 @@
         <v>0.03001</v>
       </c>
       <c r="P71" s="15" t="n">
-        <v>49533579.64</v>
+        <v>94427986.83</v>
       </c>
       <c r="Q71" s="16" t="n">
-        <v>0.05501</v>
+        <v>0.04542</v>
       </c>
       <c r="R71" s="15" t="n">
-        <v>8209318.63</v>
+        <v>32305010.2</v>
       </c>
       <c r="S71" s="16" t="n">
-        <v>0.06825000000000001</v>
+        <v>0.13156</v>
       </c>
       <c r="T71" s="15" t="n">
-        <v>3931048.41</v>
+        <v>10881225.19</v>
       </c>
       <c r="U71" s="16" t="n">
-        <v>0.08989</v>
-      </c>
-      <c r="V71" s="15" t="n"/>
-      <c r="W71" s="16" t="n"/>
+        <v>0.06432</v>
+      </c>
+      <c r="V71" s="15" t="n">
+        <v>11926387.78</v>
+      </c>
+      <c r="W71" s="16" t="n">
+        <v>0.0565</v>
+      </c>
       <c r="X71" s="15" t="n"/>
       <c r="Y71" s="16" t="n"/>
       <c r="Z71" s="15" t="n"/>
@@ -7465,22 +7469,22 @@
         <v>46296</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>3312535284.76</v>
+        <v>3400401948.07</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>91757446.53</v>
+        <v>98031967.43000001</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.0277</v>
+        <v>0.02883</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>935044847.6900001</v>
+        <v>935177546.49</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>176362488.32</v>
+        <v>176329463.26</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.18861</v>
+        <v>0.18855</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
@@ -7488,19 +7492,19 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>4247580132.45</v>
+        <v>4335579494.57</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>268119934.85</v>
+        <v>274361430.7</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.06312</v>
+        <v>0.06328</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>858</v>
+        <v>876</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>190</v>
+        <v>234</v>
       </c>
       <c r="N20" s="9" t="n">
         <v>1383015756.65</v>
@@ -7509,28 +7513,28 @@
         <v>0.02467</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>435519830.32</v>
+        <v>480414237.5</v>
       </c>
       <c r="Q20" s="10" t="n">
-        <v>0.03502</v>
+        <v>0.035</v>
       </c>
       <c r="R20" s="9" t="n">
-        <v>339757629.9</v>
+        <v>363853321.47</v>
       </c>
       <c r="S20" s="10" t="n">
-        <v>0.0334</v>
+        <v>0.04133</v>
       </c>
       <c r="T20" s="9" t="n">
-        <v>124576472.25</v>
+        <v>131526649.03</v>
       </c>
       <c r="U20" s="10" t="n">
-        <v>0.02989</v>
+        <v>0.03094</v>
       </c>
       <c r="V20" s="9" t="n">
-        <v>1029665595.64</v>
+        <v>1041591983.43</v>
       </c>
       <c r="W20" s="10" t="n">
-        <v>0.02653</v>
+        <v>0.02688</v>
       </c>
       <c r="X20" s="9" t="n"/>
       <c r="Y20" s="10" t="n"/>
@@ -8643,7 +8647,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-27 16:42 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-28 14:47 UTC.</t>
         </is>
       </c>
     </row>
@@ -10220,26 +10224,26 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>575012.67</v>
+        <v>577669.83</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>436351.22</v>
+        <v>440259.2</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>0.5974</v>
+        <v>0.5921999999999999</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>0.5409</v>
+        <v>0.5357</v>
       </c>
       <c r="H15" s="16" t="n"/>
       <c r="I15" s="16" t="n">
-        <v>0.0554</v>
+        <v>0.0571</v>
       </c>
       <c r="J15" s="19" t="n">
-        <v>13877</v>
+        <v>13959</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>19975</v>
+        <v>20074</v>
       </c>
       <c r="L15" s="31" t="n">
         <v>0</v>
@@ -13202,26 +13206,26 @@
         </is>
       </c>
       <c r="D86" s="9" t="n">
-        <v>40581.87</v>
+        <v>40604.68</v>
       </c>
       <c r="E86" s="9" t="n">
         <v>144830.03</v>
       </c>
       <c r="F86" s="10" t="n">
-        <v>0.892</v>
+        <v>0.8921</v>
       </c>
       <c r="G86" s="10" t="n">
-        <v>0.824</v>
+        <v>0.8241000000000001</v>
       </c>
       <c r="H86" s="10" t="n"/>
       <c r="I86" s="10" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="J86" s="13" t="n">
-        <v>3018</v>
+        <v>3025</v>
       </c>
       <c r="K86" s="13" t="n">
-        <v>4527</v>
+        <v>4534</v>
       </c>
       <c r="L86" s="32" t="n">
         <v>0</v>
@@ -13244,26 +13248,26 @@
         </is>
       </c>
       <c r="D87" s="15" t="n">
-        <v>178714.08</v>
+        <v>179401.39</v>
       </c>
       <c r="E87" s="15" t="n">
-        <v>52176.39</v>
+        <v>52270.17</v>
       </c>
       <c r="F87" s="16" t="n">
-        <v>0.5258</v>
+        <v>0.5195</v>
       </c>
       <c r="G87" s="16" t="n">
-        <v>0.4772</v>
+        <v>0.4709</v>
       </c>
       <c r="H87" s="16" t="n"/>
       <c r="I87" s="16" t="n">
-        <v>0.2835</v>
+        <v>0.2925</v>
       </c>
       <c r="J87" s="19" t="n">
-        <v>896</v>
+        <v>923</v>
       </c>
       <c r="K87" s="19" t="n">
-        <v>2391</v>
+        <v>2421</v>
       </c>
       <c r="L87" s="31" t="n">
         <v>0</v>
@@ -13286,26 +13290,26 @@
         </is>
       </c>
       <c r="D88" s="9" t="n">
-        <v>105425.46</v>
+        <v>106461</v>
       </c>
       <c r="E88" s="9" t="n">
-        <v>27838.28</v>
+        <v>30229.34</v>
       </c>
       <c r="F88" s="10" t="n">
-        <v>0.5474</v>
+        <v>0.5422</v>
       </c>
       <c r="G88" s="10" t="n">
-        <v>0.4936</v>
+        <v>0.4881</v>
       </c>
       <c r="H88" s="10" t="n"/>
       <c r="I88" s="10" t="n">
-        <v>0.1305</v>
+        <v>0.1337</v>
       </c>
       <c r="J88" s="13" t="n">
-        <v>1586</v>
+        <v>1601</v>
       </c>
       <c r="K88" s="13" t="n">
-        <v>2393</v>
+        <v>2411</v>
       </c>
       <c r="L88" s="32" t="n">
         <v>0</v>
@@ -13328,26 +13332,26 @@
         </is>
       </c>
       <c r="D89" s="15" t="n">
-        <v>79646.81</v>
+        <v>80167.35000000001</v>
       </c>
       <c r="E89" s="15" t="n">
-        <v>50994.96</v>
+        <v>51030.37</v>
       </c>
       <c r="F89" s="16" t="n">
-        <v>0.5376</v>
+        <v>0.5256999999999999</v>
       </c>
       <c r="G89" s="16" t="n">
-        <v>0.4779</v>
+        <v>0.4661</v>
       </c>
       <c r="H89" s="16" t="n"/>
       <c r="I89" s="16" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.0699</v>
       </c>
       <c r="J89" s="19" t="n">
-        <v>1625</v>
+        <v>1632</v>
       </c>
       <c r="K89" s="19" t="n">
-        <v>2123</v>
+        <v>2133</v>
       </c>
       <c r="L89" s="31" t="n">
         <v>0</v>
@@ -13370,26 +13374,26 @@
         </is>
       </c>
       <c r="D90" s="9" t="n">
-        <v>47687.4</v>
+        <v>47941.32</v>
       </c>
       <c r="E90" s="9" t="n">
-        <v>26930.46</v>
+        <v>27253.07</v>
       </c>
       <c r="F90" s="10" t="n">
-        <v>0.7556</v>
+        <v>0.7547</v>
       </c>
       <c r="G90" s="10" t="n">
-        <v>0.6956</v>
+        <v>0.6946</v>
       </c>
       <c r="H90" s="10" t="n"/>
       <c r="I90" s="10" t="n">
-        <v>0.0501</v>
+        <v>0.0505</v>
       </c>
       <c r="J90" s="13" t="n">
-        <v>1438</v>
+        <v>1446</v>
       </c>
       <c r="K90" s="13" t="n">
-        <v>1768</v>
+        <v>1779</v>
       </c>
       <c r="L90" s="32" t="n">
         <v>0</v>
@@ -13412,26 +13416,26 @@
         </is>
       </c>
       <c r="D91" s="15" t="n">
-        <v>76848.77</v>
+        <v>76937.06</v>
       </c>
       <c r="E91" s="15" t="n">
-        <v>61332.31</v>
+        <v>61916.86</v>
       </c>
       <c r="F91" s="16" t="n">
-        <v>0.4695</v>
+        <v>0.4688</v>
       </c>
       <c r="G91" s="16" t="n">
-        <v>0.4085</v>
+        <v>0.4079</v>
       </c>
       <c r="H91" s="16" t="n"/>
       <c r="I91" s="16" t="n">
-        <v>0.0257</v>
+        <v>0.0255</v>
       </c>
       <c r="J91" s="19" t="n">
-        <v>2572</v>
+        <v>2584</v>
       </c>
       <c r="K91" s="19" t="n">
-        <v>3228</v>
+        <v>3244</v>
       </c>
       <c r="L91" s="31" t="n">
         <v>0</v>
@@ -13454,26 +13458,26 @@
         </is>
       </c>
       <c r="D92" s="9" t="n">
-        <v>46108.27</v>
+        <v>46157.04</v>
       </c>
       <c r="E92" s="9" t="n">
-        <v>72248.78999999999</v>
+        <v>72729.35000000001</v>
       </c>
       <c r="F92" s="10" t="n">
-        <v>0.8826000000000001</v>
+        <v>0.879</v>
       </c>
       <c r="G92" s="10" t="n">
-        <v>0.8165</v>
+        <v>0.8128</v>
       </c>
       <c r="H92" s="10" t="n"/>
       <c r="I92" s="10" t="n">
-        <v>0.0106</v>
+        <v>0.0109</v>
       </c>
       <c r="J92" s="13" t="n">
-        <v>2742</v>
+        <v>2748</v>
       </c>
       <c r="K92" s="13" t="n">
-        <v>3545</v>
+        <v>3552</v>
       </c>
       <c r="L92" s="32" t="n">
         <v>0</v>
@@ -14882,26 +14886,26 @@
         </is>
       </c>
       <c r="D126" s="9" t="n">
-        <v>366769.33</v>
+        <v>382866.83</v>
       </c>
       <c r="E126" s="9" t="n">
-        <v>1899242.78</v>
+        <v>1919082.81</v>
       </c>
       <c r="F126" s="10" t="n">
-        <v>0.9696</v>
+        <v>0.8921</v>
       </c>
       <c r="G126" s="10" t="n">
-        <v>0.9036</v>
+        <v>0.8258</v>
       </c>
       <c r="H126" s="10" t="n"/>
       <c r="I126" s="10" t="n">
-        <v>0</v>
+        <v>0.0064</v>
       </c>
       <c r="J126" s="13" t="n">
-        <v>17608</v>
+        <v>18246</v>
       </c>
       <c r="K126" s="13" t="n">
-        <v>39373</v>
+        <v>40265</v>
       </c>
       <c r="L126" s="32" t="n">
         <v>0</v>
@@ -17360,26 +17364,26 @@
         </is>
       </c>
       <c r="D185" s="15" t="n">
-        <v>133872.16</v>
+        <v>134949.67</v>
       </c>
       <c r="E185" s="15" t="n">
-        <v>635173.98</v>
+        <v>637964.03</v>
       </c>
       <c r="F185" s="16" t="n">
-        <v>1.0205</v>
+        <v>1.0159</v>
       </c>
       <c r="G185" s="16" t="n">
-        <v>0.9491000000000001</v>
+        <v>0.9445</v>
       </c>
       <c r="H185" s="16" t="n"/>
       <c r="I185" s="16" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="J185" s="19" t="n">
-        <v>9458</v>
+        <v>9614</v>
       </c>
       <c r="K185" s="19" t="n">
-        <v>21726</v>
+        <v>21895</v>
       </c>
       <c r="L185" s="31" t="n">
         <v>0</v>
@@ -17402,26 +17406,26 @@
         </is>
       </c>
       <c r="D186" s="9" t="n">
-        <v>17563.49</v>
+        <v>26299.84</v>
       </c>
       <c r="E186" s="9" t="n">
-        <v>5504.89</v>
+        <v>7905.07</v>
       </c>
       <c r="F186" s="10" t="n">
-        <v>0.9671999999999999</v>
+        <v>0.2109</v>
       </c>
       <c r="G186" s="10" t="n">
-        <v>0.9252</v>
+        <v>0.1643</v>
       </c>
       <c r="H186" s="10" t="n"/>
       <c r="I186" s="10" t="n">
-        <v>0</v>
+        <v>0.1037</v>
       </c>
       <c r="J186" s="13" t="n">
-        <v>359</v>
+        <v>492</v>
       </c>
       <c r="K186" s="13" t="n">
-        <v>507</v>
+        <v>784</v>
       </c>
       <c r="L186" s="32" t="n">
         <v>0</v>
@@ -17444,26 +17448,26 @@
         </is>
       </c>
       <c r="D187" s="15" t="n">
-        <v>29700.27</v>
+        <v>31999.82</v>
       </c>
       <c r="E187" s="15" t="n">
-        <v>12587.03</v>
+        <v>18065.21</v>
       </c>
       <c r="F187" s="16" t="n">
-        <v>1.013</v>
+        <v>0.9594</v>
       </c>
       <c r="G187" s="16" t="n">
-        <v>0.964</v>
+        <v>0.9096</v>
       </c>
       <c r="H187" s="16" t="n"/>
       <c r="I187" s="16" t="n">
-        <v>0</v>
+        <v>0.0185</v>
       </c>
       <c r="J187" s="19" t="n">
-        <v>735</v>
+        <v>813</v>
       </c>
       <c r="K187" s="19" t="n">
-        <v>897</v>
+        <v>1027</v>
       </c>
       <c r="L187" s="31" t="n">
         <v>0</v>
@@ -17486,26 +17490,26 @@
         </is>
       </c>
       <c r="D188" s="9" t="n">
-        <v>33096.48</v>
+        <v>35185.84</v>
       </c>
       <c r="E188" s="9" t="n">
-        <v>34121.01</v>
+        <v>41544.1</v>
       </c>
       <c r="F188" s="10" t="n">
-        <v>0.8899</v>
+        <v>0.7702</v>
       </c>
       <c r="G188" s="10" t="n">
-        <v>0.8310999999999999</v>
+        <v>0.7068</v>
       </c>
       <c r="H188" s="10" t="n"/>
       <c r="I188" s="10" t="n">
-        <v>0</v>
+        <v>0.0139</v>
       </c>
       <c r="J188" s="13" t="n">
-        <v>1069</v>
+        <v>1153</v>
       </c>
       <c r="K188" s="13" t="n">
-        <v>1271</v>
+        <v>1379</v>
       </c>
       <c r="L188" s="32" t="n">
         <v>0</v>
@@ -17528,26 +17532,26 @@
         </is>
       </c>
       <c r="D189" s="15" t="n">
-        <v>30004.48</v>
+        <v>30484.5</v>
       </c>
       <c r="E189" s="15" t="n">
-        <v>45190.61</v>
+        <v>46385.28</v>
       </c>
       <c r="F189" s="16" t="n">
-        <v>0.8586</v>
+        <v>0.8103</v>
       </c>
       <c r="G189" s="16" t="n">
-        <v>0.791</v>
+        <v>0.7413999999999999</v>
       </c>
       <c r="H189" s="16" t="n"/>
       <c r="I189" s="16" t="n">
-        <v>0</v>
+        <v>0.0102</v>
       </c>
       <c r="J189" s="19" t="n">
-        <v>1137</v>
+        <v>1175</v>
       </c>
       <c r="K189" s="19" t="n">
-        <v>1681</v>
+        <v>1727</v>
       </c>
       <c r="L189" s="31" t="n">
         <v>0</v>
@@ -17570,26 +17574,26 @@
         </is>
       </c>
       <c r="D190" s="9" t="n">
-        <v>50592.24</v>
+        <v>51401.9</v>
       </c>
       <c r="E190" s="9" t="n">
-        <v>192024.07</v>
+        <v>192499.26</v>
       </c>
       <c r="F190" s="10" t="n">
-        <v>0.8993</v>
+        <v>0.8852</v>
       </c>
       <c r="G190" s="10" t="n">
-        <v>0.8293</v>
+        <v>0.8152</v>
       </c>
       <c r="H190" s="10" t="n"/>
       <c r="I190" s="10" t="n">
-        <v>0</v>
+        <v>0.0056</v>
       </c>
       <c r="J190" s="13" t="n">
-        <v>2590</v>
+        <v>2684</v>
       </c>
       <c r="K190" s="13" t="n">
-        <v>3468</v>
+        <v>3572</v>
       </c>
       <c r="L190" s="32" t="n">
         <v>0</v>
@@ -17612,26 +17616,26 @@
         </is>
       </c>
       <c r="D191" s="15" t="n">
-        <v>71940.2</v>
+        <v>72545.25999999999</v>
       </c>
       <c r="E191" s="15" t="n">
-        <v>974641.22</v>
+        <v>974719.86</v>
       </c>
       <c r="F191" s="16" t="n">
-        <v>0.9901</v>
+        <v>0.9775</v>
       </c>
       <c r="G191" s="16" t="n">
-        <v>0.9213</v>
+        <v>0.9087</v>
       </c>
       <c r="H191" s="16" t="n"/>
       <c r="I191" s="16" t="n">
-        <v>0</v>
+        <v>0.0017</v>
       </c>
       <c r="J191" s="19" t="n">
-        <v>2260</v>
+        <v>2315</v>
       </c>
       <c r="K191" s="19" t="n">
-        <v>9823</v>
+        <v>9881</v>
       </c>
       <c r="L191" s="31" t="n">
         <v>0</v>
@@ -18158,26 +18162,26 @@
         </is>
       </c>
       <c r="D204" s="9" t="n">
-        <v>892002.55</v>
+        <v>950338.08</v>
       </c>
       <c r="E204" s="9" t="n">
-        <v>184585.63</v>
+        <v>232445</v>
       </c>
       <c r="F204" s="10" t="n">
-        <v>0.1059</v>
+        <v>0.1406</v>
       </c>
       <c r="G204" s="10" t="n">
-        <v>0.0517</v>
+        <v>0.08550000000000001</v>
       </c>
       <c r="H204" s="10" t="n"/>
       <c r="I204" s="10" t="n">
-        <v>0.1007</v>
+        <v>0.1018</v>
       </c>
       <c r="J204" s="13" t="n">
-        <v>22338</v>
+        <v>22519</v>
       </c>
       <c r="K204" s="13" t="n">
-        <v>37218</v>
+        <v>40392</v>
       </c>
       <c r="L204" s="32" t="n">
         <v>0</v>
@@ -21728,26 +21732,26 @@
         </is>
       </c>
       <c r="D289" s="15" t="n">
-        <v>16045.52</v>
+        <v>16068.95</v>
       </c>
       <c r="E289" s="15" t="n">
         <v>1923.97</v>
       </c>
       <c r="F289" s="16" t="n">
-        <v>0.8179</v>
+        <v>0.8183</v>
       </c>
       <c r="G289" s="16" t="n">
-        <v>0.7528</v>
+        <v>0.7532</v>
       </c>
       <c r="H289" s="16" t="n"/>
       <c r="I289" s="16" t="n">
-        <v>0.0135</v>
+        <v>0.0134</v>
       </c>
       <c r="J289" s="19" t="n">
-        <v>1412</v>
+        <v>1413</v>
       </c>
       <c r="K289" s="19" t="n">
-        <v>2066</v>
+        <v>2067</v>
       </c>
       <c r="L289" s="31" t="n">
         <v>0</v>
@@ -21770,26 +21774,26 @@
         </is>
       </c>
       <c r="D290" s="9" t="n">
-        <v>340007.34</v>
+        <v>359202.85</v>
       </c>
       <c r="E290" s="9" t="n">
-        <v>35967.65</v>
+        <v>37737.47</v>
       </c>
       <c r="F290" s="10" t="n">
-        <v>0.1124</v>
+        <v>0.1512</v>
       </c>
       <c r="G290" s="10" t="n">
-        <v>0.06510000000000001</v>
+        <v>0.1035</v>
       </c>
       <c r="H290" s="10" t="n"/>
       <c r="I290" s="10" t="n">
-        <v>0.2674</v>
+        <v>0.2696</v>
       </c>
       <c r="J290" s="13" t="n">
-        <v>2274</v>
+        <v>2322</v>
       </c>
       <c r="K290" s="13" t="n">
-        <v>8603</v>
+        <v>9275</v>
       </c>
       <c r="L290" s="32" t="n">
         <v>0</v>
@@ -21812,26 +21816,26 @@
         </is>
       </c>
       <c r="D291" s="15" t="n">
-        <v>152924.91</v>
+        <v>166228.2</v>
       </c>
       <c r="E291" s="15" t="n">
-        <v>27728.86</v>
+        <v>35861.65</v>
       </c>
       <c r="F291" s="16" t="n">
-        <v>-0.4606</v>
+        <v>-0.3582</v>
       </c>
       <c r="G291" s="16" t="n">
-        <v>-0.514</v>
+        <v>-0.4127</v>
       </c>
       <c r="H291" s="16" t="n"/>
       <c r="I291" s="16" t="n">
-        <v>0.1937</v>
+        <v>0.1946</v>
       </c>
       <c r="J291" s="19" t="n">
-        <v>3361</v>
+        <v>3413</v>
       </c>
       <c r="K291" s="19" t="n">
-        <v>5800</v>
+        <v>6459</v>
       </c>
       <c r="L291" s="31" t="n">
         <v>0</v>
@@ -21854,26 +21858,26 @@
         </is>
       </c>
       <c r="D292" s="9" t="n">
-        <v>147987.91</v>
+        <v>173119.37</v>
       </c>
       <c r="E292" s="9" t="n">
-        <v>51248</v>
+        <v>84107.82000000001</v>
       </c>
       <c r="F292" s="10" t="n">
-        <v>-0.1336</v>
+        <v>-0.019</v>
       </c>
       <c r="G292" s="10" t="n">
-        <v>-0.1869</v>
+        <v>-0.076</v>
       </c>
       <c r="H292" s="10" t="n"/>
       <c r="I292" s="10" t="n">
-        <v>0.135</v>
+        <v>0.136</v>
       </c>
       <c r="J292" s="13" t="n">
-        <v>3564</v>
+        <v>3595</v>
       </c>
       <c r="K292" s="13" t="n">
-        <v>5659</v>
+        <v>7446</v>
       </c>
       <c r="L292" s="32" t="n">
         <v>0</v>
@@ -21896,26 +21900,26 @@
         </is>
       </c>
       <c r="D293" s="15" t="n">
-        <v>83680.81</v>
+        <v>84187.06</v>
       </c>
       <c r="E293" s="15" t="n">
-        <v>25768.92</v>
+        <v>26314.81</v>
       </c>
       <c r="F293" s="16" t="n">
-        <v>0.3209</v>
+        <v>0.2809</v>
       </c>
       <c r="G293" s="16" t="n">
-        <v>0.2583</v>
+        <v>0.2182</v>
       </c>
       <c r="H293" s="16" t="n"/>
       <c r="I293" s="16" t="n">
-        <v>0.0854</v>
+        <v>0.0853</v>
       </c>
       <c r="J293" s="19" t="n">
-        <v>3125</v>
+        <v>3153</v>
       </c>
       <c r="K293" s="19" t="n">
-        <v>4097</v>
+        <v>4129</v>
       </c>
       <c r="L293" s="31" t="n">
         <v>0</v>
@@ -21938,26 +21942,26 @@
         </is>
       </c>
       <c r="D294" s="9" t="n">
-        <v>94807.64999999999</v>
+        <v>94884.47</v>
       </c>
       <c r="E294" s="9" t="n">
-        <v>34231.72</v>
+        <v>35096.5</v>
       </c>
       <c r="F294" s="10" t="n">
-        <v>0.6177</v>
+        <v>0.6168</v>
       </c>
       <c r="G294" s="10" t="n">
-        <v>0.5531</v>
+        <v>0.5521</v>
       </c>
       <c r="H294" s="10" t="n"/>
       <c r="I294" s="10" t="n">
-        <v>0.0393</v>
+        <v>0.0396</v>
       </c>
       <c r="J294" s="13" t="n">
-        <v>4832</v>
+        <v>4850</v>
       </c>
       <c r="K294" s="13" t="n">
-        <v>6387</v>
+        <v>6407</v>
       </c>
       <c r="L294" s="32" t="n">
         <v>0</v>
@@ -21980,26 +21984,26 @@
         </is>
       </c>
       <c r="D295" s="15" t="n">
-        <v>56548.41</v>
+        <v>56647.17</v>
       </c>
       <c r="E295" s="15" t="n">
-        <v>7716.51</v>
+        <v>11402.79</v>
       </c>
       <c r="F295" s="16" t="n">
-        <v>0.8465</v>
+        <v>0.8265</v>
       </c>
       <c r="G295" s="16" t="n">
-        <v>0.7798</v>
+        <v>0.7588</v>
       </c>
       <c r="H295" s="16" t="n"/>
       <c r="I295" s="16" t="n">
         <v>0.008999999999999999</v>
       </c>
       <c r="J295" s="19" t="n">
-        <v>3770</v>
+        <v>3773</v>
       </c>
       <c r="K295" s="19" t="n">
-        <v>4606</v>
+        <v>4609</v>
       </c>
       <c r="L295" s="31" t="n">
         <v>0</v>
@@ -22736,26 +22740,26 @@
         </is>
       </c>
       <c r="D313" s="15" t="n">
-        <v>5600710.43</v>
+        <v>5614853.86</v>
       </c>
       <c r="E313" s="15" t="n">
-        <v>3611215.76</v>
+        <v>3613192.19</v>
       </c>
       <c r="F313" s="16" t="n">
-        <v>0.3779</v>
+        <v>0.3754</v>
       </c>
       <c r="G313" s="16" t="n">
-        <v>0.3216</v>
+        <v>0.3192</v>
       </c>
       <c r="H313" s="16" t="n"/>
       <c r="I313" s="16" t="n">
-        <v>0.092</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="J313" s="19" t="n">
-        <v>116546</v>
+        <v>116756</v>
       </c>
       <c r="K313" s="19" t="n">
-        <v>288635</v>
+        <v>288930</v>
       </c>
       <c r="L313" s="31" t="n">
         <v>0</v>
@@ -27608,26 +27612,26 @@
         </is>
       </c>
       <c r="D429" s="15" t="n">
-        <v>520188.7</v>
+        <v>520206.49</v>
       </c>
       <c r="E429" s="15" t="n">
         <v>210426.28</v>
       </c>
       <c r="F429" s="16" t="n">
-        <v>0.7983</v>
+        <v>0.7975</v>
       </c>
       <c r="G429" s="16" t="n">
-        <v>0.7325</v>
+        <v>0.7317</v>
       </c>
       <c r="H429" s="16" t="n"/>
       <c r="I429" s="16" t="n">
         <v>0.0174</v>
       </c>
       <c r="J429" s="19" t="n">
-        <v>35335</v>
+        <v>35336</v>
       </c>
       <c r="K429" s="19" t="n">
-        <v>68038</v>
+        <v>68039</v>
       </c>
       <c r="L429" s="31" t="n">
         <v>0</v>
@@ -27650,26 +27654,26 @@
         </is>
       </c>
       <c r="D430" s="9" t="n">
-        <v>2099482.27</v>
+        <v>2107432.08</v>
       </c>
       <c r="E430" s="9" t="n">
-        <v>1010982.05</v>
+        <v>1011521.52</v>
       </c>
       <c r="F430" s="10" t="n">
-        <v>-0.0206</v>
+        <v>-0.0226</v>
       </c>
       <c r="G430" s="10" t="n">
-        <v>-0.0733</v>
+        <v>-0.0752</v>
       </c>
       <c r="H430" s="10" t="n"/>
       <c r="I430" s="10" t="n">
-        <v>0.2994</v>
+        <v>0.3008</v>
       </c>
       <c r="J430" s="13" t="n">
-        <v>9215</v>
+        <v>9274</v>
       </c>
       <c r="K430" s="13" t="n">
-        <v>33906</v>
+        <v>34012</v>
       </c>
       <c r="L430" s="32" t="n">
         <v>0</v>
@@ -27692,26 +27696,26 @@
         </is>
       </c>
       <c r="D431" s="15" t="n">
-        <v>908576.87</v>
+        <v>912040.27</v>
       </c>
       <c r="E431" s="15" t="n">
-        <v>217416.47</v>
+        <v>217419.87</v>
       </c>
       <c r="F431" s="16" t="n">
-        <v>0.4684</v>
+        <v>0.465</v>
       </c>
       <c r="G431" s="16" t="n">
-        <v>0.4178</v>
+        <v>0.4145</v>
       </c>
       <c r="H431" s="16" t="n"/>
       <c r="I431" s="16" t="n">
-        <v>0.1884</v>
+        <v>0.19</v>
       </c>
       <c r="J431" s="19" t="n">
-        <v>11613</v>
+        <v>11662</v>
       </c>
       <c r="K431" s="19" t="n">
-        <v>25911</v>
+        <v>25978</v>
       </c>
       <c r="L431" s="31" t="n">
         <v>0</v>
@@ -27734,26 +27738,26 @@
         </is>
       </c>
       <c r="D432" s="9" t="n">
-        <v>650386.8100000001</v>
+        <v>651727.04</v>
       </c>
       <c r="E432" s="9" t="n">
-        <v>156738.89</v>
+        <v>156879.23</v>
       </c>
       <c r="F432" s="10" t="n">
-        <v>0.6221</v>
+        <v>0.6195000000000001</v>
       </c>
       <c r="G432" s="10" t="n">
-        <v>0.5669</v>
+        <v>0.5644</v>
       </c>
       <c r="H432" s="10" t="n"/>
       <c r="I432" s="10" t="n">
-        <v>0.1424</v>
+        <v>0.143</v>
       </c>
       <c r="J432" s="13" t="n">
-        <v>12579</v>
+        <v>12608</v>
       </c>
       <c r="K432" s="13" t="n">
-        <v>25522</v>
+        <v>25565</v>
       </c>
       <c r="L432" s="32" t="n">
         <v>0</v>
@@ -27776,26 +27780,26 @@
         </is>
       </c>
       <c r="D433" s="15" t="n">
-        <v>373081.52</v>
+        <v>373580.46</v>
       </c>
       <c r="E433" s="15" t="n">
-        <v>212110.52</v>
+        <v>212500.3</v>
       </c>
       <c r="F433" s="16" t="n">
-        <v>0.619</v>
+        <v>0.6178</v>
       </c>
       <c r="G433" s="16" t="n">
-        <v>0.5608</v>
+        <v>0.5597</v>
       </c>
       <c r="H433" s="16" t="n"/>
       <c r="I433" s="16" t="n">
-        <v>0.1051</v>
+        <v>0.1058</v>
       </c>
       <c r="J433" s="19" t="n">
-        <v>10394</v>
+        <v>10419</v>
       </c>
       <c r="K433" s="19" t="n">
-        <v>17705</v>
+        <v>17733</v>
       </c>
       <c r="L433" s="31" t="n">
         <v>0</v>
@@ -27818,26 +27822,26 @@
         </is>
       </c>
       <c r="D434" s="9" t="n">
-        <v>521207.24</v>
+        <v>521946.32</v>
       </c>
       <c r="E434" s="9" t="n">
-        <v>336628.49</v>
+        <v>337518.48</v>
       </c>
       <c r="F434" s="10" t="n">
-        <v>0.6074000000000001</v>
+        <v>0.605</v>
       </c>
       <c r="G434" s="10" t="n">
-        <v>0.5463</v>
+        <v>0.5439000000000001</v>
       </c>
       <c r="H434" s="10" t="n"/>
       <c r="I434" s="10" t="n">
-        <v>0.0716</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="J434" s="13" t="n">
-        <v>18789</v>
+        <v>18832</v>
       </c>
       <c r="K434" s="13" t="n">
-        <v>35326</v>
+        <v>35372</v>
       </c>
       <c r="L434" s="32" t="n">
         <v>0</v>
@@ -27860,26 +27864,26 @@
         </is>
       </c>
       <c r="D435" s="15" t="n">
-        <v>527787</v>
+        <v>527921.2</v>
       </c>
       <c r="E435" s="15" t="n">
-        <v>1466913.05</v>
+        <v>1466926.51</v>
       </c>
       <c r="F435" s="16" t="n">
-        <v>0.6944</v>
+        <v>0.6932</v>
       </c>
       <c r="G435" s="16" t="n">
-        <v>0.6284</v>
+        <v>0.6272</v>
       </c>
       <c r="H435" s="16" t="n"/>
       <c r="I435" s="16" t="n">
-        <v>0.0504</v>
+        <v>0.0506</v>
       </c>
       <c r="J435" s="19" t="n">
-        <v>18621</v>
+        <v>18625</v>
       </c>
       <c r="K435" s="19" t="n">
-        <v>82227</v>
+        <v>82231</v>
       </c>
       <c r="L435" s="31" t="n">
         <v>0</v>
@@ -39222,29 +39226,29 @@
         </is>
       </c>
       <c r="D694" s="9" t="n">
-        <v>13555738.91</v>
+        <v>13563124.8</v>
       </c>
       <c r="E694" s="9" t="n">
-        <v>78769140.43000001</v>
+        <v>78794857.51000001</v>
       </c>
       <c r="F694" s="10" t="n">
-        <v>0.2923</v>
+        <v>0.2912</v>
       </c>
       <c r="G694" s="10" t="n">
-        <v>0.226</v>
+        <v>0.2249</v>
       </c>
       <c r="H694" s="10" t="n"/>
       <c r="I694" s="10" t="n">
-        <v>0.0689</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="J694" s="13" t="n">
-        <v>485748</v>
+        <v>485822</v>
       </c>
       <c r="K694" s="13" t="n">
-        <v>669193</v>
+        <v>669298</v>
       </c>
       <c r="L694" s="32" t="n">
-        <v>0.527</v>
+        <v>0.5271</v>
       </c>
     </row>
     <row r="695">
@@ -39264,29 +39268,29 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>2286443.2</v>
+        <v>2325254.86</v>
       </c>
       <c r="E695" s="15" t="n">
-        <v>14425593.65</v>
+        <v>14545221.86</v>
       </c>
       <c r="F695" s="16" t="n">
-        <v>0.3191</v>
+        <v>0.2543</v>
       </c>
       <c r="G695" s="16" t="n">
-        <v>0.2523</v>
+        <v>0.1878</v>
       </c>
       <c r="H695" s="16" t="n"/>
       <c r="I695" s="16" t="n">
-        <v>0.0374</v>
+        <v>0.0419</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>109527</v>
+        <v>110450</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>146057</v>
+        <v>147323</v>
       </c>
       <c r="L695" s="31" t="n">
-        <v>0.7869</v>
+        <v>0.7877</v>
       </c>
     </row>
     <row r="696">
@@ -42834,29 +42838,29 @@
         </is>
       </c>
       <c r="D780" s="9" t="n">
-        <v>3103056.95</v>
+        <v>3103435.12</v>
       </c>
       <c r="E780" s="9" t="n">
-        <v>49897945.68</v>
+        <v>49923181.25</v>
       </c>
       <c r="F780" s="10" t="n">
-        <v>0.5425</v>
+        <v>0.5415</v>
       </c>
       <c r="G780" s="10" t="n">
-        <v>0.4621</v>
+        <v>0.4611</v>
       </c>
       <c r="H780" s="10" t="n"/>
       <c r="I780" s="10" t="n">
-        <v>0.0183</v>
+        <v>0.0184</v>
       </c>
       <c r="J780" s="13" t="n">
-        <v>250222</v>
+        <v>250240</v>
       </c>
       <c r="K780" s="13" t="n">
-        <v>337767</v>
+        <v>337791</v>
       </c>
       <c r="L780" s="32" t="n">
-        <v>0.5719</v>
+        <v>0.572</v>
       </c>
     </row>
     <row r="781">
@@ -42876,29 +42880,29 @@
         </is>
       </c>
       <c r="D781" s="15" t="n">
-        <v>1914031.08</v>
+        <v>1917224.51</v>
       </c>
       <c r="E781" s="15" t="n">
-        <v>1048138.13</v>
+        <v>1048139.89</v>
       </c>
       <c r="F781" s="16" t="n">
-        <v>0.212</v>
+        <v>0.2102</v>
       </c>
       <c r="G781" s="16" t="n">
-        <v>0.169</v>
+        <v>0.1672</v>
       </c>
       <c r="H781" s="16" t="n"/>
       <c r="I781" s="16" t="n">
-        <v>0.3292</v>
+        <v>0.3296</v>
       </c>
       <c r="J781" s="19" t="n">
-        <v>9871</v>
+        <v>9876</v>
       </c>
       <c r="K781" s="19" t="n">
-        <v>25455</v>
+        <v>25462</v>
       </c>
       <c r="L781" s="31" t="n">
-        <v>0.4786</v>
+        <v>0.4795</v>
       </c>
     </row>
     <row r="782">
@@ -42918,29 +42922,29 @@
         </is>
       </c>
       <c r="D782" s="9" t="n">
-        <v>1953157.41</v>
+        <v>1956078.89</v>
       </c>
       <c r="E782" s="9" t="n">
-        <v>2022283.53</v>
+        <v>2022379.17</v>
       </c>
       <c r="F782" s="10" t="n">
-        <v>0.1389</v>
+        <v>0.1364</v>
       </c>
       <c r="G782" s="10" t="n">
-        <v>0.0844</v>
+        <v>0.0819</v>
       </c>
       <c r="H782" s="10" t="n"/>
       <c r="I782" s="10" t="n">
-        <v>0.2451</v>
+        <v>0.2455</v>
       </c>
       <c r="J782" s="13" t="n">
-        <v>20995</v>
+        <v>21007</v>
       </c>
       <c r="K782" s="13" t="n">
-        <v>38546</v>
+        <v>38564</v>
       </c>
       <c r="L782" s="32" t="n">
-        <v>0.5301</v>
+        <v>0.5303</v>
       </c>
     </row>
     <row r="783">
@@ -42960,29 +42964,29 @@
         </is>
       </c>
       <c r="D783" s="15" t="n">
-        <v>1550894.83</v>
+        <v>1551278.28</v>
       </c>
       <c r="E783" s="15" t="n">
-        <v>2905915.81</v>
+        <v>2905920.09</v>
       </c>
       <c r="F783" s="16" t="n">
-        <v>0.1737</v>
+        <v>0.1729</v>
       </c>
       <c r="G783" s="16" t="n">
-        <v>0.1097</v>
+        <v>0.1089</v>
       </c>
       <c r="H783" s="16" t="n"/>
       <c r="I783" s="16" t="n">
-        <v>0.1834</v>
+        <v>0.1837</v>
       </c>
       <c r="J783" s="19" t="n">
-        <v>28049</v>
+        <v>28057</v>
       </c>
       <c r="K783" s="19" t="n">
-        <v>41160</v>
+        <v>41170</v>
       </c>
       <c r="L783" s="31" t="n">
-        <v>0.5454</v>
+        <v>0.5453</v>
       </c>
     </row>
     <row r="784">
@@ -43002,26 +43006,26 @@
         </is>
       </c>
       <c r="D784" s="9" t="n">
-        <v>1259857.94</v>
+        <v>1259986.53</v>
       </c>
       <c r="E784" s="9" t="n">
-        <v>3415532.04</v>
+        <v>3415554.13</v>
       </c>
       <c r="F784" s="10" t="n">
-        <v>0.1874</v>
+        <v>0.1871</v>
       </c>
       <c r="G784" s="10" t="n">
-        <v>0.1198</v>
+        <v>0.1195</v>
       </c>
       <c r="H784" s="10" t="n"/>
       <c r="I784" s="10" t="n">
-        <v>0.1443</v>
+        <v>0.1444</v>
       </c>
       <c r="J784" s="13" t="n">
-        <v>30275</v>
+        <v>30281</v>
       </c>
       <c r="K784" s="13" t="n">
-        <v>40867</v>
+        <v>40875</v>
       </c>
       <c r="L784" s="32" t="n">
         <v>0.5073</v>
@@ -43044,26 +43048,26 @@
         </is>
       </c>
       <c r="D785" s="15" t="n">
-        <v>2012592.08</v>
+        <v>2012842.27</v>
       </c>
       <c r="E785" s="15" t="n">
-        <v>7497972.48</v>
+        <v>7498203.38</v>
       </c>
       <c r="F785" s="16" t="n">
-        <v>0.1848</v>
+        <v>0.1846</v>
       </c>
       <c r="G785" s="16" t="n">
-        <v>0.1152</v>
+        <v>0.115</v>
       </c>
       <c r="H785" s="16" t="n"/>
       <c r="I785" s="16" t="n">
-        <v>0.0978</v>
+        <v>0.09810000000000001</v>
       </c>
       <c r="J785" s="19" t="n">
-        <v>64298</v>
+        <v>64314</v>
       </c>
       <c r="K785" s="19" t="n">
-        <v>82610</v>
+        <v>82635</v>
       </c>
       <c r="L785" s="31" t="n">
         <v>0.509</v>
@@ -43086,26 +43090,26 @@
         </is>
       </c>
       <c r="D786" s="9" t="n">
-        <v>1762148.64</v>
+        <v>1762279.2</v>
       </c>
       <c r="E786" s="9" t="n">
-        <v>11981352.77</v>
+        <v>11981479.59</v>
       </c>
       <c r="F786" s="10" t="n">
-        <v>0.4113</v>
+        <v>0.411</v>
       </c>
       <c r="G786" s="10" t="n">
-        <v>0.3336</v>
+        <v>0.3333</v>
       </c>
       <c r="H786" s="10" t="n"/>
       <c r="I786" s="10" t="n">
-        <v>0.057</v>
+        <v>0.0571</v>
       </c>
       <c r="J786" s="13" t="n">
-        <v>82038</v>
+        <v>82047</v>
       </c>
       <c r="K786" s="13" t="n">
-        <v>102788</v>
+        <v>102801</v>
       </c>
       <c r="L786" s="32" t="n">
         <v>0.5152</v>
@@ -43128,29 +43132,29 @@
         </is>
       </c>
       <c r="D787" s="15" t="n">
-        <v>691808.91</v>
+        <v>702518.55</v>
       </c>
       <c r="E787" s="15" t="n">
-        <v>10560558.16</v>
+        <v>10661798.39</v>
       </c>
       <c r="F787" s="16" t="n">
-        <v>0.6709000000000001</v>
+        <v>0.6118</v>
       </c>
       <c r="G787" s="16" t="n">
-        <v>0.5954</v>
+        <v>0.5366</v>
       </c>
       <c r="H787" s="16" t="n"/>
       <c r="I787" s="16" t="n">
-        <v>0.011</v>
+        <v>0.0131</v>
       </c>
       <c r="J787" s="19" t="n">
-        <v>66290</v>
+        <v>66711</v>
       </c>
       <c r="K787" s="19" t="n">
-        <v>85687</v>
+        <v>86254</v>
       </c>
       <c r="L787" s="31" t="n">
-        <v>0.6266</v>
+        <v>0.6288</v>
       </c>
     </row>
     <row r="788">
@@ -43170,29 +43174,29 @@
         </is>
       </c>
       <c r="D788" s="9" t="n">
-        <v>224066.16</v>
+        <v>227093.56</v>
       </c>
       <c r="E788" s="9" t="n">
-        <v>651962.35</v>
+        <v>654005.79</v>
       </c>
       <c r="F788" s="10" t="n">
-        <v>-0.4034</v>
+        <v>-0.3844</v>
       </c>
       <c r="G788" s="10" t="n">
-        <v>-0.4665</v>
+        <v>-0.4474</v>
       </c>
       <c r="H788" s="10" t="n"/>
       <c r="I788" s="10" t="n">
-        <v>0.3184</v>
+        <v>0.3273</v>
       </c>
       <c r="J788" s="13" t="n">
-        <v>1187</v>
+        <v>1207</v>
       </c>
       <c r="K788" s="13" t="n">
-        <v>2945</v>
+        <v>3014</v>
       </c>
       <c r="L788" s="32" t="n">
-        <v>0.9471000000000001</v>
+        <v>0.9476</v>
       </c>
     </row>
     <row r="789">
@@ -43212,29 +43216,29 @@
         </is>
       </c>
       <c r="D789" s="15" t="n">
-        <v>289364.23</v>
+        <v>291639.01</v>
       </c>
       <c r="E789" s="15" t="n">
-        <v>101302.99</v>
+        <v>101358.54</v>
       </c>
       <c r="F789" s="16" t="n">
-        <v>0.0415</v>
+        <v>0.0274</v>
       </c>
       <c r="G789" s="16" t="n">
-        <v>-0.0047</v>
+        <v>-0.0188</v>
       </c>
       <c r="H789" s="16" t="n"/>
       <c r="I789" s="16" t="n">
-        <v>0.2109</v>
+        <v>0.2201</v>
       </c>
       <c r="J789" s="19" t="n">
-        <v>2864</v>
+        <v>2912</v>
       </c>
       <c r="K789" s="19" t="n">
-        <v>4801</v>
+        <v>4869</v>
       </c>
       <c r="L789" s="31" t="n">
-        <v>0.9386</v>
+        <v>0.9389</v>
       </c>
     </row>
     <row r="790">
@@ -43254,29 +43258,29 @@
         </is>
       </c>
       <c r="D790" s="9" t="n">
-        <v>229793.07</v>
+        <v>235046.37</v>
       </c>
       <c r="E790" s="9" t="n">
-        <v>263346.96</v>
+        <v>263750.87</v>
       </c>
       <c r="F790" s="10" t="n">
-        <v>0.1891</v>
+        <v>0.1606</v>
       </c>
       <c r="G790" s="10" t="n">
-        <v>0.1279</v>
+        <v>0.1</v>
       </c>
       <c r="H790" s="10" t="n"/>
       <c r="I790" s="10" t="n">
-        <v>0.1389</v>
+        <v>0.1488</v>
       </c>
       <c r="J790" s="13" t="n">
-        <v>4212</v>
+        <v>4275</v>
       </c>
       <c r="K790" s="13" t="n">
-        <v>5822</v>
+        <v>5894</v>
       </c>
       <c r="L790" s="32" t="n">
-        <v>0.8488</v>
+        <v>0.8516</v>
       </c>
     </row>
     <row r="791">
@@ -43296,29 +43300,29 @@
         </is>
       </c>
       <c r="D791" s="15" t="n">
-        <v>231834.61</v>
+        <v>234203.3</v>
       </c>
       <c r="E791" s="15" t="n">
-        <v>232242.15</v>
+        <v>233816.11</v>
       </c>
       <c r="F791" s="16" t="n">
-        <v>0.2537</v>
+        <v>0.212</v>
       </c>
       <c r="G791" s="16" t="n">
-        <v>0.1895</v>
+        <v>0.1477</v>
       </c>
       <c r="H791" s="16" t="n"/>
       <c r="I791" s="16" t="n">
-        <v>0.0961</v>
+        <v>0.1051</v>
       </c>
       <c r="J791" s="19" t="n">
-        <v>5320</v>
+        <v>5393</v>
       </c>
       <c r="K791" s="19" t="n">
-        <v>11067</v>
+        <v>11156</v>
       </c>
       <c r="L791" s="31" t="n">
-        <v>0.906</v>
+        <v>0.9046</v>
       </c>
     </row>
     <row r="792">
@@ -43338,29 +43342,29 @@
         </is>
       </c>
       <c r="D792" s="9" t="n">
-        <v>315458.88</v>
+        <v>324551.56</v>
       </c>
       <c r="E792" s="9" t="n">
-        <v>833171.25</v>
+        <v>836709.71</v>
       </c>
       <c r="F792" s="10" t="n">
-        <v>0.3182</v>
+        <v>0.221</v>
       </c>
       <c r="G792" s="10" t="n">
-        <v>0.2493</v>
+        <v>0.1527</v>
       </c>
       <c r="H792" s="10" t="n"/>
       <c r="I792" s="10" t="n">
-        <v>0.0574</v>
+        <v>0.0654</v>
       </c>
       <c r="J792" s="13" t="n">
-        <v>12415</v>
+        <v>12549</v>
       </c>
       <c r="K792" s="13" t="n">
-        <v>15200</v>
+        <v>15386</v>
       </c>
       <c r="L792" s="32" t="n">
-        <v>0.7922</v>
+        <v>0.7971</v>
       </c>
     </row>
     <row r="793">
@@ -43380,29 +43384,29 @@
         </is>
       </c>
       <c r="D793" s="15" t="n">
-        <v>304117.35</v>
+        <v>310202.51</v>
       </c>
       <c r="E793" s="15" t="n">
-        <v>1783009.79</v>
+        <v>1793782.44</v>
       </c>
       <c r="F793" s="16" t="n">
-        <v>0.4639</v>
+        <v>0.2633</v>
       </c>
       <c r="G793" s="16" t="n">
-        <v>0.3912</v>
+        <v>0.1907</v>
       </c>
       <c r="H793" s="16" t="n"/>
       <c r="I793" s="16" t="n">
-        <v>0.0335</v>
+        <v>0.0396</v>
       </c>
       <c r="J793" s="19" t="n">
-        <v>17239</v>
+        <v>17403</v>
       </c>
       <c r="K793" s="19" t="n">
-        <v>20535</v>
+        <v>20750</v>
       </c>
       <c r="L793" s="31" t="n">
-        <v>0.7465000000000001</v>
+        <v>0.7419</v>
       </c>
     </row>
     <row r="794">
@@ -44346,29 +44350,29 @@
         </is>
       </c>
       <c r="D816" s="9" t="n">
-        <v>6223349.88</v>
+        <v>6248821.51</v>
       </c>
       <c r="E816" s="9" t="n">
-        <v>8002346.45</v>
+        <v>8007787.59</v>
       </c>
       <c r="F816" s="10" t="n">
-        <v>0.3736</v>
+        <v>0.3664</v>
       </c>
       <c r="G816" s="10" t="n">
-        <v>0.3177</v>
+        <v>0.3105</v>
       </c>
       <c r="H816" s="10" t="n"/>
       <c r="I816" s="10" t="n">
-        <v>0.0636</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="J816" s="13" t="n">
-        <v>121077</v>
+        <v>121320</v>
       </c>
       <c r="K816" s="13" t="n">
-        <v>223478</v>
+        <v>223804</v>
       </c>
       <c r="L816" s="32" t="n">
-        <v>0.9233</v>
+        <v>0.9224</v>
       </c>
     </row>
     <row r="817">
@@ -50856,26 +50860,26 @@
         </is>
       </c>
       <c r="D971" s="15" t="n">
-        <v>613263.3</v>
+        <v>613628.21</v>
       </c>
       <c r="E971" s="15" t="n">
-        <v>3919612.15</v>
+        <v>3923100.42</v>
       </c>
       <c r="F971" s="16" t="n">
-        <v>0.6985</v>
+        <v>0.6973</v>
       </c>
       <c r="G971" s="16" t="n">
-        <v>0.6294</v>
+        <v>0.6283</v>
       </c>
       <c r="H971" s="16" t="n"/>
       <c r="I971" s="16" t="n">
-        <v>0.0165</v>
+        <v>0.0167</v>
       </c>
       <c r="J971" s="19" t="n">
-        <v>42630</v>
+        <v>42664</v>
       </c>
       <c r="K971" s="19" t="n">
-        <v>80655</v>
+        <v>80692</v>
       </c>
       <c r="L971" s="31" t="n">
         <v>0.8226</v>
@@ -50898,26 +50902,26 @@
         </is>
       </c>
       <c r="D972" s="9" t="n">
-        <v>2043139.43</v>
+        <v>2054736.72</v>
       </c>
       <c r="E972" s="9" t="n">
-        <v>506299.15</v>
+        <v>506959.58</v>
       </c>
       <c r="F972" s="10" t="n">
-        <v>0.1699</v>
+        <v>0.1576</v>
       </c>
       <c r="G972" s="10" t="n">
-        <v>0.1233</v>
+        <v>0.111</v>
       </c>
       <c r="H972" s="10" t="n"/>
       <c r="I972" s="10" t="n">
-        <v>0.3047</v>
+        <v>0.3058</v>
       </c>
       <c r="J972" s="13" t="n">
-        <v>4037</v>
+        <v>4078</v>
       </c>
       <c r="K972" s="13" t="n">
-        <v>21552</v>
+        <v>21632</v>
       </c>
       <c r="L972" s="32" t="n">
         <v>0.9654</v>
@@ -50940,29 +50944,29 @@
         </is>
       </c>
       <c r="D973" s="15" t="n">
-        <v>1041608.2</v>
+        <v>1044036.57</v>
       </c>
       <c r="E973" s="15" t="n">
-        <v>316220.83</v>
+        <v>316272.67</v>
       </c>
       <c r="F973" s="16" t="n">
-        <v>0.2819</v>
+        <v>0.2818</v>
       </c>
       <c r="G973" s="16" t="n">
-        <v>0.2296</v>
+        <v>0.2295</v>
       </c>
       <c r="H973" s="16" t="n"/>
       <c r="I973" s="16" t="n">
-        <v>0.1816</v>
+        <v>0.1832</v>
       </c>
       <c r="J973" s="19" t="n">
-        <v>8342</v>
+        <v>8394</v>
       </c>
       <c r="K973" s="19" t="n">
-        <v>15936</v>
+        <v>16010</v>
       </c>
       <c r="L973" s="31" t="n">
-        <v>0.9456</v>
+        <v>0.9455</v>
       </c>
     </row>
     <row r="974">
@@ -50982,29 +50986,29 @@
         </is>
       </c>
       <c r="D974" s="9" t="n">
-        <v>792138.55</v>
+        <v>799689.71</v>
       </c>
       <c r="E974" s="9" t="n">
-        <v>265931.49</v>
+        <v>265967.82</v>
       </c>
       <c r="F974" s="10" t="n">
-        <v>0.3786</v>
+        <v>0.365</v>
       </c>
       <c r="G974" s="10" t="n">
-        <v>0.3217</v>
+        <v>0.3083</v>
       </c>
       <c r="H974" s="10" t="n"/>
       <c r="I974" s="10" t="n">
-        <v>0.1197</v>
+        <v>0.1203</v>
       </c>
       <c r="J974" s="13" t="n">
-        <v>12060</v>
+        <v>12105</v>
       </c>
       <c r="K974" s="13" t="n">
-        <v>20126</v>
+        <v>20181</v>
       </c>
       <c r="L974" s="32" t="n">
-        <v>0.9409</v>
+        <v>0.9329</v>
       </c>
     </row>
     <row r="975">
@@ -51024,29 +51028,29 @@
         </is>
       </c>
       <c r="D975" s="15" t="n">
-        <v>531006.38</v>
+        <v>532341.37</v>
       </c>
       <c r="E975" s="15" t="n">
-        <v>331085.8</v>
+        <v>331751.44</v>
       </c>
       <c r="F975" s="16" t="n">
-        <v>0.4792</v>
+        <v>0.4732</v>
       </c>
       <c r="G975" s="16" t="n">
-        <v>0.4188</v>
+        <v>0.4128</v>
       </c>
       <c r="H975" s="16" t="n"/>
       <c r="I975" s="16" t="n">
-        <v>0.0883</v>
+        <v>0.0886</v>
       </c>
       <c r="J975" s="19" t="n">
-        <v>10642</v>
+        <v>10664</v>
       </c>
       <c r="K975" s="19" t="n">
-        <v>14473</v>
+        <v>14499</v>
       </c>
       <c r="L975" s="31" t="n">
-        <v>0.9205</v>
+        <v>0.9206</v>
       </c>
     </row>
     <row r="976">
@@ -51066,26 +51070,26 @@
         </is>
       </c>
       <c r="D976" s="9" t="n">
-        <v>688524.01</v>
+        <v>688939.83</v>
       </c>
       <c r="E976" s="9" t="n">
-        <v>696951.3100000001</v>
+        <v>697333.22</v>
       </c>
       <c r="F976" s="10" t="n">
-        <v>0.5625</v>
+        <v>0.5612</v>
       </c>
       <c r="G976" s="10" t="n">
-        <v>0.5002</v>
+        <v>0.4989</v>
       </c>
       <c r="H976" s="10" t="n"/>
       <c r="I976" s="10" t="n">
-        <v>0.0548</v>
+        <v>0.055</v>
       </c>
       <c r="J976" s="13" t="n">
-        <v>20978</v>
+        <v>21007</v>
       </c>
       <c r="K976" s="13" t="n">
-        <v>27963</v>
+        <v>27996</v>
       </c>
       <c r="L976" s="32" t="n">
         <v>0.8843</v>
@@ -51108,29 +51112,29 @@
         </is>
       </c>
       <c r="D977" s="15" t="n">
-        <v>513670</v>
+        <v>515449.09</v>
       </c>
       <c r="E977" s="15" t="n">
-        <v>1966245.73</v>
+        <v>1966402.44</v>
       </c>
       <c r="F977" s="16" t="n">
-        <v>0.6119</v>
+        <v>0.6075</v>
       </c>
       <c r="G977" s="16" t="n">
-        <v>0.5423</v>
+        <v>0.538</v>
       </c>
       <c r="H977" s="16" t="n"/>
       <c r="I977" s="16" t="n">
-        <v>0.0325</v>
+        <v>0.0328</v>
       </c>
       <c r="J977" s="19" t="n">
-        <v>22388</v>
+        <v>22408</v>
       </c>
       <c r="K977" s="19" t="n">
-        <v>42773</v>
+        <v>42794</v>
       </c>
       <c r="L977" s="31" t="n">
-        <v>0.859</v>
+        <v>0.8594000000000001</v>
       </c>
     </row>
     <row r="978">
@@ -51612,29 +51616,29 @@
         </is>
       </c>
       <c r="D989" s="15" t="n">
-        <v>479726.24</v>
+        <v>485456.77</v>
       </c>
       <c r="E989" s="15" t="n">
-        <v>2413154.35</v>
+        <v>2413953.61</v>
       </c>
       <c r="F989" s="16" t="n">
-        <v>0.6395</v>
+        <v>0.6264</v>
       </c>
       <c r="G989" s="16" t="n">
-        <v>0.5718</v>
+        <v>0.5589</v>
       </c>
       <c r="H989" s="16" t="n"/>
       <c r="I989" s="16" t="n">
-        <v>0.0218</v>
+        <v>0.0246</v>
       </c>
       <c r="J989" s="19" t="n">
-        <v>15963</v>
+        <v>16155</v>
       </c>
       <c r="K989" s="19" t="n">
-        <v>18896</v>
+        <v>19198</v>
       </c>
       <c r="L989" s="31" t="n">
-        <v>0.4235</v>
+        <v>0.4289</v>
       </c>
     </row>
     <row r="990">
@@ -54888,29 +54892,29 @@
         </is>
       </c>
       <c r="D1067" s="15" t="n">
-        <v>233161.51</v>
+        <v>233555.74</v>
       </c>
       <c r="E1067" s="15" t="n">
         <v>1837871.31</v>
       </c>
       <c r="F1067" s="16" t="n">
-        <v>0.8172</v>
+        <v>0.8175</v>
       </c>
       <c r="G1067" s="16" t="n">
-        <v>0.7465000000000001</v>
+        <v>0.7468</v>
       </c>
       <c r="H1067" s="16" t="n"/>
       <c r="I1067" s="16" t="n">
         <v>0.0119</v>
       </c>
       <c r="J1067" s="19" t="n">
-        <v>11030</v>
+        <v>11073</v>
       </c>
       <c r="K1067" s="19" t="n">
-        <v>13106</v>
+        <v>13196</v>
       </c>
       <c r="L1067" s="31" t="n">
-        <v>0.3854</v>
+        <v>0.3861</v>
       </c>
     </row>
     <row r="1068">
@@ -54930,29 +54934,29 @@
         </is>
       </c>
       <c r="D1068" s="9" t="n">
-        <v>62865.35</v>
+        <v>64292.31</v>
       </c>
       <c r="E1068" s="9" t="n">
-        <v>71345.60000000001</v>
+        <v>71370.85000000001</v>
       </c>
       <c r="F1068" s="10" t="n">
-        <v>0.3934</v>
+        <v>0.3889</v>
       </c>
       <c r="G1068" s="10" t="n">
-        <v>0.3453</v>
+        <v>0.3412</v>
       </c>
       <c r="H1068" s="10" t="n"/>
       <c r="I1068" s="10" t="n">
-        <v>0.1498</v>
+        <v>0.1868</v>
       </c>
       <c r="J1068" s="13" t="n">
-        <v>247</v>
+        <v>273</v>
       </c>
       <c r="K1068" s="13" t="n">
-        <v>438</v>
+        <v>482</v>
       </c>
       <c r="L1068" s="32" t="n">
-        <v>0.3498</v>
+        <v>0.3631</v>
       </c>
     </row>
     <row r="1069">
@@ -54972,29 +54976,29 @@
         </is>
       </c>
       <c r="D1069" s="15" t="n">
-        <v>19872.63</v>
+        <v>20946.59</v>
       </c>
       <c r="E1069" s="15" t="n">
-        <v>20581.87</v>
+        <v>20730.88</v>
       </c>
       <c r="F1069" s="16" t="n">
-        <v>0.4844</v>
+        <v>0.4019</v>
       </c>
       <c r="G1069" s="16" t="n">
-        <v>0.4243</v>
+        <v>0.342</v>
       </c>
       <c r="H1069" s="16" t="n"/>
       <c r="I1069" s="16" t="n">
-        <v>0.1152</v>
+        <v>0.133</v>
       </c>
       <c r="J1069" s="19" t="n">
-        <v>356</v>
+        <v>376</v>
       </c>
       <c r="K1069" s="19" t="n">
-        <v>392</v>
+        <v>435</v>
       </c>
       <c r="L1069" s="31" t="n">
-        <v>0.6694</v>
+        <v>0.6827</v>
       </c>
     </row>
     <row r="1070">
@@ -55014,29 +55018,29 @@
         </is>
       </c>
       <c r="D1070" s="9" t="n">
-        <v>20872.71</v>
+        <v>21422.82</v>
       </c>
       <c r="E1070" s="9" t="n">
-        <v>25687.12</v>
+        <v>25909.37</v>
       </c>
       <c r="F1070" s="10" t="n">
-        <v>0.3482</v>
+        <v>0.2956</v>
       </c>
       <c r="G1070" s="10" t="n">
-        <v>0.2806</v>
+        <v>0.2282</v>
       </c>
       <c r="H1070" s="10" t="n"/>
       <c r="I1070" s="10" t="n">
-        <v>0.0847</v>
+        <v>0.0959</v>
       </c>
       <c r="J1070" s="13" t="n">
-        <v>472</v>
+        <v>490</v>
       </c>
       <c r="K1070" s="13" t="n">
-        <v>529</v>
+        <v>557</v>
       </c>
       <c r="L1070" s="32" t="n">
-        <v>0.5947</v>
+        <v>0.6012999999999999</v>
       </c>
     </row>
     <row r="1071">
@@ -55056,29 +55060,29 @@
         </is>
       </c>
       <c r="D1071" s="15" t="n">
-        <v>26457.86</v>
+        <v>26886.56</v>
       </c>
       <c r="E1071" s="15" t="n">
-        <v>41545.73</v>
+        <v>41633.96</v>
       </c>
       <c r="F1071" s="16" t="n">
-        <v>0.3725</v>
+        <v>0.3707</v>
       </c>
       <c r="G1071" s="16" t="n">
-        <v>0.3104</v>
+        <v>0.3086</v>
       </c>
       <c r="H1071" s="16" t="n"/>
       <c r="I1071" s="16" t="n">
-        <v>0.0703</v>
+        <v>0.0798</v>
       </c>
       <c r="J1071" s="19" t="n">
-        <v>498</v>
+        <v>526</v>
       </c>
       <c r="K1071" s="19" t="n">
-        <v>554</v>
+        <v>587</v>
       </c>
       <c r="L1071" s="31" t="n">
-        <v>0.708</v>
+        <v>0.7076</v>
       </c>
     </row>
     <row r="1072">
@@ -55098,29 +55102,29 @@
         </is>
       </c>
       <c r="D1072" s="9" t="n">
-        <v>47067.56</v>
+        <v>48565.08</v>
       </c>
       <c r="E1072" s="9" t="n">
-        <v>127087.23</v>
+        <v>127324.03</v>
       </c>
       <c r="F1072" s="10" t="n">
-        <v>0.1405</v>
+        <v>0.144</v>
       </c>
       <c r="G1072" s="10" t="n">
-        <v>0.06569999999999999</v>
+        <v>0.0694</v>
       </c>
       <c r="H1072" s="10" t="n"/>
       <c r="I1072" s="10" t="n">
-        <v>0.0283</v>
+        <v>0.0331</v>
       </c>
       <c r="J1072" s="13" t="n">
-        <v>1413</v>
+        <v>1448</v>
       </c>
       <c r="K1072" s="13" t="n">
-        <v>1604</v>
+        <v>1644</v>
       </c>
       <c r="L1072" s="32" t="n">
-        <v>0.5881</v>
+        <v>0.5958</v>
       </c>
     </row>
     <row r="1073">
@@ -55140,29 +55144,29 @@
         </is>
       </c>
       <c r="D1073" s="15" t="n">
-        <v>69428.62</v>
+        <v>69787.64999999999</v>
       </c>
       <c r="E1073" s="15" t="n">
-        <v>289035.49</v>
+        <v>289113.2</v>
       </c>
       <c r="F1073" s="16" t="n">
-        <v>0.8375</v>
+        <v>0.8089</v>
       </c>
       <c r="G1073" s="16" t="n">
-        <v>0.7625</v>
+        <v>0.734</v>
       </c>
       <c r="H1073" s="16" t="n"/>
       <c r="I1073" s="16" t="n">
-        <v>0.0123</v>
+        <v>0.0142</v>
       </c>
       <c r="J1073" s="19" t="n">
-        <v>1947</v>
+        <v>1969</v>
       </c>
       <c r="K1073" s="19" t="n">
-        <v>2273</v>
+        <v>2297</v>
       </c>
       <c r="L1073" s="31" t="n">
-        <v>0.2768</v>
+        <v>0.2799</v>
       </c>
     </row>
     <row r="1074">
@@ -55602,26 +55606,26 @@
         </is>
       </c>
       <c r="D1084" s="9" t="n">
-        <v>333156.22</v>
+        <v>341357.47</v>
       </c>
       <c r="E1084" s="9" t="n">
-        <v>295931.41</v>
+        <v>298924.53</v>
       </c>
       <c r="F1084" s="10" t="n">
-        <v>0.3674</v>
+        <v>0.3574</v>
       </c>
       <c r="G1084" s="10" t="n">
-        <v>0.3122</v>
+        <v>0.3023</v>
       </c>
       <c r="H1084" s="10" t="n"/>
       <c r="I1084" s="10" t="n">
-        <v>0.0673</v>
+        <v>0.0747</v>
       </c>
       <c r="J1084" s="13" t="n">
-        <v>6254</v>
+        <v>6611</v>
       </c>
       <c r="K1084" s="13" t="n">
-        <v>13124</v>
+        <v>13560</v>
       </c>
       <c r="L1084" s="32" t="n">
         <v>0</v>
@@ -58584,26 +58588,26 @@
         </is>
       </c>
       <c r="D1155" s="15" t="n">
-        <v>4768.62</v>
+        <v>6842.13</v>
       </c>
       <c r="E1155" s="15" t="n">
-        <v>24162.78</v>
+        <v>24626.87</v>
       </c>
       <c r="F1155" s="16" t="n">
-        <v>1.0128</v>
+        <v>0.8296</v>
       </c>
       <c r="G1155" s="16" t="n">
-        <v>0.9455</v>
+        <v>0.7726</v>
       </c>
       <c r="H1155" s="16" t="n"/>
       <c r="I1155" s="16" t="n">
-        <v>0.0028</v>
+        <v>0.0098</v>
       </c>
       <c r="J1155" s="19" t="n">
-        <v>723</v>
+        <v>813</v>
       </c>
       <c r="K1155" s="19" t="n">
-        <v>880</v>
+        <v>982</v>
       </c>
       <c r="L1155" s="31" t="n">
         <v>0</v>
@@ -58626,26 +58630,26 @@
         </is>
       </c>
       <c r="D1156" s="9" t="n">
-        <v>142449.59</v>
+        <v>146538.16</v>
       </c>
       <c r="E1156" s="9" t="n">
-        <v>36234.92</v>
+        <v>36315.91</v>
       </c>
       <c r="F1156" s="10" t="n">
-        <v>0.1095</v>
+        <v>0.1192</v>
       </c>
       <c r="G1156" s="10" t="n">
-        <v>0.0629</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="H1156" s="10" t="n"/>
       <c r="I1156" s="10" t="n">
-        <v>0.1823</v>
+        <v>0.1978</v>
       </c>
       <c r="J1156" s="13" t="n">
-        <v>1086</v>
+        <v>1188</v>
       </c>
       <c r="K1156" s="13" t="n">
-        <v>3780</v>
+        <v>3920</v>
       </c>
       <c r="L1156" s="32" t="n">
         <v>0</v>
@@ -58668,26 +58672,26 @@
         </is>
       </c>
       <c r="D1157" s="15" t="n">
-        <v>131304.81</v>
+        <v>131959.37</v>
       </c>
       <c r="E1157" s="15" t="n">
-        <v>113575.54</v>
+        <v>113710.5</v>
       </c>
       <c r="F1157" s="16" t="n">
-        <v>0.4676</v>
+        <v>0.4629</v>
       </c>
       <c r="G1157" s="16" t="n">
-        <v>0.4086</v>
+        <v>0.404</v>
       </c>
       <c r="H1157" s="16" t="n"/>
       <c r="I1157" s="16" t="n">
-        <v>0.1017</v>
+        <v>0.1065</v>
       </c>
       <c r="J1157" s="19" t="n">
-        <v>1367</v>
+        <v>1418</v>
       </c>
       <c r="K1157" s="19" t="n">
-        <v>4373</v>
+        <v>4426</v>
       </c>
       <c r="L1157" s="31" t="n">
         <v>0</v>
@@ -58710,26 +58714,26 @@
         </is>
       </c>
       <c r="D1158" s="9" t="n">
-        <v>19408.91</v>
+        <v>19785.36</v>
       </c>
       <c r="E1158" s="9" t="n">
-        <v>56400.6</v>
+        <v>56586.86</v>
       </c>
       <c r="F1158" s="10" t="n">
-        <v>0.5647</v>
+        <v>0.4445</v>
       </c>
       <c r="G1158" s="10" t="n">
-        <v>0.4939</v>
+        <v>0.3739</v>
       </c>
       <c r="H1158" s="10" t="n"/>
       <c r="I1158" s="10" t="n">
-        <v>0.0428</v>
+        <v>0.0519</v>
       </c>
       <c r="J1158" s="13" t="n">
-        <v>887</v>
+        <v>924</v>
       </c>
       <c r="K1158" s="13" t="n">
-        <v>1168</v>
+        <v>1218</v>
       </c>
       <c r="L1158" s="32" t="n">
         <v>0</v>
@@ -58752,26 +58756,26 @@
         </is>
       </c>
       <c r="D1159" s="15" t="n">
-        <v>14030.8</v>
+        <v>14721.92</v>
       </c>
       <c r="E1159" s="15" t="n">
-        <v>17060.46</v>
+        <v>17102.7</v>
       </c>
       <c r="F1159" s="16" t="n">
-        <v>0.9079</v>
+        <v>0.8147</v>
       </c>
       <c r="G1159" s="16" t="n">
-        <v>0.8411999999999999</v>
+        <v>0.748</v>
       </c>
       <c r="H1159" s="16" t="n"/>
       <c r="I1159" s="16" t="n">
-        <v>0.0179</v>
+        <v>0.0235</v>
       </c>
       <c r="J1159" s="19" t="n">
-        <v>615</v>
+        <v>637</v>
       </c>
       <c r="K1159" s="19" t="n">
-        <v>846</v>
+        <v>880</v>
       </c>
       <c r="L1159" s="31" t="n">
         <v>0</v>
@@ -58794,26 +58798,26 @@
         </is>
       </c>
       <c r="D1160" s="9" t="n">
-        <v>15939.63</v>
+        <v>16118.25</v>
       </c>
       <c r="E1160" s="9" t="n">
-        <v>40956.02</v>
+        <v>41377.33</v>
       </c>
       <c r="F1160" s="10" t="n">
-        <v>0.7713</v>
+        <v>0.7606000000000001</v>
       </c>
       <c r="G1160" s="10" t="n">
-        <v>0.7065</v>
+        <v>0.6954</v>
       </c>
       <c r="H1160" s="10" t="n"/>
       <c r="I1160" s="10" t="n">
-        <v>0.0197</v>
+        <v>0.022</v>
       </c>
       <c r="J1160" s="13" t="n">
-        <v>1017</v>
+        <v>1047</v>
       </c>
       <c r="K1160" s="13" t="n">
-        <v>1367</v>
+        <v>1398</v>
       </c>
       <c r="L1160" s="32" t="n">
         <v>0</v>
@@ -58836,26 +58840,26 @@
         </is>
       </c>
       <c r="D1161" s="15" t="n">
-        <v>5253.86</v>
+        <v>5392.27</v>
       </c>
       <c r="E1161" s="15" t="n">
-        <v>7541.1</v>
+        <v>9204.34</v>
       </c>
       <c r="F1161" s="16" t="n">
-        <v>0.8744</v>
+        <v>0.8774</v>
       </c>
       <c r="G1161" s="16" t="n">
-        <v>0.8075</v>
+        <v>0.8104</v>
       </c>
       <c r="H1161" s="16" t="n"/>
       <c r="I1161" s="16" t="n">
-        <v>0.0233</v>
+        <v>0.024</v>
       </c>
       <c r="J1161" s="19" t="n">
-        <v>559</v>
+        <v>584</v>
       </c>
       <c r="K1161" s="19" t="n">
-        <v>710</v>
+        <v>736</v>
       </c>
       <c r="L1161" s="31" t="n">
         <v>0</v>
@@ -59382,26 +59386,26 @@
         </is>
       </c>
       <c r="D1174" s="9" t="n">
-        <v>175252539.5</v>
+        <v>175384057.38</v>
       </c>
       <c r="E1174" s="9" t="n">
-        <v>770228291.42</v>
+        <v>770270375.92</v>
       </c>
       <c r="F1174" s="10" t="n">
-        <v>0.1453</v>
+        <v>0.1445</v>
       </c>
       <c r="G1174" s="10" t="n">
-        <v>0.08649999999999999</v>
+        <v>0.0857</v>
       </c>
       <c r="H1174" s="10" t="n"/>
       <c r="I1174" s="10" t="n">
-        <v>0.098</v>
+        <v>0.09810000000000001</v>
       </c>
       <c r="J1174" s="13" t="n">
-        <v>4200121</v>
+        <v>4200989</v>
       </c>
       <c r="K1174" s="13" t="n">
-        <v>8132679</v>
+        <v>8135143</v>
       </c>
       <c r="L1174" s="32" t="n">
         <v>0</v>
@@ -59424,26 +59428,26 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>13879812.87</v>
+        <v>14330317.02</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>61259108.46</v>
+        <v>62000825.03</v>
       </c>
       <c r="F1175" s="16" t="n">
-        <v>0.1001</v>
+        <v>0.0129</v>
       </c>
       <c r="G1175" s="16" t="n">
-        <v>0.0461</v>
+        <v>-0.0414</v>
       </c>
       <c r="H1175" s="16" t="n"/>
       <c r="I1175" s="16" t="n">
-        <v>0.09320000000000001</v>
+        <v>0.1043</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>367860</v>
+        <v>376159</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>701881</v>
+        <v>716742</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -62994,26 +62998,26 @@
         </is>
       </c>
       <c r="D1260" s="9" t="n">
-        <v>21411475.03</v>
+        <v>21415851.66</v>
       </c>
       <c r="E1260" s="9" t="n">
-        <v>387414252.67</v>
+        <v>387438289.48</v>
       </c>
       <c r="F1260" s="10" t="n">
-        <v>0.4393</v>
+        <v>0.4388</v>
       </c>
       <c r="G1260" s="10" t="n">
-        <v>0.359</v>
+        <v>0.3585</v>
       </c>
       <c r="H1260" s="10" t="n"/>
       <c r="I1260" s="10" t="n">
         <v>0.0283</v>
       </c>
       <c r="J1260" s="13" t="n">
-        <v>1575453</v>
+        <v>1575565</v>
       </c>
       <c r="K1260" s="13" t="n">
-        <v>2452803</v>
+        <v>2453731</v>
       </c>
       <c r="L1260" s="32" t="n">
         <v>0</v>
@@ -63036,26 +63040,26 @@
         </is>
       </c>
       <c r="D1261" s="15" t="n">
-        <v>46103396.01</v>
+        <v>46199586</v>
       </c>
       <c r="E1261" s="15" t="n">
-        <v>24144787.24</v>
+        <v>24146336.19</v>
       </c>
       <c r="F1261" s="16" t="n">
-        <v>0.0355</v>
+        <v>0.0338</v>
       </c>
       <c r="G1261" s="16" t="n">
-        <v>-0.0063</v>
+        <v>-0.008</v>
       </c>
       <c r="H1261" s="16" t="n"/>
       <c r="I1261" s="16" t="n">
-        <v>0.3098</v>
+        <v>0.3101</v>
       </c>
       <c r="J1261" s="19" t="n">
-        <v>196940</v>
+        <v>197064</v>
       </c>
       <c r="K1261" s="19" t="n">
-        <v>884593</v>
+        <v>884832</v>
       </c>
       <c r="L1261" s="31" t="n">
         <v>0</v>
@@ -63078,26 +63082,26 @@
         </is>
       </c>
       <c r="D1262" s="9" t="n">
-        <v>29711834.7</v>
+        <v>29720590.67</v>
       </c>
       <c r="E1262" s="9" t="n">
-        <v>30951396.85</v>
+        <v>30953272.04</v>
       </c>
       <c r="F1262" s="10" t="n">
-        <v>0.0467</v>
+        <v>0.0464</v>
       </c>
       <c r="G1262" s="10" t="n">
-        <v>-0.0048</v>
+        <v>-0.0051</v>
       </c>
       <c r="H1262" s="10" t="n"/>
       <c r="I1262" s="10" t="n">
-        <v>0.2368</v>
+        <v>0.237</v>
       </c>
       <c r="J1262" s="13" t="n">
-        <v>294013</v>
+        <v>294137</v>
       </c>
       <c r="K1262" s="13" t="n">
-        <v>778748</v>
+        <v>778971</v>
       </c>
       <c r="L1262" s="32" t="n">
         <v>0</v>
@@ -63120,26 +63124,26 @@
         </is>
       </c>
       <c r="D1263" s="15" t="n">
-        <v>22401808.11</v>
+        <v>22409375.51</v>
       </c>
       <c r="E1263" s="15" t="n">
-        <v>37031435.68</v>
+        <v>37033124.46</v>
       </c>
       <c r="F1263" s="16" t="n">
-        <v>0.0699</v>
+        <v>0.0694</v>
       </c>
       <c r="G1263" s="16" t="n">
-        <v>0.0124</v>
+        <v>0.012</v>
       </c>
       <c r="H1263" s="16" t="n"/>
       <c r="I1263" s="16" t="n">
-        <v>0.1884</v>
+        <v>0.1886</v>
       </c>
       <c r="J1263" s="19" t="n">
-        <v>343022</v>
+        <v>343150</v>
       </c>
       <c r="K1263" s="19" t="n">
-        <v>747861</v>
+        <v>748063</v>
       </c>
       <c r="L1263" s="31" t="n">
         <v>0</v>
@@ -63162,26 +63166,26 @@
         </is>
       </c>
       <c r="D1264" s="9" t="n">
-        <v>15048492.89</v>
+        <v>15054492.07</v>
       </c>
       <c r="E1264" s="9" t="n">
-        <v>40861294.77</v>
+        <v>40863131.74</v>
       </c>
       <c r="F1264" s="10" t="n">
-        <v>0.0842</v>
+        <v>0.0834</v>
       </c>
       <c r="G1264" s="10" t="n">
-        <v>0.0197</v>
+        <v>0.0188</v>
       </c>
       <c r="H1264" s="10" t="n"/>
       <c r="I1264" s="10" t="n">
-        <v>0.1497</v>
+        <v>0.1499</v>
       </c>
       <c r="J1264" s="13" t="n">
-        <v>332642</v>
+        <v>332735</v>
       </c>
       <c r="K1264" s="13" t="n">
-        <v>634081</v>
+        <v>634237</v>
       </c>
       <c r="L1264" s="32" t="n">
         <v>0</v>
@@ -63204,26 +63208,26 @@
         </is>
       </c>
       <c r="D1265" s="15" t="n">
-        <v>21124358.98</v>
+        <v>21131567.97</v>
       </c>
       <c r="E1265" s="15" t="n">
-        <v>93730129.16</v>
+        <v>93737989.83</v>
       </c>
       <c r="F1265" s="16" t="n">
-        <v>0.1842</v>
+        <v>0.1836</v>
       </c>
       <c r="G1265" s="16" t="n">
-        <v>0.1156</v>
+        <v>0.115</v>
       </c>
       <c r="H1265" s="16" t="n"/>
       <c r="I1265" s="16" t="n">
-        <v>0.109</v>
+        <v>0.1092</v>
       </c>
       <c r="J1265" s="19" t="n">
-        <v>644440</v>
+        <v>644621</v>
       </c>
       <c r="K1265" s="19" t="n">
-        <v>1132723</v>
+        <v>1133242</v>
       </c>
       <c r="L1265" s="31" t="n">
         <v>0</v>
@@ -63246,26 +63250,26 @@
         </is>
       </c>
       <c r="D1266" s="9" t="n">
-        <v>19451173.78</v>
+        <v>19452593.49</v>
       </c>
       <c r="E1266" s="9" t="n">
-        <v>156094995.05</v>
+        <v>156098232.18</v>
       </c>
       <c r="F1266" s="10" t="n">
-        <v>0.3245</v>
+        <v>0.3243</v>
       </c>
       <c r="G1266" s="10" t="n">
-        <v>0.2512</v>
+        <v>0.251</v>
       </c>
       <c r="H1266" s="10" t="n"/>
       <c r="I1266" s="10" t="n">
         <v>0.0636</v>
       </c>
       <c r="J1266" s="13" t="n">
-        <v>813611</v>
+        <v>813717</v>
       </c>
       <c r="K1266" s="13" t="n">
-        <v>1501870</v>
+        <v>1502067</v>
       </c>
       <c r="L1266" s="32" t="n">
         <v>0</v>
@@ -63288,26 +63292,26 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>2009383.67</v>
+        <v>2051386.45</v>
       </c>
       <c r="E1267" s="15" t="n">
-        <v>35039198.49</v>
+        <v>35266537.96</v>
       </c>
       <c r="F1267" s="16" t="n">
-        <v>0.4623</v>
+        <v>0.3245</v>
       </c>
       <c r="G1267" s="16" t="n">
-        <v>0.3882</v>
+        <v>0.2499</v>
       </c>
       <c r="H1267" s="16" t="n"/>
       <c r="I1267" s="16" t="n">
-        <v>0.0236</v>
+        <v>0.0282</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>162743</v>
+        <v>164982</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>276160</v>
+        <v>279434</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63330,26 +63334,26 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>4395851.78</v>
+        <v>4490203.27</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>1781437.19</v>
+        <v>1796608.85</v>
       </c>
       <c r="F1268" s="10" t="n">
-        <v>0.0203</v>
+        <v>0.0101</v>
       </c>
       <c r="G1268" s="10" t="n">
-        <v>-0.0157</v>
+        <v>-0.0259</v>
       </c>
       <c r="H1268" s="10" t="n"/>
       <c r="I1268" s="10" t="n">
-        <v>0.302</v>
+        <v>0.3104</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>16141</v>
+        <v>16523</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>65576</v>
+        <v>66441</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63372,26 +63376,26 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>2109995.51</v>
+        <v>2209056.75</v>
       </c>
       <c r="E1269" s="15" t="n">
-        <v>1810514.38</v>
+        <v>1866943.24</v>
       </c>
       <c r="F1269" s="16" t="n">
-        <v>0.0449</v>
+        <v>-0.0148</v>
       </c>
       <c r="G1269" s="16" t="n">
-        <v>-0.005</v>
+        <v>-0.0648</v>
       </c>
       <c r="H1269" s="16" t="n"/>
       <c r="I1269" s="16" t="n">
-        <v>0.2457</v>
+        <v>0.2579</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>23097</v>
+        <v>23736</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>56915</v>
+        <v>58721</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63414,26 +63418,26 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>1521131.26</v>
+        <v>1586344.51</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>2389107.02</v>
+        <v>2508367.86</v>
       </c>
       <c r="F1270" s="10" t="n">
-        <v>0.0313</v>
+        <v>-0.0426</v>
       </c>
       <c r="G1270" s="10" t="n">
-        <v>-0.0257</v>
+        <v>-0.0999</v>
       </c>
       <c r="H1270" s="10" t="n"/>
       <c r="I1270" s="10" t="n">
-        <v>0.201</v>
+        <v>0.218</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>25990</v>
+        <v>26838</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>50707</v>
+        <v>52680</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63456,26 +63460,26 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>965471.36</v>
+        <v>1015132.99</v>
       </c>
       <c r="E1271" s="15" t="n">
-        <v>2282222.09</v>
+        <v>2332279.58</v>
       </c>
       <c r="F1271" s="16" t="n">
-        <v>-0.0468</v>
+        <v>-0.178</v>
       </c>
       <c r="G1271" s="16" t="n">
-        <v>-0.1076</v>
+        <v>-0.2391</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
-        <v>0.1647</v>
+        <v>0.1832</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>25401</v>
+        <v>26305</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>42325</v>
+        <v>44217</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63498,26 +63502,26 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>1379294.2</v>
+        <v>1444363.28</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>5445208.45</v>
+        <v>5565420.19</v>
       </c>
       <c r="F1272" s="10" t="n">
-        <v>0.012</v>
+        <v>-0.1555</v>
       </c>
       <c r="G1272" s="10" t="n">
-        <v>-0.0546</v>
+        <v>-0.2227</v>
       </c>
       <c r="H1272" s="10" t="n"/>
       <c r="I1272" s="10" t="n">
-        <v>0.1208</v>
+        <v>0.1399</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>49306</v>
+        <v>51023</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>80594</v>
+        <v>83371</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63540,26 +63544,26 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>1498685.09</v>
+        <v>1533829.78</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>12511420.84</v>
+        <v>12664667.34</v>
       </c>
       <c r="F1273" s="16" t="n">
-        <v>0.1715</v>
+        <v>-0.0132</v>
       </c>
       <c r="G1273" s="16" t="n">
-        <v>0.1048</v>
+        <v>-0.0805</v>
       </c>
       <c r="H1273" s="16" t="n"/>
       <c r="I1273" s="16" t="n">
-        <v>0.0693</v>
+        <v>0.0824</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>65182</v>
+        <v>66752</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>129604</v>
+        <v>131878</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -64086,26 +64090,26 @@
         </is>
       </c>
       <c r="D1286" s="9" t="n">
-        <v>56720.67</v>
+        <v>60762.19</v>
       </c>
       <c r="E1286" s="9" t="n">
-        <v>188633.95</v>
+        <v>197146.71</v>
       </c>
       <c r="F1286" s="10" t="n">
-        <v>0.714</v>
+        <v>0.5455</v>
       </c>
       <c r="G1286" s="10" t="n">
-        <v>0.6482</v>
+        <v>0.4763</v>
       </c>
       <c r="H1286" s="10" t="n"/>
       <c r="I1286" s="10" t="n">
-        <v>0.0132</v>
+        <v>0.0259</v>
       </c>
       <c r="J1286" s="13" t="n">
-        <v>2721</v>
+        <v>2816</v>
       </c>
       <c r="K1286" s="13" t="n">
-        <v>3210</v>
+        <v>3329</v>
       </c>
       <c r="L1286" s="32" t="n">
         <v>0</v>
@@ -67656,26 +67660,26 @@
         </is>
       </c>
       <c r="D1371" s="15" t="n">
-        <v>14558.78</v>
+        <v>14613.5</v>
       </c>
       <c r="E1371" s="15" t="n">
-        <v>121362.39</v>
+        <v>122019.12</v>
       </c>
       <c r="F1371" s="16" t="n">
-        <v>0.9434</v>
+        <v>0.9053</v>
       </c>
       <c r="G1371" s="16" t="n">
-        <v>0.8687</v>
+        <v>0.8302</v>
       </c>
       <c r="H1371" s="16" t="n"/>
       <c r="I1371" s="16" t="n">
-        <v>0.0007</v>
+        <v>0.002</v>
       </c>
       <c r="J1371" s="19" t="n">
-        <v>1532</v>
+        <v>1538</v>
       </c>
       <c r="K1371" s="19" t="n">
-        <v>1833</v>
+        <v>1840</v>
       </c>
       <c r="L1371" s="31" t="n">
         <v>0</v>
@@ -67698,26 +67702,26 @@
         </is>
       </c>
       <c r="D1372" s="9" t="n">
-        <v>13118.47</v>
+        <v>14147.5</v>
       </c>
       <c r="E1372" s="9" t="n">
-        <v>9817.07</v>
+        <v>9973.35</v>
       </c>
       <c r="F1372" s="10" t="n">
-        <v>0.5326</v>
+        <v>0.4777</v>
       </c>
       <c r="G1372" s="10" t="n">
-        <v>0.4755</v>
+        <v>0.421</v>
       </c>
       <c r="H1372" s="10" t="n"/>
       <c r="I1372" s="10" t="n">
-        <v>0.065</v>
+        <v>0.131</v>
       </c>
       <c r="J1372" s="13" t="n">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="K1372" s="13" t="n">
-        <v>188</v>
+        <v>216</v>
       </c>
       <c r="L1372" s="32" t="n">
         <v>0</v>
@@ -67740,26 +67744,26 @@
         </is>
       </c>
       <c r="D1373" s="15" t="n">
-        <v>4123.12</v>
+        <v>4904.21</v>
       </c>
       <c r="E1373" s="15" t="n">
-        <v>12691.16</v>
+        <v>14348.4</v>
       </c>
       <c r="F1373" s="16" t="n">
-        <v>0.4596</v>
+        <v>0.3593</v>
       </c>
       <c r="G1373" s="16" t="n">
-        <v>0.3796</v>
+        <v>0.2757</v>
       </c>
       <c r="H1373" s="16" t="n"/>
       <c r="I1373" s="16" t="n">
-        <v>0.0609</v>
+        <v>0.1203</v>
       </c>
       <c r="J1373" s="19" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="K1373" s="19" t="n">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="L1373" s="31" t="n">
         <v>0</v>
@@ -67782,26 +67786,26 @@
         </is>
       </c>
       <c r="D1374" s="9" t="n">
-        <v>3217.37</v>
+        <v>3472.59</v>
       </c>
       <c r="E1374" s="9" t="n">
-        <v>3115.85</v>
+        <v>3681.65</v>
       </c>
       <c r="F1374" s="10" t="n">
-        <v>0.9</v>
+        <v>0.866</v>
       </c>
       <c r="G1374" s="10" t="n">
-        <v>0.835</v>
+        <v>0.7985</v>
       </c>
       <c r="H1374" s="10" t="n"/>
       <c r="I1374" s="10" t="n">
-        <v>0.0473</v>
+        <v>0.0494</v>
       </c>
       <c r="J1374" s="13" t="n">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="K1374" s="13" t="n">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="L1374" s="32" t="n">
         <v>0</v>
@@ -67824,26 +67828,26 @@
         </is>
       </c>
       <c r="D1375" s="15" t="n">
-        <v>9007.65</v>
+        <v>10310.05</v>
       </c>
       <c r="E1375" s="15" t="n">
-        <v>9371.01</v>
+        <v>13666.38</v>
       </c>
       <c r="F1375" s="16" t="n">
-        <v>0.9512</v>
+        <v>0.2874</v>
       </c>
       <c r="G1375" s="16" t="n">
-        <v>0.8938</v>
+        <v>0.2131</v>
       </c>
       <c r="H1375" s="16" t="n"/>
       <c r="I1375" s="16" t="n">
-        <v>0.0464</v>
+        <v>0.0679</v>
       </c>
       <c r="J1375" s="19" t="n">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="K1375" s="19" t="n">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="L1375" s="31" t="n">
         <v>0</v>
@@ -67866,26 +67870,26 @@
         </is>
       </c>
       <c r="D1376" s="9" t="n">
-        <v>7200.44</v>
+        <v>7785.6</v>
       </c>
       <c r="E1376" s="9" t="n">
-        <v>7374.27</v>
+        <v>8274.549999999999</v>
       </c>
       <c r="F1376" s="10" t="n">
-        <v>0.1912</v>
+        <v>0.0823</v>
       </c>
       <c r="G1376" s="10" t="n">
-        <v>0.1292</v>
+        <v>0.0191</v>
       </c>
       <c r="H1376" s="10" t="n"/>
       <c r="I1376" s="10" t="n">
-        <v>0.0185</v>
+        <v>0.0351</v>
       </c>
       <c r="J1376" s="13" t="n">
-        <v>325</v>
+        <v>342</v>
       </c>
       <c r="K1376" s="13" t="n">
-        <v>360</v>
+        <v>381</v>
       </c>
       <c r="L1376" s="32" t="n">
         <v>0</v>
@@ -67908,26 +67912,26 @@
         </is>
       </c>
       <c r="D1377" s="15" t="n">
-        <v>5494.84</v>
+        <v>5528.74</v>
       </c>
       <c r="E1377" s="15" t="n">
-        <v>24902.18</v>
+        <v>25183.26</v>
       </c>
       <c r="F1377" s="16" t="n">
-        <v>0.9177999999999999</v>
+        <v>0.8656</v>
       </c>
       <c r="G1377" s="16" t="n">
-        <v>0.8458</v>
+        <v>0.7921</v>
       </c>
       <c r="H1377" s="16" t="n"/>
       <c r="I1377" s="16" t="n">
-        <v>0</v>
+        <v>0.012</v>
       </c>
       <c r="J1377" s="19" t="n">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="K1377" s="19" t="n">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="L1377" s="31" t="n">
         <v>0</v>
@@ -68747,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-27 16:42 UTC</t>
+          <t>2026-10-28 14:47 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-28 16:13 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -6019,13 +6019,13 @@
         <v>0.05772</v>
       </c>
       <c r="E71" s="15" t="n">
-        <v>23752659.5</v>
+        <v>51158805.46</v>
       </c>
       <c r="F71" s="15" t="n">
-        <v>5029166.96</v>
+        <v>7539875.03</v>
       </c>
       <c r="G71" s="16" t="n">
-        <v>0.21173</v>
+        <v>0.14738</v>
       </c>
       <c r="H71" s="17" t="inlineStr">
         <is>
@@ -6033,13 +6033,13 @@
         </is>
       </c>
       <c r="I71" s="15" t="n">
-        <v>219529620.32</v>
+        <v>246935766.29</v>
       </c>
       <c r="J71" s="15" t="n">
-        <v>16329931.35</v>
+        <v>18840639.43</v>
       </c>
       <c r="K71" s="18" t="n">
-        <v>0.07439</v>
+        <v>0.07630000000000001</v>
       </c>
       <c r="L71" s="19" t="n">
         <v>32</v>
@@ -7478,13 +7478,13 @@
         <v>0.02883</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>935177546.49</v>
+        <v>962458191.3200001</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>176329463.26</v>
+        <v>178726710.71</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.18855</v>
+        <v>0.1857</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
@@ -7492,13 +7492,13 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>4335579494.57</v>
+        <v>4362860139.39</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>274361430.7</v>
+        <v>276758678.14</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.06328</v>
+        <v>0.06344</v>
       </c>
       <c r="L20" s="13" t="n">
         <v>876</v>
@@ -8116,10 +8116,10 @@
         <v>5.2</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>9142841.539999999</v>
+        <v>14901097.86</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>-0.0645</v>
+        <v>-0.09429999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -8647,7 +8647,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-28 14:47 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-28 16:13 UTC.</t>
         </is>
       </c>
     </row>
@@ -10224,26 +10224,26 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>577669.83</v>
+        <v>3384519.55</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>440259.2</v>
+        <v>4455000.07</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>0.5921999999999999</v>
+        <v>0.2516</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>0.5357</v>
+        <v>0.1954</v>
       </c>
       <c r="H15" s="16" t="n"/>
       <c r="I15" s="16" t="n">
-        <v>0.0571</v>
+        <v>0.07920000000000001</v>
       </c>
       <c r="J15" s="19" t="n">
-        <v>13959</v>
+        <v>63872</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>20074</v>
+        <v>98756</v>
       </c>
       <c r="L15" s="31" t="n">
         <v>0</v>
@@ -13206,26 +13206,26 @@
         </is>
       </c>
       <c r="D86" s="9" t="n">
-        <v>40604.68</v>
+        <v>228934.05</v>
       </c>
       <c r="E86" s="9" t="n">
-        <v>144830.03</v>
+        <v>1050327.49</v>
       </c>
       <c r="F86" s="10" t="n">
-        <v>0.8921</v>
+        <v>0.379</v>
       </c>
       <c r="G86" s="10" t="n">
-        <v>0.8241000000000001</v>
+        <v>0.3142</v>
       </c>
       <c r="H86" s="10" t="n"/>
       <c r="I86" s="10" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0252</v>
       </c>
       <c r="J86" s="13" t="n">
-        <v>3025</v>
+        <v>15881</v>
       </c>
       <c r="K86" s="13" t="n">
-        <v>4534</v>
+        <v>22101</v>
       </c>
       <c r="L86" s="32" t="n">
         <v>0</v>
@@ -13248,26 +13248,26 @@
         </is>
       </c>
       <c r="D87" s="15" t="n">
-        <v>179401.39</v>
+        <v>1030476.39</v>
       </c>
       <c r="E87" s="15" t="n">
-        <v>52270.17</v>
+        <v>685888.86</v>
       </c>
       <c r="F87" s="16" t="n">
-        <v>0.5195</v>
+        <v>0.2599</v>
       </c>
       <c r="G87" s="16" t="n">
-        <v>0.4709</v>
+        <v>0.2096</v>
       </c>
       <c r="H87" s="16" t="n"/>
       <c r="I87" s="16" t="n">
-        <v>0.2925</v>
+        <v>0.2973</v>
       </c>
       <c r="J87" s="19" t="n">
-        <v>923</v>
+        <v>3636</v>
       </c>
       <c r="K87" s="19" t="n">
-        <v>2421</v>
+        <v>12542</v>
       </c>
       <c r="L87" s="31" t="n">
         <v>0</v>
@@ -13290,26 +13290,26 @@
         </is>
       </c>
       <c r="D88" s="9" t="n">
-        <v>106461</v>
+        <v>673906.62</v>
       </c>
       <c r="E88" s="9" t="n">
-        <v>30229.34</v>
+        <v>323939.15</v>
       </c>
       <c r="F88" s="10" t="n">
-        <v>0.5422</v>
+        <v>0.2298</v>
       </c>
       <c r="G88" s="10" t="n">
-        <v>0.4881</v>
+        <v>0.1781</v>
       </c>
       <c r="H88" s="10" t="n"/>
       <c r="I88" s="10" t="n">
-        <v>0.1337</v>
+        <v>0.1725</v>
       </c>
       <c r="J88" s="13" t="n">
-        <v>1601</v>
+        <v>6904</v>
       </c>
       <c r="K88" s="13" t="n">
-        <v>2411</v>
+        <v>12745</v>
       </c>
       <c r="L88" s="32" t="n">
         <v>0</v>
@@ -13332,26 +13332,26 @@
         </is>
       </c>
       <c r="D89" s="15" t="n">
-        <v>80167.35000000001</v>
+        <v>538952.58</v>
       </c>
       <c r="E89" s="15" t="n">
-        <v>51030.37</v>
+        <v>883222.1899999999</v>
       </c>
       <c r="F89" s="16" t="n">
-        <v>0.5256999999999999</v>
+        <v>-0.0495</v>
       </c>
       <c r="G89" s="16" t="n">
-        <v>0.4661</v>
+        <v>-0.1079</v>
       </c>
       <c r="H89" s="16" t="n"/>
       <c r="I89" s="16" t="n">
-        <v>0.0699</v>
+        <v>0.1136</v>
       </c>
       <c r="J89" s="19" t="n">
-        <v>1632</v>
+        <v>7516</v>
       </c>
       <c r="K89" s="19" t="n">
-        <v>2133</v>
+        <v>11573</v>
       </c>
       <c r="L89" s="31" t="n">
         <v>0</v>
@@ -13374,26 +13374,26 @@
         </is>
       </c>
       <c r="D90" s="9" t="n">
-        <v>47941.32</v>
+        <v>329735.87</v>
       </c>
       <c r="E90" s="9" t="n">
-        <v>27253.07</v>
+        <v>353294.7</v>
       </c>
       <c r="F90" s="10" t="n">
-        <v>0.7547</v>
+        <v>0.2583</v>
       </c>
       <c r="G90" s="10" t="n">
-        <v>0.6946</v>
+        <v>0.1963</v>
       </c>
       <c r="H90" s="10" t="n"/>
       <c r="I90" s="10" t="n">
-        <v>0.0505</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="J90" s="13" t="n">
-        <v>1446</v>
+        <v>6896</v>
       </c>
       <c r="K90" s="13" t="n">
-        <v>1779</v>
+        <v>10581</v>
       </c>
       <c r="L90" s="32" t="n">
         <v>0</v>
@@ -13416,26 +13416,26 @@
         </is>
       </c>
       <c r="D91" s="15" t="n">
-        <v>76937.06</v>
+        <v>355382.2</v>
       </c>
       <c r="E91" s="15" t="n">
-        <v>61916.86</v>
+        <v>479145.76</v>
       </c>
       <c r="F91" s="16" t="n">
-        <v>0.4688</v>
+        <v>0.4163</v>
       </c>
       <c r="G91" s="16" t="n">
-        <v>0.4079</v>
+        <v>0.3553</v>
       </c>
       <c r="H91" s="16" t="n"/>
       <c r="I91" s="16" t="n">
-        <v>0.0255</v>
+        <v>0.0491</v>
       </c>
       <c r="J91" s="19" t="n">
-        <v>2584</v>
+        <v>11771</v>
       </c>
       <c r="K91" s="19" t="n">
-        <v>3244</v>
+        <v>15177</v>
       </c>
       <c r="L91" s="31" t="n">
         <v>0</v>
@@ -13458,26 +13458,26 @@
         </is>
       </c>
       <c r="D92" s="9" t="n">
-        <v>46157.04</v>
+        <v>227131.85</v>
       </c>
       <c r="E92" s="9" t="n">
-        <v>72729.35000000001</v>
+        <v>679181.9300000001</v>
       </c>
       <c r="F92" s="10" t="n">
-        <v>0.879</v>
+        <v>0.5968</v>
       </c>
       <c r="G92" s="10" t="n">
-        <v>0.8128</v>
+        <v>0.5305</v>
       </c>
       <c r="H92" s="10" t="n"/>
       <c r="I92" s="10" t="n">
-        <v>0.0109</v>
+        <v>0.0292</v>
       </c>
       <c r="J92" s="13" t="n">
-        <v>2748</v>
+        <v>11268</v>
       </c>
       <c r="K92" s="13" t="n">
-        <v>3552</v>
+        <v>14037</v>
       </c>
       <c r="L92" s="32" t="n">
         <v>0</v>
@@ -14886,26 +14886,26 @@
         </is>
       </c>
       <c r="D126" s="9" t="n">
-        <v>382866.83</v>
+        <v>977439.04</v>
       </c>
       <c r="E126" s="9" t="n">
-        <v>1919082.81</v>
+        <v>1986991.04</v>
       </c>
       <c r="F126" s="10" t="n">
-        <v>0.8921</v>
+        <v>0.509</v>
       </c>
       <c r="G126" s="10" t="n">
-        <v>0.8258</v>
+        <v>0.4564</v>
       </c>
       <c r="H126" s="10" t="n"/>
       <c r="I126" s="10" t="n">
-        <v>0.0064</v>
+        <v>0.0379</v>
       </c>
       <c r="J126" s="13" t="n">
-        <v>18246</v>
+        <v>23254</v>
       </c>
       <c r="K126" s="13" t="n">
-        <v>40265</v>
+        <v>52318</v>
       </c>
       <c r="L126" s="32" t="n">
         <v>0</v>
@@ -17364,26 +17364,26 @@
         </is>
       </c>
       <c r="D185" s="15" t="n">
-        <v>134949.67</v>
+        <v>139897.04</v>
       </c>
       <c r="E185" s="15" t="n">
         <v>637964.03</v>
       </c>
       <c r="F185" s="16" t="n">
-        <v>1.0159</v>
+        <v>1.0178</v>
       </c>
       <c r="G185" s="16" t="n">
-        <v>0.9445</v>
+        <v>0.9464</v>
       </c>
       <c r="H185" s="16" t="n"/>
       <c r="I185" s="16" t="n">
         <v>0.0003</v>
       </c>
       <c r="J185" s="19" t="n">
-        <v>9614</v>
+        <v>10011</v>
       </c>
       <c r="K185" s="19" t="n">
-        <v>21895</v>
+        <v>22444</v>
       </c>
       <c r="L185" s="31" t="n">
         <v>0</v>
@@ -17406,26 +17406,26 @@
         </is>
       </c>
       <c r="D186" s="9" t="n">
-        <v>26299.84</v>
+        <v>482276.1</v>
       </c>
       <c r="E186" s="9" t="n">
-        <v>7905.07</v>
+        <v>42284.94</v>
       </c>
       <c r="F186" s="10" t="n">
-        <v>0.2109</v>
+        <v>0.2265</v>
       </c>
       <c r="G186" s="10" t="n">
-        <v>0.1643</v>
+        <v>0.1852</v>
       </c>
       <c r="H186" s="10" t="n"/>
       <c r="I186" s="10" t="n">
-        <v>0.1037</v>
+        <v>0.2377</v>
       </c>
       <c r="J186" s="13" t="n">
-        <v>492</v>
+        <v>2179</v>
       </c>
       <c r="K186" s="13" t="n">
-        <v>784</v>
+        <v>8047</v>
       </c>
       <c r="L186" s="32" t="n">
         <v>0</v>
@@ -17448,26 +17448,26 @@
         </is>
       </c>
       <c r="D187" s="15" t="n">
-        <v>31999.82</v>
+        <v>91189.94</v>
       </c>
       <c r="E187" s="15" t="n">
-        <v>18065.21</v>
+        <v>36808.52</v>
       </c>
       <c r="F187" s="16" t="n">
-        <v>0.9594</v>
+        <v>0.47</v>
       </c>
       <c r="G187" s="16" t="n">
-        <v>0.9096</v>
+        <v>0.4217</v>
       </c>
       <c r="H187" s="16" t="n"/>
       <c r="I187" s="16" t="n">
-        <v>0.0185</v>
+        <v>0.0992</v>
       </c>
       <c r="J187" s="19" t="n">
-        <v>813</v>
+        <v>1724</v>
       </c>
       <c r="K187" s="19" t="n">
-        <v>1027</v>
+        <v>2451</v>
       </c>
       <c r="L187" s="31" t="n">
         <v>0</v>
@@ -17490,26 +17490,26 @@
         </is>
       </c>
       <c r="D188" s="9" t="n">
-        <v>35185.84</v>
+        <v>77614.25</v>
       </c>
       <c r="E188" s="9" t="n">
-        <v>41544.1</v>
+        <v>51545.5</v>
       </c>
       <c r="F188" s="10" t="n">
-        <v>0.7702</v>
+        <v>0.4579</v>
       </c>
       <c r="G188" s="10" t="n">
-        <v>0.7068</v>
+        <v>0.3993</v>
       </c>
       <c r="H188" s="10" t="n"/>
       <c r="I188" s="10" t="n">
-        <v>0.0139</v>
+        <v>0.0572</v>
       </c>
       <c r="J188" s="13" t="n">
-        <v>1153</v>
+        <v>2272</v>
       </c>
       <c r="K188" s="13" t="n">
-        <v>1379</v>
+        <v>3025</v>
       </c>
       <c r="L188" s="32" t="n">
         <v>0</v>
@@ -17532,26 +17532,26 @@
         </is>
       </c>
       <c r="D189" s="15" t="n">
-        <v>30484.5</v>
+        <v>47610.16</v>
       </c>
       <c r="E189" s="15" t="n">
-        <v>46385.28</v>
+        <v>49136.52</v>
       </c>
       <c r="F189" s="16" t="n">
-        <v>0.8103</v>
+        <v>0.82</v>
       </c>
       <c r="G189" s="16" t="n">
-        <v>0.7413999999999999</v>
+        <v>0.7556</v>
       </c>
       <c r="H189" s="16" t="n"/>
       <c r="I189" s="16" t="n">
-        <v>0.0102</v>
+        <v>0.0175</v>
       </c>
       <c r="J189" s="19" t="n">
-        <v>1175</v>
+        <v>1428</v>
       </c>
       <c r="K189" s="19" t="n">
-        <v>1727</v>
+        <v>2044</v>
       </c>
       <c r="L189" s="31" t="n">
         <v>0</v>
@@ -17574,26 +17574,26 @@
         </is>
       </c>
       <c r="D190" s="9" t="n">
-        <v>51401.9</v>
+        <v>62444.56</v>
       </c>
       <c r="E190" s="9" t="n">
-        <v>192499.26</v>
+        <v>193835.69</v>
       </c>
       <c r="F190" s="10" t="n">
-        <v>0.8852</v>
+        <v>0.8611</v>
       </c>
       <c r="G190" s="10" t="n">
-        <v>0.8152</v>
+        <v>0.7939000000000001</v>
       </c>
       <c r="H190" s="10" t="n"/>
       <c r="I190" s="10" t="n">
-        <v>0.0056</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="J190" s="13" t="n">
-        <v>2684</v>
+        <v>3111</v>
       </c>
       <c r="K190" s="13" t="n">
-        <v>3572</v>
+        <v>4113</v>
       </c>
       <c r="L190" s="32" t="n">
         <v>0</v>
@@ -17616,26 +17616,26 @@
         </is>
       </c>
       <c r="D191" s="15" t="n">
-        <v>72545.25999999999</v>
+        <v>76406.99000000001</v>
       </c>
       <c r="E191" s="15" t="n">
-        <v>974719.86</v>
+        <v>975415.85</v>
       </c>
       <c r="F191" s="16" t="n">
-        <v>0.9775</v>
+        <v>0.9772</v>
       </c>
       <c r="G191" s="16" t="n">
-        <v>0.9087</v>
+        <v>0.9086</v>
       </c>
       <c r="H191" s="16" t="n"/>
       <c r="I191" s="16" t="n">
-        <v>0.0017</v>
+        <v>0.0024</v>
       </c>
       <c r="J191" s="19" t="n">
-        <v>2315</v>
+        <v>2529</v>
       </c>
       <c r="K191" s="19" t="n">
-        <v>9881</v>
+        <v>10194</v>
       </c>
       <c r="L191" s="31" t="n">
         <v>0</v>
@@ -18162,26 +18162,26 @@
         </is>
       </c>
       <c r="D204" s="9" t="n">
-        <v>950338.08</v>
+        <v>2754817.64</v>
       </c>
       <c r="E204" s="9" t="n">
-        <v>232445</v>
+        <v>3284931.92</v>
       </c>
       <c r="F204" s="10" t="n">
-        <v>0.1406</v>
+        <v>0.4156</v>
       </c>
       <c r="G204" s="10" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.3592</v>
       </c>
       <c r="H204" s="10" t="n"/>
       <c r="I204" s="10" t="n">
-        <v>0.1018</v>
+        <v>0.0819</v>
       </c>
       <c r="J204" s="13" t="n">
-        <v>22519</v>
+        <v>62375</v>
       </c>
       <c r="K204" s="13" t="n">
-        <v>40392</v>
+        <v>129598</v>
       </c>
       <c r="L204" s="32" t="n">
         <v>0</v>
@@ -21732,26 +21732,26 @@
         </is>
       </c>
       <c r="D289" s="15" t="n">
-        <v>16068.95</v>
+        <v>93326.35000000001</v>
       </c>
       <c r="E289" s="15" t="n">
-        <v>1923.97</v>
+        <v>241483.01</v>
       </c>
       <c r="F289" s="16" t="n">
-        <v>0.8183</v>
+        <v>0.4366</v>
       </c>
       <c r="G289" s="16" t="n">
-        <v>0.7532</v>
+        <v>0.4023</v>
       </c>
       <c r="H289" s="16" t="n"/>
       <c r="I289" s="16" t="n">
-        <v>0.0134</v>
+        <v>0.0123</v>
       </c>
       <c r="J289" s="19" t="n">
-        <v>1413</v>
+        <v>3898</v>
       </c>
       <c r="K289" s="19" t="n">
-        <v>2067</v>
+        <v>5968</v>
       </c>
       <c r="L289" s="31" t="n">
         <v>0</v>
@@ -21774,26 +21774,26 @@
         </is>
       </c>
       <c r="D290" s="9" t="n">
-        <v>359202.85</v>
+        <v>1041133.36</v>
       </c>
       <c r="E290" s="9" t="n">
-        <v>37737.47</v>
+        <v>290888.85</v>
       </c>
       <c r="F290" s="10" t="n">
-        <v>0.1512</v>
+        <v>0.3241</v>
       </c>
       <c r="G290" s="10" t="n">
-        <v>0.1035</v>
+        <v>0.2753</v>
       </c>
       <c r="H290" s="10" t="n"/>
       <c r="I290" s="10" t="n">
-        <v>0.2696</v>
+        <v>0.2297</v>
       </c>
       <c r="J290" s="13" t="n">
-        <v>2322</v>
+        <v>6133</v>
       </c>
       <c r="K290" s="13" t="n">
-        <v>9275</v>
+        <v>26276</v>
       </c>
       <c r="L290" s="32" t="n">
         <v>0</v>
@@ -21816,26 +21816,26 @@
         </is>
       </c>
       <c r="D291" s="15" t="n">
-        <v>166228.2</v>
+        <v>521046.11</v>
       </c>
       <c r="E291" s="15" t="n">
-        <v>35861.65</v>
+        <v>273595.5</v>
       </c>
       <c r="F291" s="16" t="n">
-        <v>-0.3582</v>
+        <v>0.2446</v>
       </c>
       <c r="G291" s="16" t="n">
-        <v>-0.4127</v>
+        <v>0.1885</v>
       </c>
       <c r="H291" s="16" t="n"/>
       <c r="I291" s="16" t="n">
-        <v>0.1946</v>
+        <v>0.158</v>
       </c>
       <c r="J291" s="19" t="n">
-        <v>3413</v>
+        <v>9574</v>
       </c>
       <c r="K291" s="19" t="n">
-        <v>6459</v>
+        <v>21602</v>
       </c>
       <c r="L291" s="31" t="n">
         <v>0</v>
@@ -21858,26 +21858,26 @@
         </is>
       </c>
       <c r="D292" s="9" t="n">
-        <v>173119.37</v>
+        <v>417887.68</v>
       </c>
       <c r="E292" s="9" t="n">
-        <v>84107.82000000001</v>
+        <v>403469.06</v>
       </c>
       <c r="F292" s="10" t="n">
-        <v>-0.019</v>
+        <v>0.3556</v>
       </c>
       <c r="G292" s="10" t="n">
-        <v>-0.076</v>
+        <v>0.2945</v>
       </c>
       <c r="H292" s="10" t="n"/>
       <c r="I292" s="10" t="n">
-        <v>0.136</v>
+        <v>0.1071</v>
       </c>
       <c r="J292" s="13" t="n">
-        <v>3595</v>
+        <v>10280</v>
       </c>
       <c r="K292" s="13" t="n">
-        <v>7446</v>
+        <v>17631</v>
       </c>
       <c r="L292" s="32" t="n">
         <v>0</v>
@@ -21900,26 +21900,26 @@
         </is>
       </c>
       <c r="D293" s="15" t="n">
-        <v>84187.06</v>
+        <v>239799.3</v>
       </c>
       <c r="E293" s="15" t="n">
-        <v>26314.81</v>
+        <v>286347.52</v>
       </c>
       <c r="F293" s="16" t="n">
-        <v>0.2809</v>
+        <v>0.6019</v>
       </c>
       <c r="G293" s="16" t="n">
-        <v>0.2182</v>
+        <v>0.5359</v>
       </c>
       <c r="H293" s="16" t="n"/>
       <c r="I293" s="16" t="n">
-        <v>0.0853</v>
+        <v>0.0612</v>
       </c>
       <c r="J293" s="19" t="n">
-        <v>3153</v>
+        <v>9036</v>
       </c>
       <c r="K293" s="19" t="n">
-        <v>4129</v>
+        <v>12493</v>
       </c>
       <c r="L293" s="31" t="n">
         <v>0</v>
@@ -21942,26 +21942,26 @@
         </is>
       </c>
       <c r="D294" s="9" t="n">
-        <v>94884.47</v>
+        <v>252301.08</v>
       </c>
       <c r="E294" s="9" t="n">
-        <v>35096.5</v>
+        <v>629128.87</v>
       </c>
       <c r="F294" s="10" t="n">
-        <v>0.6168</v>
+        <v>0.7124</v>
       </c>
       <c r="G294" s="10" t="n">
-        <v>0.5521</v>
+        <v>0.6432</v>
       </c>
       <c r="H294" s="10" t="n"/>
       <c r="I294" s="10" t="n">
-        <v>0.0396</v>
+        <v>0.0299</v>
       </c>
       <c r="J294" s="13" t="n">
-        <v>4850</v>
+        <v>13514</v>
       </c>
       <c r="K294" s="13" t="n">
-        <v>6407</v>
+        <v>18704</v>
       </c>
       <c r="L294" s="32" t="n">
         <v>0</v>
@@ -21984,26 +21984,26 @@
         </is>
       </c>
       <c r="D295" s="15" t="n">
-        <v>56647.17</v>
+        <v>189323.77</v>
       </c>
       <c r="E295" s="15" t="n">
-        <v>11402.79</v>
+        <v>1160019.12</v>
       </c>
       <c r="F295" s="16" t="n">
-        <v>0.8265</v>
+        <v>0.8794</v>
       </c>
       <c r="G295" s="16" t="n">
-        <v>0.7588</v>
+        <v>0.8094</v>
       </c>
       <c r="H295" s="16" t="n"/>
       <c r="I295" s="16" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="J295" s="19" t="n">
-        <v>3773</v>
+        <v>9940</v>
       </c>
       <c r="K295" s="19" t="n">
-        <v>4609</v>
+        <v>26924</v>
       </c>
       <c r="L295" s="31" t="n">
         <v>0</v>
@@ -22740,26 +22740,26 @@
         </is>
       </c>
       <c r="D313" s="15" t="n">
-        <v>5614853.86</v>
+        <v>16036559.93</v>
       </c>
       <c r="E313" s="15" t="n">
-        <v>3613192.19</v>
+        <v>20607452.17</v>
       </c>
       <c r="F313" s="16" t="n">
-        <v>0.3754</v>
+        <v>0.1201</v>
       </c>
       <c r="G313" s="16" t="n">
-        <v>0.3192</v>
+        <v>0.06519999999999999</v>
       </c>
       <c r="H313" s="16" t="n"/>
       <c r="I313" s="16" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.1355</v>
       </c>
       <c r="J313" s="19" t="n">
-        <v>116756</v>
+        <v>339393</v>
       </c>
       <c r="K313" s="19" t="n">
-        <v>288930</v>
+        <v>754985</v>
       </c>
       <c r="L313" s="31" t="n">
         <v>0</v>
@@ -27612,26 +27612,26 @@
         </is>
       </c>
       <c r="D429" s="15" t="n">
-        <v>520206.49</v>
+        <v>1358257.72</v>
       </c>
       <c r="E429" s="15" t="n">
-        <v>210426.28</v>
+        <v>2889627.21</v>
       </c>
       <c r="F429" s="16" t="n">
-        <v>0.7975</v>
+        <v>-0.4511</v>
       </c>
       <c r="G429" s="16" t="n">
-        <v>0.7317</v>
+        <v>-0.5177</v>
       </c>
       <c r="H429" s="16" t="n"/>
       <c r="I429" s="16" t="n">
-        <v>0.0174</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="J429" s="19" t="n">
-        <v>35336</v>
+        <v>97517</v>
       </c>
       <c r="K429" s="19" t="n">
-        <v>68039</v>
+        <v>174244</v>
       </c>
       <c r="L429" s="31" t="n">
         <v>0</v>
@@ -27654,26 +27654,26 @@
         </is>
       </c>
       <c r="D430" s="9" t="n">
-        <v>2107432.08</v>
+        <v>6341223.32</v>
       </c>
       <c r="E430" s="9" t="n">
-        <v>1011521.52</v>
+        <v>3377528.75</v>
       </c>
       <c r="F430" s="10" t="n">
-        <v>-0.0226</v>
+        <v>0.0286</v>
       </c>
       <c r="G430" s="10" t="n">
-        <v>-0.0752</v>
+        <v>-0.0201</v>
       </c>
       <c r="H430" s="10" t="n"/>
       <c r="I430" s="10" t="n">
-        <v>0.3008</v>
+        <v>0.3092</v>
       </c>
       <c r="J430" s="13" t="n">
-        <v>9274</v>
+        <v>27823</v>
       </c>
       <c r="K430" s="13" t="n">
-        <v>34012</v>
+        <v>106899</v>
       </c>
       <c r="L430" s="32" t="n">
         <v>0</v>
@@ -27696,26 +27696,26 @@
         </is>
       </c>
       <c r="D431" s="15" t="n">
-        <v>912040.27</v>
+        <v>2631797.18</v>
       </c>
       <c r="E431" s="15" t="n">
-        <v>217419.87</v>
+        <v>1964228.9</v>
       </c>
       <c r="F431" s="16" t="n">
-        <v>0.465</v>
+        <v>0.1953</v>
       </c>
       <c r="G431" s="16" t="n">
-        <v>0.4145</v>
+        <v>0.1439</v>
       </c>
       <c r="H431" s="16" t="n"/>
       <c r="I431" s="16" t="n">
-        <v>0.19</v>
+        <v>0.2152</v>
       </c>
       <c r="J431" s="19" t="n">
-        <v>11662</v>
+        <v>35652</v>
       </c>
       <c r="K431" s="19" t="n">
-        <v>25978</v>
+        <v>79581</v>
       </c>
       <c r="L431" s="31" t="n">
         <v>0</v>
@@ -27738,26 +27738,26 @@
         </is>
       </c>
       <c r="D432" s="9" t="n">
-        <v>651727.04</v>
+        <v>2000251.66</v>
       </c>
       <c r="E432" s="9" t="n">
-        <v>156879.23</v>
+        <v>1600113.84</v>
       </c>
       <c r="F432" s="10" t="n">
-        <v>0.6195000000000001</v>
+        <v>0.33</v>
       </c>
       <c r="G432" s="10" t="n">
-        <v>0.5644</v>
+        <v>0.2739</v>
       </c>
       <c r="H432" s="10" t="n"/>
       <c r="I432" s="10" t="n">
-        <v>0.143</v>
+        <v>0.1715</v>
       </c>
       <c r="J432" s="13" t="n">
-        <v>12608</v>
+        <v>41083</v>
       </c>
       <c r="K432" s="13" t="n">
-        <v>25565</v>
+        <v>88141</v>
       </c>
       <c r="L432" s="32" t="n">
         <v>0</v>
@@ -27780,26 +27780,26 @@
         </is>
       </c>
       <c r="D433" s="15" t="n">
-        <v>373580.46</v>
+        <v>1043121.8</v>
       </c>
       <c r="E433" s="15" t="n">
-        <v>212500.3</v>
+        <v>1232339.51</v>
       </c>
       <c r="F433" s="16" t="n">
-        <v>0.6178</v>
+        <v>0.3472</v>
       </c>
       <c r="G433" s="16" t="n">
-        <v>0.5597</v>
+        <v>0.2873</v>
       </c>
       <c r="H433" s="16" t="n"/>
       <c r="I433" s="16" t="n">
-        <v>0.1058</v>
+        <v>0.1476</v>
       </c>
       <c r="J433" s="19" t="n">
-        <v>10419</v>
+        <v>31035</v>
       </c>
       <c r="K433" s="19" t="n">
-        <v>17733</v>
+        <v>51302</v>
       </c>
       <c r="L433" s="31" t="n">
         <v>0</v>
@@ -27822,26 +27822,26 @@
         </is>
       </c>
       <c r="D434" s="9" t="n">
-        <v>521946.32</v>
+        <v>1464923.49</v>
       </c>
       <c r="E434" s="9" t="n">
-        <v>337518.48</v>
+        <v>2763986.32</v>
       </c>
       <c r="F434" s="10" t="n">
-        <v>0.605</v>
+        <v>0.3929</v>
       </c>
       <c r="G434" s="10" t="n">
-        <v>0.5439000000000001</v>
+        <v>0.3296</v>
       </c>
       <c r="H434" s="10" t="n"/>
       <c r="I434" s="10" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.1155</v>
       </c>
       <c r="J434" s="13" t="n">
-        <v>18832</v>
+        <v>53225</v>
       </c>
       <c r="K434" s="13" t="n">
-        <v>35372</v>
+        <v>116908</v>
       </c>
       <c r="L434" s="32" t="n">
         <v>0</v>
@@ -27864,26 +27864,26 @@
         </is>
       </c>
       <c r="D435" s="15" t="n">
-        <v>527921.2</v>
+        <v>1196984.74</v>
       </c>
       <c r="E435" s="15" t="n">
-        <v>1466926.51</v>
+        <v>6779627.65</v>
       </c>
       <c r="F435" s="16" t="n">
-        <v>0.6932</v>
+        <v>0.2058</v>
       </c>
       <c r="G435" s="16" t="n">
-        <v>0.6272</v>
+        <v>0.1395</v>
       </c>
       <c r="H435" s="16" t="n"/>
       <c r="I435" s="16" t="n">
-        <v>0.0506</v>
+        <v>0.0983</v>
       </c>
       <c r="J435" s="19" t="n">
-        <v>18625</v>
+        <v>53058</v>
       </c>
       <c r="K435" s="19" t="n">
-        <v>82231</v>
+        <v>137910</v>
       </c>
       <c r="L435" s="31" t="n">
         <v>0</v>
@@ -29226,31 +29226,31 @@
         </is>
       </c>
       <c r="D466" s="9" t="n">
-        <v>9142841.539999999</v>
+        <v>14901097.86</v>
       </c>
       <c r="E466" s="9" t="n">
-        <v>30542631.86</v>
+        <v>38612880.59</v>
       </c>
       <c r="F466" s="10" t="n">
-        <v>-0.0645</v>
+        <v>-0.09429999999999999</v>
       </c>
       <c r="G466" s="10" t="n">
-        <v>-0.1297</v>
+        <v>-0.1506</v>
       </c>
       <c r="H466" s="10" t="n">
-        <v>0.1583</v>
+        <v>0.1577</v>
       </c>
       <c r="I466" s="10" t="n">
-        <v>0.0907</v>
+        <v>0.1135</v>
       </c>
       <c r="J466" s="13" t="n">
-        <v>281494</v>
+        <v>377462</v>
       </c>
       <c r="K466" s="13" t="n">
-        <v>567178</v>
+        <v>734000</v>
       </c>
       <c r="L466" s="32" t="n">
-        <v>0.8328</v>
+        <v>0.5637</v>
       </c>
     </row>
     <row r="467">
@@ -38414,31 +38414,31 @@
         </is>
       </c>
       <c r="D675" s="15" t="n">
-        <v>1117023</v>
+        <v>1263400.75</v>
       </c>
       <c r="E675" s="15" t="n">
-        <v>14437461.7</v>
+        <v>16092576.5</v>
       </c>
       <c r="F675" s="16" t="n">
-        <v>0.6938</v>
+        <v>0.6099</v>
       </c>
       <c r="G675" s="16" t="n">
-        <v>0.6165</v>
+        <v>0.5352</v>
       </c>
       <c r="H675" s="16" t="n">
-        <v>0.5904</v>
+        <v>0.59</v>
       </c>
       <c r="I675" s="16" t="n">
-        <v>0.0187</v>
+        <v>0.0256</v>
       </c>
       <c r="J675" s="19" t="n">
-        <v>79400</v>
+        <v>88522</v>
       </c>
       <c r="K675" s="19" t="n">
-        <v>167675</v>
+        <v>179212</v>
       </c>
       <c r="L675" s="31" t="n">
-        <v>0.7542</v>
+        <v>0.6815</v>
       </c>
     </row>
     <row r="676">
@@ -38458,31 +38458,31 @@
         </is>
       </c>
       <c r="D676" s="9" t="n">
-        <v>2309706.33</v>
+        <v>4423439.96</v>
       </c>
       <c r="E676" s="9" t="n">
-        <v>1985157.13</v>
+        <v>3416598.36</v>
       </c>
       <c r="F676" s="10" t="n">
-        <v>-0.3326</v>
+        <v>-0.2302</v>
       </c>
       <c r="G676" s="10" t="n">
-        <v>-0.3933</v>
+        <v>-0.2819</v>
       </c>
       <c r="H676" s="10" t="n">
-        <v>0.0621</v>
+        <v>0.068</v>
       </c>
       <c r="I676" s="10" t="n">
-        <v>0.2512</v>
+        <v>0.2619</v>
       </c>
       <c r="J676" s="13" t="n">
-        <v>12410</v>
+        <v>21482</v>
       </c>
       <c r="K676" s="13" t="n">
-        <v>52769</v>
+        <v>92656</v>
       </c>
       <c r="L676" s="32" t="n">
-        <v>0.8638</v>
+        <v>0.5157</v>
       </c>
     </row>
     <row r="677">
@@ -38502,31 +38502,31 @@
         </is>
       </c>
       <c r="D677" s="15" t="n">
-        <v>1287828.33</v>
+        <v>2413989.85</v>
       </c>
       <c r="E677" s="15" t="n">
-        <v>3475973.03</v>
+        <v>4636579.74</v>
       </c>
       <c r="F677" s="16" t="n">
-        <v>-0.4826</v>
+        <v>-0.3412</v>
       </c>
       <c r="G677" s="16" t="n">
-        <v>-0.541</v>
+        <v>-0.3913</v>
       </c>
       <c r="H677" s="16" t="n">
-        <v>0.07480000000000001</v>
+        <v>0.0733</v>
       </c>
       <c r="I677" s="16" t="n">
-        <v>0.2101</v>
+        <v>0.2217</v>
       </c>
       <c r="J677" s="19" t="n">
-        <v>23018</v>
+        <v>38204</v>
       </c>
       <c r="K677" s="19" t="n">
-        <v>55503</v>
+        <v>85547</v>
       </c>
       <c r="L677" s="31" t="n">
-        <v>0.8753</v>
+        <v>0.5235</v>
       </c>
     </row>
     <row r="678">
@@ -38546,31 +38546,31 @@
         </is>
       </c>
       <c r="D678" s="9" t="n">
-        <v>1234183.64</v>
+        <v>2043446.47</v>
       </c>
       <c r="E678" s="9" t="n">
-        <v>1216253.68</v>
+        <v>1815308.29</v>
       </c>
       <c r="F678" s="10" t="n">
-        <v>-0.312</v>
+        <v>-0.2633</v>
       </c>
       <c r="G678" s="10" t="n">
-        <v>-0.3743</v>
+        <v>-0.3173</v>
       </c>
       <c r="H678" s="10" t="n">
-        <v>0.1467</v>
+        <v>0.1434</v>
       </c>
       <c r="I678" s="10" t="n">
-        <v>0.168</v>
+        <v>0.1814</v>
       </c>
       <c r="J678" s="13" t="n">
-        <v>30336</v>
+        <v>46818</v>
       </c>
       <c r="K678" s="13" t="n">
-        <v>52310</v>
+        <v>76563</v>
       </c>
       <c r="L678" s="32" t="n">
-        <v>0.8577</v>
+        <v>0.5703</v>
       </c>
     </row>
     <row r="679">
@@ -38590,31 +38590,31 @@
         </is>
       </c>
       <c r="D679" s="15" t="n">
-        <v>955088.46</v>
+        <v>1500413.95</v>
       </c>
       <c r="E679" s="15" t="n">
-        <v>1087210.59</v>
+        <v>1647044.73</v>
       </c>
       <c r="F679" s="16" t="n">
-        <v>-0.1041</v>
+        <v>-0.1101</v>
       </c>
       <c r="G679" s="16" t="n">
-        <v>-0.1673</v>
+        <v>-0.165</v>
       </c>
       <c r="H679" s="16" t="n">
-        <v>0.1836</v>
+        <v>0.1866</v>
       </c>
       <c r="I679" s="16" t="n">
-        <v>0.1267</v>
+        <v>0.1433</v>
       </c>
       <c r="J679" s="19" t="n">
-        <v>30078</v>
+        <v>43626</v>
       </c>
       <c r="K679" s="19" t="n">
-        <v>48117</v>
+        <v>65498</v>
       </c>
       <c r="L679" s="31" t="n">
-        <v>0.7537</v>
+        <v>0.5366</v>
       </c>
     </row>
     <row r="680">
@@ -38634,31 +38634,31 @@
         </is>
       </c>
       <c r="D680" s="9" t="n">
-        <v>1151331.83</v>
+        <v>1802024.96</v>
       </c>
       <c r="E680" s="9" t="n">
-        <v>3167613.07</v>
+        <v>4401269.39</v>
       </c>
       <c r="F680" s="10" t="n">
-        <v>0.0735</v>
+        <v>-0.015</v>
       </c>
       <c r="G680" s="10" t="n">
-        <v>0.0052</v>
+        <v>-0.074</v>
       </c>
       <c r="H680" s="10" t="n">
-        <v>0.282</v>
+        <v>0.2777</v>
       </c>
       <c r="I680" s="10" t="n">
-        <v>0.0849</v>
+        <v>0.1024</v>
       </c>
       <c r="J680" s="13" t="n">
-        <v>53621</v>
+        <v>72418</v>
       </c>
       <c r="K680" s="13" t="n">
-        <v>71982</v>
+        <v>95118</v>
       </c>
       <c r="L680" s="32" t="n">
-        <v>0.8303</v>
+        <v>0.5818</v>
       </c>
     </row>
     <row r="681">
@@ -38678,31 +38678,31 @@
         </is>
       </c>
       <c r="D681" s="15" t="n">
-        <v>1087679.95</v>
+        <v>1454381.92</v>
       </c>
       <c r="E681" s="15" t="n">
-        <v>5172962.64</v>
+        <v>6603503.57</v>
       </c>
       <c r="F681" s="16" t="n">
-        <v>0.3903</v>
+        <v>0.2729</v>
       </c>
       <c r="G681" s="16" t="n">
-        <v>0.318</v>
+        <v>0.207</v>
       </c>
       <c r="H681" s="16" t="n">
-        <v>0.4484</v>
+        <v>0.438</v>
       </c>
       <c r="I681" s="16" t="n">
-        <v>0.0499</v>
+        <v>0.0648</v>
       </c>
       <c r="J681" s="19" t="n">
-        <v>52631</v>
+        <v>66392</v>
       </c>
       <c r="K681" s="19" t="n">
-        <v>118822</v>
+        <v>139406</v>
       </c>
       <c r="L681" s="31" t="n">
-        <v>0.8409</v>
+        <v>0.6707</v>
       </c>
     </row>
     <row r="682">
@@ -39226,26 +39226,26 @@
         </is>
       </c>
       <c r="D694" s="9" t="n">
-        <v>13563124.8</v>
+        <v>13563307.28</v>
       </c>
       <c r="E694" s="9" t="n">
-        <v>78794857.51000001</v>
+        <v>78801596.06</v>
       </c>
       <c r="F694" s="10" t="n">
-        <v>0.2912</v>
+        <v>0.2913</v>
       </c>
       <c r="G694" s="10" t="n">
-        <v>0.2249</v>
+        <v>0.225</v>
       </c>
       <c r="H694" s="10" t="n"/>
       <c r="I694" s="10" t="n">
         <v>0.06900000000000001</v>
       </c>
       <c r="J694" s="13" t="n">
-        <v>485822</v>
+        <v>485863</v>
       </c>
       <c r="K694" s="13" t="n">
-        <v>669298</v>
+        <v>669343</v>
       </c>
       <c r="L694" s="32" t="n">
         <v>0.5271</v>
@@ -39268,29 +39268,29 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>2325254.86</v>
+        <v>3256603.51</v>
       </c>
       <c r="E695" s="15" t="n">
-        <v>14545221.86</v>
+        <v>24925755.65</v>
       </c>
       <c r="F695" s="16" t="n">
-        <v>0.2543</v>
+        <v>0.1703</v>
       </c>
       <c r="G695" s="16" t="n">
-        <v>0.1878</v>
+        <v>0.102</v>
       </c>
       <c r="H695" s="16" t="n"/>
       <c r="I695" s="16" t="n">
-        <v>0.0419</v>
+        <v>0.0526</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>110450</v>
+        <v>150197</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>147323</v>
+        <v>202457</v>
       </c>
       <c r="L695" s="31" t="n">
-        <v>0.7877</v>
+        <v>0.5823</v>
       </c>
     </row>
     <row r="696">
@@ -42838,13 +42838,13 @@
         </is>
       </c>
       <c r="D780" s="9" t="n">
-        <v>3103435.12</v>
+        <v>3103440.19</v>
       </c>
       <c r="E780" s="9" t="n">
-        <v>49923181.25</v>
+        <v>49927972.85</v>
       </c>
       <c r="F780" s="10" t="n">
-        <v>0.5415</v>
+        <v>0.5414</v>
       </c>
       <c r="G780" s="10" t="n">
         <v>0.4611</v>
@@ -42854,10 +42854,10 @@
         <v>0.0184</v>
       </c>
       <c r="J780" s="13" t="n">
-        <v>250240</v>
+        <v>250253</v>
       </c>
       <c r="K780" s="13" t="n">
-        <v>337791</v>
+        <v>337806</v>
       </c>
       <c r="L780" s="32" t="n">
         <v>0.572</v>
@@ -42922,26 +42922,26 @@
         </is>
       </c>
       <c r="D782" s="9" t="n">
-        <v>1956078.89</v>
+        <v>1956213.9</v>
       </c>
       <c r="E782" s="9" t="n">
-        <v>2022379.17</v>
+        <v>2022852.78</v>
       </c>
       <c r="F782" s="10" t="n">
-        <v>0.1364</v>
+        <v>0.1367</v>
       </c>
       <c r="G782" s="10" t="n">
-        <v>0.0819</v>
+        <v>0.0822</v>
       </c>
       <c r="H782" s="10" t="n"/>
       <c r="I782" s="10" t="n">
-        <v>0.2455</v>
+        <v>0.2456</v>
       </c>
       <c r="J782" s="13" t="n">
-        <v>21007</v>
+        <v>21012</v>
       </c>
       <c r="K782" s="13" t="n">
-        <v>38564</v>
+        <v>38570</v>
       </c>
       <c r="L782" s="32" t="n">
         <v>0.5303</v>
@@ -42967,23 +42967,23 @@
         <v>1551278.28</v>
       </c>
       <c r="E783" s="15" t="n">
-        <v>2905920.09</v>
+        <v>2906922.06</v>
       </c>
       <c r="F783" s="16" t="n">
-        <v>0.1729</v>
+        <v>0.1736</v>
       </c>
       <c r="G783" s="16" t="n">
-        <v>0.1089</v>
+        <v>0.1096</v>
       </c>
       <c r="H783" s="16" t="n"/>
       <c r="I783" s="16" t="n">
-        <v>0.1837</v>
+        <v>0.1838</v>
       </c>
       <c r="J783" s="19" t="n">
-        <v>28057</v>
+        <v>28064</v>
       </c>
       <c r="K783" s="19" t="n">
-        <v>41170</v>
+        <v>41177</v>
       </c>
       <c r="L783" s="31" t="n">
         <v>0.5453</v>
@@ -43006,10 +43006,10 @@
         </is>
       </c>
       <c r="D784" s="9" t="n">
-        <v>1259986.53</v>
+        <v>1259991.25</v>
       </c>
       <c r="E784" s="9" t="n">
-        <v>3415554.13</v>
+        <v>3415680.05</v>
       </c>
       <c r="F784" s="10" t="n">
         <v>0.1871</v>
@@ -43019,13 +43019,13 @@
       </c>
       <c r="H784" s="10" t="n"/>
       <c r="I784" s="10" t="n">
-        <v>0.1444</v>
+        <v>0.1445</v>
       </c>
       <c r="J784" s="13" t="n">
-        <v>30281</v>
+        <v>30284</v>
       </c>
       <c r="K784" s="13" t="n">
-        <v>40875</v>
+        <v>40878</v>
       </c>
       <c r="L784" s="32" t="n">
         <v>0.5073</v>
@@ -43048,26 +43048,26 @@
         </is>
       </c>
       <c r="D785" s="15" t="n">
-        <v>2012842.27</v>
+        <v>2012876.04</v>
       </c>
       <c r="E785" s="15" t="n">
-        <v>7498203.38</v>
+        <v>7498312.67</v>
       </c>
       <c r="F785" s="16" t="n">
         <v>0.1846</v>
       </c>
       <c r="G785" s="16" t="n">
-        <v>0.115</v>
+        <v>0.1149</v>
       </c>
       <c r="H785" s="16" t="n"/>
       <c r="I785" s="16" t="n">
         <v>0.09810000000000001</v>
       </c>
       <c r="J785" s="19" t="n">
-        <v>64314</v>
+        <v>64323</v>
       </c>
       <c r="K785" s="19" t="n">
-        <v>82635</v>
+        <v>82645</v>
       </c>
       <c r="L785" s="31" t="n">
         <v>0.509</v>
@@ -43090,26 +43090,26 @@
         </is>
       </c>
       <c r="D786" s="9" t="n">
-        <v>1762279.2</v>
+        <v>1762283.1</v>
       </c>
       <c r="E786" s="9" t="n">
-        <v>11981479.59</v>
+        <v>11981715.76</v>
       </c>
       <c r="F786" s="10" t="n">
-        <v>0.411</v>
+        <v>0.4109</v>
       </c>
       <c r="G786" s="10" t="n">
-        <v>0.3333</v>
+        <v>0.3332</v>
       </c>
       <c r="H786" s="10" t="n"/>
       <c r="I786" s="10" t="n">
         <v>0.0571</v>
       </c>
       <c r="J786" s="13" t="n">
-        <v>82047</v>
+        <v>82051</v>
       </c>
       <c r="K786" s="13" t="n">
-        <v>102801</v>
+        <v>102805</v>
       </c>
       <c r="L786" s="32" t="n">
         <v>0.5152</v>
@@ -43132,29 +43132,29 @@
         </is>
       </c>
       <c r="D787" s="15" t="n">
-        <v>702518.55</v>
+        <v>892097.1899999999</v>
       </c>
       <c r="E787" s="15" t="n">
-        <v>10661798.39</v>
+        <v>17261663.56</v>
       </c>
       <c r="F787" s="16" t="n">
-        <v>0.6118</v>
+        <v>0.6077</v>
       </c>
       <c r="G787" s="16" t="n">
-        <v>0.5366</v>
+        <v>0.5273</v>
       </c>
       <c r="H787" s="16" t="n"/>
       <c r="I787" s="16" t="n">
-        <v>0.0131</v>
+        <v>0.0167</v>
       </c>
       <c r="J787" s="19" t="n">
-        <v>66711</v>
+        <v>87406</v>
       </c>
       <c r="K787" s="19" t="n">
-        <v>86254</v>
+        <v>113453</v>
       </c>
       <c r="L787" s="31" t="n">
-        <v>0.6288</v>
+        <v>0.5084</v>
       </c>
     </row>
     <row r="788">
@@ -43174,29 +43174,29 @@
         </is>
       </c>
       <c r="D788" s="9" t="n">
-        <v>227093.56</v>
+        <v>449189.44</v>
       </c>
       <c r="E788" s="9" t="n">
-        <v>654005.79</v>
+        <v>699850.01</v>
       </c>
       <c r="F788" s="10" t="n">
-        <v>-0.3844</v>
+        <v>-0.6856</v>
       </c>
       <c r="G788" s="10" t="n">
-        <v>-0.4474</v>
+        <v>-0.7339</v>
       </c>
       <c r="H788" s="10" t="n"/>
       <c r="I788" s="10" t="n">
-        <v>0.3273</v>
+        <v>0.3582</v>
       </c>
       <c r="J788" s="13" t="n">
-        <v>1207</v>
+        <v>1823</v>
       </c>
       <c r="K788" s="13" t="n">
-        <v>3014</v>
+        <v>4686</v>
       </c>
       <c r="L788" s="32" t="n">
-        <v>0.9476</v>
+        <v>0.5084</v>
       </c>
     </row>
     <row r="789">
@@ -43216,29 +43216,29 @@
         </is>
       </c>
       <c r="D789" s="15" t="n">
-        <v>291639.01</v>
+        <v>408318.47</v>
       </c>
       <c r="E789" s="15" t="n">
-        <v>101358.54</v>
+        <v>278854.5</v>
       </c>
       <c r="F789" s="16" t="n">
-        <v>0.0274</v>
+        <v>-0.0408</v>
       </c>
       <c r="G789" s="16" t="n">
-        <v>-0.0188</v>
+        <v>-0.0888</v>
       </c>
       <c r="H789" s="16" t="n"/>
       <c r="I789" s="16" t="n">
-        <v>0.2201</v>
+        <v>0.2435</v>
       </c>
       <c r="J789" s="19" t="n">
-        <v>2912</v>
+        <v>4275</v>
       </c>
       <c r="K789" s="19" t="n">
-        <v>4869</v>
+        <v>7463</v>
       </c>
       <c r="L789" s="31" t="n">
-        <v>0.9389</v>
+        <v>0.6884</v>
       </c>
     </row>
     <row r="790">
@@ -43258,29 +43258,29 @@
         </is>
       </c>
       <c r="D790" s="9" t="n">
-        <v>235046.37</v>
+        <v>331577.13</v>
       </c>
       <c r="E790" s="9" t="n">
-        <v>263750.87</v>
+        <v>557703.17</v>
       </c>
       <c r="F790" s="10" t="n">
-        <v>0.1606</v>
+        <v>0.1539</v>
       </c>
       <c r="G790" s="10" t="n">
-        <v>0.1</v>
+        <v>0.0912</v>
       </c>
       <c r="H790" s="10" t="n"/>
       <c r="I790" s="10" t="n">
-        <v>0.1488</v>
+        <v>0.1703</v>
       </c>
       <c r="J790" s="13" t="n">
-        <v>4275</v>
+        <v>6294</v>
       </c>
       <c r="K790" s="13" t="n">
-        <v>5894</v>
+        <v>8943</v>
       </c>
       <c r="L790" s="32" t="n">
-        <v>0.8516</v>
+        <v>0.6221</v>
       </c>
     </row>
     <row r="791">
@@ -43300,29 +43300,29 @@
         </is>
       </c>
       <c r="D791" s="15" t="n">
-        <v>234203.3</v>
+        <v>306445.25</v>
       </c>
       <c r="E791" s="15" t="n">
-        <v>233816.11</v>
+        <v>712672.14</v>
       </c>
       <c r="F791" s="16" t="n">
-        <v>0.212</v>
+        <v>0.1804</v>
       </c>
       <c r="G791" s="16" t="n">
-        <v>0.1477</v>
+        <v>0.1103</v>
       </c>
       <c r="H791" s="16" t="n"/>
       <c r="I791" s="16" t="n">
-        <v>0.1051</v>
+        <v>0.1247</v>
       </c>
       <c r="J791" s="19" t="n">
-        <v>5393</v>
+        <v>7778</v>
       </c>
       <c r="K791" s="19" t="n">
-        <v>11156</v>
+        <v>14745</v>
       </c>
       <c r="L791" s="31" t="n">
-        <v>0.9046</v>
+        <v>0.7181999999999999</v>
       </c>
     </row>
     <row r="792">
@@ -43342,29 +43342,29 @@
         </is>
       </c>
       <c r="D792" s="9" t="n">
-        <v>324551.56</v>
+        <v>454959.55</v>
       </c>
       <c r="E792" s="9" t="n">
-        <v>836709.71</v>
+        <v>1818681.79</v>
       </c>
       <c r="F792" s="10" t="n">
-        <v>0.221</v>
+        <v>0.2041</v>
       </c>
       <c r="G792" s="10" t="n">
-        <v>0.1527</v>
+        <v>0.1301</v>
       </c>
       <c r="H792" s="10" t="n"/>
       <c r="I792" s="10" t="n">
-        <v>0.0654</v>
+        <v>0.0801</v>
       </c>
       <c r="J792" s="13" t="n">
-        <v>12549</v>
+        <v>17942</v>
       </c>
       <c r="K792" s="13" t="n">
-        <v>15386</v>
+        <v>22626</v>
       </c>
       <c r="L792" s="32" t="n">
-        <v>0.7971</v>
+        <v>0.5926</v>
       </c>
     </row>
     <row r="793">
@@ -43384,29 +43384,29 @@
         </is>
       </c>
       <c r="D793" s="15" t="n">
-        <v>310202.51</v>
+        <v>414016.48</v>
       </c>
       <c r="E793" s="15" t="n">
-        <v>1793782.44</v>
+        <v>3596330.48</v>
       </c>
       <c r="F793" s="16" t="n">
-        <v>0.2633</v>
+        <v>0.3329</v>
       </c>
       <c r="G793" s="16" t="n">
-        <v>0.1907</v>
+        <v>0.2525</v>
       </c>
       <c r="H793" s="16" t="n"/>
       <c r="I793" s="16" t="n">
-        <v>0.0396</v>
+        <v>0.0511</v>
       </c>
       <c r="J793" s="19" t="n">
-        <v>17403</v>
+        <v>24679</v>
       </c>
       <c r="K793" s="19" t="n">
-        <v>20750</v>
+        <v>30541</v>
       </c>
       <c r="L793" s="31" t="n">
-        <v>0.7419</v>
+        <v>0.5736</v>
       </c>
     </row>
     <row r="794">
@@ -44350,29 +44350,29 @@
         </is>
       </c>
       <c r="D816" s="9" t="n">
-        <v>6248821.51</v>
+        <v>9785449.689999999</v>
       </c>
       <c r="E816" s="9" t="n">
-        <v>8007787.59</v>
+        <v>25733893.86</v>
       </c>
       <c r="F816" s="10" t="n">
-        <v>0.3664</v>
+        <v>0.3582</v>
       </c>
       <c r="G816" s="10" t="n">
-        <v>0.3105</v>
+        <v>0.2993</v>
       </c>
       <c r="H816" s="10" t="n"/>
       <c r="I816" s="10" t="n">
-        <v>0.06419999999999999</v>
+        <v>0.0757</v>
       </c>
       <c r="J816" s="13" t="n">
-        <v>121320</v>
+        <v>188680</v>
       </c>
       <c r="K816" s="13" t="n">
-        <v>223804</v>
+        <v>349180</v>
       </c>
       <c r="L816" s="32" t="n">
-        <v>0.9224</v>
+        <v>0.6321</v>
       </c>
     </row>
     <row r="817">
@@ -50860,29 +50860,29 @@
         </is>
       </c>
       <c r="D971" s="15" t="n">
-        <v>613628.21</v>
+        <v>822143.49</v>
       </c>
       <c r="E971" s="15" t="n">
-        <v>3923100.42</v>
+        <v>9792780.220000001</v>
       </c>
       <c r="F971" s="16" t="n">
-        <v>0.6973</v>
+        <v>0.7091</v>
       </c>
       <c r="G971" s="16" t="n">
-        <v>0.6283</v>
+        <v>0.6358</v>
       </c>
       <c r="H971" s="16" t="n"/>
       <c r="I971" s="16" t="n">
-        <v>0.0167</v>
+        <v>0.0194</v>
       </c>
       <c r="J971" s="19" t="n">
-        <v>42664</v>
+        <v>59470</v>
       </c>
       <c r="K971" s="19" t="n">
-        <v>80692</v>
+        <v>107776</v>
       </c>
       <c r="L971" s="31" t="n">
-        <v>0.8226</v>
+        <v>0.6428</v>
       </c>
     </row>
     <row r="972">
@@ -50902,29 +50902,29 @@
         </is>
       </c>
       <c r="D972" s="9" t="n">
-        <v>2054736.72</v>
+        <v>3098919.71</v>
       </c>
       <c r="E972" s="9" t="n">
-        <v>506959.58</v>
+        <v>1727684.53</v>
       </c>
       <c r="F972" s="10" t="n">
-        <v>0.1576</v>
+        <v>0.1849</v>
       </c>
       <c r="G972" s="10" t="n">
-        <v>0.111</v>
+        <v>0.1364</v>
       </c>
       <c r="H972" s="10" t="n"/>
       <c r="I972" s="10" t="n">
-        <v>0.3058</v>
+        <v>0.3118</v>
       </c>
       <c r="J972" s="13" t="n">
-        <v>4078</v>
+        <v>7621</v>
       </c>
       <c r="K972" s="13" t="n">
-        <v>21632</v>
+        <v>37175</v>
       </c>
       <c r="L972" s="32" t="n">
-        <v>0.9654</v>
+        <v>0.6946</v>
       </c>
     </row>
     <row r="973">
@@ -50944,29 +50944,29 @@
         </is>
       </c>
       <c r="D973" s="15" t="n">
-        <v>1044036.57</v>
+        <v>1893375.46</v>
       </c>
       <c r="E973" s="15" t="n">
-        <v>316272.67</v>
+        <v>1722796.65</v>
       </c>
       <c r="F973" s="16" t="n">
-        <v>0.2818</v>
+        <v>0.2911</v>
       </c>
       <c r="G973" s="16" t="n">
-        <v>0.2295</v>
+        <v>0.2368</v>
       </c>
       <c r="H973" s="16" t="n"/>
       <c r="I973" s="16" t="n">
-        <v>0.1832</v>
+        <v>0.1983</v>
       </c>
       <c r="J973" s="19" t="n">
-        <v>8394</v>
+        <v>15139</v>
       </c>
       <c r="K973" s="19" t="n">
-        <v>16010</v>
+        <v>31640</v>
       </c>
       <c r="L973" s="31" t="n">
-        <v>0.9455</v>
+        <v>0.5717</v>
       </c>
     </row>
     <row r="974">
@@ -50986,29 +50986,29 @@
         </is>
       </c>
       <c r="D974" s="9" t="n">
-        <v>799689.71</v>
+        <v>1322275.92</v>
       </c>
       <c r="E974" s="9" t="n">
-        <v>265967.82</v>
+        <v>1750299.99</v>
       </c>
       <c r="F974" s="10" t="n">
-        <v>0.365</v>
+        <v>0.3881</v>
       </c>
       <c r="G974" s="10" t="n">
-        <v>0.3083</v>
+        <v>0.3269</v>
       </c>
       <c r="H974" s="10" t="n"/>
       <c r="I974" s="10" t="n">
-        <v>0.1203</v>
+        <v>0.1314</v>
       </c>
       <c r="J974" s="13" t="n">
-        <v>12105</v>
+        <v>20318</v>
       </c>
       <c r="K974" s="13" t="n">
-        <v>20181</v>
+        <v>35967</v>
       </c>
       <c r="L974" s="32" t="n">
-        <v>0.9329</v>
+        <v>0.6012999999999999</v>
       </c>
     </row>
     <row r="975">
@@ -51028,29 +51028,29 @@
         </is>
       </c>
       <c r="D975" s="15" t="n">
-        <v>532341.37</v>
+        <v>866172.11</v>
       </c>
       <c r="E975" s="15" t="n">
-        <v>331751.44</v>
+        <v>1899469.56</v>
       </c>
       <c r="F975" s="16" t="n">
-        <v>0.4732</v>
+        <v>0.4376</v>
       </c>
       <c r="G975" s="16" t="n">
-        <v>0.4128</v>
+        <v>0.3722</v>
       </c>
       <c r="H975" s="16" t="n"/>
       <c r="I975" s="16" t="n">
-        <v>0.0886</v>
+        <v>0.0946</v>
       </c>
       <c r="J975" s="19" t="n">
-        <v>10664</v>
+        <v>18006</v>
       </c>
       <c r="K975" s="19" t="n">
-        <v>14499</v>
+        <v>26843</v>
       </c>
       <c r="L975" s="31" t="n">
-        <v>0.9206</v>
+        <v>0.595</v>
       </c>
     </row>
     <row r="976">
@@ -51070,29 +51070,29 @@
         </is>
       </c>
       <c r="D976" s="9" t="n">
-        <v>688939.83</v>
+        <v>1038086.27</v>
       </c>
       <c r="E976" s="9" t="n">
-        <v>697333.22</v>
+        <v>3147754.11</v>
       </c>
       <c r="F976" s="10" t="n">
-        <v>0.5612</v>
+        <v>0.4741</v>
       </c>
       <c r="G976" s="10" t="n">
-        <v>0.4989</v>
+        <v>0.4057</v>
       </c>
       <c r="H976" s="10" t="n"/>
       <c r="I976" s="10" t="n">
-        <v>0.055</v>
+        <v>0.0617</v>
       </c>
       <c r="J976" s="13" t="n">
-        <v>21007</v>
+        <v>33490</v>
       </c>
       <c r="K976" s="13" t="n">
-        <v>27996</v>
+        <v>47624</v>
       </c>
       <c r="L976" s="32" t="n">
-        <v>0.8843</v>
+        <v>0.624</v>
       </c>
     </row>
     <row r="977">
@@ -51112,29 +51112,29 @@
         </is>
       </c>
       <c r="D977" s="15" t="n">
-        <v>515449.09</v>
+        <v>744476.73</v>
       </c>
       <c r="E977" s="15" t="n">
-        <v>1966402.44</v>
+        <v>5693108.79</v>
       </c>
       <c r="F977" s="16" t="n">
-        <v>0.6075</v>
+        <v>0.5562</v>
       </c>
       <c r="G977" s="16" t="n">
-        <v>0.538</v>
+        <v>0.4828</v>
       </c>
       <c r="H977" s="16" t="n"/>
       <c r="I977" s="16" t="n">
-        <v>0.0328</v>
+        <v>0.0376</v>
       </c>
       <c r="J977" s="19" t="n">
-        <v>22408</v>
+        <v>34636</v>
       </c>
       <c r="K977" s="19" t="n">
-        <v>42794</v>
+        <v>62155</v>
       </c>
       <c r="L977" s="31" t="n">
-        <v>0.8594000000000001</v>
+        <v>0.6231</v>
       </c>
     </row>
     <row r="978">
@@ -51616,29 +51616,29 @@
         </is>
       </c>
       <c r="D989" s="15" t="n">
-        <v>485456.77</v>
+        <v>544428.1800000001</v>
       </c>
       <c r="E989" s="15" t="n">
-        <v>2413953.61</v>
+        <v>2623023.49</v>
       </c>
       <c r="F989" s="16" t="n">
-        <v>0.6264</v>
+        <v>0.6686</v>
       </c>
       <c r="G989" s="16" t="n">
-        <v>0.5589</v>
+        <v>0.6016</v>
       </c>
       <c r="H989" s="16" t="n"/>
       <c r="I989" s="16" t="n">
-        <v>0.0246</v>
+        <v>0.0242</v>
       </c>
       <c r="J989" s="19" t="n">
-        <v>16155</v>
+        <v>18022</v>
       </c>
       <c r="K989" s="19" t="n">
-        <v>19198</v>
+        <v>21431</v>
       </c>
       <c r="L989" s="31" t="n">
-        <v>0.4289</v>
+        <v>0.3839</v>
       </c>
     </row>
     <row r="990">
@@ -54892,29 +54892,29 @@
         </is>
       </c>
       <c r="D1067" s="15" t="n">
-        <v>233555.74</v>
+        <v>249179.56</v>
       </c>
       <c r="E1067" s="15" t="n">
-        <v>1837871.31</v>
+        <v>1946944.03</v>
       </c>
       <c r="F1067" s="16" t="n">
-        <v>0.8175</v>
+        <v>0.8401</v>
       </c>
       <c r="G1067" s="16" t="n">
-        <v>0.7468</v>
+        <v>0.7693</v>
       </c>
       <c r="H1067" s="16" t="n"/>
       <c r="I1067" s="16" t="n">
-        <v>0.0119</v>
+        <v>0.011</v>
       </c>
       <c r="J1067" s="19" t="n">
-        <v>11073</v>
+        <v>12079</v>
       </c>
       <c r="K1067" s="19" t="n">
-        <v>13196</v>
+        <v>14429</v>
       </c>
       <c r="L1067" s="31" t="n">
-        <v>0.3861</v>
+        <v>0.3628</v>
       </c>
     </row>
     <row r="1068">
@@ -54934,29 +54934,29 @@
         </is>
       </c>
       <c r="D1068" s="9" t="n">
-        <v>64292.31</v>
+        <v>76632.17999999999</v>
       </c>
       <c r="E1068" s="9" t="n">
-        <v>71370.85000000001</v>
+        <v>83156.49000000001</v>
       </c>
       <c r="F1068" s="10" t="n">
-        <v>0.3889</v>
+        <v>0.4546</v>
       </c>
       <c r="G1068" s="10" t="n">
-        <v>0.3412</v>
+        <v>0.4079</v>
       </c>
       <c r="H1068" s="10" t="n"/>
       <c r="I1068" s="10" t="n">
-        <v>0.1868</v>
+        <v>0.1777</v>
       </c>
       <c r="J1068" s="13" t="n">
-        <v>273</v>
+        <v>332</v>
       </c>
       <c r="K1068" s="13" t="n">
-        <v>482</v>
+        <v>569</v>
       </c>
       <c r="L1068" s="32" t="n">
-        <v>0.3631</v>
+        <v>0.3046</v>
       </c>
     </row>
     <row r="1069">
@@ -54976,29 +54976,29 @@
         </is>
       </c>
       <c r="D1069" s="15" t="n">
-        <v>20946.59</v>
+        <v>24026.03</v>
       </c>
       <c r="E1069" s="15" t="n">
-        <v>20730.88</v>
+        <v>25021.86</v>
       </c>
       <c r="F1069" s="16" t="n">
-        <v>0.4019</v>
+        <v>0.4426</v>
       </c>
       <c r="G1069" s="16" t="n">
-        <v>0.342</v>
+        <v>0.3821</v>
       </c>
       <c r="H1069" s="16" t="n"/>
       <c r="I1069" s="16" t="n">
-        <v>0.133</v>
+        <v>0.131</v>
       </c>
       <c r="J1069" s="19" t="n">
-        <v>376</v>
+        <v>458</v>
       </c>
       <c r="K1069" s="19" t="n">
-        <v>435</v>
+        <v>532</v>
       </c>
       <c r="L1069" s="31" t="n">
-        <v>0.6827</v>
+        <v>0.5961</v>
       </c>
     </row>
     <row r="1070">
@@ -55018,29 +55018,29 @@
         </is>
       </c>
       <c r="D1070" s="9" t="n">
-        <v>21422.82</v>
+        <v>32180.74</v>
       </c>
       <c r="E1070" s="9" t="n">
-        <v>25909.37</v>
+        <v>28169.35</v>
       </c>
       <c r="F1070" s="10" t="n">
-        <v>0.2956</v>
+        <v>0.5504</v>
       </c>
       <c r="G1070" s="10" t="n">
-        <v>0.2282</v>
+        <v>0.4894</v>
       </c>
       <c r="H1070" s="10" t="n"/>
       <c r="I1070" s="10" t="n">
-        <v>0.0959</v>
+        <v>0.0917</v>
       </c>
       <c r="J1070" s="13" t="n">
-        <v>490</v>
+        <v>567</v>
       </c>
       <c r="K1070" s="13" t="n">
-        <v>557</v>
+        <v>648</v>
       </c>
       <c r="L1070" s="32" t="n">
-        <v>0.6012999999999999</v>
+        <v>0.4004</v>
       </c>
     </row>
     <row r="1071">
@@ -55060,29 +55060,29 @@
         </is>
       </c>
       <c r="D1071" s="15" t="n">
-        <v>26886.56</v>
+        <v>29554.14</v>
       </c>
       <c r="E1071" s="15" t="n">
-        <v>41633.96</v>
+        <v>54507.76</v>
       </c>
       <c r="F1071" s="16" t="n">
-        <v>0.3707</v>
+        <v>0.3852</v>
       </c>
       <c r="G1071" s="16" t="n">
-        <v>0.3086</v>
+        <v>0.3216</v>
       </c>
       <c r="H1071" s="16" t="n"/>
       <c r="I1071" s="16" t="n">
-        <v>0.0798</v>
+        <v>0.0752</v>
       </c>
       <c r="J1071" s="19" t="n">
-        <v>526</v>
+        <v>625</v>
       </c>
       <c r="K1071" s="19" t="n">
-        <v>587</v>
+        <v>700</v>
       </c>
       <c r="L1071" s="31" t="n">
-        <v>0.7076</v>
+        <v>0.6516</v>
       </c>
     </row>
     <row r="1072">
@@ -55102,29 +55102,29 @@
         </is>
       </c>
       <c r="D1072" s="9" t="n">
-        <v>48565.08</v>
+        <v>54806.31</v>
       </c>
       <c r="E1072" s="9" t="n">
-        <v>127324.03</v>
+        <v>158053.05</v>
       </c>
       <c r="F1072" s="10" t="n">
-        <v>0.144</v>
+        <v>0.2775</v>
       </c>
       <c r="G1072" s="10" t="n">
-        <v>0.0694</v>
+        <v>0.2014</v>
       </c>
       <c r="H1072" s="10" t="n"/>
       <c r="I1072" s="10" t="n">
-        <v>0.0331</v>
+        <v>0.032</v>
       </c>
       <c r="J1072" s="13" t="n">
-        <v>1448</v>
+        <v>1687</v>
       </c>
       <c r="K1072" s="13" t="n">
-        <v>1644</v>
+        <v>1913</v>
       </c>
       <c r="L1072" s="32" t="n">
-        <v>0.5958</v>
+        <v>0.5329</v>
       </c>
     </row>
     <row r="1073">
@@ -55144,29 +55144,29 @@
         </is>
       </c>
       <c r="D1073" s="15" t="n">
-        <v>69787.64999999999</v>
+        <v>78049.23</v>
       </c>
       <c r="E1073" s="15" t="n">
-        <v>289113.2</v>
+        <v>327170.95</v>
       </c>
       <c r="F1073" s="16" t="n">
-        <v>0.8089</v>
+        <v>0.8315</v>
       </c>
       <c r="G1073" s="16" t="n">
-        <v>0.734</v>
+        <v>0.7574</v>
       </c>
       <c r="H1073" s="16" t="n"/>
       <c r="I1073" s="16" t="n">
-        <v>0.0142</v>
+        <v>0.0136</v>
       </c>
       <c r="J1073" s="19" t="n">
-        <v>1969</v>
+        <v>2274</v>
       </c>
       <c r="K1073" s="19" t="n">
-        <v>2297</v>
+        <v>2640</v>
       </c>
       <c r="L1073" s="31" t="n">
-        <v>0.2799</v>
+        <v>0.2512</v>
       </c>
     </row>
     <row r="1074">
@@ -55606,26 +55606,26 @@
         </is>
       </c>
       <c r="D1084" s="9" t="n">
-        <v>341357.47</v>
+        <v>1461637.68</v>
       </c>
       <c r="E1084" s="9" t="n">
-        <v>298924.53</v>
+        <v>2177367.67</v>
       </c>
       <c r="F1084" s="10" t="n">
-        <v>0.3574</v>
+        <v>0.3151</v>
       </c>
       <c r="G1084" s="10" t="n">
-        <v>0.3023</v>
+        <v>0.2565</v>
       </c>
       <c r="H1084" s="10" t="n"/>
       <c r="I1084" s="10" t="n">
-        <v>0.0747</v>
+        <v>0.073</v>
       </c>
       <c r="J1084" s="13" t="n">
-        <v>6611</v>
+        <v>29249</v>
       </c>
       <c r="K1084" s="13" t="n">
-        <v>13560</v>
+        <v>91830</v>
       </c>
       <c r="L1084" s="32" t="n">
         <v>0</v>
@@ -58588,26 +58588,26 @@
         </is>
       </c>
       <c r="D1155" s="15" t="n">
-        <v>6842.13</v>
+        <v>118952.97</v>
       </c>
       <c r="E1155" s="15" t="n">
-        <v>24626.87</v>
+        <v>790417.48</v>
       </c>
       <c r="F1155" s="16" t="n">
-        <v>0.8296</v>
+        <v>1.0167</v>
       </c>
       <c r="G1155" s="16" t="n">
-        <v>0.7726</v>
+        <v>0.9515</v>
       </c>
       <c r="H1155" s="16" t="n"/>
       <c r="I1155" s="16" t="n">
-        <v>0.0098</v>
+        <v>0.0059</v>
       </c>
       <c r="J1155" s="19" t="n">
-        <v>813</v>
+        <v>3914</v>
       </c>
       <c r="K1155" s="19" t="n">
-        <v>982</v>
+        <v>40419</v>
       </c>
       <c r="L1155" s="31" t="n">
         <v>0</v>
@@ -58630,26 +58630,26 @@
         </is>
       </c>
       <c r="D1156" s="9" t="n">
-        <v>146538.16</v>
+        <v>589216.15</v>
       </c>
       <c r="E1156" s="9" t="n">
-        <v>36315.91</v>
+        <v>685551.1899999999</v>
       </c>
       <c r="F1156" s="10" t="n">
-        <v>0.1192</v>
+        <v>0.1193</v>
       </c>
       <c r="G1156" s="10" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.0619</v>
       </c>
       <c r="H1156" s="10" t="n"/>
       <c r="I1156" s="10" t="n">
-        <v>0.1978</v>
+        <v>0.1897</v>
       </c>
       <c r="J1156" s="13" t="n">
-        <v>1188</v>
+        <v>4954</v>
       </c>
       <c r="K1156" s="13" t="n">
-        <v>3920</v>
+        <v>14651</v>
       </c>
       <c r="L1156" s="32" t="n">
         <v>0</v>
@@ -58672,26 +58672,26 @@
         </is>
       </c>
       <c r="D1157" s="15" t="n">
-        <v>131959.37</v>
+        <v>415663.92</v>
       </c>
       <c r="E1157" s="15" t="n">
-        <v>113710.5</v>
+        <v>226861.09</v>
       </c>
       <c r="F1157" s="16" t="n">
-        <v>0.4629</v>
+        <v>0.3773</v>
       </c>
       <c r="G1157" s="16" t="n">
-        <v>0.404</v>
+        <v>0.3198</v>
       </c>
       <c r="H1157" s="16" t="n"/>
       <c r="I1157" s="16" t="n">
-        <v>0.1065</v>
+        <v>0.108</v>
       </c>
       <c r="J1157" s="19" t="n">
-        <v>1418</v>
+        <v>5619</v>
       </c>
       <c r="K1157" s="19" t="n">
-        <v>4426</v>
+        <v>13081</v>
       </c>
       <c r="L1157" s="31" t="n">
         <v>0</v>
@@ -58714,26 +58714,26 @@
         </is>
       </c>
       <c r="D1158" s="9" t="n">
-        <v>19785.36</v>
+        <v>126542.03</v>
       </c>
       <c r="E1158" s="9" t="n">
-        <v>56586.86</v>
+        <v>109910.39</v>
       </c>
       <c r="F1158" s="10" t="n">
-        <v>0.4445</v>
+        <v>-0.1241</v>
       </c>
       <c r="G1158" s="10" t="n">
-        <v>0.3739</v>
+        <v>-0.1872</v>
       </c>
       <c r="H1158" s="10" t="n"/>
       <c r="I1158" s="10" t="n">
-        <v>0.0519</v>
+        <v>0.0674</v>
       </c>
       <c r="J1158" s="13" t="n">
-        <v>924</v>
+        <v>4109</v>
       </c>
       <c r="K1158" s="13" t="n">
-        <v>1218</v>
+        <v>6415</v>
       </c>
       <c r="L1158" s="32" t="n">
         <v>0</v>
@@ -58756,26 +58756,26 @@
         </is>
       </c>
       <c r="D1159" s="15" t="n">
-        <v>14721.92</v>
+        <v>70630.2</v>
       </c>
       <c r="E1159" s="15" t="n">
-        <v>17102.7</v>
+        <v>43364.71</v>
       </c>
       <c r="F1159" s="16" t="n">
-        <v>0.8147</v>
+        <v>0.6441</v>
       </c>
       <c r="G1159" s="16" t="n">
-        <v>0.748</v>
+        <v>0.5861</v>
       </c>
       <c r="H1159" s="16" t="n"/>
       <c r="I1159" s="16" t="n">
-        <v>0.0235</v>
+        <v>0.0427</v>
       </c>
       <c r="J1159" s="19" t="n">
-        <v>637</v>
+        <v>2717</v>
       </c>
       <c r="K1159" s="19" t="n">
-        <v>880</v>
+        <v>3573</v>
       </c>
       <c r="L1159" s="31" t="n">
         <v>0</v>
@@ -58798,26 +58798,26 @@
         </is>
       </c>
       <c r="D1160" s="9" t="n">
-        <v>16118.25</v>
+        <v>78728.50999999999</v>
       </c>
       <c r="E1160" s="9" t="n">
-        <v>41377.33</v>
+        <v>163313.85</v>
       </c>
       <c r="F1160" s="10" t="n">
-        <v>0.7606000000000001</v>
+        <v>0.4926</v>
       </c>
       <c r="G1160" s="10" t="n">
-        <v>0.6954</v>
+        <v>0.4346</v>
       </c>
       <c r="H1160" s="10" t="n"/>
       <c r="I1160" s="10" t="n">
-        <v>0.022</v>
+        <v>0.0288</v>
       </c>
       <c r="J1160" s="13" t="n">
-        <v>1047</v>
+        <v>4270</v>
       </c>
       <c r="K1160" s="13" t="n">
-        <v>1398</v>
+        <v>5781</v>
       </c>
       <c r="L1160" s="32" t="n">
         <v>0</v>
@@ -58840,26 +58840,26 @@
         </is>
       </c>
       <c r="D1161" s="15" t="n">
-        <v>5392.27</v>
+        <v>61903.91</v>
       </c>
       <c r="E1161" s="15" t="n">
-        <v>9204.34</v>
+        <v>157948.97</v>
       </c>
       <c r="F1161" s="16" t="n">
-        <v>0.8774</v>
+        <v>0.711</v>
       </c>
       <c r="G1161" s="16" t="n">
-        <v>0.8104</v>
+        <v>0.6525</v>
       </c>
       <c r="H1161" s="16" t="n"/>
       <c r="I1161" s="16" t="n">
-        <v>0.024</v>
+        <v>0.0134</v>
       </c>
       <c r="J1161" s="19" t="n">
-        <v>584</v>
+        <v>3666</v>
       </c>
       <c r="K1161" s="19" t="n">
-        <v>736</v>
+        <v>7910</v>
       </c>
       <c r="L1161" s="31" t="n">
         <v>0</v>
@@ -59386,26 +59386,26 @@
         </is>
       </c>
       <c r="D1174" s="9" t="n">
-        <v>175384057.38</v>
+        <v>176373261.15</v>
       </c>
       <c r="E1174" s="9" t="n">
-        <v>770270375.92</v>
+        <v>773209780.41</v>
       </c>
       <c r="F1174" s="10" t="n">
-        <v>0.1445</v>
+        <v>0.1429</v>
       </c>
       <c r="G1174" s="10" t="n">
-        <v>0.0857</v>
+        <v>0.08409999999999999</v>
       </c>
       <c r="H1174" s="10" t="n"/>
       <c r="I1174" s="10" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.0983</v>
       </c>
       <c r="J1174" s="13" t="n">
-        <v>4200989</v>
+        <v>4205576</v>
       </c>
       <c r="K1174" s="13" t="n">
-        <v>8135143</v>
+        <v>8170415</v>
       </c>
       <c r="L1174" s="32" t="n">
         <v>0</v>
@@ -59428,26 +59428,26 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>14330317.02</v>
+        <v>34154509.52</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>62000825.03</v>
+        <v>128339336.36</v>
       </c>
       <c r="F1175" s="16" t="n">
-        <v>0.0129</v>
+        <v>0.0248</v>
       </c>
       <c r="G1175" s="16" t="n">
-        <v>-0.0414</v>
+        <v>-0.0297</v>
       </c>
       <c r="H1175" s="16" t="n"/>
       <c r="I1175" s="16" t="n">
-        <v>0.1043</v>
+        <v>0.113</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>376159</v>
+        <v>780027</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>716742</v>
+        <v>1488069</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -62998,26 +62998,26 @@
         </is>
       </c>
       <c r="D1260" s="9" t="n">
-        <v>21415851.66</v>
+        <v>21453018.56</v>
       </c>
       <c r="E1260" s="9" t="n">
-        <v>387438289.48</v>
+        <v>389674509.32</v>
       </c>
       <c r="F1260" s="10" t="n">
-        <v>0.4388</v>
+        <v>0.4377</v>
       </c>
       <c r="G1260" s="10" t="n">
-        <v>0.3585</v>
+        <v>0.3573</v>
       </c>
       <c r="H1260" s="10" t="n"/>
       <c r="I1260" s="10" t="n">
         <v>0.0283</v>
       </c>
       <c r="J1260" s="13" t="n">
-        <v>1575565</v>
+        <v>1575927</v>
       </c>
       <c r="K1260" s="13" t="n">
-        <v>2453731</v>
+        <v>2465999</v>
       </c>
       <c r="L1260" s="32" t="n">
         <v>0</v>
@@ -63040,26 +63040,26 @@
         </is>
       </c>
       <c r="D1261" s="15" t="n">
-        <v>46199586</v>
+        <v>46788644.17</v>
       </c>
       <c r="E1261" s="15" t="n">
-        <v>24146336.19</v>
+        <v>24363916.93</v>
       </c>
       <c r="F1261" s="16" t="n">
-        <v>0.0338</v>
+        <v>0.0321</v>
       </c>
       <c r="G1261" s="16" t="n">
-        <v>-0.008</v>
+        <v>-0.0097</v>
       </c>
       <c r="H1261" s="16" t="n"/>
       <c r="I1261" s="16" t="n">
-        <v>0.3101</v>
+        <v>0.3104</v>
       </c>
       <c r="J1261" s="19" t="n">
-        <v>197064</v>
+        <v>198391</v>
       </c>
       <c r="K1261" s="19" t="n">
-        <v>884832</v>
+        <v>892353</v>
       </c>
       <c r="L1261" s="31" t="n">
         <v>0</v>
@@ -63082,26 +63082,26 @@
         </is>
       </c>
       <c r="D1262" s="9" t="n">
-        <v>29720590.67</v>
+        <v>29940421.86</v>
       </c>
       <c r="E1262" s="9" t="n">
-        <v>30953272.04</v>
+        <v>31119391.9</v>
       </c>
       <c r="F1262" s="10" t="n">
-        <v>0.0464</v>
+        <v>0.0437</v>
       </c>
       <c r="G1262" s="10" t="n">
-        <v>-0.0051</v>
+        <v>-0.0078</v>
       </c>
       <c r="H1262" s="10" t="n"/>
       <c r="I1262" s="10" t="n">
-        <v>0.237</v>
+        <v>0.2374</v>
       </c>
       <c r="J1262" s="13" t="n">
-        <v>294137</v>
+        <v>295224</v>
       </c>
       <c r="K1262" s="13" t="n">
-        <v>778971</v>
+        <v>782205</v>
       </c>
       <c r="L1262" s="32" t="n">
         <v>0</v>
@@ -63124,26 +63124,26 @@
         </is>
       </c>
       <c r="D1263" s="15" t="n">
-        <v>22409375.51</v>
+        <v>22479595.61</v>
       </c>
       <c r="E1263" s="15" t="n">
-        <v>37033124.46</v>
+        <v>37079999.04</v>
       </c>
       <c r="F1263" s="16" t="n">
-        <v>0.0694</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="G1263" s="16" t="n">
-        <v>0.012</v>
+        <v>0.0102</v>
       </c>
       <c r="H1263" s="16" t="n"/>
       <c r="I1263" s="16" t="n">
-        <v>0.1886</v>
+        <v>0.189</v>
       </c>
       <c r="J1263" s="19" t="n">
-        <v>343150</v>
+        <v>343841</v>
       </c>
       <c r="K1263" s="19" t="n">
-        <v>748063</v>
+        <v>749572</v>
       </c>
       <c r="L1263" s="31" t="n">
         <v>0</v>
@@ -63166,26 +63166,26 @@
         </is>
       </c>
       <c r="D1264" s="9" t="n">
-        <v>15054492.07</v>
+        <v>15069885.63</v>
       </c>
       <c r="E1264" s="9" t="n">
-        <v>40863131.74</v>
+        <v>40879842.98</v>
       </c>
       <c r="F1264" s="10" t="n">
-        <v>0.0834</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="G1264" s="10" t="n">
-        <v>0.0188</v>
+        <v>0.0185</v>
       </c>
       <c r="H1264" s="10" t="n"/>
       <c r="I1264" s="10" t="n">
-        <v>0.1499</v>
+        <v>0.15</v>
       </c>
       <c r="J1264" s="13" t="n">
-        <v>332735</v>
+        <v>333083</v>
       </c>
       <c r="K1264" s="13" t="n">
-        <v>634237</v>
+        <v>635196</v>
       </c>
       <c r="L1264" s="32" t="n">
         <v>0</v>
@@ -63208,26 +63208,26 @@
         </is>
       </c>
       <c r="D1265" s="15" t="n">
-        <v>21131567.97</v>
+        <v>21147289.46</v>
       </c>
       <c r="E1265" s="15" t="n">
-        <v>93737989.83</v>
+        <v>93769954.95</v>
       </c>
       <c r="F1265" s="16" t="n">
-        <v>0.1836</v>
+        <v>0.184</v>
       </c>
       <c r="G1265" s="16" t="n">
-        <v>0.115</v>
+        <v>0.1153</v>
       </c>
       <c r="H1265" s="16" t="n"/>
       <c r="I1265" s="16" t="n">
-        <v>0.1092</v>
+        <v>0.1093</v>
       </c>
       <c r="J1265" s="19" t="n">
-        <v>644621</v>
+        <v>645082</v>
       </c>
       <c r="K1265" s="19" t="n">
-        <v>1133242</v>
+        <v>1135102</v>
       </c>
       <c r="L1265" s="31" t="n">
         <v>0</v>
@@ -63250,26 +63250,26 @@
         </is>
       </c>
       <c r="D1266" s="9" t="n">
-        <v>19452593.49</v>
+        <v>19494405.87</v>
       </c>
       <c r="E1266" s="9" t="n">
-        <v>156098232.18</v>
+        <v>156322165.29</v>
       </c>
       <c r="F1266" s="10" t="n">
-        <v>0.3243</v>
+        <v>0.3252</v>
       </c>
       <c r="G1266" s="10" t="n">
-        <v>0.251</v>
+        <v>0.2518</v>
       </c>
       <c r="H1266" s="10" t="n"/>
       <c r="I1266" s="10" t="n">
         <v>0.0636</v>
       </c>
       <c r="J1266" s="13" t="n">
-        <v>813717</v>
+        <v>814028</v>
       </c>
       <c r="K1266" s="13" t="n">
-        <v>1502067</v>
+        <v>1509988</v>
       </c>
       <c r="L1266" s="32" t="n">
         <v>0</v>
@@ -63292,26 +63292,26 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>2051386.45</v>
+        <v>4293137.14</v>
       </c>
       <c r="E1267" s="15" t="n">
-        <v>35266537.96</v>
+        <v>69964337.86</v>
       </c>
       <c r="F1267" s="16" t="n">
-        <v>0.3245</v>
+        <v>0.4633</v>
       </c>
       <c r="G1267" s="16" t="n">
-        <v>0.2499</v>
+        <v>0.3911</v>
       </c>
       <c r="H1267" s="16" t="n"/>
       <c r="I1267" s="16" t="n">
-        <v>0.0282</v>
+        <v>0.0302</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>164982</v>
+        <v>321961</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>279434</v>
+        <v>517123</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63334,26 +63334,26 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>4490203.27</v>
+        <v>9747648.52</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>1796608.85</v>
+        <v>4904845.32</v>
       </c>
       <c r="F1268" s="10" t="n">
-        <v>0.0101</v>
+        <v>-0.0532</v>
       </c>
       <c r="G1268" s="10" t="n">
-        <v>-0.0259</v>
+        <v>-0.0912</v>
       </c>
       <c r="H1268" s="10" t="n"/>
       <c r="I1268" s="10" t="n">
-        <v>0.3104</v>
+        <v>0.3168</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>16523</v>
+        <v>38295</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>66441</v>
+        <v>155884</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63376,26 +63376,26 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>2209056.75</v>
+        <v>6097421.07</v>
       </c>
       <c r="E1269" s="15" t="n">
-        <v>1866943.24</v>
+        <v>5591432.89</v>
       </c>
       <c r="F1269" s="16" t="n">
-        <v>-0.0148</v>
+        <v>-0.0864</v>
       </c>
       <c r="G1269" s="16" t="n">
-        <v>-0.0648</v>
+        <v>-0.1357</v>
       </c>
       <c r="H1269" s="16" t="n"/>
       <c r="I1269" s="16" t="n">
-        <v>0.2579</v>
+        <v>0.2653</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>23736</v>
+        <v>54160</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>58721</v>
+        <v>144752</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63418,26 +63418,26 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>1586344.51</v>
+        <v>4463138.75</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>2508367.86</v>
+        <v>6104734.79</v>
       </c>
       <c r="F1270" s="10" t="n">
-        <v>-0.0426</v>
+        <v>-0.1134</v>
       </c>
       <c r="G1270" s="10" t="n">
-        <v>-0.0999</v>
+        <v>-0.1686</v>
       </c>
       <c r="H1270" s="10" t="n"/>
       <c r="I1270" s="10" t="n">
-        <v>0.218</v>
+        <v>0.2273</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>26838</v>
+        <v>59816</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>52680</v>
+        <v>123730</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63460,26 +63460,26 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>1015132.99</v>
+        <v>2588859.97</v>
       </c>
       <c r="E1271" s="15" t="n">
-        <v>2332279.58</v>
+        <v>5690834.77</v>
       </c>
       <c r="F1271" s="16" t="n">
-        <v>-0.178</v>
+        <v>-0.1058</v>
       </c>
       <c r="G1271" s="16" t="n">
-        <v>-0.2391</v>
+        <v>-0.167</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
-        <v>0.1832</v>
+        <v>0.1904</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>26305</v>
+        <v>57184</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>44217</v>
+        <v>98990</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63502,26 +63502,26 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>1444363.28</v>
+        <v>3573668.34</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>5565420.19</v>
+        <v>12252556.11</v>
       </c>
       <c r="F1272" s="10" t="n">
-        <v>-0.1555</v>
+        <v>-0.0102</v>
       </c>
       <c r="G1272" s="10" t="n">
-        <v>-0.2227</v>
+        <v>-0.07829999999999999</v>
       </c>
       <c r="H1272" s="10" t="n"/>
       <c r="I1272" s="10" t="n">
-        <v>0.1399</v>
+        <v>0.1445</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>51023</v>
+        <v>109968</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>83371</v>
+        <v>184225</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63544,26 +63544,26 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>1533829.78</v>
+        <v>3390635.74</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>12664667.34</v>
+        <v>23830594.62</v>
       </c>
       <c r="F1273" s="16" t="n">
-        <v>-0.0132</v>
+        <v>0.2116</v>
       </c>
       <c r="G1273" s="16" t="n">
-        <v>-0.0805</v>
+        <v>0.144</v>
       </c>
       <c r="H1273" s="16" t="n"/>
       <c r="I1273" s="16" t="n">
-        <v>0.0824</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>66752</v>
+        <v>138643</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>131878</v>
+        <v>263365</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -64090,26 +64090,26 @@
         </is>
       </c>
       <c r="D1286" s="9" t="n">
-        <v>60762.19</v>
+        <v>1388858.16</v>
       </c>
       <c r="E1286" s="9" t="n">
-        <v>197146.71</v>
+        <v>616574.1899999999</v>
       </c>
       <c r="F1286" s="10" t="n">
-        <v>0.5455</v>
+        <v>0.1971</v>
       </c>
       <c r="G1286" s="10" t="n">
-        <v>0.4763</v>
+        <v>0.1432</v>
       </c>
       <c r="H1286" s="10" t="n"/>
       <c r="I1286" s="10" t="n">
-        <v>0.0259</v>
+        <v>0.0858</v>
       </c>
       <c r="J1286" s="13" t="n">
-        <v>2816</v>
+        <v>25877</v>
       </c>
       <c r="K1286" s="13" t="n">
-        <v>3329</v>
+        <v>37764</v>
       </c>
       <c r="L1286" s="32" t="n">
         <v>0</v>
@@ -67660,26 +67660,26 @@
         </is>
       </c>
       <c r="D1371" s="15" t="n">
-        <v>14613.5</v>
+        <v>105248.54</v>
       </c>
       <c r="E1371" s="15" t="n">
-        <v>122019.12</v>
+        <v>209938.5</v>
       </c>
       <c r="F1371" s="16" t="n">
-        <v>0.9053</v>
+        <v>0.318</v>
       </c>
       <c r="G1371" s="16" t="n">
-        <v>0.8302</v>
+        <v>0.2531</v>
       </c>
       <c r="H1371" s="16" t="n"/>
       <c r="I1371" s="16" t="n">
-        <v>0.002</v>
+        <v>0.0242</v>
       </c>
       <c r="J1371" s="19" t="n">
-        <v>1538</v>
+        <v>7197</v>
       </c>
       <c r="K1371" s="19" t="n">
-        <v>1840</v>
+        <v>10402</v>
       </c>
       <c r="L1371" s="31" t="n">
         <v>0</v>
@@ -67702,26 +67702,26 @@
         </is>
       </c>
       <c r="D1372" s="9" t="n">
-        <v>14147.5</v>
+        <v>290505.8</v>
       </c>
       <c r="E1372" s="9" t="n">
-        <v>9973.35</v>
+        <v>47779.85</v>
       </c>
       <c r="F1372" s="10" t="n">
-        <v>0.4777</v>
+        <v>0.293</v>
       </c>
       <c r="G1372" s="10" t="n">
-        <v>0.421</v>
+        <v>0.2448</v>
       </c>
       <c r="H1372" s="10" t="n"/>
       <c r="I1372" s="10" t="n">
-        <v>0.131</v>
+        <v>0.2733</v>
       </c>
       <c r="J1372" s="13" t="n">
-        <v>145</v>
+        <v>1317</v>
       </c>
       <c r="K1372" s="13" t="n">
-        <v>216</v>
+        <v>2710</v>
       </c>
       <c r="L1372" s="32" t="n">
         <v>0</v>
@@ -67744,26 +67744,26 @@
         </is>
       </c>
       <c r="D1373" s="15" t="n">
-        <v>4904.21</v>
+        <v>341164.66</v>
       </c>
       <c r="E1373" s="15" t="n">
-        <v>14348.4</v>
+        <v>51045.95</v>
       </c>
       <c r="F1373" s="16" t="n">
-        <v>0.3593</v>
+        <v>-0.012</v>
       </c>
       <c r="G1373" s="16" t="n">
-        <v>0.2757</v>
+        <v>-0.0614</v>
       </c>
       <c r="H1373" s="16" t="n"/>
       <c r="I1373" s="16" t="n">
-        <v>0.1203</v>
+        <v>0.2054</v>
       </c>
       <c r="J1373" s="19" t="n">
-        <v>133</v>
+        <v>2468</v>
       </c>
       <c r="K1373" s="19" t="n">
-        <v>148</v>
+        <v>3971</v>
       </c>
       <c r="L1373" s="31" t="n">
         <v>0</v>
@@ -67786,26 +67786,26 @@
         </is>
       </c>
       <c r="D1374" s="9" t="n">
-        <v>3472.59</v>
+        <v>206521.35</v>
       </c>
       <c r="E1374" s="9" t="n">
-        <v>3681.65</v>
+        <v>59996.41</v>
       </c>
       <c r="F1374" s="10" t="n">
-        <v>0.866</v>
+        <v>0.1624</v>
       </c>
       <c r="G1374" s="10" t="n">
-        <v>0.7985</v>
+        <v>0.1063</v>
       </c>
       <c r="H1374" s="10" t="n"/>
       <c r="I1374" s="10" t="n">
-        <v>0.0494</v>
+        <v>0.1418</v>
       </c>
       <c r="J1374" s="13" t="n">
-        <v>162</v>
+        <v>2947</v>
       </c>
       <c r="K1374" s="13" t="n">
-        <v>188</v>
+        <v>3958</v>
       </c>
       <c r="L1374" s="32" t="n">
         <v>0</v>
@@ -67828,26 +67828,26 @@
         </is>
       </c>
       <c r="D1375" s="15" t="n">
-        <v>10310.05</v>
+        <v>169901.13</v>
       </c>
       <c r="E1375" s="15" t="n">
-        <v>13666.38</v>
+        <v>82069.41</v>
       </c>
       <c r="F1375" s="16" t="n">
-        <v>0.2874</v>
+        <v>0.3462</v>
       </c>
       <c r="G1375" s="16" t="n">
-        <v>0.2131</v>
+        <v>0.2931</v>
       </c>
       <c r="H1375" s="16" t="n"/>
       <c r="I1375" s="16" t="n">
-        <v>0.0679</v>
+        <v>0.0968</v>
       </c>
       <c r="J1375" s="19" t="n">
-        <v>162</v>
+        <v>2645</v>
       </c>
       <c r="K1375" s="19" t="n">
-        <v>183</v>
+        <v>3756</v>
       </c>
       <c r="L1375" s="31" t="n">
         <v>0</v>
@@ -67870,26 +67870,26 @@
         </is>
       </c>
       <c r="D1376" s="9" t="n">
-        <v>7785.6</v>
+        <v>185942.32</v>
       </c>
       <c r="E1376" s="9" t="n">
-        <v>8274.549999999999</v>
+        <v>87038.3</v>
       </c>
       <c r="F1376" s="10" t="n">
-        <v>0.0823</v>
+        <v>0.2646</v>
       </c>
       <c r="G1376" s="10" t="n">
-        <v>0.0191</v>
+        <v>0.2056</v>
       </c>
       <c r="H1376" s="10" t="n"/>
       <c r="I1376" s="10" t="n">
-        <v>0.0351</v>
+        <v>0.06469999999999999</v>
       </c>
       <c r="J1376" s="13" t="n">
-        <v>342</v>
+        <v>5237</v>
       </c>
       <c r="K1376" s="13" t="n">
-        <v>381</v>
+        <v>8143</v>
       </c>
       <c r="L1376" s="32" t="n">
         <v>0</v>
@@ -67912,26 +67912,26 @@
         </is>
       </c>
       <c r="D1377" s="15" t="n">
-        <v>5528.74</v>
+        <v>89574.35000000001</v>
       </c>
       <c r="E1377" s="15" t="n">
-        <v>25183.26</v>
+        <v>78705.77</v>
       </c>
       <c r="F1377" s="16" t="n">
-        <v>0.8656</v>
+        <v>0.1972</v>
       </c>
       <c r="G1377" s="16" t="n">
-        <v>0.7921</v>
+        <v>0.135</v>
       </c>
       <c r="H1377" s="16" t="n"/>
       <c r="I1377" s="16" t="n">
-        <v>0.012</v>
+        <v>0.0411</v>
       </c>
       <c r="J1377" s="19" t="n">
-        <v>334</v>
+        <v>4066</v>
       </c>
       <c r="K1377" s="19" t="n">
-        <v>373</v>
+        <v>4824</v>
       </c>
       <c r="L1377" s="31" t="n">
         <v>0</v>
@@ -68751,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-28 14:47 UTC</t>
+          <t>2026-10-28 16:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-28 17:13 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8647,7 +8647,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-28 16:13 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-28 17:13 UTC.</t>
         </is>
       </c>
     </row>
@@ -39226,26 +39226,26 @@
         </is>
       </c>
       <c r="D694" s="9" t="n">
-        <v>13563307.28</v>
+        <v>13563451.25</v>
       </c>
       <c r="E694" s="9" t="n">
-        <v>78801596.06</v>
+        <v>78801851.91</v>
       </c>
       <c r="F694" s="10" t="n">
         <v>0.2913</v>
       </c>
       <c r="G694" s="10" t="n">
-        <v>0.225</v>
+        <v>0.2249</v>
       </c>
       <c r="H694" s="10" t="n"/>
       <c r="I694" s="10" t="n">
         <v>0.06900000000000001</v>
       </c>
       <c r="J694" s="13" t="n">
-        <v>485863</v>
+        <v>485873</v>
       </c>
       <c r="K694" s="13" t="n">
-        <v>669343</v>
+        <v>669361</v>
       </c>
       <c r="L694" s="32" t="n">
         <v>0.5271</v>
@@ -39268,10 +39268,10 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>3256603.51</v>
+        <v>3257626.8</v>
       </c>
       <c r="E695" s="15" t="n">
-        <v>24925755.65</v>
+        <v>24955545.1</v>
       </c>
       <c r="F695" s="16" t="n">
         <v>0.1703</v>
@@ -39284,13 +39284,13 @@
         <v>0.0526</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>150197</v>
+        <v>150253</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>202457</v>
+        <v>202545</v>
       </c>
       <c r="L695" s="31" t="n">
-        <v>0.5823</v>
+        <v>0.5822000000000001</v>
       </c>
     </row>
     <row r="696">
@@ -42838,7 +42838,7 @@
         </is>
       </c>
       <c r="D780" s="9" t="n">
-        <v>3103440.19</v>
+        <v>3103441.87</v>
       </c>
       <c r="E780" s="9" t="n">
         <v>49927972.85</v>
@@ -42854,10 +42854,10 @@
         <v>0.0184</v>
       </c>
       <c r="J780" s="13" t="n">
-        <v>250253</v>
+        <v>250254</v>
       </c>
       <c r="K780" s="13" t="n">
-        <v>337806</v>
+        <v>337807</v>
       </c>
       <c r="L780" s="32" t="n">
         <v>0.572</v>
@@ -42964,10 +42964,10 @@
         </is>
       </c>
       <c r="D783" s="15" t="n">
-        <v>1551278.28</v>
+        <v>1551374.54</v>
       </c>
       <c r="E783" s="15" t="n">
-        <v>2906922.06</v>
+        <v>2907061.32</v>
       </c>
       <c r="F783" s="16" t="n">
         <v>0.1736</v>
@@ -42980,10 +42980,10 @@
         <v>0.1838</v>
       </c>
       <c r="J783" s="19" t="n">
-        <v>28064</v>
+        <v>28066</v>
       </c>
       <c r="K783" s="19" t="n">
-        <v>41177</v>
+        <v>41180</v>
       </c>
       <c r="L783" s="31" t="n">
         <v>0.5453</v>
@@ -43006,10 +43006,10 @@
         </is>
       </c>
       <c r="D784" s="9" t="n">
-        <v>1259991.25</v>
+        <v>1260003.64</v>
       </c>
       <c r="E784" s="9" t="n">
-        <v>3415680.05</v>
+        <v>3415703.94</v>
       </c>
       <c r="F784" s="10" t="n">
         <v>0.1871</v>
@@ -43022,10 +43022,10 @@
         <v>0.1445</v>
       </c>
       <c r="J784" s="13" t="n">
-        <v>30284</v>
+        <v>30287</v>
       </c>
       <c r="K784" s="13" t="n">
-        <v>40878</v>
+        <v>40881</v>
       </c>
       <c r="L784" s="32" t="n">
         <v>0.5073</v>
@@ -43048,13 +43048,13 @@
         </is>
       </c>
       <c r="D785" s="15" t="n">
-        <v>2012876.04</v>
+        <v>2012892.34</v>
       </c>
       <c r="E785" s="15" t="n">
-        <v>7498312.67</v>
+        <v>7498326.62</v>
       </c>
       <c r="F785" s="16" t="n">
-        <v>0.1846</v>
+        <v>0.1845</v>
       </c>
       <c r="G785" s="16" t="n">
         <v>0.1149</v>
@@ -43064,10 +43064,10 @@
         <v>0.09810000000000001</v>
       </c>
       <c r="J785" s="19" t="n">
-        <v>64323</v>
+        <v>64325</v>
       </c>
       <c r="K785" s="19" t="n">
-        <v>82645</v>
+        <v>82648</v>
       </c>
       <c r="L785" s="31" t="n">
         <v>0.509</v>
@@ -43090,10 +43090,10 @@
         </is>
       </c>
       <c r="D786" s="9" t="n">
-        <v>1762283.1</v>
+        <v>1762300.44</v>
       </c>
       <c r="E786" s="9" t="n">
-        <v>11981715.76</v>
+        <v>11981794.5</v>
       </c>
       <c r="F786" s="10" t="n">
         <v>0.4109</v>
@@ -43103,13 +43103,13 @@
       </c>
       <c r="H786" s="10" t="n"/>
       <c r="I786" s="10" t="n">
-        <v>0.0571</v>
+        <v>0.0572</v>
       </c>
       <c r="J786" s="13" t="n">
-        <v>82051</v>
+        <v>82053</v>
       </c>
       <c r="K786" s="13" t="n">
-        <v>102805</v>
+        <v>102813</v>
       </c>
       <c r="L786" s="32" t="n">
         <v>0.5152</v>
@@ -43132,29 +43132,29 @@
         </is>
       </c>
       <c r="D787" s="15" t="n">
-        <v>892097.1899999999</v>
+        <v>892452.01</v>
       </c>
       <c r="E787" s="15" t="n">
-        <v>17261663.56</v>
+        <v>17284316.8</v>
       </c>
       <c r="F787" s="16" t="n">
-        <v>0.6077</v>
+        <v>0.6076</v>
       </c>
       <c r="G787" s="16" t="n">
-        <v>0.5273</v>
+        <v>0.5272</v>
       </c>
       <c r="H787" s="16" t="n"/>
       <c r="I787" s="16" t="n">
         <v>0.0167</v>
       </c>
       <c r="J787" s="19" t="n">
-        <v>87406</v>
+        <v>87446</v>
       </c>
       <c r="K787" s="19" t="n">
-        <v>113453</v>
+        <v>113521</v>
       </c>
       <c r="L787" s="31" t="n">
-        <v>0.5084</v>
+        <v>0.5083</v>
       </c>
     </row>
     <row r="788">
@@ -43216,26 +43216,26 @@
         </is>
       </c>
       <c r="D789" s="15" t="n">
-        <v>408318.47</v>
+        <v>408345.56</v>
       </c>
       <c r="E789" s="15" t="n">
         <v>278854.5</v>
       </c>
       <c r="F789" s="16" t="n">
-        <v>-0.0408</v>
+        <v>-0.0407</v>
       </c>
       <c r="G789" s="16" t="n">
-        <v>-0.0888</v>
+        <v>-0.0887</v>
       </c>
       <c r="H789" s="16" t="n"/>
       <c r="I789" s="16" t="n">
-        <v>0.2435</v>
+        <v>0.2433</v>
       </c>
       <c r="J789" s="19" t="n">
-        <v>4275</v>
+        <v>4279</v>
       </c>
       <c r="K789" s="19" t="n">
-        <v>7463</v>
+        <v>7467</v>
       </c>
       <c r="L789" s="31" t="n">
         <v>0.6884</v>
@@ -43300,10 +43300,10 @@
         </is>
       </c>
       <c r="D791" s="15" t="n">
-        <v>306445.25</v>
+        <v>306468.65</v>
       </c>
       <c r="E791" s="15" t="n">
-        <v>712672.14</v>
+        <v>712748.6899999999</v>
       </c>
       <c r="F791" s="16" t="n">
         <v>0.1804</v>
@@ -43313,13 +43313,13 @@
       </c>
       <c r="H791" s="16" t="n"/>
       <c r="I791" s="16" t="n">
-        <v>0.1247</v>
+        <v>0.1249</v>
       </c>
       <c r="J791" s="19" t="n">
-        <v>7778</v>
+        <v>7782</v>
       </c>
       <c r="K791" s="19" t="n">
-        <v>14745</v>
+        <v>14749</v>
       </c>
       <c r="L791" s="31" t="n">
         <v>0.7181999999999999</v>
@@ -43342,7 +43342,7 @@
         </is>
       </c>
       <c r="D792" s="9" t="n">
-        <v>454959.55</v>
+        <v>454981.88</v>
       </c>
       <c r="E792" s="9" t="n">
         <v>1818681.79</v>
@@ -43351,17 +43351,17 @@
         <v>0.2041</v>
       </c>
       <c r="G792" s="10" t="n">
-        <v>0.1301</v>
+        <v>0.1302</v>
       </c>
       <c r="H792" s="10" t="n"/>
       <c r="I792" s="10" t="n">
         <v>0.0801</v>
       </c>
       <c r="J792" s="13" t="n">
-        <v>17942</v>
+        <v>17944</v>
       </c>
       <c r="K792" s="13" t="n">
-        <v>22626</v>
+        <v>22628</v>
       </c>
       <c r="L792" s="32" t="n">
         <v>0.5926</v>
@@ -43384,29 +43384,29 @@
         </is>
       </c>
       <c r="D793" s="15" t="n">
-        <v>414016.48</v>
+        <v>414612.13</v>
       </c>
       <c r="E793" s="15" t="n">
-        <v>3596330.48</v>
+        <v>3603390.13</v>
       </c>
       <c r="F793" s="16" t="n">
-        <v>0.3329</v>
+        <v>0.3325</v>
       </c>
       <c r="G793" s="16" t="n">
-        <v>0.2525</v>
+        <v>0.252</v>
       </c>
       <c r="H793" s="16" t="n"/>
       <c r="I793" s="16" t="n">
         <v>0.0511</v>
       </c>
       <c r="J793" s="19" t="n">
-        <v>24679</v>
+        <v>24685</v>
       </c>
       <c r="K793" s="19" t="n">
-        <v>30541</v>
+        <v>30551</v>
       </c>
       <c r="L793" s="31" t="n">
-        <v>0.5736</v>
+        <v>0.5728</v>
       </c>
     </row>
     <row r="794">
@@ -59386,26 +59386,26 @@
         </is>
       </c>
       <c r="D1174" s="9" t="n">
-        <v>176373261.15</v>
+        <v>176379919.12</v>
       </c>
       <c r="E1174" s="9" t="n">
-        <v>773209780.41</v>
+        <v>773266594.1900001</v>
       </c>
       <c r="F1174" s="10" t="n">
-        <v>0.1429</v>
+        <v>0.1428</v>
       </c>
       <c r="G1174" s="10" t="n">
-        <v>0.08409999999999999</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="H1174" s="10" t="n"/>
       <c r="I1174" s="10" t="n">
         <v>0.0983</v>
       </c>
       <c r="J1174" s="13" t="n">
-        <v>4205576</v>
+        <v>4205792</v>
       </c>
       <c r="K1174" s="13" t="n">
-        <v>8170415</v>
+        <v>8171054</v>
       </c>
       <c r="L1174" s="32" t="n">
         <v>0</v>
@@ -59428,26 +59428,26 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>34154509.52</v>
+        <v>34170036.29</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>128339336.36</v>
+        <v>128501680.55</v>
       </c>
       <c r="F1175" s="16" t="n">
-        <v>0.0248</v>
+        <v>0.0244</v>
       </c>
       <c r="G1175" s="16" t="n">
-        <v>-0.0297</v>
+        <v>-0.0301</v>
       </c>
       <c r="H1175" s="16" t="n"/>
       <c r="I1175" s="16" t="n">
         <v>0.113</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>780027</v>
+        <v>780556</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>1488069</v>
+        <v>1489123</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -62998,26 +62998,26 @@
         </is>
       </c>
       <c r="D1260" s="9" t="n">
-        <v>21453018.56</v>
+        <v>21454066.46</v>
       </c>
       <c r="E1260" s="9" t="n">
-        <v>389674509.32</v>
+        <v>389721488.37</v>
       </c>
       <c r="F1260" s="10" t="n">
-        <v>0.4377</v>
+        <v>0.4375</v>
       </c>
       <c r="G1260" s="10" t="n">
-        <v>0.3573</v>
+        <v>0.357</v>
       </c>
       <c r="H1260" s="10" t="n"/>
       <c r="I1260" s="10" t="n">
         <v>0.0283</v>
       </c>
       <c r="J1260" s="13" t="n">
-        <v>1575927</v>
+        <v>1575954</v>
       </c>
       <c r="K1260" s="13" t="n">
-        <v>2465999</v>
+        <v>2466033</v>
       </c>
       <c r="L1260" s="32" t="n">
         <v>0</v>
@@ -63040,13 +63040,13 @@
         </is>
       </c>
       <c r="D1261" s="15" t="n">
-        <v>46788644.17</v>
+        <v>46789274.66</v>
       </c>
       <c r="E1261" s="15" t="n">
-        <v>24363916.93</v>
+        <v>24364287.56</v>
       </c>
       <c r="F1261" s="16" t="n">
-        <v>0.0321</v>
+        <v>0.032</v>
       </c>
       <c r="G1261" s="16" t="n">
         <v>-0.0097</v>
@@ -63056,10 +63056,10 @@
         <v>0.3104</v>
       </c>
       <c r="J1261" s="19" t="n">
-        <v>198391</v>
+        <v>198419</v>
       </c>
       <c r="K1261" s="19" t="n">
-        <v>892353</v>
+        <v>892393</v>
       </c>
       <c r="L1261" s="31" t="n">
         <v>0</v>
@@ -63082,10 +63082,10 @@
         </is>
       </c>
       <c r="D1262" s="9" t="n">
-        <v>29940421.86</v>
+        <v>29941215.67</v>
       </c>
       <c r="E1262" s="9" t="n">
-        <v>31119391.9</v>
+        <v>31119813.12</v>
       </c>
       <c r="F1262" s="10" t="n">
         <v>0.0437</v>
@@ -63098,10 +63098,10 @@
         <v>0.2374</v>
       </c>
       <c r="J1262" s="13" t="n">
-        <v>295224</v>
+        <v>295258</v>
       </c>
       <c r="K1262" s="13" t="n">
-        <v>782205</v>
+        <v>782276</v>
       </c>
       <c r="L1262" s="32" t="n">
         <v>0</v>
@@ -63124,26 +63124,26 @@
         </is>
       </c>
       <c r="D1263" s="15" t="n">
-        <v>22479595.61</v>
+        <v>22480778.11</v>
       </c>
       <c r="E1263" s="15" t="n">
-        <v>37079999.04</v>
+        <v>37082524</v>
       </c>
       <c r="F1263" s="16" t="n">
-        <v>0.06759999999999999</v>
+        <v>0.0675</v>
       </c>
       <c r="G1263" s="16" t="n">
-        <v>0.0102</v>
+        <v>0.0101</v>
       </c>
       <c r="H1263" s="16" t="n"/>
       <c r="I1263" s="16" t="n">
         <v>0.189</v>
       </c>
       <c r="J1263" s="19" t="n">
-        <v>343841</v>
+        <v>343874</v>
       </c>
       <c r="K1263" s="19" t="n">
-        <v>749572</v>
+        <v>749741</v>
       </c>
       <c r="L1263" s="31" t="n">
         <v>0</v>
@@ -63166,26 +63166,26 @@
         </is>
       </c>
       <c r="D1264" s="9" t="n">
-        <v>15069885.63</v>
+        <v>15071771.52</v>
       </c>
       <c r="E1264" s="9" t="n">
-        <v>40879842.98</v>
+        <v>40883477.55</v>
       </c>
       <c r="F1264" s="10" t="n">
-        <v>0.08309999999999999</v>
+        <v>0.0825</v>
       </c>
       <c r="G1264" s="10" t="n">
-        <v>0.0185</v>
+        <v>0.0179</v>
       </c>
       <c r="H1264" s="10" t="n"/>
       <c r="I1264" s="10" t="n">
         <v>0.15</v>
       </c>
       <c r="J1264" s="13" t="n">
-        <v>333083</v>
+        <v>333105</v>
       </c>
       <c r="K1264" s="13" t="n">
-        <v>635196</v>
+        <v>635396</v>
       </c>
       <c r="L1264" s="32" t="n">
         <v>0</v>
@@ -63208,10 +63208,10 @@
         </is>
       </c>
       <c r="D1265" s="15" t="n">
-        <v>21147289.46</v>
+        <v>21148024.03</v>
       </c>
       <c r="E1265" s="15" t="n">
-        <v>93769954.95</v>
+        <v>93772166.48999999</v>
       </c>
       <c r="F1265" s="16" t="n">
         <v>0.184</v>
@@ -63224,10 +63224,10 @@
         <v>0.1093</v>
       </c>
       <c r="J1265" s="19" t="n">
-        <v>645082</v>
+        <v>645117</v>
       </c>
       <c r="K1265" s="19" t="n">
-        <v>1135102</v>
+        <v>1135169</v>
       </c>
       <c r="L1265" s="31" t="n">
         <v>0</v>
@@ -63250,10 +63250,10 @@
         </is>
       </c>
       <c r="D1266" s="9" t="n">
-        <v>19494405.87</v>
+        <v>19494788.68</v>
       </c>
       <c r="E1266" s="9" t="n">
-        <v>156322165.29</v>
+        <v>156322837.09</v>
       </c>
       <c r="F1266" s="10" t="n">
         <v>0.3252</v>
@@ -63266,10 +63266,10 @@
         <v>0.0636</v>
       </c>
       <c r="J1266" s="13" t="n">
-        <v>814028</v>
+        <v>814065</v>
       </c>
       <c r="K1266" s="13" t="n">
-        <v>1509988</v>
+        <v>1510046</v>
       </c>
       <c r="L1266" s="32" t="n">
         <v>0</v>
@@ -63292,26 +63292,26 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>4293137.14</v>
+        <v>4296335.29</v>
       </c>
       <c r="E1267" s="15" t="n">
-        <v>69964337.86</v>
+        <v>70100866.36</v>
       </c>
       <c r="F1267" s="16" t="n">
-        <v>0.4633</v>
+        <v>0.4607</v>
       </c>
       <c r="G1267" s="16" t="n">
-        <v>0.3911</v>
+        <v>0.3884</v>
       </c>
       <c r="H1267" s="16" t="n"/>
       <c r="I1267" s="16" t="n">
         <v>0.0302</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>321961</v>
+        <v>322202</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>517123</v>
+        <v>517643</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63334,26 +63334,26 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>9747648.52</v>
+        <v>9750471.93</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>4904845.32</v>
+        <v>4906953.2</v>
       </c>
       <c r="F1268" s="10" t="n">
-        <v>-0.0532</v>
+        <v>-0.0533</v>
       </c>
       <c r="G1268" s="10" t="n">
-        <v>-0.0912</v>
+        <v>-0.09130000000000001</v>
       </c>
       <c r="H1268" s="10" t="n"/>
       <c r="I1268" s="10" t="n">
         <v>0.3168</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>38295</v>
+        <v>38314</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>155884</v>
+        <v>155921</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63376,26 +63376,26 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>6097421.07</v>
+        <v>6098028.15</v>
       </c>
       <c r="E1269" s="15" t="n">
-        <v>5591432.89</v>
+        <v>5591539.16</v>
       </c>
       <c r="F1269" s="16" t="n">
-        <v>-0.0864</v>
+        <v>-0.0863</v>
       </c>
       <c r="G1269" s="16" t="n">
-        <v>-0.1357</v>
+        <v>-0.1356</v>
       </c>
       <c r="H1269" s="16" t="n"/>
       <c r="I1269" s="16" t="n">
-        <v>0.2653</v>
+        <v>0.2652</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>54160</v>
+        <v>54181</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>144752</v>
+        <v>144779</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63418,26 +63418,26 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>4463138.75</v>
+        <v>4467022.78</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>6104734.79</v>
+        <v>6108282.44</v>
       </c>
       <c r="F1270" s="10" t="n">
-        <v>-0.1134</v>
+        <v>-0.1125</v>
       </c>
       <c r="G1270" s="10" t="n">
-        <v>-0.1686</v>
+        <v>-0.1677</v>
       </c>
       <c r="H1270" s="10" t="n"/>
       <c r="I1270" s="10" t="n">
         <v>0.2273</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>59816</v>
+        <v>59850</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>123730</v>
+        <v>123776</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63460,26 +63460,26 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>2588859.97</v>
+        <v>2589448.85</v>
       </c>
       <c r="E1271" s="15" t="n">
-        <v>5690834.77</v>
+        <v>5691219.84</v>
       </c>
       <c r="F1271" s="16" t="n">
-        <v>-0.1058</v>
+        <v>-0.1057</v>
       </c>
       <c r="G1271" s="16" t="n">
-        <v>-0.167</v>
+        <v>-0.1669</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
         <v>0.1904</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>57184</v>
+        <v>57216</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>98990</v>
+        <v>99035</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63502,26 +63502,26 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>3573668.34</v>
+        <v>3575352.7</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>12252556.11</v>
+        <v>12265682.24</v>
       </c>
       <c r="F1272" s="10" t="n">
-        <v>-0.0102</v>
+        <v>-0.0109</v>
       </c>
       <c r="G1272" s="10" t="n">
-        <v>-0.07829999999999999</v>
+        <v>-0.0791</v>
       </c>
       <c r="H1272" s="10" t="n"/>
       <c r="I1272" s="10" t="n">
         <v>0.1445</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>109968</v>
+        <v>110045</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>184225</v>
+        <v>184437</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63544,26 +63544,26 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>3390635.74</v>
+        <v>3393376.59</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>23830594.62</v>
+        <v>23837137.32</v>
       </c>
       <c r="F1273" s="16" t="n">
-        <v>0.2116</v>
+        <v>0.2106</v>
       </c>
       <c r="G1273" s="16" t="n">
-        <v>0.144</v>
+        <v>0.143</v>
       </c>
       <c r="H1273" s="16" t="n"/>
       <c r="I1273" s="16" t="n">
-        <v>0.08309999999999999</v>
+        <v>0.0832</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>138643</v>
+        <v>138748</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>263365</v>
+        <v>263532</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -68751,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-28 16:13 UTC</t>
+          <t>2026-10-28 17:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-29 15:13 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -5942,13 +5942,13 @@
         <v>0.04729</v>
       </c>
       <c r="E70" s="9" t="n">
-        <v>285061092.15</v>
+        <v>285082183.42</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>54965134.27</v>
+        <v>54937645.93</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>0.19282</v>
+        <v>0.19271</v>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
@@ -5956,13 +5956,13 @@
         </is>
       </c>
       <c r="I70" s="9" t="n">
-        <v>1210710659.26</v>
+        <v>1210731750.53</v>
       </c>
       <c r="J70" s="9" t="n">
-        <v>98736946.2</v>
+        <v>98709457.86</v>
       </c>
       <c r="K70" s="12" t="n">
-        <v>0.08155</v>
+        <v>0.08153000000000001</v>
       </c>
       <c r="L70" s="13" t="n">
         <v>219</v>
@@ -6010,22 +6010,22 @@
         <v>46327</v>
       </c>
       <c r="B71" s="15" t="n">
-        <v>195776960.82</v>
+        <v>290023265.3</v>
       </c>
       <c r="C71" s="15" t="n">
-        <v>11300764.39</v>
+        <v>10824463.21</v>
       </c>
       <c r="D71" s="16" t="n">
-        <v>0.05772</v>
+        <v>0.03732</v>
       </c>
       <c r="E71" s="15" t="n">
-        <v>51158805.46</v>
+        <v>77941885.75</v>
       </c>
       <c r="F71" s="15" t="n">
-        <v>7539875.03</v>
+        <v>3308922.51</v>
       </c>
       <c r="G71" s="16" t="n">
-        <v>0.14738</v>
+        <v>0.04245</v>
       </c>
       <c r="H71" s="17" t="inlineStr">
         <is>
@@ -6033,19 +6033,19 @@
         </is>
       </c>
       <c r="I71" s="15" t="n">
-        <v>246935766.29</v>
+        <v>367965151.05</v>
       </c>
       <c r="J71" s="15" t="n">
-        <v>18840639.43</v>
+        <v>14133385.72</v>
       </c>
       <c r="K71" s="18" t="n">
-        <v>0.07630000000000001</v>
+        <v>0.03841</v>
       </c>
       <c r="L71" s="19" t="n">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="M71" s="19" t="n">
-        <v>1022</v>
+        <v>320</v>
       </c>
       <c r="N71" s="15" t="n">
         <v>46236350.82</v>
@@ -6054,28 +6054,28 @@
         <v>0.03001</v>
       </c>
       <c r="P71" s="15" t="n">
-        <v>94427986.83</v>
+        <v>159809004.13</v>
       </c>
       <c r="Q71" s="16" t="n">
-        <v>0.04542</v>
+        <v>0.0246</v>
       </c>
       <c r="R71" s="15" t="n">
-        <v>32305010.2</v>
+        <v>48213465.27</v>
       </c>
       <c r="S71" s="16" t="n">
-        <v>0.13156</v>
+        <v>0.09447</v>
       </c>
       <c r="T71" s="15" t="n">
-        <v>10881225.19</v>
+        <v>14425136.43</v>
       </c>
       <c r="U71" s="16" t="n">
-        <v>0.06432</v>
+        <v>0.03938</v>
       </c>
       <c r="V71" s="15" t="n">
-        <v>11926387.78</v>
+        <v>21339308.66</v>
       </c>
       <c r="W71" s="16" t="n">
-        <v>0.0565</v>
+        <v>0.01793</v>
       </c>
       <c r="X71" s="15" t="n"/>
       <c r="Y71" s="16" t="n"/>
@@ -7469,22 +7469,22 @@
         <v>46296</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>3400401948.07</v>
+        <v>3494648252.56</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>98031967.43000001</v>
+        <v>97555666.25</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.02883</v>
+        <v>0.02792</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>962458191.3200001</v>
+        <v>989099510.4</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>178726710.71</v>
+        <v>174313449.38</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.1857</v>
+        <v>0.17623</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
@@ -7492,19 +7492,19 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>4362860139.39</v>
+        <v>4483747762.95</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>276758678.14</v>
+        <v>271869115.63</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.06344</v>
+        <v>0.06063</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>876</v>
+        <v>895</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>234</v>
+        <v>191</v>
       </c>
       <c r="N20" s="9" t="n">
         <v>1383015756.65</v>
@@ -7513,28 +7513,28 @@
         <v>0.02467</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>480414237.5</v>
+        <v>545795254.8</v>
       </c>
       <c r="Q20" s="10" t="n">
-        <v>0.035</v>
+        <v>0.03015</v>
       </c>
       <c r="R20" s="9" t="n">
-        <v>363853321.47</v>
+        <v>379761776.54</v>
       </c>
       <c r="S20" s="10" t="n">
-        <v>0.04133</v>
+        <v>0.0404</v>
       </c>
       <c r="T20" s="9" t="n">
-        <v>131526649.03</v>
+        <v>135070560.26</v>
       </c>
       <c r="U20" s="10" t="n">
-        <v>0.03094</v>
+        <v>0.02916</v>
       </c>
       <c r="V20" s="9" t="n">
-        <v>1041591983.43</v>
+        <v>1051004904.3</v>
       </c>
       <c r="W20" s="10" t="n">
-        <v>0.02688</v>
+        <v>0.02636</v>
       </c>
       <c r="X20" s="9" t="n"/>
       <c r="Y20" s="10" t="n"/>
@@ -8647,7 +8647,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-28 17:13 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-29 15:13 UTC.</t>
         </is>
       </c>
     </row>
@@ -10182,26 +10182,26 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>8024681.87</v>
+        <v>8028895.41</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>22502042.01</v>
+        <v>22503554.28</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.0896</v>
+        <v>0.0891</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.0305</v>
+        <v>0.03</v>
       </c>
       <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n">
-        <v>0.1192</v>
+        <v>0.1196</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>150478</v>
+        <v>150556</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>244272</v>
+        <v>244364</v>
       </c>
       <c r="L14" s="32" t="n">
         <v>0</v>
@@ -10224,26 +10224,26 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>3384519.55</v>
+        <v>7496682.6</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>4455000.07</v>
+        <v>17200673.39</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>0.2516</v>
+        <v>-0.0455</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>0.1954</v>
+        <v>-0.1058</v>
       </c>
       <c r="H15" s="16" t="n"/>
       <c r="I15" s="16" t="n">
-        <v>0.07920000000000001</v>
+        <v>0.1093</v>
       </c>
       <c r="J15" s="19" t="n">
-        <v>63872</v>
+        <v>140602</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>98756</v>
+        <v>229813</v>
       </c>
       <c r="L15" s="31" t="n">
         <v>0</v>
@@ -12954,26 +12954,26 @@
         </is>
       </c>
       <c r="D80" s="9" t="n">
-        <v>2299759.77</v>
+        <v>2301083.54</v>
       </c>
       <c r="E80" s="9" t="n">
-        <v>1504972.67</v>
+        <v>1505601.97</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>-0.0378</v>
+        <v>-0.038</v>
       </c>
       <c r="G80" s="10" t="n">
-        <v>-0.0848</v>
+        <v>-0.0851</v>
       </c>
       <c r="H80" s="10" t="n"/>
       <c r="I80" s="10" t="n">
-        <v>0.3412</v>
+        <v>0.3433</v>
       </c>
       <c r="J80" s="13" t="n">
-        <v>9362</v>
+        <v>9404</v>
       </c>
       <c r="K80" s="13" t="n">
-        <v>29078</v>
+        <v>29129</v>
       </c>
       <c r="L80" s="32" t="n">
         <v>0</v>
@@ -12996,26 +12996,26 @@
         </is>
       </c>
       <c r="D81" s="15" t="n">
-        <v>1854212.26</v>
+        <v>1854979.57</v>
       </c>
       <c r="E81" s="15" t="n">
-        <v>1761077.07</v>
+        <v>1761580.35</v>
       </c>
       <c r="F81" s="16" t="n">
-        <v>0.1108</v>
+        <v>0.1102</v>
       </c>
       <c r="G81" s="16" t="n">
-        <v>0.0559</v>
+        <v>0.0553</v>
       </c>
       <c r="H81" s="16" t="n"/>
       <c r="I81" s="16" t="n">
-        <v>0.241</v>
+        <v>0.2417</v>
       </c>
       <c r="J81" s="19" t="n">
-        <v>16464</v>
+        <v>16481</v>
       </c>
       <c r="K81" s="19" t="n">
-        <v>31920</v>
+        <v>31940</v>
       </c>
       <c r="L81" s="31" t="n">
         <v>0</v>
@@ -13038,26 +13038,26 @@
         </is>
       </c>
       <c r="D82" s="9" t="n">
-        <v>1224114.81</v>
+        <v>1224224.84</v>
       </c>
       <c r="E82" s="9" t="n">
-        <v>1886902.93</v>
+        <v>1886919.23</v>
       </c>
       <c r="F82" s="10" t="n">
-        <v>0.0161</v>
+        <v>0.0159</v>
       </c>
       <c r="G82" s="10" t="n">
-        <v>-0.0463</v>
+        <v>-0.0465</v>
       </c>
       <c r="H82" s="10" t="n"/>
       <c r="I82" s="10" t="n">
-        <v>0.1771</v>
+        <v>0.1774</v>
       </c>
       <c r="J82" s="13" t="n">
-        <v>18952</v>
+        <v>18959</v>
       </c>
       <c r="K82" s="13" t="n">
-        <v>30043</v>
+        <v>30051</v>
       </c>
       <c r="L82" s="32" t="n">
         <v>0</v>
@@ -13080,26 +13080,26 @@
         </is>
       </c>
       <c r="D83" s="15" t="n">
-        <v>775499.27</v>
+        <v>777445.4300000001</v>
       </c>
       <c r="E83" s="15" t="n">
-        <v>1698641.32</v>
+        <v>1698879.57</v>
       </c>
       <c r="F83" s="16" t="n">
-        <v>0.1256</v>
+        <v>0.1229</v>
       </c>
       <c r="G83" s="16" t="n">
-        <v>0.06</v>
+        <v>0.0574</v>
       </c>
       <c r="H83" s="16" t="n"/>
       <c r="I83" s="16" t="n">
-        <v>0.1308</v>
+        <v>0.1312</v>
       </c>
       <c r="J83" s="19" t="n">
-        <v>16731</v>
+        <v>16738</v>
       </c>
       <c r="K83" s="19" t="n">
-        <v>24242</v>
+        <v>24249</v>
       </c>
       <c r="L83" s="31" t="n">
         <v>0</v>
@@ -13122,26 +13122,26 @@
         </is>
       </c>
       <c r="D84" s="9" t="n">
-        <v>865560.78</v>
+        <v>865627.05</v>
       </c>
       <c r="E84" s="9" t="n">
-        <v>3367196.38</v>
+        <v>3367321.52</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>0.1048</v>
+        <v>0.1043</v>
       </c>
       <c r="G84" s="10" t="n">
-        <v>0.0334</v>
+        <v>0.0329</v>
       </c>
       <c r="H84" s="10" t="n"/>
       <c r="I84" s="10" t="n">
-        <v>0.093</v>
+        <v>0.0931</v>
       </c>
       <c r="J84" s="13" t="n">
-        <v>28676</v>
+        <v>28681</v>
       </c>
       <c r="K84" s="13" t="n">
-        <v>38831</v>
+        <v>38837</v>
       </c>
       <c r="L84" s="32" t="n">
         <v>0</v>
@@ -13206,26 +13206,26 @@
         </is>
       </c>
       <c r="D86" s="9" t="n">
-        <v>228934.05</v>
+        <v>471761.62</v>
       </c>
       <c r="E86" s="9" t="n">
-        <v>1050327.49</v>
+        <v>5920922.8</v>
       </c>
       <c r="F86" s="10" t="n">
-        <v>0.379</v>
+        <v>0.0664</v>
       </c>
       <c r="G86" s="10" t="n">
-        <v>0.3142</v>
+        <v>-0.0059</v>
       </c>
       <c r="H86" s="10" t="n"/>
       <c r="I86" s="10" t="n">
-        <v>0.0252</v>
+        <v>0.0314</v>
       </c>
       <c r="J86" s="13" t="n">
-        <v>15881</v>
+        <v>35575</v>
       </c>
       <c r="K86" s="13" t="n">
-        <v>22101</v>
+        <v>48617</v>
       </c>
       <c r="L86" s="32" t="n">
         <v>0</v>
@@ -13248,26 +13248,26 @@
         </is>
       </c>
       <c r="D87" s="15" t="n">
-        <v>1030476.39</v>
+        <v>2392245.47</v>
       </c>
       <c r="E87" s="15" t="n">
-        <v>685888.86</v>
+        <v>1537759.63</v>
       </c>
       <c r="F87" s="16" t="n">
-        <v>0.2599</v>
+        <v>0.0756</v>
       </c>
       <c r="G87" s="16" t="n">
-        <v>0.2096</v>
+        <v>0.0235</v>
       </c>
       <c r="H87" s="16" t="n"/>
       <c r="I87" s="16" t="n">
-        <v>0.2973</v>
+        <v>0.3269</v>
       </c>
       <c r="J87" s="19" t="n">
-        <v>3636</v>
+        <v>7719</v>
       </c>
       <c r="K87" s="19" t="n">
-        <v>12542</v>
+        <v>34254</v>
       </c>
       <c r="L87" s="31" t="n">
         <v>0</v>
@@ -13290,26 +13290,26 @@
         </is>
       </c>
       <c r="D88" s="9" t="n">
-        <v>673906.62</v>
+        <v>1490661.35</v>
       </c>
       <c r="E88" s="9" t="n">
-        <v>323939.15</v>
+        <v>1403813.55</v>
       </c>
       <c r="F88" s="10" t="n">
-        <v>0.2298</v>
+        <v>0.08019999999999999</v>
       </c>
       <c r="G88" s="10" t="n">
-        <v>0.1781</v>
+        <v>0.0223</v>
       </c>
       <c r="H88" s="10" t="n"/>
       <c r="I88" s="10" t="n">
-        <v>0.1725</v>
+        <v>0.2193</v>
       </c>
       <c r="J88" s="13" t="n">
-        <v>6904</v>
+        <v>15060</v>
       </c>
       <c r="K88" s="13" t="n">
-        <v>12745</v>
+        <v>30564</v>
       </c>
       <c r="L88" s="32" t="n">
         <v>0</v>
@@ -13332,26 +13332,26 @@
         </is>
       </c>
       <c r="D89" s="15" t="n">
-        <v>538952.58</v>
+        <v>1136759.77</v>
       </c>
       <c r="E89" s="15" t="n">
-        <v>883222.1899999999</v>
+        <v>1910367.84</v>
       </c>
       <c r="F89" s="16" t="n">
-        <v>-0.0495</v>
+        <v>-0.3104</v>
       </c>
       <c r="G89" s="16" t="n">
-        <v>-0.1079</v>
+        <v>-0.3727</v>
       </c>
       <c r="H89" s="16" t="n"/>
       <c r="I89" s="16" t="n">
-        <v>0.1136</v>
+        <v>0.1651</v>
       </c>
       <c r="J89" s="19" t="n">
-        <v>7516</v>
+        <v>17042</v>
       </c>
       <c r="K89" s="19" t="n">
-        <v>11573</v>
+        <v>28014</v>
       </c>
       <c r="L89" s="31" t="n">
         <v>0</v>
@@ -13374,26 +13374,26 @@
         </is>
       </c>
       <c r="D90" s="9" t="n">
-        <v>329735.87</v>
+        <v>755568.51</v>
       </c>
       <c r="E90" s="9" t="n">
-        <v>353294.7</v>
+        <v>1482815.64</v>
       </c>
       <c r="F90" s="10" t="n">
-        <v>0.2583</v>
+        <v>-0.2621</v>
       </c>
       <c r="G90" s="10" t="n">
-        <v>0.1963</v>
+        <v>-0.3288</v>
       </c>
       <c r="H90" s="10" t="n"/>
       <c r="I90" s="10" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.1314</v>
       </c>
       <c r="J90" s="13" t="n">
-        <v>6896</v>
+        <v>15544</v>
       </c>
       <c r="K90" s="13" t="n">
-        <v>10581</v>
+        <v>24290</v>
       </c>
       <c r="L90" s="32" t="n">
         <v>0</v>
@@ -13416,26 +13416,26 @@
         </is>
       </c>
       <c r="D91" s="15" t="n">
-        <v>355382.2</v>
+        <v>778101.22</v>
       </c>
       <c r="E91" s="15" t="n">
-        <v>479145.76</v>
+        <v>2146423.35</v>
       </c>
       <c r="F91" s="16" t="n">
-        <v>0.4163</v>
+        <v>-0.0916</v>
       </c>
       <c r="G91" s="16" t="n">
-        <v>0.3553</v>
+        <v>-0.1587</v>
       </c>
       <c r="H91" s="16" t="n"/>
       <c r="I91" s="16" t="n">
-        <v>0.0491</v>
+        <v>0.0888</v>
       </c>
       <c r="J91" s="19" t="n">
-        <v>11771</v>
+        <v>25911</v>
       </c>
       <c r="K91" s="19" t="n">
-        <v>15177</v>
+        <v>33752</v>
       </c>
       <c r="L91" s="31" t="n">
         <v>0</v>
@@ -13458,26 +13458,26 @@
         </is>
       </c>
       <c r="D92" s="9" t="n">
-        <v>227131.85</v>
+        <v>471584.66</v>
       </c>
       <c r="E92" s="9" t="n">
-        <v>679181.9300000001</v>
+        <v>2798570.57</v>
       </c>
       <c r="F92" s="10" t="n">
-        <v>0.5968</v>
+        <v>-0.1081</v>
       </c>
       <c r="G92" s="10" t="n">
-        <v>0.5305</v>
+        <v>-0.1787</v>
       </c>
       <c r="H92" s="10" t="n"/>
       <c r="I92" s="10" t="n">
-        <v>0.0292</v>
+        <v>0.0534</v>
       </c>
       <c r="J92" s="13" t="n">
-        <v>11268</v>
+        <v>23751</v>
       </c>
       <c r="K92" s="13" t="n">
-        <v>14037</v>
+        <v>30322</v>
       </c>
       <c r="L92" s="32" t="n">
         <v>0</v>
@@ -14886,26 +14886,26 @@
         </is>
       </c>
       <c r="D126" s="9" t="n">
-        <v>977439.04</v>
+        <v>1792564.57</v>
       </c>
       <c r="E126" s="9" t="n">
-        <v>1986991.04</v>
+        <v>3293728.48</v>
       </c>
       <c r="F126" s="10" t="n">
-        <v>0.509</v>
+        <v>0.4267</v>
       </c>
       <c r="G126" s="10" t="n">
-        <v>0.4564</v>
+        <v>0.3738</v>
       </c>
       <c r="H126" s="10" t="n"/>
       <c r="I126" s="10" t="n">
-        <v>0.0379</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="J126" s="13" t="n">
-        <v>23254</v>
+        <v>32859</v>
       </c>
       <c r="K126" s="13" t="n">
-        <v>52318</v>
+        <v>83660</v>
       </c>
       <c r="L126" s="32" t="n">
         <v>0</v>
@@ -17364,26 +17364,26 @@
         </is>
       </c>
       <c r="D185" s="15" t="n">
-        <v>139897.04</v>
+        <v>157135.21</v>
       </c>
       <c r="E185" s="15" t="n">
-        <v>637964.03</v>
+        <v>680642.9</v>
       </c>
       <c r="F185" s="16" t="n">
-        <v>1.0178</v>
+        <v>1.0167</v>
       </c>
       <c r="G185" s="16" t="n">
-        <v>0.9464</v>
+        <v>0.9456</v>
       </c>
       <c r="H185" s="16" t="n"/>
       <c r="I185" s="16" t="n">
         <v>0.0003</v>
       </c>
       <c r="J185" s="19" t="n">
-        <v>10011</v>
+        <v>11716</v>
       </c>
       <c r="K185" s="19" t="n">
-        <v>22444</v>
+        <v>24628</v>
       </c>
       <c r="L185" s="31" t="n">
         <v>0</v>
@@ -17406,26 +17406,26 @@
         </is>
       </c>
       <c r="D186" s="9" t="n">
-        <v>482276.1</v>
+        <v>1055218.31</v>
       </c>
       <c r="E186" s="9" t="n">
-        <v>42284.94</v>
+        <v>694021.84</v>
       </c>
       <c r="F186" s="10" t="n">
-        <v>0.2265</v>
+        <v>0.2034</v>
       </c>
       <c r="G186" s="10" t="n">
-        <v>0.1852</v>
+        <v>0.1572</v>
       </c>
       <c r="H186" s="10" t="n"/>
       <c r="I186" s="10" t="n">
-        <v>0.2377</v>
+        <v>0.2841</v>
       </c>
       <c r="J186" s="13" t="n">
-        <v>2179</v>
+        <v>5125</v>
       </c>
       <c r="K186" s="13" t="n">
-        <v>8047</v>
+        <v>20137</v>
       </c>
       <c r="L186" s="32" t="n">
         <v>0</v>
@@ -17448,26 +17448,26 @@
         </is>
       </c>
       <c r="D187" s="15" t="n">
-        <v>91189.94</v>
+        <v>154050.74</v>
       </c>
       <c r="E187" s="15" t="n">
-        <v>36808.52</v>
+        <v>117821.97</v>
       </c>
       <c r="F187" s="16" t="n">
-        <v>0.47</v>
+        <v>0.4205</v>
       </c>
       <c r="G187" s="16" t="n">
-        <v>0.4217</v>
+        <v>0.3692</v>
       </c>
       <c r="H187" s="16" t="n"/>
       <c r="I187" s="16" t="n">
-        <v>0.0992</v>
+        <v>0.1381</v>
       </c>
       <c r="J187" s="19" t="n">
-        <v>1724</v>
+        <v>3171</v>
       </c>
       <c r="K187" s="19" t="n">
-        <v>2451</v>
+        <v>4624</v>
       </c>
       <c r="L187" s="31" t="n">
         <v>0</v>
@@ -17490,26 +17490,26 @@
         </is>
       </c>
       <c r="D188" s="9" t="n">
-        <v>77614.25</v>
+        <v>154440.54</v>
       </c>
       <c r="E188" s="9" t="n">
-        <v>51545.5</v>
+        <v>137558.5</v>
       </c>
       <c r="F188" s="10" t="n">
-        <v>0.4579</v>
+        <v>0.5836</v>
       </c>
       <c r="G188" s="10" t="n">
-        <v>0.3993</v>
+        <v>0.5265</v>
       </c>
       <c r="H188" s="10" t="n"/>
       <c r="I188" s="10" t="n">
-        <v>0.0572</v>
+        <v>0.0774</v>
       </c>
       <c r="J188" s="13" t="n">
-        <v>2272</v>
+        <v>3967</v>
       </c>
       <c r="K188" s="13" t="n">
-        <v>3025</v>
+        <v>5638</v>
       </c>
       <c r="L188" s="32" t="n">
         <v>0</v>
@@ -17532,26 +17532,26 @@
         </is>
       </c>
       <c r="D189" s="15" t="n">
-        <v>47610.16</v>
+        <v>73402.27</v>
       </c>
       <c r="E189" s="15" t="n">
-        <v>49136.52</v>
+        <v>122618.92</v>
       </c>
       <c r="F189" s="16" t="n">
-        <v>0.82</v>
+        <v>0.6366000000000001</v>
       </c>
       <c r="G189" s="16" t="n">
-        <v>0.7556</v>
+        <v>0.5737</v>
       </c>
       <c r="H189" s="16" t="n"/>
       <c r="I189" s="16" t="n">
-        <v>0.0175</v>
+        <v>0.0288</v>
       </c>
       <c r="J189" s="19" t="n">
-        <v>1428</v>
+        <v>1877</v>
       </c>
       <c r="K189" s="19" t="n">
-        <v>2044</v>
+        <v>2687</v>
       </c>
       <c r="L189" s="31" t="n">
         <v>0</v>
@@ -17574,26 +17574,26 @@
         </is>
       </c>
       <c r="D190" s="9" t="n">
-        <v>62444.56</v>
+        <v>79146.7</v>
       </c>
       <c r="E190" s="9" t="n">
-        <v>193835.69</v>
+        <v>219614.5</v>
       </c>
       <c r="F190" s="10" t="n">
-        <v>0.8611</v>
+        <v>0.8783</v>
       </c>
       <c r="G190" s="10" t="n">
-        <v>0.7939000000000001</v>
+        <v>0.8117</v>
       </c>
       <c r="H190" s="10" t="n"/>
       <c r="I190" s="10" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.012</v>
       </c>
       <c r="J190" s="13" t="n">
-        <v>3111</v>
+        <v>3906</v>
       </c>
       <c r="K190" s="13" t="n">
-        <v>4113</v>
+        <v>5346</v>
       </c>
       <c r="L190" s="32" t="n">
         <v>0</v>
@@ -17616,26 +17616,26 @@
         </is>
       </c>
       <c r="D191" s="15" t="n">
-        <v>76406.99000000001</v>
+        <v>119170.8</v>
       </c>
       <c r="E191" s="15" t="n">
-        <v>975415.85</v>
+        <v>1321449.86</v>
       </c>
       <c r="F191" s="16" t="n">
-        <v>0.9772</v>
+        <v>1.0021</v>
       </c>
       <c r="G191" s="16" t="n">
-        <v>0.9086</v>
+        <v>0.9328</v>
       </c>
       <c r="H191" s="16" t="n"/>
       <c r="I191" s="16" t="n">
-        <v>0.0024</v>
+        <v>0.0029</v>
       </c>
       <c r="J191" s="19" t="n">
-        <v>2529</v>
+        <v>3097</v>
       </c>
       <c r="K191" s="19" t="n">
-        <v>10194</v>
+        <v>20600</v>
       </c>
       <c r="L191" s="31" t="n">
         <v>0</v>
@@ -18162,26 +18162,26 @@
         </is>
       </c>
       <c r="D204" s="9" t="n">
-        <v>2754817.64</v>
+        <v>4785450.27</v>
       </c>
       <c r="E204" s="9" t="n">
-        <v>3284931.92</v>
+        <v>6490799.19</v>
       </c>
       <c r="F204" s="10" t="n">
-        <v>0.4156</v>
+        <v>0.3278</v>
       </c>
       <c r="G204" s="10" t="n">
-        <v>0.3592</v>
+        <v>0.2718</v>
       </c>
       <c r="H204" s="10" t="n"/>
       <c r="I204" s="10" t="n">
-        <v>0.0819</v>
+        <v>0.0771</v>
       </c>
       <c r="J204" s="13" t="n">
-        <v>62375</v>
+        <v>105146</v>
       </c>
       <c r="K204" s="13" t="n">
-        <v>129598</v>
+        <v>209674</v>
       </c>
       <c r="L204" s="32" t="n">
         <v>0</v>
@@ -21732,26 +21732,26 @@
         </is>
       </c>
       <c r="D289" s="15" t="n">
-        <v>93326.35000000001</v>
+        <v>192624.19</v>
       </c>
       <c r="E289" s="15" t="n">
-        <v>241483.01</v>
+        <v>552013.54</v>
       </c>
       <c r="F289" s="16" t="n">
-        <v>0.4366</v>
+        <v>0.3029</v>
       </c>
       <c r="G289" s="16" t="n">
-        <v>0.4023</v>
+        <v>0.2743</v>
       </c>
       <c r="H289" s="16" t="n"/>
       <c r="I289" s="16" t="n">
-        <v>0.0123</v>
+        <v>0.0175</v>
       </c>
       <c r="J289" s="19" t="n">
-        <v>3898</v>
+        <v>6643</v>
       </c>
       <c r="K289" s="19" t="n">
-        <v>5968</v>
+        <v>10104</v>
       </c>
       <c r="L289" s="31" t="n">
         <v>0</v>
@@ -21774,26 +21774,26 @@
         </is>
       </c>
       <c r="D290" s="9" t="n">
-        <v>1041133.36</v>
+        <v>2014435.94</v>
       </c>
       <c r="E290" s="9" t="n">
-        <v>290888.85</v>
+        <v>921366.96</v>
       </c>
       <c r="F290" s="10" t="n">
-        <v>0.3241</v>
+        <v>0.187</v>
       </c>
       <c r="G290" s="10" t="n">
-        <v>0.2753</v>
+        <v>0.1366</v>
       </c>
       <c r="H290" s="10" t="n"/>
       <c r="I290" s="10" t="n">
-        <v>0.2297</v>
+        <v>0.211</v>
       </c>
       <c r="J290" s="13" t="n">
-        <v>6133</v>
+        <v>10294</v>
       </c>
       <c r="K290" s="13" t="n">
-        <v>26276</v>
+        <v>50520</v>
       </c>
       <c r="L290" s="32" t="n">
         <v>0</v>
@@ -21816,26 +21816,26 @@
         </is>
       </c>
       <c r="D291" s="15" t="n">
-        <v>521046.11</v>
+        <v>860991.77</v>
       </c>
       <c r="E291" s="15" t="n">
-        <v>273595.5</v>
+        <v>893154.97</v>
       </c>
       <c r="F291" s="16" t="n">
-        <v>0.2446</v>
+        <v>0.1862</v>
       </c>
       <c r="G291" s="16" t="n">
-        <v>0.1885</v>
+        <v>0.1291</v>
       </c>
       <c r="H291" s="16" t="n"/>
       <c r="I291" s="16" t="n">
-        <v>0.158</v>
+        <v>0.1483</v>
       </c>
       <c r="J291" s="19" t="n">
-        <v>9574</v>
+        <v>16888</v>
       </c>
       <c r="K291" s="19" t="n">
-        <v>21602</v>
+        <v>34814</v>
       </c>
       <c r="L291" s="31" t="n">
         <v>0</v>
@@ -21858,26 +21858,26 @@
         </is>
       </c>
       <c r="D292" s="9" t="n">
-        <v>417887.68</v>
+        <v>649130.54</v>
       </c>
       <c r="E292" s="9" t="n">
-        <v>403469.06</v>
+        <v>837729.29</v>
       </c>
       <c r="F292" s="10" t="n">
-        <v>0.3556</v>
+        <v>0.3584</v>
       </c>
       <c r="G292" s="10" t="n">
-        <v>0.2945</v>
+        <v>0.2963</v>
       </c>
       <c r="H292" s="10" t="n"/>
       <c r="I292" s="10" t="n">
-        <v>0.1071</v>
+        <v>0.0959</v>
       </c>
       <c r="J292" s="13" t="n">
-        <v>10280</v>
+        <v>17696</v>
       </c>
       <c r="K292" s="13" t="n">
-        <v>17631</v>
+        <v>28276</v>
       </c>
       <c r="L292" s="32" t="n">
         <v>0</v>
@@ -21900,26 +21900,26 @@
         </is>
       </c>
       <c r="D293" s="15" t="n">
-        <v>239799.3</v>
+        <v>381253.12</v>
       </c>
       <c r="E293" s="15" t="n">
-        <v>286347.52</v>
+        <v>568827.17</v>
       </c>
       <c r="F293" s="16" t="n">
-        <v>0.6019</v>
+        <v>0.4968</v>
       </c>
       <c r="G293" s="16" t="n">
-        <v>0.5359</v>
+        <v>0.431</v>
       </c>
       <c r="H293" s="16" t="n"/>
       <c r="I293" s="16" t="n">
-        <v>0.0612</v>
+        <v>0.057</v>
       </c>
       <c r="J293" s="19" t="n">
-        <v>9036</v>
+        <v>15221</v>
       </c>
       <c r="K293" s="19" t="n">
-        <v>12493</v>
+        <v>20365</v>
       </c>
       <c r="L293" s="31" t="n">
         <v>0</v>
@@ -21942,26 +21942,26 @@
         </is>
       </c>
       <c r="D294" s="9" t="n">
-        <v>252301.08</v>
+        <v>403444.29</v>
       </c>
       <c r="E294" s="9" t="n">
-        <v>629128.87</v>
+        <v>1092506.3</v>
       </c>
       <c r="F294" s="10" t="n">
-        <v>0.7124</v>
+        <v>0.7482</v>
       </c>
       <c r="G294" s="10" t="n">
-        <v>0.6432</v>
+        <v>0.6802</v>
       </c>
       <c r="H294" s="10" t="n"/>
       <c r="I294" s="10" t="n">
-        <v>0.0299</v>
+        <v>0.0271</v>
       </c>
       <c r="J294" s="13" t="n">
-        <v>13514</v>
+        <v>22384</v>
       </c>
       <c r="K294" s="13" t="n">
-        <v>18704</v>
+        <v>29546</v>
       </c>
       <c r="L294" s="32" t="n">
         <v>0</v>
@@ -21984,26 +21984,26 @@
         </is>
       </c>
       <c r="D295" s="15" t="n">
-        <v>189323.77</v>
+        <v>283570.42</v>
       </c>
       <c r="E295" s="15" t="n">
-        <v>1160019.12</v>
+        <v>1625200.97</v>
       </c>
       <c r="F295" s="16" t="n">
-        <v>0.8794</v>
+        <v>0.8794999999999999</v>
       </c>
       <c r="G295" s="16" t="n">
-        <v>0.8094</v>
+        <v>0.8126</v>
       </c>
       <c r="H295" s="16" t="n"/>
       <c r="I295" s="16" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.0092</v>
       </c>
       <c r="J295" s="19" t="n">
-        <v>9940</v>
+        <v>16020</v>
       </c>
       <c r="K295" s="19" t="n">
-        <v>26924</v>
+        <v>36049</v>
       </c>
       <c r="L295" s="31" t="n">
         <v>0</v>
@@ -22740,26 +22740,26 @@
         </is>
       </c>
       <c r="D313" s="15" t="n">
-        <v>16036559.93</v>
+        <v>31759806.78</v>
       </c>
       <c r="E313" s="15" t="n">
-        <v>20607452.17</v>
+        <v>43443488.49</v>
       </c>
       <c r="F313" s="16" t="n">
-        <v>0.1201</v>
+        <v>-0.0539</v>
       </c>
       <c r="G313" s="16" t="n">
-        <v>0.06519999999999999</v>
+        <v>-0.1101</v>
       </c>
       <c r="H313" s="16" t="n"/>
       <c r="I313" s="16" t="n">
-        <v>0.1355</v>
+        <v>0.1456</v>
       </c>
       <c r="J313" s="19" t="n">
-        <v>339393</v>
+        <v>706454</v>
       </c>
       <c r="K313" s="19" t="n">
-        <v>754985</v>
+        <v>1490895</v>
       </c>
       <c r="L313" s="31" t="n">
         <v>0</v>
@@ -27612,26 +27612,26 @@
         </is>
       </c>
       <c r="D429" s="15" t="n">
-        <v>1358257.72</v>
+        <v>3235977.62</v>
       </c>
       <c r="E429" s="15" t="n">
-        <v>2889627.21</v>
+        <v>11325204.28</v>
       </c>
       <c r="F429" s="16" t="n">
-        <v>-0.4511</v>
+        <v>-0.0028</v>
       </c>
       <c r="G429" s="16" t="n">
-        <v>-0.5177</v>
+        <v>-0.073</v>
       </c>
       <c r="H429" s="16" t="n"/>
       <c r="I429" s="16" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.0633</v>
       </c>
       <c r="J429" s="19" t="n">
-        <v>97517</v>
+        <v>219326</v>
       </c>
       <c r="K429" s="19" t="n">
-        <v>174244</v>
+        <v>444890</v>
       </c>
       <c r="L429" s="31" t="n">
         <v>0</v>
@@ -27654,26 +27654,26 @@
         </is>
       </c>
       <c r="D430" s="9" t="n">
-        <v>6341223.32</v>
+        <v>11918111.23</v>
       </c>
       <c r="E430" s="9" t="n">
-        <v>3377528.75</v>
+        <v>6688723.39</v>
       </c>
       <c r="F430" s="10" t="n">
-        <v>0.0286</v>
+        <v>-0.0449</v>
       </c>
       <c r="G430" s="10" t="n">
-        <v>-0.0201</v>
+        <v>-0.0944</v>
       </c>
       <c r="H430" s="10" t="n"/>
       <c r="I430" s="10" t="n">
-        <v>0.3092</v>
+        <v>0.3242</v>
       </c>
       <c r="J430" s="13" t="n">
-        <v>27823</v>
+        <v>54342</v>
       </c>
       <c r="K430" s="13" t="n">
-        <v>106899</v>
+        <v>197793</v>
       </c>
       <c r="L430" s="32" t="n">
         <v>0</v>
@@ -27696,26 +27696,26 @@
         </is>
       </c>
       <c r="D431" s="15" t="n">
-        <v>2631797.18</v>
+        <v>5286459.84</v>
       </c>
       <c r="E431" s="15" t="n">
-        <v>1964228.9</v>
+        <v>4081132.53</v>
       </c>
       <c r="F431" s="16" t="n">
-        <v>0.1953</v>
+        <v>-0.0456</v>
       </c>
       <c r="G431" s="16" t="n">
-        <v>0.1439</v>
+        <v>-0.0973</v>
       </c>
       <c r="H431" s="16" t="n"/>
       <c r="I431" s="16" t="n">
-        <v>0.2152</v>
+        <v>0.2405</v>
       </c>
       <c r="J431" s="19" t="n">
-        <v>35652</v>
+        <v>70748</v>
       </c>
       <c r="K431" s="19" t="n">
-        <v>79581</v>
+        <v>153789</v>
       </c>
       <c r="L431" s="31" t="n">
         <v>0</v>
@@ -27738,26 +27738,26 @@
         </is>
       </c>
       <c r="D432" s="9" t="n">
-        <v>2000251.66</v>
+        <v>3758471.11</v>
       </c>
       <c r="E432" s="9" t="n">
-        <v>1600113.84</v>
+        <v>4239130.46</v>
       </c>
       <c r="F432" s="10" t="n">
-        <v>0.33</v>
+        <v>0.0261</v>
       </c>
       <c r="G432" s="10" t="n">
-        <v>0.2739</v>
+        <v>-0.0314</v>
       </c>
       <c r="H432" s="10" t="n"/>
       <c r="I432" s="10" t="n">
-        <v>0.1715</v>
+        <v>0.1975</v>
       </c>
       <c r="J432" s="13" t="n">
-        <v>41083</v>
+        <v>80610</v>
       </c>
       <c r="K432" s="13" t="n">
-        <v>88141</v>
+        <v>161972</v>
       </c>
       <c r="L432" s="32" t="n">
         <v>0</v>
@@ -27780,26 +27780,26 @@
         </is>
       </c>
       <c r="D433" s="15" t="n">
-        <v>1043121.8</v>
+        <v>2171759.29</v>
       </c>
       <c r="E433" s="15" t="n">
-        <v>1232339.51</v>
+        <v>2492942.93</v>
       </c>
       <c r="F433" s="16" t="n">
-        <v>0.3472</v>
+        <v>-0.0658</v>
       </c>
       <c r="G433" s="16" t="n">
-        <v>0.2873</v>
+        <v>-0.1258</v>
       </c>
       <c r="H433" s="16" t="n"/>
       <c r="I433" s="16" t="n">
-        <v>0.1476</v>
+        <v>0.1743</v>
       </c>
       <c r="J433" s="19" t="n">
-        <v>31035</v>
+        <v>63370</v>
       </c>
       <c r="K433" s="19" t="n">
-        <v>51302</v>
+        <v>102059</v>
       </c>
       <c r="L433" s="31" t="n">
         <v>0</v>
@@ -27822,26 +27822,26 @@
         </is>
       </c>
       <c r="D434" s="9" t="n">
-        <v>1464923.49</v>
+        <v>3038315.55</v>
       </c>
       <c r="E434" s="9" t="n">
-        <v>2763986.32</v>
+        <v>5345961.14</v>
       </c>
       <c r="F434" s="10" t="n">
-        <v>0.3929</v>
+        <v>-0.1452</v>
       </c>
       <c r="G434" s="10" t="n">
-        <v>0.3296</v>
+        <v>-0.2078</v>
       </c>
       <c r="H434" s="10" t="n"/>
       <c r="I434" s="10" t="n">
-        <v>0.1155</v>
+        <v>0.1397</v>
       </c>
       <c r="J434" s="13" t="n">
-        <v>53225</v>
+        <v>109830</v>
       </c>
       <c r="K434" s="13" t="n">
-        <v>116908</v>
+        <v>204735</v>
       </c>
       <c r="L434" s="32" t="n">
         <v>0</v>
@@ -27864,26 +27864,26 @@
         </is>
       </c>
       <c r="D435" s="15" t="n">
-        <v>1196984.74</v>
+        <v>2350712.14</v>
       </c>
       <c r="E435" s="15" t="n">
-        <v>6779627.65</v>
+        <v>9270393.77</v>
       </c>
       <c r="F435" s="16" t="n">
-        <v>0.2058</v>
+        <v>-0.1878</v>
       </c>
       <c r="G435" s="16" t="n">
-        <v>0.1395</v>
+        <v>-0.2549</v>
       </c>
       <c r="H435" s="16" t="n"/>
       <c r="I435" s="16" t="n">
-        <v>0.0983</v>
+        <v>0.111</v>
       </c>
       <c r="J435" s="19" t="n">
-        <v>53058</v>
+        <v>108228</v>
       </c>
       <c r="K435" s="19" t="n">
-        <v>137910</v>
+        <v>225657</v>
       </c>
       <c r="L435" s="31" t="n">
         <v>0</v>
@@ -39226,29 +39226,29 @@
         </is>
       </c>
       <c r="D694" s="9" t="n">
-        <v>13563451.25</v>
+        <v>13569942.05</v>
       </c>
       <c r="E694" s="9" t="n">
-        <v>78801851.91</v>
+        <v>78858814.67</v>
       </c>
       <c r="F694" s="10" t="n">
-        <v>0.2913</v>
+        <v>0.2864</v>
       </c>
       <c r="G694" s="10" t="n">
-        <v>0.2249</v>
+        <v>0.22</v>
       </c>
       <c r="H694" s="10" t="n"/>
       <c r="I694" s="10" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.06909999999999999</v>
       </c>
       <c r="J694" s="13" t="n">
-        <v>485873</v>
+        <v>485923</v>
       </c>
       <c r="K694" s="13" t="n">
-        <v>669361</v>
+        <v>669421</v>
       </c>
       <c r="L694" s="32" t="n">
-        <v>0.5271</v>
+        <v>0.5269</v>
       </c>
     </row>
     <row r="695">
@@ -39268,29 +39268,29 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>3257626.8</v>
+        <v>3434190.46</v>
       </c>
       <c r="E695" s="15" t="n">
-        <v>24955545.1</v>
+        <v>26899878.68</v>
       </c>
       <c r="F695" s="16" t="n">
-        <v>0.1703</v>
+        <v>0.1941</v>
       </c>
       <c r="G695" s="16" t="n">
-        <v>0.102</v>
+        <v>0.1253</v>
       </c>
       <c r="H695" s="16" t="n"/>
       <c r="I695" s="16" t="n">
-        <v>0.0526</v>
+        <v>0.0507</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>150253</v>
+        <v>162352</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>202545</v>
+        <v>221048</v>
       </c>
       <c r="L695" s="31" t="n">
-        <v>0.5822000000000001</v>
+        <v>0.5554</v>
       </c>
     </row>
     <row r="696">
@@ -42838,26 +42838,26 @@
         </is>
       </c>
       <c r="D780" s="9" t="n">
-        <v>3103441.87</v>
+        <v>3104067.63</v>
       </c>
       <c r="E780" s="9" t="n">
-        <v>49927972.85</v>
+        <v>49984169.9</v>
       </c>
       <c r="F780" s="10" t="n">
-        <v>0.5414</v>
+        <v>0.5223</v>
       </c>
       <c r="G780" s="10" t="n">
-        <v>0.4611</v>
+        <v>0.4417</v>
       </c>
       <c r="H780" s="10" t="n"/>
       <c r="I780" s="10" t="n">
         <v>0.0184</v>
       </c>
       <c r="J780" s="13" t="n">
-        <v>250254</v>
+        <v>250271</v>
       </c>
       <c r="K780" s="13" t="n">
-        <v>337807</v>
+        <v>337831</v>
       </c>
       <c r="L780" s="32" t="n">
         <v>0.572</v>
@@ -42922,26 +42922,26 @@
         </is>
       </c>
       <c r="D782" s="9" t="n">
-        <v>1956213.9</v>
+        <v>1956433.89</v>
       </c>
       <c r="E782" s="9" t="n">
-        <v>2022852.78</v>
+        <v>2022982.02</v>
       </c>
       <c r="F782" s="10" t="n">
-        <v>0.1367</v>
+        <v>0.1366</v>
       </c>
       <c r="G782" s="10" t="n">
-        <v>0.0822</v>
+        <v>0.08210000000000001</v>
       </c>
       <c r="H782" s="10" t="n"/>
       <c r="I782" s="10" t="n">
-        <v>0.2456</v>
+        <v>0.2458</v>
       </c>
       <c r="J782" s="13" t="n">
-        <v>21012</v>
+        <v>21021</v>
       </c>
       <c r="K782" s="13" t="n">
-        <v>38570</v>
+        <v>38580</v>
       </c>
       <c r="L782" s="32" t="n">
         <v>0.5303</v>
@@ -42964,29 +42964,29 @@
         </is>
       </c>
       <c r="D783" s="15" t="n">
-        <v>1551374.54</v>
+        <v>1551860.24</v>
       </c>
       <c r="E783" s="15" t="n">
-        <v>2907061.32</v>
+        <v>2907294.15</v>
       </c>
       <c r="F783" s="16" t="n">
-        <v>0.1736</v>
+        <v>0.1732</v>
       </c>
       <c r="G783" s="16" t="n">
-        <v>0.1096</v>
+        <v>0.1092</v>
       </c>
       <c r="H783" s="16" t="n"/>
       <c r="I783" s="16" t="n">
-        <v>0.1838</v>
+        <v>0.184</v>
       </c>
       <c r="J783" s="19" t="n">
-        <v>28066</v>
+        <v>28072</v>
       </c>
       <c r="K783" s="19" t="n">
-        <v>41180</v>
+        <v>41186</v>
       </c>
       <c r="L783" s="31" t="n">
-        <v>0.5453</v>
+        <v>0.5454</v>
       </c>
     </row>
     <row r="784">
@@ -43006,29 +43006,29 @@
         </is>
       </c>
       <c r="D784" s="9" t="n">
-        <v>1260003.64</v>
+        <v>1260210.84</v>
       </c>
       <c r="E784" s="9" t="n">
-        <v>3415703.94</v>
+        <v>3415971.86</v>
       </c>
       <c r="F784" s="10" t="n">
-        <v>0.1871</v>
+        <v>0.1867</v>
       </c>
       <c r="G784" s="10" t="n">
-        <v>0.1195</v>
+        <v>0.1191</v>
       </c>
       <c r="H784" s="10" t="n"/>
       <c r="I784" s="10" t="n">
-        <v>0.1445</v>
+        <v>0.1446</v>
       </c>
       <c r="J784" s="13" t="n">
-        <v>30287</v>
+        <v>30295</v>
       </c>
       <c r="K784" s="13" t="n">
-        <v>40881</v>
+        <v>40889</v>
       </c>
       <c r="L784" s="32" t="n">
-        <v>0.5073</v>
+        <v>0.5074</v>
       </c>
     </row>
     <row r="785">
@@ -43048,29 +43048,29 @@
         </is>
       </c>
       <c r="D785" s="15" t="n">
-        <v>2012892.34</v>
+        <v>2017783.37</v>
       </c>
       <c r="E785" s="15" t="n">
-        <v>7498326.62</v>
+        <v>7498334.28</v>
       </c>
       <c r="F785" s="16" t="n">
-        <v>0.1845</v>
+        <v>0.182</v>
       </c>
       <c r="G785" s="16" t="n">
-        <v>0.1149</v>
+        <v>0.1124</v>
       </c>
       <c r="H785" s="16" t="n"/>
       <c r="I785" s="16" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.0982</v>
       </c>
       <c r="J785" s="19" t="n">
-        <v>64325</v>
+        <v>64329</v>
       </c>
       <c r="K785" s="19" t="n">
-        <v>82648</v>
+        <v>82652</v>
       </c>
       <c r="L785" s="31" t="n">
-        <v>0.509</v>
+        <v>0.5078</v>
       </c>
     </row>
     <row r="786">
@@ -43090,26 +43090,26 @@
         </is>
       </c>
       <c r="D786" s="9" t="n">
-        <v>1762300.44</v>
+        <v>1762361.57</v>
       </c>
       <c r="E786" s="9" t="n">
-        <v>11981794.5</v>
+        <v>11981922.57</v>
       </c>
       <c r="F786" s="10" t="n">
-        <v>0.4109</v>
+        <v>0.4103</v>
       </c>
       <c r="G786" s="10" t="n">
-        <v>0.3332</v>
+        <v>0.3326</v>
       </c>
       <c r="H786" s="10" t="n"/>
       <c r="I786" s="10" t="n">
         <v>0.0572</v>
       </c>
       <c r="J786" s="13" t="n">
-        <v>82053</v>
+        <v>82059</v>
       </c>
       <c r="K786" s="13" t="n">
-        <v>102813</v>
+        <v>102821</v>
       </c>
       <c r="L786" s="32" t="n">
         <v>0.5152</v>
@@ -43132,29 +43132,29 @@
         </is>
       </c>
       <c r="D787" s="15" t="n">
-        <v>892452.01</v>
+        <v>994063.02</v>
       </c>
       <c r="E787" s="15" t="n">
-        <v>17284316.8</v>
+        <v>18962832.56</v>
       </c>
       <c r="F787" s="16" t="n">
-        <v>0.6076</v>
+        <v>0.6096</v>
       </c>
       <c r="G787" s="16" t="n">
-        <v>0.5272</v>
+        <v>0.5288</v>
       </c>
       <c r="H787" s="16" t="n"/>
       <c r="I787" s="16" t="n">
-        <v>0.0167</v>
+        <v>0.0169</v>
       </c>
       <c r="J787" s="19" t="n">
-        <v>87446</v>
+        <v>96074</v>
       </c>
       <c r="K787" s="19" t="n">
-        <v>113521</v>
+        <v>127865</v>
       </c>
       <c r="L787" s="31" t="n">
-        <v>0.5083</v>
+        <v>0.4599</v>
       </c>
     </row>
     <row r="788">
@@ -43174,29 +43174,29 @@
         </is>
       </c>
       <c r="D788" s="9" t="n">
-        <v>449189.44</v>
+        <v>454072.95</v>
       </c>
       <c r="E788" s="9" t="n">
-        <v>699850.01</v>
+        <v>700562.28</v>
       </c>
       <c r="F788" s="10" t="n">
-        <v>-0.6856</v>
+        <v>-0.6693</v>
       </c>
       <c r="G788" s="10" t="n">
-        <v>-0.7339</v>
+        <v>-0.7177</v>
       </c>
       <c r="H788" s="10" t="n"/>
       <c r="I788" s="10" t="n">
-        <v>0.3582</v>
+        <v>0.3463</v>
       </c>
       <c r="J788" s="13" t="n">
-        <v>1823</v>
+        <v>1897</v>
       </c>
       <c r="K788" s="13" t="n">
-        <v>4686</v>
+        <v>4777</v>
       </c>
       <c r="L788" s="32" t="n">
-        <v>0.5084</v>
+        <v>0.5041</v>
       </c>
     </row>
     <row r="789">
@@ -43216,29 +43216,29 @@
         </is>
       </c>
       <c r="D789" s="15" t="n">
-        <v>408345.56</v>
+        <v>414325.32</v>
       </c>
       <c r="E789" s="15" t="n">
-        <v>278854.5</v>
+        <v>284326.57</v>
       </c>
       <c r="F789" s="16" t="n">
-        <v>-0.0407</v>
+        <v>-0.0328</v>
       </c>
       <c r="G789" s="16" t="n">
-        <v>-0.0887</v>
+        <v>-0.08110000000000001</v>
       </c>
       <c r="H789" s="16" t="n"/>
       <c r="I789" s="16" t="n">
-        <v>0.2433</v>
+        <v>0.2365</v>
       </c>
       <c r="J789" s="19" t="n">
-        <v>4279</v>
+        <v>4470</v>
       </c>
       <c r="K789" s="19" t="n">
-        <v>7467</v>
+        <v>7693</v>
       </c>
       <c r="L789" s="31" t="n">
-        <v>0.6884</v>
+        <v>0.6821</v>
       </c>
     </row>
     <row r="790">
@@ -43258,29 +43258,29 @@
         </is>
       </c>
       <c r="D790" s="9" t="n">
-        <v>331577.13</v>
+        <v>336941.74</v>
       </c>
       <c r="E790" s="9" t="n">
-        <v>557703.17</v>
+        <v>562369.47</v>
       </c>
       <c r="F790" s="10" t="n">
-        <v>0.1539</v>
+        <v>0.1593</v>
       </c>
       <c r="G790" s="10" t="n">
-        <v>0.0912</v>
+        <v>0.09660000000000001</v>
       </c>
       <c r="H790" s="10" t="n"/>
       <c r="I790" s="10" t="n">
-        <v>0.1703</v>
+        <v>0.1659</v>
       </c>
       <c r="J790" s="13" t="n">
-        <v>6294</v>
+        <v>6546</v>
       </c>
       <c r="K790" s="13" t="n">
-        <v>8943</v>
+        <v>9242</v>
       </c>
       <c r="L790" s="32" t="n">
-        <v>0.6221</v>
+        <v>0.6136</v>
       </c>
     </row>
     <row r="791">
@@ -43300,29 +43300,29 @@
         </is>
       </c>
       <c r="D791" s="15" t="n">
-        <v>306468.65</v>
+        <v>317188.44</v>
       </c>
       <c r="E791" s="15" t="n">
-        <v>712748.6899999999</v>
+        <v>739755.8100000001</v>
       </c>
       <c r="F791" s="16" t="n">
-        <v>0.1804</v>
+        <v>0.1999</v>
       </c>
       <c r="G791" s="16" t="n">
-        <v>0.1103</v>
+        <v>0.1298</v>
       </c>
       <c r="H791" s="16" t="n"/>
       <c r="I791" s="16" t="n">
-        <v>0.1249</v>
+        <v>0.1222</v>
       </c>
       <c r="J791" s="19" t="n">
-        <v>7782</v>
+        <v>8176</v>
       </c>
       <c r="K791" s="19" t="n">
-        <v>14749</v>
+        <v>15205</v>
       </c>
       <c r="L791" s="31" t="n">
-        <v>0.7181999999999999</v>
+        <v>0.695</v>
       </c>
     </row>
     <row r="792">
@@ -43342,29 +43342,29 @@
         </is>
       </c>
       <c r="D792" s="9" t="n">
-        <v>454981.88</v>
+        <v>472394.63</v>
       </c>
       <c r="E792" s="9" t="n">
-        <v>1818681.79</v>
+        <v>1901924.58</v>
       </c>
       <c r="F792" s="10" t="n">
-        <v>0.2041</v>
+        <v>0.2224</v>
       </c>
       <c r="G792" s="10" t="n">
-        <v>0.1302</v>
+        <v>0.1483</v>
       </c>
       <c r="H792" s="10" t="n"/>
       <c r="I792" s="10" t="n">
-        <v>0.0801</v>
+        <v>0.07779999999999999</v>
       </c>
       <c r="J792" s="13" t="n">
-        <v>17944</v>
+        <v>18865</v>
       </c>
       <c r="K792" s="13" t="n">
-        <v>22628</v>
+        <v>23674</v>
       </c>
       <c r="L792" s="32" t="n">
-        <v>0.5926</v>
+        <v>0.5726</v>
       </c>
     </row>
     <row r="793">
@@ -43384,29 +43384,29 @@
         </is>
       </c>
       <c r="D793" s="15" t="n">
-        <v>414612.13</v>
+        <v>445204.36</v>
       </c>
       <c r="E793" s="15" t="n">
-        <v>3603390.13</v>
+        <v>3748107.41</v>
       </c>
       <c r="F793" s="16" t="n">
-        <v>0.3325</v>
+        <v>0.3507</v>
       </c>
       <c r="G793" s="16" t="n">
-        <v>0.252</v>
+        <v>0.2702</v>
       </c>
       <c r="H793" s="16" t="n"/>
       <c r="I793" s="16" t="n">
-        <v>0.0511</v>
+        <v>0.051</v>
       </c>
       <c r="J793" s="19" t="n">
-        <v>24685</v>
+        <v>26324</v>
       </c>
       <c r="K793" s="19" t="n">
-        <v>30551</v>
+        <v>32592</v>
       </c>
       <c r="L793" s="31" t="n">
-        <v>0.5728</v>
+        <v>0.5412</v>
       </c>
     </row>
     <row r="794">
@@ -44308,29 +44308,29 @@
         </is>
       </c>
       <c r="D815" s="15" t="n">
-        <v>21656843.23</v>
+        <v>21671735</v>
       </c>
       <c r="E815" s="15" t="n">
-        <v>54661492.13</v>
+        <v>54663866.25</v>
       </c>
       <c r="F815" s="16" t="n">
-        <v>0.1394</v>
+        <v>0.1383</v>
       </c>
       <c r="G815" s="16" t="n">
-        <v>0.079</v>
+        <v>0.0779</v>
       </c>
       <c r="H815" s="16" t="n"/>
       <c r="I815" s="16" t="n">
-        <v>0.09429999999999999</v>
+        <v>0.0945</v>
       </c>
       <c r="J815" s="19" t="n">
-        <v>399853</v>
+        <v>399942</v>
       </c>
       <c r="K815" s="19" t="n">
-        <v>643601</v>
+        <v>643719</v>
       </c>
       <c r="L815" s="31" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.5633</v>
       </c>
     </row>
     <row r="816">
@@ -44350,29 +44350,29 @@
         </is>
       </c>
       <c r="D816" s="9" t="n">
-        <v>9785449.689999999</v>
+        <v>10064034.13</v>
       </c>
       <c r="E816" s="9" t="n">
-        <v>25733893.86</v>
+        <v>26543135.79</v>
       </c>
       <c r="F816" s="10" t="n">
-        <v>0.3582</v>
+        <v>0.3717</v>
       </c>
       <c r="G816" s="10" t="n">
-        <v>0.2993</v>
+        <v>0.3126</v>
       </c>
       <c r="H816" s="10" t="n"/>
       <c r="I816" s="10" t="n">
-        <v>0.0757</v>
+        <v>0.0741</v>
       </c>
       <c r="J816" s="13" t="n">
-        <v>188680</v>
+        <v>195156</v>
       </c>
       <c r="K816" s="13" t="n">
-        <v>349180</v>
+        <v>362605</v>
       </c>
       <c r="L816" s="32" t="n">
-        <v>0.6321</v>
+        <v>0.6153</v>
       </c>
     </row>
     <row r="817">
@@ -50608,29 +50608,29 @@
         </is>
       </c>
       <c r="D965" s="15" t="n">
-        <v>7841310.64</v>
+        <v>7850603.44</v>
       </c>
       <c r="E965" s="15" t="n">
-        <v>6197264.27</v>
+        <v>6198608.33</v>
       </c>
       <c r="F965" s="16" t="n">
-        <v>-0.0757</v>
+        <v>-0.07679999999999999</v>
       </c>
       <c r="G965" s="16" t="n">
-        <v>-0.1263</v>
+        <v>-0.1274</v>
       </c>
       <c r="H965" s="16" t="n"/>
       <c r="I965" s="16" t="n">
-        <v>0.3241</v>
+        <v>0.3252</v>
       </c>
       <c r="J965" s="19" t="n">
-        <v>19738</v>
+        <v>19788</v>
       </c>
       <c r="K965" s="19" t="n">
-        <v>88744</v>
+        <v>88823</v>
       </c>
       <c r="L965" s="31" t="n">
-        <v>0.5279</v>
+        <v>0.5283</v>
       </c>
     </row>
     <row r="966">
@@ -50650,29 +50650,29 @@
         </is>
       </c>
       <c r="D966" s="9" t="n">
-        <v>4010911.74</v>
+        <v>4016377.09</v>
       </c>
       <c r="E966" s="9" t="n">
-        <v>4092724.18</v>
+        <v>4093565.37</v>
       </c>
       <c r="F966" s="10" t="n">
-        <v>0.0199</v>
+        <v>0.0168</v>
       </c>
       <c r="G966" s="10" t="n">
-        <v>-0.0376</v>
+        <v>-0.0407</v>
       </c>
       <c r="H966" s="10" t="n"/>
       <c r="I966" s="10" t="n">
-        <v>0.2397</v>
+        <v>0.2401</v>
       </c>
       <c r="J966" s="13" t="n">
-        <v>36205</v>
+        <v>36226</v>
       </c>
       <c r="K966" s="13" t="n">
-        <v>80011</v>
+        <v>80032</v>
       </c>
       <c r="L966" s="32" t="n">
-        <v>0.5704</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="967">
@@ -50692,10 +50692,10 @@
         </is>
       </c>
       <c r="D967" s="15" t="n">
-        <v>2757629.05</v>
+        <v>2757708.77</v>
       </c>
       <c r="E967" s="15" t="n">
-        <v>3944916.14</v>
+        <v>3945082.83</v>
       </c>
       <c r="F967" s="16" t="n">
         <v>0.2192</v>
@@ -50705,13 +50705,13 @@
       </c>
       <c r="H967" s="16" t="n"/>
       <c r="I967" s="16" t="n">
-        <v>0.1698</v>
+        <v>0.17</v>
       </c>
       <c r="J967" s="19" t="n">
-        <v>42179</v>
+        <v>42192</v>
       </c>
       <c r="K967" s="19" t="n">
-        <v>62149</v>
+        <v>62162</v>
       </c>
       <c r="L967" s="31" t="n">
         <v>0.594</v>
@@ -50734,26 +50734,26 @@
         </is>
       </c>
       <c r="D968" s="9" t="n">
-        <v>1762878.9</v>
+        <v>1762927.13</v>
       </c>
       <c r="E968" s="9" t="n">
-        <v>3831254.67</v>
+        <v>3831272.03</v>
       </c>
       <c r="F968" s="10" t="n">
         <v>0.2432</v>
       </c>
       <c r="G968" s="10" t="n">
-        <v>0.1766</v>
+        <v>0.1765</v>
       </c>
       <c r="H968" s="10" t="n"/>
       <c r="I968" s="10" t="n">
         <v>0.1258</v>
       </c>
       <c r="J968" s="13" t="n">
-        <v>37788</v>
+        <v>37790</v>
       </c>
       <c r="K968" s="13" t="n">
-        <v>52540</v>
+        <v>52542</v>
       </c>
       <c r="L968" s="32" t="n">
         <v>0.5564</v>
@@ -50776,26 +50776,26 @@
         </is>
       </c>
       <c r="D969" s="15" t="n">
-        <v>2145323.38</v>
+        <v>2145329.04</v>
       </c>
       <c r="E969" s="15" t="n">
-        <v>7523568.74</v>
+        <v>7523573.55</v>
       </c>
       <c r="F969" s="16" t="n">
-        <v>0.3416</v>
+        <v>0.3415</v>
       </c>
       <c r="G969" s="16" t="n">
         <v>0.2688</v>
       </c>
       <c r="H969" s="16" t="n"/>
       <c r="I969" s="16" t="n">
-        <v>0.0798</v>
+        <v>0.0799</v>
       </c>
       <c r="J969" s="19" t="n">
-        <v>71904</v>
+        <v>71907</v>
       </c>
       <c r="K969" s="19" t="n">
-        <v>95146</v>
+        <v>95149</v>
       </c>
       <c r="L969" s="31" t="n">
         <v>0.5954</v>
@@ -50860,29 +50860,29 @@
         </is>
       </c>
       <c r="D971" s="15" t="n">
-        <v>822143.49</v>
+        <v>859811.66</v>
       </c>
       <c r="E971" s="15" t="n">
-        <v>9792780.220000001</v>
+        <v>10273208.24</v>
       </c>
       <c r="F971" s="16" t="n">
-        <v>0.7091</v>
+        <v>0.7223000000000001</v>
       </c>
       <c r="G971" s="16" t="n">
-        <v>0.6358</v>
+        <v>0.649</v>
       </c>
       <c r="H971" s="16" t="n"/>
       <c r="I971" s="16" t="n">
-        <v>0.0194</v>
+        <v>0.0189</v>
       </c>
       <c r="J971" s="19" t="n">
-        <v>59470</v>
+        <v>62213</v>
       </c>
       <c r="K971" s="19" t="n">
-        <v>107776</v>
+        <v>111271</v>
       </c>
       <c r="L971" s="31" t="n">
-        <v>0.6428</v>
+        <v>0.6149</v>
       </c>
     </row>
     <row r="972">
@@ -50902,29 +50902,29 @@
         </is>
       </c>
       <c r="D972" s="9" t="n">
-        <v>3098919.71</v>
+        <v>3231531.18</v>
       </c>
       <c r="E972" s="9" t="n">
-        <v>1727684.53</v>
+        <v>1830307.86</v>
       </c>
       <c r="F972" s="10" t="n">
-        <v>0.1849</v>
+        <v>0.209</v>
       </c>
       <c r="G972" s="10" t="n">
-        <v>0.1364</v>
+        <v>0.16</v>
       </c>
       <c r="H972" s="10" t="n"/>
       <c r="I972" s="10" t="n">
-        <v>0.3118</v>
+        <v>0.3032</v>
       </c>
       <c r="J972" s="13" t="n">
-        <v>7621</v>
+        <v>7925</v>
       </c>
       <c r="K972" s="13" t="n">
-        <v>37175</v>
+        <v>37890</v>
       </c>
       <c r="L972" s="32" t="n">
-        <v>0.6946</v>
+        <v>0.6669</v>
       </c>
     </row>
     <row r="973">
@@ -50944,29 +50944,29 @@
         </is>
       </c>
       <c r="D973" s="15" t="n">
-        <v>1893375.46</v>
+        <v>1909008.81</v>
       </c>
       <c r="E973" s="15" t="n">
-        <v>1722796.65</v>
+        <v>1732883.52</v>
       </c>
       <c r="F973" s="16" t="n">
-        <v>0.2911</v>
+        <v>0.2944</v>
       </c>
       <c r="G973" s="16" t="n">
-        <v>0.2368</v>
+        <v>0.24</v>
       </c>
       <c r="H973" s="16" t="n"/>
       <c r="I973" s="16" t="n">
-        <v>0.1983</v>
+        <v>0.1954</v>
       </c>
       <c r="J973" s="19" t="n">
-        <v>15139</v>
+        <v>15546</v>
       </c>
       <c r="K973" s="19" t="n">
-        <v>31640</v>
+        <v>32141</v>
       </c>
       <c r="L973" s="31" t="n">
-        <v>0.5717</v>
+        <v>0.5682</v>
       </c>
     </row>
     <row r="974">
@@ -50986,29 +50986,29 @@
         </is>
       </c>
       <c r="D974" s="9" t="n">
-        <v>1322275.92</v>
+        <v>1335135.71</v>
       </c>
       <c r="E974" s="9" t="n">
-        <v>1750299.99</v>
+        <v>1763738.57</v>
       </c>
       <c r="F974" s="10" t="n">
-        <v>0.3881</v>
+        <v>0.392</v>
       </c>
       <c r="G974" s="10" t="n">
-        <v>0.3269</v>
+        <v>0.3308</v>
       </c>
       <c r="H974" s="10" t="n"/>
       <c r="I974" s="10" t="n">
-        <v>0.1314</v>
+        <v>0.1295</v>
       </c>
       <c r="J974" s="13" t="n">
-        <v>20318</v>
+        <v>20833</v>
       </c>
       <c r="K974" s="13" t="n">
-        <v>35967</v>
+        <v>36552</v>
       </c>
       <c r="L974" s="32" t="n">
-        <v>0.6012999999999999</v>
+        <v>0.5959</v>
       </c>
     </row>
     <row r="975">
@@ -51028,29 +51028,29 @@
         </is>
       </c>
       <c r="D975" s="15" t="n">
-        <v>866172.11</v>
+        <v>885908.73</v>
       </c>
       <c r="E975" s="15" t="n">
-        <v>1899469.56</v>
+        <v>1921867.56</v>
       </c>
       <c r="F975" s="16" t="n">
-        <v>0.4376</v>
+        <v>0.4498</v>
       </c>
       <c r="G975" s="16" t="n">
-        <v>0.3722</v>
+        <v>0.3843</v>
       </c>
       <c r="H975" s="16" t="n"/>
       <c r="I975" s="16" t="n">
-        <v>0.0946</v>
+        <v>0.0934</v>
       </c>
       <c r="J975" s="19" t="n">
-        <v>18006</v>
+        <v>18443</v>
       </c>
       <c r="K975" s="19" t="n">
-        <v>26843</v>
+        <v>27376</v>
       </c>
       <c r="L975" s="31" t="n">
-        <v>0.595</v>
+        <v>0.582</v>
       </c>
     </row>
     <row r="976">
@@ -51070,29 +51070,29 @@
         </is>
       </c>
       <c r="D976" s="9" t="n">
-        <v>1038086.27</v>
+        <v>1060485.01</v>
       </c>
       <c r="E976" s="9" t="n">
-        <v>3147754.11</v>
+        <v>3205507.44</v>
       </c>
       <c r="F976" s="10" t="n">
-        <v>0.4741</v>
+        <v>0.4806</v>
       </c>
       <c r="G976" s="10" t="n">
-        <v>0.4057</v>
+        <v>0.4121</v>
       </c>
       <c r="H976" s="10" t="n"/>
       <c r="I976" s="10" t="n">
-        <v>0.0617</v>
+        <v>0.061</v>
       </c>
       <c r="J976" s="13" t="n">
-        <v>33490</v>
+        <v>34444</v>
       </c>
       <c r="K976" s="13" t="n">
-        <v>47624</v>
+        <v>49253</v>
       </c>
       <c r="L976" s="32" t="n">
-        <v>0.624</v>
+        <v>0.6113</v>
       </c>
     </row>
     <row r="977">
@@ -51112,29 +51112,29 @@
         </is>
       </c>
       <c r="D977" s="15" t="n">
-        <v>744476.73</v>
+        <v>782153.03</v>
       </c>
       <c r="E977" s="15" t="n">
-        <v>5693108.79</v>
+        <v>5815622.59</v>
       </c>
       <c r="F977" s="16" t="n">
-        <v>0.5562</v>
+        <v>0.5768</v>
       </c>
       <c r="G977" s="16" t="n">
-        <v>0.4828</v>
+        <v>0.5034999999999999</v>
       </c>
       <c r="H977" s="16" t="n"/>
       <c r="I977" s="16" t="n">
-        <v>0.0376</v>
+        <v>0.037</v>
       </c>
       <c r="J977" s="19" t="n">
-        <v>34636</v>
+        <v>35752</v>
       </c>
       <c r="K977" s="19" t="n">
-        <v>62155</v>
+        <v>68122</v>
       </c>
       <c r="L977" s="31" t="n">
-        <v>0.6231</v>
+        <v>0.5933</v>
       </c>
     </row>
     <row r="978">
@@ -51574,10 +51574,10 @@
         </is>
       </c>
       <c r="D988" s="9" t="n">
-        <v>6720859.86</v>
+        <v>6721050.91</v>
       </c>
       <c r="E988" s="9" t="n">
-        <v>21398902.89</v>
+        <v>21399159.66</v>
       </c>
       <c r="F988" s="10" t="n">
         <v>0.3926</v>
@@ -51590,10 +51590,10 @@
         <v>0.0594</v>
       </c>
       <c r="J988" s="13" t="n">
-        <v>137657</v>
+        <v>137663</v>
       </c>
       <c r="K988" s="13" t="n">
-        <v>200853</v>
+        <v>200864</v>
       </c>
       <c r="L988" s="32" t="n">
         <v>0.6414</v>
@@ -51616,29 +51616,29 @@
         </is>
       </c>
       <c r="D989" s="15" t="n">
-        <v>544428.1800000001</v>
+        <v>673220.78</v>
       </c>
       <c r="E989" s="15" t="n">
-        <v>2623023.49</v>
+        <v>3292035.57</v>
       </c>
       <c r="F989" s="16" t="n">
-        <v>0.6686</v>
+        <v>0.7238</v>
       </c>
       <c r="G989" s="16" t="n">
-        <v>0.6016</v>
+        <v>0.6559</v>
       </c>
       <c r="H989" s="16" t="n"/>
       <c r="I989" s="16" t="n">
-        <v>0.0242</v>
+        <v>0.0216</v>
       </c>
       <c r="J989" s="19" t="n">
-        <v>18022</v>
+        <v>21405</v>
       </c>
       <c r="K989" s="19" t="n">
-        <v>21431</v>
+        <v>47250</v>
       </c>
       <c r="L989" s="31" t="n">
-        <v>0.3839</v>
+        <v>0.3168</v>
       </c>
     </row>
     <row r="990">
@@ -54682,26 +54682,26 @@
         </is>
       </c>
       <c r="D1062" s="9" t="n">
-        <v>960500.84</v>
+        <v>960545.36</v>
       </c>
       <c r="E1062" s="9" t="n">
-        <v>1049026.46</v>
+        <v>1049058.75</v>
       </c>
       <c r="F1062" s="10" t="n">
-        <v>0.1924</v>
+        <v>0.1923</v>
       </c>
       <c r="G1062" s="10" t="n">
-        <v>0.1353</v>
+        <v>0.1352</v>
       </c>
       <c r="H1062" s="10" t="n"/>
       <c r="I1062" s="10" t="n">
-        <v>0.202</v>
+        <v>0.2022</v>
       </c>
       <c r="J1062" s="13" t="n">
-        <v>8382</v>
+        <v>8384</v>
       </c>
       <c r="K1062" s="13" t="n">
-        <v>15798</v>
+        <v>15805</v>
       </c>
       <c r="L1062" s="32" t="n">
         <v>0.5778</v>
@@ -54724,13 +54724,13 @@
         </is>
       </c>
       <c r="D1063" s="15" t="n">
-        <v>907535.95</v>
+        <v>907559.46</v>
       </c>
       <c r="E1063" s="15" t="n">
-        <v>1452663.41</v>
+        <v>1452887.89</v>
       </c>
       <c r="F1063" s="16" t="n">
-        <v>0.3594</v>
+        <v>0.3593</v>
       </c>
       <c r="G1063" s="16" t="n">
         <v>0.2966</v>
@@ -54740,10 +54740,10 @@
         <v>0.1396</v>
       </c>
       <c r="J1063" s="19" t="n">
-        <v>10667</v>
+        <v>10669</v>
       </c>
       <c r="K1063" s="19" t="n">
-        <v>18566</v>
+        <v>18568</v>
       </c>
       <c r="L1063" s="31" t="n">
         <v>0.6227</v>
@@ -54766,26 +54766,26 @@
         </is>
       </c>
       <c r="D1064" s="9" t="n">
-        <v>609403.05</v>
+        <v>609526.08</v>
       </c>
       <c r="E1064" s="9" t="n">
         <v>1751784.17</v>
       </c>
       <c r="F1064" s="10" t="n">
-        <v>0.386</v>
+        <v>0.3861</v>
       </c>
       <c r="G1064" s="10" t="n">
-        <v>0.3154</v>
+        <v>0.3156</v>
       </c>
       <c r="H1064" s="10" t="n"/>
       <c r="I1064" s="10" t="n">
         <v>0.08799999999999999</v>
       </c>
       <c r="J1064" s="13" t="n">
-        <v>10000</v>
+        <v>10002</v>
       </c>
       <c r="K1064" s="13" t="n">
-        <v>14156</v>
+        <v>14158</v>
       </c>
       <c r="L1064" s="32" t="n">
         <v>0.6883</v>
@@ -54892,29 +54892,29 @@
         </is>
       </c>
       <c r="D1067" s="15" t="n">
-        <v>249179.56</v>
+        <v>325712.16</v>
       </c>
       <c r="E1067" s="15" t="n">
-        <v>1946944.03</v>
+        <v>2465880.71</v>
       </c>
       <c r="F1067" s="16" t="n">
-        <v>0.8401</v>
+        <v>0.8907</v>
       </c>
       <c r="G1067" s="16" t="n">
-        <v>0.7693</v>
+        <v>0.8201000000000001</v>
       </c>
       <c r="H1067" s="16" t="n"/>
       <c r="I1067" s="16" t="n">
-        <v>0.011</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="J1067" s="19" t="n">
-        <v>12079</v>
+        <v>14256</v>
       </c>
       <c r="K1067" s="19" t="n">
-        <v>14429</v>
+        <v>37855</v>
       </c>
       <c r="L1067" s="31" t="n">
-        <v>0.3628</v>
+        <v>0.2798</v>
       </c>
     </row>
     <row r="1068">
@@ -54934,29 +54934,29 @@
         </is>
       </c>
       <c r="D1068" s="9" t="n">
-        <v>76632.17999999999</v>
+        <v>79380.2</v>
       </c>
       <c r="E1068" s="9" t="n">
-        <v>83156.49000000001</v>
+        <v>83178.02</v>
       </c>
       <c r="F1068" s="10" t="n">
-        <v>0.4546</v>
+        <v>0.4743</v>
       </c>
       <c r="G1068" s="10" t="n">
-        <v>0.4079</v>
+        <v>0.4277</v>
       </c>
       <c r="H1068" s="10" t="n"/>
       <c r="I1068" s="10" t="n">
-        <v>0.1777</v>
+        <v>0.1753</v>
       </c>
       <c r="J1068" s="13" t="n">
-        <v>332</v>
+        <v>365</v>
       </c>
       <c r="K1068" s="13" t="n">
-        <v>569</v>
+        <v>619</v>
       </c>
       <c r="L1068" s="32" t="n">
-        <v>0.3046</v>
+        <v>0.3002</v>
       </c>
     </row>
     <row r="1069">
@@ -54976,29 +54976,29 @@
         </is>
       </c>
       <c r="D1069" s="15" t="n">
-        <v>24026.03</v>
+        <v>33287.18</v>
       </c>
       <c r="E1069" s="15" t="n">
-        <v>25021.86</v>
+        <v>26621.29</v>
       </c>
       <c r="F1069" s="16" t="n">
-        <v>0.4426</v>
+        <v>0.5760999999999999</v>
       </c>
       <c r="G1069" s="16" t="n">
-        <v>0.3821</v>
+        <v>0.5154</v>
       </c>
       <c r="H1069" s="16" t="n"/>
       <c r="I1069" s="16" t="n">
-        <v>0.131</v>
+        <v>0.1259</v>
       </c>
       <c r="J1069" s="19" t="n">
-        <v>458</v>
+        <v>556</v>
       </c>
       <c r="K1069" s="19" t="n">
-        <v>532</v>
+        <v>667</v>
       </c>
       <c r="L1069" s="31" t="n">
-        <v>0.5961</v>
+        <v>0.4475</v>
       </c>
     </row>
     <row r="1070">
@@ -55018,29 +55018,29 @@
         </is>
       </c>
       <c r="D1070" s="9" t="n">
-        <v>32180.74</v>
+        <v>41933.29</v>
       </c>
       <c r="E1070" s="9" t="n">
-        <v>28169.35</v>
+        <v>61880.68</v>
       </c>
       <c r="F1070" s="10" t="n">
-        <v>0.5504</v>
+        <v>0.4834</v>
       </c>
       <c r="G1070" s="10" t="n">
-        <v>0.4894</v>
+        <v>0.4125</v>
       </c>
       <c r="H1070" s="10" t="n"/>
       <c r="I1070" s="10" t="n">
-        <v>0.0917</v>
+        <v>0.0785</v>
       </c>
       <c r="J1070" s="13" t="n">
-        <v>567</v>
+        <v>701</v>
       </c>
       <c r="K1070" s="13" t="n">
-        <v>648</v>
+        <v>797</v>
       </c>
       <c r="L1070" s="32" t="n">
-        <v>0.4004</v>
+        <v>0.3203</v>
       </c>
     </row>
     <row r="1071">
@@ -55060,29 +55060,29 @@
         </is>
       </c>
       <c r="D1071" s="15" t="n">
-        <v>29554.14</v>
+        <v>36970.46</v>
       </c>
       <c r="E1071" s="15" t="n">
-        <v>54507.76</v>
+        <v>56451.75</v>
       </c>
       <c r="F1071" s="16" t="n">
-        <v>0.3852</v>
+        <v>0.4983</v>
       </c>
       <c r="G1071" s="16" t="n">
-        <v>0.3216</v>
+        <v>0.4356</v>
       </c>
       <c r="H1071" s="16" t="n"/>
       <c r="I1071" s="16" t="n">
-        <v>0.0752</v>
+        <v>0.06279999999999999</v>
       </c>
       <c r="J1071" s="19" t="n">
-        <v>625</v>
+        <v>764</v>
       </c>
       <c r="K1071" s="19" t="n">
-        <v>700</v>
+        <v>856</v>
       </c>
       <c r="L1071" s="31" t="n">
-        <v>0.6516</v>
+        <v>0.5264</v>
       </c>
     </row>
     <row r="1072">
@@ -55102,29 +55102,29 @@
         </is>
       </c>
       <c r="D1072" s="9" t="n">
-        <v>54806.31</v>
+        <v>64026.64</v>
       </c>
       <c r="E1072" s="9" t="n">
-        <v>158053.05</v>
+        <v>184939.2</v>
       </c>
       <c r="F1072" s="10" t="n">
-        <v>0.2775</v>
+        <v>0.3604</v>
       </c>
       <c r="G1072" s="10" t="n">
-        <v>0.2014</v>
+        <v>0.2839</v>
       </c>
       <c r="H1072" s="10" t="n"/>
       <c r="I1072" s="10" t="n">
-        <v>0.032</v>
+        <v>0.0284</v>
       </c>
       <c r="J1072" s="13" t="n">
-        <v>1687</v>
+        <v>2039</v>
       </c>
       <c r="K1072" s="13" t="n">
-        <v>1913</v>
+        <v>2329</v>
       </c>
       <c r="L1072" s="32" t="n">
-        <v>0.5329</v>
+        <v>0.4733</v>
       </c>
     </row>
     <row r="1073">
@@ -55144,29 +55144,29 @@
         </is>
       </c>
       <c r="D1073" s="15" t="n">
-        <v>78049.23</v>
+        <v>91910.86</v>
       </c>
       <c r="E1073" s="15" t="n">
-        <v>327170.95</v>
+        <v>413083.94</v>
       </c>
       <c r="F1073" s="16" t="n">
-        <v>0.8315</v>
+        <v>0.8549</v>
       </c>
       <c r="G1073" s="16" t="n">
-        <v>0.7574</v>
+        <v>0.7806999999999999</v>
       </c>
       <c r="H1073" s="16" t="n"/>
       <c r="I1073" s="16" t="n">
-        <v>0.0136</v>
+        <v>0.0128</v>
       </c>
       <c r="J1073" s="19" t="n">
-        <v>2274</v>
+        <v>2724</v>
       </c>
       <c r="K1073" s="19" t="n">
-        <v>2640</v>
+        <v>4127</v>
       </c>
       <c r="L1073" s="31" t="n">
-        <v>0.2512</v>
+        <v>0.2199</v>
       </c>
     </row>
     <row r="1074">
@@ -55606,26 +55606,26 @@
         </is>
       </c>
       <c r="D1084" s="9" t="n">
-        <v>1461637.68</v>
+        <v>2883699.5</v>
       </c>
       <c r="E1084" s="9" t="n">
-        <v>2177367.67</v>
+        <v>10016785.4</v>
       </c>
       <c r="F1084" s="10" t="n">
-        <v>0.3151</v>
+        <v>0.1984</v>
       </c>
       <c r="G1084" s="10" t="n">
-        <v>0.2565</v>
+        <v>0.1444</v>
       </c>
       <c r="H1084" s="10" t="n"/>
       <c r="I1084" s="10" t="n">
-        <v>0.073</v>
+        <v>0.0877</v>
       </c>
       <c r="J1084" s="13" t="n">
-        <v>29249</v>
+        <v>50033</v>
       </c>
       <c r="K1084" s="13" t="n">
-        <v>91830</v>
+        <v>140585</v>
       </c>
       <c r="L1084" s="32" t="n">
         <v>0</v>
@@ -58588,26 +58588,26 @@
         </is>
       </c>
       <c r="D1155" s="15" t="n">
-        <v>118952.97</v>
+        <v>139535.21</v>
       </c>
       <c r="E1155" s="15" t="n">
-        <v>790417.48</v>
+        <v>5299051.6</v>
       </c>
       <c r="F1155" s="16" t="n">
-        <v>1.0167</v>
+        <v>0.9021</v>
       </c>
       <c r="G1155" s="16" t="n">
-        <v>0.9515</v>
+        <v>0.8292</v>
       </c>
       <c r="H1155" s="16" t="n"/>
       <c r="I1155" s="16" t="n">
-        <v>0.0059</v>
+        <v>0.0069</v>
       </c>
       <c r="J1155" s="19" t="n">
-        <v>3914</v>
+        <v>5920</v>
       </c>
       <c r="K1155" s="19" t="n">
-        <v>40419</v>
+        <v>47350</v>
       </c>
       <c r="L1155" s="31" t="n">
         <v>0</v>
@@ -58630,26 +58630,26 @@
         </is>
       </c>
       <c r="D1156" s="9" t="n">
-        <v>589216.15</v>
+        <v>1322311.28</v>
       </c>
       <c r="E1156" s="9" t="n">
-        <v>685551.1899999999</v>
+        <v>889236.9</v>
       </c>
       <c r="F1156" s="10" t="n">
-        <v>0.1193</v>
+        <v>0.093</v>
       </c>
       <c r="G1156" s="10" t="n">
-        <v>0.0619</v>
+        <v>0.0474</v>
       </c>
       <c r="H1156" s="10" t="n"/>
       <c r="I1156" s="10" t="n">
-        <v>0.1897</v>
+        <v>0.2042</v>
       </c>
       <c r="J1156" s="13" t="n">
-        <v>4954</v>
+        <v>8588</v>
       </c>
       <c r="K1156" s="13" t="n">
-        <v>14651</v>
+        <v>25602</v>
       </c>
       <c r="L1156" s="32" t="n">
         <v>0</v>
@@ -58672,26 +58672,26 @@
         </is>
       </c>
       <c r="D1157" s="15" t="n">
-        <v>415663.92</v>
+        <v>718161.52</v>
       </c>
       <c r="E1157" s="15" t="n">
-        <v>226861.09</v>
+        <v>548438.3100000001</v>
       </c>
       <c r="F1157" s="16" t="n">
-        <v>0.3773</v>
+        <v>0.2034</v>
       </c>
       <c r="G1157" s="16" t="n">
-        <v>0.3198</v>
+        <v>0.1477</v>
       </c>
       <c r="H1157" s="16" t="n"/>
       <c r="I1157" s="16" t="n">
-        <v>0.108</v>
+        <v>0.1233</v>
       </c>
       <c r="J1157" s="19" t="n">
-        <v>5619</v>
+        <v>9675</v>
       </c>
       <c r="K1157" s="19" t="n">
-        <v>13081</v>
+        <v>22508</v>
       </c>
       <c r="L1157" s="31" t="n">
         <v>0</v>
@@ -58714,26 +58714,26 @@
         </is>
       </c>
       <c r="D1158" s="9" t="n">
-        <v>126542.03</v>
+        <v>328304.62</v>
       </c>
       <c r="E1158" s="9" t="n">
-        <v>109910.39</v>
+        <v>446997.54</v>
       </c>
       <c r="F1158" s="10" t="n">
-        <v>-0.1241</v>
+        <v>0.1137</v>
       </c>
       <c r="G1158" s="10" t="n">
-        <v>-0.1872</v>
+        <v>0.0503</v>
       </c>
       <c r="H1158" s="10" t="n"/>
       <c r="I1158" s="10" t="n">
-        <v>0.0674</v>
+        <v>0.08450000000000001</v>
       </c>
       <c r="J1158" s="13" t="n">
-        <v>4109</v>
+        <v>7631</v>
       </c>
       <c r="K1158" s="13" t="n">
-        <v>6415</v>
+        <v>14677</v>
       </c>
       <c r="L1158" s="32" t="n">
         <v>0</v>
@@ -58756,26 +58756,26 @@
         </is>
       </c>
       <c r="D1159" s="15" t="n">
-        <v>70630.2</v>
+        <v>124098.34</v>
       </c>
       <c r="E1159" s="15" t="n">
-        <v>43364.71</v>
+        <v>407706.83</v>
       </c>
       <c r="F1159" s="16" t="n">
-        <v>0.6441</v>
+        <v>0.3824</v>
       </c>
       <c r="G1159" s="16" t="n">
-        <v>0.5861</v>
+        <v>0.3164</v>
       </c>
       <c r="H1159" s="16" t="n"/>
       <c r="I1159" s="16" t="n">
-        <v>0.0427</v>
+        <v>0.066</v>
       </c>
       <c r="J1159" s="19" t="n">
-        <v>2717</v>
+        <v>4564</v>
       </c>
       <c r="K1159" s="19" t="n">
-        <v>3573</v>
+        <v>6345</v>
       </c>
       <c r="L1159" s="31" t="n">
         <v>0</v>
@@ -58798,26 +58798,26 @@
         </is>
       </c>
       <c r="D1160" s="9" t="n">
-        <v>78728.50999999999</v>
+        <v>141095.34</v>
       </c>
       <c r="E1160" s="9" t="n">
-        <v>163313.85</v>
+        <v>512589.3</v>
       </c>
       <c r="F1160" s="10" t="n">
-        <v>0.4926</v>
+        <v>0.2803</v>
       </c>
       <c r="G1160" s="10" t="n">
-        <v>0.4346</v>
+        <v>0.2161</v>
       </c>
       <c r="H1160" s="10" t="n"/>
       <c r="I1160" s="10" t="n">
-        <v>0.0288</v>
+        <v>0.0461</v>
       </c>
       <c r="J1160" s="13" t="n">
-        <v>4270</v>
+        <v>7203</v>
       </c>
       <c r="K1160" s="13" t="n">
-        <v>5781</v>
+        <v>10453</v>
       </c>
       <c r="L1160" s="32" t="n">
         <v>0</v>
@@ -58840,26 +58840,26 @@
         </is>
       </c>
       <c r="D1161" s="15" t="n">
-        <v>61903.91</v>
+        <v>110193.2</v>
       </c>
       <c r="E1161" s="15" t="n">
-        <v>157948.97</v>
+        <v>1912764.93</v>
       </c>
       <c r="F1161" s="16" t="n">
-        <v>0.711</v>
+        <v>0.4787</v>
       </c>
       <c r="G1161" s="16" t="n">
-        <v>0.6525</v>
+        <v>0.414</v>
       </c>
       <c r="H1161" s="16" t="n"/>
       <c r="I1161" s="16" t="n">
-        <v>0.0134</v>
+        <v>0.0192</v>
       </c>
       <c r="J1161" s="19" t="n">
-        <v>3666</v>
+        <v>6452</v>
       </c>
       <c r="K1161" s="19" t="n">
-        <v>7910</v>
+        <v>13650</v>
       </c>
       <c r="L1161" s="31" t="n">
         <v>0</v>
@@ -59386,26 +59386,26 @@
         </is>
       </c>
       <c r="D1174" s="9" t="n">
-        <v>176379919.12</v>
+        <v>176752961.05</v>
       </c>
       <c r="E1174" s="9" t="n">
-        <v>773266594.1900001</v>
+        <v>774561897.83</v>
       </c>
       <c r="F1174" s="10" t="n">
-        <v>0.1428</v>
+        <v>0.1419</v>
       </c>
       <c r="G1174" s="10" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="H1174" s="10" t="n"/>
       <c r="I1174" s="10" t="n">
-        <v>0.0983</v>
+        <v>0.0985</v>
       </c>
       <c r="J1174" s="13" t="n">
-        <v>4205792</v>
+        <v>4207730</v>
       </c>
       <c r="K1174" s="13" t="n">
-        <v>8171054</v>
+        <v>8186425</v>
       </c>
       <c r="L1174" s="32" t="n">
         <v>0</v>
@@ -59428,26 +59428,26 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>34170036.29</v>
+        <v>57946157.24</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>128501680.55</v>
+        <v>223674664.6</v>
       </c>
       <c r="F1175" s="16" t="n">
-        <v>0.0244</v>
+        <v>0.1258</v>
       </c>
       <c r="G1175" s="16" t="n">
-        <v>-0.0301</v>
+        <v>0.0707</v>
       </c>
       <c r="H1175" s="16" t="n"/>
       <c r="I1175" s="16" t="n">
-        <v>0.113</v>
+        <v>0.1015</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>780556</v>
+        <v>1374359</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>1489123</v>
+        <v>2555668</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -62998,26 +62998,26 @@
         </is>
       </c>
       <c r="D1260" s="9" t="n">
-        <v>21454066.46</v>
+        <v>21457462.74</v>
       </c>
       <c r="E1260" s="9" t="n">
-        <v>389721488.37</v>
+        <v>390593856.51</v>
       </c>
       <c r="F1260" s="10" t="n">
-        <v>0.4375</v>
+        <v>0.4338</v>
       </c>
       <c r="G1260" s="10" t="n">
-        <v>0.357</v>
+        <v>0.3532</v>
       </c>
       <c r="H1260" s="10" t="n"/>
       <c r="I1260" s="10" t="n">
-        <v>0.0283</v>
+        <v>0.0284</v>
       </c>
       <c r="J1260" s="13" t="n">
-        <v>1575954</v>
+        <v>1576126</v>
       </c>
       <c r="K1260" s="13" t="n">
-        <v>2466033</v>
+        <v>2468161</v>
       </c>
       <c r="L1260" s="32" t="n">
         <v>0</v>
@@ -63040,26 +63040,26 @@
         </is>
       </c>
       <c r="D1261" s="15" t="n">
-        <v>46789274.66</v>
+        <v>47038181.94</v>
       </c>
       <c r="E1261" s="15" t="n">
-        <v>24364287.56</v>
+        <v>24462981.01</v>
       </c>
       <c r="F1261" s="16" t="n">
-        <v>0.032</v>
+        <v>0.033</v>
       </c>
       <c r="G1261" s="16" t="n">
-        <v>-0.0097</v>
+        <v>-0.008800000000000001</v>
       </c>
       <c r="H1261" s="16" t="n"/>
       <c r="I1261" s="16" t="n">
-        <v>0.3104</v>
+        <v>0.3106</v>
       </c>
       <c r="J1261" s="19" t="n">
-        <v>198419</v>
+        <v>198928</v>
       </c>
       <c r="K1261" s="19" t="n">
-        <v>892393</v>
+        <v>896767</v>
       </c>
       <c r="L1261" s="31" t="n">
         <v>0</v>
@@ -63082,26 +63082,26 @@
         </is>
       </c>
       <c r="D1262" s="9" t="n">
-        <v>29941215.67</v>
+        <v>30002560.46</v>
       </c>
       <c r="E1262" s="9" t="n">
-        <v>31119813.12</v>
+        <v>31177325.75</v>
       </c>
       <c r="F1262" s="10" t="n">
-        <v>0.0437</v>
+        <v>0.0438</v>
       </c>
       <c r="G1262" s="10" t="n">
-        <v>-0.0078</v>
+        <v>-0.0077</v>
       </c>
       <c r="H1262" s="10" t="n"/>
       <c r="I1262" s="10" t="n">
-        <v>0.2374</v>
+        <v>0.2376</v>
       </c>
       <c r="J1262" s="13" t="n">
-        <v>295258</v>
+        <v>295705</v>
       </c>
       <c r="K1262" s="13" t="n">
-        <v>782276</v>
+        <v>783776</v>
       </c>
       <c r="L1262" s="32" t="n">
         <v>0</v>
@@ -63124,26 +63124,26 @@
         </is>
       </c>
       <c r="D1263" s="15" t="n">
-        <v>22480778.11</v>
+        <v>22499210.51</v>
       </c>
       <c r="E1263" s="15" t="n">
-        <v>37082524</v>
+        <v>37108422.3</v>
       </c>
       <c r="F1263" s="16" t="n">
-        <v>0.0675</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="G1263" s="16" t="n">
         <v>0.0101</v>
       </c>
       <c r="H1263" s="16" t="n"/>
       <c r="I1263" s="16" t="n">
-        <v>0.189</v>
+        <v>0.1892</v>
       </c>
       <c r="J1263" s="19" t="n">
-        <v>343874</v>
+        <v>344121</v>
       </c>
       <c r="K1263" s="19" t="n">
-        <v>749741</v>
+        <v>750766</v>
       </c>
       <c r="L1263" s="31" t="n">
         <v>0</v>
@@ -63166,26 +63166,26 @@
         </is>
       </c>
       <c r="D1264" s="9" t="n">
-        <v>15071771.52</v>
+        <v>15087009.88</v>
       </c>
       <c r="E1264" s="9" t="n">
-        <v>40883477.55</v>
+        <v>40911895.96</v>
       </c>
       <c r="F1264" s="10" t="n">
-        <v>0.0825</v>
+        <v>0.0829</v>
       </c>
       <c r="G1264" s="10" t="n">
-        <v>0.0179</v>
+        <v>0.0183</v>
       </c>
       <c r="H1264" s="10" t="n"/>
       <c r="I1264" s="10" t="n">
-        <v>0.15</v>
+        <v>0.1502</v>
       </c>
       <c r="J1264" s="13" t="n">
-        <v>333105</v>
+        <v>333265</v>
       </c>
       <c r="K1264" s="13" t="n">
-        <v>635396</v>
+        <v>637271</v>
       </c>
       <c r="L1264" s="32" t="n">
         <v>0</v>
@@ -63208,26 +63208,26 @@
         </is>
       </c>
       <c r="D1265" s="15" t="n">
-        <v>21148024.03</v>
+        <v>21159263.18</v>
       </c>
       <c r="E1265" s="15" t="n">
-        <v>93772166.48999999</v>
+        <v>93814929.09999999</v>
       </c>
       <c r="F1265" s="16" t="n">
-        <v>0.184</v>
+        <v>0.1831</v>
       </c>
       <c r="G1265" s="16" t="n">
-        <v>0.1153</v>
+        <v>0.1144</v>
       </c>
       <c r="H1265" s="16" t="n"/>
       <c r="I1265" s="16" t="n">
-        <v>0.1093</v>
+        <v>0.1095</v>
       </c>
       <c r="J1265" s="19" t="n">
-        <v>645117</v>
+        <v>645336</v>
       </c>
       <c r="K1265" s="19" t="n">
-        <v>1135169</v>
+        <v>1136063</v>
       </c>
       <c r="L1265" s="31" t="n">
         <v>0</v>
@@ -63250,26 +63250,26 @@
         </is>
       </c>
       <c r="D1266" s="9" t="n">
-        <v>19494788.68</v>
+        <v>19509272.35</v>
       </c>
       <c r="E1266" s="9" t="n">
-        <v>156322837.09</v>
+        <v>156492487.2</v>
       </c>
       <c r="F1266" s="10" t="n">
-        <v>0.3252</v>
+        <v>0.3211</v>
       </c>
       <c r="G1266" s="10" t="n">
-        <v>0.2518</v>
+        <v>0.2477</v>
       </c>
       <c r="H1266" s="10" t="n"/>
       <c r="I1266" s="10" t="n">
-        <v>0.0636</v>
+        <v>0.0638</v>
       </c>
       <c r="J1266" s="13" t="n">
-        <v>814065</v>
+        <v>814249</v>
       </c>
       <c r="K1266" s="13" t="n">
-        <v>1510046</v>
+        <v>1513621</v>
       </c>
       <c r="L1266" s="32" t="n">
         <v>0</v>
@@ -63292,26 +63292,26 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>4296335.29</v>
+        <v>7611818.21</v>
       </c>
       <c r="E1267" s="15" t="n">
-        <v>70100866.36</v>
+        <v>126703083.65</v>
       </c>
       <c r="F1267" s="16" t="n">
-        <v>0.4607</v>
+        <v>0.443</v>
       </c>
       <c r="G1267" s="16" t="n">
-        <v>0.3884</v>
+        <v>0.3696</v>
       </c>
       <c r="H1267" s="16" t="n"/>
       <c r="I1267" s="16" t="n">
-        <v>0.0302</v>
+        <v>0.0281</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>322202</v>
+        <v>577683</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>517643</v>
+        <v>924052</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63334,26 +63334,26 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>9750471.93</v>
+        <v>16243166.73</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>4906953.2</v>
+        <v>7813796.59</v>
       </c>
       <c r="F1268" s="10" t="n">
-        <v>-0.0533</v>
+        <v>0.0242</v>
       </c>
       <c r="G1268" s="10" t="n">
-        <v>-0.09130000000000001</v>
+        <v>-0.0147</v>
       </c>
       <c r="H1268" s="10" t="n"/>
       <c r="I1268" s="10" t="n">
-        <v>0.3168</v>
+        <v>0.3127</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>38314</v>
+        <v>64250</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>155921</v>
+        <v>255671</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63376,26 +63376,26 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>6098028.15</v>
+        <v>10245295.77</v>
       </c>
       <c r="E1269" s="15" t="n">
-        <v>5591539.16</v>
+        <v>8807401.199999999</v>
       </c>
       <c r="F1269" s="16" t="n">
-        <v>-0.0863</v>
+        <v>0.0444</v>
       </c>
       <c r="G1269" s="16" t="n">
-        <v>-0.1356</v>
+        <v>-0.0046</v>
       </c>
       <c r="H1269" s="16" t="n"/>
       <c r="I1269" s="16" t="n">
-        <v>0.2652</v>
+        <v>0.2514</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>54181</v>
+        <v>92249</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>144779</v>
+        <v>234600</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63418,26 +63418,26 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>4467022.78</v>
+        <v>7373654.78</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>6108282.44</v>
+        <v>10571661.18</v>
       </c>
       <c r="F1270" s="10" t="n">
-        <v>-0.1125</v>
+        <v>0.0324</v>
       </c>
       <c r="G1270" s="10" t="n">
-        <v>-0.1677</v>
+        <v>-0.0239</v>
       </c>
       <c r="H1270" s="10" t="n"/>
       <c r="I1270" s="10" t="n">
-        <v>0.2273</v>
+        <v>0.2066</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>59850</v>
+        <v>102565</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>123776</v>
+        <v>215200</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63460,26 +63460,26 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>2589448.85</v>
+        <v>4617625.16</v>
       </c>
       <c r="E1271" s="15" t="n">
-        <v>5691219.84</v>
+        <v>10995519.04</v>
       </c>
       <c r="F1271" s="16" t="n">
-        <v>-0.1057</v>
+        <v>0.1056</v>
       </c>
       <c r="G1271" s="16" t="n">
-        <v>-0.1669</v>
+        <v>0.0436</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
-        <v>0.1904</v>
+        <v>0.1673</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>57216</v>
+        <v>100099</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>99035</v>
+        <v>189929</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63502,26 +63502,26 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>3575352.7</v>
+        <v>6110574.78</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>12265682.24</v>
+        <v>20801367.55</v>
       </c>
       <c r="F1272" s="10" t="n">
-        <v>-0.0109</v>
+        <v>0.1454</v>
       </c>
       <c r="G1272" s="10" t="n">
-        <v>-0.0791</v>
+        <v>0.07829999999999999</v>
       </c>
       <c r="H1272" s="10" t="n"/>
       <c r="I1272" s="10" t="n">
-        <v>0.1445</v>
+        <v>0.1245</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>110045</v>
+        <v>192919</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>184437</v>
+        <v>311151</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63544,26 +63544,26 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>3393376.59</v>
+        <v>5744021.8</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>23837137.32</v>
+        <v>37981835.39</v>
       </c>
       <c r="F1273" s="16" t="n">
-        <v>0.2106</v>
+        <v>0.2537</v>
       </c>
       <c r="G1273" s="16" t="n">
-        <v>0.143</v>
+        <v>0.1858</v>
       </c>
       <c r="H1273" s="16" t="n"/>
       <c r="I1273" s="16" t="n">
-        <v>0.0832</v>
+        <v>0.0735</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>138748</v>
+        <v>244594</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>263532</v>
+        <v>425065</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -64048,26 +64048,26 @@
         </is>
       </c>
       <c r="D1285" s="15" t="n">
-        <v>17469693.82</v>
+        <v>17471488.71</v>
       </c>
       <c r="E1285" s="15" t="n">
-        <v>50447851.19</v>
+        <v>50450647.22</v>
       </c>
       <c r="F1285" s="16" t="n">
         <v>0.1857</v>
       </c>
       <c r="G1285" s="16" t="n">
-        <v>0.1246</v>
+        <v>0.1245</v>
       </c>
       <c r="H1285" s="16" t="n"/>
       <c r="I1285" s="16" t="n">
-        <v>0.1135</v>
+        <v>0.1136</v>
       </c>
       <c r="J1285" s="19" t="n">
-        <v>291010</v>
+        <v>291055</v>
       </c>
       <c r="K1285" s="19" t="n">
-        <v>435945</v>
+        <v>435995</v>
       </c>
       <c r="L1285" s="31" t="n">
         <v>0</v>
@@ -64090,26 +64090,26 @@
         </is>
       </c>
       <c r="D1286" s="9" t="n">
-        <v>1388858.16</v>
+        <v>3710208.95</v>
       </c>
       <c r="E1286" s="9" t="n">
-        <v>616574.1899999999</v>
+        <v>9237620.09</v>
       </c>
       <c r="F1286" s="10" t="n">
-        <v>0.1971</v>
+        <v>-0.06320000000000001</v>
       </c>
       <c r="G1286" s="10" t="n">
-        <v>0.1432</v>
+        <v>-0.1225</v>
       </c>
       <c r="H1286" s="10" t="n"/>
       <c r="I1286" s="10" t="n">
-        <v>0.0858</v>
+        <v>0.116</v>
       </c>
       <c r="J1286" s="13" t="n">
-        <v>25877</v>
+        <v>71342</v>
       </c>
       <c r="K1286" s="13" t="n">
-        <v>37764</v>
+        <v>107873</v>
       </c>
       <c r="L1286" s="32" t="n">
         <v>0</v>
@@ -67408,26 +67408,26 @@
         </is>
       </c>
       <c r="D1365" s="15" t="n">
-        <v>5143464.56</v>
+        <v>5144479.24</v>
       </c>
       <c r="E1365" s="15" t="n">
-        <v>3967339.44</v>
+        <v>3968083.12</v>
       </c>
       <c r="F1365" s="16" t="n">
-        <v>0.06619999999999999</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="G1365" s="16" t="n">
-        <v>0.013</v>
+        <v>0.0129</v>
       </c>
       <c r="H1365" s="16" t="n"/>
       <c r="I1365" s="16" t="n">
-        <v>0.3521</v>
+        <v>0.3526</v>
       </c>
       <c r="J1365" s="19" t="n">
-        <v>16667</v>
+        <v>16697</v>
       </c>
       <c r="K1365" s="19" t="n">
-        <v>51800</v>
+        <v>51833</v>
       </c>
       <c r="L1365" s="31" t="n">
         <v>0</v>
@@ -67450,10 +67450,10 @@
         </is>
       </c>
       <c r="D1366" s="9" t="n">
-        <v>3532875.81</v>
+        <v>3533297.8</v>
       </c>
       <c r="E1366" s="9" t="n">
-        <v>3872405.78</v>
+        <v>3873643</v>
       </c>
       <c r="F1366" s="10" t="n">
         <v>0.1447</v>
@@ -67463,13 +67463,13 @@
       </c>
       <c r="H1366" s="10" t="n"/>
       <c r="I1366" s="10" t="n">
-        <v>0.2296</v>
+        <v>0.2298</v>
       </c>
       <c r="J1366" s="13" t="n">
-        <v>28881</v>
+        <v>28889</v>
       </c>
       <c r="K1366" s="13" t="n">
-        <v>52094</v>
+        <v>52103</v>
       </c>
       <c r="L1366" s="32" t="n">
         <v>0</v>
@@ -67492,26 +67492,26 @@
         </is>
       </c>
       <c r="D1367" s="15" t="n">
-        <v>2486832.05</v>
+        <v>2487134.42</v>
       </c>
       <c r="E1367" s="15" t="n">
-        <v>4179544.07</v>
+        <v>4179715.77</v>
       </c>
       <c r="F1367" s="16" t="n">
-        <v>0.1198</v>
+        <v>0.1195</v>
       </c>
       <c r="G1367" s="16" t="n">
-        <v>0.0582</v>
+        <v>0.0579</v>
       </c>
       <c r="H1367" s="16" t="n"/>
       <c r="I1367" s="16" t="n">
-        <v>0.172</v>
+        <v>0.1721</v>
       </c>
       <c r="J1367" s="19" t="n">
-        <v>33669</v>
+        <v>33674</v>
       </c>
       <c r="K1367" s="19" t="n">
-        <v>52216</v>
+        <v>52222</v>
       </c>
       <c r="L1367" s="31" t="n">
         <v>0</v>
@@ -67534,10 +67534,10 @@
         </is>
       </c>
       <c r="D1368" s="9" t="n">
-        <v>1777600.35</v>
+        <v>1777656.21</v>
       </c>
       <c r="E1368" s="9" t="n">
-        <v>4221664.98</v>
+        <v>4222308.41</v>
       </c>
       <c r="F1368" s="10" t="n">
         <v>0.3156</v>
@@ -67550,10 +67550,10 @@
         <v>0.1372</v>
       </c>
       <c r="J1368" s="13" t="n">
-        <v>28900</v>
+        <v>28902</v>
       </c>
       <c r="K1368" s="13" t="n">
-        <v>42232</v>
+        <v>42234</v>
       </c>
       <c r="L1368" s="32" t="n">
         <v>0</v>
@@ -67660,26 +67660,26 @@
         </is>
       </c>
       <c r="D1371" s="15" t="n">
-        <v>105248.54</v>
+        <v>270801.02</v>
       </c>
       <c r="E1371" s="15" t="n">
-        <v>209938.5</v>
+        <v>3589976.92</v>
       </c>
       <c r="F1371" s="16" t="n">
-        <v>0.318</v>
+        <v>0.1302</v>
       </c>
       <c r="G1371" s="16" t="n">
-        <v>0.2531</v>
+        <v>0.0571</v>
       </c>
       <c r="H1371" s="16" t="n"/>
       <c r="I1371" s="16" t="n">
-        <v>0.0242</v>
+        <v>0.0286</v>
       </c>
       <c r="J1371" s="19" t="n">
-        <v>7197</v>
+        <v>20011</v>
       </c>
       <c r="K1371" s="19" t="n">
-        <v>10402</v>
+        <v>27084</v>
       </c>
       <c r="L1371" s="31" t="n">
         <v>0</v>
@@ -67702,26 +67702,26 @@
         </is>
       </c>
       <c r="D1372" s="9" t="n">
-        <v>290505.8</v>
+        <v>904072.1</v>
       </c>
       <c r="E1372" s="9" t="n">
-        <v>47779.85</v>
+        <v>361397.1</v>
       </c>
       <c r="F1372" s="10" t="n">
-        <v>0.293</v>
+        <v>0.0122</v>
       </c>
       <c r="G1372" s="10" t="n">
-        <v>0.2448</v>
+        <v>-0.0359</v>
       </c>
       <c r="H1372" s="10" t="n"/>
       <c r="I1372" s="10" t="n">
-        <v>0.2733</v>
+        <v>0.3279</v>
       </c>
       <c r="J1372" s="13" t="n">
-        <v>1317</v>
+        <v>3605</v>
       </c>
       <c r="K1372" s="13" t="n">
-        <v>2710</v>
+        <v>8805</v>
       </c>
       <c r="L1372" s="32" t="n">
         <v>0</v>
@@ -67744,26 +67744,26 @@
         </is>
       </c>
       <c r="D1373" s="15" t="n">
-        <v>341164.66</v>
+        <v>889168.15</v>
       </c>
       <c r="E1373" s="15" t="n">
-        <v>51045.95</v>
+        <v>505953.04</v>
       </c>
       <c r="F1373" s="16" t="n">
-        <v>-0.012</v>
+        <v>-0.1606</v>
       </c>
       <c r="G1373" s="16" t="n">
-        <v>-0.0614</v>
+        <v>-0.215</v>
       </c>
       <c r="H1373" s="16" t="n"/>
       <c r="I1373" s="16" t="n">
-        <v>0.2054</v>
+        <v>0.2622</v>
       </c>
       <c r="J1373" s="19" t="n">
-        <v>2468</v>
+        <v>6919</v>
       </c>
       <c r="K1373" s="19" t="n">
-        <v>3971</v>
+        <v>12529</v>
       </c>
       <c r="L1373" s="31" t="n">
         <v>0</v>
@@ -67786,26 +67786,26 @@
         </is>
       </c>
       <c r="D1374" s="9" t="n">
-        <v>206521.35</v>
+        <v>551521.1899999999</v>
       </c>
       <c r="E1374" s="9" t="n">
-        <v>59996.41</v>
+        <v>745263.37</v>
       </c>
       <c r="F1374" s="10" t="n">
-        <v>0.1624</v>
+        <v>-0.0551</v>
       </c>
       <c r="G1374" s="10" t="n">
-        <v>0.1063</v>
+        <v>-0.1175</v>
       </c>
       <c r="H1374" s="10" t="n"/>
       <c r="I1374" s="10" t="n">
-        <v>0.1418</v>
+        <v>0.1821</v>
       </c>
       <c r="J1374" s="13" t="n">
-        <v>2947</v>
+        <v>8090</v>
       </c>
       <c r="K1374" s="13" t="n">
-        <v>3958</v>
+        <v>11876</v>
       </c>
       <c r="L1374" s="32" t="n">
         <v>0</v>
@@ -67828,26 +67828,26 @@
         </is>
       </c>
       <c r="D1375" s="15" t="n">
-        <v>169901.13</v>
+        <v>406579.19</v>
       </c>
       <c r="E1375" s="15" t="n">
-        <v>82069.41</v>
+        <v>758895.9399999999</v>
       </c>
       <c r="F1375" s="16" t="n">
-        <v>0.3462</v>
+        <v>-0.0999</v>
       </c>
       <c r="G1375" s="16" t="n">
-        <v>0.2931</v>
+        <v>-0.1615</v>
       </c>
       <c r="H1375" s="16" t="n"/>
       <c r="I1375" s="16" t="n">
-        <v>0.0968</v>
+        <v>0.1464</v>
       </c>
       <c r="J1375" s="19" t="n">
-        <v>2645</v>
+        <v>7330</v>
       </c>
       <c r="K1375" s="19" t="n">
-        <v>3756</v>
+        <v>11748</v>
       </c>
       <c r="L1375" s="31" t="n">
         <v>0</v>
@@ -67870,26 +67870,26 @@
         </is>
       </c>
       <c r="D1376" s="9" t="n">
-        <v>185942.32</v>
+        <v>442202.7</v>
       </c>
       <c r="E1376" s="9" t="n">
-        <v>87038.3</v>
+        <v>1833111.58</v>
       </c>
       <c r="F1376" s="10" t="n">
-        <v>0.2646</v>
+        <v>-0.0053</v>
       </c>
       <c r="G1376" s="10" t="n">
-        <v>0.2056</v>
+        <v>-0.07539999999999999</v>
       </c>
       <c r="H1376" s="10" t="n"/>
       <c r="I1376" s="10" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.1009</v>
       </c>
       <c r="J1376" s="13" t="n">
-        <v>5237</v>
+        <v>14024</v>
       </c>
       <c r="K1376" s="13" t="n">
-        <v>8143</v>
+        <v>21372</v>
       </c>
       <c r="L1376" s="32" t="n">
         <v>0</v>
@@ -67912,26 +67912,26 @@
         </is>
       </c>
       <c r="D1377" s="15" t="n">
-        <v>89574.35000000001</v>
+        <v>245864.62</v>
       </c>
       <c r="E1377" s="15" t="n">
-        <v>78705.77</v>
+        <v>1443022.15</v>
       </c>
       <c r="F1377" s="16" t="n">
-        <v>0.1972</v>
+        <v>-0.2627</v>
       </c>
       <c r="G1377" s="16" t="n">
-        <v>0.135</v>
+        <v>-0.336</v>
       </c>
       <c r="H1377" s="16" t="n"/>
       <c r="I1377" s="16" t="n">
-        <v>0.0411</v>
+        <v>0.06569999999999999</v>
       </c>
       <c r="J1377" s="19" t="n">
-        <v>4066</v>
+        <v>11363</v>
       </c>
       <c r="K1377" s="19" t="n">
-        <v>4824</v>
+        <v>14459</v>
       </c>
       <c r="L1377" s="31" t="n">
         <v>0</v>
@@ -68751,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-28 17:13 UTC</t>
+          <t>2026-10-29 15:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-29 16:19 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8647,7 +8647,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-29 15:13 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-29 16:19 UTC.</t>
         </is>
       </c>
     </row>
@@ -59386,10 +59386,10 @@
         </is>
       </c>
       <c r="D1174" s="9" t="n">
-        <v>176752961.05</v>
+        <v>176753035.71</v>
       </c>
       <c r="E1174" s="9" t="n">
-        <v>774561897.83</v>
+        <v>774561992.42</v>
       </c>
       <c r="F1174" s="10" t="n">
         <v>0.1419</v>
@@ -59402,10 +59402,10 @@
         <v>0.0985</v>
       </c>
       <c r="J1174" s="13" t="n">
-        <v>4207730</v>
+        <v>4207739</v>
       </c>
       <c r="K1174" s="13" t="n">
-        <v>8186425</v>
+        <v>8186439</v>
       </c>
       <c r="L1174" s="32" t="n">
         <v>0</v>
@@ -59428,26 +59428,26 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>57946157.24</v>
+        <v>57947776.67</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>223674664.6</v>
+        <v>223676093.34</v>
       </c>
       <c r="F1175" s="16" t="n">
         <v>0.1258</v>
       </c>
       <c r="G1175" s="16" t="n">
-        <v>0.0707</v>
+        <v>0.0706</v>
       </c>
       <c r="H1175" s="16" t="n"/>
       <c r="I1175" s="16" t="n">
         <v>0.1015</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>1374359</v>
+        <v>1374420</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>2555668</v>
+        <v>2555757</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -63040,7 +63040,7 @@
         </is>
       </c>
       <c r="D1261" s="15" t="n">
-        <v>47038181.94</v>
+        <v>47038186.7</v>
       </c>
       <c r="E1261" s="15" t="n">
         <v>24462981.01</v>
@@ -63056,10 +63056,10 @@
         <v>0.3106</v>
       </c>
       <c r="J1261" s="19" t="n">
-        <v>198928</v>
+        <v>198929</v>
       </c>
       <c r="K1261" s="19" t="n">
-        <v>896767</v>
+        <v>896768</v>
       </c>
       <c r="L1261" s="31" t="n">
         <v>0</v>
@@ -63082,10 +63082,10 @@
         </is>
       </c>
       <c r="D1262" s="9" t="n">
-        <v>30002560.46</v>
+        <v>30002596.96</v>
       </c>
       <c r="E1262" s="9" t="n">
-        <v>31177325.75</v>
+        <v>31177345.55</v>
       </c>
       <c r="F1262" s="10" t="n">
         <v>0.0438</v>
@@ -63095,13 +63095,13 @@
       </c>
       <c r="H1262" s="10" t="n"/>
       <c r="I1262" s="10" t="n">
-        <v>0.2376</v>
+        <v>0.2377</v>
       </c>
       <c r="J1262" s="13" t="n">
-        <v>295705</v>
+        <v>295709</v>
       </c>
       <c r="K1262" s="13" t="n">
-        <v>783776</v>
+        <v>783783</v>
       </c>
       <c r="L1262" s="32" t="n">
         <v>0</v>
@@ -63166,10 +63166,10 @@
         </is>
       </c>
       <c r="D1264" s="9" t="n">
-        <v>15087009.88</v>
+        <v>15087039.61</v>
       </c>
       <c r="E1264" s="9" t="n">
-        <v>40911895.96</v>
+        <v>40911911.69</v>
       </c>
       <c r="F1264" s="10" t="n">
         <v>0.0829</v>
@@ -63182,10 +63182,10 @@
         <v>0.1502</v>
       </c>
       <c r="J1264" s="13" t="n">
-        <v>333265</v>
+        <v>333268</v>
       </c>
       <c r="K1264" s="13" t="n">
-        <v>637271</v>
+        <v>637275</v>
       </c>
       <c r="L1264" s="32" t="n">
         <v>0</v>
@@ -63208,10 +63208,10 @@
         </is>
       </c>
       <c r="D1265" s="15" t="n">
-        <v>21159263.18</v>
+        <v>21159266.84</v>
       </c>
       <c r="E1265" s="15" t="n">
-        <v>93814929.09999999</v>
+        <v>93814988.16</v>
       </c>
       <c r="F1265" s="16" t="n">
         <v>0.1831</v>
@@ -63224,10 +63224,10 @@
         <v>0.1095</v>
       </c>
       <c r="J1265" s="19" t="n">
-        <v>645336</v>
+        <v>645337</v>
       </c>
       <c r="K1265" s="19" t="n">
-        <v>1136063</v>
+        <v>1136065</v>
       </c>
       <c r="L1265" s="31" t="n">
         <v>0</v>
@@ -63292,13 +63292,13 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>7611818.21</v>
+        <v>7611841.61</v>
       </c>
       <c r="E1267" s="15" t="n">
         <v>126703083.65</v>
       </c>
       <c r="F1267" s="16" t="n">
-        <v>0.443</v>
+        <v>0.4429</v>
       </c>
       <c r="G1267" s="16" t="n">
         <v>0.3696</v>
@@ -63308,10 +63308,10 @@
         <v>0.0281</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>577683</v>
+        <v>577685</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>924052</v>
+        <v>924054</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63334,26 +63334,26 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>16243166.73</v>
+        <v>16243566.1</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>7813796.59</v>
+        <v>7814050.31</v>
       </c>
       <c r="F1268" s="10" t="n">
         <v>0.0242</v>
       </c>
       <c r="G1268" s="10" t="n">
-        <v>-0.0147</v>
+        <v>-0.0148</v>
       </c>
       <c r="H1268" s="10" t="n"/>
       <c r="I1268" s="10" t="n">
-        <v>0.3127</v>
+        <v>0.3128</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>64250</v>
+        <v>64257</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>255671</v>
+        <v>255684</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63376,10 +63376,10 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>10245295.77</v>
+        <v>10245462.62</v>
       </c>
       <c r="E1269" s="15" t="n">
-        <v>8807401.199999999</v>
+        <v>8807409.08</v>
       </c>
       <c r="F1269" s="16" t="n">
         <v>0.0444</v>
@@ -63392,10 +63392,10 @@
         <v>0.2514</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>92249</v>
+        <v>92260</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>234600</v>
+        <v>234613</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63418,26 +63418,26 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>7373654.78</v>
+        <v>7374048.53</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>10571661.18</v>
+        <v>10571888.78</v>
       </c>
       <c r="F1270" s="10" t="n">
-        <v>0.0324</v>
+        <v>0.0323</v>
       </c>
       <c r="G1270" s="10" t="n">
-        <v>-0.0239</v>
+        <v>-0.024</v>
       </c>
       <c r="H1270" s="10" t="n"/>
       <c r="I1270" s="10" t="n">
-        <v>0.2066</v>
+        <v>0.2067</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>102565</v>
+        <v>102574</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>215200</v>
+        <v>215213</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63460,26 +63460,26 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>4617625.16</v>
+        <v>4617796.22</v>
       </c>
       <c r="E1271" s="15" t="n">
-        <v>10995519.04</v>
+        <v>10995666.72</v>
       </c>
       <c r="F1271" s="16" t="n">
-        <v>0.1056</v>
+        <v>0.1055</v>
       </c>
       <c r="G1271" s="16" t="n">
         <v>0.0436</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
-        <v>0.1673</v>
+        <v>0.1674</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>100099</v>
+        <v>100106</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>189929</v>
+        <v>189941</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63502,26 +63502,26 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>6110574.78</v>
+        <v>6110804.24</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>20801367.55</v>
+        <v>20801670.83</v>
       </c>
       <c r="F1272" s="10" t="n">
-        <v>0.1454</v>
+        <v>0.1452</v>
       </c>
       <c r="G1272" s="10" t="n">
-        <v>0.07829999999999999</v>
+        <v>0.07820000000000001</v>
       </c>
       <c r="H1272" s="10" t="n"/>
       <c r="I1272" s="10" t="n">
-        <v>0.1245</v>
+        <v>0.1246</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>192919</v>
+        <v>192931</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>311151</v>
+        <v>311171</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63544,26 +63544,26 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>5744021.8</v>
+        <v>5744257.35</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>37981835.39</v>
+        <v>37982323.98</v>
       </c>
       <c r="F1273" s="16" t="n">
-        <v>0.2537</v>
+        <v>0.2533</v>
       </c>
       <c r="G1273" s="16" t="n">
-        <v>0.1858</v>
+        <v>0.1854</v>
       </c>
       <c r="H1273" s="16" t="n"/>
       <c r="I1273" s="16" t="n">
-        <v>0.0735</v>
+        <v>0.0736</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>244594</v>
+        <v>244607</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>425065</v>
+        <v>425081</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -68751,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-29 15:13 UTC</t>
+          <t>2026-10-29 16:19 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-29 17:29 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8647,7 +8647,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-29 16:19 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-29 17:29 UTC.</t>
         </is>
       </c>
     </row>
@@ -39268,13 +39268,13 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>3434190.46</v>
+        <v>3434206.39</v>
       </c>
       <c r="E695" s="15" t="n">
-        <v>26899878.68</v>
+        <v>26899974.2</v>
       </c>
       <c r="F695" s="16" t="n">
-        <v>0.1941</v>
+        <v>0.1942</v>
       </c>
       <c r="G695" s="16" t="n">
         <v>0.1253</v>
@@ -39284,10 +39284,10 @@
         <v>0.0507</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>162352</v>
+        <v>162355</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>221048</v>
+        <v>221052</v>
       </c>
       <c r="L695" s="31" t="n">
         <v>0.5554</v>
@@ -43132,7 +43132,7 @@
         </is>
       </c>
       <c r="D787" s="15" t="n">
-        <v>994063.02</v>
+        <v>994073.34</v>
       </c>
       <c r="E787" s="15" t="n">
         <v>18962832.56</v>
@@ -43148,10 +43148,10 @@
         <v>0.0169</v>
       </c>
       <c r="J787" s="19" t="n">
-        <v>96074</v>
+        <v>96076</v>
       </c>
       <c r="K787" s="19" t="n">
-        <v>127865</v>
+        <v>127867</v>
       </c>
       <c r="L787" s="31" t="n">
         <v>0.4599</v>
@@ -43342,10 +43342,10 @@
         </is>
       </c>
       <c r="D792" s="9" t="n">
-        <v>472394.63</v>
+        <v>472400.25</v>
       </c>
       <c r="E792" s="9" t="n">
-        <v>1901924.58</v>
+        <v>1902020.09</v>
       </c>
       <c r="F792" s="10" t="n">
         <v>0.2224</v>
@@ -43358,10 +43358,10 @@
         <v>0.07779999999999999</v>
       </c>
       <c r="J792" s="13" t="n">
-        <v>18865</v>
+        <v>18866</v>
       </c>
       <c r="K792" s="13" t="n">
-        <v>23674</v>
+        <v>23676</v>
       </c>
       <c r="L792" s="32" t="n">
         <v>0.5726</v>
@@ -59428,26 +59428,26 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>57947776.67</v>
+        <v>57997127.37</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>223676093.34</v>
+        <v>223721677.52</v>
       </c>
       <c r="F1175" s="16" t="n">
-        <v>0.1258</v>
+        <v>0.1245</v>
       </c>
       <c r="G1175" s="16" t="n">
-        <v>0.0706</v>
+        <v>0.0693</v>
       </c>
       <c r="H1175" s="16" t="n"/>
       <c r="I1175" s="16" t="n">
-        <v>0.1015</v>
+        <v>0.1016</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>1374420</v>
+        <v>1374952</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>2555757</v>
+        <v>2556692</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -63292,26 +63292,26 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>7611841.61</v>
+        <v>7612662.76</v>
       </c>
       <c r="E1267" s="15" t="n">
-        <v>126703083.65</v>
+        <v>126706759.4</v>
       </c>
       <c r="F1267" s="16" t="n">
-        <v>0.4429</v>
+        <v>0.4423</v>
       </c>
       <c r="G1267" s="16" t="n">
-        <v>0.3696</v>
+        <v>0.3689</v>
       </c>
       <c r="H1267" s="16" t="n"/>
       <c r="I1267" s="16" t="n">
         <v>0.0281</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>577685</v>
+        <v>577783</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>924054</v>
+        <v>924196</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63334,26 +63334,26 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>16243566.1</v>
+        <v>16263666.15</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>7814050.31</v>
+        <v>7822396.76</v>
       </c>
       <c r="F1268" s="10" t="n">
-        <v>0.0242</v>
+        <v>0.0237</v>
       </c>
       <c r="G1268" s="10" t="n">
-        <v>-0.0148</v>
+        <v>-0.0152</v>
       </c>
       <c r="H1268" s="10" t="n"/>
       <c r="I1268" s="10" t="n">
         <v>0.3128</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>64257</v>
+        <v>64309</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>255684</v>
+        <v>255834</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63376,26 +63376,26 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>10245462.62</v>
+        <v>10250417.67</v>
       </c>
       <c r="E1269" s="15" t="n">
-        <v>8807409.08</v>
+        <v>8814110.49</v>
       </c>
       <c r="F1269" s="16" t="n">
-        <v>0.0444</v>
+        <v>0.0443</v>
       </c>
       <c r="G1269" s="16" t="n">
-        <v>-0.0046</v>
+        <v>-0.0048</v>
       </c>
       <c r="H1269" s="16" t="n"/>
       <c r="I1269" s="16" t="n">
-        <v>0.2514</v>
+        <v>0.2515</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>92260</v>
+        <v>92346</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>234613</v>
+        <v>234781</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63418,26 +63418,26 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>7374048.53</v>
+        <v>7391430.73</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>10571888.78</v>
+        <v>10589434.91</v>
       </c>
       <c r="F1270" s="10" t="n">
-        <v>0.0323</v>
+        <v>0.0341</v>
       </c>
       <c r="G1270" s="10" t="n">
-        <v>-0.024</v>
+        <v>-0.0222</v>
       </c>
       <c r="H1270" s="10" t="n"/>
       <c r="I1270" s="10" t="n">
         <v>0.2067</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>102574</v>
+        <v>102644</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>215213</v>
+        <v>215334</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63460,26 +63460,26 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>4617796.22</v>
+        <v>4619485.08</v>
       </c>
       <c r="E1271" s="15" t="n">
-        <v>10995666.72</v>
+        <v>10997091.41</v>
       </c>
       <c r="F1271" s="16" t="n">
-        <v>0.1055</v>
+        <v>0.1054</v>
       </c>
       <c r="G1271" s="16" t="n">
-        <v>0.0436</v>
+        <v>0.0434</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
-        <v>0.1674</v>
+        <v>0.1673</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>100106</v>
+        <v>100151</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>189941</v>
+        <v>190014</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63502,26 +63502,26 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>6110804.24</v>
+        <v>6113109.08</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>20801670.83</v>
+        <v>20803826.57</v>
       </c>
       <c r="F1272" s="10" t="n">
-        <v>0.1452</v>
+        <v>0.1449</v>
       </c>
       <c r="G1272" s="10" t="n">
-        <v>0.07820000000000001</v>
+        <v>0.0779</v>
       </c>
       <c r="H1272" s="10" t="n"/>
       <c r="I1272" s="10" t="n">
         <v>0.1246</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>192931</v>
+        <v>193023</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>311171</v>
+        <v>311311</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63544,26 +63544,26 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>5744257.35</v>
+        <v>5746355.89</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>37982323.98</v>
+        <v>37988057.97</v>
       </c>
       <c r="F1273" s="16" t="n">
-        <v>0.2533</v>
+        <v>0.2412</v>
       </c>
       <c r="G1273" s="16" t="n">
-        <v>0.1854</v>
+        <v>0.1733</v>
       </c>
       <c r="H1273" s="16" t="n"/>
       <c r="I1273" s="16" t="n">
         <v>0.0736</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>244607</v>
+        <v>244696</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>425081</v>
+        <v>425222</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -68751,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-29 16:19 UTC</t>
+          <t>2026-10-29 17:29 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-30 13:36 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -6010,13 +6010,13 @@
         <v>46327</v>
       </c>
       <c r="B71" s="15" t="n">
-        <v>290023265.3</v>
+        <v>388768367.54</v>
       </c>
       <c r="C71" s="15" t="n">
-        <v>10824463.21</v>
+        <v>13448275.08</v>
       </c>
       <c r="D71" s="16" t="n">
-        <v>0.03732</v>
+        <v>0.03459</v>
       </c>
       <c r="E71" s="15" t="n">
         <v>77941885.75</v>
@@ -6033,31 +6033,31 @@
         </is>
       </c>
       <c r="I71" s="15" t="n">
-        <v>367965151.05</v>
+        <v>466710253.29</v>
       </c>
       <c r="J71" s="15" t="n">
-        <v>14133385.72</v>
+        <v>16757197.59</v>
       </c>
       <c r="K71" s="18" t="n">
-        <v>0.03841</v>
+        <v>0.0359</v>
       </c>
       <c r="L71" s="19" t="n">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="M71" s="19" t="n">
-        <v>320</v>
+        <v>275</v>
       </c>
       <c r="N71" s="15" t="n">
-        <v>46236350.82</v>
+        <v>94893876.34999999</v>
       </c>
       <c r="O71" s="16" t="n">
-        <v>0.03001</v>
+        <v>0.03309</v>
       </c>
       <c r="P71" s="15" t="n">
-        <v>159809004.13</v>
+        <v>186611185.43</v>
       </c>
       <c r="Q71" s="16" t="n">
-        <v>0.0246</v>
+        <v>0.02881</v>
       </c>
       <c r="R71" s="15" t="n">
         <v>48213465.27</v>
@@ -6066,16 +6066,16 @@
         <v>0.09447</v>
       </c>
       <c r="T71" s="15" t="n">
-        <v>14425136.43</v>
+        <v>22516612.21</v>
       </c>
       <c r="U71" s="16" t="n">
-        <v>0.03938</v>
+        <v>0.03578</v>
       </c>
       <c r="V71" s="15" t="n">
-        <v>21339308.66</v>
+        <v>36533228.28</v>
       </c>
       <c r="W71" s="16" t="n">
-        <v>0.01793</v>
+        <v>-0.01175</v>
       </c>
       <c r="X71" s="15" t="n"/>
       <c r="Y71" s="16" t="n"/>
@@ -7469,13 +7469,13 @@
         <v>46296</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>3494648252.56</v>
+        <v>3593393354.79</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>97555666.25</v>
+        <v>100179478.11</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.02792</v>
+        <v>0.02788</v>
       </c>
       <c r="E20" s="9" t="n">
         <v>989099510.4</v>
@@ -7492,31 +7492,31 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>4483747762.95</v>
+        <v>4582492865.19</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>271869115.63</v>
+        <v>274492927.49</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.06063</v>
+        <v>0.0599</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>895</v>
+        <v>913</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="N20" s="9" t="n">
-        <v>1383015756.65</v>
+        <v>1431673282.18</v>
       </c>
       <c r="O20" s="10" t="n">
-        <v>0.02467</v>
+        <v>0.02505</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>545795254.8</v>
+        <v>572597436.11</v>
       </c>
       <c r="Q20" s="10" t="n">
-        <v>0.03015</v>
+        <v>0.03127</v>
       </c>
       <c r="R20" s="9" t="n">
         <v>379761776.54</v>
@@ -7525,16 +7525,16 @@
         <v>0.0404</v>
       </c>
       <c r="T20" s="9" t="n">
-        <v>135070560.26</v>
+        <v>143162036.05</v>
       </c>
       <c r="U20" s="10" t="n">
-        <v>0.02916</v>
+        <v>0.02917</v>
       </c>
       <c r="V20" s="9" t="n">
-        <v>1051004904.3</v>
+        <v>1066198823.92</v>
       </c>
       <c r="W20" s="10" t="n">
-        <v>0.02636</v>
+        <v>0.02522</v>
       </c>
       <c r="X20" s="9" t="n"/>
       <c r="Y20" s="10" t="n"/>
@@ -8104,16 +8104,16 @@
         <v>0.1512</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>46236350.84</v>
+        <v>94893876.36</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>0.03</v>
+        <v>0.0331</v>
       </c>
       <c r="J12" s="13" t="n">
-        <v>221</v>
+        <v>179</v>
       </c>
       <c r="K12" s="26" t="n">
-        <v>5.2</v>
+        <v>4.6</v>
       </c>
       <c r="L12" s="9" t="n">
         <v>14901097.86</v>
@@ -8647,14 +8647,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-29 17:29 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-30 13:35 UTC.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>Season 2026 to date  ·  107 games</t>
+          <t>Season 2026 to date  ·  108 games</t>
         </is>
       </c>
     </row>
@@ -8717,31 +8717,31 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>1222920230.620002</v>
+        <v>1242148986.830002</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.03404194278386737</v>
+        <v>0.03414252607348797</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.009039838497393479</v>
+        <v>0.009209379238148975</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0.06037493218330366</v>
+        <v>0.05800499158414313</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>0.006968689250286157</v>
+        <v>0.00706927871311936</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>534.0624293301751</v>
+        <v>509.3571287102377</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>-0.002074811568598865</v>
+        <v>-0.001358699631071073</v>
       </c>
       <c r="I6" s="29" t="n">
-        <v>-6.148847194268542</v>
+        <v>-5.780773251111782</v>
       </c>
       <c r="J6" s="15" t="n">
-        <v>38219473.94999999</v>
+        <v>38713353.87999999</v>
       </c>
     </row>
     <row r="7">
@@ -8751,31 +8751,31 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>345301505.5900002</v>
+        <v>352825195.7700002</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.05820100122546935</v>
+        <v>0.05927148860319046</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>0.02891891636249267</v>
+        <v>0.03001278584113064</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.07070640341451558</v>
+        <v>0.07341357804171743</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.00121011320371372</v>
+        <v>0.001284147911845718</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>694.9629021080185</v>
+        <v>721.2943012987171</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>0.0008355540812259088</v>
+        <v>0.0007603501655704837</v>
       </c>
       <c r="I7" s="30" t="n">
-        <v>-7.233698673677703</v>
+        <v>-7.472572125270251</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>12638934.98</v>
+        <v>12904009.41</v>
       </c>
     </row>
     <row r="8">
@@ -8785,31 +8785,31 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>179565673.55</v>
+        <v>182795051.14</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.01693368604302492</v>
+        <v>0.01852958080033504</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>-0.01075434665112806</v>
+        <v>-0.009195987416051864</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>-0.04330797116837722</v>
+        <v>-0.03919452277885934</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>-0.009469878460504582</v>
+        <v>-0.009267089483668568</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>-338.3809270787264</v>
+        <v>-299.2743329519077</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>0.004648676925084292</v>
+        <v>0.004978644497512434</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>2.560108322595374</v>
+        <v>2.288052276752405</v>
       </c>
       <c r="J8" s="15" t="n">
-        <v>6214775.340000003</v>
+        <v>6335120.860000003</v>
       </c>
     </row>
     <row r="9">
@@ -8819,31 +8819,31 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>346346080.4</v>
+        <v>359657881.4</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>0.001824353748338238</v>
+        <v>0.001353932932331388</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>-0.02144233164533888</v>
+        <v>-0.02159652072621035</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>-0.02784298349082149</v>
+        <v>-0.02845774903697743</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>-0.009129245738717894</v>
+        <v>-0.009127565060159396</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-187.1373775210359</v>
+        <v>-193.3018397681803</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-0.01731253779212512</v>
+        <v>-0.01729053022507779</v>
       </c>
       <c r="I9" s="30" t="n">
-        <v>1.165126677544536</v>
+        <v>1.219707056616253</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>8216388.200000001</v>
+        <v>8418692.32</v>
       </c>
     </row>
     <row r="10">
@@ -8853,31 +8853,31 @@
         </is>
       </c>
       <c r="B10" s="15" t="n">
-        <v>146005654.84</v>
+        <v>148758742.44</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>0.05145533656373001</v>
+        <v>0.05002108688167529</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>0.02765169721970201</v>
+        <v>0.02617430482494471</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>0.05522358936650015</v>
+        <v>0.04979888046030893</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>0.007509571301164498</v>
+        <v>0.007549610435221038</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>477.1401806533566</v>
+        <v>422.492700250879</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>0.01949776159889655</v>
+        <v>0.01918376670634628</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>-3.427671862018092</v>
+        <v>-2.957949698613085</v>
       </c>
       <c r="J10" s="15" t="n">
-        <v>3475465.949999998</v>
+        <v>3547417.309999999</v>
       </c>
     </row>
     <row r="11">
@@ -8887,31 +8887,31 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>43361261.79</v>
+        <v>45972074.73999999</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.005174308604915702</v>
+        <v>0.005474498843555989</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>-0.0148828229013582</v>
+        <v>-0.01385246029468193</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0.0549229467682824</v>
+        <v>0.05511096312786019</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.003449239542388056</v>
+        <v>0.003509968750666112</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>514.7370722589434</v>
+        <v>516.0099437719407</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-0.03376440569841296</v>
+        <v>-0.03172761804996298</v>
       </c>
       <c r="I11" s="30" t="n">
-        <v>-4.164503123756305</v>
+        <v>-4.025313301042278</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>869702.5299999997</v>
+        <v>888500.4099999997</v>
       </c>
     </row>
     <row r="12">
@@ -8921,31 +8921,31 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>2283500406.789998</v>
+        <v>2332157932.319999</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>0.0320285360241348</v>
+        <v>0.0321116310658691</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>0.006601765366528518</v>
+        <v>0.006790783059981442</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>0.03210404513997277</v>
+        <v>0.03182867630774563</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>0.0003048262263836474</v>
+        <v>0.0003740526171751907</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>317.9921891358912</v>
+        <v>314.5462369057044</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>-0.00233380249877931</v>
+        <v>-0.001959245545720535</v>
       </c>
       <c r="I12" s="29" t="n">
-        <v>-3.643565526010595</v>
+        <v>-3.496222746052172</v>
       </c>
       <c r="J12" s="15" t="n">
-        <v>69634740.94999996</v>
+        <v>70807094.18999995</v>
       </c>
     </row>
     <row r="14">
@@ -9325,11 +9325,11 @@
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>W07 (Mon)</t>
+          <t>W07 (Mon) + W08 (Thu)</t>
         </is>
       </c>
       <c r="D26" s="19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
@@ -9337,25 +9337,25 @@
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>46236350.84</v>
+        <v>94893876.36</v>
       </c>
       <c r="G26" s="16" t="n">
-        <v>0.03</v>
+        <v>0.0331</v>
       </c>
       <c r="H26" s="16" t="n">
-        <v>0.0073</v>
+        <v>0.0116</v>
       </c>
       <c r="I26" s="15" t="n">
-        <v>-339609.72</v>
+        <v>-1101654.39</v>
       </c>
       <c r="J26" s="15" t="n">
-        <v>11581068.34</v>
+        <v>23039476.94</v>
       </c>
       <c r="K26" s="16" t="n">
-        <v>0.0267</v>
+        <v>0.0222</v>
       </c>
       <c r="L26" s="16" t="n">
-        <v>0.0047</v>
+        <v>0.0043</v>
       </c>
     </row>
     <row r="27">
@@ -68692,22 +68692,22 @@
         </is>
       </c>
       <c r="B12" s="33" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C12" s="34" t="n">
-        <v>1383015756.650002</v>
+        <v>1431673282.180002</v>
       </c>
       <c r="D12" s="35" t="n">
-        <v>0.02466700909658066</v>
+        <v>0.02505256106015008</v>
       </c>
       <c r="E12" s="35" t="n">
-        <v>0.01437533470975423</v>
+        <v>0.01448305115939996</v>
       </c>
       <c r="F12" s="35" t="n">
-        <v>-0.002234954162736131</v>
+        <v>-0.002027570201007317</v>
       </c>
       <c r="G12" s="33" t="n">
-        <v>166.1028887249036</v>
+        <v>165.1062136040727</v>
       </c>
       <c r="H12" s="36" t="n"/>
       <c r="I12" s="36" t="n"/>
@@ -68751,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-29 17:29 UTC</t>
+          <t>2026-10-30 13:35 UTC</t>
         </is>
       </c>
     </row>
@@ -68787,7 +68787,7 @@
       </c>
       <c r="B4" s="38" t="inlineStr">
         <is>
-          <t>491 (2025 post: from 2026-01-10, 2025 pre: from 2025-07-31, 2025 reg: from 2025-09-04, 2026 pre: from 2026-08-06, 2026 reg: from 2026-09-09)</t>
+          <t>492 (2025 post: from 2026-01-10, 2025 pre: from 2025-07-31, 2025 reg: from 2025-09-04, 2026 pre: from 2026-08-06, 2026 reg: from 2026-09-09)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-30 14:56 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -6019,13 +6019,13 @@
         <v>0.03459</v>
       </c>
       <c r="E71" s="15" t="n">
-        <v>77941885.75</v>
+        <v>108039933.87</v>
       </c>
       <c r="F71" s="15" t="n">
-        <v>3308922.51</v>
+        <v>7323492.1</v>
       </c>
       <c r="G71" s="16" t="n">
-        <v>0.04245</v>
+        <v>0.06779</v>
       </c>
       <c r="H71" s="17" t="inlineStr">
         <is>
@@ -6033,13 +6033,13 @@
         </is>
       </c>
       <c r="I71" s="15" t="n">
-        <v>466710253.29</v>
+        <v>496808301.41</v>
       </c>
       <c r="J71" s="15" t="n">
-        <v>16757197.59</v>
+        <v>20771767.18</v>
       </c>
       <c r="K71" s="18" t="n">
-        <v>0.0359</v>
+        <v>0.04181</v>
       </c>
       <c r="L71" s="19" t="n">
         <v>69</v>
@@ -7478,13 +7478,13 @@
         <v>0.02788</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>989099510.4</v>
+        <v>1018716501.02</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>174313449.38</v>
+        <v>177846829.26</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.17623</v>
+        <v>0.17458</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
@@ -7492,13 +7492,13 @@
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>4582492865.19</v>
+        <v>4612109855.82</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>274492927.49</v>
+        <v>278026307.37</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.0599</v>
+        <v>0.06028</v>
       </c>
       <c r="L20" s="13" t="n">
         <v>913</v>
@@ -8116,10 +8116,10 @@
         <v>4.6</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>14901097.86</v>
+        <v>22276768.18</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>-0.09429999999999999</v>
+        <v>-0.1308</v>
       </c>
     </row>
     <row r="13">
@@ -8647,7 +8647,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-30 13:35 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-30 14:56 UTC.</t>
         </is>
       </c>
     </row>
@@ -10224,26 +10224,26 @@
         </is>
       </c>
       <c r="D15" s="15" t="n">
-        <v>7496682.6</v>
+        <v>9628202.810000001</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>17200673.39</v>
+        <v>28147629.99</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>-0.0455</v>
+        <v>-0.0133</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>-0.1058</v>
+        <v>-0.07530000000000001</v>
       </c>
       <c r="H15" s="16" t="n"/>
       <c r="I15" s="16" t="n">
-        <v>0.1093</v>
+        <v>0.1235</v>
       </c>
       <c r="J15" s="19" t="n">
-        <v>140602</v>
+        <v>181952</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>229813</v>
+        <v>303383</v>
       </c>
       <c r="L15" s="31" t="n">
         <v>0</v>
@@ -13206,26 +13206,26 @@
         </is>
       </c>
       <c r="D86" s="9" t="n">
-        <v>471761.62</v>
+        <v>594314.1800000001</v>
       </c>
       <c r="E86" s="9" t="n">
-        <v>5920922.8</v>
+        <v>11116093.02</v>
       </c>
       <c r="F86" s="10" t="n">
-        <v>0.0664</v>
+        <v>0.2357</v>
       </c>
       <c r="G86" s="10" t="n">
-        <v>-0.0059</v>
+        <v>0.1517</v>
       </c>
       <c r="H86" s="10" t="n"/>
       <c r="I86" s="10" t="n">
-        <v>0.0314</v>
+        <v>0.0332</v>
       </c>
       <c r="J86" s="13" t="n">
-        <v>35575</v>
+        <v>45679</v>
       </c>
       <c r="K86" s="13" t="n">
-        <v>48617</v>
+        <v>67102</v>
       </c>
       <c r="L86" s="32" t="n">
         <v>0</v>
@@ -13248,26 +13248,26 @@
         </is>
       </c>
       <c r="D87" s="15" t="n">
-        <v>2392245.47</v>
+        <v>2941756.92</v>
       </c>
       <c r="E87" s="15" t="n">
-        <v>1537759.63</v>
+        <v>1861535.65</v>
       </c>
       <c r="F87" s="16" t="n">
-        <v>0.0756</v>
+        <v>0.0359</v>
       </c>
       <c r="G87" s="16" t="n">
-        <v>0.0235</v>
+        <v>-0.0152</v>
       </c>
       <c r="H87" s="16" t="n"/>
       <c r="I87" s="16" t="n">
-        <v>0.3269</v>
+        <v>0.3391</v>
       </c>
       <c r="J87" s="19" t="n">
-        <v>7719</v>
+        <v>9984</v>
       </c>
       <c r="K87" s="19" t="n">
-        <v>34254</v>
+        <v>41634</v>
       </c>
       <c r="L87" s="31" t="n">
         <v>0</v>
@@ -13290,26 +13290,26 @@
         </is>
       </c>
       <c r="D88" s="9" t="n">
-        <v>1490661.35</v>
+        <v>2011290.18</v>
       </c>
       <c r="E88" s="9" t="n">
-        <v>1403813.55</v>
+        <v>1970125.99</v>
       </c>
       <c r="F88" s="10" t="n">
-        <v>0.08019999999999999</v>
+        <v>0.0625</v>
       </c>
       <c r="G88" s="10" t="n">
-        <v>0.0223</v>
+        <v>0.0058</v>
       </c>
       <c r="H88" s="10" t="n"/>
       <c r="I88" s="10" t="n">
-        <v>0.2193</v>
+        <v>0.239</v>
       </c>
       <c r="J88" s="13" t="n">
-        <v>15060</v>
+        <v>19223</v>
       </c>
       <c r="K88" s="13" t="n">
-        <v>30564</v>
+        <v>39502</v>
       </c>
       <c r="L88" s="32" t="n">
         <v>0</v>
@@ -13332,26 +13332,26 @@
         </is>
       </c>
       <c r="D89" s="15" t="n">
-        <v>1136759.77</v>
+        <v>1471586.89</v>
       </c>
       <c r="E89" s="15" t="n">
-        <v>1910367.84</v>
+        <v>2656210.57</v>
       </c>
       <c r="F89" s="16" t="n">
-        <v>-0.3104</v>
+        <v>-0.2358</v>
       </c>
       <c r="G89" s="16" t="n">
-        <v>-0.3727</v>
+        <v>-0.2991</v>
       </c>
       <c r="H89" s="16" t="n"/>
       <c r="I89" s="16" t="n">
-        <v>0.1651</v>
+        <v>0.1841</v>
       </c>
       <c r="J89" s="19" t="n">
-        <v>17042</v>
+        <v>22068</v>
       </c>
       <c r="K89" s="19" t="n">
-        <v>28014</v>
+        <v>37115</v>
       </c>
       <c r="L89" s="31" t="n">
         <v>0</v>
@@ -13374,26 +13374,26 @@
         </is>
       </c>
       <c r="D90" s="9" t="n">
-        <v>755568.51</v>
+        <v>964113.25</v>
       </c>
       <c r="E90" s="9" t="n">
-        <v>1482815.64</v>
+        <v>2304002.46</v>
       </c>
       <c r="F90" s="10" t="n">
-        <v>-0.2621</v>
+        <v>-0.1571</v>
       </c>
       <c r="G90" s="10" t="n">
-        <v>-0.3288</v>
+        <v>-0.2262</v>
       </c>
       <c r="H90" s="10" t="n"/>
       <c r="I90" s="10" t="n">
-        <v>0.1314</v>
+        <v>0.1531</v>
       </c>
       <c r="J90" s="13" t="n">
-        <v>15544</v>
+        <v>20081</v>
       </c>
       <c r="K90" s="13" t="n">
-        <v>24290</v>
+        <v>31908</v>
       </c>
       <c r="L90" s="32" t="n">
         <v>0</v>
@@ -13416,26 +13416,26 @@
         </is>
       </c>
       <c r="D91" s="15" t="n">
-        <v>778101.22</v>
+        <v>1026499.18</v>
       </c>
       <c r="E91" s="15" t="n">
-        <v>2146423.35</v>
+        <v>3573596.74</v>
       </c>
       <c r="F91" s="16" t="n">
-        <v>-0.0916</v>
+        <v>0.0027</v>
       </c>
       <c r="G91" s="16" t="n">
-        <v>-0.1587</v>
+        <v>-0.06850000000000001</v>
       </c>
       <c r="H91" s="16" t="n"/>
       <c r="I91" s="16" t="n">
-        <v>0.0888</v>
+        <v>0.1088</v>
       </c>
       <c r="J91" s="19" t="n">
-        <v>25911</v>
+        <v>33968</v>
       </c>
       <c r="K91" s="19" t="n">
-        <v>33752</v>
+        <v>45424</v>
       </c>
       <c r="L91" s="31" t="n">
         <v>0</v>
@@ -13458,26 +13458,26 @@
         </is>
       </c>
       <c r="D92" s="9" t="n">
-        <v>471584.66</v>
+        <v>618642.21</v>
       </c>
       <c r="E92" s="9" t="n">
-        <v>2798570.57</v>
+        <v>4666065.55</v>
       </c>
       <c r="F92" s="10" t="n">
-        <v>-0.1081</v>
+        <v>-0.0056</v>
       </c>
       <c r="G92" s="10" t="n">
-        <v>-0.1787</v>
+        <v>-0.0863</v>
       </c>
       <c r="H92" s="10" t="n"/>
       <c r="I92" s="10" t="n">
-        <v>0.0534</v>
+        <v>0.0693</v>
       </c>
       <c r="J92" s="13" t="n">
-        <v>23751</v>
+        <v>30949</v>
       </c>
       <c r="K92" s="13" t="n">
-        <v>30322</v>
+        <v>40698</v>
       </c>
       <c r="L92" s="32" t="n">
         <v>0</v>
@@ -14886,26 +14886,26 @@
         </is>
       </c>
       <c r="D126" s="9" t="n">
-        <v>1792564.57</v>
+        <v>2898713.32</v>
       </c>
       <c r="E126" s="9" t="n">
-        <v>3293728.48</v>
+        <v>4296507.65</v>
       </c>
       <c r="F126" s="10" t="n">
-        <v>0.4267</v>
+        <v>0.4684</v>
       </c>
       <c r="G126" s="10" t="n">
-        <v>0.3738</v>
+        <v>0.4197</v>
       </c>
       <c r="H126" s="10" t="n"/>
       <c r="I126" s="10" t="n">
-        <v>0.07049999999999999</v>
+        <v>0.0775</v>
       </c>
       <c r="J126" s="13" t="n">
-        <v>32859</v>
+        <v>48555</v>
       </c>
       <c r="K126" s="13" t="n">
-        <v>83660</v>
+        <v>112684</v>
       </c>
       <c r="L126" s="32" t="n">
         <v>0</v>
@@ -17364,26 +17364,26 @@
         </is>
       </c>
       <c r="D185" s="15" t="n">
-        <v>157135.21</v>
+        <v>241960.38</v>
       </c>
       <c r="E185" s="15" t="n">
-        <v>680642.9</v>
+        <v>789319.26</v>
       </c>
       <c r="F185" s="16" t="n">
-        <v>1.0167</v>
+        <v>1.0267</v>
       </c>
       <c r="G185" s="16" t="n">
-        <v>0.9456</v>
+        <v>0.9569</v>
       </c>
       <c r="H185" s="16" t="n"/>
       <c r="I185" s="16" t="n">
         <v>0.0003</v>
       </c>
       <c r="J185" s="19" t="n">
-        <v>11716</v>
+        <v>17093</v>
       </c>
       <c r="K185" s="19" t="n">
-        <v>24628</v>
+        <v>31560</v>
       </c>
       <c r="L185" s="31" t="n">
         <v>0</v>
@@ -17406,26 +17406,26 @@
         </is>
       </c>
       <c r="D186" s="9" t="n">
-        <v>1055218.31</v>
+        <v>1576011.3</v>
       </c>
       <c r="E186" s="9" t="n">
-        <v>694021.84</v>
+        <v>1062192.68</v>
       </c>
       <c r="F186" s="10" t="n">
-        <v>0.2034</v>
+        <v>0.2619</v>
       </c>
       <c r="G186" s="10" t="n">
-        <v>0.1572</v>
+        <v>0.2179</v>
       </c>
       <c r="H186" s="10" t="n"/>
       <c r="I186" s="10" t="n">
-        <v>0.2841</v>
+        <v>0.2927</v>
       </c>
       <c r="J186" s="13" t="n">
-        <v>5125</v>
+        <v>7926</v>
       </c>
       <c r="K186" s="13" t="n">
-        <v>20137</v>
+        <v>29323</v>
       </c>
       <c r="L186" s="32" t="n">
         <v>0</v>
@@ -17448,26 +17448,26 @@
         </is>
       </c>
       <c r="D187" s="15" t="n">
-        <v>154050.74</v>
+        <v>429103.12</v>
       </c>
       <c r="E187" s="15" t="n">
-        <v>117821.97</v>
+        <v>188035.3</v>
       </c>
       <c r="F187" s="16" t="n">
-        <v>0.4205</v>
+        <v>0.4783</v>
       </c>
       <c r="G187" s="16" t="n">
-        <v>0.3692</v>
+        <v>0.4363</v>
       </c>
       <c r="H187" s="16" t="n"/>
       <c r="I187" s="16" t="n">
-        <v>0.1381</v>
+        <v>0.1522</v>
       </c>
       <c r="J187" s="19" t="n">
-        <v>3171</v>
+        <v>5236</v>
       </c>
       <c r="K187" s="19" t="n">
-        <v>4624</v>
+        <v>10198</v>
       </c>
       <c r="L187" s="31" t="n">
         <v>0</v>
@@ -17490,26 +17490,26 @@
         </is>
       </c>
       <c r="D188" s="9" t="n">
-        <v>154440.54</v>
+        <v>266826.92</v>
       </c>
       <c r="E188" s="9" t="n">
-        <v>137558.5</v>
+        <v>242737.54</v>
       </c>
       <c r="F188" s="10" t="n">
-        <v>0.5836</v>
+        <v>0.5897</v>
       </c>
       <c r="G188" s="10" t="n">
-        <v>0.5265</v>
+        <v>0.5409</v>
       </c>
       <c r="H188" s="10" t="n"/>
       <c r="I188" s="10" t="n">
-        <v>0.0774</v>
+        <v>0.08260000000000001</v>
       </c>
       <c r="J188" s="13" t="n">
-        <v>3967</v>
+        <v>5689</v>
       </c>
       <c r="K188" s="13" t="n">
-        <v>5638</v>
+        <v>7857</v>
       </c>
       <c r="L188" s="32" t="n">
         <v>0</v>
@@ -17532,26 +17532,26 @@
         </is>
       </c>
       <c r="D189" s="15" t="n">
-        <v>73402.27</v>
+        <v>110772.87</v>
       </c>
       <c r="E189" s="15" t="n">
-        <v>122618.92</v>
+        <v>171760.8</v>
       </c>
       <c r="F189" s="16" t="n">
-        <v>0.6366000000000001</v>
+        <v>0.6961000000000001</v>
       </c>
       <c r="G189" s="16" t="n">
-        <v>0.5737</v>
+        <v>0.6385</v>
       </c>
       <c r="H189" s="16" t="n"/>
       <c r="I189" s="16" t="n">
-        <v>0.0288</v>
+        <v>0.0297</v>
       </c>
       <c r="J189" s="19" t="n">
-        <v>1877</v>
+        <v>2792</v>
       </c>
       <c r="K189" s="19" t="n">
-        <v>2687</v>
+        <v>3914</v>
       </c>
       <c r="L189" s="31" t="n">
         <v>0</v>
@@ -17574,26 +17574,26 @@
         </is>
       </c>
       <c r="D190" s="9" t="n">
-        <v>79146.7</v>
+        <v>131930.68</v>
       </c>
       <c r="E190" s="9" t="n">
-        <v>219614.5</v>
+        <v>243626.86</v>
       </c>
       <c r="F190" s="10" t="n">
-        <v>0.8783</v>
+        <v>0.8801</v>
       </c>
       <c r="G190" s="10" t="n">
-        <v>0.8117</v>
+        <v>0.8214</v>
       </c>
       <c r="H190" s="10" t="n"/>
       <c r="I190" s="10" t="n">
-        <v>0.012</v>
+        <v>0.0124</v>
       </c>
       <c r="J190" s="13" t="n">
-        <v>3906</v>
+        <v>5703</v>
       </c>
       <c r="K190" s="13" t="n">
-        <v>5346</v>
+        <v>7589</v>
       </c>
       <c r="L190" s="32" t="n">
         <v>0</v>
@@ -17616,26 +17616,26 @@
         </is>
       </c>
       <c r="D191" s="15" t="n">
-        <v>119170.8</v>
+        <v>142108.05</v>
       </c>
       <c r="E191" s="15" t="n">
-        <v>1321449.86</v>
+        <v>1598835.2</v>
       </c>
       <c r="F191" s="16" t="n">
-        <v>1.0021</v>
+        <v>0.99</v>
       </c>
       <c r="G191" s="16" t="n">
-        <v>0.9328</v>
+        <v>0.9219000000000001</v>
       </c>
       <c r="H191" s="16" t="n"/>
       <c r="I191" s="16" t="n">
-        <v>0.0029</v>
+        <v>0.0036</v>
       </c>
       <c r="J191" s="19" t="n">
-        <v>3097</v>
+        <v>4116</v>
       </c>
       <c r="K191" s="19" t="n">
-        <v>20600</v>
+        <v>22243</v>
       </c>
       <c r="L191" s="31" t="n">
         <v>0</v>
@@ -18162,26 +18162,26 @@
         </is>
       </c>
       <c r="D204" s="9" t="n">
-        <v>4785450.27</v>
+        <v>5415885.44</v>
       </c>
       <c r="E204" s="9" t="n">
-        <v>6490799.19</v>
+        <v>8917091.09</v>
       </c>
       <c r="F204" s="10" t="n">
-        <v>0.3278</v>
+        <v>0.3167</v>
       </c>
       <c r="G204" s="10" t="n">
-        <v>0.2718</v>
+        <v>0.2602</v>
       </c>
       <c r="H204" s="10" t="n"/>
       <c r="I204" s="10" t="n">
-        <v>0.0771</v>
+        <v>0.08119999999999999</v>
       </c>
       <c r="J204" s="13" t="n">
-        <v>105146</v>
+        <v>120649</v>
       </c>
       <c r="K204" s="13" t="n">
-        <v>209674</v>
+        <v>238598</v>
       </c>
       <c r="L204" s="32" t="n">
         <v>0</v>
@@ -21732,26 +21732,26 @@
         </is>
       </c>
       <c r="D289" s="15" t="n">
-        <v>192624.19</v>
+        <v>209923.61</v>
       </c>
       <c r="E289" s="15" t="n">
-        <v>552013.54</v>
+        <v>853036.86</v>
       </c>
       <c r="F289" s="16" t="n">
-        <v>0.3029</v>
+        <v>0.3141</v>
       </c>
       <c r="G289" s="16" t="n">
-        <v>0.2743</v>
+        <v>0.2845</v>
       </c>
       <c r="H289" s="16" t="n"/>
       <c r="I289" s="16" t="n">
-        <v>0.0175</v>
+        <v>0.0226</v>
       </c>
       <c r="J289" s="19" t="n">
-        <v>6643</v>
+        <v>7480</v>
       </c>
       <c r="K289" s="19" t="n">
-        <v>10104</v>
+        <v>11504</v>
       </c>
       <c r="L289" s="31" t="n">
         <v>0</v>
@@ -21774,26 +21774,26 @@
         </is>
       </c>
       <c r="D290" s="9" t="n">
-        <v>2014435.94</v>
+        <v>2375780.34</v>
       </c>
       <c r="E290" s="9" t="n">
-        <v>921366.96</v>
+        <v>1341098.49</v>
       </c>
       <c r="F290" s="10" t="n">
-        <v>0.187</v>
+        <v>0.1835</v>
       </c>
       <c r="G290" s="10" t="n">
-        <v>0.1366</v>
+        <v>0.1328</v>
       </c>
       <c r="H290" s="10" t="n"/>
       <c r="I290" s="10" t="n">
-        <v>0.211</v>
+        <v>0.2128</v>
       </c>
       <c r="J290" s="13" t="n">
-        <v>10294</v>
+        <v>12213</v>
       </c>
       <c r="K290" s="13" t="n">
-        <v>50520</v>
+        <v>60154</v>
       </c>
       <c r="L290" s="32" t="n">
         <v>0</v>
@@ -21816,26 +21816,26 @@
         </is>
       </c>
       <c r="D291" s="15" t="n">
-        <v>860991.77</v>
+        <v>958980.28</v>
       </c>
       <c r="E291" s="15" t="n">
-        <v>893154.97</v>
+        <v>1182009.17</v>
       </c>
       <c r="F291" s="16" t="n">
-        <v>0.1862</v>
+        <v>0.1867</v>
       </c>
       <c r="G291" s="16" t="n">
-        <v>0.1291</v>
+        <v>0.1284</v>
       </c>
       <c r="H291" s="16" t="n"/>
       <c r="I291" s="16" t="n">
-        <v>0.1483</v>
+        <v>0.1521</v>
       </c>
       <c r="J291" s="19" t="n">
-        <v>16888</v>
+        <v>19863</v>
       </c>
       <c r="K291" s="19" t="n">
-        <v>34814</v>
+        <v>39801</v>
       </c>
       <c r="L291" s="31" t="n">
         <v>0</v>
@@ -21858,26 +21858,26 @@
         </is>
       </c>
       <c r="D292" s="9" t="n">
-        <v>649130.54</v>
+        <v>705454.28</v>
       </c>
       <c r="E292" s="9" t="n">
-        <v>837729.29</v>
+        <v>1125651.61</v>
       </c>
       <c r="F292" s="10" t="n">
-        <v>0.3584</v>
+        <v>0.3573</v>
       </c>
       <c r="G292" s="10" t="n">
-        <v>0.2963</v>
+        <v>0.2935</v>
       </c>
       <c r="H292" s="10" t="n"/>
       <c r="I292" s="10" t="n">
-        <v>0.0959</v>
+        <v>0.0999</v>
       </c>
       <c r="J292" s="13" t="n">
-        <v>17696</v>
+        <v>20486</v>
       </c>
       <c r="K292" s="13" t="n">
-        <v>28276</v>
+        <v>32269</v>
       </c>
       <c r="L292" s="32" t="n">
         <v>0</v>
@@ -21900,26 +21900,26 @@
         </is>
       </c>
       <c r="D293" s="15" t="n">
-        <v>381253.12</v>
+        <v>410173.48</v>
       </c>
       <c r="E293" s="15" t="n">
-        <v>568827.17</v>
+        <v>814636.27</v>
       </c>
       <c r="F293" s="16" t="n">
-        <v>0.4968</v>
+        <v>0.4934</v>
       </c>
       <c r="G293" s="16" t="n">
-        <v>0.431</v>
+        <v>0.4261</v>
       </c>
       <c r="H293" s="16" t="n"/>
       <c r="I293" s="16" t="n">
-        <v>0.057</v>
+        <v>0.0605</v>
       </c>
       <c r="J293" s="19" t="n">
-        <v>15221</v>
+        <v>17391</v>
       </c>
       <c r="K293" s="19" t="n">
-        <v>20365</v>
+        <v>23108</v>
       </c>
       <c r="L293" s="31" t="n">
         <v>0</v>
@@ -21942,26 +21942,26 @@
         </is>
       </c>
       <c r="D294" s="9" t="n">
-        <v>403444.29</v>
+        <v>452272.86</v>
       </c>
       <c r="E294" s="9" t="n">
-        <v>1092506.3</v>
+        <v>1596515.11</v>
       </c>
       <c r="F294" s="10" t="n">
-        <v>0.7482</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="G294" s="10" t="n">
-        <v>0.6802</v>
+        <v>0.6254</v>
       </c>
       <c r="H294" s="10" t="n"/>
       <c r="I294" s="10" t="n">
-        <v>0.0271</v>
+        <v>0.0288</v>
       </c>
       <c r="J294" s="13" t="n">
-        <v>22384</v>
+        <v>25359</v>
       </c>
       <c r="K294" s="13" t="n">
-        <v>29546</v>
+        <v>33269</v>
       </c>
       <c r="L294" s="32" t="n">
         <v>0</v>
@@ -21984,26 +21984,26 @@
         </is>
       </c>
       <c r="D295" s="15" t="n">
-        <v>283570.42</v>
+        <v>303300.6</v>
       </c>
       <c r="E295" s="15" t="n">
-        <v>1625200.97</v>
+        <v>2004143.57</v>
       </c>
       <c r="F295" s="16" t="n">
-        <v>0.8794999999999999</v>
+        <v>0.8796</v>
       </c>
       <c r="G295" s="16" t="n">
-        <v>0.8126</v>
+        <v>0.8125</v>
       </c>
       <c r="H295" s="16" t="n"/>
       <c r="I295" s="16" t="n">
-        <v>0.0092</v>
+        <v>0.01</v>
       </c>
       <c r="J295" s="19" t="n">
-        <v>16020</v>
+        <v>17857</v>
       </c>
       <c r="K295" s="19" t="n">
-        <v>36049</v>
+        <v>38493</v>
       </c>
       <c r="L295" s="31" t="n">
         <v>0</v>
@@ -22740,26 +22740,26 @@
         </is>
       </c>
       <c r="D313" s="15" t="n">
-        <v>31759806.78</v>
+        <v>42823625</v>
       </c>
       <c r="E313" s="15" t="n">
-        <v>43443488.49</v>
+        <v>85152288.59999999</v>
       </c>
       <c r="F313" s="16" t="n">
-        <v>-0.0539</v>
+        <v>0.0349</v>
       </c>
       <c r="G313" s="16" t="n">
-        <v>-0.1101</v>
+        <v>-0.0229</v>
       </c>
       <c r="H313" s="16" t="n"/>
       <c r="I313" s="16" t="n">
-        <v>0.1456</v>
+        <v>0.1353</v>
       </c>
       <c r="J313" s="19" t="n">
-        <v>706454</v>
+        <v>955582</v>
       </c>
       <c r="K313" s="19" t="n">
-        <v>1490895</v>
+        <v>2014819</v>
       </c>
       <c r="L313" s="31" t="n">
         <v>0</v>
@@ -27612,26 +27612,26 @@
         </is>
       </c>
       <c r="D429" s="15" t="n">
-        <v>3235977.62</v>
+        <v>4252594.38</v>
       </c>
       <c r="E429" s="15" t="n">
-        <v>11325204.28</v>
+        <v>29914459.76</v>
       </c>
       <c r="F429" s="16" t="n">
-        <v>-0.0028</v>
+        <v>0.2094</v>
       </c>
       <c r="G429" s="16" t="n">
-        <v>-0.073</v>
+        <v>0.1351</v>
       </c>
       <c r="H429" s="16" t="n"/>
       <c r="I429" s="16" t="n">
-        <v>0.0633</v>
+        <v>0.0529</v>
       </c>
       <c r="J429" s="19" t="n">
-        <v>219326</v>
+        <v>291514</v>
       </c>
       <c r="K429" s="19" t="n">
-        <v>444890</v>
+        <v>603672</v>
       </c>
       <c r="L429" s="31" t="n">
         <v>0</v>
@@ -27654,26 +27654,26 @@
         </is>
       </c>
       <c r="D430" s="9" t="n">
-        <v>11918111.23</v>
+        <v>16102145.12</v>
       </c>
       <c r="E430" s="9" t="n">
-        <v>6688723.39</v>
+        <v>9767879.119999999</v>
       </c>
       <c r="F430" s="10" t="n">
-        <v>-0.0449</v>
+        <v>-0.0363</v>
       </c>
       <c r="G430" s="10" t="n">
-        <v>-0.0944</v>
+        <v>-0.0856</v>
       </c>
       <c r="H430" s="10" t="n"/>
       <c r="I430" s="10" t="n">
-        <v>0.3242</v>
+        <v>0.3196</v>
       </c>
       <c r="J430" s="13" t="n">
-        <v>54342</v>
+        <v>75150</v>
       </c>
       <c r="K430" s="13" t="n">
-        <v>197793</v>
+        <v>271580</v>
       </c>
       <c r="L430" s="32" t="n">
         <v>0</v>
@@ -27696,26 +27696,26 @@
         </is>
       </c>
       <c r="D431" s="15" t="n">
-        <v>5286459.84</v>
+        <v>7519401.81</v>
       </c>
       <c r="E431" s="15" t="n">
-        <v>4081132.53</v>
+        <v>6894779.71</v>
       </c>
       <c r="F431" s="16" t="n">
-        <v>-0.0456</v>
+        <v>0.0391</v>
       </c>
       <c r="G431" s="16" t="n">
-        <v>-0.0973</v>
+        <v>-0.0145</v>
       </c>
       <c r="H431" s="16" t="n"/>
       <c r="I431" s="16" t="n">
-        <v>0.2405</v>
+        <v>0.2308</v>
       </c>
       <c r="J431" s="19" t="n">
-        <v>70748</v>
+        <v>97824</v>
       </c>
       <c r="K431" s="19" t="n">
-        <v>153789</v>
+        <v>234837</v>
       </c>
       <c r="L431" s="31" t="n">
         <v>0</v>
@@ -27738,26 +27738,26 @@
         </is>
       </c>
       <c r="D432" s="9" t="n">
-        <v>3758471.11</v>
+        <v>4896348.64</v>
       </c>
       <c r="E432" s="9" t="n">
-        <v>4239130.46</v>
+        <v>7262291.97</v>
       </c>
       <c r="F432" s="10" t="n">
-        <v>0.0261</v>
+        <v>0.1033</v>
       </c>
       <c r="G432" s="10" t="n">
-        <v>-0.0314</v>
+        <v>0.0435</v>
       </c>
       <c r="H432" s="10" t="n"/>
       <c r="I432" s="10" t="n">
-        <v>0.1975</v>
+        <v>0.1852</v>
       </c>
       <c r="J432" s="13" t="n">
-        <v>80610</v>
+        <v>108540</v>
       </c>
       <c r="K432" s="13" t="n">
-        <v>161972</v>
+        <v>209924</v>
       </c>
       <c r="L432" s="32" t="n">
         <v>0</v>
@@ -27780,26 +27780,26 @@
         </is>
       </c>
       <c r="D433" s="15" t="n">
-        <v>2171759.29</v>
+        <v>2935759.79</v>
       </c>
       <c r="E433" s="15" t="n">
-        <v>2492942.93</v>
+        <v>4877075.14</v>
       </c>
       <c r="F433" s="16" t="n">
-        <v>-0.0658</v>
+        <v>0.043</v>
       </c>
       <c r="G433" s="16" t="n">
-        <v>-0.1258</v>
+        <v>-0.019</v>
       </c>
       <c r="H433" s="16" t="n"/>
       <c r="I433" s="16" t="n">
-        <v>0.1743</v>
+        <v>0.1612</v>
       </c>
       <c r="J433" s="19" t="n">
-        <v>63370</v>
+        <v>86333</v>
       </c>
       <c r="K433" s="19" t="n">
-        <v>102059</v>
+        <v>140741</v>
       </c>
       <c r="L433" s="31" t="n">
         <v>0</v>
@@ -27822,26 +27822,26 @@
         </is>
       </c>
       <c r="D434" s="9" t="n">
-        <v>3038315.55</v>
+        <v>4029877.54</v>
       </c>
       <c r="E434" s="9" t="n">
-        <v>5345961.14</v>
+        <v>9658321.09</v>
       </c>
       <c r="F434" s="10" t="n">
-        <v>-0.1452</v>
+        <v>0.0394</v>
       </c>
       <c r="G434" s="10" t="n">
-        <v>-0.2078</v>
+        <v>-0.0267</v>
       </c>
       <c r="H434" s="10" t="n"/>
       <c r="I434" s="10" t="n">
-        <v>0.1397</v>
+        <v>0.1272</v>
       </c>
       <c r="J434" s="13" t="n">
-        <v>109830</v>
+        <v>149554</v>
       </c>
       <c r="K434" s="13" t="n">
-        <v>204735</v>
+        <v>267106</v>
       </c>
       <c r="L434" s="32" t="n">
         <v>0</v>
@@ -27864,26 +27864,26 @@
         </is>
       </c>
       <c r="D435" s="15" t="n">
-        <v>2350712.14</v>
+        <v>3087497.73</v>
       </c>
       <c r="E435" s="15" t="n">
-        <v>9270393.77</v>
+        <v>16777481.81</v>
       </c>
       <c r="F435" s="16" t="n">
-        <v>-0.1878</v>
+        <v>0.0336</v>
       </c>
       <c r="G435" s="16" t="n">
-        <v>-0.2549</v>
+        <v>-0.0381</v>
       </c>
       <c r="H435" s="16" t="n"/>
       <c r="I435" s="16" t="n">
-        <v>0.111</v>
+        <v>0.0969</v>
       </c>
       <c r="J435" s="19" t="n">
-        <v>108228</v>
+        <v>146667</v>
       </c>
       <c r="K435" s="19" t="n">
-        <v>225657</v>
+        <v>286959</v>
       </c>
       <c r="L435" s="31" t="n">
         <v>0</v>
@@ -29226,31 +29226,31 @@
         </is>
       </c>
       <c r="D466" s="9" t="n">
-        <v>14901097.86</v>
+        <v>22276768.18</v>
       </c>
       <c r="E466" s="9" t="n">
-        <v>38612880.59</v>
+        <v>52409451.1</v>
       </c>
       <c r="F466" s="10" t="n">
-        <v>-0.09429999999999999</v>
+        <v>-0.1308</v>
       </c>
       <c r="G466" s="10" t="n">
-        <v>-0.1506</v>
+        <v>-0.1882</v>
       </c>
       <c r="H466" s="10" t="n">
-        <v>0.1577</v>
+        <v>0.1448</v>
       </c>
       <c r="I466" s="10" t="n">
-        <v>0.1135</v>
+        <v>0.1298</v>
       </c>
       <c r="J466" s="13" t="n">
-        <v>377462</v>
+        <v>569390</v>
       </c>
       <c r="K466" s="13" t="n">
-        <v>734000</v>
+        <v>1076453</v>
       </c>
       <c r="L466" s="32" t="n">
-        <v>0.5637</v>
+        <v>0.706</v>
       </c>
     </row>
     <row r="467">
@@ -38414,31 +38414,31 @@
         </is>
       </c>
       <c r="D675" s="15" t="n">
-        <v>1263400.75</v>
+        <v>1712501.55</v>
       </c>
       <c r="E675" s="15" t="n">
-        <v>16092576.5</v>
+        <v>19027244.59</v>
       </c>
       <c r="F675" s="16" t="n">
-        <v>0.6099</v>
+        <v>0.4217</v>
       </c>
       <c r="G675" s="16" t="n">
-        <v>0.5352</v>
+        <v>0.3477</v>
       </c>
       <c r="H675" s="16" t="n">
-        <v>0.59</v>
+        <v>0.5787</v>
       </c>
       <c r="I675" s="16" t="n">
-        <v>0.0256</v>
+        <v>0.0379</v>
       </c>
       <c r="J675" s="19" t="n">
-        <v>88522</v>
+        <v>120441</v>
       </c>
       <c r="K675" s="19" t="n">
-        <v>179212</v>
+        <v>232528</v>
       </c>
       <c r="L675" s="31" t="n">
-        <v>0.6815</v>
+        <v>0.7635999999999999</v>
       </c>
     </row>
     <row r="676">
@@ -38458,31 +38458,31 @@
         </is>
       </c>
       <c r="D676" s="9" t="n">
-        <v>4423439.96</v>
+        <v>6610352.87</v>
       </c>
       <c r="E676" s="9" t="n">
-        <v>3416598.36</v>
+        <v>4311485.79</v>
       </c>
       <c r="F676" s="10" t="n">
-        <v>-0.2302</v>
+        <v>-0.1646</v>
       </c>
       <c r="G676" s="10" t="n">
-        <v>-0.2819</v>
+        <v>-0.217</v>
       </c>
       <c r="H676" s="10" t="n">
-        <v>0.068</v>
+        <v>0.0589</v>
       </c>
       <c r="I676" s="10" t="n">
-        <v>0.2619</v>
+        <v>0.2728</v>
       </c>
       <c r="J676" s="13" t="n">
-        <v>21482</v>
+        <v>32565</v>
       </c>
       <c r="K676" s="13" t="n">
-        <v>92656</v>
+        <v>142527</v>
       </c>
       <c r="L676" s="32" t="n">
-        <v>0.5157</v>
+        <v>0.6732</v>
       </c>
     </row>
     <row r="677">
@@ -38502,31 +38502,31 @@
         </is>
       </c>
       <c r="D677" s="15" t="n">
-        <v>2413989.85</v>
+        <v>3583045.23</v>
       </c>
       <c r="E677" s="15" t="n">
-        <v>4636579.74</v>
+        <v>5225597.01</v>
       </c>
       <c r="F677" s="16" t="n">
-        <v>-0.3412</v>
+        <v>-0.2784</v>
       </c>
       <c r="G677" s="16" t="n">
-        <v>-0.3913</v>
+        <v>-0.3306</v>
       </c>
       <c r="H677" s="16" t="n">
-        <v>0.0733</v>
+        <v>0.06510000000000001</v>
       </c>
       <c r="I677" s="16" t="n">
-        <v>0.2217</v>
+        <v>0.231</v>
       </c>
       <c r="J677" s="19" t="n">
-        <v>38204</v>
+        <v>58450</v>
       </c>
       <c r="K677" s="19" t="n">
-        <v>85547</v>
+        <v>125030</v>
       </c>
       <c r="L677" s="31" t="n">
-        <v>0.5235</v>
+        <v>0.6775</v>
       </c>
     </row>
     <row r="678">
@@ -38546,31 +38546,31 @@
         </is>
       </c>
       <c r="D678" s="9" t="n">
-        <v>2043446.47</v>
+        <v>3234938.39</v>
       </c>
       <c r="E678" s="9" t="n">
-        <v>1815308.29</v>
+        <v>2526511.03</v>
       </c>
       <c r="F678" s="10" t="n">
-        <v>-0.2633</v>
+        <v>-0.298</v>
       </c>
       <c r="G678" s="10" t="n">
-        <v>-0.3173</v>
+        <v>-0.354</v>
       </c>
       <c r="H678" s="10" t="n">
-        <v>0.1434</v>
+        <v>0.1083</v>
       </c>
       <c r="I678" s="10" t="n">
-        <v>0.1814</v>
+        <v>0.1897</v>
       </c>
       <c r="J678" s="13" t="n">
-        <v>46818</v>
+        <v>74041</v>
       </c>
       <c r="K678" s="13" t="n">
-        <v>76563</v>
+        <v>126166</v>
       </c>
       <c r="L678" s="32" t="n">
-        <v>0.5703</v>
+        <v>0.7262999999999999</v>
       </c>
     </row>
     <row r="679">
@@ -38590,31 +38590,31 @@
         </is>
       </c>
       <c r="D679" s="15" t="n">
-        <v>1500413.95</v>
+        <v>2230726.28</v>
       </c>
       <c r="E679" s="15" t="n">
-        <v>1647044.73</v>
+        <v>2505235.27</v>
       </c>
       <c r="F679" s="16" t="n">
-        <v>-0.1101</v>
+        <v>-0.1692</v>
       </c>
       <c r="G679" s="16" t="n">
-        <v>-0.165</v>
+        <v>-0.2263</v>
       </c>
       <c r="H679" s="16" t="n">
-        <v>0.1866</v>
+        <v>0.155</v>
       </c>
       <c r="I679" s="16" t="n">
-        <v>0.1433</v>
+        <v>0.1568</v>
       </c>
       <c r="J679" s="19" t="n">
-        <v>43626</v>
+        <v>68352</v>
       </c>
       <c r="K679" s="19" t="n">
-        <v>65498</v>
+        <v>99160</v>
       </c>
       <c r="L679" s="31" t="n">
-        <v>0.5366</v>
+        <v>0.6862</v>
       </c>
     </row>
     <row r="680">
@@ -38634,31 +38634,31 @@
         </is>
       </c>
       <c r="D680" s="9" t="n">
-        <v>1802024.96</v>
+        <v>2746606.44</v>
       </c>
       <c r="E680" s="9" t="n">
-        <v>4401269.39</v>
+        <v>7012804.35</v>
       </c>
       <c r="F680" s="10" t="n">
-        <v>-0.015</v>
+        <v>-0.09520000000000001</v>
       </c>
       <c r="G680" s="10" t="n">
-        <v>-0.074</v>
+        <v>-0.1558</v>
       </c>
       <c r="H680" s="10" t="n">
-        <v>0.2777</v>
+        <v>0.2387</v>
       </c>
       <c r="I680" s="10" t="n">
-        <v>0.1024</v>
+        <v>0.1189</v>
       </c>
       <c r="J680" s="13" t="n">
-        <v>72418</v>
+        <v>112197</v>
       </c>
       <c r="K680" s="13" t="n">
-        <v>95118</v>
+        <v>154576</v>
       </c>
       <c r="L680" s="32" t="n">
-        <v>0.5818</v>
+        <v>0.7225</v>
       </c>
     </row>
     <row r="681">
@@ -38678,31 +38678,31 @@
         </is>
       </c>
       <c r="D681" s="15" t="n">
-        <v>1454381.92</v>
+        <v>2158597.43</v>
       </c>
       <c r="E681" s="15" t="n">
-        <v>6603503.57</v>
+        <v>11800573.07</v>
       </c>
       <c r="F681" s="16" t="n">
-        <v>0.2729</v>
+        <v>0.0238</v>
       </c>
       <c r="G681" s="16" t="n">
-        <v>0.207</v>
+        <v>-0.0425</v>
       </c>
       <c r="H681" s="16" t="n">
-        <v>0.438</v>
+        <v>0.3814</v>
       </c>
       <c r="I681" s="16" t="n">
-        <v>0.0648</v>
+        <v>0.0859</v>
       </c>
       <c r="J681" s="19" t="n">
-        <v>66392</v>
+        <v>103344</v>
       </c>
       <c r="K681" s="19" t="n">
-        <v>139406</v>
+        <v>196466</v>
       </c>
       <c r="L681" s="31" t="n">
-        <v>0.6707</v>
+        <v>0.7769</v>
       </c>
     </row>
     <row r="682">
@@ -39268,29 +39268,29 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>3434206.39</v>
+        <v>5066549.86</v>
       </c>
       <c r="E695" s="15" t="n">
-        <v>26899974.2</v>
+        <v>33654585.55</v>
       </c>
       <c r="F695" s="16" t="n">
-        <v>0.1942</v>
+        <v>0.2433</v>
       </c>
       <c r="G695" s="16" t="n">
-        <v>0.1253</v>
+        <v>0.1758</v>
       </c>
       <c r="H695" s="16" t="n"/>
       <c r="I695" s="16" t="n">
-        <v>0.0507</v>
+        <v>0.0506</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>162355</v>
+        <v>219820</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>221052</v>
+        <v>303664</v>
       </c>
       <c r="L695" s="31" t="n">
-        <v>0.5554</v>
+        <v>0.6791</v>
       </c>
     </row>
     <row r="696">
@@ -43132,29 +43132,29 @@
         </is>
       </c>
       <c r="D787" s="15" t="n">
-        <v>994073.34</v>
+        <v>1429125.21</v>
       </c>
       <c r="E787" s="15" t="n">
-        <v>18962832.56</v>
+        <v>23552639.9</v>
       </c>
       <c r="F787" s="16" t="n">
-        <v>0.6096</v>
+        <v>0.6092</v>
       </c>
       <c r="G787" s="16" t="n">
-        <v>0.5288</v>
+        <v>0.5314</v>
       </c>
       <c r="H787" s="16" t="n"/>
       <c r="I787" s="16" t="n">
-        <v>0.0169</v>
+        <v>0.0166</v>
       </c>
       <c r="J787" s="19" t="n">
-        <v>96076</v>
+        <v>128165</v>
       </c>
       <c r="K787" s="19" t="n">
-        <v>127867</v>
+        <v>174111</v>
       </c>
       <c r="L787" s="31" t="n">
-        <v>0.4599</v>
+        <v>0.5848</v>
       </c>
     </row>
     <row r="788">
@@ -43174,29 +43174,29 @@
         </is>
       </c>
       <c r="D788" s="9" t="n">
-        <v>454072.95</v>
+        <v>633364.6</v>
       </c>
       <c r="E788" s="9" t="n">
-        <v>700562.28</v>
+        <v>772415.95</v>
       </c>
       <c r="F788" s="10" t="n">
-        <v>-0.6693</v>
+        <v>-0.4263</v>
       </c>
       <c r="G788" s="10" t="n">
-        <v>-0.7177</v>
+        <v>-0.475</v>
       </c>
       <c r="H788" s="10" t="n"/>
       <c r="I788" s="10" t="n">
-        <v>0.3463</v>
+        <v>0.3506</v>
       </c>
       <c r="J788" s="13" t="n">
-        <v>1897</v>
+        <v>2955</v>
       </c>
       <c r="K788" s="13" t="n">
-        <v>4777</v>
+        <v>7294</v>
       </c>
       <c r="L788" s="32" t="n">
-        <v>0.5041</v>
+        <v>0.6375</v>
       </c>
     </row>
     <row r="789">
@@ -43216,29 +43216,29 @@
         </is>
       </c>
       <c r="D789" s="15" t="n">
-        <v>414325.32</v>
+        <v>617007.66</v>
       </c>
       <c r="E789" s="15" t="n">
-        <v>284326.57</v>
+        <v>447141.6</v>
       </c>
       <c r="F789" s="16" t="n">
-        <v>-0.0328</v>
+        <v>0.0477</v>
       </c>
       <c r="G789" s="16" t="n">
-        <v>-0.08110000000000001</v>
+        <v>-0.0047</v>
       </c>
       <c r="H789" s="16" t="n"/>
       <c r="I789" s="16" t="n">
-        <v>0.2365</v>
+        <v>0.2261</v>
       </c>
       <c r="J789" s="19" t="n">
-        <v>4470</v>
+        <v>6776</v>
       </c>
       <c r="K789" s="19" t="n">
-        <v>7693</v>
+        <v>11223</v>
       </c>
       <c r="L789" s="31" t="n">
-        <v>0.6821</v>
+        <v>0.7779</v>
       </c>
     </row>
     <row r="790">
@@ -43258,29 +43258,29 @@
         </is>
       </c>
       <c r="D790" s="9" t="n">
-        <v>336941.74</v>
+        <v>578968.53</v>
       </c>
       <c r="E790" s="9" t="n">
-        <v>562369.47</v>
+        <v>798054.73</v>
       </c>
       <c r="F790" s="10" t="n">
-        <v>0.1593</v>
+        <v>0.2309</v>
       </c>
       <c r="G790" s="10" t="n">
-        <v>0.09660000000000001</v>
+        <v>0.1698</v>
       </c>
       <c r="H790" s="10" t="n"/>
       <c r="I790" s="10" t="n">
-        <v>0.1659</v>
+        <v>0.1616</v>
       </c>
       <c r="J790" s="13" t="n">
-        <v>6546</v>
+        <v>9513</v>
       </c>
       <c r="K790" s="13" t="n">
-        <v>9242</v>
+        <v>13551</v>
       </c>
       <c r="L790" s="32" t="n">
-        <v>0.6136</v>
+        <v>0.7548</v>
       </c>
     </row>
     <row r="791">
@@ -43300,29 +43300,29 @@
         </is>
       </c>
       <c r="D791" s="15" t="n">
-        <v>317188.44</v>
+        <v>472588.67</v>
       </c>
       <c r="E791" s="15" t="n">
-        <v>739755.8100000001</v>
+        <v>964506.48</v>
       </c>
       <c r="F791" s="16" t="n">
-        <v>0.1999</v>
+        <v>0.2834</v>
       </c>
       <c r="G791" s="16" t="n">
-        <v>0.1298</v>
+        <v>0.2152</v>
       </c>
       <c r="H791" s="16" t="n"/>
       <c r="I791" s="16" t="n">
-        <v>0.1222</v>
+        <v>0.1139</v>
       </c>
       <c r="J791" s="19" t="n">
-        <v>8176</v>
+        <v>11374</v>
       </c>
       <c r="K791" s="19" t="n">
-        <v>15205</v>
+        <v>19574</v>
       </c>
       <c r="L791" s="31" t="n">
-        <v>0.695</v>
+        <v>0.7914</v>
       </c>
     </row>
     <row r="792">
@@ -43342,29 +43342,29 @@
         </is>
       </c>
       <c r="D792" s="9" t="n">
-        <v>472400.25</v>
+        <v>678280.29</v>
       </c>
       <c r="E792" s="9" t="n">
-        <v>1902020.09</v>
+        <v>2332051.08</v>
       </c>
       <c r="F792" s="10" t="n">
-        <v>0.2224</v>
+        <v>0.2305</v>
       </c>
       <c r="G792" s="10" t="n">
-        <v>0.1483</v>
+        <v>0.1585</v>
       </c>
       <c r="H792" s="10" t="n"/>
       <c r="I792" s="10" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.074</v>
       </c>
       <c r="J792" s="13" t="n">
-        <v>18866</v>
+        <v>25608</v>
       </c>
       <c r="K792" s="13" t="n">
-        <v>23676</v>
+        <v>31864</v>
       </c>
       <c r="L792" s="32" t="n">
-        <v>0.5726</v>
+        <v>0.6948</v>
       </c>
     </row>
     <row r="793">
@@ -43384,29 +43384,29 @@
         </is>
       </c>
       <c r="D793" s="15" t="n">
-        <v>445204.36</v>
+        <v>657214.91</v>
       </c>
       <c r="E793" s="15" t="n">
-        <v>3748107.41</v>
+        <v>4787775.8</v>
       </c>
       <c r="F793" s="16" t="n">
-        <v>0.3507</v>
+        <v>0.2715</v>
       </c>
       <c r="G793" s="16" t="n">
-        <v>0.2702</v>
+        <v>0.1938</v>
       </c>
       <c r="H793" s="16" t="n"/>
       <c r="I793" s="16" t="n">
-        <v>0.051</v>
+        <v>0.0479</v>
       </c>
       <c r="J793" s="19" t="n">
-        <v>26324</v>
+        <v>35429</v>
       </c>
       <c r="K793" s="19" t="n">
-        <v>32592</v>
+        <v>46047</v>
       </c>
       <c r="L793" s="31" t="n">
-        <v>0.5412</v>
+        <v>0.6681</v>
       </c>
     </row>
     <row r="794">
@@ -44350,29 +44350,29 @@
         </is>
       </c>
       <c r="D816" s="9" t="n">
-        <v>10064034.13</v>
+        <v>13339658.55</v>
       </c>
       <c r="E816" s="9" t="n">
-        <v>26543135.79</v>
+        <v>29524400.32</v>
       </c>
       <c r="F816" s="10" t="n">
-        <v>0.3717</v>
+        <v>0.2978</v>
       </c>
       <c r="G816" s="10" t="n">
-        <v>0.3126</v>
+        <v>0.2387</v>
       </c>
       <c r="H816" s="10" t="n"/>
       <c r="I816" s="10" t="n">
-        <v>0.0741</v>
+        <v>0.0767</v>
       </c>
       <c r="J816" s="13" t="n">
-        <v>195156</v>
+        <v>262359</v>
       </c>
       <c r="K816" s="13" t="n">
-        <v>362605</v>
+        <v>499346</v>
       </c>
       <c r="L816" s="32" t="n">
-        <v>0.6153</v>
+        <v>0.7060999999999999</v>
       </c>
     </row>
     <row r="817">
@@ -50860,29 +50860,29 @@
         </is>
       </c>
       <c r="D971" s="15" t="n">
-        <v>859811.66</v>
+        <v>1240535.33</v>
       </c>
       <c r="E971" s="15" t="n">
-        <v>10273208.24</v>
+        <v>11160154.03</v>
       </c>
       <c r="F971" s="16" t="n">
-        <v>0.7223000000000001</v>
+        <v>0.6786</v>
       </c>
       <c r="G971" s="16" t="n">
-        <v>0.649</v>
+        <v>0.6075</v>
       </c>
       <c r="H971" s="16" t="n"/>
       <c r="I971" s="16" t="n">
-        <v>0.0189</v>
+        <v>0.0199</v>
       </c>
       <c r="J971" s="19" t="n">
-        <v>62213</v>
+        <v>86017</v>
       </c>
       <c r="K971" s="19" t="n">
-        <v>111271</v>
+        <v>150642</v>
       </c>
       <c r="L971" s="31" t="n">
-        <v>0.6149</v>
+        <v>0.7304</v>
       </c>
     </row>
     <row r="972">
@@ -50902,29 +50902,29 @@
         </is>
       </c>
       <c r="D972" s="9" t="n">
-        <v>3231531.18</v>
+        <v>4269866.1</v>
       </c>
       <c r="E972" s="9" t="n">
-        <v>1830307.86</v>
+        <v>2365428.41</v>
       </c>
       <c r="F972" s="10" t="n">
-        <v>0.209</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="G972" s="10" t="n">
-        <v>0.16</v>
+        <v>0.0343</v>
       </c>
       <c r="H972" s="10" t="n"/>
       <c r="I972" s="10" t="n">
-        <v>0.3032</v>
+        <v>0.3233</v>
       </c>
       <c r="J972" s="13" t="n">
-        <v>7925</v>
+        <v>10841</v>
       </c>
       <c r="K972" s="13" t="n">
-        <v>37890</v>
+        <v>48039</v>
       </c>
       <c r="L972" s="32" t="n">
-        <v>0.6669</v>
+        <v>0.7445000000000001</v>
       </c>
     </row>
     <row r="973">
@@ -50944,29 +50944,29 @@
         </is>
       </c>
       <c r="D973" s="15" t="n">
-        <v>1909008.81</v>
+        <v>2390782.89</v>
       </c>
       <c r="E973" s="15" t="n">
-        <v>1732883.52</v>
+        <v>1881433.99</v>
       </c>
       <c r="F973" s="16" t="n">
-        <v>0.2944</v>
+        <v>0.303</v>
       </c>
       <c r="G973" s="16" t="n">
-        <v>0.24</v>
+        <v>0.2484</v>
       </c>
       <c r="H973" s="16" t="n"/>
       <c r="I973" s="16" t="n">
-        <v>0.1954</v>
+        <v>0.1994</v>
       </c>
       <c r="J973" s="19" t="n">
-        <v>15546</v>
+        <v>20901</v>
       </c>
       <c r="K973" s="19" t="n">
-        <v>32141</v>
+        <v>42724</v>
       </c>
       <c r="L973" s="31" t="n">
-        <v>0.5682</v>
+        <v>0.6525</v>
       </c>
     </row>
     <row r="974">
@@ -50986,29 +50986,29 @@
         </is>
       </c>
       <c r="D974" s="9" t="n">
-        <v>1335135.71</v>
+        <v>1816826.34</v>
       </c>
       <c r="E974" s="9" t="n">
-        <v>1763738.57</v>
+        <v>1887245.08</v>
       </c>
       <c r="F974" s="10" t="n">
-        <v>0.392</v>
+        <v>0.4069</v>
       </c>
       <c r="G974" s="10" t="n">
-        <v>0.3308</v>
+        <v>0.3466</v>
       </c>
       <c r="H974" s="10" t="n"/>
       <c r="I974" s="10" t="n">
-        <v>0.1295</v>
+        <v>0.1316</v>
       </c>
       <c r="J974" s="13" t="n">
-        <v>20833</v>
+        <v>27856</v>
       </c>
       <c r="K974" s="13" t="n">
-        <v>36552</v>
+        <v>52125</v>
       </c>
       <c r="L974" s="32" t="n">
-        <v>0.5959</v>
+        <v>0.7006</v>
       </c>
     </row>
     <row r="975">
@@ -51028,29 +51028,29 @@
         </is>
       </c>
       <c r="D975" s="15" t="n">
-        <v>885908.73</v>
+        <v>1120309.96</v>
       </c>
       <c r="E975" s="15" t="n">
-        <v>1921867.56</v>
+        <v>2123824.86</v>
       </c>
       <c r="F975" s="16" t="n">
-        <v>0.4498</v>
+        <v>0.3949</v>
       </c>
       <c r="G975" s="16" t="n">
-        <v>0.3843</v>
+        <v>0.3303</v>
       </c>
       <c r="H975" s="16" t="n"/>
       <c r="I975" s="16" t="n">
-        <v>0.0934</v>
+        <v>0.096</v>
       </c>
       <c r="J975" s="19" t="n">
-        <v>18443</v>
+        <v>24544</v>
       </c>
       <c r="K975" s="19" t="n">
-        <v>27376</v>
+        <v>35743</v>
       </c>
       <c r="L975" s="31" t="n">
-        <v>0.582</v>
+        <v>0.6657</v>
       </c>
     </row>
     <row r="976">
@@ -51070,29 +51070,29 @@
         </is>
       </c>
       <c r="D976" s="9" t="n">
-        <v>1060485.01</v>
+        <v>1468784.97</v>
       </c>
       <c r="E976" s="9" t="n">
-        <v>3205507.44</v>
+        <v>3774012.68</v>
       </c>
       <c r="F976" s="10" t="n">
-        <v>0.4806</v>
+        <v>0.2078</v>
       </c>
       <c r="G976" s="10" t="n">
-        <v>0.4121</v>
+        <v>0.1408</v>
       </c>
       <c r="H976" s="10" t="n"/>
       <c r="I976" s="10" t="n">
-        <v>0.061</v>
+        <v>0.0626</v>
       </c>
       <c r="J976" s="13" t="n">
-        <v>34444</v>
+        <v>45458</v>
       </c>
       <c r="K976" s="13" t="n">
-        <v>49253</v>
+        <v>87381</v>
       </c>
       <c r="L976" s="32" t="n">
-        <v>0.6113</v>
+        <v>0.7159</v>
       </c>
     </row>
     <row r="977">
@@ -51112,29 +51112,29 @@
         </is>
       </c>
       <c r="D977" s="15" t="n">
-        <v>782153.03</v>
+        <v>1032552.96</v>
       </c>
       <c r="E977" s="15" t="n">
-        <v>5815622.59</v>
+        <v>6332301.28</v>
       </c>
       <c r="F977" s="16" t="n">
-        <v>0.5768</v>
+        <v>0.5393</v>
       </c>
       <c r="G977" s="16" t="n">
-        <v>0.5034999999999999</v>
+        <v>0.4684</v>
       </c>
       <c r="H977" s="16" t="n"/>
       <c r="I977" s="16" t="n">
-        <v>0.037</v>
+        <v>0.0398</v>
       </c>
       <c r="J977" s="19" t="n">
-        <v>35752</v>
+        <v>46742</v>
       </c>
       <c r="K977" s="19" t="n">
-        <v>68122</v>
+        <v>82692</v>
       </c>
       <c r="L977" s="31" t="n">
-        <v>0.5933</v>
+        <v>0.6822</v>
       </c>
     </row>
     <row r="978">
@@ -51616,29 +51616,29 @@
         </is>
       </c>
       <c r="D989" s="15" t="n">
-        <v>673220.78</v>
+        <v>2491457.06</v>
       </c>
       <c r="E989" s="15" t="n">
-        <v>3292035.57</v>
+        <v>4621964.29</v>
       </c>
       <c r="F989" s="16" t="n">
-        <v>0.7238</v>
+        <v>0.6272</v>
       </c>
       <c r="G989" s="16" t="n">
-        <v>0.6559</v>
+        <v>0.5706</v>
       </c>
       <c r="H989" s="16" t="n"/>
       <c r="I989" s="16" t="n">
-        <v>0.0216</v>
+        <v>0.0379</v>
       </c>
       <c r="J989" s="19" t="n">
-        <v>21405</v>
+        <v>55189</v>
       </c>
       <c r="K989" s="19" t="n">
-        <v>47250</v>
+        <v>98455</v>
       </c>
       <c r="L989" s="31" t="n">
-        <v>0.3168</v>
+        <v>0.7925</v>
       </c>
     </row>
     <row r="990">
@@ -54892,29 +54892,29 @@
         </is>
       </c>
       <c r="D1067" s="15" t="n">
-        <v>325712.16</v>
+        <v>569865.76</v>
       </c>
       <c r="E1067" s="15" t="n">
-        <v>2465880.71</v>
+        <v>3384023.25</v>
       </c>
       <c r="F1067" s="16" t="n">
-        <v>0.8907</v>
+        <v>0.8547</v>
       </c>
       <c r="G1067" s="16" t="n">
-        <v>0.8201000000000001</v>
+        <v>0.786</v>
       </c>
       <c r="H1067" s="16" t="n"/>
       <c r="I1067" s="16" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="J1067" s="19" t="n">
-        <v>14256</v>
+        <v>27710</v>
       </c>
       <c r="K1067" s="19" t="n">
-        <v>37855</v>
+        <v>58086</v>
       </c>
       <c r="L1067" s="31" t="n">
-        <v>0.2798</v>
+        <v>0.5374</v>
       </c>
     </row>
     <row r="1068">
@@ -54934,29 +54934,29 @@
         </is>
       </c>
       <c r="D1068" s="9" t="n">
-        <v>79380.2</v>
+        <v>351172.99</v>
       </c>
       <c r="E1068" s="9" t="n">
-        <v>83178.02</v>
+        <v>94658.64999999999</v>
       </c>
       <c r="F1068" s="10" t="n">
-        <v>0.4743</v>
+        <v>0.285</v>
       </c>
       <c r="G1068" s="10" t="n">
-        <v>0.4277</v>
+        <v>0.2466</v>
       </c>
       <c r="H1068" s="10" t="n"/>
       <c r="I1068" s="10" t="n">
-        <v>0.1753</v>
+        <v>0.2733</v>
       </c>
       <c r="J1068" s="13" t="n">
-        <v>365</v>
+        <v>1266</v>
       </c>
       <c r="K1068" s="13" t="n">
-        <v>619</v>
+        <v>2973</v>
       </c>
       <c r="L1068" s="32" t="n">
-        <v>0.3002</v>
+        <v>0.8405</v>
       </c>
     </row>
     <row r="1069">
@@ -54976,29 +54976,29 @@
         </is>
       </c>
       <c r="D1069" s="15" t="n">
-        <v>33287.18</v>
+        <v>360617.94</v>
       </c>
       <c r="E1069" s="15" t="n">
-        <v>26621.29</v>
+        <v>60233.64</v>
       </c>
       <c r="F1069" s="16" t="n">
-        <v>0.5760999999999999</v>
+        <v>0.4595</v>
       </c>
       <c r="G1069" s="16" t="n">
-        <v>0.5154</v>
+        <v>0.4134</v>
       </c>
       <c r="H1069" s="16" t="n"/>
       <c r="I1069" s="16" t="n">
-        <v>0.1259</v>
+        <v>0.1736</v>
       </c>
       <c r="J1069" s="19" t="n">
-        <v>556</v>
+        <v>2909</v>
       </c>
       <c r="K1069" s="19" t="n">
-        <v>667</v>
+        <v>4323</v>
       </c>
       <c r="L1069" s="31" t="n">
-        <v>0.4475</v>
+        <v>0.925</v>
       </c>
     </row>
     <row r="1070">
@@ -55018,29 +55018,29 @@
         </is>
       </c>
       <c r="D1070" s="9" t="n">
-        <v>41933.29</v>
+        <v>317428.44</v>
       </c>
       <c r="E1070" s="9" t="n">
-        <v>61880.68</v>
+        <v>139843.75</v>
       </c>
       <c r="F1070" s="10" t="n">
-        <v>0.4834</v>
+        <v>0.5173</v>
       </c>
       <c r="G1070" s="10" t="n">
-        <v>0.4125</v>
+        <v>0.4654</v>
       </c>
       <c r="H1070" s="10" t="n"/>
       <c r="I1070" s="10" t="n">
-        <v>0.0785</v>
+        <v>0.1078</v>
       </c>
       <c r="J1070" s="13" t="n">
-        <v>701</v>
+        <v>3617</v>
       </c>
       <c r="K1070" s="13" t="n">
-        <v>797</v>
+        <v>5350</v>
       </c>
       <c r="L1070" s="32" t="n">
-        <v>0.3203</v>
+        <v>0.9006</v>
       </c>
     </row>
     <row r="1071">
@@ -55060,29 +55060,29 @@
         </is>
       </c>
       <c r="D1071" s="15" t="n">
-        <v>36970.46</v>
+        <v>275724.31</v>
       </c>
       <c r="E1071" s="15" t="n">
-        <v>56451.75</v>
+        <v>89579.85000000001</v>
       </c>
       <c r="F1071" s="16" t="n">
-        <v>0.4983</v>
+        <v>0.668</v>
       </c>
       <c r="G1071" s="16" t="n">
-        <v>0.4356</v>
+        <v>0.6096</v>
       </c>
       <c r="H1071" s="16" t="n"/>
       <c r="I1071" s="16" t="n">
-        <v>0.06279999999999999</v>
+        <v>0.0586</v>
       </c>
       <c r="J1071" s="19" t="n">
-        <v>764</v>
+        <v>3600</v>
       </c>
       <c r="K1071" s="19" t="n">
-        <v>856</v>
+        <v>5062</v>
       </c>
       <c r="L1071" s="31" t="n">
-        <v>0.5264</v>
+        <v>0.9306</v>
       </c>
     </row>
     <row r="1072">
@@ -55102,29 +55102,29 @@
         </is>
       </c>
       <c r="D1072" s="9" t="n">
-        <v>64026.64</v>
+        <v>333327.35</v>
       </c>
       <c r="E1072" s="9" t="n">
-        <v>184939.2</v>
+        <v>321079.75</v>
       </c>
       <c r="F1072" s="10" t="n">
-        <v>0.3604</v>
+        <v>0.6971000000000001</v>
       </c>
       <c r="G1072" s="10" t="n">
-        <v>0.2839</v>
+        <v>0.6344</v>
       </c>
       <c r="H1072" s="10" t="n"/>
       <c r="I1072" s="10" t="n">
-        <v>0.0284</v>
+        <v>0.0337</v>
       </c>
       <c r="J1072" s="13" t="n">
-        <v>2039</v>
+        <v>8108</v>
       </c>
       <c r="K1072" s="13" t="n">
-        <v>2329</v>
+        <v>12301</v>
       </c>
       <c r="L1072" s="32" t="n">
-        <v>0.4733</v>
+        <v>0.8861</v>
       </c>
     </row>
     <row r="1073">
@@ -55144,29 +55144,29 @@
         </is>
       </c>
       <c r="D1073" s="15" t="n">
-        <v>91910.86</v>
+        <v>283320.26</v>
       </c>
       <c r="E1073" s="15" t="n">
-        <v>413083.94</v>
+        <v>532545.42</v>
       </c>
       <c r="F1073" s="16" t="n">
-        <v>0.8549</v>
+        <v>0.8087</v>
       </c>
       <c r="G1073" s="16" t="n">
-        <v>0.7806999999999999</v>
+        <v>0.7438</v>
       </c>
       <c r="H1073" s="16" t="n"/>
       <c r="I1073" s="16" t="n">
-        <v>0.0128</v>
+        <v>0.0175</v>
       </c>
       <c r="J1073" s="19" t="n">
-        <v>2724</v>
+        <v>7979</v>
       </c>
       <c r="K1073" s="19" t="n">
-        <v>4127</v>
+        <v>10360</v>
       </c>
       <c r="L1073" s="31" t="n">
-        <v>0.2199</v>
+        <v>0.7121</v>
       </c>
     </row>
     <row r="1074">
@@ -55606,26 +55606,26 @@
         </is>
       </c>
       <c r="D1084" s="9" t="n">
-        <v>2883699.5</v>
+        <v>3997751.11</v>
       </c>
       <c r="E1084" s="9" t="n">
-        <v>10016785.4</v>
+        <v>11354044.82</v>
       </c>
       <c r="F1084" s="10" t="n">
-        <v>0.1984</v>
+        <v>0.1424</v>
       </c>
       <c r="G1084" s="10" t="n">
-        <v>0.1444</v>
+        <v>0.0877</v>
       </c>
       <c r="H1084" s="10" t="n"/>
       <c r="I1084" s="10" t="n">
-        <v>0.0877</v>
+        <v>0.09719999999999999</v>
       </c>
       <c r="J1084" s="13" t="n">
-        <v>50033</v>
+        <v>71157</v>
       </c>
       <c r="K1084" s="13" t="n">
-        <v>140585</v>
+        <v>188250</v>
       </c>
       <c r="L1084" s="32" t="n">
         <v>0</v>
@@ -58588,26 +58588,26 @@
         </is>
       </c>
       <c r="D1155" s="15" t="n">
-        <v>139535.21</v>
+        <v>190980.97</v>
       </c>
       <c r="E1155" s="15" t="n">
-        <v>5299051.6</v>
+        <v>5421977.3</v>
       </c>
       <c r="F1155" s="16" t="n">
-        <v>0.9021</v>
+        <v>0.6982</v>
       </c>
       <c r="G1155" s="16" t="n">
-        <v>0.8292</v>
+        <v>0.6304999999999999</v>
       </c>
       <c r="H1155" s="16" t="n"/>
       <c r="I1155" s="16" t="n">
-        <v>0.0069</v>
+        <v>0.0198</v>
       </c>
       <c r="J1155" s="19" t="n">
-        <v>5920</v>
+        <v>8892</v>
       </c>
       <c r="K1155" s="19" t="n">
-        <v>47350</v>
+        <v>54348</v>
       </c>
       <c r="L1155" s="31" t="n">
         <v>0</v>
@@ -58630,26 +58630,26 @@
         </is>
       </c>
       <c r="D1156" s="9" t="n">
-        <v>1322311.28</v>
+        <v>1770217.32</v>
       </c>
       <c r="E1156" s="9" t="n">
-        <v>889236.9</v>
+        <v>1506051.88</v>
       </c>
       <c r="F1156" s="10" t="n">
-        <v>0.093</v>
+        <v>0.032</v>
       </c>
       <c r="G1156" s="10" t="n">
-        <v>0.0474</v>
+        <v>-0.0157</v>
       </c>
       <c r="H1156" s="10" t="n"/>
       <c r="I1156" s="10" t="n">
-        <v>0.2042</v>
+        <v>0.2183</v>
       </c>
       <c r="J1156" s="13" t="n">
-        <v>8588</v>
+        <v>12513</v>
       </c>
       <c r="K1156" s="13" t="n">
-        <v>25602</v>
+        <v>37519</v>
       </c>
       <c r="L1156" s="32" t="n">
         <v>0</v>
@@ -58672,26 +58672,26 @@
         </is>
       </c>
       <c r="D1157" s="15" t="n">
-        <v>718161.52</v>
+        <v>1031643.58</v>
       </c>
       <c r="E1157" s="15" t="n">
-        <v>548438.3100000001</v>
+        <v>669329.89</v>
       </c>
       <c r="F1157" s="16" t="n">
-        <v>0.2034</v>
+        <v>0.0785</v>
       </c>
       <c r="G1157" s="16" t="n">
-        <v>0.1477</v>
+        <v>0.0236</v>
       </c>
       <c r="H1157" s="16" t="n"/>
       <c r="I1157" s="16" t="n">
-        <v>0.1233</v>
+        <v>0.1343</v>
       </c>
       <c r="J1157" s="19" t="n">
-        <v>9675</v>
+        <v>13596</v>
       </c>
       <c r="K1157" s="19" t="n">
-        <v>22508</v>
+        <v>31727</v>
       </c>
       <c r="L1157" s="31" t="n">
         <v>0</v>
@@ -58714,26 +58714,26 @@
         </is>
       </c>
       <c r="D1158" s="9" t="n">
-        <v>328304.62</v>
+        <v>446726.93</v>
       </c>
       <c r="E1158" s="9" t="n">
-        <v>446997.54</v>
+        <v>579901.15</v>
       </c>
       <c r="F1158" s="10" t="n">
-        <v>0.1137</v>
+        <v>0.1383</v>
       </c>
       <c r="G1158" s="10" t="n">
-        <v>0.0503</v>
+        <v>0.0747</v>
       </c>
       <c r="H1158" s="10" t="n"/>
       <c r="I1158" s="10" t="n">
-        <v>0.08450000000000001</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="J1158" s="13" t="n">
-        <v>7631</v>
+        <v>10492</v>
       </c>
       <c r="K1158" s="13" t="n">
-        <v>14677</v>
+        <v>19893</v>
       </c>
       <c r="L1158" s="32" t="n">
         <v>0</v>
@@ -58756,26 +58756,26 @@
         </is>
       </c>
       <c r="D1159" s="15" t="n">
-        <v>124098.34</v>
+        <v>187294.5</v>
       </c>
       <c r="E1159" s="15" t="n">
-        <v>407706.83</v>
+        <v>440225.24</v>
       </c>
       <c r="F1159" s="16" t="n">
-        <v>0.3824</v>
+        <v>0.3948</v>
       </c>
       <c r="G1159" s="16" t="n">
-        <v>0.3164</v>
+        <v>0.3304</v>
       </c>
       <c r="H1159" s="16" t="n"/>
       <c r="I1159" s="16" t="n">
-        <v>0.066</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="J1159" s="19" t="n">
-        <v>4564</v>
+        <v>6425</v>
       </c>
       <c r="K1159" s="19" t="n">
-        <v>6345</v>
+        <v>9509</v>
       </c>
       <c r="L1159" s="31" t="n">
         <v>0</v>
@@ -58798,26 +58798,26 @@
         </is>
       </c>
       <c r="D1160" s="9" t="n">
-        <v>141095.34</v>
+        <v>202588.16</v>
       </c>
       <c r="E1160" s="9" t="n">
-        <v>512589.3</v>
+        <v>597138.1899999999</v>
       </c>
       <c r="F1160" s="10" t="n">
-        <v>0.2803</v>
+        <v>0.3567</v>
       </c>
       <c r="G1160" s="10" t="n">
-        <v>0.2161</v>
+        <v>0.2929</v>
       </c>
       <c r="H1160" s="10" t="n"/>
       <c r="I1160" s="10" t="n">
-        <v>0.0461</v>
+        <v>0.05</v>
       </c>
       <c r="J1160" s="13" t="n">
-        <v>7203</v>
+        <v>10165</v>
       </c>
       <c r="K1160" s="13" t="n">
-        <v>10453</v>
+        <v>14872</v>
       </c>
       <c r="L1160" s="32" t="n">
         <v>0</v>
@@ -58840,26 +58840,26 @@
         </is>
       </c>
       <c r="D1161" s="15" t="n">
-        <v>110193.2</v>
+        <v>168299.65</v>
       </c>
       <c r="E1161" s="15" t="n">
-        <v>1912764.93</v>
+        <v>2139421.18</v>
       </c>
       <c r="F1161" s="16" t="n">
-        <v>0.4787</v>
+        <v>0.5357</v>
       </c>
       <c r="G1161" s="16" t="n">
-        <v>0.414</v>
+        <v>0.4706</v>
       </c>
       <c r="H1161" s="16" t="n"/>
       <c r="I1161" s="16" t="n">
-        <v>0.0192</v>
+        <v>0.0241</v>
       </c>
       <c r="J1161" s="19" t="n">
-        <v>6452</v>
+        <v>9074</v>
       </c>
       <c r="K1161" s="19" t="n">
-        <v>13650</v>
+        <v>20382</v>
       </c>
       <c r="L1161" s="31" t="n">
         <v>0</v>
@@ -59386,10 +59386,10 @@
         </is>
       </c>
       <c r="D1174" s="9" t="n">
-        <v>176753035.71</v>
+        <v>176753150.06</v>
       </c>
       <c r="E1174" s="9" t="n">
-        <v>774561992.42</v>
+        <v>774562265.72</v>
       </c>
       <c r="F1174" s="10" t="n">
         <v>0.1419</v>
@@ -59402,10 +59402,10 @@
         <v>0.0985</v>
       </c>
       <c r="J1174" s="13" t="n">
-        <v>4207739</v>
+        <v>4207750</v>
       </c>
       <c r="K1174" s="13" t="n">
-        <v>8186439</v>
+        <v>8186452</v>
       </c>
       <c r="L1174" s="32" t="n">
         <v>0</v>
@@ -59428,26 +59428,26 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>57997127.37</v>
+        <v>79307281.97</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>223721677.52</v>
+        <v>309733183.15</v>
       </c>
       <c r="F1175" s="16" t="n">
-        <v>0.1245</v>
+        <v>0.1419</v>
       </c>
       <c r="G1175" s="16" t="n">
-        <v>0.0693</v>
+        <v>0.08690000000000001</v>
       </c>
       <c r="H1175" s="16" t="n"/>
       <c r="I1175" s="16" t="n">
-        <v>0.1016</v>
+        <v>0.1064</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>1374952</v>
+        <v>1820002</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>2556692</v>
+        <v>3390647</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -62998,7 +62998,7 @@
         </is>
       </c>
       <c r="D1260" s="9" t="n">
-        <v>21457462.74</v>
+        <v>21457467.5</v>
       </c>
       <c r="E1260" s="9" t="n">
         <v>390593856.51</v>
@@ -63014,10 +63014,10 @@
         <v>0.0284</v>
       </c>
       <c r="J1260" s="13" t="n">
-        <v>1576126</v>
+        <v>1576127</v>
       </c>
       <c r="K1260" s="13" t="n">
-        <v>2468161</v>
+        <v>2468162</v>
       </c>
       <c r="L1260" s="32" t="n">
         <v>0</v>
@@ -63040,7 +63040,7 @@
         </is>
       </c>
       <c r="D1261" s="15" t="n">
-        <v>47038186.7</v>
+        <v>47038229.58</v>
       </c>
       <c r="E1261" s="15" t="n">
         <v>24462981.01</v>
@@ -63056,10 +63056,10 @@
         <v>0.3106</v>
       </c>
       <c r="J1261" s="19" t="n">
-        <v>198929</v>
+        <v>198932</v>
       </c>
       <c r="K1261" s="19" t="n">
-        <v>896768</v>
+        <v>896771</v>
       </c>
       <c r="L1261" s="31" t="n">
         <v>0</v>
@@ -63082,10 +63082,10 @@
         </is>
       </c>
       <c r="D1262" s="9" t="n">
-        <v>30002596.96</v>
+        <v>30002644.23</v>
       </c>
       <c r="E1262" s="9" t="n">
-        <v>31177345.55</v>
+        <v>31177418.43</v>
       </c>
       <c r="F1262" s="10" t="n">
         <v>0.0438</v>
@@ -63098,10 +63098,10 @@
         <v>0.2377</v>
       </c>
       <c r="J1262" s="13" t="n">
-        <v>295709</v>
+        <v>295710</v>
       </c>
       <c r="K1262" s="13" t="n">
-        <v>783783</v>
+        <v>783785</v>
       </c>
       <c r="L1262" s="32" t="n">
         <v>0</v>
@@ -63124,10 +63124,10 @@
         </is>
       </c>
       <c r="D1263" s="15" t="n">
-        <v>22499210.51</v>
+        <v>22499229.94</v>
       </c>
       <c r="E1263" s="15" t="n">
-        <v>37108422.3</v>
+        <v>37108520.54</v>
       </c>
       <c r="F1263" s="16" t="n">
         <v>0.06759999999999999</v>
@@ -63140,10 +63140,10 @@
         <v>0.1892</v>
       </c>
       <c r="J1263" s="19" t="n">
-        <v>344121</v>
+        <v>344124</v>
       </c>
       <c r="K1263" s="19" t="n">
-        <v>750766</v>
+        <v>750770</v>
       </c>
       <c r="L1263" s="31" t="n">
         <v>0</v>
@@ -63169,7 +63169,7 @@
         <v>15087039.61</v>
       </c>
       <c r="E1264" s="9" t="n">
-        <v>40911911.69</v>
+        <v>40911923.08</v>
       </c>
       <c r="F1264" s="10" t="n">
         <v>0.0829</v>
@@ -63182,10 +63182,10 @@
         <v>0.1502</v>
       </c>
       <c r="J1264" s="13" t="n">
-        <v>333268</v>
+        <v>333269</v>
       </c>
       <c r="K1264" s="13" t="n">
-        <v>637275</v>
+        <v>637276</v>
       </c>
       <c r="L1264" s="32" t="n">
         <v>0</v>
@@ -63253,7 +63253,7 @@
         <v>19509272.35</v>
       </c>
       <c r="E1266" s="9" t="n">
-        <v>156492487.2</v>
+        <v>156492577.99</v>
       </c>
       <c r="F1266" s="10" t="n">
         <v>0.3211</v>
@@ -63266,10 +63266,10 @@
         <v>0.0638</v>
       </c>
       <c r="J1266" s="13" t="n">
-        <v>814249</v>
+        <v>814251</v>
       </c>
       <c r="K1266" s="13" t="n">
-        <v>1513621</v>
+        <v>1513623</v>
       </c>
       <c r="L1266" s="32" t="n">
         <v>0</v>
@@ -63292,26 +63292,26 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>7612662.76</v>
+        <v>9676047.439999999</v>
       </c>
       <c r="E1267" s="15" t="n">
-        <v>126706759.4</v>
+        <v>174625916.12</v>
       </c>
       <c r="F1267" s="16" t="n">
-        <v>0.4423</v>
+        <v>0.4011</v>
       </c>
       <c r="G1267" s="16" t="n">
-        <v>0.3689</v>
+        <v>0.3266</v>
       </c>
       <c r="H1267" s="16" t="n"/>
       <c r="I1267" s="16" t="n">
-        <v>0.0281</v>
+        <v>0.0302</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>577783</v>
+        <v>727676</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>924196</v>
+        <v>1167300</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63334,26 +63334,26 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>16263666.15</v>
+        <v>22559469.15</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>7822396.76</v>
+        <v>11100977.89</v>
       </c>
       <c r="F1268" s="10" t="n">
-        <v>0.0237</v>
+        <v>0.0667</v>
       </c>
       <c r="G1268" s="10" t="n">
-        <v>-0.0152</v>
+        <v>0.0273</v>
       </c>
       <c r="H1268" s="10" t="n"/>
       <c r="I1268" s="10" t="n">
-        <v>0.3128</v>
+        <v>0.313</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>64309</v>
+        <v>91922</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>255834</v>
+        <v>366829</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63376,26 +63376,26 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>10250417.67</v>
+        <v>14657755.99</v>
       </c>
       <c r="E1269" s="15" t="n">
-        <v>8814110.49</v>
+        <v>12788990.96</v>
       </c>
       <c r="F1269" s="16" t="n">
-        <v>0.0443</v>
+        <v>0.0927</v>
       </c>
       <c r="G1269" s="16" t="n">
-        <v>-0.0048</v>
+        <v>0.0441</v>
       </c>
       <c r="H1269" s="16" t="n"/>
       <c r="I1269" s="16" t="n">
-        <v>0.2515</v>
+        <v>0.2491</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>92346</v>
+        <v>131316</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>234781</v>
+        <v>326878</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63418,26 +63418,26 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>7391430.73</v>
+        <v>10094693.99</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>10589434.91</v>
+        <v>14843318.68</v>
       </c>
       <c r="F1270" s="10" t="n">
-        <v>0.0341</v>
+        <v>0.0702</v>
       </c>
       <c r="G1270" s="10" t="n">
-        <v>-0.0222</v>
+        <v>0.0139</v>
       </c>
       <c r="H1270" s="10" t="n"/>
       <c r="I1270" s="10" t="n">
-        <v>0.2067</v>
+        <v>0.2039</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>102644</v>
+        <v>144778</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>215334</v>
+        <v>296114</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63460,26 +63460,26 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>4619485.08</v>
+        <v>6475423.93</v>
       </c>
       <c r="E1271" s="15" t="n">
-        <v>10997091.41</v>
+        <v>15078900.22</v>
       </c>
       <c r="F1271" s="16" t="n">
-        <v>0.1054</v>
+        <v>0.1396</v>
       </c>
       <c r="G1271" s="16" t="n">
-        <v>0.0434</v>
+        <v>0.07829999999999999</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
-        <v>0.1673</v>
+        <v>0.1676</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>100151</v>
+        <v>138722</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>190014</v>
+        <v>253594</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63502,26 +63502,26 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>6113109.08</v>
+        <v>8248799.35</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>20803826.57</v>
+        <v>29062267.28</v>
       </c>
       <c r="F1272" s="10" t="n">
-        <v>0.1449</v>
+        <v>0.1424</v>
       </c>
       <c r="G1272" s="10" t="n">
-        <v>0.0779</v>
+        <v>0.0757</v>
       </c>
       <c r="H1272" s="10" t="n"/>
       <c r="I1272" s="10" t="n">
-        <v>0.1246</v>
+        <v>0.125</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>193023</v>
+        <v>262440</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>311311</v>
+        <v>417580</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63544,26 +63544,26 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>5746355.89</v>
+        <v>7595092.11</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>37988057.97</v>
+        <v>52232812.01</v>
       </c>
       <c r="F1273" s="16" t="n">
-        <v>0.2412</v>
+        <v>0.2262</v>
       </c>
       <c r="G1273" s="16" t="n">
-        <v>0.1733</v>
+        <v>0.1578</v>
       </c>
       <c r="H1273" s="16" t="n"/>
       <c r="I1273" s="16" t="n">
-        <v>0.0736</v>
+        <v>0.0761</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>244696</v>
+        <v>323148</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>425222</v>
+        <v>562352</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -64090,26 +64090,26 @@
         </is>
       </c>
       <c r="D1286" s="9" t="n">
-        <v>3710208.95</v>
+        <v>5406822.66</v>
       </c>
       <c r="E1286" s="9" t="n">
-        <v>9237620.09</v>
+        <v>18309456.55</v>
       </c>
       <c r="F1286" s="10" t="n">
-        <v>-0.06320000000000001</v>
+        <v>-0.0098</v>
       </c>
       <c r="G1286" s="10" t="n">
-        <v>-0.1225</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="H1286" s="10" t="n"/>
       <c r="I1286" s="10" t="n">
-        <v>0.116</v>
+        <v>0.1275</v>
       </c>
       <c r="J1286" s="13" t="n">
-        <v>71342</v>
+        <v>102092</v>
       </c>
       <c r="K1286" s="13" t="n">
-        <v>107873</v>
+        <v>155466</v>
       </c>
       <c r="L1286" s="32" t="n">
         <v>0</v>
@@ -67660,26 +67660,26 @@
         </is>
       </c>
       <c r="D1371" s="15" t="n">
-        <v>270801.02</v>
+        <v>399402.74</v>
       </c>
       <c r="E1371" s="15" t="n">
-        <v>3589976.92</v>
+        <v>8339238.73</v>
       </c>
       <c r="F1371" s="16" t="n">
-        <v>0.1302</v>
+        <v>0.1007</v>
       </c>
       <c r="G1371" s="16" t="n">
-        <v>0.0571</v>
+        <v>0.0185</v>
       </c>
       <c r="H1371" s="16" t="n"/>
       <c r="I1371" s="16" t="n">
-        <v>0.0286</v>
+        <v>0.0318</v>
       </c>
       <c r="J1371" s="19" t="n">
-        <v>20011</v>
+        <v>29145</v>
       </c>
       <c r="K1371" s="19" t="n">
-        <v>27084</v>
+        <v>39815</v>
       </c>
       <c r="L1371" s="31" t="n">
         <v>0</v>
@@ -67702,26 +67702,26 @@
         </is>
       </c>
       <c r="D1372" s="9" t="n">
-        <v>904072.1</v>
+        <v>1377748.11</v>
       </c>
       <c r="E1372" s="9" t="n">
-        <v>361397.1</v>
+        <v>684607.09</v>
       </c>
       <c r="F1372" s="10" t="n">
-        <v>0.0122</v>
+        <v>0.0095</v>
       </c>
       <c r="G1372" s="10" t="n">
-        <v>-0.0359</v>
+        <v>-0.0364</v>
       </c>
       <c r="H1372" s="10" t="n"/>
       <c r="I1372" s="10" t="n">
-        <v>0.3279</v>
+        <v>0.3351</v>
       </c>
       <c r="J1372" s="13" t="n">
-        <v>3605</v>
+        <v>5220</v>
       </c>
       <c r="K1372" s="13" t="n">
-        <v>8805</v>
+        <v>12503</v>
       </c>
       <c r="L1372" s="32" t="n">
         <v>0</v>
@@ -67744,26 +67744,26 @@
         </is>
       </c>
       <c r="D1373" s="15" t="n">
-        <v>889168.15</v>
+        <v>1274693.73</v>
       </c>
       <c r="E1373" s="15" t="n">
-        <v>505953.04</v>
+        <v>870355.16</v>
       </c>
       <c r="F1373" s="16" t="n">
-        <v>-0.1606</v>
+        <v>-0.0867</v>
       </c>
       <c r="G1373" s="16" t="n">
-        <v>-0.215</v>
+        <v>-0.1372</v>
       </c>
       <c r="H1373" s="16" t="n"/>
       <c r="I1373" s="16" t="n">
-        <v>0.2622</v>
+        <v>0.2708</v>
       </c>
       <c r="J1373" s="19" t="n">
-        <v>6919</v>
+        <v>9645</v>
       </c>
       <c r="K1373" s="19" t="n">
-        <v>12529</v>
+        <v>17886</v>
       </c>
       <c r="L1373" s="31" t="n">
         <v>0</v>
@@ -67786,26 +67786,26 @@
         </is>
       </c>
       <c r="D1374" s="9" t="n">
-        <v>551521.1899999999</v>
+        <v>771511.77</v>
       </c>
       <c r="E1374" s="9" t="n">
-        <v>745263.37</v>
+        <v>1197416.16</v>
       </c>
       <c r="F1374" s="10" t="n">
-        <v>-0.0551</v>
+        <v>0.0393</v>
       </c>
       <c r="G1374" s="10" t="n">
-        <v>-0.1175</v>
+        <v>-0.0229</v>
       </c>
       <c r="H1374" s="10" t="n"/>
       <c r="I1374" s="10" t="n">
-        <v>0.1821</v>
+        <v>0.1977</v>
       </c>
       <c r="J1374" s="13" t="n">
-        <v>8090</v>
+        <v>11260</v>
       </c>
       <c r="K1374" s="13" t="n">
-        <v>11876</v>
+        <v>16867</v>
       </c>
       <c r="L1374" s="32" t="n">
         <v>0</v>
@@ -67828,26 +67828,26 @@
         </is>
       </c>
       <c r="D1375" s="15" t="n">
-        <v>406579.19</v>
+        <v>553119.9</v>
       </c>
       <c r="E1375" s="15" t="n">
-        <v>758895.9399999999</v>
+        <v>1318711.43</v>
       </c>
       <c r="F1375" s="16" t="n">
-        <v>-0.0999</v>
+        <v>0.0083</v>
       </c>
       <c r="G1375" s="16" t="n">
-        <v>-0.1615</v>
+        <v>-0.056</v>
       </c>
       <c r="H1375" s="16" t="n"/>
       <c r="I1375" s="16" t="n">
-        <v>0.1464</v>
+        <v>0.1662</v>
       </c>
       <c r="J1375" s="19" t="n">
-        <v>7330</v>
+        <v>10351</v>
       </c>
       <c r="K1375" s="19" t="n">
-        <v>11748</v>
+        <v>16392</v>
       </c>
       <c r="L1375" s="31" t="n">
         <v>0</v>
@@ -67870,26 +67870,26 @@
         </is>
       </c>
       <c r="D1376" s="9" t="n">
-        <v>442202.7</v>
+        <v>674063.51</v>
       </c>
       <c r="E1376" s="9" t="n">
-        <v>1833111.58</v>
+        <v>3006281.64</v>
       </c>
       <c r="F1376" s="10" t="n">
-        <v>-0.0053</v>
+        <v>-0.0098</v>
       </c>
       <c r="G1376" s="10" t="n">
-        <v>-0.07539999999999999</v>
+        <v>-0.08019999999999999</v>
       </c>
       <c r="H1376" s="10" t="n"/>
       <c r="I1376" s="10" t="n">
-        <v>0.1009</v>
+        <v>0.1193</v>
       </c>
       <c r="J1376" s="13" t="n">
-        <v>14024</v>
+        <v>19766</v>
       </c>
       <c r="K1376" s="13" t="n">
-        <v>21372</v>
+        <v>29767</v>
       </c>
       <c r="L1376" s="32" t="n">
         <v>0</v>
@@ -67912,26 +67912,26 @@
         </is>
       </c>
       <c r="D1377" s="15" t="n">
-        <v>245864.62</v>
+        <v>356282.91</v>
       </c>
       <c r="E1377" s="15" t="n">
-        <v>1443022.15</v>
+        <v>2892846.34</v>
       </c>
       <c r="F1377" s="16" t="n">
-        <v>-0.2627</v>
+        <v>-0.067</v>
       </c>
       <c r="G1377" s="16" t="n">
-        <v>-0.336</v>
+        <v>-0.1472</v>
       </c>
       <c r="H1377" s="16" t="n"/>
       <c r="I1377" s="16" t="n">
-        <v>0.06569999999999999</v>
+        <v>0.0851</v>
       </c>
       <c r="J1377" s="19" t="n">
-        <v>11363</v>
+        <v>16705</v>
       </c>
       <c r="K1377" s="19" t="n">
-        <v>14459</v>
+        <v>22236</v>
       </c>
       <c r="L1377" s="31" t="n">
         <v>0</v>
@@ -68751,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-30 13:35 UTC</t>
+          <t>2026-10-30 14:56 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-30 16:05 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8647,7 +8647,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-30 14:56 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-30 16:05 UTC.</t>
         </is>
       </c>
     </row>
@@ -39268,13 +39268,13 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>5066549.86</v>
+        <v>5066660.07</v>
       </c>
       <c r="E695" s="15" t="n">
         <v>33654585.55</v>
       </c>
       <c r="F695" s="16" t="n">
-        <v>0.2433</v>
+        <v>0.2432</v>
       </c>
       <c r="G695" s="16" t="n">
         <v>0.1758</v>
@@ -39284,13 +39284,13 @@
         <v>0.0506</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>219820</v>
+        <v>219830</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>303664</v>
+        <v>303674</v>
       </c>
       <c r="L695" s="31" t="n">
-        <v>0.6791</v>
+        <v>0.6792</v>
       </c>
     </row>
     <row r="696">
@@ -43132,7 +43132,7 @@
         </is>
       </c>
       <c r="D787" s="15" t="n">
-        <v>1429125.21</v>
+        <v>1429187.6</v>
       </c>
       <c r="E787" s="15" t="n">
         <v>23552639.9</v>
@@ -43148,13 +43148,13 @@
         <v>0.0166</v>
       </c>
       <c r="J787" s="19" t="n">
-        <v>128165</v>
+        <v>128168</v>
       </c>
       <c r="K787" s="19" t="n">
-        <v>174111</v>
+        <v>174114</v>
       </c>
       <c r="L787" s="31" t="n">
-        <v>0.5848</v>
+        <v>0.5849</v>
       </c>
     </row>
     <row r="788">
@@ -43216,26 +43216,26 @@
         </is>
       </c>
       <c r="D789" s="15" t="n">
-        <v>617007.66</v>
+        <v>617041.6899999999</v>
       </c>
       <c r="E789" s="15" t="n">
         <v>447141.6</v>
       </c>
       <c r="F789" s="16" t="n">
-        <v>0.0477</v>
+        <v>0.0478</v>
       </c>
       <c r="G789" s="16" t="n">
-        <v>-0.0047</v>
+        <v>-0.0046</v>
       </c>
       <c r="H789" s="16" t="n"/>
       <c r="I789" s="16" t="n">
-        <v>0.2261</v>
+        <v>0.226</v>
       </c>
       <c r="J789" s="19" t="n">
-        <v>6776</v>
+        <v>6780</v>
       </c>
       <c r="K789" s="19" t="n">
-        <v>11223</v>
+        <v>11227</v>
       </c>
       <c r="L789" s="31" t="n">
         <v>0.7779</v>
@@ -43258,7 +43258,7 @@
         </is>
       </c>
       <c r="D790" s="9" t="n">
-        <v>578968.53</v>
+        <v>578971.98</v>
       </c>
       <c r="E790" s="9" t="n">
         <v>798054.73</v>
@@ -43274,10 +43274,10 @@
         <v>0.1616</v>
       </c>
       <c r="J790" s="13" t="n">
-        <v>9513</v>
+        <v>9514</v>
       </c>
       <c r="K790" s="13" t="n">
-        <v>13551</v>
+        <v>13552</v>
       </c>
       <c r="L790" s="32" t="n">
         <v>0.7548</v>
@@ -43342,7 +43342,7 @@
         </is>
       </c>
       <c r="D792" s="9" t="n">
-        <v>678280.29</v>
+        <v>678281.22</v>
       </c>
       <c r="E792" s="9" t="n">
         <v>2332051.08</v>
@@ -43358,10 +43358,10 @@
         <v>0.074</v>
       </c>
       <c r="J792" s="13" t="n">
-        <v>25608</v>
+        <v>25609</v>
       </c>
       <c r="K792" s="13" t="n">
-        <v>31864</v>
+        <v>31865</v>
       </c>
       <c r="L792" s="32" t="n">
         <v>0.6948</v>
@@ -43384,26 +43384,26 @@
         </is>
       </c>
       <c r="D793" s="15" t="n">
-        <v>657214.91</v>
+        <v>657224.3100000001</v>
       </c>
       <c r="E793" s="15" t="n">
         <v>4787775.8</v>
       </c>
       <c r="F793" s="16" t="n">
-        <v>0.2715</v>
+        <v>0.2713</v>
       </c>
       <c r="G793" s="16" t="n">
-        <v>0.1938</v>
+        <v>0.1937</v>
       </c>
       <c r="H793" s="16" t="n"/>
       <c r="I793" s="16" t="n">
-        <v>0.0479</v>
+        <v>0.048</v>
       </c>
       <c r="J793" s="19" t="n">
-        <v>35429</v>
+        <v>35430</v>
       </c>
       <c r="K793" s="19" t="n">
-        <v>46047</v>
+        <v>46048</v>
       </c>
       <c r="L793" s="31" t="n">
         <v>0.6681</v>
@@ -59428,13 +59428,13 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>79307281.97</v>
+        <v>79309028.84</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>309733183.15</v>
+        <v>309735891.85</v>
       </c>
       <c r="F1175" s="16" t="n">
-        <v>0.1419</v>
+        <v>0.1418</v>
       </c>
       <c r="G1175" s="16" t="n">
         <v>0.08690000000000001</v>
@@ -59444,10 +59444,10 @@
         <v>0.1064</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>1820002</v>
+        <v>1820082</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>3390647</v>
+        <v>3390748</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -63292,10 +63292,10 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>9676047.439999999</v>
+        <v>9676086.789999999</v>
       </c>
       <c r="E1267" s="15" t="n">
-        <v>174625916.12</v>
+        <v>174628159.3</v>
       </c>
       <c r="F1267" s="16" t="n">
         <v>0.4011</v>
@@ -63308,10 +63308,10 @@
         <v>0.0302</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>727676</v>
+        <v>727684</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>1167300</v>
+        <v>1167309</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63334,10 +63334,10 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>22559469.15</v>
+        <v>22560125.91</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>11100977.89</v>
+        <v>11101281.38</v>
       </c>
       <c r="F1268" s="10" t="n">
         <v>0.0667</v>
@@ -63347,13 +63347,13 @@
       </c>
       <c r="H1268" s="10" t="n"/>
       <c r="I1268" s="10" t="n">
-        <v>0.313</v>
+        <v>0.3131</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>91922</v>
+        <v>91944</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>366829</v>
+        <v>366863</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63376,10 +63376,10 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>14657755.99</v>
+        <v>14657942.52</v>
       </c>
       <c r="E1269" s="15" t="n">
-        <v>12788990.96</v>
+        <v>12789129.68</v>
       </c>
       <c r="F1269" s="16" t="n">
         <v>0.0927</v>
@@ -63392,10 +63392,10 @@
         <v>0.2491</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>131316</v>
+        <v>131330</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>326878</v>
+        <v>326898</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63418,26 +63418,26 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>10094693.99</v>
+        <v>10095172.32</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>14843318.68</v>
+        <v>14843337.67</v>
       </c>
       <c r="F1270" s="10" t="n">
-        <v>0.0702</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G1270" s="10" t="n">
-        <v>0.0139</v>
+        <v>0.0137</v>
       </c>
       <c r="H1270" s="10" t="n"/>
       <c r="I1270" s="10" t="n">
         <v>0.2039</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>144778</v>
+        <v>144788</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>296114</v>
+        <v>296125</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63460,7 +63460,7 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>6475423.93</v>
+        <v>6475565.4</v>
       </c>
       <c r="E1271" s="15" t="n">
         <v>15078900.22</v>
@@ -63469,17 +63469,17 @@
         <v>0.1396</v>
       </c>
       <c r="G1271" s="16" t="n">
-        <v>0.07829999999999999</v>
+        <v>0.07820000000000001</v>
       </c>
       <c r="H1271" s="16" t="n"/>
       <c r="I1271" s="16" t="n">
         <v>0.1676</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>138722</v>
+        <v>138728</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>253594</v>
+        <v>253600</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63502,10 +63502,10 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>8248799.35</v>
+        <v>8248997.09</v>
       </c>
       <c r="E1272" s="9" t="n">
-        <v>29062267.28</v>
+        <v>29062271.59</v>
       </c>
       <c r="F1272" s="10" t="n">
         <v>0.1424</v>
@@ -63518,10 +63518,10 @@
         <v>0.125</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>262440</v>
+        <v>262455</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>417580</v>
+        <v>417596</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63544,7 +63544,7 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>7595092.11</v>
+        <v>7595138.8</v>
       </c>
       <c r="E1273" s="15" t="n">
         <v>52232812.01</v>
@@ -63560,10 +63560,10 @@
         <v>0.0761</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>323148</v>
+        <v>323153</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>562352</v>
+        <v>562357</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -68751,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-30 14:56 UTC</t>
+          <t>2026-10-30 16:05 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-30 17:04 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8647,7 +8647,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-30 16:05 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-30 17:04 UTC.</t>
         </is>
       </c>
     </row>
@@ -39268,26 +39268,26 @@
         </is>
       </c>
       <c r="D695" s="15" t="n">
-        <v>5066660.07</v>
+        <v>5066921.94</v>
       </c>
       <c r="E695" s="15" t="n">
         <v>33654585.55</v>
       </c>
       <c r="F695" s="16" t="n">
-        <v>0.2432</v>
+        <v>0.243</v>
       </c>
       <c r="G695" s="16" t="n">
-        <v>0.1758</v>
+        <v>0.1756</v>
       </c>
       <c r="H695" s="16" t="n"/>
       <c r="I695" s="16" t="n">
         <v>0.0506</v>
       </c>
       <c r="J695" s="19" t="n">
-        <v>219830</v>
+        <v>219841</v>
       </c>
       <c r="K695" s="19" t="n">
-        <v>303674</v>
+        <v>303685</v>
       </c>
       <c r="L695" s="31" t="n">
         <v>0.6792</v>
@@ -43132,26 +43132,26 @@
         </is>
       </c>
       <c r="D787" s="15" t="n">
-        <v>1429187.6</v>
+        <v>1429290.44</v>
       </c>
       <c r="E787" s="15" t="n">
         <v>23552639.9</v>
       </c>
       <c r="F787" s="16" t="n">
-        <v>0.6092</v>
+        <v>0.6084000000000001</v>
       </c>
       <c r="G787" s="16" t="n">
-        <v>0.5314</v>
+        <v>0.5306</v>
       </c>
       <c r="H787" s="16" t="n"/>
       <c r="I787" s="16" t="n">
         <v>0.0166</v>
       </c>
       <c r="J787" s="19" t="n">
-        <v>128168</v>
+        <v>128170</v>
       </c>
       <c r="K787" s="19" t="n">
-        <v>174114</v>
+        <v>174116</v>
       </c>
       <c r="L787" s="31" t="n">
         <v>0.5849</v>
@@ -43216,7 +43216,7 @@
         </is>
       </c>
       <c r="D789" s="15" t="n">
-        <v>617041.6899999999</v>
+        <v>617062.91</v>
       </c>
       <c r="E789" s="15" t="n">
         <v>447141.6</v>
@@ -43232,10 +43232,10 @@
         <v>0.226</v>
       </c>
       <c r="J789" s="19" t="n">
-        <v>6780</v>
+        <v>6783</v>
       </c>
       <c r="K789" s="19" t="n">
-        <v>11227</v>
+        <v>11230</v>
       </c>
       <c r="L789" s="31" t="n">
         <v>0.7779</v>
@@ -43258,7 +43258,7 @@
         </is>
       </c>
       <c r="D790" s="9" t="n">
-        <v>578971.98</v>
+        <v>578986.04</v>
       </c>
       <c r="E790" s="9" t="n">
         <v>798054.73</v>
@@ -43271,13 +43271,13 @@
       </c>
       <c r="H790" s="10" t="n"/>
       <c r="I790" s="10" t="n">
-        <v>0.1616</v>
+        <v>0.1615</v>
       </c>
       <c r="J790" s="13" t="n">
-        <v>9514</v>
+        <v>9516</v>
       </c>
       <c r="K790" s="13" t="n">
-        <v>13552</v>
+        <v>13554</v>
       </c>
       <c r="L790" s="32" t="n">
         <v>0.7548</v>
@@ -43300,26 +43300,26 @@
         </is>
       </c>
       <c r="D791" s="15" t="n">
-        <v>472588.67</v>
+        <v>472682.47</v>
       </c>
       <c r="E791" s="15" t="n">
         <v>964506.48</v>
       </c>
       <c r="F791" s="16" t="n">
-        <v>0.2834</v>
+        <v>0.2836</v>
       </c>
       <c r="G791" s="16" t="n">
-        <v>0.2152</v>
+        <v>0.2153</v>
       </c>
       <c r="H791" s="16" t="n"/>
       <c r="I791" s="16" t="n">
-        <v>0.1139</v>
+        <v>0.1138</v>
       </c>
       <c r="J791" s="19" t="n">
-        <v>11374</v>
+        <v>11375</v>
       </c>
       <c r="K791" s="19" t="n">
-        <v>19574</v>
+        <v>19575</v>
       </c>
       <c r="L791" s="31" t="n">
         <v>0.7914</v>
@@ -43342,13 +43342,13 @@
         </is>
       </c>
       <c r="D792" s="9" t="n">
-        <v>678281.22</v>
+        <v>678310.71</v>
       </c>
       <c r="E792" s="9" t="n">
         <v>2332051.08</v>
       </c>
       <c r="F792" s="10" t="n">
-        <v>0.2305</v>
+        <v>0.2306</v>
       </c>
       <c r="G792" s="10" t="n">
         <v>0.1585</v>
@@ -43358,10 +43358,10 @@
         <v>0.074</v>
       </c>
       <c r="J792" s="13" t="n">
-        <v>25609</v>
+        <v>25611</v>
       </c>
       <c r="K792" s="13" t="n">
-        <v>31865</v>
+        <v>31867</v>
       </c>
       <c r="L792" s="32" t="n">
         <v>0.6948</v>
@@ -43384,7 +43384,7 @@
         </is>
       </c>
       <c r="D793" s="15" t="n">
-        <v>657224.3100000001</v>
+        <v>657224.77</v>
       </c>
       <c r="E793" s="15" t="n">
         <v>4787775.8</v>
@@ -43400,10 +43400,10 @@
         <v>0.048</v>
       </c>
       <c r="J793" s="19" t="n">
-        <v>35430</v>
+        <v>35431</v>
       </c>
       <c r="K793" s="19" t="n">
-        <v>46048</v>
+        <v>46049</v>
       </c>
       <c r="L793" s="31" t="n">
         <v>0.6681</v>
@@ -59428,10 +59428,10 @@
         </is>
       </c>
       <c r="D1175" s="15" t="n">
-        <v>79309028.84</v>
+        <v>79309875.31999999</v>
       </c>
       <c r="E1175" s="15" t="n">
-        <v>309735891.85</v>
+        <v>309736363.93</v>
       </c>
       <c r="F1175" s="16" t="n">
         <v>0.1418</v>
@@ -59444,10 +59444,10 @@
         <v>0.1064</v>
       </c>
       <c r="J1175" s="19" t="n">
-        <v>1820082</v>
+        <v>1820129</v>
       </c>
       <c r="K1175" s="19" t="n">
-        <v>3390748</v>
+        <v>3390814</v>
       </c>
       <c r="L1175" s="31" t="n">
         <v>0</v>
@@ -63292,7 +63292,7 @@
         </is>
       </c>
       <c r="D1267" s="15" t="n">
-        <v>9676086.789999999</v>
+        <v>9676132.15</v>
       </c>
       <c r="E1267" s="15" t="n">
         <v>174628159.3</v>
@@ -63308,10 +63308,10 @@
         <v>0.0302</v>
       </c>
       <c r="J1267" s="19" t="n">
-        <v>727684</v>
+        <v>727693</v>
       </c>
       <c r="K1267" s="19" t="n">
-        <v>1167309</v>
+        <v>1167318</v>
       </c>
       <c r="L1267" s="31" t="n">
         <v>0</v>
@@ -63334,10 +63334,10 @@
         </is>
       </c>
       <c r="D1268" s="9" t="n">
-        <v>22560125.91</v>
+        <v>22560470.46</v>
       </c>
       <c r="E1268" s="9" t="n">
-        <v>11101281.38</v>
+        <v>11101516.7</v>
       </c>
       <c r="F1268" s="10" t="n">
         <v>0.0667</v>
@@ -63350,10 +63350,10 @@
         <v>0.3131</v>
       </c>
       <c r="J1268" s="13" t="n">
-        <v>91944</v>
+        <v>91954</v>
       </c>
       <c r="K1268" s="13" t="n">
-        <v>366863</v>
+        <v>366881</v>
       </c>
       <c r="L1268" s="32" t="n">
         <v>0</v>
@@ -63376,7 +63376,7 @@
         </is>
       </c>
       <c r="D1269" s="15" t="n">
-        <v>14657942.52</v>
+        <v>14658098.41</v>
       </c>
       <c r="E1269" s="15" t="n">
         <v>12789129.68</v>
@@ -63392,10 +63392,10 @@
         <v>0.2491</v>
       </c>
       <c r="J1269" s="19" t="n">
-        <v>131330</v>
+        <v>131334</v>
       </c>
       <c r="K1269" s="19" t="n">
-        <v>326898</v>
+        <v>326904</v>
       </c>
       <c r="L1269" s="31" t="n">
         <v>0</v>
@@ -63418,10 +63418,10 @@
         </is>
       </c>
       <c r="D1270" s="9" t="n">
-        <v>10095172.32</v>
+        <v>10095229.1</v>
       </c>
       <c r="E1270" s="9" t="n">
-        <v>14843337.67</v>
+        <v>14843344</v>
       </c>
       <c r="F1270" s="10" t="n">
         <v>0.07000000000000001</v>
@@ -63434,10 +63434,10 @@
         <v>0.2039</v>
       </c>
       <c r="J1270" s="13" t="n">
-        <v>144788</v>
+        <v>144793</v>
       </c>
       <c r="K1270" s="13" t="n">
-        <v>296125</v>
+        <v>296134</v>
       </c>
       <c r="L1270" s="32" t="n">
         <v>0</v>
@@ -63460,7 +63460,7 @@
         </is>
       </c>
       <c r="D1271" s="15" t="n">
-        <v>6475565.4</v>
+        <v>6475578.55</v>
       </c>
       <c r="E1271" s="15" t="n">
         <v>15078900.22</v>
@@ -63476,10 +63476,10 @@
         <v>0.1676</v>
       </c>
       <c r="J1271" s="19" t="n">
-        <v>138728</v>
+        <v>138732</v>
       </c>
       <c r="K1271" s="19" t="n">
-        <v>253600</v>
+        <v>253605</v>
       </c>
       <c r="L1271" s="31" t="n">
         <v>0</v>
@@ -63502,13 +63502,13 @@
         </is>
       </c>
       <c r="D1272" s="9" t="n">
-        <v>8248997.09</v>
+        <v>8249146.83</v>
       </c>
       <c r="E1272" s="9" t="n">
         <v>29062271.59</v>
       </c>
       <c r="F1272" s="10" t="n">
-        <v>0.1424</v>
+        <v>0.1425</v>
       </c>
       <c r="G1272" s="10" t="n">
         <v>0.0757</v>
@@ -63518,10 +63518,10 @@
         <v>0.125</v>
       </c>
       <c r="J1272" s="13" t="n">
-        <v>262455</v>
+        <v>262466</v>
       </c>
       <c r="K1272" s="13" t="n">
-        <v>417596</v>
+        <v>417609</v>
       </c>
       <c r="L1272" s="32" t="n">
         <v>0</v>
@@ -63544,10 +63544,10 @@
         </is>
       </c>
       <c r="D1273" s="15" t="n">
-        <v>7595138.8</v>
+        <v>7595219.82</v>
       </c>
       <c r="E1273" s="15" t="n">
-        <v>52232812.01</v>
+        <v>52233042.45</v>
       </c>
       <c r="F1273" s="16" t="n">
         <v>0.2262</v>
@@ -63560,10 +63560,10 @@
         <v>0.0761</v>
       </c>
       <c r="J1273" s="19" t="n">
-        <v>323153</v>
+        <v>323157</v>
       </c>
       <c r="K1273" s="19" t="n">
-        <v>562357</v>
+        <v>562363</v>
       </c>
       <c r="L1273" s="31" t="n">
         <v>0</v>
@@ -68751,7 +68751,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-30 16:05 UTC</t>
+          <t>2026-10-30 17:04 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-31 15:28 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8641,7 +8641,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-31 14:27 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-31 15:28 UTC.</t>
         </is>
       </c>
     </row>
@@ -66847,7 +66847,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-31 14:27 UTC</t>
+          <t>2026-10-31 15:28 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
nfl hold refresh 2026-10-31 16:11 UTC
</commit_message>
<xml_diff>
--- a/nfl_hold.xlsx
+++ b/nfl_hold.xlsx
@@ -8641,7 +8641,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-31 15:28 UTC.</t>
+          <t>Hold = share of taker $ that takers lost (a sportsbook's hold). Green = house/makers won, red = takers won. Regular season + playoffs. Updated 2026-10-31 16:10 UTC.</t>
         </is>
       </c>
     </row>
@@ -66847,7 +66847,7 @@
       </c>
       <c r="B1" s="38" t="inlineStr">
         <is>
-          <t>2026-10-31 15:28 UTC</t>
+          <t>2026-10-31 16:10 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>